<commit_message>
add (exploratroy_DAG) (codebook) added more variables to the DAG
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Vaccine Uptake - R\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52FE9BDB-56C1-45FB-89BB-16B7F3A83CD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B878E925-4527-48F2-B61E-018908ACAF97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10890" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1310" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1294" uniqueCount="407">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -1246,9 +1246,6 @@
     <t xml:space="preserve">derive the time period in which the parent last received a dose of the covid vaccine: covid_vaccination_within6m and covid_vaccination_within1y bot == 0 (&gt;1y), covid_vaccination_6m == 0 and covid_vaccination_within_1y == 1 (&gt;6m and &lt;1y), covid_vacciantion_within6m == 1 (&lt;6m) </t>
   </si>
   <si>
-    <t>Ancestors/Descendants</t>
-  </si>
-  <si>
     <t>Legend</t>
   </si>
   <si>
@@ -1307,6 +1304,15 @@
   </si>
   <si>
     <t>Junior/Technical college</t>
+  </si>
+  <si>
+    <t>From (col) \ To (row)</t>
+  </si>
+  <si>
+    <t>Summary?</t>
+  </si>
+  <si>
+    <t>Vaccine uptake varies based on 3 different categories, can we leave it as a standalone variable</t>
   </si>
 </sst>
 </file>
@@ -1428,7 +1434,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1459,25 +1465,18 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <font>
-        <color theme="2" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <font>
         <color theme="2" tint="-0.24994659260841701"/>
@@ -1864,8 +1863,7 @@
     <col min="69" max="69" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="70" max="72" width="35.81640625" bestFit="1" customWidth="1"/>
     <col min="73" max="73" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="35.81640625" style="18" bestFit="1" customWidth="1"/>
-    <col min="75" max="77" width="35.81640625" bestFit="1" customWidth="1"/>
+    <col min="74" max="77" width="35.81640625" bestFit="1" customWidth="1"/>
     <col min="78" max="80" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="81" max="84" width="35.81640625" bestFit="1" customWidth="1"/>
     <col min="85" max="86" width="35.81640625" style="6" customWidth="1"/>
@@ -1912,7 +1910,7 @@
         <v>15</v>
       </c>
       <c r="M1" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="N1" t="s">
         <v>17</v>
@@ -2094,7 +2092,7 @@
       <c r="BU1" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="BV1" s="18" t="s">
+      <c r="BV1" t="s">
         <v>77</v>
       </c>
       <c r="BW1" t="s">
@@ -2128,10 +2126,10 @@
         <v>87</v>
       </c>
       <c r="CG1" s="6" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="CH1" s="6" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="CI1" s="8" t="s">
         <v>88</v>
@@ -2379,7 +2377,7 @@
       <c r="BU2" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="BV2" s="18" t="s">
+      <c r="BV2" t="s">
         <v>96</v>
       </c>
       <c r="BW2" t="s">
@@ -2482,7 +2480,7 @@
         <v>117</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="N3" s="2" t="s">
         <v>118</v>
@@ -2600,7 +2598,6 @@
       <c r="BU3" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="BV3" s="19"/>
       <c r="BW3" s="2" t="s">
         <v>144</v>
       </c>
@@ -2632,10 +2629,10 @@
         <v>153</v>
       </c>
       <c r="CG3" s="5" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="CH3" s="5" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="CI3" s="7"/>
       <c r="CJ3" s="2" t="s">
@@ -2876,8 +2873,8 @@
       <c r="BU4" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="BV4" s="18" t="s">
-        <v>401</v>
+      <c r="BV4" t="s">
+        <v>400</v>
       </c>
       <c r="BW4" t="s">
         <v>99</v>
@@ -3519,7 +3516,7 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C14" t="s">
         <v>268</v>
@@ -3528,10 +3525,10 @@
         <v>109</v>
       </c>
       <c r="E14" t="s">
+        <v>397</v>
+      </c>
+      <c r="F14" t="s">
         <v>398</v>
-      </c>
-      <c r="F14" t="s">
-        <v>399</v>
       </c>
       <c r="G14" t="s">
         <v>291</v>
@@ -4412,80 +4409,80 @@
         <v>183</v>
       </c>
     </row>
-    <row r="55" spans="1:13" s="18" customFormat="1">
-      <c r="A55" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="B55" s="18" t="s">
+    <row r="55" spans="1:13">
+      <c r="A55" t="s">
+        <v>96</v>
+      </c>
+      <c r="B55" t="s">
         <v>71</v>
       </c>
-      <c r="C55" s="18" t="s">
+      <c r="C55" t="s">
         <v>269</v>
       </c>
-      <c r="D55" s="18">
+      <c r="D55">
         <v>0</v>
       </c>
-      <c r="E55" s="18" t="s">
+      <c r="E55" t="s">
         <v>175</v>
       </c>
-      <c r="F55" s="18" t="s">
+      <c r="F55" t="s">
         <v>362</v>
       </c>
-      <c r="G55" s="18" t="s">
+      <c r="G55" t="s">
         <v>66</v>
       </c>
-      <c r="H55" s="18" t="s">
+      <c r="H55" t="s">
         <v>315</v>
       </c>
-      <c r="I55" s="18" t="s">
+      <c r="I55" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="56" spans="1:13" s="18" customFormat="1">
-      <c r="A56" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D56" s="18">
+    <row r="56" spans="1:13">
+      <c r="A56" t="s">
+        <v>96</v>
+      </c>
+      <c r="D56">
         <v>1</v>
       </c>
-      <c r="E56" s="18" t="s">
+      <c r="E56" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="57" spans="1:13" s="18" customFormat="1">
-      <c r="A57" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D57" s="18" t="s">
+    <row r="57" spans="1:13">
+      <c r="A57" t="s">
+        <v>96</v>
+      </c>
+      <c r="D57" t="s">
         <v>172</v>
       </c>
-      <c r="E57" s="18" t="s">
+      <c r="E57" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="58" spans="1:13" s="18" customFormat="1">
-      <c r="A58" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="B58" s="18" t="s">
+    <row r="58" spans="1:13">
+      <c r="A58" t="s">
+        <v>96</v>
+      </c>
+      <c r="B58" t="s">
         <v>73</v>
       </c>
-      <c r="C58" s="18" t="s">
+      <c r="C58" t="s">
         <v>269</v>
       </c>
-      <c r="D58" s="18">
+      <c r="D58">
         <v>0</v>
       </c>
-      <c r="E58" s="18" t="s">
+      <c r="E58" t="s">
         <v>170</v>
       </c>
-      <c r="F58" s="18" t="s">
+      <c r="F58" t="s">
         <v>363</v>
       </c>
-      <c r="G58" s="18" t="s">
+      <c r="G58" t="s">
         <v>58</v>
       </c>
-      <c r="H58" s="18" t="s">
+      <c r="H58" t="s">
         <v>315</v>
       </c>
     </row>
@@ -4764,244 +4761,244 @@
         <v>197</v>
       </c>
     </row>
-    <row r="79" spans="1:8" s="18" customFormat="1">
-      <c r="A79" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="B79" s="18" t="s">
+    <row r="79" spans="1:8">
+      <c r="A79" t="s">
+        <v>96</v>
+      </c>
+      <c r="B79" t="s">
         <v>77</v>
       </c>
-      <c r="C79" s="18" t="s">
+      <c r="C79" t="s">
         <v>269</v>
       </c>
-      <c r="D79" s="18">
+      <c r="D79">
         <v>1</v>
       </c>
-      <c r="E79" s="18" t="s">
+      <c r="E79" t="s">
         <v>184</v>
       </c>
-      <c r="F79" s="18" t="s">
+      <c r="F79" t="s">
         <v>367</v>
       </c>
-      <c r="G79" s="18" t="s">
+      <c r="G79" t="s">
         <v>330</v>
       </c>
-      <c r="H79" s="18" t="s">
+      <c r="H79" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="80" spans="1:8" s="18" customFormat="1">
-      <c r="A80" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D80" s="18">
+    <row r="80" spans="1:8">
+      <c r="A80" t="s">
+        <v>96</v>
+      </c>
+      <c r="D80">
         <f>D79 +1</f>
         <v>2</v>
       </c>
-      <c r="E80" s="18" t="s">
+      <c r="E80" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="81" spans="1:5" s="18" customFormat="1">
-      <c r="A81" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D81" s="18">
+    <row r="81" spans="1:5">
+      <c r="A81" t="s">
+        <v>96</v>
+      </c>
+      <c r="D81">
         <f t="shared" ref="D81:D96" si="0">D80 +1</f>
         <v>3</v>
       </c>
-      <c r="E81" s="18" t="s">
+      <c r="E81" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="82" spans="1:5" s="18" customFormat="1">
-      <c r="A82" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D82" s="18">
+    <row r="82" spans="1:5">
+      <c r="A82" t="s">
+        <v>96</v>
+      </c>
+      <c r="D82">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="E82" s="18" t="s">
+      <c r="E82" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="83" spans="1:5" s="18" customFormat="1">
-      <c r="A83" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D83" s="18">
+    <row r="83" spans="1:5">
+      <c r="A83" t="s">
+        <v>96</v>
+      </c>
+      <c r="D83">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="E83" s="18" t="s">
+      <c r="E83" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="84" spans="1:5" s="18" customFormat="1">
-      <c r="A84" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D84" s="18">
+    <row r="84" spans="1:5">
+      <c r="A84" t="s">
+        <v>96</v>
+      </c>
+      <c r="D84">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="E84" s="18" t="s">
+      <c r="E84" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="85" spans="1:5" s="18" customFormat="1">
-      <c r="A85" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D85" s="18">
+    <row r="85" spans="1:5">
+      <c r="A85" t="s">
+        <v>96</v>
+      </c>
+      <c r="D85">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="E85" s="18" t="s">
+      <c r="E85" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="86" spans="1:5" s="18" customFormat="1">
-      <c r="A86" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D86" s="18">
+    <row r="86" spans="1:5">
+      <c r="A86" t="s">
+        <v>96</v>
+      </c>
+      <c r="D86">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="E86" s="18" t="s">
+      <c r="E86" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="87" spans="1:5" s="18" customFormat="1">
-      <c r="A87" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D87" s="18">
+    <row r="87" spans="1:5">
+      <c r="A87" t="s">
+        <v>96</v>
+      </c>
+      <c r="D87">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="E87" s="18" t="s">
+      <c r="E87" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="88" spans="1:5" s="18" customFormat="1">
-      <c r="A88" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D88" s="18">
+    <row r="88" spans="1:5">
+      <c r="A88" t="s">
+        <v>96</v>
+      </c>
+      <c r="D88">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="E88" s="18" t="s">
+      <c r="E88" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="89" spans="1:5" s="18" customFormat="1">
-      <c r="A89" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D89" s="18">
+    <row r="89" spans="1:5">
+      <c r="A89" t="s">
+        <v>96</v>
+      </c>
+      <c r="D89">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="E89" s="18" t="s">
+      <c r="E89" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="90" spans="1:5" s="18" customFormat="1">
-      <c r="A90" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D90" s="18">
+    <row r="90" spans="1:5">
+      <c r="A90" t="s">
+        <v>96</v>
+      </c>
+      <c r="D90">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="E90" s="18" t="s">
+      <c r="E90" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="91" spans="1:5" s="18" customFormat="1">
-      <c r="A91" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D91" s="18">
+    <row r="91" spans="1:5">
+      <c r="A91" t="s">
+        <v>96</v>
+      </c>
+      <c r="D91">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="E91" s="18" t="s">
+      <c r="E91" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="92" spans="1:5" s="18" customFormat="1">
-      <c r="A92" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D92" s="18">
+    <row r="92" spans="1:5">
+      <c r="A92" t="s">
+        <v>96</v>
+      </c>
+      <c r="D92">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="E92" s="18" t="s">
+      <c r="E92" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="93" spans="1:5" s="18" customFormat="1">
-      <c r="A93" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D93" s="18">
+    <row r="93" spans="1:5">
+      <c r="A93" t="s">
+        <v>96</v>
+      </c>
+      <c r="D93">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="E93" s="18" t="s">
+      <c r="E93" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="94" spans="1:5" s="18" customFormat="1">
-      <c r="A94" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D94" s="18">
+    <row r="94" spans="1:5">
+      <c r="A94" t="s">
+        <v>96</v>
+      </c>
+      <c r="D94">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="E94" s="18" t="s">
+      <c r="E94" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="95" spans="1:5" s="18" customFormat="1">
-      <c r="A95" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D95" s="18">
+    <row r="95" spans="1:5">
+      <c r="A95" t="s">
+        <v>96</v>
+      </c>
+      <c r="D95">
         <f>D94 +1</f>
         <v>17</v>
       </c>
-      <c r="E95" s="18" t="s">
+      <c r="E95" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="96" spans="1:5" s="18" customFormat="1">
-      <c r="A96" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D96" s="18">
+    <row r="96" spans="1:5">
+      <c r="A96" t="s">
+        <v>96</v>
+      </c>
+      <c r="D96">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="E96" s="18" t="s">
+      <c r="E96" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="97" spans="1:17" s="18" customFormat="1">
-      <c r="A97" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D97" s="18" t="s">
+    <row r="97" spans="1:17">
+      <c r="A97" t="s">
+        <v>96</v>
+      </c>
+      <c r="D97" t="s">
         <v>172</v>
       </c>
-      <c r="E97" s="18" t="s">
+      <c r="E97" t="s">
         <v>197</v>
       </c>
     </row>
@@ -5720,7 +5717,7 @@
         <v>0</v>
       </c>
       <c r="E134" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="F134" t="s">
         <v>376</v>
@@ -5764,7 +5761,7 @@
         <v>1</v>
       </c>
       <c r="E135" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="136" spans="1:16">
@@ -5814,7 +5811,7 @@
         <v>0</v>
       </c>
       <c r="E139" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="F139" t="s">
         <v>377</v>
@@ -5858,7 +5855,7 @@
         <v>1</v>
       </c>
       <c r="E140" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="141" spans="1:16">
@@ -5908,7 +5905,7 @@
         <v>0</v>
       </c>
       <c r="E144" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="F144" t="s">
         <v>378</v>
@@ -5940,7 +5937,7 @@
         <v>1</v>
       </c>
       <c r="E145" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="146" spans="1:10">
@@ -6327,35 +6324,36 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9521944E-28B4-4113-A27F-3B841E118807}">
-  <dimension ref="A1:AW57"/>
+  <dimension ref="A1:AO48"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.36328125" customWidth="1"/>
     <col min="4" max="6" width="8.6328125" customWidth="1"/>
-    <col min="24" max="24" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8.36328125" customWidth="1"/>
-    <col min="35" max="35" width="11.08984375" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="9.26953125" customWidth="1"/>
-    <col min="41" max="41" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="42" max="43" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="8.6328125" customWidth="1"/>
-    <col min="45" max="45" width="9.26953125" customWidth="1"/>
-    <col min="46" max="46" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="18" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8.36328125" customWidth="1"/>
+    <col min="26" max="26" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="9.26953125" customWidth="1"/>
+    <col min="32" max="32" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="33" max="34" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="8.6328125" customWidth="1"/>
+    <col min="36" max="36" width="9.26953125" customWidth="1"/>
+    <col min="37" max="37" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="18" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="8.7265625" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" s="2" customFormat="1" ht="30" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>384</v>
+    <row r="1" spans="1:41" s="2" customFormat="1" ht="30" customHeight="1">
+      <c r="A1" s="18" t="s">
+        <v>404</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>5</v>
@@ -6391,485 +6389,1881 @@
         <v>15</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>19</v>
+        <v>62</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>26</v>
+        <v>71</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>63</v>
+        <v>75</v>
+      </c>
+      <c r="Z1" s="17" t="s">
+        <v>77</v>
       </c>
       <c r="AA1" s="2" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="AB1" s="2" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="AC1" s="2" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="AD1" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AE1" s="19" t="s">
-        <v>71</v>
+        <v>84</v>
+      </c>
+      <c r="AE1" s="2" t="s">
+        <v>85</v>
       </c>
       <c r="AF1" s="2" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="AG1" s="2" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="AH1" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="AI1" s="17" t="s">
-        <v>77</v>
+        <v>89</v>
+      </c>
+      <c r="AI1" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="AJ1" s="2" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="AK1" s="2" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="AL1" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="AM1" s="2" t="s">
-        <v>84</v>
+        <v>93</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>389</v>
       </c>
       <c r="AN1" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AO1" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="AP1" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="AQ1" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AR1" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="AS1" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AT1" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="AU1" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="AV1" t="s">
-        <v>390</v>
-      </c>
-      <c r="AW1" s="2" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="2" spans="1:49">
+        <v>388</v>
+      </c>
+      <c r="AO1" s="20" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="2" spans="1:41">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:49">
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="19"/>
+      <c r="S2" s="19"/>
+      <c r="T2" s="19"/>
+      <c r="U2" s="19"/>
+      <c r="V2" s="19"/>
+      <c r="W2" s="19"/>
+      <c r="X2" s="19"/>
+      <c r="Y2" s="19"/>
+      <c r="Z2" s="19"/>
+      <c r="AA2" s="19"/>
+      <c r="AB2" s="19"/>
+      <c r="AC2" s="19"/>
+      <c r="AD2" s="19"/>
+      <c r="AE2" s="19"/>
+      <c r="AF2" s="19"/>
+      <c r="AG2" s="19"/>
+      <c r="AH2" s="19"/>
+      <c r="AI2" s="19"/>
+      <c r="AJ2" s="19"/>
+      <c r="AK2" s="19"/>
+      <c r="AL2" s="19"/>
+      <c r="AM2" s="19"/>
+      <c r="AN2" s="19"/>
+    </row>
+    <row r="3" spans="1:41">
       <c r="A3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:49">
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19"/>
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+      <c r="W3" s="19"/>
+      <c r="X3" s="19"/>
+      <c r="Y3" s="19"/>
+      <c r="Z3" s="19"/>
+      <c r="AA3" s="19"/>
+      <c r="AB3" s="19"/>
+      <c r="AC3" s="19"/>
+      <c r="AD3" s="19"/>
+      <c r="AE3" s="19"/>
+      <c r="AF3" s="19"/>
+      <c r="AG3" s="19"/>
+      <c r="AH3" s="19"/>
+      <c r="AI3" s="19"/>
+      <c r="AJ3" s="19"/>
+      <c r="AK3" s="19"/>
+      <c r="AL3" s="19"/>
+      <c r="AM3" s="19"/>
+      <c r="AN3" s="19"/>
+    </row>
+    <row r="4" spans="1:41">
       <c r="A4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:49">
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="19"/>
+      <c r="W4" s="19"/>
+      <c r="X4" s="19"/>
+      <c r="Y4" s="19"/>
+      <c r="Z4" s="19"/>
+      <c r="AA4" s="19"/>
+      <c r="AB4" s="19"/>
+      <c r="AC4" s="19"/>
+      <c r="AD4" s="19"/>
+      <c r="AE4" s="19"/>
+      <c r="AF4" s="19"/>
+      <c r="AG4" s="19"/>
+      <c r="AH4" s="19"/>
+      <c r="AI4" s="19"/>
+      <c r="AJ4" s="19"/>
+      <c r="AK4" s="19"/>
+      <c r="AL4" s="19"/>
+      <c r="AM4" s="19"/>
+      <c r="AN4" s="19"/>
+    </row>
+    <row r="5" spans="1:41">
       <c r="A5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:49">
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+      <c r="V5" s="19"/>
+      <c r="W5" s="19"/>
+      <c r="X5" s="19"/>
+      <c r="Y5" s="19"/>
+      <c r="Z5" s="19"/>
+      <c r="AA5" s="19"/>
+      <c r="AB5" s="19"/>
+      <c r="AC5" s="19"/>
+      <c r="AD5" s="19"/>
+      <c r="AE5" s="19"/>
+      <c r="AF5" s="19"/>
+      <c r="AG5" s="19"/>
+      <c r="AH5" s="19"/>
+      <c r="AI5" s="19"/>
+      <c r="AJ5" s="19"/>
+      <c r="AK5" s="19"/>
+      <c r="AL5" s="19"/>
+      <c r="AM5" s="19"/>
+      <c r="AN5" s="19"/>
+    </row>
+    <row r="6" spans="1:41">
       <c r="A6" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:49">
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="19"/>
+      <c r="Q6" s="19"/>
+      <c r="R6" s="19"/>
+      <c r="S6" s="19"/>
+      <c r="T6" s="19"/>
+      <c r="U6" s="19"/>
+      <c r="V6" s="19"/>
+      <c r="W6" s="19"/>
+      <c r="X6" s="19"/>
+      <c r="Y6" s="19"/>
+      <c r="Z6" s="19"/>
+      <c r="AA6" s="19"/>
+      <c r="AB6" s="19"/>
+      <c r="AC6" s="19"/>
+      <c r="AD6" s="19"/>
+      <c r="AE6" s="19"/>
+      <c r="AF6" s="19"/>
+      <c r="AG6" s="19"/>
+      <c r="AH6" s="19"/>
+      <c r="AI6" s="19"/>
+      <c r="AJ6" s="19"/>
+      <c r="AK6" s="19"/>
+      <c r="AL6" s="19"/>
+      <c r="AM6" s="19"/>
+      <c r="AN6" s="19"/>
+    </row>
+    <row r="7" spans="1:41">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:49">
+      <c r="B7" s="19"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="19"/>
+      <c r="T7" s="19"/>
+      <c r="U7" s="19"/>
+      <c r="V7" s="19"/>
+      <c r="W7" s="19"/>
+      <c r="X7" s="19"/>
+      <c r="Y7" s="19"/>
+      <c r="Z7" s="19"/>
+      <c r="AA7" s="19"/>
+      <c r="AB7" s="19"/>
+      <c r="AC7" s="19"/>
+      <c r="AD7" s="19"/>
+      <c r="AE7" s="19"/>
+      <c r="AF7" s="19"/>
+      <c r="AG7" s="19"/>
+      <c r="AH7" s="19"/>
+      <c r="AI7" s="19"/>
+      <c r="AJ7" s="19"/>
+      <c r="AK7" s="19"/>
+      <c r="AL7" s="19"/>
+      <c r="AM7" s="19"/>
+      <c r="AN7" s="19"/>
+    </row>
+    <row r="8" spans="1:41">
       <c r="A8" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:49">
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="19"/>
+      <c r="S8" s="19"/>
+      <c r="T8" s="19"/>
+      <c r="U8" s="19"/>
+      <c r="V8" s="19"/>
+      <c r="W8" s="19"/>
+      <c r="X8" s="19"/>
+      <c r="Y8" s="19"/>
+      <c r="Z8" s="19"/>
+      <c r="AA8" s="19"/>
+      <c r="AB8" s="19"/>
+      <c r="AC8" s="19"/>
+      <c r="AD8" s="19"/>
+      <c r="AE8" s="19"/>
+      <c r="AF8" s="19"/>
+      <c r="AG8" s="19"/>
+      <c r="AH8" s="19"/>
+      <c r="AI8" s="19"/>
+      <c r="AJ8" s="19"/>
+      <c r="AK8" s="19"/>
+      <c r="AL8" s="19"/>
+      <c r="AM8" s="19"/>
+      <c r="AN8" s="19"/>
+    </row>
+    <row r="9" spans="1:41">
       <c r="A9" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="10" spans="1:49">
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="19"/>
+      <c r="U9" s="19"/>
+      <c r="V9" s="19"/>
+      <c r="W9" s="19"/>
+      <c r="X9" s="19"/>
+      <c r="Y9" s="19"/>
+      <c r="Z9" s="19"/>
+      <c r="AA9" s="19"/>
+      <c r="AB9" s="19"/>
+      <c r="AC9" s="19"/>
+      <c r="AD9" s="19"/>
+      <c r="AE9" s="19"/>
+      <c r="AF9" s="19"/>
+      <c r="AG9" s="19"/>
+      <c r="AH9" s="19"/>
+      <c r="AI9" s="19"/>
+      <c r="AJ9" s="19"/>
+      <c r="AK9" s="19"/>
+      <c r="AL9" s="19"/>
+      <c r="AM9" s="19"/>
+      <c r="AN9" s="19"/>
+    </row>
+    <row r="10" spans="1:41">
       <c r="A10" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="11" spans="1:49">
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="19"/>
+      <c r="Q10" s="19"/>
+      <c r="R10" s="19"/>
+      <c r="S10" s="19"/>
+      <c r="T10" s="19"/>
+      <c r="U10" s="19"/>
+      <c r="V10" s="19"/>
+      <c r="W10" s="19"/>
+      <c r="X10" s="19"/>
+      <c r="Y10" s="19"/>
+      <c r="Z10" s="19"/>
+      <c r="AA10" s="19"/>
+      <c r="AB10" s="19"/>
+      <c r="AC10" s="19"/>
+      <c r="AD10" s="19"/>
+      <c r="AE10" s="19"/>
+      <c r="AF10" s="19"/>
+      <c r="AG10" s="19"/>
+      <c r="AH10" s="19"/>
+      <c r="AI10" s="19"/>
+      <c r="AJ10" s="19"/>
+      <c r="AK10" s="19"/>
+      <c r="AL10" s="19"/>
+      <c r="AM10" s="19"/>
+      <c r="AN10" s="19"/>
+    </row>
+    <row r="11" spans="1:41">
       <c r="A11" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="12" spans="1:49">
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
+      <c r="L11" s="19"/>
+      <c r="M11" s="19"/>
+      <c r="N11" s="19"/>
+      <c r="O11" s="19"/>
+      <c r="P11" s="19"/>
+      <c r="Q11" s="19"/>
+      <c r="R11" s="19"/>
+      <c r="S11" s="19"/>
+      <c r="T11" s="19"/>
+      <c r="U11" s="19"/>
+      <c r="V11" s="19"/>
+      <c r="W11" s="19"/>
+      <c r="X11" s="19"/>
+      <c r="Y11" s="19"/>
+      <c r="Z11" s="19"/>
+      <c r="AA11" s="19"/>
+      <c r="AB11" s="19"/>
+      <c r="AC11" s="19"/>
+      <c r="AD11" s="19"/>
+      <c r="AE11" s="19"/>
+      <c r="AF11" s="19"/>
+      <c r="AG11" s="19"/>
+      <c r="AH11" s="19"/>
+      <c r="AI11" s="19"/>
+      <c r="AJ11" s="19"/>
+      <c r="AK11" s="19"/>
+      <c r="AL11" s="19"/>
+      <c r="AM11" s="19"/>
+      <c r="AN11" s="19"/>
+    </row>
+    <row r="12" spans="1:41">
       <c r="A12" t="s">
         <v>15</v>
       </c>
-      <c r="AH12" s="16"/>
-      <c r="AW12" s="16"/>
-    </row>
-    <row r="13" spans="1:49">
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="19"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="19"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="19"/>
+      <c r="Q12" s="19"/>
+      <c r="R12" s="19"/>
+      <c r="S12" s="19"/>
+      <c r="T12" s="19"/>
+      <c r="U12" s="19"/>
+      <c r="V12" s="19"/>
+      <c r="W12" s="19"/>
+      <c r="X12" s="19"/>
+      <c r="Y12" s="19"/>
+      <c r="Z12" s="19"/>
+      <c r="AA12" s="19"/>
+      <c r="AB12" s="19"/>
+      <c r="AC12" s="19"/>
+      <c r="AD12" s="19"/>
+      <c r="AE12" s="19"/>
+      <c r="AF12" s="19"/>
+      <c r="AG12" s="19"/>
+      <c r="AH12" s="19"/>
+      <c r="AI12" s="19"/>
+      <c r="AJ12" s="19"/>
+      <c r="AK12" s="19"/>
+      <c r="AL12" s="19"/>
+      <c r="AM12" s="19"/>
+      <c r="AN12" s="16"/>
+      <c r="AO12" s="11" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="13" spans="1:41">
       <c r="A13" t="s">
-        <v>397</v>
-      </c>
-      <c r="AW13" s="16"/>
-    </row>
-    <row r="14" spans="1:49">
+        <v>396</v>
+      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="19"/>
+      <c r="N13" s="19"/>
+      <c r="O13" s="19"/>
+      <c r="P13" s="19"/>
+      <c r="Q13" s="19"/>
+      <c r="R13" s="19"/>
+      <c r="S13" s="19"/>
+      <c r="T13" s="19"/>
+      <c r="U13" s="19"/>
+      <c r="V13" s="19"/>
+      <c r="W13" s="19"/>
+      <c r="X13" s="19"/>
+      <c r="Y13" s="19"/>
+      <c r="Z13" s="19"/>
+      <c r="AA13" s="19"/>
+      <c r="AB13" s="19"/>
+      <c r="AC13" s="19"/>
+      <c r="AD13" s="19"/>
+      <c r="AE13" s="19"/>
+      <c r="AF13" s="19"/>
+      <c r="AG13" s="19"/>
+      <c r="AH13" s="19"/>
+      <c r="AI13" s="19"/>
+      <c r="AJ13" s="19"/>
+      <c r="AK13" s="19"/>
+      <c r="AL13" s="19"/>
+      <c r="AM13" s="19"/>
+      <c r="AN13" s="16"/>
+    </row>
+    <row r="14" spans="1:41">
       <c r="A14" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="1:49">
+        <v>60</v>
+      </c>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="19"/>
+      <c r="L14" s="19"/>
+      <c r="M14" s="19"/>
+      <c r="N14" s="19"/>
+      <c r="O14" s="19"/>
+      <c r="P14" s="19"/>
+      <c r="Q14" s="19"/>
+      <c r="R14" s="16"/>
+      <c r="S14" s="19"/>
+      <c r="T14" s="19"/>
+      <c r="U14" s="19"/>
+      <c r="V14" s="19"/>
+      <c r="W14" s="19"/>
+      <c r="X14" s="19"/>
+      <c r="Y14" s="19"/>
+      <c r="Z14" s="16"/>
+      <c r="AA14" s="19"/>
+      <c r="AB14" s="19"/>
+      <c r="AC14" s="16"/>
+      <c r="AD14" s="16"/>
+      <c r="AE14" s="19"/>
+      <c r="AF14" s="19"/>
+      <c r="AG14" s="19"/>
+      <c r="AH14" s="19"/>
+      <c r="AI14" s="19"/>
+      <c r="AJ14" s="19"/>
+      <c r="AK14" s="19"/>
+      <c r="AL14" s="19"/>
+      <c r="AM14" s="19"/>
+      <c r="AN14" s="16"/>
+    </row>
+    <row r="15" spans="1:41">
       <c r="A15" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:49">
+        <v>61</v>
+      </c>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
+      <c r="I15" s="19"/>
+      <c r="J15" s="19"/>
+      <c r="K15" s="19"/>
+      <c r="L15" s="19"/>
+      <c r="M15" s="19"/>
+      <c r="N15" s="19"/>
+      <c r="O15" s="19"/>
+      <c r="P15" s="19"/>
+      <c r="Q15" s="19"/>
+      <c r="R15" s="19"/>
+      <c r="S15" s="19"/>
+      <c r="T15" s="19"/>
+      <c r="U15" s="19"/>
+      <c r="V15" s="19"/>
+      <c r="W15" s="19"/>
+      <c r="X15" s="19"/>
+      <c r="Y15" s="19"/>
+      <c r="Z15" s="19"/>
+      <c r="AA15" s="19"/>
+      <c r="AB15" s="19"/>
+      <c r="AC15" s="19"/>
+      <c r="AD15" s="19"/>
+      <c r="AE15" s="19"/>
+      <c r="AF15" s="19"/>
+      <c r="AG15" s="19"/>
+      <c r="AH15" s="19"/>
+      <c r="AI15" s="19"/>
+      <c r="AJ15" s="19"/>
+      <c r="AK15" s="19"/>
+      <c r="AL15" s="19"/>
+      <c r="AM15" s="19"/>
+      <c r="AN15" s="19"/>
+    </row>
+    <row r="16" spans="1:41">
       <c r="A16" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:49">
+        <v>62</v>
+      </c>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
+      <c r="O16" s="19"/>
+      <c r="P16" s="19"/>
+      <c r="Q16" s="19"/>
+      <c r="R16" s="19"/>
+      <c r="S16" s="19"/>
+      <c r="T16" s="19"/>
+      <c r="U16" s="19"/>
+      <c r="V16" s="19"/>
+      <c r="W16" s="19"/>
+      <c r="X16" s="19"/>
+      <c r="Y16" s="19"/>
+      <c r="Z16" s="19"/>
+      <c r="AA16" s="19"/>
+      <c r="AB16" s="19"/>
+      <c r="AC16" s="19"/>
+      <c r="AD16" s="19"/>
+      <c r="AE16" s="19"/>
+      <c r="AF16" s="19"/>
+      <c r="AG16" s="19"/>
+      <c r="AH16" s="19"/>
+      <c r="AI16" s="19"/>
+      <c r="AJ16" s="19"/>
+      <c r="AK16" s="19"/>
+      <c r="AL16" s="19"/>
+      <c r="AM16" s="16"/>
+      <c r="AN16" s="19"/>
+    </row>
+    <row r="17" spans="1:40">
       <c r="A17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:49">
+        <v>63</v>
+      </c>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="19"/>
+      <c r="K17" s="19"/>
+      <c r="L17" s="19"/>
+      <c r="M17" s="19"/>
+      <c r="N17" s="19"/>
+      <c r="O17" s="19"/>
+      <c r="P17" s="19"/>
+      <c r="Q17" s="19"/>
+      <c r="R17" s="19"/>
+      <c r="S17" s="19"/>
+      <c r="T17" s="19"/>
+      <c r="U17" s="19"/>
+      <c r="V17" s="19"/>
+      <c r="W17" s="19"/>
+      <c r="X17" s="19"/>
+      <c r="Y17" s="19"/>
+      <c r="Z17" s="19"/>
+      <c r="AA17" s="19"/>
+      <c r="AB17" s="19"/>
+      <c r="AC17" s="19"/>
+      <c r="AD17" s="19"/>
+      <c r="AE17" s="19"/>
+      <c r="AF17" s="19"/>
+      <c r="AG17" s="19"/>
+      <c r="AH17" s="19"/>
+      <c r="AI17" s="19"/>
+      <c r="AJ17" s="19"/>
+      <c r="AK17" s="19"/>
+      <c r="AL17" s="19"/>
+      <c r="AM17" s="16"/>
+      <c r="AN17" s="19"/>
+    </row>
+    <row r="18" spans="1:40">
       <c r="A18" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="19" spans="1:49">
+        <v>64</v>
+      </c>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="19"/>
+      <c r="L18" s="19"/>
+      <c r="M18" s="19"/>
+      <c r="N18" s="19"/>
+      <c r="O18" s="19"/>
+      <c r="P18" s="16"/>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="19"/>
+      <c r="S18" s="19"/>
+      <c r="T18" s="19"/>
+      <c r="U18" s="19"/>
+      <c r="V18" s="19"/>
+      <c r="W18" s="19"/>
+      <c r="X18" s="19"/>
+      <c r="Y18" s="19"/>
+      <c r="Z18" s="19"/>
+      <c r="AA18" s="19"/>
+      <c r="AB18" s="19"/>
+      <c r="AC18" s="19"/>
+      <c r="AD18" s="19"/>
+      <c r="AE18" s="19"/>
+      <c r="AF18" s="19"/>
+      <c r="AG18" s="19"/>
+      <c r="AH18" s="19"/>
+      <c r="AI18" s="19"/>
+      <c r="AJ18" s="19"/>
+      <c r="AK18" s="19"/>
+      <c r="AL18" s="19"/>
+      <c r="AM18" s="16"/>
+      <c r="AN18" s="19"/>
+    </row>
+    <row r="19" spans="1:40">
       <c r="A19" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" spans="1:49">
+        <v>65</v>
+      </c>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="19"/>
+      <c r="N19" s="19"/>
+      <c r="O19" s="19"/>
+      <c r="P19" s="19"/>
+      <c r="Q19" s="19"/>
+      <c r="R19" s="19"/>
+      <c r="S19" s="19"/>
+      <c r="T19" s="19"/>
+      <c r="U19" s="19"/>
+      <c r="V19" s="19"/>
+      <c r="W19" s="19"/>
+      <c r="X19" s="19"/>
+      <c r="Y19" s="19"/>
+      <c r="Z19" s="19"/>
+      <c r="AA19" s="19"/>
+      <c r="AB19" s="19"/>
+      <c r="AC19" s="19"/>
+      <c r="AD19" s="19"/>
+      <c r="AE19" s="19"/>
+      <c r="AF19" s="19"/>
+      <c r="AG19" s="19"/>
+      <c r="AH19" s="19"/>
+      <c r="AI19" s="19"/>
+      <c r="AJ19" s="19"/>
+      <c r="AK19" s="19"/>
+      <c r="AL19" s="19"/>
+      <c r="AM19" s="19"/>
+      <c r="AN19" s="19"/>
+    </row>
+    <row r="20" spans="1:40">
       <c r="A20" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="21" spans="1:49">
+        <v>66</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="19"/>
+      <c r="N20" s="19"/>
+      <c r="O20" s="19"/>
+      <c r="P20" s="19"/>
+      <c r="Q20" s="19"/>
+      <c r="R20" s="19"/>
+      <c r="S20" s="19"/>
+      <c r="T20" s="19"/>
+      <c r="U20" s="19"/>
+      <c r="V20" s="19"/>
+      <c r="W20" s="19"/>
+      <c r="X20" s="19"/>
+      <c r="Y20" s="19"/>
+      <c r="Z20" s="19"/>
+      <c r="AA20" s="19"/>
+      <c r="AB20" s="19"/>
+      <c r="AC20" s="19"/>
+      <c r="AD20" s="19"/>
+      <c r="AE20" s="19"/>
+      <c r="AF20" s="19"/>
+      <c r="AG20" s="19"/>
+      <c r="AH20" s="19"/>
+      <c r="AI20" s="19"/>
+      <c r="AJ20" s="19"/>
+      <c r="AK20" s="19"/>
+      <c r="AL20" s="19"/>
+      <c r="AM20" s="19"/>
+      <c r="AN20" s="19"/>
+    </row>
+    <row r="21" spans="1:40">
       <c r="A21" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" spans="1:49">
+        <v>69</v>
+      </c>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="19"/>
+      <c r="J21" s="19"/>
+      <c r="K21" s="19"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
+      <c r="N21" s="19"/>
+      <c r="O21" s="19"/>
+      <c r="P21" s="19"/>
+      <c r="Q21" s="16"/>
+      <c r="R21" s="19"/>
+      <c r="S21" s="19"/>
+      <c r="T21" s="19"/>
+      <c r="U21" s="19"/>
+      <c r="V21" s="19"/>
+      <c r="W21" s="19"/>
+      <c r="X21" s="19"/>
+      <c r="Y21" s="19"/>
+      <c r="Z21" s="19"/>
+      <c r="AA21" s="19"/>
+      <c r="AB21" s="19"/>
+      <c r="AC21" s="19"/>
+      <c r="AD21" s="19"/>
+      <c r="AE21" s="19"/>
+      <c r="AF21" s="19"/>
+      <c r="AG21" s="19"/>
+      <c r="AH21" s="19"/>
+      <c r="AI21" s="19"/>
+      <c r="AJ21" s="19"/>
+      <c r="AK21" s="19"/>
+      <c r="AL21" s="19"/>
+      <c r="AM21" s="16"/>
+      <c r="AN21" s="19"/>
+    </row>
+    <row r="22" spans="1:40">
       <c r="A22" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="23" spans="1:49">
+        <v>71</v>
+      </c>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="19"/>
+      <c r="K22" s="19"/>
+      <c r="L22" s="19"/>
+      <c r="M22" s="19"/>
+      <c r="N22" s="16"/>
+      <c r="O22" s="19"/>
+      <c r="P22" s="19"/>
+      <c r="Q22" s="16"/>
+      <c r="R22" s="19"/>
+      <c r="S22" s="19"/>
+      <c r="T22" s="19"/>
+      <c r="U22" s="19"/>
+      <c r="V22" s="19"/>
+      <c r="W22" s="19"/>
+      <c r="X22" s="19"/>
+      <c r="Y22" s="19"/>
+      <c r="Z22" s="16"/>
+      <c r="AA22" s="16"/>
+      <c r="AB22" s="19"/>
+      <c r="AC22" s="19"/>
+      <c r="AD22" s="16"/>
+      <c r="AE22" s="19"/>
+      <c r="AF22" s="19"/>
+      <c r="AG22" s="19"/>
+      <c r="AH22" s="19"/>
+      <c r="AI22" s="19"/>
+      <c r="AJ22" s="19"/>
+      <c r="AK22" s="19"/>
+      <c r="AL22" s="19"/>
+      <c r="AM22" s="16"/>
+      <c r="AN22" s="19"/>
+    </row>
+    <row r="23" spans="1:40">
       <c r="A23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AI23" s="16"/>
-      <c r="AM23" s="16"/>
-      <c r="AW23" s="16"/>
-    </row>
-    <row r="24" spans="1:49">
+        <v>73</v>
+      </c>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
+      <c r="L23" s="19"/>
+      <c r="M23" s="19"/>
+      <c r="N23" s="19"/>
+      <c r="O23" s="19"/>
+      <c r="P23" s="19"/>
+      <c r="Q23" s="19"/>
+      <c r="R23" s="19"/>
+      <c r="S23" s="19"/>
+      <c r="T23" s="19"/>
+      <c r="U23" s="19"/>
+      <c r="V23" s="19"/>
+      <c r="W23" s="19"/>
+      <c r="X23" s="19"/>
+      <c r="Y23" s="19"/>
+      <c r="Z23" s="19"/>
+      <c r="AA23" s="19"/>
+      <c r="AB23" s="19"/>
+      <c r="AC23" s="19"/>
+      <c r="AD23" s="19"/>
+      <c r="AE23" s="19"/>
+      <c r="AF23" s="19"/>
+      <c r="AG23" s="19"/>
+      <c r="AH23" s="19"/>
+      <c r="AI23" s="19"/>
+      <c r="AJ23" s="19"/>
+      <c r="AK23" s="19"/>
+      <c r="AL23" s="19"/>
+      <c r="AM23" s="19"/>
+      <c r="AN23" s="19"/>
+    </row>
+    <row r="24" spans="1:40">
       <c r="A24" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="25" spans="1:49">
+        <v>74</v>
+      </c>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19"/>
+      <c r="J24" s="19"/>
+      <c r="K24" s="19"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="19"/>
+      <c r="N24" s="19"/>
+      <c r="O24" s="19"/>
+      <c r="P24" s="19"/>
+      <c r="Q24" s="19"/>
+      <c r="R24" s="19"/>
+      <c r="S24" s="19"/>
+      <c r="T24" s="19"/>
+      <c r="U24" s="19"/>
+      <c r="V24" s="19"/>
+      <c r="W24" s="19"/>
+      <c r="X24" s="19"/>
+      <c r="Y24" s="19"/>
+      <c r="Z24" s="19"/>
+      <c r="AA24" s="19"/>
+      <c r="AB24" s="19"/>
+      <c r="AC24" s="19"/>
+      <c r="AD24" s="19"/>
+      <c r="AE24" s="19"/>
+      <c r="AF24" s="19"/>
+      <c r="AG24" s="19"/>
+      <c r="AH24" s="19"/>
+      <c r="AI24" s="19"/>
+      <c r="AJ24" s="19"/>
+      <c r="AK24" s="19"/>
+      <c r="AL24" s="19"/>
+      <c r="AM24" s="19"/>
+      <c r="AN24" s="19"/>
+    </row>
+    <row r="25" spans="1:40">
       <c r="A25" t="s">
-        <v>62</v>
-      </c>
-      <c r="AV25" s="16"/>
-    </row>
-    <row r="26" spans="1:49">
+        <v>75</v>
+      </c>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="19"/>
+      <c r="J25" s="19"/>
+      <c r="K25" s="19"/>
+      <c r="L25" s="19"/>
+      <c r="M25" s="19"/>
+      <c r="N25" s="19"/>
+      <c r="O25" s="19"/>
+      <c r="P25" s="16"/>
+      <c r="Q25" s="19"/>
+      <c r="R25" s="19"/>
+      <c r="S25" s="19"/>
+      <c r="T25" s="19"/>
+      <c r="U25" s="19"/>
+      <c r="V25" s="19"/>
+      <c r="W25" s="19"/>
+      <c r="X25" s="19"/>
+      <c r="Y25" s="19"/>
+      <c r="Z25" s="19"/>
+      <c r="AA25" s="16"/>
+      <c r="AB25" s="19"/>
+      <c r="AC25" s="19"/>
+      <c r="AD25" s="19"/>
+      <c r="AE25" s="19"/>
+      <c r="AF25" s="19"/>
+      <c r="AG25" s="19"/>
+      <c r="AH25" s="19"/>
+      <c r="AI25" s="19"/>
+      <c r="AJ25" s="19"/>
+      <c r="AK25" s="19"/>
+      <c r="AL25" s="19"/>
+      <c r="AM25" s="16"/>
+      <c r="AN25" s="19"/>
+    </row>
+    <row r="26" spans="1:40">
       <c r="A26" t="s">
-        <v>63</v>
-      </c>
-      <c r="AV26" s="16"/>
-    </row>
-    <row r="27" spans="1:49">
+        <v>77</v>
+      </c>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="19"/>
+      <c r="J26" s="19"/>
+      <c r="K26" s="19"/>
+      <c r="L26" s="19"/>
+      <c r="M26" s="19"/>
+      <c r="N26" s="19"/>
+      <c r="O26" s="19"/>
+      <c r="P26" s="19"/>
+      <c r="Q26" s="19"/>
+      <c r="R26" s="16"/>
+      <c r="S26" s="19"/>
+      <c r="T26" s="19"/>
+      <c r="U26" s="16"/>
+      <c r="V26" s="19"/>
+      <c r="W26" s="19"/>
+      <c r="X26" s="19"/>
+      <c r="Y26" s="19"/>
+      <c r="Z26" s="19"/>
+      <c r="AA26" s="19"/>
+      <c r="AB26" s="19"/>
+      <c r="AC26" s="19"/>
+      <c r="AD26" s="19"/>
+      <c r="AE26" s="19"/>
+      <c r="AF26" s="19"/>
+      <c r="AG26" s="19"/>
+      <c r="AH26" s="19"/>
+      <c r="AI26" s="19"/>
+      <c r="AJ26" s="19"/>
+      <c r="AK26" s="19"/>
+      <c r="AL26" s="19"/>
+      <c r="AM26" s="16"/>
+      <c r="AN26" s="16"/>
+    </row>
+    <row r="27" spans="1:40">
       <c r="A27" t="s">
-        <v>64</v>
-      </c>
-      <c r="Y27" s="16"/>
-      <c r="Z27" s="16"/>
-      <c r="AV27" s="16"/>
-    </row>
-    <row r="28" spans="1:49">
+        <v>78</v>
+      </c>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="19"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="19"/>
+      <c r="K27" s="19"/>
+      <c r="L27" s="19"/>
+      <c r="M27" s="19"/>
+      <c r="N27" s="19"/>
+      <c r="O27" s="19"/>
+      <c r="P27" s="16"/>
+      <c r="Q27" s="19"/>
+      <c r="R27" s="19"/>
+      <c r="S27" s="19"/>
+      <c r="T27" s="19"/>
+      <c r="U27" s="19"/>
+      <c r="V27" s="16"/>
+      <c r="W27" s="19"/>
+      <c r="X27" s="19"/>
+      <c r="Y27" s="19"/>
+      <c r="Z27" s="19"/>
+      <c r="AA27" s="19"/>
+      <c r="AB27" s="19"/>
+      <c r="AC27" s="19"/>
+      <c r="AD27" s="19"/>
+      <c r="AE27" s="19"/>
+      <c r="AF27" s="19"/>
+      <c r="AG27" s="19"/>
+      <c r="AH27" s="19"/>
+      <c r="AI27" s="16"/>
+      <c r="AJ27" s="16"/>
+      <c r="AK27" s="16"/>
+      <c r="AL27" s="19"/>
+      <c r="AM27" s="19"/>
+      <c r="AN27" s="16"/>
+    </row>
+    <row r="28" spans="1:40">
       <c r="A28" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="29" spans="1:49">
+        <v>79</v>
+      </c>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="19"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="19"/>
+      <c r="N28" s="19"/>
+      <c r="O28" s="19"/>
+      <c r="P28" s="19"/>
+      <c r="Q28" s="19"/>
+      <c r="R28" s="16"/>
+      <c r="S28" s="19"/>
+      <c r="T28" s="19"/>
+      <c r="U28" s="19"/>
+      <c r="V28" s="19"/>
+      <c r="W28" s="19"/>
+      <c r="X28" s="19"/>
+      <c r="Y28" s="19"/>
+      <c r="Z28" s="16"/>
+      <c r="AA28" s="19"/>
+      <c r="AB28" s="19"/>
+      <c r="AC28" s="19"/>
+      <c r="AD28" s="19"/>
+      <c r="AE28" s="19"/>
+      <c r="AF28" s="19"/>
+      <c r="AG28" s="19"/>
+      <c r="AH28" s="19"/>
+      <c r="AI28" s="19"/>
+      <c r="AJ28" s="19"/>
+      <c r="AK28" s="19"/>
+      <c r="AL28" s="19"/>
+      <c r="AM28" s="19"/>
+      <c r="AN28" s="19"/>
+    </row>
+    <row r="29" spans="1:40">
       <c r="A29" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="30" spans="1:49">
+        <v>80</v>
+      </c>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="19"/>
+      <c r="K29" s="19"/>
+      <c r="L29" s="19"/>
+      <c r="M29" s="19"/>
+      <c r="N29" s="19"/>
+      <c r="O29" s="19"/>
+      <c r="P29" s="19"/>
+      <c r="Q29" s="19"/>
+      <c r="R29" s="16"/>
+      <c r="S29" s="19"/>
+      <c r="T29" s="19"/>
+      <c r="U29" s="19"/>
+      <c r="V29" s="19"/>
+      <c r="W29" s="19"/>
+      <c r="X29" s="19"/>
+      <c r="Y29" s="19"/>
+      <c r="Z29" s="16"/>
+      <c r="AA29" s="19"/>
+      <c r="AB29" s="19"/>
+      <c r="AC29" s="19"/>
+      <c r="AD29" s="16" t="s">
+        <v>395</v>
+      </c>
+      <c r="AE29" s="19"/>
+      <c r="AF29" s="19"/>
+      <c r="AG29" s="19"/>
+      <c r="AH29" s="19"/>
+      <c r="AI29" s="19"/>
+      <c r="AJ29" s="19"/>
+      <c r="AK29" s="19"/>
+      <c r="AL29" s="19"/>
+      <c r="AM29" s="19"/>
+      <c r="AN29" s="19"/>
+    </row>
+    <row r="30" spans="1:40">
       <c r="A30" t="s">
-        <v>69</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
+      <c r="G30" s="19"/>
+      <c r="H30" s="19"/>
+      <c r="I30" s="19"/>
+      <c r="J30" s="19"/>
+      <c r="K30" s="19"/>
       <c r="L30" s="16"/>
-      <c r="AV30" s="16"/>
-    </row>
-    <row r="31" spans="1:49">
-      <c r="A31" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="W31" s="16"/>
-      <c r="Z31" s="16"/>
-      <c r="AI31" s="16"/>
-      <c r="AJ31" s="16"/>
-      <c r="AM31" s="16"/>
-      <c r="AV31" s="16"/>
-    </row>
-    <row r="32" spans="1:49">
+      <c r="M30" s="19"/>
+      <c r="N30" s="19"/>
+      <c r="O30" s="19"/>
+      <c r="P30" s="19"/>
+      <c r="Q30" s="19"/>
+      <c r="R30" s="16"/>
+      <c r="S30" s="19"/>
+      <c r="T30" s="19"/>
+      <c r="U30" s="19"/>
+      <c r="V30" s="19"/>
+      <c r="W30" s="19"/>
+      <c r="X30" s="19"/>
+      <c r="Y30" s="19"/>
+      <c r="Z30" s="16"/>
+      <c r="AA30" s="19"/>
+      <c r="AB30" s="19"/>
+      <c r="AC30" s="19"/>
+      <c r="AD30" s="19"/>
+      <c r="AE30" s="19"/>
+      <c r="AF30" s="19"/>
+      <c r="AG30" s="19"/>
+      <c r="AH30" s="19"/>
+      <c r="AI30" s="19"/>
+      <c r="AJ30" s="19"/>
+      <c r="AK30" s="19"/>
+      <c r="AL30" s="19"/>
+      <c r="AM30" s="19"/>
+      <c r="AN30" s="19"/>
+    </row>
+    <row r="31" spans="1:40">
+      <c r="A31" t="s">
+        <v>85</v>
+      </c>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="19"/>
+      <c r="K31" s="19"/>
+      <c r="L31" s="19"/>
+      <c r="M31" s="19"/>
+      <c r="N31" s="19"/>
+      <c r="O31" s="19"/>
+      <c r="P31" s="19"/>
+      <c r="Q31" s="19"/>
+      <c r="R31" s="19"/>
+      <c r="S31" s="19"/>
+      <c r="T31" s="19"/>
+      <c r="U31" s="19"/>
+      <c r="V31" s="19"/>
+      <c r="W31" s="19"/>
+      <c r="X31" s="19"/>
+      <c r="Y31" s="19"/>
+      <c r="Z31" s="19"/>
+      <c r="AA31" s="19"/>
+      <c r="AB31" s="19"/>
+      <c r="AC31" s="19"/>
+      <c r="AD31" s="19"/>
+      <c r="AE31" s="19"/>
+      <c r="AF31" s="19"/>
+      <c r="AG31" s="19"/>
+      <c r="AH31" s="19"/>
+      <c r="AI31" s="19"/>
+      <c r="AJ31" s="19"/>
+      <c r="AK31" s="19"/>
+      <c r="AL31" s="19"/>
+      <c r="AM31" s="19"/>
+      <c r="AN31" s="19"/>
+    </row>
+    <row r="32" spans="1:40">
       <c r="A32" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="33" spans="1:49">
+        <v>86</v>
+      </c>
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
+      <c r="G32" s="19"/>
+      <c r="H32" s="19"/>
+      <c r="I32" s="19"/>
+      <c r="J32" s="19"/>
+      <c r="K32" s="19"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="19"/>
+      <c r="N32" s="19"/>
+      <c r="O32" s="19"/>
+      <c r="P32" s="19"/>
+      <c r="Q32" s="19"/>
+      <c r="R32" s="19"/>
+      <c r="S32" s="19"/>
+      <c r="T32" s="19"/>
+      <c r="U32" s="16"/>
+      <c r="V32" s="19"/>
+      <c r="W32" s="19"/>
+      <c r="X32" s="19"/>
+      <c r="Y32" s="19"/>
+      <c r="Z32" s="16"/>
+      <c r="AA32" s="19"/>
+      <c r="AB32" s="16"/>
+      <c r="AC32" s="19"/>
+      <c r="AD32" s="19"/>
+      <c r="AE32" s="19"/>
+      <c r="AF32" s="19"/>
+      <c r="AG32" s="19"/>
+      <c r="AH32" s="16"/>
+      <c r="AI32" s="19"/>
+      <c r="AJ32" s="19"/>
+      <c r="AK32" s="19"/>
+      <c r="AL32" s="19"/>
+      <c r="AM32" s="19"/>
+      <c r="AN32" s="16"/>
+    </row>
+    <row r="33" spans="1:40">
       <c r="A33" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="34" spans="1:49">
+        <v>87</v>
+      </c>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="19"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="19"/>
+      <c r="J33" s="19"/>
+      <c r="K33" s="19"/>
+      <c r="L33" s="19"/>
+      <c r="M33" s="19"/>
+      <c r="N33" s="19"/>
+      <c r="O33" s="19"/>
+      <c r="P33" s="19"/>
+      <c r="Q33" s="19"/>
+      <c r="R33" s="19"/>
+      <c r="S33" s="19"/>
+      <c r="T33" s="19"/>
+      <c r="U33" s="16"/>
+      <c r="V33" s="19"/>
+      <c r="W33" s="19"/>
+      <c r="X33" s="19"/>
+      <c r="Y33" s="19"/>
+      <c r="Z33" s="16"/>
+      <c r="AA33" s="19"/>
+      <c r="AB33" s="19"/>
+      <c r="AC33" s="16"/>
+      <c r="AD33" s="16"/>
+      <c r="AE33" s="19"/>
+      <c r="AF33" s="19"/>
+      <c r="AG33" s="19"/>
+      <c r="AH33" s="16"/>
+      <c r="AI33" s="19"/>
+      <c r="AJ33" s="19"/>
+      <c r="AK33" s="19"/>
+      <c r="AL33" s="19"/>
+      <c r="AM33" s="19"/>
+      <c r="AN33" s="16"/>
+    </row>
+    <row r="34" spans="1:40">
       <c r="A34" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="35" spans="1:49">
-      <c r="A35" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="AD35" s="16"/>
-      <c r="AV35" s="16"/>
-      <c r="AW35" s="16"/>
-    </row>
-    <row r="36" spans="1:49">
+        <v>89</v>
+      </c>
+      <c r="B34" s="19"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+      <c r="F34" s="19"/>
+      <c r="G34" s="19"/>
+      <c r="H34" s="19"/>
+      <c r="I34" s="19"/>
+      <c r="J34" s="19"/>
+      <c r="K34" s="19"/>
+      <c r="L34" s="19"/>
+      <c r="M34" s="19"/>
+      <c r="N34" s="19"/>
+      <c r="O34" s="19"/>
+      <c r="P34" s="19"/>
+      <c r="Q34" s="19"/>
+      <c r="R34" s="19"/>
+      <c r="S34" s="19"/>
+      <c r="T34" s="19"/>
+      <c r="U34" s="19"/>
+      <c r="V34" s="19"/>
+      <c r="W34" s="19"/>
+      <c r="X34" s="19"/>
+      <c r="Y34" s="19"/>
+      <c r="Z34" s="19"/>
+      <c r="AA34" s="19"/>
+      <c r="AB34" s="19"/>
+      <c r="AC34" s="19"/>
+      <c r="AD34" s="19"/>
+      <c r="AE34" s="19"/>
+      <c r="AF34" s="19"/>
+      <c r="AG34" s="19"/>
+      <c r="AH34" s="19"/>
+      <c r="AI34" s="19"/>
+      <c r="AJ34" s="19"/>
+      <c r="AK34" s="19"/>
+      <c r="AL34" s="19"/>
+      <c r="AM34" s="19"/>
+      <c r="AN34" s="19"/>
+    </row>
+    <row r="35" spans="1:40">
+      <c r="A35" t="s">
+        <v>90</v>
+      </c>
+      <c r="B35" s="19"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="19"/>
+      <c r="G35" s="19"/>
+      <c r="H35" s="19"/>
+      <c r="I35" s="19"/>
+      <c r="J35" s="19"/>
+      <c r="K35" s="19"/>
+      <c r="L35" s="19"/>
+      <c r="M35" s="19"/>
+      <c r="N35" s="19"/>
+      <c r="O35" s="19"/>
+      <c r="P35" s="19"/>
+      <c r="Q35" s="19"/>
+      <c r="R35" s="19"/>
+      <c r="S35" s="19"/>
+      <c r="T35" s="19"/>
+      <c r="U35" s="19"/>
+      <c r="V35" s="19"/>
+      <c r="W35" s="19"/>
+      <c r="X35" s="19"/>
+      <c r="Y35" s="19"/>
+      <c r="Z35" s="19"/>
+      <c r="AA35" s="19"/>
+      <c r="AB35" s="19"/>
+      <c r="AC35" s="19"/>
+      <c r="AD35" s="19"/>
+      <c r="AE35" s="19"/>
+      <c r="AF35" s="19"/>
+      <c r="AG35" s="19"/>
+      <c r="AH35" s="19"/>
+      <c r="AI35" s="19"/>
+      <c r="AJ35" s="19"/>
+      <c r="AK35" s="19"/>
+      <c r="AL35" s="19"/>
+      <c r="AM35" s="19"/>
+      <c r="AN35" s="16"/>
+    </row>
+    <row r="36" spans="1:40">
       <c r="A36" t="s">
-        <v>78</v>
-      </c>
-      <c r="AE36" s="16"/>
-      <c r="AW36" s="16"/>
-    </row>
-    <row r="37" spans="1:49">
+        <v>91</v>
+      </c>
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="19"/>
+      <c r="G36" s="19"/>
+      <c r="H36" s="19"/>
+      <c r="I36" s="19"/>
+      <c r="J36" s="19"/>
+      <c r="K36" s="19"/>
+      <c r="L36" s="19"/>
+      <c r="M36" s="19"/>
+      <c r="N36" s="19"/>
+      <c r="O36" s="19"/>
+      <c r="P36" s="19"/>
+      <c r="Q36" s="19"/>
+      <c r="R36" s="19"/>
+      <c r="S36" s="19"/>
+      <c r="T36" s="19"/>
+      <c r="U36" s="19"/>
+      <c r="V36" s="19"/>
+      <c r="W36" s="19"/>
+      <c r="X36" s="19"/>
+      <c r="Y36" s="19"/>
+      <c r="Z36" s="19"/>
+      <c r="AA36" s="19"/>
+      <c r="AB36" s="19"/>
+      <c r="AC36" s="19"/>
+      <c r="AD36" s="19"/>
+      <c r="AE36" s="19"/>
+      <c r="AF36" s="19"/>
+      <c r="AG36" s="19"/>
+      <c r="AH36" s="19"/>
+      <c r="AI36" s="19"/>
+      <c r="AJ36" s="19"/>
+      <c r="AK36" s="19"/>
+      <c r="AL36" s="19"/>
+      <c r="AM36" s="19"/>
+      <c r="AN36" s="16"/>
+    </row>
+    <row r="37" spans="1:40">
       <c r="A37" t="s">
-        <v>79</v>
-      </c>
-      <c r="AI37" s="16"/>
-    </row>
-    <row r="38" spans="1:49">
+        <v>92</v>
+      </c>
+      <c r="B37" s="19"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="19"/>
+      <c r="E37" s="19"/>
+      <c r="F37" s="19"/>
+      <c r="G37" s="19"/>
+      <c r="H37" s="19"/>
+      <c r="I37" s="19"/>
+      <c r="J37" s="19"/>
+      <c r="K37" s="19"/>
+      <c r="L37" s="19"/>
+      <c r="M37" s="19"/>
+      <c r="N37" s="19"/>
+      <c r="O37" s="19"/>
+      <c r="P37" s="19"/>
+      <c r="Q37" s="19"/>
+      <c r="R37" s="19"/>
+      <c r="S37" s="19"/>
+      <c r="T37" s="19"/>
+      <c r="U37" s="19"/>
+      <c r="V37" s="19"/>
+      <c r="W37" s="19"/>
+      <c r="X37" s="19"/>
+      <c r="Y37" s="19"/>
+      <c r="Z37" s="19"/>
+      <c r="AA37" s="19"/>
+      <c r="AB37" s="19"/>
+      <c r="AC37" s="19"/>
+      <c r="AD37" s="19"/>
+      <c r="AE37" s="19"/>
+      <c r="AF37" s="19"/>
+      <c r="AG37" s="19"/>
+      <c r="AH37" s="19"/>
+      <c r="AI37" s="19"/>
+      <c r="AJ37" s="19"/>
+      <c r="AK37" s="19"/>
+      <c r="AL37" s="19"/>
+      <c r="AM37" s="19"/>
+      <c r="AN37" s="16"/>
+    </row>
+    <row r="38" spans="1:40">
       <c r="A38" t="s">
-        <v>80</v>
-      </c>
-      <c r="AI38" s="16"/>
-      <c r="AM38" s="16" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="39" spans="1:49">
+        <v>93</v>
+      </c>
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="19"/>
+      <c r="H38" s="19"/>
+      <c r="I38" s="19"/>
+      <c r="J38" s="19"/>
+      <c r="K38" s="19"/>
+      <c r="L38" s="19"/>
+      <c r="M38" s="19"/>
+      <c r="N38" s="19"/>
+      <c r="O38" s="19"/>
+      <c r="P38" s="19"/>
+      <c r="Q38" s="19"/>
+      <c r="R38" s="19"/>
+      <c r="S38" s="19"/>
+      <c r="T38" s="19"/>
+      <c r="U38" s="19"/>
+      <c r="V38" s="19"/>
+      <c r="W38" s="19"/>
+      <c r="X38" s="19"/>
+      <c r="Y38" s="19"/>
+      <c r="Z38" s="19"/>
+      <c r="AA38" s="19"/>
+      <c r="AB38" s="19"/>
+      <c r="AC38" s="19"/>
+      <c r="AD38" s="19"/>
+      <c r="AE38" s="19"/>
+      <c r="AF38" s="19"/>
+      <c r="AG38" s="19"/>
+      <c r="AH38" s="19"/>
+      <c r="AI38" s="19"/>
+      <c r="AJ38" s="19"/>
+      <c r="AK38" s="19"/>
+      <c r="AL38" s="19"/>
+      <c r="AM38" s="19"/>
+      <c r="AN38" s="16"/>
+    </row>
+    <row r="39" spans="1:40">
       <c r="A39" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="40" spans="1:49">
+        <v>389</v>
+      </c>
+      <c r="B39" s="19"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="19"/>
+      <c r="F39" s="19"/>
+      <c r="G39" s="19"/>
+      <c r="H39" s="19"/>
+      <c r="I39" s="19"/>
+      <c r="J39" s="19"/>
+      <c r="K39" s="19"/>
+      <c r="L39" s="19"/>
+      <c r="M39" s="19"/>
+      <c r="N39" s="19"/>
+      <c r="O39" s="19"/>
+      <c r="P39" s="19"/>
+      <c r="Q39" s="19"/>
+      <c r="R39" s="19"/>
+      <c r="S39" s="19"/>
+      <c r="T39" s="19"/>
+      <c r="U39" s="19"/>
+      <c r="V39" s="19"/>
+      <c r="W39" s="19"/>
+      <c r="X39" s="19"/>
+      <c r="Y39" s="19"/>
+      <c r="Z39" s="19"/>
+      <c r="AA39" s="19"/>
+      <c r="AB39" s="19"/>
+      <c r="AC39" s="19"/>
+      <c r="AD39" s="19"/>
+      <c r="AE39" s="19"/>
+      <c r="AF39" s="19"/>
+      <c r="AG39" s="19"/>
+      <c r="AH39" s="19"/>
+      <c r="AI39" s="19"/>
+      <c r="AJ39" s="19"/>
+      <c r="AK39" s="19"/>
+      <c r="AL39" s="19"/>
+      <c r="AM39" s="19"/>
+      <c r="AN39" s="19"/>
+    </row>
+    <row r="40" spans="1:40">
       <c r="A40" t="s">
-        <v>85</v>
-      </c>
-      <c r="AR40" s="16"/>
-      <c r="AS40" s="16"/>
-      <c r="AT40" s="16"/>
-      <c r="AU40" s="16"/>
-      <c r="AW40" s="16"/>
-    </row>
-    <row r="41" spans="1:49">
-      <c r="A41" t="s">
-        <v>86</v>
-      </c>
-      <c r="AD41" s="16"/>
-      <c r="AK41" s="16"/>
-      <c r="AQ41" s="16"/>
-      <c r="AW41" s="16"/>
-    </row>
-    <row r="42" spans="1:49">
-      <c r="A42" t="s">
-        <v>87</v>
-      </c>
-      <c r="L42" s="16"/>
-      <c r="M42" s="16"/>
-      <c r="AD42" s="16"/>
-      <c r="AI42" s="16"/>
-      <c r="AL42" s="16"/>
-      <c r="AM42" s="16"/>
-      <c r="AQ42" s="16"/>
-      <c r="AW42" s="16"/>
-    </row>
-    <row r="43" spans="1:49">
-      <c r="A43" t="s">
-        <v>89</v>
-      </c>
-      <c r="Z43" s="16"/>
-      <c r="AD43" s="16"/>
-      <c r="AI43" s="16"/>
-      <c r="AM43" s="16"/>
-    </row>
-    <row r="44" spans="1:49">
-      <c r="A44" t="s">
-        <v>90</v>
-      </c>
-      <c r="AW44" s="16"/>
-    </row>
-    <row r="45" spans="1:49">
-      <c r="A45" t="s">
-        <v>91</v>
-      </c>
-      <c r="AW45" s="16"/>
-    </row>
-    <row r="46" spans="1:49">
-      <c r="A46" t="s">
-        <v>92</v>
-      </c>
-      <c r="AW46" s="16"/>
-    </row>
-    <row r="47" spans="1:49">
-      <c r="A47" t="s">
-        <v>93</v>
-      </c>
-      <c r="AS47" s="16"/>
-      <c r="AW47" s="16"/>
-    </row>
-    <row r="48" spans="1:49">
-      <c r="A48" t="s">
+        <v>388</v>
+      </c>
+      <c r="B40" s="19"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="19"/>
+      <c r="H40" s="19"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="19"/>
+      <c r="K40" s="19"/>
+      <c r="L40" s="19"/>
+      <c r="M40" s="19"/>
+      <c r="N40" s="19"/>
+      <c r="O40" s="19"/>
+      <c r="P40" s="19"/>
+      <c r="Q40" s="19"/>
+      <c r="R40" s="19"/>
+      <c r="S40" s="19"/>
+      <c r="T40" s="19"/>
+      <c r="U40" s="19"/>
+      <c r="V40" s="19"/>
+      <c r="W40" s="19"/>
+      <c r="X40" s="19"/>
+      <c r="Y40" s="19"/>
+      <c r="Z40" s="19"/>
+      <c r="AA40" s="19"/>
+      <c r="AB40" s="19"/>
+      <c r="AC40" s="19"/>
+      <c r="AD40" s="19"/>
+      <c r="AE40" s="19"/>
+      <c r="AF40" s="19"/>
+      <c r="AG40" s="19"/>
+      <c r="AH40" s="19"/>
+      <c r="AI40" s="19"/>
+      <c r="AJ40" s="19"/>
+      <c r="AK40" s="19"/>
+      <c r="AL40" s="19"/>
+      <c r="AM40" s="19"/>
+      <c r="AN40" s="19"/>
+    </row>
+    <row r="43" spans="1:40">
+      <c r="B43" s="12" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="44" spans="1:40">
+      <c r="A44" s="12"/>
+      <c r="B44" s="13"/>
+      <c r="C44" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="45" spans="1:40">
+      <c r="B45" s="14"/>
+      <c r="C45" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="46" spans="1:40">
+      <c r="B46" s="15"/>
+      <c r="C46" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="47" spans="1:40">
+      <c r="B47" s="16"/>
+      <c r="C47" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="48" spans="1:40">
+      <c r="B48" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="AW48" s="16"/>
-    </row>
-    <row r="49" spans="1:3">
-      <c r="A49" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="B52" s="12" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53" s="12"/>
-      <c r="B53" s="13"/>
-      <c r="C53" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3">
-      <c r="B54" s="14"/>
-      <c r="C54" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="B55" s="15"/>
-      <c r="C55" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3">
-      <c r="B56" s="16"/>
-      <c r="C56" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3">
-      <c r="B57" s="1" t="s">
+      <c r="C48" t="s">
         <v>391</v>
       </c>
-      <c r="C57" t="s">
-        <v>392</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B31:V31 X31:Y31 AD36 B35:AC36 B23:AH23 AA31:AH31 B37:AH38 B42:AH43 B2:AW22 AJ23:AW23 B24:AW30 AK31:AL31 AN31:AU31 AW31 B32:AW34 AE35:AU35 AF36:AW36 AJ37:AW38 B39:AW41 B44:AW49 AJ42:AW43">
-    <cfRule type="expression" dxfId="6" priority="2">
-      <formula>$A2=B$1</formula>
+  <conditionalFormatting sqref="N22 Q22 AA22 AD22 AM22 AM26:AN26">
+    <cfRule type="expression" dxfId="5" priority="6">
+      <formula>#REF!=N$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AE36">
-    <cfRule type="expression" dxfId="5" priority="4">
-      <formula>$A36=#REF!</formula>
+  <conditionalFormatting sqref="U26">
+    <cfRule type="expression" dxfId="4" priority="29">
+      <formula>#REF!=U$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W31 Z31 AJ31 AM31 AV31">
-    <cfRule type="expression" dxfId="4" priority="6">
-      <formula>#REF!=W$1</formula>
+  <conditionalFormatting sqref="V27">
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula>$A27=#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI31">
-    <cfRule type="expression" dxfId="3" priority="15">
+  <conditionalFormatting sqref="Z14 Z29 Z33:Z34">
+    <cfRule type="expression" dxfId="2" priority="50">
+      <formula>$A14=#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z22">
+    <cfRule type="expression" dxfId="1" priority="15">
       <formula>#REF!=#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AV35:AW35 AD35">
-    <cfRule type="expression" dxfId="2" priority="29">
-      <formula>#REF!=AD$1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI38 AI42:AI43 AI23">
-    <cfRule type="expression" dxfId="1" priority="50">
-      <formula>$A23=#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B56">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>$A56=B$1</formula>
+  <conditionalFormatting sqref="B47 N2:AN13 N14:Y14 AA14:AN14 N15:AN21 B2:M22 O22:P22 R22:Y22 AB22:AC22 AE22:AL22 AN22 B23:AN25 V26:AL26 B26:T27 U27 B28:Y29 AA28:AN29 B30:AN32 B33:Y34 AA33:AN34 W27:AN27 B35:AN40">
+    <cfRule type="expression" dxfId="0" priority="57">
+      <formula>$A2=B$1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix (03_transform_data) (codeboook) updated test_household_income to be a numerical value of their yearly earnings, that corresponds to the middle value of the income bin they fall into
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Vaccine Uptake - R\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B878E925-4527-48F2-B61E-018908ACAF97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D979DE-9EF0-4082-B8A6-7A689E30934C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10890" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
     <sheet name="Values&amp;Labels" sheetId="2" r:id="rId2"/>
     <sheet name="causal relationships" sheetId="3" r:id="rId3"/>
+    <sheet name="relationships" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -87,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1294" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1307" uniqueCount="425">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -688,21 +689,6 @@
     <t>No household income data was provided</t>
   </si>
   <si>
-    <t>10,000,000 yen or more and less than 12,000,000 yen</t>
-  </si>
-  <si>
-    <t>12,000,000 yen or more and less than 14,000,000 yen</t>
-  </si>
-  <si>
-    <t>14,000,000 yen or more and less than 16,000,000 yen</t>
-  </si>
-  <si>
-    <t>16,000,000 yen or more and less than 18,000,000 yen</t>
-  </si>
-  <si>
-    <t>18,000,000 yen or more and less than 20,000,000 yen</t>
-  </si>
-  <si>
     <t>20,000,000 yen and above</t>
   </si>
   <si>
@@ -1195,9 +1181,6 @@
     <t>take the annual hosuehold income categories as responded up till 10,000,000 yen a year which corresponds with the top 10% percentile of earners</t>
   </si>
   <si>
-    <t>take the annual hosuehold income categories as responded</t>
-  </si>
-  <si>
     <t>where "chronic_illness" represents the 20 chronic illnesses asked about in the survey, we derive the responding parent's experience with chronic illnesses as: never (for never had for all 20 illnesses), previously had (if not currently having a chronic illness and previously had at least one chronic illness), currently having (when at least 1 chronic illness corresponds to currently have)</t>
   </si>
   <si>
@@ -1313,6 +1296,78 @@
   </si>
   <si>
     <t>Vaccine uptake varies based on 3 different categories, can we leave it as a standalone variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unmarried have a lower mean income </t>
+  </si>
+  <si>
+    <t>single parent households have a lower income (mean category 6.9 vs 9.8)</t>
+  </si>
+  <si>
+    <t>interaction variables</t>
+  </si>
+  <si>
+    <t>variable</t>
+  </si>
+  <si>
+    <t>Relationship</t>
+  </si>
+  <si>
+    <t>Single fathers have about the same mean income as dual parent families whilst, single mothers experience a much lower mean income</t>
+  </si>
+  <si>
+    <t>&lt; 250,000 JPY</t>
+  </si>
+  <si>
+    <t>1,500,000 JPY</t>
+  </si>
+  <si>
+    <t>750,000 JPY</t>
+  </si>
+  <si>
+    <t>2,500,000 JPY</t>
+  </si>
+  <si>
+    <t>3,500,000 JPY</t>
+  </si>
+  <si>
+    <t>4,500,000 JPY</t>
+  </si>
+  <si>
+    <t>5,500,000 JPY</t>
+  </si>
+  <si>
+    <t>6,500,000 JPY</t>
+  </si>
+  <si>
+    <t>7,500,000 JPY</t>
+  </si>
+  <si>
+    <t>8,500,000 JPY</t>
+  </si>
+  <si>
+    <t>9,500,000 JPY</t>
+  </si>
+  <si>
+    <t>11,000,000 JPY</t>
+  </si>
+  <si>
+    <t>13,000,000 JPY</t>
+  </si>
+  <si>
+    <t>17,000,000 JPY</t>
+  </si>
+  <si>
+    <t>15,000,000 JPY</t>
+  </si>
+  <si>
+    <t>19,000,000 JPY</t>
+  </si>
+  <si>
+    <t>assign them the middle value of the income category that they fall into</t>
+  </si>
+  <si>
+    <t>JPY</t>
   </si>
 </sst>
 </file>
@@ -1366,7 +1421,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1421,6 +1476,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1434,7 +1495,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1468,10 +1529,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1910,7 +1972,7 @@
         <v>15</v>
       </c>
       <c r="M1" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="N1" t="s">
         <v>17</v>
@@ -2126,10 +2188,10 @@
         <v>87</v>
       </c>
       <c r="CG1" s="6" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="CH1" s="6" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="CI1" s="8" t="s">
         <v>88</v>
@@ -2480,7 +2542,7 @@
         <v>117</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="N3" s="2" t="s">
         <v>118</v>
@@ -2629,10 +2691,10 @@
         <v>153</v>
       </c>
       <c r="CG3" s="5" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="CH3" s="5" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="CI3" s="7"/>
       <c r="CJ3" s="2" t="s">
@@ -2871,10 +2933,10 @@
         <v>100</v>
       </c>
       <c r="BU4" s="4" t="s">
-        <v>99</v>
+        <v>263</v>
       </c>
       <c r="BV4" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="BW4" t="s">
         <v>99</v>
@@ -3048,6 +3110,9 @@
       </c>
       <c r="BT7" t="s">
         <v>108</v>
+      </c>
+      <c r="BU7" s="4" t="s">
+        <v>424</v>
       </c>
       <c r="CO7" s="8"/>
       <c r="CP7" s="8"/>
@@ -3094,37 +3159,37 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>159</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>160</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" spans="1:16">
@@ -3135,34 +3200,34 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -3182,19 +3247,19 @@
         <v>102</v>
       </c>
       <c r="F3" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="G3" t="s">
+        <v>273</v>
+      </c>
+      <c r="H3" t="s">
         <v>278</v>
       </c>
-      <c r="H3" t="s">
-        <v>283</v>
-      </c>
       <c r="I3" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="J3" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -3214,19 +3279,19 @@
         <v>104</v>
       </c>
       <c r="F4" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="G4" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="H4" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="I4" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="J4" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -3246,19 +3311,19 @@
         <v>105</v>
       </c>
       <c r="F5" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="G5" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="H5" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="I5" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="J5" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -3278,19 +3343,19 @@
         <v>110</v>
       </c>
       <c r="F6" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="G6" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="H6" t="s">
+        <v>278</v>
+      </c>
+      <c r="I6" t="s">
         <v>283</v>
       </c>
-      <c r="I6" t="s">
-        <v>288</v>
-      </c>
       <c r="J6" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -3310,19 +3375,19 @@
         <v>111</v>
       </c>
       <c r="F7" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="G7" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="H7" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="I7" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="J7" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:16">
@@ -3333,7 +3398,7 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D8" t="s">
         <v>108</v>
@@ -3342,19 +3407,19 @@
         <v>112</v>
       </c>
       <c r="F8" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="G8" t="s">
         <v>5</v>
       </c>
       <c r="H8" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="I8" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="J8" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -3365,7 +3430,7 @@
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D9" t="s">
         <v>108</v>
@@ -3374,19 +3439,19 @@
         <v>113</v>
       </c>
       <c r="F9" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="G9" t="s">
         <v>6</v>
       </c>
       <c r="H9" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="I9" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="J9" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -3397,7 +3462,7 @@
         <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D10" t="s">
         <v>108</v>
@@ -3406,19 +3471,19 @@
         <v>114</v>
       </c>
       <c r="F10" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="G10" t="s">
         <v>7</v>
       </c>
       <c r="H10" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="I10" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="J10" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -3429,7 +3494,7 @@
         <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D11" t="s">
         <v>108</v>
@@ -3438,19 +3503,19 @@
         <v>115</v>
       </c>
       <c r="F11" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="G11" t="s">
         <v>8</v>
       </c>
       <c r="H11" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="I11" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="J11" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -3461,7 +3526,7 @@
         <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D12" t="s">
         <v>108</v>
@@ -3470,19 +3535,19 @@
         <v>116</v>
       </c>
       <c r="F12" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="G12" t="s">
         <v>9</v>
       </c>
       <c r="H12" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="I12" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="J12" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" spans="1:16">
@@ -3493,22 +3558,22 @@
         <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D13" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E13" t="s">
         <v>117</v>
       </c>
       <c r="F13" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="G13" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="H13" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="14" spans="1:16">
@@ -3516,25 +3581,25 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="C14" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D14" t="s">
         <v>109</v>
       </c>
       <c r="E14" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="F14" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="G14" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="H14" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="15" spans="1:16">
@@ -3554,19 +3619,19 @@
         <v>118</v>
       </c>
       <c r="F15" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="G15" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="H15" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="I15" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="J15" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="16" spans="1:16">
@@ -3586,19 +3651,19 @@
         <v>119</v>
       </c>
       <c r="F16" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="G16" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="H16" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="I16" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="J16" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -3618,19 +3683,19 @@
         <v>120</v>
       </c>
       <c r="F17" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="G17" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="H17" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="I17" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="J17" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -3641,7 +3706,7 @@
         <v>20</v>
       </c>
       <c r="C18" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -3650,25 +3715,25 @@
         <v>162</v>
       </c>
       <c r="F18" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="G18" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="H18" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="I18" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="J18" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="K18" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="L18" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -3723,16 +3788,16 @@
         <v>21</v>
       </c>
       <c r="C23" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D23">
         <v>0</v>
       </c>
       <c r="E23" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="F23" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="G23" t="s">
         <v>15</v>
@@ -3741,22 +3806,22 @@
         <v>16</v>
       </c>
       <c r="I23" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="J23" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="K23" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="L23" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="M23" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="N23" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="24" spans="1:14">
@@ -3809,19 +3874,19 @@
         <v>122</v>
       </c>
       <c r="F27" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="G27" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="H27" t="s">
+        <v>298</v>
+      </c>
+      <c r="I27" t="s">
         <v>303</v>
       </c>
-      <c r="I27" t="s">
-        <v>308</v>
-      </c>
       <c r="J27" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -3841,19 +3906,19 @@
         <v>123</v>
       </c>
       <c r="F28" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="G28" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="H28" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="I28" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="J28" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -3864,7 +3929,7 @@
         <v>25</v>
       </c>
       <c r="C29" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D29">
         <v>0</v>
@@ -3873,25 +3938,25 @@
         <v>162</v>
       </c>
       <c r="F29" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="G29" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="H29" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="I29" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="J29" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="K29" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="L29" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -3935,7 +4000,7 @@
         <v>26</v>
       </c>
       <c r="C33" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D33">
         <v>0</v>
@@ -3944,7 +4009,7 @@
         <v>169</v>
       </c>
       <c r="F33" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="G33" t="s">
         <v>15</v>
@@ -3953,22 +4018,22 @@
         <v>16</v>
       </c>
       <c r="I33" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J33" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="K33" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="L33" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="M33" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="N33" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -4012,7 +4077,7 @@
         <v>60</v>
       </c>
       <c r="C37" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D37" t="s">
         <v>109</v>
@@ -4021,13 +4086,13 @@
         <v>127</v>
       </c>
       <c r="F37" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="G37" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="H37" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -4038,7 +4103,7 @@
         <v>61</v>
       </c>
       <c r="C38" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D38" t="s">
         <v>109</v>
@@ -4047,13 +4112,13 @@
         <v>128</v>
       </c>
       <c r="F38" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="G38" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="H38" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -4064,7 +4129,7 @@
         <v>62</v>
       </c>
       <c r="C39" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D39" t="s">
         <v>109</v>
@@ -4073,25 +4138,25 @@
         <v>129</v>
       </c>
       <c r="F39" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="G39" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="H39" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I39" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="J39" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K39" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="L39" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -4102,7 +4167,7 @@
         <v>63</v>
       </c>
       <c r="C40" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D40" t="s">
         <v>109</v>
@@ -4111,13 +4176,13 @@
         <v>130</v>
       </c>
       <c r="F40" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="G40" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="H40" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -4128,7 +4193,7 @@
         <v>64</v>
       </c>
       <c r="C41" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D41" t="s">
         <v>109</v>
@@ -4137,19 +4202,19 @@
         <v>131</v>
       </c>
       <c r="F41" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="G41" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="H41" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I41" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="J41" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -4160,7 +4225,7 @@
         <v>65</v>
       </c>
       <c r="C42" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D42">
         <v>0</v>
@@ -4169,16 +4234,16 @@
         <v>170</v>
       </c>
       <c r="F42" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="G42" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="H42" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I42" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="J42" t="s">
         <v>16</v>
@@ -4220,7 +4285,7 @@
         <v>66</v>
       </c>
       <c r="C45" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D45">
         <v>0</v>
@@ -4229,13 +4294,13 @@
         <v>173</v>
       </c>
       <c r="F45" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="G45" t="s">
         <v>65</v>
       </c>
       <c r="H45" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -4257,25 +4322,25 @@
         <v>67</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D47" s="4" t="s">
         <v>109</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I47" s="4" t="s">
         <v>65</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="48" spans="1:14" s="4" customFormat="1">
@@ -4286,25 +4351,25 @@
         <v>68</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>109</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I48" s="4" t="s">
         <v>65</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -4315,25 +4380,25 @@
         <v>69</v>
       </c>
       <c r="C49" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D49" t="s">
         <v>109</v>
       </c>
       <c r="F49" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="G49" t="s">
         <v>68</v>
       </c>
       <c r="H49" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I49" t="s">
         <v>67</v>
       </c>
       <c r="J49" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="50" spans="1:13" s="4" customFormat="1">
@@ -4344,7 +4409,7 @@
         <v>70</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D50" s="4">
         <v>0</v>
@@ -4353,16 +4418,16 @@
         <v>175</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="G50" s="4" t="s">
         <v>66</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
     </row>
     <row r="51" spans="1:13" s="4" customFormat="1">
@@ -4417,7 +4482,7 @@
         <v>71</v>
       </c>
       <c r="C55" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D55">
         <v>0</v>
@@ -4426,16 +4491,16 @@
         <v>175</v>
       </c>
       <c r="F55" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="G55" t="s">
         <v>66</v>
       </c>
       <c r="H55" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I55" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -4468,7 +4533,7 @@
         <v>73</v>
       </c>
       <c r="C58" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D58">
         <v>0</v>
@@ -4477,13 +4542,13 @@
         <v>170</v>
       </c>
       <c r="F58" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="G58" t="s">
         <v>58</v>
       </c>
       <c r="H58" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="59" spans="1:13">
@@ -4505,7 +4570,7 @@
         <v>172</v>
       </c>
       <c r="E60" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
     </row>
     <row r="61" spans="1:13">
@@ -4516,7 +4581,7 @@
         <v>74</v>
       </c>
       <c r="C61" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D61">
         <v>0</v>
@@ -4525,25 +4590,25 @@
         <v>170</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="G61" s="11" t="s">
         <v>73</v>
       </c>
       <c r="H61" s="11" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I61" s="11" t="s">
         <v>70</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>60</v>
       </c>
       <c r="L61" s="11" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="M61" s="11"/>
     </row>
@@ -4566,7 +4631,7 @@
         <v>172</v>
       </c>
       <c r="E63" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -4577,19 +4642,19 @@
         <v>75</v>
       </c>
       <c r="C64" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D64" t="s">
         <v>108</v>
       </c>
       <c r="F64" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="G64" t="s">
         <v>59</v>
       </c>
       <c r="H64" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="65" spans="1:8" s="4" customFormat="1">
@@ -4600,22 +4665,22 @@
         <v>76</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D65" s="4">
         <v>1</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="66" spans="1:8" s="4" customFormat="1">
@@ -4769,7 +4834,7 @@
         <v>77</v>
       </c>
       <c r="C79" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="D79">
         <v>1</v>
@@ -4778,13 +4843,13 @@
         <v>184</v>
       </c>
       <c r="F79" t="s">
-        <v>367</v>
+        <v>423</v>
       </c>
       <c r="G79" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="H79" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="80" spans="1:8">
@@ -4796,7 +4861,7 @@
         <v>2</v>
       </c>
       <c r="E80" t="s">
-        <v>185</v>
+        <v>407</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -4808,7 +4873,7 @@
         <v>3</v>
       </c>
       <c r="E81" t="s">
-        <v>186</v>
+        <v>409</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -4820,7 +4885,7 @@
         <v>4</v>
       </c>
       <c r="E82" t="s">
-        <v>187</v>
+        <v>408</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -4832,7 +4897,7 @@
         <v>5</v>
       </c>
       <c r="E83" t="s">
-        <v>188</v>
+        <v>410</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -4844,7 +4909,7 @@
         <v>6</v>
       </c>
       <c r="E84" t="s">
-        <v>189</v>
+        <v>411</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -4856,7 +4921,7 @@
         <v>7</v>
       </c>
       <c r="E85" t="s">
-        <v>190</v>
+        <v>412</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -4868,7 +4933,7 @@
         <v>8</v>
       </c>
       <c r="E86" t="s">
-        <v>191</v>
+        <v>413</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -4880,7 +4945,7 @@
         <v>9</v>
       </c>
       <c r="E87" t="s">
-        <v>192</v>
+        <v>414</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -4892,7 +4957,7 @@
         <v>10</v>
       </c>
       <c r="E88" t="s">
-        <v>193</v>
+        <v>415</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -4904,7 +4969,7 @@
         <v>11</v>
       </c>
       <c r="E89" t="s">
-        <v>194</v>
+        <v>416</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -4916,7 +4981,7 @@
         <v>12</v>
       </c>
       <c r="E90" t="s">
-        <v>195</v>
+        <v>417</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -4928,7 +4993,7 @@
         <v>13</v>
       </c>
       <c r="E91" t="s">
-        <v>198</v>
+        <v>418</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -4940,7 +5005,7 @@
         <v>14</v>
       </c>
       <c r="E92" t="s">
-        <v>199</v>
+        <v>419</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -4951,8 +5016,8 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="E93" t="s">
-        <v>200</v>
+      <c r="E93" s="21" t="s">
+        <v>421</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -4964,7 +5029,7 @@
         <v>16</v>
       </c>
       <c r="E94" t="s">
-        <v>201</v>
+        <v>420</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -4976,7 +5041,7 @@
         <v>17</v>
       </c>
       <c r="E95" t="s">
-        <v>202</v>
+        <v>422</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -4988,7 +5053,7 @@
         <v>18</v>
       </c>
       <c r="E96" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="97" spans="1:17">
@@ -5010,25 +5075,25 @@
         <v>78</v>
       </c>
       <c r="C98" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D98">
         <v>0</v>
       </c>
       <c r="E98" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="F98" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
       <c r="G98" t="s">
         <v>66</v>
       </c>
       <c r="H98" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I98" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
     </row>
     <row r="99" spans="1:17">
@@ -5039,7 +5104,7 @@
         <v>1</v>
       </c>
       <c r="E99" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="100" spans="1:17">
@@ -5050,7 +5115,7 @@
         <v>2</v>
       </c>
       <c r="E100" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="101" spans="1:17">
@@ -5061,7 +5126,7 @@
         <v>172</v>
       </c>
       <c r="E101" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="102" spans="1:17">
@@ -5072,46 +5137,46 @@
         <v>79</v>
       </c>
       <c r="C102" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D102">
         <v>0</v>
       </c>
       <c r="E102" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="F102" t="s">
-        <v>369</v>
+        <v>363</v>
       </c>
       <c r="G102" t="s">
         <v>66</v>
       </c>
       <c r="H102" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I102" t="s">
         <v>73</v>
       </c>
       <c r="J102" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K102" t="s">
         <v>74</v>
       </c>
       <c r="L102" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="M102" t="s">
         <v>48</v>
       </c>
       <c r="N102" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="O102" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="P102" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="103" spans="1:17">
@@ -5122,7 +5187,7 @@
         <v>1</v>
       </c>
       <c r="E103" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="104" spans="1:17">
@@ -5133,7 +5198,7 @@
         <v>2</v>
       </c>
       <c r="E104" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="105" spans="1:17">
@@ -5144,7 +5209,7 @@
         <v>3</v>
       </c>
       <c r="E105" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="106" spans="1:17">
@@ -5155,7 +5220,7 @@
         <v>172</v>
       </c>
       <c r="E106" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="107" spans="1:17">
@@ -5166,46 +5231,46 @@
         <v>80</v>
       </c>
       <c r="C107" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D107">
         <v>0</v>
       </c>
       <c r="E107" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="F107" t="s">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="G107" t="s">
         <v>66</v>
       </c>
       <c r="H107" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I107" t="s">
         <v>73</v>
       </c>
       <c r="J107" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K107" t="s">
         <v>74</v>
       </c>
       <c r="L107" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="M107" t="s">
         <v>48</v>
       </c>
       <c r="N107" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="O107" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="P107" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="108" spans="1:17">
@@ -5216,7 +5281,7 @@
         <v>1</v>
       </c>
       <c r="E108" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="109" spans="1:17">
@@ -5227,7 +5292,7 @@
         <v>2</v>
       </c>
       <c r="E109" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="110" spans="1:17">
@@ -5238,7 +5303,7 @@
         <v>3</v>
       </c>
       <c r="E110" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="111" spans="1:17" s="6" customFormat="1">
@@ -5251,7 +5316,7 @@
         <v>172</v>
       </c>
       <c r="E111" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="F111"/>
       <c r="G111"/>
@@ -5274,46 +5339,46 @@
         <v>81</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D112" s="4">
         <v>0</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>371</v>
+        <v>365</v>
       </c>
       <c r="G112" s="4" t="s">
         <v>66</v>
       </c>
       <c r="H112" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I112" s="4" t="s">
         <v>73</v>
       </c>
       <c r="J112" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K112" s="4" t="s">
         <v>74</v>
       </c>
       <c r="L112" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="M112" s="4" t="s">
         <v>48</v>
       </c>
       <c r="N112" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="O112" s="4" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="P112" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="113" spans="1:16" s="4" customFormat="1">
@@ -5324,7 +5389,7 @@
         <v>1</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="114" spans="1:16" s="4" customFormat="1">
@@ -5335,7 +5400,7 @@
         <v>2</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="115" spans="1:16" s="4" customFormat="1">
@@ -5346,7 +5411,7 @@
         <v>3</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="116" spans="1:16" s="4" customFormat="1">
@@ -5357,7 +5422,7 @@
         <v>172</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
     </row>
     <row r="117" spans="1:16" s="4" customFormat="1">
@@ -5368,46 +5433,46 @@
         <v>82</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D117" s="4">
         <v>0</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>372</v>
+        <v>366</v>
       </c>
       <c r="G117" s="4" t="s">
         <v>66</v>
       </c>
       <c r="H117" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I117" s="4" t="s">
         <v>73</v>
       </c>
       <c r="J117" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K117" s="4" t="s">
         <v>74</v>
       </c>
       <c r="L117" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="M117" s="4" t="s">
         <v>48</v>
       </c>
       <c r="N117" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="O117" s="4" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="P117" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="118" spans="1:16" s="4" customFormat="1">
@@ -5418,7 +5483,7 @@
         <v>1</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
     </row>
     <row r="119" spans="1:16" s="4" customFormat="1">
@@ -5429,7 +5494,7 @@
         <v>2</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
     </row>
     <row r="120" spans="1:16" s="4" customFormat="1">
@@ -5440,7 +5505,7 @@
         <v>3</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="121" spans="1:16" s="4" customFormat="1">
@@ -5451,7 +5516,7 @@
         <v>172</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="122" spans="1:16" s="4" customFormat="1">
@@ -5462,46 +5527,46 @@
         <v>83</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D122" s="4">
         <v>0</v>
       </c>
       <c r="E122" s="4" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>373</v>
+        <v>367</v>
       </c>
       <c r="G122" s="4" t="s">
         <v>66</v>
       </c>
       <c r="H122" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I122" s="4" t="s">
         <v>73</v>
       </c>
       <c r="J122" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K122" s="4" t="s">
         <v>74</v>
       </c>
       <c r="L122" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="M122" s="4" t="s">
         <v>48</v>
       </c>
       <c r="N122" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="O122" s="4" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="P122" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="123" spans="1:16" s="4" customFormat="1">
@@ -5512,7 +5577,7 @@
         <v>1</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
     </row>
     <row r="124" spans="1:16" s="4" customFormat="1">
@@ -5523,7 +5588,7 @@
         <v>2</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="125" spans="1:16" s="4" customFormat="1">
@@ -5534,7 +5599,7 @@
         <v>3</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
     </row>
     <row r="126" spans="1:16" s="4" customFormat="1">
@@ -5545,7 +5610,7 @@
         <v>172</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
     </row>
     <row r="127" spans="1:16">
@@ -5556,46 +5621,46 @@
         <v>84</v>
       </c>
       <c r="C127" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D127">
         <v>0</v>
       </c>
       <c r="E127" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="F127" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
       <c r="G127" t="s">
         <v>66</v>
       </c>
       <c r="H127" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I127" t="s">
         <v>73</v>
       </c>
       <c r="J127" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K127" t="s">
         <v>74</v>
       </c>
       <c r="L127" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="M127" t="s">
         <v>48</v>
       </c>
       <c r="N127" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="O127" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="P127" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="128" spans="1:16">
@@ -5606,7 +5671,7 @@
         <v>1</v>
       </c>
       <c r="E128" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
     </row>
     <row r="129" spans="1:16">
@@ -5617,7 +5682,7 @@
         <v>172</v>
       </c>
       <c r="E129" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
     </row>
     <row r="130" spans="1:16">
@@ -5628,46 +5693,46 @@
         <v>85</v>
       </c>
       <c r="C130" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D130">
         <v>0</v>
       </c>
       <c r="E130" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="F130" t="s">
-        <v>375</v>
+        <v>369</v>
       </c>
       <c r="G130" t="s">
         <v>66</v>
       </c>
       <c r="H130" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I130" t="s">
         <v>73</v>
       </c>
       <c r="J130" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K130" t="s">
         <v>74</v>
       </c>
       <c r="L130" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="M130" t="s">
         <v>48</v>
       </c>
       <c r="N130" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="O130" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="P130" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="131" spans="1:16">
@@ -5678,7 +5743,7 @@
         <v>1</v>
       </c>
       <c r="E131" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
     </row>
     <row r="132" spans="1:16">
@@ -5689,7 +5754,7 @@
         <v>2</v>
       </c>
       <c r="E132" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
     </row>
     <row r="133" spans="1:16">
@@ -5700,7 +5765,7 @@
         <v>172</v>
       </c>
       <c r="E133" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="134" spans="1:16">
@@ -5711,46 +5776,46 @@
         <v>86</v>
       </c>
       <c r="C134" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D134">
         <v>0</v>
       </c>
       <c r="E134" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="F134" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="G134" t="s">
         <v>66</v>
       </c>
       <c r="H134" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I134" t="s">
         <v>73</v>
       </c>
       <c r="J134" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K134" t="s">
         <v>74</v>
       </c>
       <c r="L134" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="M134" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="N134" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="O134" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="P134" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="135" spans="1:16">
@@ -5761,7 +5826,7 @@
         <v>1</v>
       </c>
       <c r="E135" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
     </row>
     <row r="136" spans="1:16">
@@ -5772,7 +5837,7 @@
         <v>2</v>
       </c>
       <c r="E136" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
     </row>
     <row r="137" spans="1:16">
@@ -5783,7 +5848,7 @@
         <v>3</v>
       </c>
       <c r="E137" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="138" spans="1:16">
@@ -5794,7 +5859,7 @@
         <v>172</v>
       </c>
       <c r="E138" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
     </row>
     <row r="139" spans="1:16">
@@ -5805,46 +5870,46 @@
         <v>87</v>
       </c>
       <c r="C139" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D139">
         <v>0</v>
       </c>
       <c r="E139" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="F139" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="G139" t="s">
         <v>66</v>
       </c>
       <c r="H139" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I139" t="s">
         <v>73</v>
       </c>
       <c r="J139" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K139" t="s">
         <v>74</v>
       </c>
       <c r="L139" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="M139" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="N139" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="O139" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="P139" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="140" spans="1:16">
@@ -5855,7 +5920,7 @@
         <v>1</v>
       </c>
       <c r="E140" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
     </row>
     <row r="141" spans="1:16">
@@ -5866,7 +5931,7 @@
         <v>2</v>
       </c>
       <c r="E141" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
     </row>
     <row r="142" spans="1:16">
@@ -5877,7 +5942,7 @@
         <v>3</v>
       </c>
       <c r="E142" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="143" spans="1:16">
@@ -5888,7 +5953,7 @@
         <v>172</v>
       </c>
       <c r="E143" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
     </row>
     <row r="144" spans="1:16">
@@ -5899,34 +5964,34 @@
         <v>89</v>
       </c>
       <c r="C144" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D144">
         <v>0</v>
       </c>
       <c r="E144" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="F144" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="G144" t="s">
         <v>66</v>
       </c>
       <c r="H144" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="I144" t="s">
         <v>86</v>
       </c>
       <c r="J144" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K144" t="s">
         <v>87</v>
       </c>
       <c r="L144" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="145" spans="1:10">
@@ -5937,7 +6002,7 @@
         <v>1</v>
       </c>
       <c r="E145" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
     </row>
     <row r="146" spans="1:10">
@@ -5948,7 +6013,7 @@
         <v>2</v>
       </c>
       <c r="E146" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
     </row>
     <row r="147" spans="1:10">
@@ -5959,7 +6024,7 @@
         <v>3</v>
       </c>
       <c r="E147" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="148" spans="1:10">
@@ -5970,7 +6035,7 @@
         <v>172</v>
       </c>
       <c r="E148" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
     </row>
     <row r="149" spans="1:10">
@@ -5981,28 +6046,28 @@
         <v>90</v>
       </c>
       <c r="C149" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D149">
         <v>0</v>
       </c>
       <c r="E149" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F149" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="G149" t="s">
         <v>66</v>
       </c>
       <c r="H149" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I149" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="J149" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="150" spans="1:10">
@@ -6013,7 +6078,7 @@
         <v>1</v>
       </c>
       <c r="E150" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
     </row>
     <row r="151" spans="1:10">
@@ -6024,7 +6089,7 @@
         <v>172</v>
       </c>
       <c r="E151" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
     </row>
     <row r="152" spans="1:10">
@@ -6035,28 +6100,28 @@
         <v>91</v>
       </c>
       <c r="C152" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D152">
         <v>0</v>
       </c>
       <c r="E152" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="F152" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="G152" t="s">
         <v>66</v>
       </c>
       <c r="H152" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I152" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="J152" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="153" spans="1:10">
@@ -6067,7 +6132,7 @@
         <v>1</v>
       </c>
       <c r="E153" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
     </row>
     <row r="154" spans="1:10">
@@ -6078,7 +6143,7 @@
         <v>2</v>
       </c>
       <c r="E154" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="155" spans="1:10">
@@ -6089,7 +6154,7 @@
         <v>3</v>
       </c>
       <c r="E155" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
     </row>
     <row r="156" spans="1:10">
@@ -6100,7 +6165,7 @@
         <v>4</v>
       </c>
       <c r="E156" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
     </row>
     <row r="157" spans="1:10">
@@ -6111,7 +6176,7 @@
         <v>5</v>
       </c>
       <c r="E157" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
     </row>
     <row r="158" spans="1:10">
@@ -6122,7 +6187,7 @@
         <v>6</v>
       </c>
       <c r="E158" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="159" spans="1:10">
@@ -6133,7 +6198,7 @@
         <v>7</v>
       </c>
       <c r="E159" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
     <row r="160" spans="1:10">
@@ -6144,7 +6209,7 @@
         <v>172</v>
       </c>
       <c r="E160" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
     </row>
     <row r="161" spans="1:12">
@@ -6155,28 +6220,28 @@
         <v>92</v>
       </c>
       <c r="C161" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D161">
         <v>0</v>
       </c>
       <c r="E161" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="F161" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="G161" t="s">
         <v>66</v>
       </c>
       <c r="H161" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I161" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="J161" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="162" spans="1:12">
@@ -6187,7 +6252,7 @@
         <v>1</v>
       </c>
       <c r="E162" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
     </row>
     <row r="163" spans="1:12">
@@ -6198,7 +6263,7 @@
         <v>2</v>
       </c>
       <c r="E163" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
     </row>
     <row r="164" spans="1:12">
@@ -6209,7 +6274,7 @@
         <v>3</v>
       </c>
       <c r="E164" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
     </row>
     <row r="165" spans="1:12">
@@ -6220,7 +6285,7 @@
         <v>4</v>
       </c>
       <c r="E165" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="166" spans="1:12">
@@ -6231,7 +6296,7 @@
         <v>5</v>
       </c>
       <c r="E166" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="167" spans="1:12">
@@ -6242,7 +6307,7 @@
         <v>172</v>
       </c>
       <c r="E167" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
     </row>
     <row r="168" spans="1:12">
@@ -6253,34 +6318,34 @@
         <v>93</v>
       </c>
       <c r="C168" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D168">
         <v>0</v>
       </c>
       <c r="E168" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="F168" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="G168" t="s">
         <v>66</v>
       </c>
       <c r="H168" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="I168" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="J168" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="K168" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="L168" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="169" spans="1:12">
@@ -6291,7 +6356,7 @@
         <v>1</v>
       </c>
       <c r="E169" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="170" spans="1:12">
@@ -6302,7 +6367,7 @@
         <v>2</v>
       </c>
       <c r="E170" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
     </row>
     <row r="171" spans="1:12">
@@ -6313,7 +6378,7 @@
         <v>172</v>
       </c>
       <c r="E171" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -6353,7 +6418,7 @@
   <sheetData>
     <row r="1" spans="1:41" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A1" s="18" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>5</v>
@@ -6389,7 +6454,7 @@
         <v>15</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="N1" s="2" t="s">
         <v>60</v>
@@ -6467,1115 +6532,173 @@
         <v>93</v>
       </c>
       <c r="AM1" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="AN1" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="AO1" s="20" t="s">
-        <v>405</v>
+        <v>382</v>
+      </c>
+      <c r="AO1" s="19" t="s">
+        <v>399</v>
       </c>
     </row>
     <row r="2" spans="1:41">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="19"/>
-      <c r="W2" s="19"/>
-      <c r="X2" s="19"/>
-      <c r="Y2" s="19"/>
-      <c r="Z2" s="19"/>
-      <c r="AA2" s="19"/>
-      <c r="AB2" s="19"/>
-      <c r="AC2" s="19"/>
-      <c r="AD2" s="19"/>
-      <c r="AE2" s="19"/>
-      <c r="AF2" s="19"/>
-      <c r="AG2" s="19"/>
-      <c r="AH2" s="19"/>
-      <c r="AI2" s="19"/>
-      <c r="AJ2" s="19"/>
-      <c r="AK2" s="19"/>
-      <c r="AL2" s="19"/>
-      <c r="AM2" s="19"/>
-      <c r="AN2" s="19"/>
     </row>
     <row r="3" spans="1:41">
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="19"/>
-      <c r="S3" s="19"/>
-      <c r="T3" s="19"/>
-      <c r="U3" s="19"/>
-      <c r="V3" s="19"/>
-      <c r="W3" s="19"/>
-      <c r="X3" s="19"/>
-      <c r="Y3" s="19"/>
-      <c r="Z3" s="19"/>
-      <c r="AA3" s="19"/>
-      <c r="AB3" s="19"/>
-      <c r="AC3" s="19"/>
-      <c r="AD3" s="19"/>
-      <c r="AE3" s="19"/>
-      <c r="AF3" s="19"/>
-      <c r="AG3" s="19"/>
-      <c r="AH3" s="19"/>
-      <c r="AI3" s="19"/>
-      <c r="AJ3" s="19"/>
-      <c r="AK3" s="19"/>
-      <c r="AL3" s="19"/>
-      <c r="AM3" s="19"/>
-      <c r="AN3" s="19"/>
     </row>
     <row r="4" spans="1:41">
       <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="19"/>
-      <c r="U4" s="19"/>
-      <c r="V4" s="19"/>
-      <c r="W4" s="19"/>
-      <c r="X4" s="19"/>
-      <c r="Y4" s="19"/>
-      <c r="Z4" s="19"/>
-      <c r="AA4" s="19"/>
-      <c r="AB4" s="19"/>
-      <c r="AC4" s="19"/>
-      <c r="AD4" s="19"/>
-      <c r="AE4" s="19"/>
-      <c r="AF4" s="19"/>
-      <c r="AG4" s="19"/>
-      <c r="AH4" s="19"/>
-      <c r="AI4" s="19"/>
-      <c r="AJ4" s="19"/>
-      <c r="AK4" s="19"/>
-      <c r="AL4" s="19"/>
-      <c r="AM4" s="19"/>
-      <c r="AN4" s="19"/>
     </row>
     <row r="5" spans="1:41">
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="19"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
-      <c r="W5" s="19"/>
-      <c r="X5" s="19"/>
-      <c r="Y5" s="19"/>
-      <c r="Z5" s="19"/>
-      <c r="AA5" s="19"/>
-      <c r="AB5" s="19"/>
-      <c r="AC5" s="19"/>
-      <c r="AD5" s="19"/>
-      <c r="AE5" s="19"/>
-      <c r="AF5" s="19"/>
-      <c r="AG5" s="19"/>
-      <c r="AH5" s="19"/>
-      <c r="AI5" s="19"/>
-      <c r="AJ5" s="19"/>
-      <c r="AK5" s="19"/>
-      <c r="AL5" s="19"/>
-      <c r="AM5" s="19"/>
-      <c r="AN5" s="19"/>
     </row>
     <row r="6" spans="1:41">
       <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
-      <c r="P6" s="19"/>
-      <c r="Q6" s="19"/>
-      <c r="R6" s="19"/>
-      <c r="S6" s="19"/>
-      <c r="T6" s="19"/>
-      <c r="U6" s="19"/>
-      <c r="V6" s="19"/>
-      <c r="W6" s="19"/>
-      <c r="X6" s="19"/>
-      <c r="Y6" s="19"/>
-      <c r="Z6" s="19"/>
-      <c r="AA6" s="19"/>
-      <c r="AB6" s="19"/>
-      <c r="AC6" s="19"/>
-      <c r="AD6" s="19"/>
-      <c r="AE6" s="19"/>
-      <c r="AF6" s="19"/>
-      <c r="AG6" s="19"/>
-      <c r="AH6" s="19"/>
-      <c r="AI6" s="19"/>
-      <c r="AJ6" s="19"/>
-      <c r="AK6" s="19"/>
-      <c r="AL6" s="19"/>
-      <c r="AM6" s="19"/>
-      <c r="AN6" s="19"/>
     </row>
     <row r="7" spans="1:41">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="19"/>
-      <c r="P7" s="19"/>
-      <c r="Q7" s="19"/>
-      <c r="R7" s="19"/>
-      <c r="S7" s="19"/>
-      <c r="T7" s="19"/>
-      <c r="U7" s="19"/>
-      <c r="V7" s="19"/>
-      <c r="W7" s="19"/>
-      <c r="X7" s="19"/>
-      <c r="Y7" s="19"/>
-      <c r="Z7" s="19"/>
-      <c r="AA7" s="19"/>
-      <c r="AB7" s="19"/>
-      <c r="AC7" s="19"/>
-      <c r="AD7" s="19"/>
-      <c r="AE7" s="19"/>
-      <c r="AF7" s="19"/>
-      <c r="AG7" s="19"/>
-      <c r="AH7" s="19"/>
-      <c r="AI7" s="19"/>
-      <c r="AJ7" s="19"/>
-      <c r="AK7" s="19"/>
-      <c r="AL7" s="19"/>
-      <c r="AM7" s="19"/>
-      <c r="AN7" s="19"/>
     </row>
     <row r="8" spans="1:41">
       <c r="A8" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19"/>
-      <c r="M8" s="19"/>
-      <c r="N8" s="19"/>
-      <c r="O8" s="19"/>
-      <c r="P8" s="19"/>
-      <c r="Q8" s="19"/>
-      <c r="R8" s="19"/>
-      <c r="S8" s="19"/>
-      <c r="T8" s="19"/>
-      <c r="U8" s="19"/>
-      <c r="V8" s="19"/>
-      <c r="W8" s="19"/>
-      <c r="X8" s="19"/>
-      <c r="Y8" s="19"/>
-      <c r="Z8" s="19"/>
-      <c r="AA8" s="19"/>
-      <c r="AB8" s="19"/>
-      <c r="AC8" s="19"/>
-      <c r="AD8" s="19"/>
-      <c r="AE8" s="19"/>
-      <c r="AF8" s="19"/>
-      <c r="AG8" s="19"/>
-      <c r="AH8" s="19"/>
-      <c r="AI8" s="19"/>
-      <c r="AJ8" s="19"/>
-      <c r="AK8" s="19"/>
-      <c r="AL8" s="19"/>
-      <c r="AM8" s="19"/>
-      <c r="AN8" s="19"/>
     </row>
     <row r="9" spans="1:41">
       <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
-      <c r="N9" s="19"/>
-      <c r="O9" s="19"/>
-      <c r="P9" s="19"/>
-      <c r="Q9" s="19"/>
-      <c r="R9" s="19"/>
-      <c r="S9" s="19"/>
-      <c r="T9" s="19"/>
-      <c r="U9" s="19"/>
-      <c r="V9" s="19"/>
-      <c r="W9" s="19"/>
-      <c r="X9" s="19"/>
-      <c r="Y9" s="19"/>
-      <c r="Z9" s="19"/>
-      <c r="AA9" s="19"/>
-      <c r="AB9" s="19"/>
-      <c r="AC9" s="19"/>
-      <c r="AD9" s="19"/>
-      <c r="AE9" s="19"/>
-      <c r="AF9" s="19"/>
-      <c r="AG9" s="19"/>
-      <c r="AH9" s="19"/>
-      <c r="AI9" s="19"/>
-      <c r="AJ9" s="19"/>
-      <c r="AK9" s="19"/>
-      <c r="AL9" s="19"/>
-      <c r="AM9" s="19"/>
-      <c r="AN9" s="19"/>
     </row>
     <row r="10" spans="1:41">
       <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
-      <c r="N10" s="19"/>
-      <c r="O10" s="19"/>
-      <c r="P10" s="19"/>
-      <c r="Q10" s="19"/>
-      <c r="R10" s="19"/>
-      <c r="S10" s="19"/>
-      <c r="T10" s="19"/>
-      <c r="U10" s="19"/>
-      <c r="V10" s="19"/>
-      <c r="W10" s="19"/>
-      <c r="X10" s="19"/>
-      <c r="Y10" s="19"/>
-      <c r="Z10" s="19"/>
-      <c r="AA10" s="19"/>
-      <c r="AB10" s="19"/>
-      <c r="AC10" s="19"/>
-      <c r="AD10" s="19"/>
-      <c r="AE10" s="19"/>
-      <c r="AF10" s="19"/>
-      <c r="AG10" s="19"/>
-      <c r="AH10" s="19"/>
-      <c r="AI10" s="19"/>
-      <c r="AJ10" s="19"/>
-      <c r="AK10" s="19"/>
-      <c r="AL10" s="19"/>
-      <c r="AM10" s="19"/>
-      <c r="AN10" s="19"/>
     </row>
     <row r="11" spans="1:41">
       <c r="A11" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="19"/>
-      <c r="L11" s="19"/>
-      <c r="M11" s="19"/>
-      <c r="N11" s="19"/>
-      <c r="O11" s="19"/>
-      <c r="P11" s="19"/>
-      <c r="Q11" s="19"/>
-      <c r="R11" s="19"/>
-      <c r="S11" s="19"/>
-      <c r="T11" s="19"/>
-      <c r="U11" s="19"/>
-      <c r="V11" s="19"/>
-      <c r="W11" s="19"/>
-      <c r="X11" s="19"/>
-      <c r="Y11" s="19"/>
-      <c r="Z11" s="19"/>
-      <c r="AA11" s="19"/>
-      <c r="AB11" s="19"/>
-      <c r="AC11" s="19"/>
-      <c r="AD11" s="19"/>
-      <c r="AE11" s="19"/>
-      <c r="AF11" s="19"/>
-      <c r="AG11" s="19"/>
-      <c r="AH11" s="19"/>
-      <c r="AI11" s="19"/>
-      <c r="AJ11" s="19"/>
-      <c r="AK11" s="19"/>
-      <c r="AL11" s="19"/>
-      <c r="AM11" s="19"/>
-      <c r="AN11" s="19"/>
     </row>
     <row r="12" spans="1:41">
       <c r="A12" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="19"/>
-      <c r="M12" s="19"/>
-      <c r="N12" s="19"/>
-      <c r="O12" s="19"/>
-      <c r="P12" s="19"/>
-      <c r="Q12" s="19"/>
-      <c r="R12" s="19"/>
-      <c r="S12" s="19"/>
-      <c r="T12" s="19"/>
-      <c r="U12" s="19"/>
-      <c r="V12" s="19"/>
-      <c r="W12" s="19"/>
-      <c r="X12" s="19"/>
-      <c r="Y12" s="19"/>
-      <c r="Z12" s="19"/>
-      <c r="AA12" s="19"/>
-      <c r="AB12" s="19"/>
-      <c r="AC12" s="19"/>
-      <c r="AD12" s="19"/>
-      <c r="AE12" s="19"/>
-      <c r="AF12" s="19"/>
-      <c r="AG12" s="19"/>
-      <c r="AH12" s="19"/>
-      <c r="AI12" s="19"/>
-      <c r="AJ12" s="19"/>
-      <c r="AK12" s="19"/>
-      <c r="AL12" s="19"/>
-      <c r="AM12" s="19"/>
       <c r="AN12" s="16"/>
       <c r="AO12" s="11" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
     </row>
     <row r="13" spans="1:41">
       <c r="A13" t="s">
-        <v>396</v>
-      </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="19"/>
-      <c r="J13" s="19"/>
-      <c r="K13" s="19"/>
-      <c r="L13" s="19"/>
-      <c r="M13" s="19"/>
-      <c r="N13" s="19"/>
-      <c r="O13" s="19"/>
-      <c r="P13" s="19"/>
-      <c r="Q13" s="19"/>
-      <c r="R13" s="19"/>
-      <c r="S13" s="19"/>
-      <c r="T13" s="19"/>
-      <c r="U13" s="19"/>
-      <c r="V13" s="19"/>
-      <c r="W13" s="19"/>
-      <c r="X13" s="19"/>
-      <c r="Y13" s="19"/>
-      <c r="Z13" s="19"/>
-      <c r="AA13" s="19"/>
-      <c r="AB13" s="19"/>
-      <c r="AC13" s="19"/>
-      <c r="AD13" s="19"/>
-      <c r="AE13" s="19"/>
-      <c r="AF13" s="19"/>
-      <c r="AG13" s="19"/>
-      <c r="AH13" s="19"/>
-      <c r="AI13" s="19"/>
-      <c r="AJ13" s="19"/>
-      <c r="AK13" s="19"/>
-      <c r="AL13" s="19"/>
-      <c r="AM13" s="19"/>
+        <v>390</v>
+      </c>
       <c r="AN13" s="16"/>
     </row>
     <row r="14" spans="1:41">
       <c r="A14" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="19"/>
-      <c r="I14" s="19"/>
-      <c r="J14" s="19"/>
-      <c r="K14" s="19"/>
-      <c r="L14" s="19"/>
-      <c r="M14" s="19"/>
-      <c r="N14" s="19"/>
-      <c r="O14" s="19"/>
-      <c r="P14" s="19"/>
-      <c r="Q14" s="19"/>
       <c r="R14" s="16"/>
-      <c r="S14" s="19"/>
-      <c r="T14" s="19"/>
-      <c r="U14" s="19"/>
-      <c r="V14" s="19"/>
-      <c r="W14" s="19"/>
-      <c r="X14" s="19"/>
-      <c r="Y14" s="19"/>
-      <c r="Z14" s="16"/>
-      <c r="AA14" s="19"/>
-      <c r="AB14" s="19"/>
+      <c r="Z14" s="16" t="s">
+        <v>402</v>
+      </c>
       <c r="AC14" s="16"/>
       <c r="AD14" s="16"/>
-      <c r="AE14" s="19"/>
-      <c r="AF14" s="19"/>
-      <c r="AG14" s="19"/>
-      <c r="AH14" s="19"/>
-      <c r="AI14" s="19"/>
-      <c r="AJ14" s="19"/>
-      <c r="AK14" s="19"/>
-      <c r="AL14" s="19"/>
-      <c r="AM14" s="19"/>
       <c r="AN14" s="16"/>
     </row>
     <row r="15" spans="1:41">
       <c r="A15" t="s">
         <v>61</v>
       </c>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
-      <c r="J15" s="19"/>
-      <c r="K15" s="19"/>
-      <c r="L15" s="19"/>
-      <c r="M15" s="19"/>
-      <c r="N15" s="19"/>
-      <c r="O15" s="19"/>
-      <c r="P15" s="19"/>
-      <c r="Q15" s="19"/>
-      <c r="R15" s="19"/>
-      <c r="S15" s="19"/>
-      <c r="T15" s="19"/>
-      <c r="U15" s="19"/>
-      <c r="V15" s="19"/>
-      <c r="W15" s="19"/>
-      <c r="X15" s="19"/>
-      <c r="Y15" s="19"/>
-      <c r="Z15" s="19"/>
-      <c r="AA15" s="19"/>
-      <c r="AB15" s="19"/>
-      <c r="AC15" s="19"/>
-      <c r="AD15" s="19"/>
-      <c r="AE15" s="19"/>
-      <c r="AF15" s="19"/>
-      <c r="AG15" s="19"/>
-      <c r="AH15" s="19"/>
-      <c r="AI15" s="19"/>
-      <c r="AJ15" s="19"/>
-      <c r="AK15" s="19"/>
-      <c r="AL15" s="19"/>
-      <c r="AM15" s="19"/>
-      <c r="AN15" s="19"/>
     </row>
     <row r="16" spans="1:41">
       <c r="A16" t="s">
         <v>62</v>
       </c>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
-      <c r="L16" s="19"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="19"/>
-      <c r="O16" s="19"/>
-      <c r="P16" s="19"/>
-      <c r="Q16" s="19"/>
-      <c r="R16" s="19"/>
-      <c r="S16" s="19"/>
-      <c r="T16" s="19"/>
-      <c r="U16" s="19"/>
-      <c r="V16" s="19"/>
-      <c r="W16" s="19"/>
-      <c r="X16" s="19"/>
-      <c r="Y16" s="19"/>
-      <c r="Z16" s="19"/>
-      <c r="AA16" s="19"/>
-      <c r="AB16" s="19"/>
-      <c r="AC16" s="19"/>
-      <c r="AD16" s="19"/>
-      <c r="AE16" s="19"/>
-      <c r="AF16" s="19"/>
-      <c r="AG16" s="19"/>
-      <c r="AH16" s="19"/>
-      <c r="AI16" s="19"/>
-      <c r="AJ16" s="19"/>
-      <c r="AK16" s="19"/>
-      <c r="AL16" s="19"/>
       <c r="AM16" s="16"/>
-      <c r="AN16" s="19"/>
     </row>
     <row r="17" spans="1:40">
       <c r="A17" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="19"/>
-      <c r="K17" s="19"/>
-      <c r="L17" s="19"/>
-      <c r="M17" s="19"/>
-      <c r="N17" s="19"/>
-      <c r="O17" s="19"/>
-      <c r="P17" s="19"/>
-      <c r="Q17" s="19"/>
-      <c r="R17" s="19"/>
-      <c r="S17" s="19"/>
-      <c r="T17" s="19"/>
-      <c r="U17" s="19"/>
-      <c r="V17" s="19"/>
-      <c r="W17" s="19"/>
-      <c r="X17" s="19"/>
-      <c r="Y17" s="19"/>
-      <c r="Z17" s="19"/>
-      <c r="AA17" s="19"/>
-      <c r="AB17" s="19"/>
-      <c r="AC17" s="19"/>
-      <c r="AD17" s="19"/>
-      <c r="AE17" s="19"/>
-      <c r="AF17" s="19"/>
-      <c r="AG17" s="19"/>
-      <c r="AH17" s="19"/>
-      <c r="AI17" s="19"/>
-      <c r="AJ17" s="19"/>
-      <c r="AK17" s="19"/>
-      <c r="AL17" s="19"/>
       <c r="AM17" s="16"/>
-      <c r="AN17" s="19"/>
     </row>
     <row r="18" spans="1:40">
       <c r="A18" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="19"/>
-      <c r="O18" s="19"/>
       <c r="P18" s="16"/>
       <c r="Q18" s="16"/>
-      <c r="R18" s="19"/>
-      <c r="S18" s="19"/>
-      <c r="T18" s="19"/>
-      <c r="U18" s="19"/>
-      <c r="V18" s="19"/>
-      <c r="W18" s="19"/>
-      <c r="X18" s="19"/>
-      <c r="Y18" s="19"/>
-      <c r="Z18" s="19"/>
-      <c r="AA18" s="19"/>
-      <c r="AB18" s="19"/>
-      <c r="AC18" s="19"/>
-      <c r="AD18" s="19"/>
-      <c r="AE18" s="19"/>
-      <c r="AF18" s="19"/>
-      <c r="AG18" s="19"/>
-      <c r="AH18" s="19"/>
-      <c r="AI18" s="19"/>
-      <c r="AJ18" s="19"/>
-      <c r="AK18" s="19"/>
-      <c r="AL18" s="19"/>
       <c r="AM18" s="16"/>
-      <c r="AN18" s="19"/>
     </row>
     <row r="19" spans="1:40">
       <c r="A19" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="19"/>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="19"/>
-      <c r="N19" s="19"/>
-      <c r="O19" s="19"/>
-      <c r="P19" s="19"/>
-      <c r="Q19" s="19"/>
-      <c r="R19" s="19"/>
-      <c r="S19" s="19"/>
-      <c r="T19" s="19"/>
-      <c r="U19" s="19"/>
-      <c r="V19" s="19"/>
-      <c r="W19" s="19"/>
-      <c r="X19" s="19"/>
-      <c r="Y19" s="19"/>
-      <c r="Z19" s="19"/>
-      <c r="AA19" s="19"/>
-      <c r="AB19" s="19"/>
-      <c r="AC19" s="19"/>
-      <c r="AD19" s="19"/>
-      <c r="AE19" s="19"/>
-      <c r="AF19" s="19"/>
-      <c r="AG19" s="19"/>
-      <c r="AH19" s="19"/>
-      <c r="AI19" s="19"/>
-      <c r="AJ19" s="19"/>
-      <c r="AK19" s="19"/>
-      <c r="AL19" s="19"/>
-      <c r="AM19" s="19"/>
-      <c r="AN19" s="19"/>
     </row>
     <row r="20" spans="1:40">
       <c r="A20" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="19"/>
-      <c r="O20" s="19"/>
-      <c r="P20" s="19"/>
-      <c r="Q20" s="19"/>
-      <c r="R20" s="19"/>
-      <c r="S20" s="19"/>
-      <c r="T20" s="19"/>
-      <c r="U20" s="19"/>
-      <c r="V20" s="19"/>
-      <c r="W20" s="19"/>
-      <c r="X20" s="19"/>
-      <c r="Y20" s="19"/>
-      <c r="Z20" s="19"/>
-      <c r="AA20" s="19"/>
-      <c r="AB20" s="19"/>
-      <c r="AC20" s="19"/>
-      <c r="AD20" s="19"/>
-      <c r="AE20" s="19"/>
-      <c r="AF20" s="19"/>
-      <c r="AG20" s="19"/>
-      <c r="AH20" s="19"/>
-      <c r="AI20" s="19"/>
-      <c r="AJ20" s="19"/>
-      <c r="AK20" s="19"/>
-      <c r="AL20" s="19"/>
-      <c r="AM20" s="19"/>
-      <c r="AN20" s="19"/>
     </row>
     <row r="21" spans="1:40">
       <c r="A21" t="s">
         <v>69</v>
       </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="19"/>
       <c r="L21" s="16"/>
       <c r="M21" s="16"/>
-      <c r="N21" s="19"/>
-      <c r="O21" s="19"/>
-      <c r="P21" s="19"/>
       <c r="Q21" s="16"/>
-      <c r="R21" s="19"/>
-      <c r="S21" s="19"/>
-      <c r="T21" s="19"/>
-      <c r="U21" s="19"/>
-      <c r="V21" s="19"/>
-      <c r="W21" s="19"/>
-      <c r="X21" s="19"/>
-      <c r="Y21" s="19"/>
-      <c r="Z21" s="19"/>
-      <c r="AA21" s="19"/>
-      <c r="AB21" s="19"/>
-      <c r="AC21" s="19"/>
-      <c r="AD21" s="19"/>
-      <c r="AE21" s="19"/>
-      <c r="AF21" s="19"/>
-      <c r="AG21" s="19"/>
-      <c r="AH21" s="19"/>
-      <c r="AI21" s="19"/>
-      <c r="AJ21" s="19"/>
-      <c r="AK21" s="19"/>
-      <c r="AL21" s="19"/>
       <c r="AM21" s="16"/>
-      <c r="AN21" s="19"/>
     </row>
     <row r="22" spans="1:40">
       <c r="A22" t="s">
         <v>71</v>
       </c>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="19"/>
-      <c r="J22" s="19"/>
-      <c r="K22" s="19"/>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19"/>
       <c r="N22" s="16"/>
-      <c r="O22" s="19"/>
-      <c r="P22" s="19"/>
       <c r="Q22" s="16"/>
-      <c r="R22" s="19"/>
-      <c r="S22" s="19"/>
-      <c r="T22" s="19"/>
-      <c r="U22" s="19"/>
-      <c r="V22" s="19"/>
-      <c r="W22" s="19"/>
-      <c r="X22" s="19"/>
-      <c r="Y22" s="19"/>
-      <c r="Z22" s="16"/>
+      <c r="Z22" s="20" t="s">
+        <v>401</v>
+      </c>
       <c r="AA22" s="16"/>
-      <c r="AB22" s="19"/>
-      <c r="AC22" s="19"/>
       <c r="AD22" s="16"/>
-      <c r="AE22" s="19"/>
-      <c r="AF22" s="19"/>
-      <c r="AG22" s="19"/>
-      <c r="AH22" s="19"/>
-      <c r="AI22" s="19"/>
-      <c r="AJ22" s="19"/>
-      <c r="AK22" s="19"/>
-      <c r="AL22" s="19"/>
       <c r="AM22" s="16"/>
-      <c r="AN22" s="19"/>
     </row>
     <row r="23" spans="1:40">
       <c r="A23" t="s">
         <v>73</v>
       </c>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="19"/>
-      <c r="O23" s="19"/>
-      <c r="P23" s="19"/>
-      <c r="Q23" s="19"/>
-      <c r="R23" s="19"/>
-      <c r="S23" s="19"/>
-      <c r="T23" s="19"/>
-      <c r="U23" s="19"/>
-      <c r="V23" s="19"/>
-      <c r="W23" s="19"/>
-      <c r="X23" s="19"/>
-      <c r="Y23" s="19"/>
-      <c r="Z23" s="19"/>
-      <c r="AA23" s="19"/>
-      <c r="AB23" s="19"/>
-      <c r="AC23" s="19"/>
-      <c r="AD23" s="19"/>
-      <c r="AE23" s="19"/>
-      <c r="AF23" s="19"/>
-      <c r="AG23" s="19"/>
-      <c r="AH23" s="19"/>
-      <c r="AI23" s="19"/>
-      <c r="AJ23" s="19"/>
-      <c r="AK23" s="19"/>
-      <c r="AL23" s="19"/>
-      <c r="AM23" s="19"/>
-      <c r="AN23" s="19"/>
     </row>
     <row r="24" spans="1:40">
       <c r="A24" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="19"/>
-      <c r="I24" s="19"/>
-      <c r="J24" s="19"/>
-      <c r="K24" s="19"/>
-      <c r="L24" s="19"/>
-      <c r="M24" s="19"/>
-      <c r="N24" s="19"/>
-      <c r="O24" s="19"/>
-      <c r="P24" s="19"/>
-      <c r="Q24" s="19"/>
-      <c r="R24" s="19"/>
-      <c r="S24" s="19"/>
-      <c r="T24" s="19"/>
-      <c r="U24" s="19"/>
-      <c r="V24" s="19"/>
-      <c r="W24" s="19"/>
-      <c r="X24" s="19"/>
-      <c r="Y24" s="19"/>
-      <c r="Z24" s="19"/>
-      <c r="AA24" s="19"/>
-      <c r="AB24" s="19"/>
-      <c r="AC24" s="19"/>
-      <c r="AD24" s="19"/>
-      <c r="AE24" s="19"/>
-      <c r="AF24" s="19"/>
-      <c r="AG24" s="19"/>
-      <c r="AH24" s="19"/>
-      <c r="AI24" s="19"/>
-      <c r="AJ24" s="19"/>
-      <c r="AK24" s="19"/>
-      <c r="AL24" s="19"/>
-      <c r="AM24" s="19"/>
-      <c r="AN24" s="19"/>
     </row>
     <row r="25" spans="1:40">
       <c r="A25" t="s">
         <v>75</v>
       </c>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
-      <c r="J25" s="19"/>
-      <c r="K25" s="19"/>
-      <c r="L25" s="19"/>
-      <c r="M25" s="19"/>
-      <c r="N25" s="19"/>
-      <c r="O25" s="19"/>
       <c r="P25" s="16"/>
-      <c r="Q25" s="19"/>
-      <c r="R25" s="19"/>
-      <c r="S25" s="19"/>
-      <c r="T25" s="19"/>
-      <c r="U25" s="19"/>
-      <c r="V25" s="19"/>
-      <c r="W25" s="19"/>
-      <c r="X25" s="19"/>
-      <c r="Y25" s="19"/>
-      <c r="Z25" s="19"/>
       <c r="AA25" s="16"/>
-      <c r="AB25" s="19"/>
-      <c r="AC25" s="19"/>
-      <c r="AD25" s="19"/>
-      <c r="AE25" s="19"/>
-      <c r="AF25" s="19"/>
-      <c r="AG25" s="19"/>
-      <c r="AH25" s="19"/>
-      <c r="AI25" s="19"/>
-      <c r="AJ25" s="19"/>
-      <c r="AK25" s="19"/>
-      <c r="AL25" s="19"/>
       <c r="AM25" s="16"/>
-      <c r="AN25" s="19"/>
     </row>
     <row r="26" spans="1:40">
       <c r="A26" t="s">
         <v>77</v>
       </c>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="19"/>
-      <c r="I26" s="19"/>
-      <c r="J26" s="19"/>
-      <c r="K26" s="19"/>
-      <c r="L26" s="19"/>
-      <c r="M26" s="19"/>
-      <c r="N26" s="19"/>
-      <c r="O26" s="19"/>
-      <c r="P26" s="19"/>
-      <c r="Q26" s="19"/>
       <c r="R26" s="16"/>
-      <c r="S26" s="19"/>
-      <c r="T26" s="19"/>
       <c r="U26" s="16"/>
-      <c r="V26" s="19"/>
-      <c r="W26" s="19"/>
-      <c r="X26" s="19"/>
-      <c r="Y26" s="19"/>
-      <c r="Z26" s="19"/>
-      <c r="AA26" s="19"/>
-      <c r="AB26" s="19"/>
-      <c r="AC26" s="19"/>
-      <c r="AD26" s="19"/>
-      <c r="AE26" s="19"/>
-      <c r="AF26" s="19"/>
-      <c r="AG26" s="19"/>
-      <c r="AH26" s="19"/>
-      <c r="AI26" s="19"/>
-      <c r="AJ26" s="19"/>
-      <c r="AK26" s="19"/>
-      <c r="AL26" s="19"/>
       <c r="AM26" s="16"/>
       <c r="AN26" s="16"/>
     </row>
@@ -7583,656 +6706,139 @@
       <c r="A27" t="s">
         <v>78</v>
       </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19"/>
-      <c r="I27" s="19"/>
-      <c r="J27" s="19"/>
-      <c r="K27" s="19"/>
-      <c r="L27" s="19"/>
-      <c r="M27" s="19"/>
-      <c r="N27" s="19"/>
-      <c r="O27" s="19"/>
       <c r="P27" s="16"/>
-      <c r="Q27" s="19"/>
-      <c r="R27" s="19"/>
-      <c r="S27" s="19"/>
-      <c r="T27" s="19"/>
-      <c r="U27" s="19"/>
       <c r="V27" s="16"/>
-      <c r="W27" s="19"/>
-      <c r="X27" s="19"/>
-      <c r="Y27" s="19"/>
-      <c r="Z27" s="19"/>
-      <c r="AA27" s="19"/>
-      <c r="AB27" s="19"/>
-      <c r="AC27" s="19"/>
-      <c r="AD27" s="19"/>
-      <c r="AE27" s="19"/>
-      <c r="AF27" s="19"/>
-      <c r="AG27" s="19"/>
-      <c r="AH27" s="19"/>
       <c r="AI27" s="16"/>
       <c r="AJ27" s="16"/>
       <c r="AK27" s="16"/>
-      <c r="AL27" s="19"/>
-      <c r="AM27" s="19"/>
       <c r="AN27" s="16"/>
     </row>
     <row r="28" spans="1:40">
       <c r="A28" t="s">
         <v>79</v>
       </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
-      <c r="L28" s="19"/>
-      <c r="M28" s="19"/>
-      <c r="N28" s="19"/>
-      <c r="O28" s="19"/>
-      <c r="P28" s="19"/>
-      <c r="Q28" s="19"/>
       <c r="R28" s="16"/>
-      <c r="S28" s="19"/>
-      <c r="T28" s="19"/>
-      <c r="U28" s="19"/>
-      <c r="V28" s="19"/>
-      <c r="W28" s="19"/>
-      <c r="X28" s="19"/>
-      <c r="Y28" s="19"/>
       <c r="Z28" s="16"/>
-      <c r="AA28" s="19"/>
-      <c r="AB28" s="19"/>
-      <c r="AC28" s="19"/>
-      <c r="AD28" s="19"/>
-      <c r="AE28" s="19"/>
-      <c r="AF28" s="19"/>
-      <c r="AG28" s="19"/>
-      <c r="AH28" s="19"/>
-      <c r="AI28" s="19"/>
-      <c r="AJ28" s="19"/>
-      <c r="AK28" s="19"/>
-      <c r="AL28" s="19"/>
-      <c r="AM28" s="19"/>
-      <c r="AN28" s="19"/>
     </row>
     <row r="29" spans="1:40">
       <c r="A29" t="s">
         <v>80</v>
       </c>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="19"/>
-      <c r="I29" s="19"/>
-      <c r="J29" s="19"/>
-      <c r="K29" s="19"/>
-      <c r="L29" s="19"/>
-      <c r="M29" s="19"/>
-      <c r="N29" s="19"/>
-      <c r="O29" s="19"/>
-      <c r="P29" s="19"/>
-      <c r="Q29" s="19"/>
       <c r="R29" s="16"/>
-      <c r="S29" s="19"/>
-      <c r="T29" s="19"/>
-      <c r="U29" s="19"/>
-      <c r="V29" s="19"/>
-      <c r="W29" s="19"/>
-      <c r="X29" s="19"/>
-      <c r="Y29" s="19"/>
       <c r="Z29" s="16"/>
-      <c r="AA29" s="19"/>
-      <c r="AB29" s="19"/>
-      <c r="AC29" s="19"/>
       <c r="AD29" s="16" t="s">
-        <v>395</v>
-      </c>
-      <c r="AE29" s="19"/>
-      <c r="AF29" s="19"/>
-      <c r="AG29" s="19"/>
-      <c r="AH29" s="19"/>
-      <c r="AI29" s="19"/>
-      <c r="AJ29" s="19"/>
-      <c r="AK29" s="19"/>
-      <c r="AL29" s="19"/>
-      <c r="AM29" s="19"/>
-      <c r="AN29" s="19"/>
+        <v>389</v>
+      </c>
     </row>
     <row r="30" spans="1:40">
       <c r="A30" t="s">
         <v>84</v>
       </c>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="19"/>
-      <c r="J30" s="19"/>
-      <c r="K30" s="19"/>
       <c r="L30" s="16"/>
-      <c r="M30" s="19"/>
-      <c r="N30" s="19"/>
-      <c r="O30" s="19"/>
-      <c r="P30" s="19"/>
-      <c r="Q30" s="19"/>
       <c r="R30" s="16"/>
-      <c r="S30" s="19"/>
-      <c r="T30" s="19"/>
-      <c r="U30" s="19"/>
-      <c r="V30" s="19"/>
-      <c r="W30" s="19"/>
-      <c r="X30" s="19"/>
-      <c r="Y30" s="19"/>
       <c r="Z30" s="16"/>
-      <c r="AA30" s="19"/>
-      <c r="AB30" s="19"/>
-      <c r="AC30" s="19"/>
-      <c r="AD30" s="19"/>
-      <c r="AE30" s="19"/>
-      <c r="AF30" s="19"/>
-      <c r="AG30" s="19"/>
-      <c r="AH30" s="19"/>
-      <c r="AI30" s="19"/>
-      <c r="AJ30" s="19"/>
-      <c r="AK30" s="19"/>
-      <c r="AL30" s="19"/>
-      <c r="AM30" s="19"/>
-      <c r="AN30" s="19"/>
     </row>
     <row r="31" spans="1:40">
       <c r="A31" t="s">
         <v>85</v>
       </c>
-      <c r="B31" s="19"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="19"/>
-      <c r="I31" s="19"/>
-      <c r="J31" s="19"/>
-      <c r="K31" s="19"/>
-      <c r="L31" s="19"/>
-      <c r="M31" s="19"/>
-      <c r="N31" s="19"/>
-      <c r="O31" s="19"/>
-      <c r="P31" s="19"/>
-      <c r="Q31" s="19"/>
-      <c r="R31" s="19"/>
-      <c r="S31" s="19"/>
-      <c r="T31" s="19"/>
-      <c r="U31" s="19"/>
-      <c r="V31" s="19"/>
-      <c r="W31" s="19"/>
-      <c r="X31" s="19"/>
-      <c r="Y31" s="19"/>
-      <c r="Z31" s="19"/>
-      <c r="AA31" s="19"/>
-      <c r="AB31" s="19"/>
-      <c r="AC31" s="19"/>
-      <c r="AD31" s="19"/>
-      <c r="AE31" s="19"/>
-      <c r="AF31" s="19"/>
-      <c r="AG31" s="19"/>
-      <c r="AH31" s="19"/>
-      <c r="AI31" s="19"/>
-      <c r="AJ31" s="19"/>
-      <c r="AK31" s="19"/>
-      <c r="AL31" s="19"/>
-      <c r="AM31" s="19"/>
-      <c r="AN31" s="19"/>
     </row>
     <row r="32" spans="1:40">
       <c r="A32" t="s">
         <v>86</v>
       </c>
-      <c r="B32" s="19"/>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="19"/>
-      <c r="J32" s="19"/>
-      <c r="K32" s="19"/>
-      <c r="L32" s="19"/>
-      <c r="M32" s="19"/>
-      <c r="N32" s="19"/>
-      <c r="O32" s="19"/>
-      <c r="P32" s="19"/>
-      <c r="Q32" s="19"/>
-      <c r="R32" s="19"/>
-      <c r="S32" s="19"/>
-      <c r="T32" s="19"/>
       <c r="U32" s="16"/>
-      <c r="V32" s="19"/>
-      <c r="W32" s="19"/>
-      <c r="X32" s="19"/>
-      <c r="Y32" s="19"/>
       <c r="Z32" s="16"/>
-      <c r="AA32" s="19"/>
       <c r="AB32" s="16"/>
-      <c r="AC32" s="19"/>
-      <c r="AD32" s="19"/>
-      <c r="AE32" s="19"/>
-      <c r="AF32" s="19"/>
-      <c r="AG32" s="19"/>
       <c r="AH32" s="16"/>
-      <c r="AI32" s="19"/>
-      <c r="AJ32" s="19"/>
-      <c r="AK32" s="19"/>
-      <c r="AL32" s="19"/>
-      <c r="AM32" s="19"/>
       <c r="AN32" s="16"/>
     </row>
     <row r="33" spans="1:40">
       <c r="A33" t="s">
         <v>87</v>
       </c>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="19"/>
-      <c r="J33" s="19"/>
-      <c r="K33" s="19"/>
-      <c r="L33" s="19"/>
-      <c r="M33" s="19"/>
-      <c r="N33" s="19"/>
-      <c r="O33" s="19"/>
-      <c r="P33" s="19"/>
-      <c r="Q33" s="19"/>
-      <c r="R33" s="19"/>
-      <c r="S33" s="19"/>
-      <c r="T33" s="19"/>
       <c r="U33" s="16"/>
-      <c r="V33" s="19"/>
-      <c r="W33" s="19"/>
-      <c r="X33" s="19"/>
-      <c r="Y33" s="19"/>
       <c r="Z33" s="16"/>
-      <c r="AA33" s="19"/>
-      <c r="AB33" s="19"/>
       <c r="AC33" s="16"/>
       <c r="AD33" s="16"/>
-      <c r="AE33" s="19"/>
-      <c r="AF33" s="19"/>
-      <c r="AG33" s="19"/>
       <c r="AH33" s="16"/>
-      <c r="AI33" s="19"/>
-      <c r="AJ33" s="19"/>
-      <c r="AK33" s="19"/>
-      <c r="AL33" s="19"/>
-      <c r="AM33" s="19"/>
       <c r="AN33" s="16"/>
     </row>
     <row r="34" spans="1:40">
       <c r="A34" t="s">
         <v>89</v>
       </c>
-      <c r="B34" s="19"/>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="19"/>
-      <c r="I34" s="19"/>
-      <c r="J34" s="19"/>
-      <c r="K34" s="19"/>
-      <c r="L34" s="19"/>
-      <c r="M34" s="19"/>
-      <c r="N34" s="19"/>
-      <c r="O34" s="19"/>
-      <c r="P34" s="19"/>
-      <c r="Q34" s="19"/>
-      <c r="R34" s="19"/>
-      <c r="S34" s="19"/>
-      <c r="T34" s="19"/>
-      <c r="U34" s="19"/>
-      <c r="V34" s="19"/>
-      <c r="W34" s="19"/>
-      <c r="X34" s="19"/>
-      <c r="Y34" s="19"/>
-      <c r="Z34" s="19"/>
-      <c r="AA34" s="19"/>
-      <c r="AB34" s="19"/>
-      <c r="AC34" s="19"/>
-      <c r="AD34" s="19"/>
-      <c r="AE34" s="19"/>
-      <c r="AF34" s="19"/>
-      <c r="AG34" s="19"/>
-      <c r="AH34" s="19"/>
-      <c r="AI34" s="19"/>
-      <c r="AJ34" s="19"/>
-      <c r="AK34" s="19"/>
-      <c r="AL34" s="19"/>
-      <c r="AM34" s="19"/>
-      <c r="AN34" s="19"/>
     </row>
     <row r="35" spans="1:40">
       <c r="A35" t="s">
         <v>90</v>
       </c>
-      <c r="B35" s="19"/>
-      <c r="C35" s="19"/>
-      <c r="D35" s="19"/>
-      <c r="E35" s="19"/>
-      <c r="F35" s="19"/>
-      <c r="G35" s="19"/>
-      <c r="H35" s="19"/>
-      <c r="I35" s="19"/>
-      <c r="J35" s="19"/>
-      <c r="K35" s="19"/>
-      <c r="L35" s="19"/>
-      <c r="M35" s="19"/>
-      <c r="N35" s="19"/>
-      <c r="O35" s="19"/>
-      <c r="P35" s="19"/>
-      <c r="Q35" s="19"/>
-      <c r="R35" s="19"/>
-      <c r="S35" s="19"/>
-      <c r="T35" s="19"/>
-      <c r="U35" s="19"/>
-      <c r="V35" s="19"/>
-      <c r="W35" s="19"/>
-      <c r="X35" s="19"/>
-      <c r="Y35" s="19"/>
-      <c r="Z35" s="19"/>
-      <c r="AA35" s="19"/>
-      <c r="AB35" s="19"/>
-      <c r="AC35" s="19"/>
-      <c r="AD35" s="19"/>
-      <c r="AE35" s="19"/>
-      <c r="AF35" s="19"/>
-      <c r="AG35" s="19"/>
-      <c r="AH35" s="19"/>
-      <c r="AI35" s="19"/>
-      <c r="AJ35" s="19"/>
-      <c r="AK35" s="19"/>
-      <c r="AL35" s="19"/>
-      <c r="AM35" s="19"/>
       <c r="AN35" s="16"/>
     </row>
     <row r="36" spans="1:40">
       <c r="A36" t="s">
         <v>91</v>
       </c>
-      <c r="B36" s="19"/>
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="19"/>
-      <c r="G36" s="19"/>
-      <c r="H36" s="19"/>
-      <c r="I36" s="19"/>
-      <c r="J36" s="19"/>
-      <c r="K36" s="19"/>
-      <c r="L36" s="19"/>
-      <c r="M36" s="19"/>
-      <c r="N36" s="19"/>
-      <c r="O36" s="19"/>
-      <c r="P36" s="19"/>
-      <c r="Q36" s="19"/>
-      <c r="R36" s="19"/>
-      <c r="S36" s="19"/>
-      <c r="T36" s="19"/>
-      <c r="U36" s="19"/>
-      <c r="V36" s="19"/>
-      <c r="W36" s="19"/>
-      <c r="X36" s="19"/>
-      <c r="Y36" s="19"/>
-      <c r="Z36" s="19"/>
-      <c r="AA36" s="19"/>
-      <c r="AB36" s="19"/>
-      <c r="AC36" s="19"/>
-      <c r="AD36" s="19"/>
-      <c r="AE36" s="19"/>
-      <c r="AF36" s="19"/>
-      <c r="AG36" s="19"/>
-      <c r="AH36" s="19"/>
-      <c r="AI36" s="19"/>
-      <c r="AJ36" s="19"/>
-      <c r="AK36" s="19"/>
-      <c r="AL36" s="19"/>
-      <c r="AM36" s="19"/>
       <c r="AN36" s="16"/>
     </row>
     <row r="37" spans="1:40">
       <c r="A37" t="s">
         <v>92</v>
       </c>
-      <c r="B37" s="19"/>
-      <c r="C37" s="19"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="19"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="19"/>
-      <c r="H37" s="19"/>
-      <c r="I37" s="19"/>
-      <c r="J37" s="19"/>
-      <c r="K37" s="19"/>
-      <c r="L37" s="19"/>
-      <c r="M37" s="19"/>
-      <c r="N37" s="19"/>
-      <c r="O37" s="19"/>
-      <c r="P37" s="19"/>
-      <c r="Q37" s="19"/>
-      <c r="R37" s="19"/>
-      <c r="S37" s="19"/>
-      <c r="T37" s="19"/>
-      <c r="U37" s="19"/>
-      <c r="V37" s="19"/>
-      <c r="W37" s="19"/>
-      <c r="X37" s="19"/>
-      <c r="Y37" s="19"/>
-      <c r="Z37" s="19"/>
-      <c r="AA37" s="19"/>
-      <c r="AB37" s="19"/>
-      <c r="AC37" s="19"/>
-      <c r="AD37" s="19"/>
-      <c r="AE37" s="19"/>
-      <c r="AF37" s="19"/>
-      <c r="AG37" s="19"/>
-      <c r="AH37" s="19"/>
-      <c r="AI37" s="19"/>
-      <c r="AJ37" s="19"/>
-      <c r="AK37" s="19"/>
-      <c r="AL37" s="19"/>
-      <c r="AM37" s="19"/>
       <c r="AN37" s="16"/>
     </row>
     <row r="38" spans="1:40">
       <c r="A38" t="s">
         <v>93</v>
       </c>
-      <c r="B38" s="19"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="19"/>
-      <c r="J38" s="19"/>
-      <c r="K38" s="19"/>
-      <c r="L38" s="19"/>
-      <c r="M38" s="19"/>
-      <c r="N38" s="19"/>
-      <c r="O38" s="19"/>
-      <c r="P38" s="19"/>
-      <c r="Q38" s="19"/>
-      <c r="R38" s="19"/>
-      <c r="S38" s="19"/>
-      <c r="T38" s="19"/>
-      <c r="U38" s="19"/>
-      <c r="V38" s="19"/>
-      <c r="W38" s="19"/>
-      <c r="X38" s="19"/>
-      <c r="Y38" s="19"/>
-      <c r="Z38" s="19"/>
-      <c r="AA38" s="19"/>
-      <c r="AB38" s="19"/>
-      <c r="AC38" s="19"/>
-      <c r="AD38" s="19"/>
-      <c r="AE38" s="19"/>
-      <c r="AF38" s="19"/>
-      <c r="AG38" s="19"/>
-      <c r="AH38" s="19"/>
-      <c r="AI38" s="19"/>
-      <c r="AJ38" s="19"/>
-      <c r="AK38" s="19"/>
-      <c r="AL38" s="19"/>
-      <c r="AM38" s="19"/>
       <c r="AN38" s="16"/>
     </row>
     <row r="39" spans="1:40">
       <c r="A39" t="s">
-        <v>389</v>
-      </c>
-      <c r="B39" s="19"/>
-      <c r="C39" s="19"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="19"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="19"/>
-      <c r="J39" s="19"/>
-      <c r="K39" s="19"/>
-      <c r="L39" s="19"/>
-      <c r="M39" s="19"/>
-      <c r="N39" s="19"/>
-      <c r="O39" s="19"/>
-      <c r="P39" s="19"/>
-      <c r="Q39" s="19"/>
-      <c r="R39" s="19"/>
-      <c r="S39" s="19"/>
-      <c r="T39" s="19"/>
-      <c r="U39" s="19"/>
-      <c r="V39" s="19"/>
-      <c r="W39" s="19"/>
-      <c r="X39" s="19"/>
-      <c r="Y39" s="19"/>
-      <c r="Z39" s="19"/>
-      <c r="AA39" s="19"/>
-      <c r="AB39" s="19"/>
-      <c r="AC39" s="19"/>
-      <c r="AD39" s="19"/>
-      <c r="AE39" s="19"/>
-      <c r="AF39" s="19"/>
-      <c r="AG39" s="19"/>
-      <c r="AH39" s="19"/>
-      <c r="AI39" s="19"/>
-      <c r="AJ39" s="19"/>
-      <c r="AK39" s="19"/>
-      <c r="AL39" s="19"/>
-      <c r="AM39" s="19"/>
-      <c r="AN39" s="19"/>
+        <v>383</v>
+      </c>
     </row>
     <row r="40" spans="1:40">
       <c r="A40" t="s">
-        <v>388</v>
-      </c>
-      <c r="B40" s="19"/>
-      <c r="C40" s="19"/>
-      <c r="D40" s="19"/>
-      <c r="E40" s="19"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="19"/>
-      <c r="H40" s="19"/>
-      <c r="I40" s="19"/>
-      <c r="J40" s="19"/>
-      <c r="K40" s="19"/>
-      <c r="L40" s="19"/>
-      <c r="M40" s="19"/>
-      <c r="N40" s="19"/>
-      <c r="O40" s="19"/>
-      <c r="P40" s="19"/>
-      <c r="Q40" s="19"/>
-      <c r="R40" s="19"/>
-      <c r="S40" s="19"/>
-      <c r="T40" s="19"/>
-      <c r="U40" s="19"/>
-      <c r="V40" s="19"/>
-      <c r="W40" s="19"/>
-      <c r="X40" s="19"/>
-      <c r="Y40" s="19"/>
-      <c r="Z40" s="19"/>
-      <c r="AA40" s="19"/>
-      <c r="AB40" s="19"/>
-      <c r="AC40" s="19"/>
-      <c r="AD40" s="19"/>
-      <c r="AE40" s="19"/>
-      <c r="AF40" s="19"/>
-      <c r="AG40" s="19"/>
-      <c r="AH40" s="19"/>
-      <c r="AI40" s="19"/>
-      <c r="AJ40" s="19"/>
-      <c r="AK40" s="19"/>
-      <c r="AL40" s="19"/>
-      <c r="AM40" s="19"/>
-      <c r="AN40" s="19"/>
+        <v>382</v>
+      </c>
     </row>
     <row r="43" spans="1:40">
       <c r="B43" s="12" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
     </row>
     <row r="44" spans="1:40">
       <c r="A44" s="12"/>
       <c r="B44" s="13"/>
       <c r="C44" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
     </row>
     <row r="45" spans="1:40">
       <c r="B45" s="14"/>
       <c r="C45" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
     </row>
     <row r="46" spans="1:40">
       <c r="B46" s="15"/>
       <c r="C46" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
     </row>
     <row r="47" spans="1:40">
       <c r="B47" s="16"/>
       <c r="C47" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
     </row>
     <row r="48" spans="1:40">
       <c r="B48" s="1" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="C48" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>
@@ -8241,32 +6847,84 @@
       <formula>#REF!=N$1</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="N2:AN13 B2:M22 N14:Y14 AA14:AN14 N15:AN21 O22:P22 R22:Y22 AB22:AC22 AE22:AL22 AN22 B23:AN25 V26:AL26 B26:T27 U27 W27:AN27 B28:Y29 AA28:AN29 B30:AN32 B33:Y34 AA33:AN34 B35:AN40 B47">
+    <cfRule type="expression" dxfId="4" priority="57">
+      <formula>$A2=B$1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="U26">
-    <cfRule type="expression" dxfId="4" priority="29">
+    <cfRule type="expression" dxfId="3" priority="29">
       <formula>#REF!=U$1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V27">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>$A27=#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z14 Z29 Z33:Z34">
-    <cfRule type="expression" dxfId="2" priority="50">
+    <cfRule type="expression" dxfId="1" priority="50">
       <formula>$A14=#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z22">
-    <cfRule type="expression" dxfId="1" priority="15">
+    <cfRule type="expression" dxfId="0" priority="15">
       <formula>#REF!=#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B47 N2:AN13 N14:Y14 AA14:AN14 N15:AN21 B2:M22 O22:P22 R22:Y22 AB22:AC22 AE22:AL22 AN22 B23:AN25 V26:AL26 B26:T27 U27 B28:Y29 AA28:AN29 B30:AN32 B33:Y34 AA33:AN34 W27:AN27 B35:AN40">
-    <cfRule type="expression" dxfId="0" priority="57">
-      <formula>$A2=B$1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{190E22E7-7A59-41CD-BCD3-4F2AC304728D}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="37.36328125" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.81640625" customWidth="1"/>
+    <col min="4" max="4" width="20.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>405</v>
+      </c>
+      <c r="B1" t="s">
+        <v>404</v>
+      </c>
+      <c r="C1" t="s">
+        <v>403</v>
+      </c>
+      <c r="D1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="C3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix (transform_data.R) (codebook) changed the definition of birth order to include siblings who are over 18 too
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Vaccine Uptake - R\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D979DE-9EF0-4082-B8A6-7A689E30934C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{374112D8-A43A-4F4C-8518-0ADD8197B2AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1307" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1358" uniqueCount="457">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -497,15 +497,6 @@
     <t xml:space="preserve">The presence of a child of interest in the response </t>
   </si>
   <si>
-    <t>The number of sisters the child of interest has</t>
-  </si>
-  <si>
-    <t>The number of brothers the child of interest has</t>
-  </si>
-  <si>
-    <t>The number of siblings the child of interest has</t>
-  </si>
-  <si>
     <t>The marital status of the child of interest's parents</t>
   </si>
   <si>
@@ -1064,9 +1055,6 @@
     <t>where "x"in child_x_sex corresponds to a value from 1 to 5, sum the number of children that are male and account for the sex of interest (if the child of interest is male) to get the number of brothers that the child of interest has</t>
   </si>
   <si>
-    <t>sum the number of brothers and sisters that the child of interest has</t>
-  </si>
-  <si>
     <t>marital_status</t>
   </si>
   <si>
@@ -1271,12 +1259,6 @@
     <t>The chronological order of the COI's birth in the family</t>
   </si>
   <si>
-    <t>find the child that matches the age of interest e.g. if the age of interest is associated with child_1_age then it is the first child, where x in child_x_age is a value from 1 to 5</t>
-  </si>
-  <si>
-    <t>The position that the COI is in by chronological order of births in their family</t>
-  </si>
-  <si>
     <t>continuous</t>
   </si>
   <si>
@@ -1298,18 +1280,9 @@
     <t>Vaccine uptake varies based on 3 different categories, can we leave it as a standalone variable</t>
   </si>
   <si>
-    <t xml:space="preserve">unmarried have a lower mean income </t>
-  </si>
-  <si>
     <t>single parent households have a lower income (mean category 6.9 vs 9.8)</t>
   </si>
   <si>
-    <t>interaction variables</t>
-  </si>
-  <si>
-    <t>variable</t>
-  </si>
-  <si>
     <t>Relationship</t>
   </si>
   <si>
@@ -1368,13 +1341,136 @@
   </si>
   <si>
     <t>JPY</t>
+  </si>
+  <si>
+    <t>unmarried have a lower mean income (4.6 M JPY/Y vs 7.6 M JPY/Y)</t>
+  </si>
+  <si>
+    <t>almost no mothers stay home if they're divorced vs ~25% stay home if they’re married</t>
+  </si>
+  <si>
+    <t>mean household size increases with marriage (3.2 v 3.9)</t>
+  </si>
+  <si>
+    <t>children with married parents have 2 parents and vice versa</t>
+  </si>
+  <si>
+    <t>siblings = -(income)^2</t>
+  </si>
+  <si>
+    <t>parents highest education doesn't impact the proportion of mothers who stay home (26% to 33%)</t>
+  </si>
+  <si>
+    <t>mean size doesn't change but more highsch/junior high have larger families (&gt;= 5)</t>
+  </si>
+  <si>
+    <t>mean no of siblings inversley proportional to parents education</t>
+  </si>
+  <si>
+    <t xml:space="preserve">income isn't related with the number of grandparents </t>
+  </si>
+  <si>
+    <t>fathers (more so) and mothers being in healthcare are predictive of more recent covid vccinations</t>
+  </si>
+  <si>
+    <t>fathers (more) and mothers in healthcare are much more likely to get the influenza vaccine</t>
+  </si>
+  <si>
+    <t>parents in healthcare received a greater number of doses of the covid vaccine (3.5 vs 2.6)</t>
+  </si>
+  <si>
+    <t>parents in healthcare harbour less negative sentiments toward the covid vaccine</t>
+  </si>
+  <si>
+    <t>a more recen t covid vaccination is associated with having obtained more doses of the vaccine</t>
+  </si>
+  <si>
+    <t>having a parent with chronic illness isn't assocaited with vulnerable individuals</t>
+  </si>
+  <si>
+    <t>fathers and mothers with chronic illnesses were more likely to have the influenza vaccine</t>
+  </si>
+  <si>
+    <t>parents without a chronic illnes were more opposed (5) to getting the covid vaccine, all else is equal</t>
+  </si>
+  <si>
+    <t>being unmarried is associated with current chronic illness</t>
+  </si>
+  <si>
+    <t>mothers staying home is associated with lower income</t>
+  </si>
+  <si>
+    <t>no stay-home mum is associated with more grandparents at home (6.8 %  vs 3.6%)</t>
+  </si>
+  <si>
+    <t>the age of children of single fathers Is much higher</t>
+  </si>
+  <si>
+    <t>postgrad (11) &gt; tertiary (8.2) &gt; JC (6.8) &gt;= HS (6.2)</t>
+  </si>
+  <si>
+    <t>postgrad (9.8) &gt; tertiary (8.0) &gt; JC (6.3) &gt;= HS (6.2)</t>
+  </si>
+  <si>
+    <t>postgrad (9.7) &gt; tertiary (8) &gt; JC (6) &gt; HS  (5.8)</t>
+  </si>
+  <si>
+    <t>A higher educational attainment by mothers results in a greater increase in mean annual household income vs the equivalent educational attainment by fathers</t>
+  </si>
+  <si>
+    <t>Mothers of single parent children are more likely to have a lower educational attainment (JC and HS)</t>
+  </si>
+  <si>
+    <t>The household income is more in line with the income levels as provided by the fathers highest educational level</t>
+  </si>
+  <si>
+    <t>variable (###)</t>
+  </si>
+  <si>
+    <t>interaction variables (####)</t>
+  </si>
+  <si>
+    <t>education</t>
+  </si>
+  <si>
+    <t>The proportion of married mothers who stay home decreases as the mother's educational attainment increases whilst the proportion of unmarried mothers who stay home stay low regardless of educational attainment</t>
+  </si>
+  <si>
+    <t>find the child that matches the age of interest e.g. if the age of interest is associated with child_1_age then it is the first child, where x in child_x_age is a value from 1 to 5. And then, add the number of children over 18</t>
+  </si>
+  <si>
+    <t>children_over_18</t>
+  </si>
+  <si>
+    <t>sum the number of brothers and sisters (&lt;18 Y/o) that the child of interest has</t>
+  </si>
+  <si>
+    <t>The position that the COI is in by chronological order of births in their family (for children both under and over 18)</t>
+  </si>
+  <si>
+    <t>The number of siblings (&lt;18y/o) the child of interest has</t>
+  </si>
+  <si>
+    <t>The number of sisters (&lt;18 y/o) the child of interest has</t>
+  </si>
+  <si>
+    <t>The number of brothers (&lt; 18 y/o) the child of interest has</t>
+  </si>
+  <si>
+    <t>The number of siblings (&lt;18y.o) that the child of interest has</t>
+  </si>
+  <si>
+    <t>The number of brothers (&lt; 18y.o) that the child of interest has</t>
+  </si>
+  <si>
+    <t>The number of sisters (&lt;18 y.o) that the child of interest has</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1416,6 +1512,12 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1495,7 +1597,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1534,11 +1636,30 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <color theme="2" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="2" tint="-0.24994659260841701"/>
@@ -1919,8 +2040,11 @@
     <col min="21" max="21" width="25.453125" bestFit="1" customWidth="1"/>
     <col min="22" max="24" width="24.90625" bestFit="1" customWidth="1"/>
     <col min="25" max="56" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="57" max="64" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="65" max="67" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="57" max="63" width="35.81640625" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="35.81640625" style="25" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="35.81640625" style="23" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="68" max="68" width="35.81640625" style="13" bestFit="1" customWidth="1"/>
     <col min="69" max="69" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="70" max="72" width="35.81640625" bestFit="1" customWidth="1"/>
@@ -1972,7 +2096,7 @@
         <v>15</v>
       </c>
       <c r="M1" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="N1" t="s">
         <v>17</v>
@@ -2124,13 +2248,13 @@
       <c r="BK1" t="s">
         <v>66</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BL1" s="25" t="s">
         <v>67</v>
       </c>
       <c r="BM1" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="BN1" s="4" t="s">
+      <c r="BN1" s="23" t="s">
         <v>69</v>
       </c>
       <c r="BO1" s="4" t="s">
@@ -2188,10 +2312,10 @@
         <v>87</v>
       </c>
       <c r="CG1" s="6" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="CH1" s="6" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="CI1" s="8" t="s">
         <v>88</v>
@@ -2409,13 +2533,13 @@
       <c r="BK2" t="s">
         <v>96</v>
       </c>
-      <c r="BL2" t="s">
+      <c r="BL2" s="25" t="s">
         <v>96</v>
       </c>
       <c r="BM2" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="BN2" s="4" t="s">
+      <c r="BN2" s="23" t="s">
         <v>96</v>
       </c>
       <c r="BO2" s="4" t="s">
@@ -2542,7 +2666,7 @@
         <v>117</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>393</v>
+        <v>450</v>
       </c>
       <c r="N3" s="2" t="s">
         <v>118</v>
@@ -2630,87 +2754,87 @@
       <c r="BK3" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="BL3" s="2" t="s">
+      <c r="BL3" s="26" t="s">
+        <v>452</v>
+      </c>
+      <c r="BM3" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="BN3" s="24" t="s">
+        <v>451</v>
+      </c>
+      <c r="BO3" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="BM3" s="3" t="s">
+      <c r="BP3" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="BN3" s="3" t="s">
+      <c r="BQ3" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="BO3" s="3" t="s">
+      <c r="BR3" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="BP3" s="17" t="s">
+      <c r="BS3" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="BQ3" s="3" t="s">
+      <c r="BT3" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="BR3" s="2" t="s">
+      <c r="BU3" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="BS3" s="2" t="s">
+      <c r="BW3" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="BT3" s="2" t="s">
+      <c r="BX3" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="BU3" s="3" t="s">
+      <c r="BY3" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="BW3" s="2" t="s">
+      <c r="BZ3" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="BX3" s="2" t="s">
+      <c r="CA3" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="BY3" s="2" t="s">
+      <c r="CB3" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="BZ3" s="3" t="s">
+      <c r="CC3" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="CA3" s="3" t="s">
+      <c r="CD3" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="CB3" s="3" t="s">
+      <c r="CE3" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="CC3" s="2" t="s">
+      <c r="CF3" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="CD3" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="CE3" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="CF3" s="2" t="s">
-        <v>153</v>
-      </c>
       <c r="CG3" s="5" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="CH3" s="5" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="CI3" s="7"/>
       <c r="CJ3" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="CK3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="CL3" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="CM3" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="CK3" s="2" t="s">
+      <c r="CN3" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="CL3" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="CM3" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="CN3" s="2" t="s">
-        <v>158</v>
       </c>
       <c r="CO3" s="7"/>
       <c r="CP3" s="7"/>
@@ -2905,13 +3029,13 @@
       <c r="BK4" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="BL4" t="s">
+      <c r="BL4" s="25" t="s">
         <v>98</v>
       </c>
       <c r="BM4" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="BN4" s="4" t="s">
+      <c r="BN4" s="23" t="s">
         <v>98</v>
       </c>
       <c r="BO4" s="4" t="s">
@@ -2933,10 +3057,10 @@
         <v>100</v>
       </c>
       <c r="BU4" s="4" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="BV4" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="BW4" t="s">
         <v>99</v>
@@ -3099,20 +3223,20 @@
       <c r="BI7" t="s">
         <v>109</v>
       </c>
-      <c r="BL7" t="s">
+      <c r="BL7" s="25" t="s">
         <v>109</v>
       </c>
       <c r="BM7" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="BN7" s="4" t="s">
+      <c r="BN7" s="23" t="s">
         <v>109</v>
       </c>
       <c r="BT7" t="s">
         <v>108</v>
       </c>
       <c r="BU7" s="4" t="s">
-        <v>424</v>
+        <v>415</v>
       </c>
       <c r="CO7" s="8"/>
       <c r="CP7" s="8"/>
@@ -3159,37 +3283,37 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>270</v>
-      </c>
       <c r="M1" s="1" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="2" spans="1:16">
@@ -3200,34 +3324,34 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -3247,19 +3371,19 @@
         <v>102</v>
       </c>
       <c r="F3" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="G3" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="H3" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="I3" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="J3" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -3279,19 +3403,19 @@
         <v>104</v>
       </c>
       <c r="F4" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="G4" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="H4" t="s">
+        <v>275</v>
+      </c>
+      <c r="I4" t="s">
         <v>278</v>
       </c>
-      <c r="I4" t="s">
-        <v>281</v>
-      </c>
       <c r="J4" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -3311,19 +3435,19 @@
         <v>105</v>
       </c>
       <c r="F5" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="G5" t="s">
+        <v>272</v>
+      </c>
+      <c r="H5" t="s">
         <v>275</v>
       </c>
-      <c r="H5" t="s">
-        <v>278</v>
-      </c>
       <c r="I5" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="J5" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -3343,19 +3467,19 @@
         <v>110</v>
       </c>
       <c r="F6" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="G6" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="H6" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="I6" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="J6" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -3375,19 +3499,19 @@
         <v>111</v>
       </c>
       <c r="F7" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="G7" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="H7" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="I7" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="J7" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="8" spans="1:16">
@@ -3398,7 +3522,7 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D8" t="s">
         <v>108</v>
@@ -3407,19 +3531,19 @@
         <v>112</v>
       </c>
       <c r="F8" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="G8" t="s">
         <v>5</v>
       </c>
       <c r="H8" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="I8" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="J8" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -3430,7 +3554,7 @@
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D9" t="s">
         <v>108</v>
@@ -3439,19 +3563,19 @@
         <v>113</v>
       </c>
       <c r="F9" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="G9" t="s">
         <v>6</v>
       </c>
       <c r="H9" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="I9" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="J9" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -3462,7 +3586,7 @@
         <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D10" t="s">
         <v>108</v>
@@ -3471,19 +3595,19 @@
         <v>114</v>
       </c>
       <c r="F10" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="G10" t="s">
         <v>7</v>
       </c>
       <c r="H10" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="I10" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="J10" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -3494,7 +3618,7 @@
         <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D11" t="s">
         <v>108</v>
@@ -3503,19 +3627,19 @@
         <v>115</v>
       </c>
       <c r="F11" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="G11" t="s">
         <v>8</v>
       </c>
       <c r="H11" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="I11" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="J11" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -3526,7 +3650,7 @@
         <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D12" t="s">
         <v>108</v>
@@ -3535,19 +3659,19 @@
         <v>116</v>
       </c>
       <c r="F12" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="G12" t="s">
         <v>9</v>
       </c>
       <c r="H12" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="I12" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="J12" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13" spans="1:16">
@@ -3558,22 +3682,22 @@
         <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D13" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E13" t="s">
         <v>117</v>
       </c>
       <c r="F13" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="G13" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="H13" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="14" spans="1:16">
@@ -3581,25 +3705,31 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="C14" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D14" t="s">
         <v>109</v>
       </c>
       <c r="E14" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="F14" t="s">
-        <v>392</v>
+        <v>447</v>
       </c>
       <c r="G14" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="H14" t="s">
-        <v>278</v>
+        <v>275</v>
+      </c>
+      <c r="I14" t="s">
+        <v>448</v>
+      </c>
+      <c r="J14" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="15" spans="1:16">
@@ -3619,19 +3749,19 @@
         <v>118</v>
       </c>
       <c r="F15" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="G15" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="H15" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="I15" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="J15" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="16" spans="1:16">
@@ -3651,19 +3781,19 @@
         <v>119</v>
       </c>
       <c r="F16" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="G16" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="H16" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="I16" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="J16" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -3683,19 +3813,19 @@
         <v>120</v>
       </c>
       <c r="F17" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="G17" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="H17" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="I17" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="J17" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -3706,34 +3836,34 @@
         <v>20</v>
       </c>
       <c r="C18" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D18">
         <v>0</v>
       </c>
       <c r="E18" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="F18" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="G18" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="H18" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="I18" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="J18" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="K18" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="L18" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -3744,7 +3874,7 @@
         <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -3755,7 +3885,7 @@
         <v>2</v>
       </c>
       <c r="E20" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -3766,7 +3896,7 @@
         <v>3</v>
       </c>
       <c r="E21" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -3774,10 +3904,10 @@
         <v>22</v>
       </c>
       <c r="D22" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E22" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" spans="1:14">
@@ -3788,16 +3918,16 @@
         <v>21</v>
       </c>
       <c r="C23" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D23">
         <v>0</v>
       </c>
       <c r="E23" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="F23" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="G23" t="s">
         <v>15</v>
@@ -3806,22 +3936,22 @@
         <v>16</v>
       </c>
       <c r="I23" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="J23" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="K23" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="L23" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="M23" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="N23" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="24" spans="1:14">
@@ -3832,7 +3962,7 @@
         <v>1</v>
       </c>
       <c r="E24" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:14">
@@ -3843,7 +3973,7 @@
         <v>2</v>
       </c>
       <c r="E25" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -3851,10 +3981,10 @@
         <v>22</v>
       </c>
       <c r="D26" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E26" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="27" spans="1:14">
@@ -3874,19 +4004,19 @@
         <v>122</v>
       </c>
       <c r="F27" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="G27" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="H27" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="I27" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="J27" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -3906,19 +4036,19 @@
         <v>123</v>
       </c>
       <c r="F28" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="G28" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="H28" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="I28" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="J28" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -3929,34 +4059,34 @@
         <v>25</v>
       </c>
       <c r="C29" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D29">
         <v>0</v>
       </c>
       <c r="E29" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="F29" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="G29" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="H29" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="I29" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="J29" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="K29" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="L29" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -3967,7 +4097,7 @@
         <v>1</v>
       </c>
       <c r="E30" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -3978,7 +4108,7 @@
         <v>2</v>
       </c>
       <c r="E31" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -3986,10 +4116,10 @@
         <v>27</v>
       </c>
       <c r="D32" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E32" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -4000,16 +4130,16 @@
         <v>26</v>
       </c>
       <c r="C33" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D33">
         <v>0</v>
       </c>
       <c r="E33" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="F33" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="G33" t="s">
         <v>15</v>
@@ -4018,22 +4148,22 @@
         <v>16</v>
       </c>
       <c r="I33" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="J33" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="K33" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="L33" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="M33" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="N33" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -4044,7 +4174,7 @@
         <v>1</v>
       </c>
       <c r="E34" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -4055,7 +4185,7 @@
         <v>2</v>
       </c>
       <c r="E35" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -4063,10 +4193,10 @@
         <v>27</v>
       </c>
       <c r="D36" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E36" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -4077,7 +4207,7 @@
         <v>60</v>
       </c>
       <c r="C37" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D37" t="s">
         <v>109</v>
@@ -4086,13 +4216,13 @@
         <v>127</v>
       </c>
       <c r="F37" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="G37" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="H37" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -4103,7 +4233,7 @@
         <v>61</v>
       </c>
       <c r="C38" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D38" t="s">
         <v>109</v>
@@ -4112,13 +4242,13 @@
         <v>128</v>
       </c>
       <c r="F38" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="G38" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="H38" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -4129,7 +4259,7 @@
         <v>62</v>
       </c>
       <c r="C39" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D39" t="s">
         <v>109</v>
@@ -4138,25 +4268,25 @@
         <v>129</v>
       </c>
       <c r="F39" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="G39" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="H39" t="s">
+        <v>307</v>
+      </c>
+      <c r="I39" t="s">
         <v>310</v>
       </c>
-      <c r="I39" t="s">
-        <v>313</v>
-      </c>
       <c r="J39" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K39" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="L39" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -4167,7 +4297,7 @@
         <v>63</v>
       </c>
       <c r="C40" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D40" t="s">
         <v>109</v>
@@ -4176,13 +4306,13 @@
         <v>130</v>
       </c>
       <c r="F40" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="G40" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="H40" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -4193,7 +4323,7 @@
         <v>64</v>
       </c>
       <c r="C41" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D41" t="s">
         <v>109</v>
@@ -4202,19 +4332,19 @@
         <v>131</v>
       </c>
       <c r="F41" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="G41" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="H41" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I41" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="J41" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -4225,25 +4355,25 @@
         <v>65</v>
       </c>
       <c r="C42" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D42">
         <v>0</v>
       </c>
       <c r="E42" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="F42" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="G42" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="H42" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I42" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="J42" t="s">
         <v>16</v>
@@ -4263,7 +4393,7 @@
         <v>1</v>
       </c>
       <c r="E43" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -4271,10 +4401,10 @@
         <v>96</v>
       </c>
       <c r="D44" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E44" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -4285,22 +4415,22 @@
         <v>66</v>
       </c>
       <c r="C45" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D45">
         <v>0</v>
       </c>
       <c r="E45" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F45" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="G45" t="s">
         <v>65</v>
       </c>
       <c r="H45" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -4311,7 +4441,7 @@
         <v>1</v>
       </c>
       <c r="E46" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="47" spans="1:14" s="4" customFormat="1">
@@ -4322,25 +4452,28 @@
         <v>67</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D47" s="4" t="s">
         <v>109</v>
       </c>
+      <c r="E47" s="4" t="s">
+        <v>455</v>
+      </c>
       <c r="F47" s="4" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I47" s="4" t="s">
         <v>65</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="48" spans="1:14" s="4" customFormat="1">
@@ -4351,25 +4484,28 @@
         <v>68</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>109</v>
       </c>
+      <c r="E48" s="4" t="s">
+        <v>456</v>
+      </c>
       <c r="F48" s="4" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I48" s="4" t="s">
         <v>65</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -4380,25 +4516,28 @@
         <v>69</v>
       </c>
       <c r="C49" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D49" t="s">
         <v>109</v>
       </c>
+      <c r="E49" t="s">
+        <v>454</v>
+      </c>
       <c r="F49" t="s">
-        <v>323</v>
+        <v>449</v>
       </c>
       <c r="G49" t="s">
         <v>68</v>
       </c>
       <c r="H49" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I49" t="s">
         <v>67</v>
       </c>
       <c r="J49" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="50" spans="1:13" s="4" customFormat="1">
@@ -4409,25 +4548,25 @@
         <v>70</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D50" s="4">
         <v>0</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="G50" s="4" t="s">
         <v>66</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
     </row>
     <row r="51" spans="1:13" s="4" customFormat="1">
@@ -4438,7 +4577,7 @@
         <v>1</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="52" spans="1:13" s="4" customFormat="1">
@@ -4449,7 +4588,7 @@
         <v>2</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="53" spans="1:13" s="4" customFormat="1">
@@ -4460,7 +4599,7 @@
         <v>3</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="54" spans="1:13" s="4" customFormat="1">
@@ -4468,10 +4607,10 @@
         <v>96</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -4482,25 +4621,25 @@
         <v>71</v>
       </c>
       <c r="C55" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D55">
         <v>0</v>
       </c>
       <c r="E55" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="F55" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="G55" t="s">
         <v>66</v>
       </c>
       <c r="H55" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I55" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -4511,7 +4650,7 @@
         <v>1</v>
       </c>
       <c r="E56" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -4519,10 +4658,10 @@
         <v>96</v>
       </c>
       <c r="D57" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E57" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="58" spans="1:13">
@@ -4533,22 +4672,22 @@
         <v>73</v>
       </c>
       <c r="C58" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D58">
         <v>0</v>
       </c>
       <c r="E58" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="F58" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="G58" t="s">
         <v>58</v>
       </c>
       <c r="H58" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="59" spans="1:13">
@@ -4559,7 +4698,7 @@
         <v>1</v>
       </c>
       <c r="E59" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="60" spans="1:13">
@@ -4567,10 +4706,10 @@
         <v>96</v>
       </c>
       <c r="D60" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E60" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="61" spans="1:13">
@@ -4581,34 +4720,34 @@
         <v>74</v>
       </c>
       <c r="C61" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D61">
         <v>0</v>
       </c>
       <c r="E61" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="G61" s="11" t="s">
         <v>73</v>
       </c>
       <c r="H61" s="11" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I61" s="11" t="s">
         <v>70</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>60</v>
       </c>
       <c r="L61" s="11" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="M61" s="11"/>
     </row>
@@ -4620,7 +4759,7 @@
         <v>1</v>
       </c>
       <c r="E62" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="63" spans="1:13">
@@ -4628,10 +4767,10 @@
         <v>96</v>
       </c>
       <c r="D63" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E63" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -4642,19 +4781,19 @@
         <v>75</v>
       </c>
       <c r="C64" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D64" t="s">
         <v>108</v>
       </c>
       <c r="F64" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="G64" t="s">
         <v>59</v>
       </c>
       <c r="H64" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="65" spans="1:8" s="4" customFormat="1">
@@ -4665,22 +4804,22 @@
         <v>76</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D65" s="4">
         <v>1</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="66" spans="1:8" s="4" customFormat="1">
@@ -4691,7 +4830,7 @@
         <v>2</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="67" spans="1:8" s="4" customFormat="1">
@@ -4702,7 +4841,7 @@
         <v>3</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="68" spans="1:8" s="4" customFormat="1">
@@ -4713,7 +4852,7 @@
         <v>4</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="69" spans="1:8" s="4" customFormat="1">
@@ -4724,7 +4863,7 @@
         <v>5</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="70" spans="1:8" s="4" customFormat="1">
@@ -4735,7 +4874,7 @@
         <v>6</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="71" spans="1:8" s="4" customFormat="1">
@@ -4746,7 +4885,7 @@
         <v>7</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="72" spans="1:8" s="4" customFormat="1">
@@ -4757,7 +4896,7 @@
         <v>8</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="73" spans="1:8" s="4" customFormat="1">
@@ -4768,7 +4907,7 @@
         <v>9</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="74" spans="1:8" s="4" customFormat="1">
@@ -4779,7 +4918,7 @@
         <v>10</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="75" spans="1:8" s="4" customFormat="1">
@@ -4790,7 +4929,7 @@
         <v>11</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="76" spans="1:8" s="4" customFormat="1">
@@ -4801,7 +4940,7 @@
         <v>12</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="77" spans="1:8" s="4" customFormat="1">
@@ -4812,7 +4951,7 @@
         <v>13</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="78" spans="1:8" s="4" customFormat="1">
@@ -4820,10 +4959,10 @@
         <v>96</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="79" spans="1:8">
@@ -4834,22 +4973,22 @@
         <v>77</v>
       </c>
       <c r="C79" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D79">
         <v>1</v>
       </c>
       <c r="E79" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="F79" t="s">
-        <v>423</v>
+        <v>414</v>
       </c>
       <c r="G79" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="H79" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="80" spans="1:8">
@@ -4861,7 +5000,7 @@
         <v>2</v>
       </c>
       <c r="E80" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -4873,7 +5012,7 @@
         <v>3</v>
       </c>
       <c r="E81" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -4885,7 +5024,7 @@
         <v>4</v>
       </c>
       <c r="E82" t="s">
-        <v>408</v>
+        <v>399</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -4897,7 +5036,7 @@
         <v>5</v>
       </c>
       <c r="E83" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -4909,7 +5048,7 @@
         <v>6</v>
       </c>
       <c r="E84" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -4921,7 +5060,7 @@
         <v>7</v>
       </c>
       <c r="E85" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -4933,7 +5072,7 @@
         <v>8</v>
       </c>
       <c r="E86" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -4945,7 +5084,7 @@
         <v>9</v>
       </c>
       <c r="E87" t="s">
-        <v>414</v>
+        <v>405</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -4957,7 +5096,7 @@
         <v>10</v>
       </c>
       <c r="E88" t="s">
-        <v>415</v>
+        <v>406</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -4969,7 +5108,7 @@
         <v>11</v>
       </c>
       <c r="E89" t="s">
-        <v>416</v>
+        <v>407</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -4981,7 +5120,7 @@
         <v>12</v>
       </c>
       <c r="E90" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -4993,7 +5132,7 @@
         <v>13</v>
       </c>
       <c r="E91" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -5005,7 +5144,7 @@
         <v>14</v>
       </c>
       <c r="E92" t="s">
-        <v>419</v>
+        <v>410</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -5017,7 +5156,7 @@
         <v>15</v>
       </c>
       <c r="E93" s="21" t="s">
-        <v>421</v>
+        <v>412</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -5029,7 +5168,7 @@
         <v>16</v>
       </c>
       <c r="E94" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -5041,7 +5180,7 @@
         <v>17</v>
       </c>
       <c r="E95" t="s">
-        <v>422</v>
+        <v>413</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -5053,7 +5192,7 @@
         <v>18</v>
       </c>
       <c r="E96" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="97" spans="1:17">
@@ -5061,10 +5200,10 @@
         <v>96</v>
       </c>
       <c r="D97" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E97" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="98" spans="1:17">
@@ -5075,25 +5214,25 @@
         <v>78</v>
       </c>
       <c r="C98" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D98">
         <v>0</v>
       </c>
       <c r="E98" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="F98" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="G98" t="s">
         <v>66</v>
       </c>
       <c r="H98" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I98" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
     </row>
     <row r="99" spans="1:17">
@@ -5104,7 +5243,7 @@
         <v>1</v>
       </c>
       <c r="E99" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="100" spans="1:17">
@@ -5115,7 +5254,7 @@
         <v>2</v>
       </c>
       <c r="E100" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="101" spans="1:17">
@@ -5123,10 +5262,10 @@
         <v>96</v>
       </c>
       <c r="D101" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E101" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="102" spans="1:17">
@@ -5137,46 +5276,46 @@
         <v>79</v>
       </c>
       <c r="C102" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D102">
         <v>0</v>
       </c>
       <c r="E102" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F102" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="G102" t="s">
         <v>66</v>
       </c>
       <c r="H102" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I102" t="s">
         <v>73</v>
       </c>
       <c r="J102" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K102" t="s">
         <v>74</v>
       </c>
       <c r="L102" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="M102" t="s">
         <v>48</v>
       </c>
       <c r="N102" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="O102" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="P102" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="103" spans="1:17">
@@ -5187,7 +5326,7 @@
         <v>1</v>
       </c>
       <c r="E103" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="104" spans="1:17">
@@ -5198,7 +5337,7 @@
         <v>2</v>
       </c>
       <c r="E104" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="105" spans="1:17">
@@ -5209,7 +5348,7 @@
         <v>3</v>
       </c>
       <c r="E105" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="106" spans="1:17">
@@ -5217,10 +5356,10 @@
         <v>96</v>
       </c>
       <c r="D106" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E106" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="107" spans="1:17">
@@ -5231,46 +5370,46 @@
         <v>80</v>
       </c>
       <c r="C107" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D107">
         <v>0</v>
       </c>
       <c r="E107" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F107" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="G107" t="s">
         <v>66</v>
       </c>
       <c r="H107" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I107" t="s">
         <v>73</v>
       </c>
       <c r="J107" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K107" t="s">
         <v>74</v>
       </c>
       <c r="L107" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="M107" t="s">
         <v>48</v>
       </c>
       <c r="N107" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="O107" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="P107" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="108" spans="1:17">
@@ -5281,7 +5420,7 @@
         <v>1</v>
       </c>
       <c r="E108" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="109" spans="1:17">
@@ -5292,7 +5431,7 @@
         <v>2</v>
       </c>
       <c r="E109" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="110" spans="1:17">
@@ -5303,7 +5442,7 @@
         <v>3</v>
       </c>
       <c r="E110" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="111" spans="1:17" s="6" customFormat="1">
@@ -5313,10 +5452,10 @@
       <c r="B111"/>
       <c r="C111"/>
       <c r="D111" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E111" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F111"/>
       <c r="G111"/>
@@ -5339,46 +5478,46 @@
         <v>81</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D112" s="4">
         <v>0</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="G112" s="4" t="s">
         <v>66</v>
       </c>
       <c r="H112" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I112" s="4" t="s">
         <v>73</v>
       </c>
       <c r="J112" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K112" s="4" t="s">
         <v>74</v>
       </c>
       <c r="L112" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="M112" s="4" t="s">
         <v>48</v>
       </c>
       <c r="N112" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="O112" s="4" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="P112" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="113" spans="1:16" s="4" customFormat="1">
@@ -5389,7 +5528,7 @@
         <v>1</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="114" spans="1:16" s="4" customFormat="1">
@@ -5400,7 +5539,7 @@
         <v>2</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
     </row>
     <row r="115" spans="1:16" s="4" customFormat="1">
@@ -5411,7 +5550,7 @@
         <v>3</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="116" spans="1:16" s="4" customFormat="1">
@@ -5419,10 +5558,10 @@
         <v>96</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="117" spans="1:16" s="4" customFormat="1">
@@ -5433,46 +5572,46 @@
         <v>82</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D117" s="4">
         <v>0</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="G117" s="4" t="s">
         <v>66</v>
       </c>
       <c r="H117" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I117" s="4" t="s">
         <v>73</v>
       </c>
       <c r="J117" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K117" s="4" t="s">
         <v>74</v>
       </c>
       <c r="L117" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="M117" s="4" t="s">
         <v>48</v>
       </c>
       <c r="N117" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="O117" s="4" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="P117" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="118" spans="1:16" s="4" customFormat="1">
@@ -5483,7 +5622,7 @@
         <v>1</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="119" spans="1:16" s="4" customFormat="1">
@@ -5494,7 +5633,7 @@
         <v>2</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="120" spans="1:16" s="4" customFormat="1">
@@ -5505,7 +5644,7 @@
         <v>3</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="121" spans="1:16" s="4" customFormat="1">
@@ -5513,10 +5652,10 @@
         <v>96</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="122" spans="1:16" s="4" customFormat="1">
@@ -5527,46 +5666,46 @@
         <v>83</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D122" s="4">
         <v>0</v>
       </c>
       <c r="E122" s="4" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="G122" s="4" t="s">
         <v>66</v>
       </c>
       <c r="H122" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I122" s="4" t="s">
         <v>73</v>
       </c>
       <c r="J122" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K122" s="4" t="s">
         <v>74</v>
       </c>
       <c r="L122" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="M122" s="4" t="s">
         <v>48</v>
       </c>
       <c r="N122" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="O122" s="4" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="P122" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="123" spans="1:16" s="4" customFormat="1">
@@ -5577,7 +5716,7 @@
         <v>1</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="124" spans="1:16" s="4" customFormat="1">
@@ -5588,7 +5727,7 @@
         <v>2</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="125" spans="1:16" s="4" customFormat="1">
@@ -5599,7 +5738,7 @@
         <v>3</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="126" spans="1:16" s="4" customFormat="1">
@@ -5607,10 +5746,10 @@
         <v>96</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="127" spans="1:16">
@@ -5621,46 +5760,46 @@
         <v>84</v>
       </c>
       <c r="C127" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D127">
         <v>0</v>
       </c>
       <c r="E127" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="F127" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="G127" t="s">
         <v>66</v>
       </c>
       <c r="H127" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I127" t="s">
         <v>73</v>
       </c>
       <c r="J127" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K127" t="s">
         <v>74</v>
       </c>
       <c r="L127" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="M127" t="s">
         <v>48</v>
       </c>
       <c r="N127" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="O127" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="P127" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="128" spans="1:16">
@@ -5671,7 +5810,7 @@
         <v>1</v>
       </c>
       <c r="E128" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="129" spans="1:16">
@@ -5679,10 +5818,10 @@
         <v>96</v>
       </c>
       <c r="D129" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E129" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="130" spans="1:16">
@@ -5693,46 +5832,46 @@
         <v>85</v>
       </c>
       <c r="C130" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D130">
         <v>0</v>
       </c>
       <c r="E130" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="F130" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="G130" t="s">
         <v>66</v>
       </c>
       <c r="H130" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I130" t="s">
         <v>73</v>
       </c>
       <c r="J130" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K130" t="s">
         <v>74</v>
       </c>
       <c r="L130" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="M130" t="s">
         <v>48</v>
       </c>
       <c r="N130" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="O130" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="P130" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="131" spans="1:16">
@@ -5743,7 +5882,7 @@
         <v>1</v>
       </c>
       <c r="E131" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="132" spans="1:16">
@@ -5754,7 +5893,7 @@
         <v>2</v>
       </c>
       <c r="E132" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="133" spans="1:16">
@@ -5762,10 +5901,10 @@
         <v>96</v>
       </c>
       <c r="D133" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E133" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="134" spans="1:16">
@@ -5776,46 +5915,46 @@
         <v>86</v>
       </c>
       <c r="C134" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D134">
         <v>0</v>
       </c>
       <c r="E134" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="F134" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="G134" t="s">
         <v>66</v>
       </c>
       <c r="H134" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I134" t="s">
         <v>73</v>
       </c>
       <c r="J134" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K134" t="s">
         <v>74</v>
       </c>
       <c r="L134" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="M134" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="N134" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="O134" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="P134" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="135" spans="1:16">
@@ -5826,7 +5965,7 @@
         <v>1</v>
       </c>
       <c r="E135" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
     </row>
     <row r="136" spans="1:16">
@@ -5837,7 +5976,7 @@
         <v>2</v>
       </c>
       <c r="E136" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="137" spans="1:16">
@@ -5848,7 +5987,7 @@
         <v>3</v>
       </c>
       <c r="E137" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="138" spans="1:16">
@@ -5856,10 +5995,10 @@
         <v>96</v>
       </c>
       <c r="D138" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E138" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="139" spans="1:16">
@@ -5870,46 +6009,46 @@
         <v>87</v>
       </c>
       <c r="C139" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D139">
         <v>0</v>
       </c>
       <c r="E139" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="F139" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="G139" t="s">
         <v>66</v>
       </c>
       <c r="H139" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I139" t="s">
         <v>73</v>
       </c>
       <c r="J139" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K139" t="s">
         <v>74</v>
       </c>
       <c r="L139" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="M139" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="N139" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="O139" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="P139" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="140" spans="1:16">
@@ -5920,7 +6059,7 @@
         <v>1</v>
       </c>
       <c r="E140" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
     </row>
     <row r="141" spans="1:16">
@@ -5931,7 +6070,7 @@
         <v>2</v>
       </c>
       <c r="E141" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="142" spans="1:16">
@@ -5942,7 +6081,7 @@
         <v>3</v>
       </c>
       <c r="E142" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="143" spans="1:16">
@@ -5950,10 +6089,10 @@
         <v>96</v>
       </c>
       <c r="D143" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E143" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="144" spans="1:16">
@@ -5964,34 +6103,34 @@
         <v>89</v>
       </c>
       <c r="C144" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D144">
         <v>0</v>
       </c>
       <c r="E144" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="F144" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="G144" t="s">
         <v>66</v>
       </c>
       <c r="H144" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="I144" t="s">
         <v>86</v>
       </c>
       <c r="J144" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K144" t="s">
         <v>87</v>
       </c>
       <c r="L144" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="145" spans="1:10">
@@ -6002,7 +6141,7 @@
         <v>1</v>
       </c>
       <c r="E145" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
     </row>
     <row r="146" spans="1:10">
@@ -6013,7 +6152,7 @@
         <v>2</v>
       </c>
       <c r="E146" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="147" spans="1:10">
@@ -6024,7 +6163,7 @@
         <v>3</v>
       </c>
       <c r="E147" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="148" spans="1:10">
@@ -6032,10 +6171,10 @@
         <v>96</v>
       </c>
       <c r="D148" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E148" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="149" spans="1:10">
@@ -6046,28 +6185,28 @@
         <v>90</v>
       </c>
       <c r="C149" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D149">
         <v>0</v>
       </c>
       <c r="E149" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="F149" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="G149" t="s">
         <v>66</v>
       </c>
       <c r="H149" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I149" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="J149" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="150" spans="1:10">
@@ -6078,7 +6217,7 @@
         <v>1</v>
       </c>
       <c r="E150" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="151" spans="1:10">
@@ -6086,10 +6225,10 @@
         <v>96</v>
       </c>
       <c r="D151" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E151" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="152" spans="1:10">
@@ -6100,28 +6239,28 @@
         <v>91</v>
       </c>
       <c r="C152" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D152">
         <v>0</v>
       </c>
       <c r="E152" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="F152" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="G152" t="s">
         <v>66</v>
       </c>
       <c r="H152" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I152" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="J152" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="153" spans="1:10">
@@ -6132,7 +6271,7 @@
         <v>1</v>
       </c>
       <c r="E153" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
     </row>
     <row r="154" spans="1:10">
@@ -6143,7 +6282,7 @@
         <v>2</v>
       </c>
       <c r="E154" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="155" spans="1:10">
@@ -6154,7 +6293,7 @@
         <v>3</v>
       </c>
       <c r="E155" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
     </row>
     <row r="156" spans="1:10">
@@ -6165,7 +6304,7 @@
         <v>4</v>
       </c>
       <c r="E156" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="157" spans="1:10">
@@ -6176,7 +6315,7 @@
         <v>5</v>
       </c>
       <c r="E157" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="158" spans="1:10">
@@ -6187,7 +6326,7 @@
         <v>6</v>
       </c>
       <c r="E158" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="159" spans="1:10">
@@ -6198,7 +6337,7 @@
         <v>7</v>
       </c>
       <c r="E159" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="160" spans="1:10">
@@ -6206,10 +6345,10 @@
         <v>96</v>
       </c>
       <c r="D160" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E160" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="161" spans="1:12">
@@ -6220,28 +6359,28 @@
         <v>92</v>
       </c>
       <c r="C161" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D161">
         <v>0</v>
       </c>
       <c r="E161" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F161" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="G161" t="s">
         <v>66</v>
       </c>
       <c r="H161" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I161" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="J161" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="162" spans="1:12">
@@ -6252,7 +6391,7 @@
         <v>1</v>
       </c>
       <c r="E162" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="163" spans="1:12">
@@ -6263,7 +6402,7 @@
         <v>2</v>
       </c>
       <c r="E163" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
     </row>
     <row r="164" spans="1:12">
@@ -6274,7 +6413,7 @@
         <v>3</v>
       </c>
       <c r="E164" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="165" spans="1:12">
@@ -6285,7 +6424,7 @@
         <v>4</v>
       </c>
       <c r="E165" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="166" spans="1:12">
@@ -6296,7 +6435,7 @@
         <v>5</v>
       </c>
       <c r="E166" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="167" spans="1:12">
@@ -6304,10 +6443,10 @@
         <v>96</v>
       </c>
       <c r="D167" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E167" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="168" spans="1:12">
@@ -6318,34 +6457,34 @@
         <v>93</v>
       </c>
       <c r="C168" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D168">
         <v>0</v>
       </c>
       <c r="E168" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="F168" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="G168" t="s">
         <v>66</v>
       </c>
       <c r="H168" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="I168" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="J168" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="K168" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="L168" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="169" spans="1:12">
@@ -6356,7 +6495,7 @@
         <v>1</v>
       </c>
       <c r="E169" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="170" spans="1:12">
@@ -6367,7 +6506,7 @@
         <v>2</v>
       </c>
       <c r="E170" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
     </row>
     <row r="171" spans="1:12">
@@ -6375,10 +6514,10 @@
         <v>96</v>
       </c>
       <c r="D171" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E171" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -6418,7 +6557,7 @@
   <sheetData>
     <row r="1" spans="1:41" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A1" s="18" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>5</v>
@@ -6454,7 +6593,7 @@
         <v>15</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="N1" s="2" t="s">
         <v>60</v>
@@ -6532,13 +6671,13 @@
         <v>93</v>
       </c>
       <c r="AM1" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="AN1" s="2" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="AO1" s="19" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
     </row>
     <row r="2" spans="1:41">
@@ -6597,12 +6736,12 @@
       </c>
       <c r="AN12" s="16"/>
       <c r="AO12" s="11" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
     </row>
     <row r="13" spans="1:41">
       <c r="A13" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="AN13" s="16"/>
     </row>
@@ -6611,8 +6750,8 @@
         <v>60</v>
       </c>
       <c r="R14" s="16"/>
-      <c r="Z14" s="16" t="s">
-        <v>402</v>
+      <c r="Z14" s="20" t="s">
+        <v>395</v>
       </c>
       <c r="AC14" s="16"/>
       <c r="AD14" s="16"/>
@@ -6666,13 +6805,21 @@
       <c r="A22" t="s">
         <v>71</v>
       </c>
-      <c r="N22" s="16"/>
-      <c r="Q22" s="16"/>
+      <c r="N22" s="20" t="s">
+        <v>419</v>
+      </c>
+      <c r="Q22" s="20" t="s">
+        <v>418</v>
+      </c>
       <c r="Z22" s="20" t="s">
-        <v>401</v>
-      </c>
-      <c r="AA22" s="16"/>
-      <c r="AD22" s="16"/>
+        <v>416</v>
+      </c>
+      <c r="AA22" s="20" t="s">
+        <v>433</v>
+      </c>
+      <c r="AD22" s="20" t="s">
+        <v>417</v>
+      </c>
       <c r="AM22" s="16"/>
     </row>
     <row r="23" spans="1:40">
@@ -6689,16 +6836,20 @@
       <c r="A25" t="s">
         <v>75</v>
       </c>
-      <c r="P25" s="16"/>
-      <c r="AA25" s="16"/>
+      <c r="P25" s="22"/>
+      <c r="AA25" s="22"/>
       <c r="AM25" s="16"/>
     </row>
     <row r="26" spans="1:40">
       <c r="A26" t="s">
         <v>77</v>
       </c>
-      <c r="R26" s="16"/>
-      <c r="U26" s="16"/>
+      <c r="R26" s="22" t="s">
+        <v>424</v>
+      </c>
+      <c r="U26" s="20" t="s">
+        <v>420</v>
+      </c>
       <c r="AM26" s="16"/>
       <c r="AN26" s="16"/>
     </row>
@@ -6706,11 +6857,17 @@
       <c r="A27" t="s">
         <v>78</v>
       </c>
-      <c r="P27" s="16"/>
+      <c r="P27" s="22" t="s">
+        <v>430</v>
+      </c>
       <c r="V27" s="16"/>
-      <c r="AI27" s="16"/>
-      <c r="AJ27" s="16"/>
-      <c r="AK27" s="16"/>
+      <c r="AI27" s="20" t="s">
+        <v>431</v>
+      </c>
+      <c r="AJ27" s="22"/>
+      <c r="AK27" s="20" t="s">
+        <v>432</v>
+      </c>
       <c r="AN27" s="16"/>
     </row>
     <row r="28" spans="1:40">
@@ -6727,28 +6884,46 @@
       <c r="R29" s="16"/>
       <c r="Z29" s="16"/>
       <c r="AD29" s="16" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
     </row>
     <row r="30" spans="1:40">
       <c r="A30" t="s">
         <v>84</v>
       </c>
-      <c r="L30" s="16"/>
-      <c r="R30" s="16"/>
-      <c r="Z30" s="16"/>
+      <c r="L30" s="22"/>
+      <c r="R30" s="20" t="s">
+        <v>435</v>
+      </c>
+      <c r="Z30" s="20" t="s">
+        <v>434</v>
+      </c>
     </row>
     <row r="31" spans="1:40">
       <c r="A31" t="s">
         <v>85</v>
       </c>
+      <c r="AI31" s="20" t="s">
+        <v>426</v>
+      </c>
+      <c r="AJ31" s="20" t="s">
+        <v>427</v>
+      </c>
+      <c r="AK31" s="20" t="s">
+        <v>428</v>
+      </c>
+      <c r="AL31" s="20" t="s">
+        <v>425</v>
+      </c>
     </row>
     <row r="32" spans="1:40">
       <c r="A32" t="s">
         <v>86</v>
       </c>
       <c r="U32" s="16"/>
-      <c r="Z32" s="16"/>
+      <c r="Z32" s="20" t="s">
+        <v>438</v>
+      </c>
       <c r="AB32" s="16"/>
       <c r="AH32" s="16"/>
       <c r="AN32" s="16"/>
@@ -6758,15 +6933,29 @@
         <v>87</v>
       </c>
       <c r="U33" s="16"/>
-      <c r="Z33" s="16"/>
+      <c r="Z33" s="20" t="s">
+        <v>437</v>
+      </c>
       <c r="AC33" s="16"/>
       <c r="AD33" s="16"/>
       <c r="AH33" s="16"/>
       <c r="AN33" s="16"/>
     </row>
-    <row r="34" spans="1:40">
+    <row r="34" spans="1:40" ht="14" customHeight="1">
       <c r="A34" t="s">
         <v>89</v>
+      </c>
+      <c r="Q34" s="22" t="s">
+        <v>422</v>
+      </c>
+      <c r="U34" s="20" t="s">
+        <v>423</v>
+      </c>
+      <c r="Z34" s="20" t="s">
+        <v>439</v>
+      </c>
+      <c r="AD34" s="22" t="s">
+        <v>421</v>
       </c>
     </row>
     <row r="35" spans="1:40">
@@ -6791,85 +6980,93 @@
       <c r="A38" t="s">
         <v>93</v>
       </c>
+      <c r="AI38" s="20" t="s">
+        <v>429</v>
+      </c>
       <c r="AN38" s="16"/>
     </row>
     <row r="39" spans="1:40">
       <c r="A39" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
     </row>
     <row r="40" spans="1:40">
       <c r="A40" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
     </row>
     <row r="43" spans="1:40">
       <c r="B43" s="12" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
     </row>
     <row r="44" spans="1:40">
       <c r="A44" s="12"/>
       <c r="B44" s="13"/>
       <c r="C44" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
     </row>
     <row r="45" spans="1:40">
       <c r="B45" s="14"/>
       <c r="C45" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
     </row>
     <row r="46" spans="1:40">
       <c r="B46" s="15"/>
       <c r="C46" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
     </row>
     <row r="47" spans="1:40">
       <c r="B47" s="16"/>
       <c r="C47" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
     </row>
     <row r="48" spans="1:40">
       <c r="B48" s="1" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="C48" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="N22 Q22 AA22 AD22 AM22 AM26:AN26">
-    <cfRule type="expression" dxfId="5" priority="6">
+    <cfRule type="expression" dxfId="6" priority="6">
       <formula>#REF!=N$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:AN13 B2:M22 N14:Y14 AA14:AN14 N15:AN21 O22:P22 R22:Y22 AB22:AC22 AE22:AL22 AN22 B23:AN25 V26:AL26 B26:T27 U27 W27:AN27 B28:Y29 AA28:AN29 B30:AN32 B33:Y34 AA33:AN34 B35:AN40 B47">
-    <cfRule type="expression" dxfId="4" priority="57">
+  <conditionalFormatting sqref="N2:AN13 B2:M22 N14:Y14 AA14:AN14 N15:AN21 O22:P22 R22:Y22 AB22:AC22 AE22:AL22 AN22 B23:AN25 V26:AL26 B26:T27 U27 W27:AN27 B28:Y29 AA28:AN29 B30:AN30 B31:AJ32 AL31:AN32 B33:Y35 AA33:AN35 B36:AN40 B47">
+    <cfRule type="expression" dxfId="5" priority="57">
       <formula>$A2=B$1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U26">
-    <cfRule type="expression" dxfId="3" priority="29">
+    <cfRule type="expression" dxfId="4" priority="29">
       <formula>#REF!=U$1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V27">
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>$A27=#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z14 Z29 Z33:Z34">
-    <cfRule type="expression" dxfId="1" priority="50">
+    <cfRule type="expression" dxfId="2" priority="50">
       <formula>$A14=#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z22">
-    <cfRule type="expression" dxfId="0" priority="15">
+    <cfRule type="expression" dxfId="1" priority="15">
       <formula>#REF!=#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AK31 Z34">
+    <cfRule type="expression" dxfId="0" priority="60">
+      <formula>$A32=Z$1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6879,49 +7076,134 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{190E22E7-7A59-41CD-BCD3-4F2AC304728D}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="B1:F17"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="37.36328125" customWidth="1"/>
-    <col min="2" max="2" width="16.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.81640625" customWidth="1"/>
-    <col min="4" max="4" width="20.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="72.81640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="28.6328125" customWidth="1"/>
+    <col min="4" max="4" width="23.1796875" customWidth="1"/>
+    <col min="5" max="5" width="30.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>405</v>
-      </c>
-      <c r="B1" t="s">
-        <v>404</v>
+    <row r="1" spans="2:6">
+      <c r="B1" s="2" t="s">
+        <v>396</v>
       </c>
       <c r="C1" t="s">
-        <v>403</v>
+        <v>443</v>
       </c>
       <c r="D1" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>406</v>
-      </c>
-      <c r="B2" t="s">
-        <v>76</v>
+        <v>444</v>
+      </c>
+    </row>
+    <row r="2" spans="2:6" ht="29">
+      <c r="B2" s="2" t="s">
+        <v>397</v>
       </c>
       <c r="C2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" t="s">
         <v>60</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="2:6" ht="29">
+      <c r="B3" s="2" t="s">
+        <v>397</v>
+      </c>
       <c r="C3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" t="s">
         <v>70</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" s="11" customFormat="1">
+      <c r="B5" s="19" t="s">
+        <v>436</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="29">
+      <c r="B7" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="29">
+      <c r="B8" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="C8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D8" t="s">
+        <v>87</v>
+      </c>
+      <c r="E8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6">
+      <c r="C9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="29">
+      <c r="B12" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="C12" t="s">
+        <v>87</v>
+      </c>
+      <c r="D12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="43.5">
+      <c r="B17" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="C17" t="s">
+        <v>84</v>
+      </c>
+      <c r="D17" t="s">
+        <v>320</v>
+      </c>
+      <c r="E17" t="s">
+        <v>445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add (03_transform_data.R) (04_exploratory_DAG.qmd) (codebook.xlsx) added an age_cat variable that indicates the child's schooling based on their age at the time of response
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Vaccine Uptake - R\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD065058-854C-480E-8AC9-A2A356E79A5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6915FECE-D1A6-4DC2-BD61-03A4E3D7C71E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
     Remove once we’ve determined how to stratify by disease</t>
       </text>
     </comment>
-    <comment ref="CB1" authorId="1" shapeId="0" xr:uid="{E5BA077E-7025-4391-8B23-A38BD7E65674}">
+    <comment ref="CC1" authorId="1" shapeId="0" xr:uid="{E5BA077E-7025-4391-8B23-A38BD7E65674}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -73,7 +73,7 @@
     <author>tc={869B55B9-3B1F-4453-9A39-E466CC7906FC}</author>
   </authors>
   <commentList>
-    <comment ref="L63" authorId="0" shapeId="0" xr:uid="{869B55B9-3B1F-4453-9A39-E466CC7906FC}">
+    <comment ref="L67" authorId="0" shapeId="0" xr:uid="{869B55B9-3B1F-4453-9A39-E466CC7906FC}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1452" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1480" uniqueCount="517">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -1609,6 +1609,42 @@
   </si>
   <si>
     <t>Taken from transformed_age_data</t>
+  </si>
+  <si>
+    <t>age_cat</t>
+  </si>
+  <si>
+    <t>category of schooling that the COI falls into based on their age as of Apr 2nd 2023</t>
+  </si>
+  <si>
+    <t>pre</t>
+  </si>
+  <si>
+    <t>primary</t>
+  </si>
+  <si>
+    <t>high</t>
+  </si>
+  <si>
+    <t>Child is of the age to be in preschool</t>
+  </si>
+  <si>
+    <t>Child is of the age to be in primary school</t>
+  </si>
+  <si>
+    <t>Child is of the age to be in junior high or high school</t>
+  </si>
+  <si>
+    <t>No COI to derive age and thus age_cat data from</t>
+  </si>
+  <si>
+    <t>child &lt; 6 y/o as of 2nd April 2023</t>
+  </si>
+  <si>
+    <t>child &gt; 6 y/o and &lt; 12 y/o as of 2nd April 2023</t>
+  </si>
+  <si>
+    <t>child &gt; 12 y/o as of 2nd April 2023</t>
   </si>
 </sst>
 </file>
@@ -1763,7 +1799,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1808,7 +1844,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2149,7 +2184,7 @@
   <threadedComment ref="AZ1" dT="2025-04-17T06:44:16.29" personId="{018BAD65-E158-4456-AEB2-B6F599AC9FA9}" id="{F627B11A-9966-4DAF-9CD9-36B5D028D9EE}" done="1">
     <text>Remove once we’ve determined how to stratify by disease</text>
   </threadedComment>
-  <threadedComment ref="CB1" dT="2025-04-17T05:57:08.19" personId="{018BAD65-E158-4456-AEB2-B6F599AC9FA9}" id="{E5BA077E-7025-4391-8B23-A38BD7E65674}" done="1">
+  <threadedComment ref="CC1" dT="2025-04-17T05:57:08.19" personId="{018BAD65-E158-4456-AEB2-B6F599AC9FA9}" id="{E5BA077E-7025-4391-8B23-A38BD7E65674}" done="1">
     <text xml:space="preserve">Remove retired status and student status? (due to the low number of respondents who fall into these categories)
 </text>
   </threadedComment>
@@ -2158,7 +2193,7 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="L63" dT="2025-04-22T08:11:08.78" personId="{018BAD65-E158-4456-AEB2-B6F599AC9FA9}" id="{869B55B9-3B1F-4453-9A39-E466CC7906FC}">
+  <threadedComment ref="L67" dT="2025-04-22T08:11:08.78" personId="{018BAD65-E158-4456-AEB2-B6F599AC9FA9}" id="{869B55B9-3B1F-4453-9A39-E466CC7906FC}">
     <text xml:space="preserve">How should we define the number of parents a child has, the numebr of spouses livignin the same household? Or the marital status of the responding parent
 there are cases where parents = 1 but the responding parent is still married, and in such cases where the other parent isn’t living in the same hosuehold as them they still may have an influence on their childs’vaccination
 cases where parents = 2 but they arent married, i.e. divorced both parents might still have a say in the child’s vaccination
@@ -2169,7 +2204,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CQ9"/>
+  <dimension ref="A1:CR9"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="20.1796875" bestFit="1" customWidth="1"/>
@@ -2186,25 +2221,26 @@
     <col min="23" max="54" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="55" max="61" width="35.81640625" bestFit="1" customWidth="1"/>
     <col min="62" max="62" width="22.90625" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="35.81640625" style="21" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="35.81640625" customWidth="1"/>
-    <col min="67" max="67" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="35.81640625" style="13" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="70" max="72" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="74" max="77" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="78" max="80" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="81" max="84" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="85" max="86" width="35.81640625" style="6" customWidth="1"/>
-    <col min="87" max="87" width="35.81640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="88" max="92" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="93" max="94" width="35.81640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="22.90625" customWidth="1"/>
+    <col min="64" max="64" width="35.81640625" style="21" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="35.81640625" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="35.81640625" customWidth="1"/>
+    <col min="68" max="68" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="35.81640625" style="13" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="71" max="73" width="35.81640625" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="75" max="78" width="35.81640625" bestFit="1" customWidth="1"/>
+    <col min="79" max="81" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="82" max="85" width="35.81640625" bestFit="1" customWidth="1"/>
+    <col min="86" max="87" width="35.81640625" style="6" customWidth="1"/>
+    <col min="88" max="88" width="35.81640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="89" max="93" width="35.81640625" bestFit="1" customWidth="1"/>
+    <col min="94" max="95" width="35.81640625" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:95">
+    <row r="1" spans="1:96">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2391,105 +2427,108 @@
       <c r="BJ1" t="s">
         <v>15</v>
       </c>
-      <c r="BK1" s="21" t="s">
+      <c r="BK1" t="s">
+        <v>505</v>
+      </c>
+      <c r="BL1" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="BL1" s="4" t="s">
+      <c r="BM1" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BN1" t="s">
         <v>69</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BO1" t="s">
         <v>497</v>
       </c>
-      <c r="BO1" s="4" t="s">
+      <c r="BP1" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="BP1" s="13" t="s">
+      <c r="BQ1" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="BQ1" s="4" t="s">
+      <c r="BR1" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BS1" t="s">
         <v>73</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BT1" t="s">
         <v>74</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BU1" t="s">
         <v>75</v>
       </c>
-      <c r="BU1" s="4" t="s">
+      <c r="BV1" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="BW1" t="s">
         <v>77</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="BX1" t="s">
         <v>78</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="BY1" t="s">
         <v>79</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="BZ1" t="s">
         <v>80</v>
       </c>
-      <c r="BZ1" s="4" t="s">
+      <c r="CA1" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="CA1" s="4" t="s">
+      <c r="CB1" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="CB1" s="4" t="s">
+      <c r="CC1" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CD1" t="s">
         <v>84</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CE1" t="s">
         <v>85</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CF1" t="s">
         <v>86</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CG1" t="s">
         <v>87</v>
       </c>
-      <c r="CG1" s="6" t="s">
+      <c r="CH1" s="6" t="s">
         <v>382</v>
       </c>
-      <c r="CH1" s="6" t="s">
+      <c r="CI1" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="CI1" s="8" t="s">
+      <c r="CJ1" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CK1" t="s">
         <v>89</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CL1" t="s">
         <v>90</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CM1" t="s">
         <v>91</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CN1" t="s">
         <v>92</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CO1" t="s">
         <v>93</v>
       </c>
-      <c r="CO1" s="8" t="s">
+      <c r="CP1" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="CP1" s="8" t="s">
+      <c r="CQ1" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="CQ1" s="2"/>
-    </row>
-    <row r="2" spans="1:95">
+      <c r="CR1" s="2"/>
+    </row>
+    <row r="2" spans="1:96">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -2674,30 +2713,30 @@
         <v>96</v>
       </c>
       <c r="BJ2" t="s">
-        <v>16</v>
-      </c>
-      <c r="BK2" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="BL2" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="BM2" t="s">
+        <v>96</v>
+      </c>
+      <c r="BK2" t="s">
+        <v>96</v>
+      </c>
+      <c r="BL2" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="BM2" s="4" t="s">
         <v>96</v>
       </c>
       <c r="BN2" t="s">
+        <v>96</v>
+      </c>
+      <c r="BO2" t="s">
         <v>498</v>
       </c>
-      <c r="BO2" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="BP2" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="BQ2" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="BR2" t="s">
+      <c r="BP2" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="BQ2" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="BR2" s="4" t="s">
         <v>96</v>
       </c>
       <c r="BS2" t="s">
@@ -2706,10 +2745,10 @@
       <c r="BT2" t="s">
         <v>96</v>
       </c>
-      <c r="BU2" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="BV2" t="s">
+      <c r="BU2" t="s">
+        <v>96</v>
+      </c>
+      <c r="BV2" s="4" t="s">
         <v>96</v>
       </c>
       <c r="BW2" t="s">
@@ -2721,7 +2760,7 @@
       <c r="BY2" t="s">
         <v>96</v>
       </c>
-      <c r="BZ2" s="4" t="s">
+      <c r="BZ2" t="s">
         <v>96</v>
       </c>
       <c r="CA2" s="4" t="s">
@@ -2730,7 +2769,7 @@
       <c r="CB2" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="CC2" t="s">
+      <c r="CC2" s="4" t="s">
         <v>96</v>
       </c>
       <c r="CD2" t="s">
@@ -2742,16 +2781,16 @@
       <c r="CF2" t="s">
         <v>96</v>
       </c>
-      <c r="CG2" s="6" t="s">
+      <c r="CG2" t="s">
         <v>96</v>
       </c>
       <c r="CH2" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="CI2" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="CJ2" t="s">
+      <c r="CI2" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="CJ2" s="8" t="s">
         <v>96</v>
       </c>
       <c r="CK2" t="s">
@@ -2766,15 +2805,18 @@
       <c r="CN2" t="s">
         <v>96</v>
       </c>
-      <c r="CO2" s="8" t="s">
+      <c r="CO2" t="s">
         <v>96</v>
       </c>
       <c r="CP2" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="CQ2" s="2"/>
-    </row>
-    <row r="3" spans="1:95" s="2" customFormat="1" ht="101.5">
+      <c r="CQ2" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="CR2" s="2"/>
+    </row>
+    <row r="3" spans="1:96" s="2" customFormat="1" ht="101.5">
       <c r="A3" s="9" t="s">
         <v>1</v>
       </c>
@@ -2897,95 +2939,98 @@
       <c r="BJ3" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="BK3" s="22" t="s">
+      <c r="BK3" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="BL3" s="22" t="s">
         <v>452</v>
       </c>
-      <c r="BL3" s="3" t="s">
+      <c r="BM3" s="3" t="s">
         <v>453</v>
       </c>
-      <c r="BM3" s="2" t="s">
+      <c r="BN3" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="BN3" t="s">
+      <c r="BO3" t="s">
         <v>499</v>
       </c>
-      <c r="BO3" s="3" t="s">
+      <c r="BP3" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="BP3" s="17" t="s">
+      <c r="BQ3" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="BQ3" s="3" t="s">
+      <c r="BR3" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="BR3" s="2" t="s">
+      <c r="BS3" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="BS3" s="2" t="s">
+      <c r="BT3" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="BT3" s="2" t="s">
+      <c r="BU3" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="BU3" s="3" t="s">
+      <c r="BV3" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="BW3" s="2" t="s">
+      <c r="BX3" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="BX3" s="2" t="s">
+      <c r="BY3" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="BY3" s="2" t="s">
+      <c r="BZ3" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="BZ3" s="3" t="s">
+      <c r="CA3" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="CA3" s="3" t="s">
+      <c r="CB3" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="CB3" s="3" t="s">
+      <c r="CC3" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="CC3" s="2" t="s">
+      <c r="CD3" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="CD3" s="2" t="s">
+      <c r="CE3" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="CE3" s="2" t="s">
+      <c r="CF3" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="CF3" s="2" t="s">
+      <c r="CG3" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="CG3" s="5" t="s">
-        <v>383</v>
       </c>
       <c r="CH3" s="5" t="s">
         <v>383</v>
       </c>
-      <c r="CI3" s="7"/>
-      <c r="CJ3" s="2" t="s">
+      <c r="CI3" s="5" t="s">
+        <v>383</v>
+      </c>
+      <c r="CJ3" s="7"/>
+      <c r="CK3" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="CK3" s="2" t="s">
+      <c r="CL3" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="CL3" s="2" t="s">
+      <c r="CM3" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="CM3" s="2" t="s">
+      <c r="CN3" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="CN3" s="2" t="s">
+      <c r="CO3" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="CO3" s="7"/>
       <c r="CP3" s="7"/>
-    </row>
-    <row r="4" spans="1:95">
+      <c r="CQ3" s="7"/>
+    </row>
+    <row r="4" spans="1:96">
       <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
@@ -3172,44 +3217,44 @@
       <c r="BJ4" t="s">
         <v>98</v>
       </c>
-      <c r="BK4" s="21" t="s">
+      <c r="BK4" t="s">
+        <v>99</v>
+      </c>
+      <c r="BL4" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="BL4" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="BM4" t="s">
+      <c r="BM4" s="4" t="s">
         <v>98</v>
       </c>
       <c r="BN4" t="s">
         <v>98</v>
       </c>
-      <c r="BO4" s="4" t="s">
+      <c r="BO4" t="s">
+        <v>98</v>
+      </c>
+      <c r="BP4" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="BP4" s="13" t="s">
+      <c r="BQ4" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="BQ4" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="BR4" s="11" t="s">
+      <c r="BR4" s="4" t="s">
         <v>99</v>
       </c>
       <c r="BS4" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="BT4" t="s">
+      <c r="BT4" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="BU4" t="s">
         <v>100</v>
       </c>
-      <c r="BU4" s="4" t="s">
+      <c r="BV4" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="BV4" t="s">
+      <c r="BW4" t="s">
         <v>388</v>
-      </c>
-      <c r="BW4" t="s">
-        <v>99</v>
       </c>
       <c r="BX4" t="s">
         <v>99</v>
@@ -3217,7 +3262,7 @@
       <c r="BY4" t="s">
         <v>99</v>
       </c>
-      <c r="BZ4" s="4" t="s">
+      <c r="BZ4" t="s">
         <v>99</v>
       </c>
       <c r="CA4" s="4" t="s">
@@ -3226,10 +3271,10 @@
       <c r="CB4" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="CC4" s="11" t="s">
+      <c r="CC4" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="CD4" t="s">
+      <c r="CD4" s="11" t="s">
         <v>99</v>
       </c>
       <c r="CE4" t="s">
@@ -3238,38 +3283,41 @@
       <c r="CF4" t="s">
         <v>99</v>
       </c>
-      <c r="CG4" s="6" t="s">
+      <c r="CG4" t="s">
         <v>99</v>
       </c>
       <c r="CH4" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="CI4" s="8" t="s">
+      <c r="CI4" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="CJ4" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="CJ4" s="11" t="s">
+      <c r="CK4" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="CK4" t="s">
+      <c r="CL4" t="s">
         <v>99</v>
       </c>
-      <c r="CL4" t="s">
+      <c r="CM4" t="s">
         <v>98</v>
-      </c>
-      <c r="CM4" t="s">
-        <v>99</v>
       </c>
       <c r="CN4" t="s">
         <v>99</v>
       </c>
-      <c r="CO4" s="8" t="s">
+      <c r="CO4" t="s">
+        <v>99</v>
+      </c>
+      <c r="CP4" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="CP4" s="8" t="s">
+      <c r="CQ4" s="8" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="1:95">
+    <row r="5" spans="1:96">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -3288,15 +3336,15 @@
       <c r="F5" t="s">
         <v>103</v>
       </c>
-      <c r="CO5" s="8"/>
       <c r="CP5" s="8"/>
-    </row>
-    <row r="6" spans="1:95">
+      <c r="CQ5" s="8"/>
+    </row>
+    <row r="6" spans="1:96">
       <c r="A6" s="1"/>
-      <c r="CO6" s="8"/>
       <c r="CP6" s="8"/>
-    </row>
-    <row r="7" spans="1:95">
+      <c r="CQ6" s="8"/>
+    </row>
+    <row r="7" spans="1:96">
       <c r="A7" s="1" t="s">
         <v>106</v>
       </c>
@@ -3366,36 +3414,36 @@
       <c r="BJ7" t="s">
         <v>108</v>
       </c>
-      <c r="BK7" s="21" t="s">
+      <c r="BL7" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="BL7" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="BM7" t="s">
+      <c r="BM7" s="4" t="s">
         <v>109</v>
       </c>
       <c r="BN7" t="s">
         <v>109</v>
       </c>
-      <c r="BT7" t="s">
+      <c r="BO7" t="s">
+        <v>109</v>
+      </c>
+      <c r="BU7" t="s">
         <v>108</v>
       </c>
-      <c r="BU7" s="4" t="s">
+      <c r="BV7" s="4" t="s">
         <v>415</v>
       </c>
-      <c r="CO7" s="8"/>
       <c r="CP7" s="8"/>
-    </row>
-    <row r="8" spans="1:95">
+      <c r="CQ7" s="8"/>
+    </row>
+    <row r="8" spans="1:96">
       <c r="A8" s="1"/>
-      <c r="CO8" s="8"/>
       <c r="CP8" s="8"/>
-    </row>
-    <row r="9" spans="1:95">
+      <c r="CQ8" s="8"/>
+    </row>
+    <row r="9" spans="1:96">
       <c r="A9" s="1"/>
-      <c r="CO9" s="8"/>
       <c r="CP9" s="8"/>
+      <c r="CQ9" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
@@ -3406,7 +3454,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83406F25-8B9E-4B45-BE5A-CFE07640E852}">
-  <dimension ref="A1:Q173"/>
+  <dimension ref="A1:Q177"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="35.81640625" bestFit="1" customWidth="1"/>
@@ -4616,855 +4664,867 @@
         <v>16</v>
       </c>
     </row>
-    <row r="48" spans="1:14" s="4" customFormat="1">
-      <c r="A48" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B48" s="4" t="s">
+    <row r="48" spans="1:14">
+      <c r="A48" t="s">
+        <v>96</v>
+      </c>
+      <c r="B48" t="s">
+        <v>505</v>
+      </c>
+      <c r="C48" t="s">
+        <v>261</v>
+      </c>
+      <c r="D48" t="s">
+        <v>507</v>
+      </c>
+      <c r="E48" t="s">
+        <v>510</v>
+      </c>
+      <c r="F48" t="s">
+        <v>514</v>
+      </c>
+      <c r="G48" t="s">
+        <v>15</v>
+      </c>
+      <c r="H48" t="s">
+        <v>16</v>
+      </c>
+      <c r="I48" t="s">
+        <v>282</v>
+      </c>
+      <c r="J48" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12">
+      <c r="A49" t="s">
+        <v>96</v>
+      </c>
+      <c r="D49" t="s">
+        <v>508</v>
+      </c>
+      <c r="E49" t="s">
+        <v>511</v>
+      </c>
+      <c r="F49" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12">
+      <c r="A50" t="s">
+        <v>96</v>
+      </c>
+      <c r="D50" t="s">
+        <v>509</v>
+      </c>
+      <c r="E50" t="s">
+        <v>512</v>
+      </c>
+      <c r="F50" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12">
+      <c r="A51" t="s">
+        <v>96</v>
+      </c>
+      <c r="D51" t="s">
+        <v>169</v>
+      </c>
+      <c r="E51" t="s">
+        <v>169</v>
+      </c>
+      <c r="F51" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" s="4" customFormat="1">
+      <c r="A52" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B52" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C48" s="4" t="s">
+      <c r="C52" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="D48" s="4" t="s">
+      <c r="D52" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="E48" s="4" t="s">
+      <c r="E52" s="4" t="s">
         <v>454</v>
       </c>
-      <c r="F48" s="4" t="s">
+      <c r="F52" s="4" t="s">
         <v>318</v>
       </c>
-      <c r="G48" s="4" t="s">
+      <c r="G52" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="H48" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="I48" s="4" t="s">
+      <c r="H52" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="I52" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="J48" s="4" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13" s="4" customFormat="1">
-      <c r="A49" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B49" s="4" t="s">
+      <c r="J52" s="4" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" s="4" customFormat="1">
+      <c r="A53" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B53" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C49" s="4" t="s">
+      <c r="C53" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="D49" s="4" t="s">
+      <c r="D53" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="E49" s="4" t="s">
+      <c r="E53" s="4" t="s">
         <v>455</v>
       </c>
-      <c r="F49" s="4" t="s">
+      <c r="F53" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="G49" s="4" t="s">
+      <c r="G53" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="H49" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="I49" s="4" t="s">
+      <c r="H53" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="I53" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="J49" s="4" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="50" spans="1:13" s="26" customFormat="1">
-      <c r="A50" s="26" t="s">
-        <v>96</v>
-      </c>
-      <c r="B50" s="26" t="s">
+      <c r="J53" s="4" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12">
+      <c r="A54" t="s">
+        <v>96</v>
+      </c>
+      <c r="B54" t="s">
         <v>500</v>
       </c>
-      <c r="C50" s="26" t="s">
+      <c r="C54" t="s">
         <v>260</v>
       </c>
-      <c r="D50" s="26" t="s">
+      <c r="D54" t="s">
         <v>109</v>
       </c>
-      <c r="E50" s="26" t="s">
+      <c r="E54" t="s">
         <v>501</v>
       </c>
-      <c r="F50" s="26" t="s">
+      <c r="F54" t="s">
         <v>503</v>
       </c>
-      <c r="G50" t="s">
+      <c r="G54" t="s">
         <v>68</v>
       </c>
-      <c r="H50" t="s">
-        <v>307</v>
-      </c>
-      <c r="I50" t="s">
+      <c r="H54" t="s">
+        <v>307</v>
+      </c>
+      <c r="I54" t="s">
         <v>67</v>
       </c>
-      <c r="J50" t="s">
-        <v>307</v>
-      </c>
-      <c r="K50" s="26" t="s">
+      <c r="J54" t="s">
+        <v>307</v>
+      </c>
+      <c r="K54" t="s">
         <v>448</v>
       </c>
-      <c r="L50" s="26" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="51" spans="1:13">
-      <c r="A51" t="s">
-        <v>96</v>
-      </c>
-      <c r="B51" t="s">
+      <c r="L54" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12">
+      <c r="A55" t="s">
+        <v>96</v>
+      </c>
+      <c r="B55" t="s">
         <v>69</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C55" t="s">
         <v>260</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D55" t="s">
         <v>109</v>
       </c>
-      <c r="E51" t="s">
+      <c r="E55" t="s">
         <v>502</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F55" t="s">
         <v>449</v>
       </c>
-      <c r="G51" t="s">
+      <c r="G55" t="s">
         <v>68</v>
       </c>
-      <c r="H51" t="s">
-        <v>307</v>
-      </c>
-      <c r="I51" t="s">
+      <c r="H55" t="s">
+        <v>307</v>
+      </c>
+      <c r="I55" t="s">
         <v>67</v>
       </c>
-      <c r="J51" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="52" spans="1:13" s="4" customFormat="1">
-      <c r="A52" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B52" s="4" t="s">
+      <c r="J55" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" s="4" customFormat="1">
+      <c r="A56" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B56" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="C56" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="D52" s="4">
+      <c r="D56" s="4">
         <v>0</v>
       </c>
-      <c r="E52" s="4" t="s">
+      <c r="E56" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="F52" s="4" t="s">
+      <c r="F56" s="4" t="s">
         <v>352</v>
       </c>
-      <c r="G52" s="4" t="s">
+      <c r="G56" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="H52" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="I52" s="4" t="s">
+      <c r="H56" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="I56" s="4" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="53" spans="1:13" s="4" customFormat="1">
-      <c r="A53" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D53" s="4">
+    <row r="57" spans="1:12" s="4" customFormat="1">
+      <c r="A57" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D57" s="4">
         <v>1</v>
       </c>
-      <c r="E53" s="4" t="s">
+      <c r="E57" s="4" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="54" spans="1:13" s="4" customFormat="1">
-      <c r="A54" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D54" s="4">
+    <row r="58" spans="1:12" s="4" customFormat="1">
+      <c r="A58" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D58" s="4">
         <v>2</v>
       </c>
-      <c r="E54" s="4" t="s">
+      <c r="E58" s="4" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="55" spans="1:13" s="4" customFormat="1">
-      <c r="A55" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D55" s="4">
+    <row r="59" spans="1:12" s="4" customFormat="1">
+      <c r="A59" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D59" s="4">
         <v>3</v>
       </c>
-      <c r="E55" s="4" t="s">
+      <c r="E59" s="4" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="56" spans="1:13" s="4" customFormat="1">
-      <c r="A56" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D56" s="4" t="s">
+    <row r="60" spans="1:12" s="4" customFormat="1">
+      <c r="A60" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D60" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="E56" s="4" t="s">
+      <c r="E60" s="4" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="57" spans="1:13">
-      <c r="A57" t="s">
-        <v>96</v>
-      </c>
-      <c r="B57" t="s">
+    <row r="61" spans="1:12">
+      <c r="A61" t="s">
+        <v>96</v>
+      </c>
+      <c r="B61" t="s">
         <v>71</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C61" t="s">
         <v>261</v>
       </c>
-      <c r="D57">
+      <c r="D61">
         <v>0</v>
       </c>
-      <c r="E57" t="s">
+      <c r="E61" t="s">
         <v>172</v>
       </c>
-      <c r="F57" t="s">
+      <c r="F61" t="s">
         <v>353</v>
       </c>
-      <c r="G57" t="s">
+      <c r="G61" t="s">
         <v>66</v>
       </c>
-      <c r="H57" t="s">
-        <v>307</v>
-      </c>
-      <c r="I57" t="s">
+      <c r="H61" t="s">
+        <v>307</v>
+      </c>
+      <c r="I61" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="58" spans="1:13">
-      <c r="A58" t="s">
-        <v>96</v>
-      </c>
-      <c r="D58">
+    <row r="62" spans="1:12">
+      <c r="A62" t="s">
+        <v>96</v>
+      </c>
+      <c r="D62">
         <v>1</v>
       </c>
-      <c r="E58" t="s">
+      <c r="E62" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="59" spans="1:13">
-      <c r="A59" t="s">
-        <v>96</v>
-      </c>
-      <c r="D59" t="s">
+    <row r="63" spans="1:12">
+      <c r="A63" t="s">
+        <v>96</v>
+      </c>
+      <c r="D63" t="s">
         <v>169</v>
       </c>
-      <c r="E59" t="s">
+      <c r="E63" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="60" spans="1:13">
-      <c r="A60" t="s">
-        <v>96</v>
-      </c>
-      <c r="B60" t="s">
+    <row r="64" spans="1:12">
+      <c r="A64" t="s">
+        <v>96</v>
+      </c>
+      <c r="B64" t="s">
         <v>73</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C64" t="s">
         <v>261</v>
       </c>
-      <c r="D60">
+      <c r="D64">
         <v>0</v>
       </c>
-      <c r="E60" t="s">
+      <c r="E64" t="s">
         <v>167</v>
       </c>
-      <c r="F60" t="s">
+      <c r="F64" t="s">
         <v>354</v>
       </c>
-      <c r="G60" t="s">
+      <c r="G64" t="s">
         <v>58</v>
       </c>
-      <c r="H60" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="61" spans="1:13">
-      <c r="A61" t="s">
-        <v>96</v>
-      </c>
-      <c r="D61">
+      <c r="H64" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13">
+      <c r="A65" t="s">
+        <v>96</v>
+      </c>
+      <c r="D65">
         <v>1</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E65" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="62" spans="1:13">
-      <c r="A62" t="s">
-        <v>96</v>
-      </c>
-      <c r="D62" t="s">
+    <row r="66" spans="1:13">
+      <c r="A66" t="s">
+        <v>96</v>
+      </c>
+      <c r="D66" t="s">
         <v>169</v>
       </c>
-      <c r="E62" t="s">
+      <c r="E66" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="63" spans="1:13">
-      <c r="A63" t="s">
-        <v>96</v>
-      </c>
-      <c r="B63" t="s">
+    <row r="67" spans="1:13">
+      <c r="A67" t="s">
+        <v>96</v>
+      </c>
+      <c r="B67" t="s">
         <v>74</v>
       </c>
-      <c r="C63" t="s">
+      <c r="C67" t="s">
         <v>261</v>
       </c>
-      <c r="D63">
+      <c r="D67">
         <v>0</v>
       </c>
-      <c r="E63" t="s">
+      <c r="E67" t="s">
         <v>167</v>
       </c>
-      <c r="F63" s="11" t="s">
+      <c r="F67" s="11" t="s">
         <v>355</v>
       </c>
-      <c r="G63" s="11" t="s">
+      <c r="G67" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="H63" s="11" t="s">
-        <v>307</v>
-      </c>
-      <c r="I63" s="11" t="s">
+      <c r="H67" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="I67" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="J63" s="11" t="s">
-        <v>307</v>
-      </c>
-      <c r="K63" s="11" t="s">
+      <c r="J67" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="K67" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="L63" s="11" t="s">
-        <v>307</v>
-      </c>
-      <c r="M63" s="11"/>
-    </row>
-    <row r="64" spans="1:13">
-      <c r="A64" t="s">
-        <v>96</v>
-      </c>
-      <c r="D64">
+      <c r="L67" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="M67" s="11"/>
+    </row>
+    <row r="68" spans="1:13">
+      <c r="A68" t="s">
+        <v>96</v>
+      </c>
+      <c r="D68">
         <v>1</v>
       </c>
-      <c r="E64" t="s">
+      <c r="E68" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="65" spans="1:8">
-      <c r="A65" t="s">
-        <v>96</v>
-      </c>
-      <c r="D65" t="s">
+    <row r="69" spans="1:13">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="D69" t="s">
         <v>169</v>
       </c>
-      <c r="E65" t="s">
+      <c r="E69" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="66" spans="1:8">
-      <c r="A66" t="s">
-        <v>96</v>
-      </c>
-      <c r="B66" t="s">
+    <row r="70" spans="1:13">
+      <c r="A70" t="s">
+        <v>96</v>
+      </c>
+      <c r="B70" t="s">
         <v>75</v>
       </c>
-      <c r="C66" t="s">
+      <c r="C70" t="s">
         <v>260</v>
       </c>
-      <c r="D66" t="s">
+      <c r="D70" t="s">
         <v>108</v>
       </c>
-      <c r="F66" t="s">
+      <c r="F70" t="s">
         <v>356</v>
       </c>
-      <c r="G66" t="s">
+      <c r="G70" t="s">
         <v>59</v>
       </c>
-      <c r="H66" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8" s="4" customFormat="1">
-      <c r="A67" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B67" s="4" t="s">
+      <c r="H70" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" s="4" customFormat="1">
+      <c r="A71" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B71" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C67" s="4" t="s">
+      <c r="C71" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="D67" s="4">
+      <c r="D71" s="4">
         <v>1</v>
       </c>
-      <c r="E67" s="4" t="s">
+      <c r="E71" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="F67" s="4" t="s">
+      <c r="F71" s="4" t="s">
         <v>357</v>
       </c>
-      <c r="G67" s="4" t="s">
+      <c r="G71" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="H67" s="4" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8" s="4" customFormat="1">
-      <c r="A68" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D68" s="4">
+      <c r="H71" s="4" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" s="4" customFormat="1">
+      <c r="A72" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D72" s="4">
         <v>2</v>
       </c>
-      <c r="E68" s="4" t="s">
+      <c r="E72" s="4" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="69" spans="1:8" s="4" customFormat="1">
-      <c r="A69" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D69" s="4">
+    <row r="73" spans="1:13" s="4" customFormat="1">
+      <c r="A73" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D73" s="4">
         <v>3</v>
       </c>
-      <c r="E69" s="4" t="s">
+      <c r="E73" s="4" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="70" spans="1:8" s="4" customFormat="1">
-      <c r="A70" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D70" s="4">
+    <row r="74" spans="1:13" s="4" customFormat="1">
+      <c r="A74" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D74" s="4">
         <v>4</v>
       </c>
-      <c r="E70" s="4" t="s">
+      <c r="E74" s="4" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="71" spans="1:8" s="4" customFormat="1">
-      <c r="A71" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D71" s="4">
+    <row r="75" spans="1:13" s="4" customFormat="1">
+      <c r="A75" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D75" s="4">
         <v>5</v>
       </c>
-      <c r="E71" s="4" t="s">
+      <c r="E75" s="4" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="72" spans="1:8" s="4" customFormat="1">
-      <c r="A72" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D72" s="4">
+    <row r="76" spans="1:13" s="4" customFormat="1">
+      <c r="A76" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D76" s="4">
         <v>6</v>
       </c>
-      <c r="E72" s="4" t="s">
+      <c r="E76" s="4" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="73" spans="1:8" s="4" customFormat="1">
-      <c r="A73" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D73" s="4">
+    <row r="77" spans="1:13" s="4" customFormat="1">
+      <c r="A77" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D77" s="4">
         <v>7</v>
       </c>
-      <c r="E73" s="4" t="s">
+      <c r="E77" s="4" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="74" spans="1:8" s="4" customFormat="1">
-      <c r="A74" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D74" s="4">
+    <row r="78" spans="1:13" s="4" customFormat="1">
+      <c r="A78" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D78" s="4">
         <v>8</v>
       </c>
-      <c r="E74" s="4" t="s">
+      <c r="E78" s="4" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="75" spans="1:8" s="4" customFormat="1">
-      <c r="A75" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D75" s="4">
+    <row r="79" spans="1:13" s="4" customFormat="1">
+      <c r="A79" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D79" s="4">
         <v>9</v>
       </c>
-      <c r="E75" s="4" t="s">
+      <c r="E79" s="4" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="76" spans="1:8" s="4" customFormat="1">
-      <c r="A76" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D76" s="4">
+    <row r="80" spans="1:13" s="4" customFormat="1">
+      <c r="A80" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D80" s="4">
         <v>10</v>
       </c>
-      <c r="E76" s="4" t="s">
+      <c r="E80" s="4" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="77" spans="1:8" s="4" customFormat="1">
-      <c r="A77" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D77" s="4">
+    <row r="81" spans="1:8" s="4" customFormat="1">
+      <c r="A81" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D81" s="4">
         <v>11</v>
       </c>
-      <c r="E77" s="4" t="s">
+      <c r="E81" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="78" spans="1:8" s="4" customFormat="1">
-      <c r="A78" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D78" s="4">
+    <row r="82" spans="1:8" s="4" customFormat="1">
+      <c r="A82" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D82" s="4">
         <v>12</v>
       </c>
-      <c r="E78" s="4" t="s">
+      <c r="E82" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="79" spans="1:8" s="4" customFormat="1">
-      <c r="A79" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D79" s="4">
+    <row r="83" spans="1:8" s="4" customFormat="1">
+      <c r="A83" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D83" s="4">
         <v>13</v>
       </c>
-      <c r="E79" s="4" t="s">
+      <c r="E83" s="4" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="80" spans="1:8" s="4" customFormat="1">
-      <c r="A80" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D80" s="4" t="s">
+    <row r="84" spans="1:8" s="4" customFormat="1">
+      <c r="A84" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D84" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="E80" s="4" t="s">
+      <c r="E84" s="4" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="81" spans="1:8">
-      <c r="A81" t="s">
-        <v>96</v>
-      </c>
-      <c r="B81" t="s">
+    <row r="85" spans="1:8">
+      <c r="A85" t="s">
+        <v>96</v>
+      </c>
+      <c r="B85" t="s">
         <v>77</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C85" t="s">
         <v>260</v>
       </c>
-      <c r="D81">
+      <c r="D85">
         <v>1</v>
       </c>
-      <c r="E81" t="s">
+      <c r="E85" t="s">
         <v>181</v>
       </c>
-      <c r="F81" t="s">
+      <c r="F85" t="s">
         <v>414</v>
       </c>
-      <c r="G81" t="s">
+      <c r="G85" t="s">
         <v>321</v>
       </c>
-      <c r="H81" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="82" spans="1:8">
-      <c r="A82" t="s">
-        <v>96</v>
-      </c>
-      <c r="D82">
-        <f>D81 +1</f>
+      <c r="H85" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8">
+      <c r="A86" t="s">
+        <v>96</v>
+      </c>
+      <c r="D86">
+        <f>D85 +1</f>
         <v>2</v>
       </c>
-      <c r="E82" t="s">
+      <c r="E86" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="83" spans="1:8">
-      <c r="A83" t="s">
-        <v>96</v>
-      </c>
-      <c r="D83">
-        <f t="shared" ref="D83:D98" si="0">D82 +1</f>
+    <row r="87" spans="1:8">
+      <c r="A87" t="s">
+        <v>96</v>
+      </c>
+      <c r="D87">
+        <f t="shared" ref="D87:D102" si="0">D86 +1</f>
         <v>3</v>
       </c>
-      <c r="E83" t="s">
+      <c r="E87" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="84" spans="1:8">
-      <c r="A84" t="s">
-        <v>96</v>
-      </c>
-      <c r="D84">
+    <row r="88" spans="1:8">
+      <c r="A88" t="s">
+        <v>96</v>
+      </c>
+      <c r="D88">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="E84" t="s">
+      <c r="E88" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="85" spans="1:8">
-      <c r="A85" t="s">
-        <v>96</v>
-      </c>
-      <c r="D85">
+    <row r="89" spans="1:8">
+      <c r="A89" t="s">
+        <v>96</v>
+      </c>
+      <c r="D89">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="E85" t="s">
+      <c r="E89" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="86" spans="1:8">
-      <c r="A86" t="s">
-        <v>96</v>
-      </c>
-      <c r="D86">
+    <row r="90" spans="1:8">
+      <c r="A90" t="s">
+        <v>96</v>
+      </c>
+      <c r="D90">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="E86" t="s">
+      <c r="E90" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="87" spans="1:8">
-      <c r="A87" t="s">
-        <v>96</v>
-      </c>
-      <c r="D87">
+    <row r="91" spans="1:8">
+      <c r="A91" t="s">
+        <v>96</v>
+      </c>
+      <c r="D91">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="E87" t="s">
+      <c r="E91" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="88" spans="1:8">
-      <c r="A88" t="s">
-        <v>96</v>
-      </c>
-      <c r="D88">
+    <row r="92" spans="1:8">
+      <c r="A92" t="s">
+        <v>96</v>
+      </c>
+      <c r="D92">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="E88" t="s">
+      <c r="E92" t="s">
         <v>404</v>
       </c>
     </row>
-    <row r="89" spans="1:8">
-      <c r="A89" t="s">
-        <v>96</v>
-      </c>
-      <c r="D89">
+    <row r="93" spans="1:8">
+      <c r="A93" t="s">
+        <v>96</v>
+      </c>
+      <c r="D93">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="E89" t="s">
+      <c r="E93" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="90" spans="1:8">
-      <c r="A90" t="s">
-        <v>96</v>
-      </c>
-      <c r="D90">
+    <row r="94" spans="1:8">
+      <c r="A94" t="s">
+        <v>96</v>
+      </c>
+      <c r="D94">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="E90" t="s">
+      <c r="E94" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="91" spans="1:8">
-      <c r="A91" t="s">
-        <v>96</v>
-      </c>
-      <c r="D91">
+    <row r="95" spans="1:8">
+      <c r="A95" t="s">
+        <v>96</v>
+      </c>
+      <c r="D95">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="E91" t="s">
+      <c r="E95" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="92" spans="1:8">
-      <c r="A92" t="s">
-        <v>96</v>
-      </c>
-      <c r="D92">
+    <row r="96" spans="1:8">
+      <c r="A96" t="s">
+        <v>96</v>
+      </c>
+      <c r="D96">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="E92" t="s">
+      <c r="E96" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="93" spans="1:8">
-      <c r="A93" t="s">
-        <v>96</v>
-      </c>
-      <c r="D93">
+    <row r="97" spans="1:16">
+      <c r="A97" t="s">
+        <v>96</v>
+      </c>
+      <c r="D97">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="E93" t="s">
+      <c r="E97" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="94" spans="1:8">
-      <c r="A94" t="s">
-        <v>96</v>
-      </c>
-      <c r="D94">
+    <row r="98" spans="1:16">
+      <c r="A98" t="s">
+        <v>96</v>
+      </c>
+      <c r="D98">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="E94" t="s">
+      <c r="E98" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="95" spans="1:8">
-      <c r="A95" t="s">
-        <v>96</v>
-      </c>
-      <c r="D95">
+    <row r="99" spans="1:16">
+      <c r="A99" t="s">
+        <v>96</v>
+      </c>
+      <c r="D99">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="E95" s="20" t="s">
+      <c r="E99" s="20" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="96" spans="1:8">
-      <c r="A96" t="s">
-        <v>96</v>
-      </c>
-      <c r="D96">
+    <row r="100" spans="1:16">
+      <c r="A100" t="s">
+        <v>96</v>
+      </c>
+      <c r="D100">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="E96" t="s">
+      <c r="E100" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="97" spans="1:16">
-      <c r="A97" t="s">
-        <v>96</v>
-      </c>
-      <c r="D97">
-        <f>D96 +1</f>
+    <row r="101" spans="1:16">
+      <c r="A101" t="s">
+        <v>96</v>
+      </c>
+      <c r="D101">
+        <f>D100 +1</f>
         <v>17</v>
       </c>
-      <c r="E97" t="s">
+      <c r="E101" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="98" spans="1:16">
-      <c r="A98" t="s">
-        <v>96</v>
-      </c>
-      <c r="D98">
+    <row r="102" spans="1:16">
+      <c r="A102" t="s">
+        <v>96</v>
+      </c>
+      <c r="D102">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="E98" t="s">
+      <c r="E102" t="s">
         <v>195</v>
-      </c>
-    </row>
-    <row r="99" spans="1:16">
-      <c r="A99" t="s">
-        <v>96</v>
-      </c>
-      <c r="D99" t="s">
-        <v>169</v>
-      </c>
-      <c r="E99" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="100" spans="1:16">
-      <c r="A100" t="s">
-        <v>96</v>
-      </c>
-      <c r="B100" t="s">
-        <v>78</v>
-      </c>
-      <c r="C100" t="s">
-        <v>261</v>
-      </c>
-      <c r="D100">
-        <v>0</v>
-      </c>
-      <c r="E100" t="s">
-        <v>197</v>
-      </c>
-      <c r="F100" t="s">
-        <v>358</v>
-      </c>
-      <c r="G100" t="s">
-        <v>66</v>
-      </c>
-      <c r="H100" t="s">
-        <v>307</v>
-      </c>
-      <c r="I100" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="101" spans="1:16">
-      <c r="A101" t="s">
-        <v>96</v>
-      </c>
-      <c r="D101">
-        <v>1</v>
-      </c>
-      <c r="E101" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="102" spans="1:16">
-      <c r="A102" t="s">
-        <v>96</v>
-      </c>
-      <c r="D102">
-        <v>2</v>
-      </c>
-      <c r="E102" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="103" spans="1:16">
@@ -5475,7 +5535,7 @@
         <v>169</v>
       </c>
       <c r="E103" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="104" spans="1:16">
@@ -5483,7 +5543,7 @@
         <v>96</v>
       </c>
       <c r="B104" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C104" t="s">
         <v>261</v>
@@ -5492,10 +5552,10 @@
         <v>0</v>
       </c>
       <c r="E104" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F104" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G104" t="s">
         <v>66</v>
@@ -5504,28 +5564,7 @@
         <v>307</v>
       </c>
       <c r="I104" t="s">
-        <v>73</v>
-      </c>
-      <c r="J104" t="s">
-        <v>307</v>
-      </c>
-      <c r="K104" t="s">
-        <v>74</v>
-      </c>
-      <c r="L104" t="s">
-        <v>307</v>
-      </c>
-      <c r="M104" t="s">
-        <v>48</v>
-      </c>
-      <c r="N104" t="s">
-        <v>307</v>
-      </c>
-      <c r="O104" t="s">
-        <v>323</v>
-      </c>
-      <c r="P104" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
     </row>
     <row r="105" spans="1:16">
@@ -5536,7 +5575,7 @@
         <v>1</v>
       </c>
       <c r="E105" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="106" spans="1:16">
@@ -5547,79 +5586,79 @@
         <v>2</v>
       </c>
       <c r="E106" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="107" spans="1:16">
       <c r="A107" t="s">
         <v>96</v>
       </c>
-      <c r="D107">
-        <v>3</v>
+      <c r="D107" t="s">
+        <v>169</v>
       </c>
       <c r="E107" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="108" spans="1:16">
       <c r="A108" t="s">
         <v>96</v>
       </c>
-      <c r="D108" t="s">
-        <v>169</v>
+      <c r="B108" t="s">
+        <v>79</v>
+      </c>
+      <c r="C108" t="s">
+        <v>261</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
       </c>
       <c r="E108" t="s">
-        <v>200</v>
+        <v>201</v>
+      </c>
+      <c r="F108" t="s">
+        <v>359</v>
+      </c>
+      <c r="G108" t="s">
+        <v>66</v>
+      </c>
+      <c r="H108" t="s">
+        <v>307</v>
+      </c>
+      <c r="I108" t="s">
+        <v>73</v>
+      </c>
+      <c r="J108" t="s">
+        <v>307</v>
+      </c>
+      <c r="K108" t="s">
+        <v>74</v>
+      </c>
+      <c r="L108" t="s">
+        <v>307</v>
+      </c>
+      <c r="M108" t="s">
+        <v>48</v>
+      </c>
+      <c r="N108" t="s">
+        <v>307</v>
+      </c>
+      <c r="O108" t="s">
+        <v>323</v>
+      </c>
+      <c r="P108" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="109" spans="1:16">
       <c r="A109" t="s">
         <v>96</v>
       </c>
-      <c r="B109" t="s">
-        <v>80</v>
-      </c>
-      <c r="C109" t="s">
-        <v>261</v>
-      </c>
       <c r="D109">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E109" t="s">
-        <v>201</v>
-      </c>
-      <c r="F109" t="s">
-        <v>360</v>
-      </c>
-      <c r="G109" t="s">
-        <v>66</v>
-      </c>
-      <c r="H109" t="s">
-        <v>307</v>
-      </c>
-      <c r="I109" t="s">
-        <v>73</v>
-      </c>
-      <c r="J109" t="s">
-        <v>307</v>
-      </c>
-      <c r="K109" t="s">
-        <v>74</v>
-      </c>
-      <c r="L109" t="s">
-        <v>307</v>
-      </c>
-      <c r="M109" t="s">
-        <v>48</v>
-      </c>
-      <c r="N109" t="s">
-        <v>307</v>
-      </c>
-      <c r="O109" t="s">
-        <v>323</v>
-      </c>
-      <c r="P109" t="s">
-        <v>307</v>
+        <v>202</v>
       </c>
     </row>
     <row r="110" spans="1:16">
@@ -5627,10 +5666,10 @@
         <v>96</v>
       </c>
       <c r="D110">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E110" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="111" spans="1:16">
@@ -5638,190 +5677,190 @@
         <v>96</v>
       </c>
       <c r="D111">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E111" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="112" spans="1:16">
       <c r="A112" t="s">
         <v>96</v>
       </c>
-      <c r="D112">
+      <c r="D112" t="s">
+        <v>169</v>
+      </c>
+      <c r="E112" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="113" spans="1:17">
+      <c r="A113" t="s">
+        <v>96</v>
+      </c>
+      <c r="B113" t="s">
+        <v>80</v>
+      </c>
+      <c r="C113" t="s">
+        <v>261</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113" t="s">
+        <v>201</v>
+      </c>
+      <c r="F113" t="s">
+        <v>360</v>
+      </c>
+      <c r="G113" t="s">
+        <v>66</v>
+      </c>
+      <c r="H113" t="s">
+        <v>307</v>
+      </c>
+      <c r="I113" t="s">
+        <v>73</v>
+      </c>
+      <c r="J113" t="s">
+        <v>307</v>
+      </c>
+      <c r="K113" t="s">
+        <v>74</v>
+      </c>
+      <c r="L113" t="s">
+        <v>307</v>
+      </c>
+      <c r="M113" t="s">
+        <v>48</v>
+      </c>
+      <c r="N113" t="s">
+        <v>307</v>
+      </c>
+      <c r="O113" t="s">
+        <v>323</v>
+      </c>
+      <c r="P113" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="114" spans="1:17">
+      <c r="A114" t="s">
+        <v>96</v>
+      </c>
+      <c r="D114">
+        <v>1</v>
+      </c>
+      <c r="E114" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="115" spans="1:17">
+      <c r="A115" t="s">
+        <v>96</v>
+      </c>
+      <c r="D115">
+        <v>2</v>
+      </c>
+      <c r="E115" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="116" spans="1:17">
+      <c r="A116" t="s">
+        <v>96</v>
+      </c>
+      <c r="D116">
         <v>3</v>
       </c>
-      <c r="E112" t="s">
+      <c r="E116" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="113" spans="1:17" s="6" customFormat="1">
-      <c r="A113" t="s">
-        <v>96</v>
-      </c>
-      <c r="B113"/>
-      <c r="C113"/>
-      <c r="D113" t="s">
+    <row r="117" spans="1:17" s="6" customFormat="1">
+      <c r="A117" t="s">
+        <v>96</v>
+      </c>
+      <c r="B117"/>
+      <c r="C117"/>
+      <c r="D117" t="s">
         <v>169</v>
       </c>
-      <c r="E113" t="s">
+      <c r="E117" t="s">
         <v>205</v>
       </c>
-      <c r="F113"/>
-      <c r="G113"/>
-      <c r="H113"/>
-      <c r="I113"/>
-      <c r="J113"/>
-      <c r="K113"/>
-      <c r="L113"/>
-      <c r="M113"/>
-      <c r="N113"/>
-      <c r="O113"/>
-      <c r="P113"/>
-      <c r="Q113"/>
-    </row>
-    <row r="114" spans="1:17" s="4" customFormat="1">
-      <c r="A114" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B114" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C114" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="D114" s="4">
-        <v>0</v>
-      </c>
-      <c r="E114" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="F114" s="4" t="s">
-        <v>361</v>
-      </c>
-      <c r="G114" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H114" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="I114" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="J114" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="K114" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="L114" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="M114" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="N114" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="O114" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="P114" s="4" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="115" spans="1:17" s="4" customFormat="1">
-      <c r="A115" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D115" s="4">
-        <v>1</v>
-      </c>
-      <c r="E115" s="4" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="116" spans="1:17" s="4" customFormat="1">
-      <c r="A116" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D116" s="4">
-        <v>2</v>
-      </c>
-      <c r="E116" s="4" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="117" spans="1:17" s="4" customFormat="1">
-      <c r="A117" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D117" s="4">
-        <v>3</v>
-      </c>
-      <c r="E117" s="4" t="s">
-        <v>209</v>
-      </c>
+      <c r="F117"/>
+      <c r="G117"/>
+      <c r="H117"/>
+      <c r="I117"/>
+      <c r="J117"/>
+      <c r="K117"/>
+      <c r="L117"/>
+      <c r="M117"/>
+      <c r="N117"/>
+      <c r="O117"/>
+      <c r="P117"/>
+      <c r="Q117"/>
     </row>
     <row r="118" spans="1:17" s="4" customFormat="1">
       <c r="A118" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D118" s="4" t="s">
-        <v>169</v>
+      <c r="B118" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="D118" s="4">
+        <v>0</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>206</v>
+        <v>217</v>
+      </c>
+      <c r="F118" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="G118" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H118" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="I118" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J118" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="K118" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="L118" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="M118" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="N118" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="O118" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="P118" s="4" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="119" spans="1:17" s="4" customFormat="1">
       <c r="A119" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B119" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C119" s="4" t="s">
-        <v>261</v>
-      </c>
       <c r="D119" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="F119" s="4" t="s">
-        <v>362</v>
-      </c>
-      <c r="G119" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H119" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="I119" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="J119" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="K119" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="L119" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="M119" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="N119" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="O119" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="P119" s="4" t="s">
-        <v>307</v>
+        <v>208</v>
       </c>
     </row>
     <row r="120" spans="1:17" s="4" customFormat="1">
@@ -5829,10 +5868,10 @@
         <v>96</v>
       </c>
       <c r="D120" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="121" spans="1:17" s="4" customFormat="1">
@@ -5840,82 +5879,82 @@
         <v>96</v>
       </c>
       <c r="D121" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="122" spans="1:17" s="4" customFormat="1">
       <c r="A122" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D122" s="4">
-        <v>3</v>
+      <c r="D122" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="E122" s="4" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
     </row>
     <row r="123" spans="1:17" s="4" customFormat="1">
       <c r="A123" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D123" s="4" t="s">
-        <v>169</v>
+      <c r="B123" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="D123" s="4">
+        <v>0</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
+      </c>
+      <c r="F123" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="G123" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H123" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="I123" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J123" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="K123" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="L123" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="M123" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="N123" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="O123" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="P123" s="4" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="124" spans="1:17" s="4" customFormat="1">
       <c r="A124" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B124" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C124" s="4" t="s">
-        <v>261</v>
-      </c>
       <c r="D124" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="F124" s="4" t="s">
-        <v>363</v>
-      </c>
-      <c r="G124" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H124" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="I124" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="J124" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="K124" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="L124" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="M124" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="N124" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="O124" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="P124" s="4" t="s">
-        <v>307</v>
+        <v>212</v>
       </c>
     </row>
     <row r="125" spans="1:17" s="4" customFormat="1">
@@ -5923,10 +5962,10 @@
         <v>96</v>
       </c>
       <c r="D125" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="126" spans="1:17" s="4" customFormat="1">
@@ -5934,165 +5973,165 @@
         <v>96</v>
       </c>
       <c r="D126" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
     </row>
     <row r="127" spans="1:17" s="4" customFormat="1">
       <c r="A127" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D127" s="4">
-        <v>3</v>
+      <c r="D127" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="E127" s="4" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
     </row>
     <row r="128" spans="1:17" s="4" customFormat="1">
       <c r="A128" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D128" s="4" t="s">
+      <c r="B128" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="D128" s="4">
+        <v>0</v>
+      </c>
+      <c r="E128" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="F128" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="G128" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H128" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="I128" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J128" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="K128" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="L128" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="M128" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="N128" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="O128" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="P128" s="4" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="129" spans="1:16" s="4" customFormat="1">
+      <c r="A129" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D129" s="4">
+        <v>1</v>
+      </c>
+      <c r="E129" s="4" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="130" spans="1:16" s="4" customFormat="1">
+      <c r="A130" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D130" s="4">
+        <v>2</v>
+      </c>
+      <c r="E130" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="131" spans="1:16" s="4" customFormat="1">
+      <c r="A131" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D131" s="4">
+        <v>3</v>
+      </c>
+      <c r="E131" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="132" spans="1:16" s="4" customFormat="1">
+      <c r="A132" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D132" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="E128" s="4" t="s">
+      <c r="E132" s="4" t="s">
         <v>215</v>
-      </c>
-    </row>
-    <row r="129" spans="1:16">
-      <c r="A129" t="s">
-        <v>96</v>
-      </c>
-      <c r="B129" t="s">
-        <v>84</v>
-      </c>
-      <c r="C129" t="s">
-        <v>261</v>
-      </c>
-      <c r="D129">
-        <v>0</v>
-      </c>
-      <c r="E129" t="s">
-        <v>221</v>
-      </c>
-      <c r="F129" t="s">
-        <v>364</v>
-      </c>
-      <c r="G129" t="s">
-        <v>66</v>
-      </c>
-      <c r="H129" t="s">
-        <v>307</v>
-      </c>
-      <c r="I129" t="s">
-        <v>73</v>
-      </c>
-      <c r="J129" t="s">
-        <v>307</v>
-      </c>
-      <c r="K129" t="s">
-        <v>74</v>
-      </c>
-      <c r="L129" t="s">
-        <v>307</v>
-      </c>
-      <c r="M129" t="s">
-        <v>48</v>
-      </c>
-      <c r="N129" t="s">
-        <v>307</v>
-      </c>
-      <c r="O129" t="s">
-        <v>323</v>
-      </c>
-      <c r="P129" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="130" spans="1:16">
-      <c r="A130" t="s">
-        <v>96</v>
-      </c>
-      <c r="D130">
-        <v>1</v>
-      </c>
-      <c r="E130" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="131" spans="1:16">
-      <c r="A131" t="s">
-        <v>96</v>
-      </c>
-      <c r="D131" t="s">
-        <v>169</v>
-      </c>
-      <c r="E131" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="132" spans="1:16">
-      <c r="A132" t="s">
-        <v>96</v>
-      </c>
-      <c r="B132" t="s">
-        <v>85</v>
-      </c>
-      <c r="C132" t="s">
-        <v>261</v>
-      </c>
-      <c r="D132">
-        <v>0</v>
-      </c>
-      <c r="E132" t="s">
-        <v>225</v>
-      </c>
-      <c r="F132" t="s">
-        <v>365</v>
-      </c>
-      <c r="G132" t="s">
-        <v>66</v>
-      </c>
-      <c r="H132" t="s">
-        <v>307</v>
-      </c>
-      <c r="I132" t="s">
-        <v>73</v>
-      </c>
-      <c r="J132" t="s">
-        <v>307</v>
-      </c>
-      <c r="K132" t="s">
-        <v>74</v>
-      </c>
-      <c r="L132" t="s">
-        <v>307</v>
-      </c>
-      <c r="M132" t="s">
-        <v>48</v>
-      </c>
-      <c r="N132" t="s">
-        <v>307</v>
-      </c>
-      <c r="O132" t="s">
-        <v>323</v>
-      </c>
-      <c r="P132" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="133" spans="1:16">
       <c r="A133" t="s">
         <v>96</v>
       </c>
+      <c r="B133" t="s">
+        <v>84</v>
+      </c>
+      <c r="C133" t="s">
+        <v>261</v>
+      </c>
       <c r="D133">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E133" t="s">
-        <v>226</v>
+        <v>221</v>
+      </c>
+      <c r="F133" t="s">
+        <v>364</v>
+      </c>
+      <c r="G133" t="s">
+        <v>66</v>
+      </c>
+      <c r="H133" t="s">
+        <v>307</v>
+      </c>
+      <c r="I133" t="s">
+        <v>73</v>
+      </c>
+      <c r="J133" t="s">
+        <v>307</v>
+      </c>
+      <c r="K133" t="s">
+        <v>74</v>
+      </c>
+      <c r="L133" t="s">
+        <v>307</v>
+      </c>
+      <c r="M133" t="s">
+        <v>48</v>
+      </c>
+      <c r="N133" t="s">
+        <v>307</v>
+      </c>
+      <c r="O133" t="s">
+        <v>323</v>
+      </c>
+      <c r="P133" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="134" spans="1:16">
@@ -6100,10 +6139,10 @@
         <v>96</v>
       </c>
       <c r="D134">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E134" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="135" spans="1:16">
@@ -6114,7 +6153,7 @@
         <v>169</v>
       </c>
       <c r="E135" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="136" spans="1:16">
@@ -6122,7 +6161,7 @@
         <v>96</v>
       </c>
       <c r="B136" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C136" t="s">
         <v>261</v>
@@ -6131,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="E136" t="s">
-        <v>390</v>
+        <v>225</v>
       </c>
       <c r="F136" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="G136" t="s">
         <v>66</v>
@@ -6155,13 +6194,13 @@
         <v>307</v>
       </c>
       <c r="M136" t="s">
-        <v>325</v>
+        <v>48</v>
       </c>
       <c r="N136" t="s">
         <v>307</v>
       </c>
       <c r="O136" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="P136" t="s">
         <v>307</v>
@@ -6175,7 +6214,7 @@
         <v>1</v>
       </c>
       <c r="E137" t="s">
-        <v>391</v>
+        <v>226</v>
       </c>
     </row>
     <row r="138" spans="1:16">
@@ -6186,79 +6225,79 @@
         <v>2</v>
       </c>
       <c r="E138" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="139" spans="1:16">
       <c r="A139" t="s">
         <v>96</v>
       </c>
-      <c r="D139">
-        <v>3</v>
+      <c r="D139" t="s">
+        <v>169</v>
       </c>
       <c r="E139" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="140" spans="1:16">
       <c r="A140" t="s">
         <v>96</v>
       </c>
-      <c r="D140" t="s">
-        <v>169</v>
+      <c r="B140" t="s">
+        <v>86</v>
+      </c>
+      <c r="C140" t="s">
+        <v>261</v>
+      </c>
+      <c r="D140">
+        <v>0</v>
       </c>
       <c r="E140" t="s">
-        <v>228</v>
+        <v>390</v>
+      </c>
+      <c r="F140" t="s">
+        <v>366</v>
+      </c>
+      <c r="G140" t="s">
+        <v>66</v>
+      </c>
+      <c r="H140" t="s">
+        <v>307</v>
+      </c>
+      <c r="I140" t="s">
+        <v>73</v>
+      </c>
+      <c r="J140" t="s">
+        <v>307</v>
+      </c>
+      <c r="K140" t="s">
+        <v>74</v>
+      </c>
+      <c r="L140" t="s">
+        <v>307</v>
+      </c>
+      <c r="M140" t="s">
+        <v>325</v>
+      </c>
+      <c r="N140" t="s">
+        <v>307</v>
+      </c>
+      <c r="O140" t="s">
+        <v>326</v>
+      </c>
+      <c r="P140" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="141" spans="1:16">
       <c r="A141" t="s">
         <v>96</v>
       </c>
-      <c r="B141" t="s">
-        <v>87</v>
-      </c>
-      <c r="C141" t="s">
-        <v>261</v>
-      </c>
       <c r="D141">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E141" t="s">
-        <v>390</v>
-      </c>
-      <c r="F141" t="s">
-        <v>367</v>
-      </c>
-      <c r="G141" t="s">
-        <v>66</v>
-      </c>
-      <c r="H141" t="s">
-        <v>307</v>
-      </c>
-      <c r="I141" t="s">
-        <v>73</v>
-      </c>
-      <c r="J141" t="s">
-        <v>307</v>
-      </c>
-      <c r="K141" t="s">
-        <v>74</v>
-      </c>
-      <c r="L141" t="s">
-        <v>307</v>
-      </c>
-      <c r="M141" t="s">
-        <v>325</v>
-      </c>
-      <c r="N141" t="s">
-        <v>307</v>
-      </c>
-      <c r="O141" t="s">
-        <v>326</v>
-      </c>
-      <c r="P141" t="s">
-        <v>307</v>
+        <v>391</v>
       </c>
     </row>
     <row r="142" spans="1:16">
@@ -6266,10 +6305,10 @@
         <v>96</v>
       </c>
       <c r="D142">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E142" t="s">
-        <v>391</v>
+        <v>229</v>
       </c>
     </row>
     <row r="143" spans="1:16">
@@ -6277,266 +6316,305 @@
         <v>96</v>
       </c>
       <c r="D143">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E143" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="144" spans="1:16">
       <c r="A144" t="s">
         <v>96</v>
       </c>
-      <c r="D144">
+      <c r="D144" t="s">
+        <v>169</v>
+      </c>
+      <c r="E144" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="145" spans="1:16">
+      <c r="A145" t="s">
+        <v>96</v>
+      </c>
+      <c r="B145" t="s">
+        <v>87</v>
+      </c>
+      <c r="C145" t="s">
+        <v>261</v>
+      </c>
+      <c r="D145">
+        <v>0</v>
+      </c>
+      <c r="E145" t="s">
+        <v>390</v>
+      </c>
+      <c r="F145" t="s">
+        <v>367</v>
+      </c>
+      <c r="G145" t="s">
+        <v>66</v>
+      </c>
+      <c r="H145" t="s">
+        <v>307</v>
+      </c>
+      <c r="I145" t="s">
+        <v>73</v>
+      </c>
+      <c r="J145" t="s">
+        <v>307</v>
+      </c>
+      <c r="K145" t="s">
+        <v>74</v>
+      </c>
+      <c r="L145" t="s">
+        <v>307</v>
+      </c>
+      <c r="M145" t="s">
+        <v>325</v>
+      </c>
+      <c r="N145" t="s">
+        <v>307</v>
+      </c>
+      <c r="O145" t="s">
+        <v>326</v>
+      </c>
+      <c r="P145" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="146" spans="1:16">
+      <c r="A146" t="s">
+        <v>96</v>
+      </c>
+      <c r="D146">
+        <v>1</v>
+      </c>
+      <c r="E146" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="147" spans="1:16">
+      <c r="A147" t="s">
+        <v>96</v>
+      </c>
+      <c r="D147">
+        <v>2</v>
+      </c>
+      <c r="E147" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="148" spans="1:16">
+      <c r="A148" t="s">
+        <v>96</v>
+      </c>
+      <c r="D148">
         <v>3</v>
       </c>
-      <c r="E144" t="s">
+      <c r="E148" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="145" spans="1:12">
-      <c r="A145" t="s">
-        <v>96</v>
-      </c>
-      <c r="D145" t="s">
+    <row r="149" spans="1:16">
+      <c r="A149" t="s">
+        <v>96</v>
+      </c>
+      <c r="D149" t="s">
         <v>169</v>
       </c>
-      <c r="E145" t="s">
+      <c r="E149" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="146" spans="1:12">
-      <c r="A146" t="s">
-        <v>96</v>
-      </c>
-      <c r="B146" t="s">
+    <row r="150" spans="1:16">
+      <c r="A150" t="s">
+        <v>96</v>
+      </c>
+      <c r="B150" t="s">
         <v>89</v>
       </c>
-      <c r="C146" t="s">
+      <c r="C150" t="s">
         <v>261</v>
       </c>
-      <c r="D146">
+      <c r="D150">
         <v>0</v>
       </c>
-      <c r="E146" t="s">
+      <c r="E150" t="s">
         <v>390</v>
       </c>
-      <c r="F146" t="s">
+      <c r="F150" t="s">
         <v>368</v>
       </c>
-      <c r="G146" t="s">
+      <c r="G150" t="s">
         <v>66</v>
       </c>
-      <c r="H146" t="s">
+      <c r="H150" t="s">
         <v>327</v>
       </c>
-      <c r="I146" t="s">
+      <c r="I150" t="s">
         <v>86</v>
       </c>
-      <c r="J146" t="s">
-        <v>307</v>
-      </c>
-      <c r="K146" t="s">
+      <c r="J150" t="s">
+        <v>307</v>
+      </c>
+      <c r="K150" t="s">
         <v>87</v>
       </c>
-      <c r="L146" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="147" spans="1:12">
-      <c r="A147" t="s">
-        <v>96</v>
-      </c>
-      <c r="D147">
+      <c r="L150" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="151" spans="1:16">
+      <c r="A151" t="s">
+        <v>96</v>
+      </c>
+      <c r="D151">
         <v>1</v>
       </c>
-      <c r="E147" t="s">
+      <c r="E151" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="148" spans="1:12">
-      <c r="A148" t="s">
-        <v>96</v>
-      </c>
-      <c r="D148">
+    <row r="152" spans="1:16">
+      <c r="A152" t="s">
+        <v>96</v>
+      </c>
+      <c r="D152">
         <v>2</v>
       </c>
-      <c r="E148" t="s">
+      <c r="E152" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="149" spans="1:12">
-      <c r="A149" t="s">
-        <v>96</v>
-      </c>
-      <c r="D149">
+    <row r="153" spans="1:16">
+      <c r="A153" t="s">
+        <v>96</v>
+      </c>
+      <c r="D153">
         <v>3</v>
       </c>
-      <c r="E149" t="s">
+      <c r="E153" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="150" spans="1:12">
-      <c r="A150" t="s">
-        <v>96</v>
-      </c>
-      <c r="D150" t="s">
+    <row r="154" spans="1:16">
+      <c r="A154" t="s">
+        <v>96</v>
+      </c>
+      <c r="D154" t="s">
         <v>169</v>
       </c>
-      <c r="E150" t="s">
+      <c r="E154" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="151" spans="1:12">
-      <c r="A151" t="s">
-        <v>96</v>
-      </c>
-      <c r="B151" t="s">
+    <row r="155" spans="1:16">
+      <c r="A155" t="s">
+        <v>96</v>
+      </c>
+      <c r="B155" t="s">
         <v>90</v>
       </c>
-      <c r="C151" t="s">
+      <c r="C155" t="s">
         <v>261</v>
       </c>
-      <c r="D151">
+      <c r="D155">
         <v>0</v>
       </c>
-      <c r="E151" t="s">
+      <c r="E155" t="s">
         <v>235</v>
       </c>
-      <c r="F151" t="s">
+      <c r="F155" t="s">
         <v>369</v>
       </c>
-      <c r="G151" t="s">
+      <c r="G155" t="s">
         <v>66</v>
       </c>
-      <c r="H151" t="s">
-        <v>307</v>
-      </c>
-      <c r="I151" t="s">
+      <c r="H155" t="s">
+        <v>307</v>
+      </c>
+      <c r="I155" t="s">
         <v>328</v>
       </c>
-      <c r="J151" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="152" spans="1:12">
-      <c r="A152" t="s">
-        <v>96</v>
-      </c>
-      <c r="D152">
+      <c r="J155" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="156" spans="1:16">
+      <c r="A156" t="s">
+        <v>96</v>
+      </c>
+      <c r="D156">
         <v>1</v>
       </c>
-      <c r="E152" t="s">
+      <c r="E156" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="153" spans="1:12">
-      <c r="A153" t="s">
-        <v>96</v>
-      </c>
-      <c r="D153" t="s">
+    <row r="157" spans="1:16">
+      <c r="A157" t="s">
+        <v>96</v>
+      </c>
+      <c r="D157" t="s">
         <v>169</v>
       </c>
-      <c r="E153" t="s">
+      <c r="E157" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="154" spans="1:12">
-      <c r="A154" t="s">
-        <v>96</v>
-      </c>
-      <c r="B154" t="s">
+    <row r="158" spans="1:16">
+      <c r="A158" t="s">
+        <v>96</v>
+      </c>
+      <c r="B158" t="s">
         <v>91</v>
       </c>
-      <c r="C154" t="s">
+      <c r="C158" t="s">
         <v>261</v>
       </c>
-      <c r="D154">
+      <c r="D158">
         <v>0</v>
       </c>
-      <c r="E154" t="s">
+      <c r="E158" t="s">
         <v>233</v>
       </c>
-      <c r="F154" t="s">
+      <c r="F158" t="s">
         <v>370</v>
       </c>
-      <c r="G154" t="s">
+      <c r="G158" t="s">
         <v>66</v>
       </c>
-      <c r="H154" t="s">
-        <v>307</v>
-      </c>
-      <c r="I154" t="s">
+      <c r="H158" t="s">
+        <v>307</v>
+      </c>
+      <c r="I158" t="s">
         <v>329</v>
       </c>
-      <c r="J154" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="155" spans="1:12">
-      <c r="A155" t="s">
-        <v>96</v>
-      </c>
-      <c r="D155">
+      <c r="J158" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="159" spans="1:16">
+      <c r="A159" t="s">
+        <v>96</v>
+      </c>
+      <c r="D159">
         <v>1</v>
       </c>
-      <c r="E155" t="s">
+      <c r="E159" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="156" spans="1:12">
-      <c r="A156" t="s">
-        <v>96</v>
-      </c>
-      <c r="D156">
+    <row r="160" spans="1:16">
+      <c r="A160" t="s">
+        <v>96</v>
+      </c>
+      <c r="D160">
         <v>2</v>
       </c>
-      <c r="E156" t="s">
+      <c r="E160" t="s">
         <v>238</v>
-      </c>
-    </row>
-    <row r="157" spans="1:12">
-      <c r="A157" t="s">
-        <v>96</v>
-      </c>
-      <c r="D157">
-        <v>3</v>
-      </c>
-      <c r="E157" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="158" spans="1:12">
-      <c r="A158" t="s">
-        <v>96</v>
-      </c>
-      <c r="D158">
-        <v>4</v>
-      </c>
-      <c r="E158" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="159" spans="1:12">
-      <c r="A159" t="s">
-        <v>96</v>
-      </c>
-      <c r="D159">
-        <v>5</v>
-      </c>
-      <c r="E159" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="160" spans="1:12">
-      <c r="A160" t="s">
-        <v>96</v>
-      </c>
-      <c r="D160">
-        <v>6</v>
-      </c>
-      <c r="E160" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="161" spans="1:12">
@@ -6544,53 +6622,32 @@
         <v>96</v>
       </c>
       <c r="D161">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E161" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="162" spans="1:12">
       <c r="A162" t="s">
         <v>96</v>
       </c>
-      <c r="D162" t="s">
-        <v>169</v>
+      <c r="D162">
+        <v>4</v>
       </c>
       <c r="E162" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="163" spans="1:12">
       <c r="A163" t="s">
         <v>96</v>
       </c>
-      <c r="B163" t="s">
-        <v>92</v>
-      </c>
-      <c r="C163" t="s">
-        <v>261</v>
-      </c>
       <c r="D163">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E163" t="s">
-        <v>245</v>
-      </c>
-      <c r="F163" t="s">
-        <v>371</v>
-      </c>
-      <c r="G163" t="s">
-        <v>66</v>
-      </c>
-      <c r="H163" t="s">
-        <v>307</v>
-      </c>
-      <c r="I163" t="s">
-        <v>329</v>
-      </c>
-      <c r="J163" t="s">
-        <v>307</v>
+        <v>241</v>
       </c>
     </row>
     <row r="164" spans="1:12">
@@ -6598,10 +6655,10 @@
         <v>96</v>
       </c>
       <c r="D164">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E164" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
     </row>
     <row r="165" spans="1:12">
@@ -6609,32 +6666,53 @@
         <v>96</v>
       </c>
       <c r="D165">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E165" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
     </row>
     <row r="166" spans="1:12">
       <c r="A166" t="s">
         <v>96</v>
       </c>
-      <c r="D166">
-        <v>3</v>
+      <c r="D166" t="s">
+        <v>169</v>
       </c>
       <c r="E166" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="167" spans="1:12">
       <c r="A167" t="s">
         <v>96</v>
       </c>
+      <c r="B167" t="s">
+        <v>92</v>
+      </c>
+      <c r="C167" t="s">
+        <v>261</v>
+      </c>
       <c r="D167">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E167" t="s">
-        <v>249</v>
+        <v>245</v>
+      </c>
+      <c r="F167" t="s">
+        <v>371</v>
+      </c>
+      <c r="G167" t="s">
+        <v>66</v>
+      </c>
+      <c r="H167" t="s">
+        <v>307</v>
+      </c>
+      <c r="I167" t="s">
+        <v>329</v>
+      </c>
+      <c r="J167" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="168" spans="1:12">
@@ -6642,59 +6720,32 @@
         <v>96</v>
       </c>
       <c r="D168">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E168" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
     </row>
     <row r="169" spans="1:12">
       <c r="A169" t="s">
         <v>96</v>
       </c>
-      <c r="D169" t="s">
-        <v>169</v>
+      <c r="D169">
+        <v>2</v>
       </c>
       <c r="E169" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="170" spans="1:12">
       <c r="A170" t="s">
         <v>96</v>
       </c>
-      <c r="B170" t="s">
-        <v>93</v>
-      </c>
-      <c r="C170" t="s">
-        <v>261</v>
-      </c>
       <c r="D170">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E170" t="s">
-        <v>251</v>
-      </c>
-      <c r="F170" t="s">
-        <v>373</v>
-      </c>
-      <c r="G170" t="s">
-        <v>66</v>
-      </c>
-      <c r="H170" t="s">
-        <v>307</v>
-      </c>
-      <c r="I170" t="s">
-        <v>330</v>
-      </c>
-      <c r="J170" t="s">
-        <v>307</v>
-      </c>
-      <c r="K170" t="s">
-        <v>331</v>
-      </c>
-      <c r="L170" t="s">
-        <v>307</v>
+        <v>248</v>
       </c>
     </row>
     <row r="171" spans="1:12">
@@ -6702,10 +6753,10 @@
         <v>96</v>
       </c>
       <c r="D171">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E171" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="172" spans="1:12">
@@ -6713,10 +6764,10 @@
         <v>96</v>
       </c>
       <c r="D172">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E172" t="s">
-        <v>372</v>
+        <v>250</v>
       </c>
     </row>
     <row r="173" spans="1:12">
@@ -6727,6 +6778,77 @@
         <v>169</v>
       </c>
       <c r="E173" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="174" spans="1:12">
+      <c r="A174" t="s">
+        <v>96</v>
+      </c>
+      <c r="B174" t="s">
+        <v>93</v>
+      </c>
+      <c r="C174" t="s">
+        <v>261</v>
+      </c>
+      <c r="D174">
+        <v>0</v>
+      </c>
+      <c r="E174" t="s">
+        <v>251</v>
+      </c>
+      <c r="F174" t="s">
+        <v>373</v>
+      </c>
+      <c r="G174" t="s">
+        <v>66</v>
+      </c>
+      <c r="H174" t="s">
+        <v>307</v>
+      </c>
+      <c r="I174" t="s">
+        <v>330</v>
+      </c>
+      <c r="J174" t="s">
+        <v>307</v>
+      </c>
+      <c r="K174" t="s">
+        <v>331</v>
+      </c>
+      <c r="L174" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="175" spans="1:12">
+      <c r="A175" t="s">
+        <v>96</v>
+      </c>
+      <c r="D175">
+        <v>1</v>
+      </c>
+      <c r="E175" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="176" spans="1:12">
+      <c r="A176" t="s">
+        <v>96</v>
+      </c>
+      <c r="D176">
+        <v>2</v>
+      </c>
+      <c r="E176" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5">
+      <c r="A177" t="s">
+        <v>96</v>
+      </c>
+      <c r="D177" t="s">
+        <v>169</v>
+      </c>
+      <c r="E177" t="s">
         <v>253</v>
       </c>
     </row>
@@ -6738,7 +6860,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9521944E-28B4-4113-A27F-3B841E118807}">
-  <dimension ref="A1:AP51"/>
+  <dimension ref="A1:AQ52"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
@@ -6746,26 +6868,26 @@
     <col min="4" max="6" width="8.6328125" customWidth="1"/>
     <col min="15" max="15" width="8.6328125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.36328125" customWidth="1"/>
-    <col min="27" max="27" width="11.08984375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="9.26953125" customWidth="1"/>
-    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="8.6328125" customWidth="1"/>
-    <col min="37" max="37" width="9.26953125" customWidth="1"/>
-    <col min="38" max="38" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="18" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="8.7265625" style="11"/>
+    <col min="23" max="23" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.36328125" customWidth="1"/>
+    <col min="28" max="28" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="9.26953125" customWidth="1"/>
+    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="8.6328125" customWidth="1"/>
+    <col min="38" max="38" width="9.26953125" customWidth="1"/>
+    <col min="39" max="39" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="18" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="8.7265625" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" s="2" customFormat="1" ht="30" customHeight="1">
+    <row r="1" spans="1:43" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A1" s="18" t="s">
         <v>392</v>
       </c>
@@ -6827,477 +6949,486 @@
         <v>66</v>
       </c>
       <c r="U1" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="V1" s="2" t="s">
         <v>497</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AA1" s="17" t="s">
+      <c r="AB1" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>379</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="AP1" s="19" t="s">
+      <c r="AQ1" s="19" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="2" spans="1:42">
+    <row r="2" spans="1:43">
       <c r="A2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:42">
+    <row r="3" spans="1:43">
       <c r="A3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:42">
+    <row r="4" spans="1:43">
       <c r="A4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:42">
+    <row r="5" spans="1:43">
       <c r="A5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:42">
+    <row r="6" spans="1:43">
       <c r="A6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:42">
+    <row r="7" spans="1:43">
       <c r="A7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:42">
+    <row r="8" spans="1:43">
       <c r="A8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:42">
+    <row r="9" spans="1:43">
       <c r="A9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:42">
+    <row r="10" spans="1:43">
       <c r="A10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:42">
+    <row r="11" spans="1:43">
       <c r="A11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:42">
+    <row r="12" spans="1:43">
       <c r="A12" t="s">
         <v>15</v>
       </c>
-      <c r="AE12" s="16"/>
-      <c r="AO12" s="16"/>
-      <c r="AP12" s="11" t="s">
+      <c r="U12" s="16"/>
+      <c r="AF12" s="16"/>
+      <c r="AP12" s="16"/>
+      <c r="AQ12" s="11" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="13" spans="1:42">
+    <row r="13" spans="1:43">
       <c r="A13" t="s">
         <v>386</v>
       </c>
       <c r="L13" s="23"/>
-      <c r="AO13" s="16"/>
-    </row>
-    <row r="14" spans="1:42">
+      <c r="AP13" s="16"/>
+    </row>
+    <row r="14" spans="1:43">
       <c r="A14" t="s">
         <v>60</v>
       </c>
       <c r="R14" s="16"/>
-      <c r="AA14" s="23" t="s">
+      <c r="AB14" s="23" t="s">
         <v>395</v>
       </c>
-      <c r="AD14" s="16"/>
       <c r="AE14" s="16"/>
-      <c r="AO14" s="16"/>
-    </row>
-    <row r="15" spans="1:42">
+      <c r="AF14" s="16"/>
+      <c r="AP14" s="16"/>
+    </row>
+    <row r="15" spans="1:43">
       <c r="A15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:42">
+    <row r="16" spans="1:43">
       <c r="A16" t="s">
         <v>62</v>
       </c>
-      <c r="AN16" s="16"/>
-    </row>
-    <row r="17" spans="1:41">
+      <c r="AO16" s="16"/>
+    </row>
+    <row r="17" spans="1:42">
       <c r="A17" t="s">
         <v>63</v>
       </c>
-      <c r="AN17" s="16"/>
-    </row>
-    <row r="18" spans="1:41">
+      <c r="AO17" s="16"/>
+    </row>
+    <row r="18" spans="1:42">
       <c r="A18" t="s">
         <v>64</v>
       </c>
       <c r="P18" s="16"/>
       <c r="Q18" s="16"/>
-      <c r="AN18" s="16"/>
-    </row>
-    <row r="19" spans="1:41">
+      <c r="AO18" s="16"/>
+    </row>
+    <row r="19" spans="1:42">
       <c r="A19" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:41">
+    <row r="20" spans="1:42">
       <c r="A20" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:41">
+    <row r="21" spans="1:42">
       <c r="A21" t="s">
+        <v>505</v>
+      </c>
+      <c r="AO21" s="16"/>
+    </row>
+    <row r="22" spans="1:42">
+      <c r="A22" t="s">
         <v>497</v>
       </c>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
-      <c r="Q21" s="16"/>
-      <c r="AN21" s="16"/>
-    </row>
-    <row r="22" spans="1:41">
-      <c r="A22" t="s">
-        <v>69</v>
-      </c>
-      <c r="L22" s="23"/>
+      <c r="L22" s="16"/>
       <c r="M22" s="16"/>
       <c r="Q22" s="16"/>
-      <c r="AN22" s="16"/>
-    </row>
-    <row r="23" spans="1:41">
+      <c r="AO22" s="16"/>
+    </row>
+    <row r="23" spans="1:42">
       <c r="A23" t="s">
+        <v>69</v>
+      </c>
+      <c r="L23" s="23"/>
+      <c r="M23" s="16"/>
+      <c r="Q23" s="16"/>
+      <c r="AO23" s="16"/>
+    </row>
+    <row r="24" spans="1:42">
+      <c r="A24" t="s">
         <v>71</v>
       </c>
-      <c r="N23" s="16" t="s">
+      <c r="N24" s="16" t="s">
         <v>419</v>
       </c>
-      <c r="Q23" s="16" t="s">
+      <c r="Q24" s="16" t="s">
         <v>418</v>
       </c>
-      <c r="AA23" s="15" t="s">
+      <c r="AB24" s="15" t="s">
         <v>416</v>
       </c>
-      <c r="AB23" s="16" t="s">
+      <c r="AC24" s="16" t="s">
         <v>433</v>
       </c>
-      <c r="AE23" s="16" t="s">
+      <c r="AF24" s="16" t="s">
         <v>417</v>
       </c>
-      <c r="AN23" s="16"/>
-    </row>
-    <row r="24" spans="1:41">
-      <c r="A24" t="s">
+      <c r="AO24" s="16"/>
+    </row>
+    <row r="25" spans="1:42">
+      <c r="A25" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="25" spans="1:41">
-      <c r="A25" t="s">
+    <row r="26" spans="1:42">
+      <c r="A26" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="26" spans="1:41">
-      <c r="A26" t="s">
+    <row r="27" spans="1:42">
+      <c r="A27" t="s">
         <v>75</v>
       </c>
-      <c r="P26" s="16"/>
-      <c r="AB26" s="16"/>
-      <c r="AN26" s="16"/>
-    </row>
-    <row r="27" spans="1:41">
-      <c r="A27" t="s">
+      <c r="P27" s="16"/>
+      <c r="AC27" s="16"/>
+      <c r="AO27" s="16"/>
+    </row>
+    <row r="28" spans="1:42">
+      <c r="A28" t="s">
         <v>77</v>
       </c>
-      <c r="R27" s="16" t="s">
+      <c r="R28" s="16" t="s">
         <v>424</v>
       </c>
-      <c r="U27" s="16"/>
-      <c r="V27" s="16" t="s">
+      <c r="V28" s="16"/>
+      <c r="W28" s="16" t="s">
         <v>420</v>
       </c>
-      <c r="AN27" s="16"/>
-      <c r="AO27" s="16"/>
-    </row>
-    <row r="28" spans="1:41">
-      <c r="A28" t="s">
+      <c r="AO28" s="16"/>
+      <c r="AP28" s="16"/>
+    </row>
+    <row r="29" spans="1:42">
+      <c r="A29" t="s">
         <v>78</v>
       </c>
-      <c r="P28" s="16" t="s">
+      <c r="P29" s="16" t="s">
         <v>430</v>
       </c>
-      <c r="W28" s="16"/>
-      <c r="AJ28" s="16" t="s">
+      <c r="X29" s="16"/>
+      <c r="AK29" s="16" t="s">
         <v>431</v>
       </c>
-      <c r="AK28" s="16"/>
-      <c r="AL28" s="16" t="s">
+      <c r="AL29" s="16"/>
+      <c r="AM29" s="16" t="s">
         <v>432</v>
       </c>
-      <c r="AO28" s="16"/>
-    </row>
-    <row r="29" spans="1:41">
-      <c r="A29" t="s">
+      <c r="AP29" s="16"/>
+    </row>
+    <row r="30" spans="1:42">
+      <c r="A30" t="s">
         <v>79</v>
       </c>
-      <c r="R29" s="16"/>
-      <c r="AA29" s="23"/>
-    </row>
-    <row r="30" spans="1:41">
-      <c r="A30" t="s">
+      <c r="R30" s="16"/>
+      <c r="AB30" s="23"/>
+    </row>
+    <row r="31" spans="1:42">
+      <c r="A31" t="s">
         <v>80</v>
       </c>
-      <c r="R30" s="16"/>
-      <c r="AA30" s="24" t="s">
+      <c r="R31" s="16"/>
+      <c r="AB31" s="24" t="s">
         <v>476</v>
       </c>
-      <c r="AE30" s="16" t="s">
+      <c r="AF31" s="16" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="31" spans="1:41">
-      <c r="A31" t="s">
+    <row r="32" spans="1:42">
+      <c r="A32" t="s">
         <v>84</v>
       </c>
-      <c r="L31" s="26"/>
-      <c r="R31" s="16" t="s">
+      <c r="R32" s="16" t="s">
         <v>435</v>
       </c>
-      <c r="AA31" s="23" t="s">
+      <c r="AB32" s="23" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="32" spans="1:41">
-      <c r="A32" t="s">
+    <row r="33" spans="1:42">
+      <c r="A33" t="s">
         <v>85</v>
       </c>
-      <c r="AJ32" s="16" t="s">
+      <c r="AK33" s="16" t="s">
         <v>426</v>
       </c>
-      <c r="AK32" s="16" t="s">
+      <c r="AL33" s="16" t="s">
         <v>427</v>
       </c>
-      <c r="AL32" s="16" t="s">
+      <c r="AM33" s="16" t="s">
         <v>428</v>
       </c>
-      <c r="AM32" s="16" t="s">
+      <c r="AN33" s="16" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="33" spans="1:41">
-      <c r="A33" t="s">
+    <row r="34" spans="1:42">
+      <c r="A34" t="s">
         <v>86</v>
       </c>
-      <c r="U33" s="16"/>
-      <c r="V33" s="16"/>
-      <c r="AA33" s="23" t="s">
+      <c r="V34" s="16"/>
+      <c r="W34" s="16"/>
+      <c r="AB34" s="23" t="s">
         <v>438</v>
       </c>
-      <c r="AC33" s="16"/>
-      <c r="AI33" s="16"/>
-      <c r="AO33" s="16"/>
-    </row>
-    <row r="34" spans="1:41">
-      <c r="A34" t="s">
+      <c r="AD34" s="16"/>
+      <c r="AJ34" s="16"/>
+      <c r="AP34" s="16"/>
+    </row>
+    <row r="35" spans="1:42">
+      <c r="A35" t="s">
         <v>87</v>
       </c>
-      <c r="U34" s="16"/>
-      <c r="V34" s="16"/>
-      <c r="AA34" s="23" t="s">
+      <c r="V35" s="16"/>
+      <c r="W35" s="16"/>
+      <c r="AB35" s="23" t="s">
         <v>437</v>
       </c>
-      <c r="AD34" s="16"/>
-      <c r="AE34" s="16"/>
-      <c r="AI34" s="16"/>
-      <c r="AO34" s="16"/>
-    </row>
-    <row r="35" spans="1:41" ht="14" customHeight="1">
-      <c r="A35" t="s">
+      <c r="AE35" s="16"/>
+      <c r="AF35" s="16"/>
+      <c r="AJ35" s="16"/>
+      <c r="AP35" s="16"/>
+    </row>
+    <row r="36" spans="1:42" ht="14" customHeight="1">
+      <c r="A36" t="s">
         <v>89</v>
       </c>
-      <c r="Q35" s="16" t="s">
+      <c r="Q36" s="16" t="s">
         <v>422</v>
       </c>
-      <c r="U35" s="16"/>
-      <c r="V35" s="16" t="s">
+      <c r="V36" s="16"/>
+      <c r="W36" s="16" t="s">
         <v>423</v>
       </c>
-      <c r="AA35" s="23" t="s">
+      <c r="AB36" s="23" t="s">
         <v>439</v>
       </c>
-      <c r="AE35" s="16" t="s">
+      <c r="AF36" s="16" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="36" spans="1:41">
-      <c r="A36" t="s">
+    <row r="37" spans="1:42">
+      <c r="A37" t="s">
         <v>90</v>
       </c>
-      <c r="AO36" s="16"/>
-    </row>
-    <row r="37" spans="1:41">
-      <c r="A37" t="s">
+      <c r="AP37" s="16"/>
+    </row>
+    <row r="38" spans="1:42">
+      <c r="A38" t="s">
         <v>91</v>
       </c>
-      <c r="AO37" s="16"/>
-    </row>
-    <row r="38" spans="1:41">
-      <c r="A38" t="s">
+      <c r="AP38" s="16"/>
+    </row>
+    <row r="39" spans="1:42">
+      <c r="A39" t="s">
         <v>92</v>
       </c>
-      <c r="AO38" s="16"/>
-    </row>
-    <row r="39" spans="1:41">
-      <c r="A39" t="s">
+      <c r="AP39" s="16"/>
+    </row>
+    <row r="40" spans="1:42">
+      <c r="A40" t="s">
         <v>93</v>
       </c>
-      <c r="AJ39" s="16" t="s">
+      <c r="AK40" s="16" t="s">
         <v>429</v>
       </c>
-      <c r="AO39" s="16"/>
-    </row>
-    <row r="40" spans="1:41">
-      <c r="A40" t="s">
+      <c r="AP40" s="16"/>
+    </row>
+    <row r="41" spans="1:42">
+      <c r="A41" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="41" spans="1:41">
-      <c r="A41" t="s">
+    <row r="42" spans="1:42">
+      <c r="A42" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="43" spans="1:41" s="11" customFormat="1">
-      <c r="A43" s="11" t="s">
+    <row r="44" spans="1:42" s="11" customFormat="1">
+      <c r="A44" s="11" t="s">
         <v>456</v>
       </c>
     </row>
-    <row r="45" spans="1:41">
-      <c r="B45" s="12" t="s">
+    <row r="46" spans="1:42">
+      <c r="B46" s="12" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="46" spans="1:41">
-      <c r="A46" s="12"/>
-      <c r="B46" s="13"/>
-      <c r="C46" t="s">
+    <row r="47" spans="1:42">
+      <c r="A47" s="12"/>
+      <c r="B47" s="13"/>
+      <c r="C47" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="47" spans="1:41">
-      <c r="B47" s="14"/>
-      <c r="C47" t="s">
+    <row r="48" spans="1:42">
+      <c r="B48" s="14"/>
+      <c r="C48" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="48" spans="1:41">
-      <c r="B48" s="15"/>
-      <c r="C48" t="s">
+    <row r="49" spans="2:3">
+      <c r="B49" s="15"/>
+      <c r="C49" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="49" spans="2:3">
-      <c r="B49" s="16"/>
-      <c r="C49" t="s">
+    <row r="50" spans="2:3">
+      <c r="B50" s="16"/>
+      <c r="C50" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="50" spans="2:3">
-      <c r="B50" s="1" t="s">
+    <row r="51" spans="2:3">
+      <c r="B51" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C51" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="51" spans="2:3">
-      <c r="B51" s="23"/>
-      <c r="C51" t="s">
+    <row r="52" spans="2:3">
+      <c r="B52" s="23"/>
+      <c r="C52" t="s">
         <v>477</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B32:AL32">
+  <conditionalFormatting sqref="B33:AM33">
     <cfRule type="expression" dxfId="4" priority="3">
-      <formula>$A32=B$1</formula>
+      <formula>$A33=B$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:AO22 B2:M23 N23:AM23 AO23 B24:AO26 W27:AM27 B27:V28 X28:AO28 B29:Z31 AB29:AO31 AM32:AO33 AB33:AK33 B33:Z36 AB34:AO36 B37:AO42 B49">
+  <conditionalFormatting sqref="N2:AP23 B2:M24 N24:AN24 AP24 B25:AP27 X28:AN28 B28:W29 Y29:AP29 B30:AA32 AC30:AP32 AN33:AP34 AC34:AL34 B34:AA37 AC35:AP37 B38:AP43 B50">
     <cfRule type="expression" dxfId="3" priority="60">
       <formula>$A2=B$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W28">
+  <conditionalFormatting sqref="X29">
     <cfRule type="expression" dxfId="2" priority="7">
-      <formula>$A28=#REF!</formula>
+      <formula>$A29=#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA35">
+  <conditionalFormatting sqref="AB36">
     <cfRule type="expression" dxfId="1" priority="1">
-      <formula>$A35=AA$1</formula>
+      <formula>$A36=AB$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AN23 AN27:AO27">
+  <conditionalFormatting sqref="AO24 AO28:AP28">
     <cfRule type="expression" dxfId="0" priority="9">
-      <formula>#REF!=AN$1</formula>
+      <formula>#REF!=AO$1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add {05_investigating_interdependence.qmd} {codebook.xslsx} added some plots for investigating interdependence and recorded the changes in the codebook
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Vaccine Uptake - R\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6915FECE-D1A6-4DC2-BD61-03A4E3D7C71E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7978386-E350-483A-9296-E0D5D3005E96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10890" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1480" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1520" uniqueCount="539">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -1536,9 +1536,6 @@
     <t>The slope for partial uptake for mothers who are self/family employed differs from the others</t>
   </si>
   <si>
-    <t>is the difference in slopes for mothers who are home employed to be considered effect modification? Esp w a small sample size</t>
-  </si>
-  <si>
     <t>The differring slopes of uptake against income  for different mother_stay_home</t>
   </si>
   <si>
@@ -1645,6 +1642,75 @@
   </si>
   <si>
     <t>child &gt; 12 y/o as of 2nd April 2023</t>
+  </si>
+  <si>
+    <t>child_sibligns</t>
+  </si>
+  <si>
+    <t>child_siblings*age_of_interest*age_cat (??)</t>
+  </si>
+  <si>
+    <t>The increase in full vaccination increases as the number of siblings increases</t>
+  </si>
+  <si>
+    <t>age_child_siblings_</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Followup</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>Having both a postgraduate mother and postgraduate father result in an increased slope</t>
+  </si>
+  <si>
+    <t>mother_highest_education(postgrad)*father_highest_education(postgrad)*test_household_income</t>
+  </si>
+  <si>
+    <t>father_highest_education(postgrad)*mother_highest_education(postgrad)</t>
+  </si>
+  <si>
+    <t>Both junior college/technical college parents results in a decreased uptake with income</t>
+  </si>
+  <si>
+    <t>father_highest_education(JCTC)*mother_highest_education(JCTC)*test_household_income</t>
+  </si>
+  <si>
+    <t>father_highest_education(JCTC)*mother_highest_education(JCTC)</t>
+  </si>
+  <si>
+    <t>father_highest_education(postgrad)</t>
+  </si>
+  <si>
+    <t>mother_highest_education(postgrad)</t>
+  </si>
+  <si>
+    <t>different slopes  for different age cats</t>
+  </si>
+  <si>
+    <t>age_cat*age_of_interest</t>
+  </si>
+  <si>
+    <t>Refer to new definitions of 0 0 employment status and stay home</t>
+  </si>
+  <si>
+    <t>Refer to ANOVA</t>
+  </si>
+  <si>
+    <t>having 2 parents for an child of an unmarried couple results in a greater increase than for having 2 parents of a child of a married couple</t>
+  </si>
+  <si>
+    <t>child_parents*test_parents_marital_status</t>
+  </si>
+  <si>
+    <t>Too little data to draw conclusions</t>
+  </si>
+  <si>
+    <t>child_parents_marital_status_</t>
   </si>
 </sst>
 </file>
@@ -1704,7 +1770,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1771,6 +1837,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1799,7 +1883,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1844,6 +1928,10 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2428,7 +2516,7 @@
         <v>15</v>
       </c>
       <c r="BK1" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="BL1" s="21" t="s">
         <v>67</v>
@@ -2440,7 +2528,7 @@
         <v>69</v>
       </c>
       <c r="BO1" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="BP1" s="4" t="s">
         <v>70</v>
@@ -2728,7 +2816,7 @@
         <v>96</v>
       </c>
       <c r="BO2" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="BP2" s="4" t="s">
         <v>96</v>
@@ -2940,7 +3028,7 @@
         <v>117</v>
       </c>
       <c r="BK3" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="BL3" s="22" t="s">
         <v>452</v>
@@ -2952,7 +3040,7 @@
         <v>451</v>
       </c>
       <c r="BO3" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="BP3" s="3" t="s">
         <v>134</v>
@@ -4655,7 +4743,7 @@
         <v>117</v>
       </c>
       <c r="F47" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="G47" t="s">
         <v>15</v>
@@ -4669,19 +4757,19 @@
         <v>96</v>
       </c>
       <c r="B48" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="C48" t="s">
         <v>261</v>
       </c>
       <c r="D48" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="E48" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="F48" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="G48" t="s">
         <v>15</v>
@@ -4701,13 +4789,13 @@
         <v>96</v>
       </c>
       <c r="D49" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="E49" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="F49" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -4715,13 +4803,13 @@
         <v>96</v>
       </c>
       <c r="D50" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="E50" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="F50" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -4735,7 +4823,7 @@
         <v>169</v>
       </c>
       <c r="F51" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="52" spans="1:12" s="4" customFormat="1">
@@ -4807,7 +4895,7 @@
         <v>96</v>
       </c>
       <c r="B54" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="C54" t="s">
         <v>260</v>
@@ -4816,10 +4904,10 @@
         <v>109</v>
       </c>
       <c r="E54" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="F54" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="G54" t="s">
         <v>68</v>
@@ -4854,7 +4942,7 @@
         <v>109</v>
       </c>
       <c r="E55" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="F55" t="s">
         <v>449</v>
@@ -6949,10 +7037,10 @@
         <v>66</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="W1" s="2" t="s">
         <v>69</v>
@@ -7135,16 +7223,17 @@
     </row>
     <row r="21" spans="1:42">
       <c r="A21" t="s">
-        <v>505</v>
-      </c>
+        <v>504</v>
+      </c>
+      <c r="L21" s="23"/>
       <c r="AO21" s="16"/>
     </row>
     <row r="22" spans="1:42">
       <c r="A22" t="s">
-        <v>497</v>
-      </c>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
+        <v>496</v>
+      </c>
+      <c r="L22" s="23"/>
+      <c r="M22" s="23"/>
       <c r="Q22" s="16"/>
       <c r="AO22" s="16"/>
     </row>
@@ -7153,7 +7242,7 @@
         <v>69</v>
       </c>
       <c r="L23" s="23"/>
-      <c r="M23" s="16"/>
+      <c r="M23" s="23"/>
       <c r="Q23" s="16"/>
       <c r="AO23" s="16"/>
     </row>
@@ -7161,7 +7250,7 @@
       <c r="A24" t="s">
         <v>71</v>
       </c>
-      <c r="N24" s="16" t="s">
+      <c r="N24" s="23" t="s">
         <v>419</v>
       </c>
       <c r="Q24" s="16" t="s">
@@ -7438,7 +7527,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313888EE-552D-40AA-8234-3B847E46EF43}">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="55.7265625" bestFit="1" customWidth="1"/>
@@ -7469,7 +7558,7 @@
         <v>462</v>
       </c>
       <c r="F1" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="G1" t="s">
         <v>458</v>
@@ -7480,16 +7569,19 @@
     </row>
     <row r="2" spans="1:10" ht="29">
       <c r="A2" t="s">
-        <v>490</v>
+        <v>489</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>522</v>
       </c>
       <c r="C2" t="s">
         <v>169</v>
       </c>
       <c r="D2" t="s">
+        <v>490</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>491</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>492</v>
       </c>
       <c r="F2" t="s">
         <v>169</v>
@@ -7505,6 +7597,9 @@
       <c r="A3" t="s">
         <v>466</v>
       </c>
+      <c r="B3" s="28" t="s">
+        <v>522</v>
+      </c>
       <c r="C3" t="s">
         <v>473</v>
       </c>
@@ -7512,10 +7607,10 @@
         <v>460</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="F3" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="G3" t="s">
         <v>475</v>
@@ -7531,6 +7626,9 @@
       </c>
     </row>
     <row r="4" spans="1:10" ht="43.5">
+      <c r="B4" s="27" t="s">
+        <v>521</v>
+      </c>
       <c r="C4" t="s">
         <v>471</v>
       </c>
@@ -7544,13 +7642,16 @@
         <v>468</v>
       </c>
       <c r="G4" t="s">
-        <v>87</v>
+        <v>530</v>
       </c>
       <c r="H4" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="43.5">
+      <c r="B5" s="27" t="s">
+        <v>521</v>
+      </c>
       <c r="C5" t="s">
         <v>471</v>
       </c>
@@ -7564,87 +7665,89 @@
         <v>469</v>
       </c>
       <c r="G5" t="s">
-        <v>86</v>
+        <v>529</v>
       </c>
       <c r="H5" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="43.5">
+      <c r="B6" s="29"/>
       <c r="C6" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="D6" t="s">
         <v>461</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>487</v>
+        <v>526</v>
       </c>
       <c r="F6" t="s">
-        <v>488</v>
+        <v>527</v>
       </c>
       <c r="G6" t="s">
-        <v>89</v>
+        <v>528</v>
       </c>
       <c r="H6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="29">
+    <row r="7" spans="1:10" ht="43.5">
+      <c r="B7" s="29"/>
       <c r="C7" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D7" t="s">
-        <v>474</v>
+        <v>461</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>481</v>
+        <v>523</v>
       </c>
       <c r="F7" t="s">
-        <v>482</v>
+        <v>524</v>
       </c>
       <c r="G7" t="s">
-        <v>84</v>
-      </c>
-      <c r="H7" t="s">
-        <v>77</v>
+        <v>525</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="43.5">
-      <c r="A8" s="2" t="s">
-        <v>480</v>
+      <c r="B8" s="26" t="s">
+        <v>520</v>
       </c>
       <c r="C8" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D8" t="s">
-        <v>478</v>
+        <v>461</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="F8" t="s">
-        <v>169</v>
+        <v>487</v>
       </c>
       <c r="G8" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H8" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="43.5">
+    <row r="9" spans="1:10" ht="29">
+      <c r="B9" s="28" t="s">
+        <v>522</v>
+      </c>
       <c r="C9" t="s">
-        <v>169</v>
+        <v>472</v>
       </c>
       <c r="D9" t="s">
-        <v>485</v>
+        <v>474</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="F9" t="s">
-        <v>169</v>
+        <v>481</v>
       </c>
       <c r="G9" t="s">
         <v>84</v>
@@ -7652,31 +7755,149 @@
       <c r="H9" t="s">
         <v>77</v>
       </c>
-      <c r="I9" t="s">
+    </row>
+    <row r="10" spans="1:10" ht="43.5">
+      <c r="A10" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>521</v>
+      </c>
+      <c r="C10" t="s">
+        <v>472</v>
+      </c>
+      <c r="D10" t="s">
+        <v>478</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="F10" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10" t="s">
+        <v>80</v>
+      </c>
+      <c r="H10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="43.5">
+      <c r="B11" s="28" t="s">
+        <v>522</v>
+      </c>
+      <c r="C11" t="s">
+        <v>169</v>
+      </c>
+      <c r="D11" t="s">
+        <v>484</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="F11" t="s">
+        <v>169</v>
+      </c>
+      <c r="G11" t="s">
+        <v>84</v>
+      </c>
+      <c r="H11" t="s">
+        <v>77</v>
+      </c>
+      <c r="I11" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="58">
-      <c r="A10" t="s">
+    <row r="12" spans="1:10" ht="58">
+      <c r="A12" t="s">
+        <v>494</v>
+      </c>
+      <c r="C12" t="s">
+        <v>473</v>
+      </c>
+      <c r="D12" t="s">
         <v>495</v>
       </c>
-      <c r="C10" t="s">
+      <c r="E12" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="F12" t="s">
+        <v>492</v>
+      </c>
+      <c r="G12" t="s">
+        <v>386</v>
+      </c>
+      <c r="H12" t="s">
+        <v>15</v>
+      </c>
+      <c r="I12" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="29">
+      <c r="A13" t="s">
+        <v>534</v>
+      </c>
+      <c r="C13" t="s">
         <v>473</v>
       </c>
-      <c r="D10" t="s">
-        <v>496</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>494</v>
-      </c>
-      <c r="F10" t="s">
-        <v>493</v>
-      </c>
-      <c r="G10" t="s">
-        <v>386</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="D13" t="s">
+        <v>519</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="F13" t="s">
+        <v>517</v>
+      </c>
+      <c r="G13" t="s">
+        <v>516</v>
+      </c>
+      <c r="H13" t="s">
         <v>15</v>
+      </c>
+      <c r="I13" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="C14" t="s">
+        <v>473</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="F14" t="s">
+        <v>532</v>
+      </c>
+      <c r="G14" t="s">
+        <v>504</v>
+      </c>
+      <c r="H14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="58">
+      <c r="A15" t="s">
+        <v>537</v>
+      </c>
+      <c r="C15" t="s">
+        <v>473</v>
+      </c>
+      <c r="D15" t="s">
+        <v>538</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="F15" t="s">
+        <v>536</v>
+      </c>
+      <c r="G15" t="s">
+        <v>71</v>
+      </c>
+      <c r="H15" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add (05_investigating_interdependence.R) added further plots in investigatin interactions
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Vaccine Uptake - R\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7978386-E350-483A-9296-E0D5D3005E96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7E2183F-ACD1-45AB-B261-AE85D2C528D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10890" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1520" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1595" uniqueCount="580">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -1698,9 +1698,6 @@
     <t>Refer to new definitions of 0 0 employment status and stay home</t>
   </si>
   <si>
-    <t>Refer to ANOVA</t>
-  </si>
-  <si>
     <t>having 2 parents for an child of an unmarried couple results in a greater increase than for having 2 parents of a child of a married couple</t>
   </si>
   <si>
@@ -1711,6 +1708,132 @@
   </si>
   <si>
     <t>child_parents_marital_status_</t>
+  </si>
+  <si>
+    <t>Refer to ANCOVA</t>
+  </si>
+  <si>
+    <t>vulnerable_indivs_child_grand_</t>
+  </si>
+  <si>
+    <t>vulnerable_individuals * child_grand</t>
+  </si>
+  <si>
+    <t>vulnerable_individauls</t>
+  </si>
+  <si>
+    <t>Having a grandparent at home when there is a vulnerable individual at home further increases uptake</t>
+  </si>
+  <si>
+    <t>Not enough data</t>
+  </si>
+  <si>
+    <t>vulnerable_indivs_income</t>
+  </si>
+  <si>
+    <t>Having a vulnerable individual increases the uptake of vaccination as income increases</t>
+  </si>
+  <si>
+    <t>vulnerable_individuals*test_household_income</t>
+  </si>
+  <si>
+    <t>Not enough data? Is it possible to run some sort of weight, based o nt</t>
+  </si>
+  <si>
+    <t>vulnerable_indivs_parent_chronic_illness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A parent who currently has a crhonic illness in a household is much less likely to have their child vaccinated </t>
+  </si>
+  <si>
+    <t>we can't really draw conclusions for parents with past chronic illnesses or even those without</t>
+  </si>
+  <si>
+    <t>vulnerable_individuals * parent_chronic_illness</t>
+  </si>
+  <si>
+    <t>vulnerable_individuals * parent_chronic_illness * child_grand * test_household_income</t>
+  </si>
+  <si>
+    <t>No conclusion to be drawn??</t>
+  </si>
+  <si>
+    <t>insufficient data to draw inferences for interactions</t>
+  </si>
+  <si>
+    <t>vulnerable_indivs_child_grand_income_parent_chronic</t>
+  </si>
+  <si>
+    <t>household_total_child_grand_</t>
+  </si>
+  <si>
+    <t>The presence of grandparents in a household directly affects the uptake of the vaccine as household_total changes</t>
+  </si>
+  <si>
+    <t>household_total*child_grand</t>
+  </si>
+  <si>
+    <t>chilg_grand</t>
+  </si>
+  <si>
+    <t>household_total*child_grand*parents_highest_education</t>
+  </si>
+  <si>
+    <t>This is just so weird man</t>
+  </si>
+  <si>
+    <t>The presence of grandparents in a household affects the uptake of the vaccine as the household changes for different highest educations of the parents themselves</t>
+  </si>
+  <si>
+    <t>household_total_child_grand_parent_education</t>
+  </si>
+  <si>
+    <t>Insufficient data to make a decision</t>
+  </si>
+  <si>
+    <t>household_total_child_grand_parent_marital</t>
+  </si>
+  <si>
+    <t>household_total*child_grand*test_paretns_marital_status</t>
+  </si>
+  <si>
+    <t>The same coloured lines are still parallel - The marital status of the responding parent doesn't really alter how the presence of grandaparents in a household changes the trends of uptake with an increasing number of individuals</t>
+  </si>
+  <si>
+    <t>househokd_total*test_parents_marital_status</t>
+  </si>
+  <si>
+    <t>Being unmarried results in a decrease in the uptake of the covid vax in the COI as the total household size increases</t>
+  </si>
+  <si>
+    <t>household_total_child_parents_marital</t>
+  </si>
+  <si>
+    <t>Too Little data to draw any sort of inference</t>
+  </si>
+  <si>
+    <t>household_total_parent_marital_income</t>
+  </si>
+  <si>
+    <t>I see no significant slope change in uptake with increasing household size. For both parents who are married and unmarried across different income groups</t>
+  </si>
+  <si>
+    <t>household_total*test_parents_marital_status*test_household_income</t>
+  </si>
+  <si>
+    <t>No?</t>
+  </si>
+  <si>
+    <t>household_total_highest_education</t>
+  </si>
+  <si>
+    <t>Education levels don’t seem to affect the uptake of the covid vaccine with increasing household sizes (all have roughly the same slope whichh is straight)</t>
+  </si>
+  <si>
+    <t>household_total*parents_higest_education</t>
+  </si>
+  <si>
+    <t>Seems to be no noticeable slope changes (based on the spread of the data points too) to indicate that there is any sort of change in uptake as the household size increases, for different parents_highest_educations</t>
   </si>
 </sst>
 </file>
@@ -7207,8 +7330,8 @@
       <c r="A18" t="s">
         <v>64</v>
       </c>
-      <c r="P18" s="16"/>
-      <c r="Q18" s="16"/>
+      <c r="P18" s="23"/>
+      <c r="Q18" s="23"/>
       <c r="AO18" s="16"/>
     </row>
     <row r="19" spans="1:42">
@@ -7253,7 +7376,7 @@
       <c r="N24" s="23" t="s">
         <v>419</v>
       </c>
-      <c r="Q24" s="16" t="s">
+      <c r="Q24" s="23" t="s">
         <v>418</v>
       </c>
       <c r="AB24" s="15" t="s">
@@ -7281,7 +7404,7 @@
       <c r="A27" t="s">
         <v>75</v>
       </c>
-      <c r="P27" s="16"/>
+      <c r="P27" s="23"/>
       <c r="AC27" s="16"/>
       <c r="AO27" s="16"/>
     </row>
@@ -7303,7 +7426,7 @@
       <c r="A29" t="s">
         <v>78</v>
       </c>
-      <c r="P29" s="16" t="s">
+      <c r="P29" s="23" t="s">
         <v>430</v>
       </c>
       <c r="X29" s="16"/>
@@ -7394,7 +7517,7 @@
       <c r="A36" t="s">
         <v>89</v>
       </c>
-      <c r="Q36" s="16" t="s">
+      <c r="Q36" s="23" t="s">
         <v>422</v>
       </c>
       <c r="V36" s="16"/>
@@ -7527,7 +7650,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313888EE-552D-40AA-8234-3B847E46EF43}">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="55.7265625" bestFit="1" customWidth="1"/>
@@ -7836,7 +7959,7 @@
     </row>
     <row r="13" spans="1:10" ht="29">
       <c r="A13" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="C13" t="s">
         <v>473</v>
@@ -7879,25 +8002,270 @@
     </row>
     <row r="15" spans="1:10" ht="58">
       <c r="A15" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="C15" t="s">
         <v>473</v>
       </c>
       <c r="D15" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="E15" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="F15" t="s">
         <v>535</v>
-      </c>
-      <c r="F15" t="s">
-        <v>536</v>
       </c>
       <c r="G15" t="s">
         <v>71</v>
       </c>
       <c r="H15" t="s">
         <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="43.5">
+      <c r="A16" t="s">
+        <v>543</v>
+      </c>
+      <c r="C16" t="s">
+        <v>471</v>
+      </c>
+      <c r="D16" t="s">
+        <v>539</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="F16" t="s">
+        <v>540</v>
+      </c>
+      <c r="G16" t="s">
+        <v>541</v>
+      </c>
+      <c r="H16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="29">
+      <c r="A17" t="s">
+        <v>547</v>
+      </c>
+      <c r="C17" t="s">
+        <v>471</v>
+      </c>
+      <c r="D17" t="s">
+        <v>544</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="F17" t="s">
+        <v>546</v>
+      </c>
+      <c r="G17" t="s">
+        <v>541</v>
+      </c>
+      <c r="H17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="43.5">
+      <c r="A18" t="s">
+        <v>550</v>
+      </c>
+      <c r="C18" t="s">
+        <v>473</v>
+      </c>
+      <c r="D18" t="s">
+        <v>548</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="F18" t="s">
+        <v>551</v>
+      </c>
+      <c r="G18" t="s">
+        <v>541</v>
+      </c>
+      <c r="H18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" t="s">
+        <v>554</v>
+      </c>
+      <c r="C19" t="s">
+        <v>473</v>
+      </c>
+      <c r="D19" t="s">
+        <v>555</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="F19" t="s">
+        <v>552</v>
+      </c>
+      <c r="G19" t="s">
+        <v>541</v>
+      </c>
+      <c r="H19" t="s">
+        <v>64</v>
+      </c>
+      <c r="I19" t="s">
+        <v>78</v>
+      </c>
+      <c r="J19" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="72.5">
+      <c r="A20" t="s">
+        <v>561</v>
+      </c>
+      <c r="C20" t="s">
+        <v>473</v>
+      </c>
+      <c r="D20" t="s">
+        <v>563</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="F20" t="s">
+        <v>560</v>
+      </c>
+      <c r="G20" t="s">
+        <v>63</v>
+      </c>
+      <c r="H20" t="s">
+        <v>559</v>
+      </c>
+      <c r="I20" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="87">
+      <c r="A21" t="s">
+        <v>564</v>
+      </c>
+      <c r="C21" t="s">
+        <v>473</v>
+      </c>
+      <c r="D21" t="s">
+        <v>565</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="F21" t="s">
+        <v>566</v>
+      </c>
+      <c r="G21" t="s">
+        <v>63</v>
+      </c>
+      <c r="H21" t="s">
+        <v>64</v>
+      </c>
+      <c r="I21" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="43.5">
+      <c r="C22" t="s">
+        <v>473</v>
+      </c>
+      <c r="D22" t="s">
+        <v>556</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="F22" t="s">
+        <v>558</v>
+      </c>
+      <c r="G22" t="s">
+        <v>63</v>
+      </c>
+      <c r="H22" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="43.5">
+      <c r="C23" t="s">
+        <v>472</v>
+      </c>
+      <c r="D23" t="s">
+        <v>570</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="F23" t="s">
+        <v>568</v>
+      </c>
+      <c r="G23" t="s">
+        <v>63</v>
+      </c>
+      <c r="H23" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="58">
+      <c r="A24" t="s">
+        <v>571</v>
+      </c>
+      <c r="B24" s="25" t="s">
+        <v>575</v>
+      </c>
+      <c r="C24" t="s">
+        <v>473</v>
+      </c>
+      <c r="D24" t="s">
+        <v>572</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="F24" t="s">
+        <v>574</v>
+      </c>
+      <c r="G24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H24" t="s">
+        <v>71</v>
+      </c>
+      <c r="I24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="58">
+      <c r="A25" t="s">
+        <v>579</v>
+      </c>
+      <c r="B25" s="25" t="s">
+        <v>575</v>
+      </c>
+      <c r="C25" t="s">
+        <v>473</v>
+      </c>
+      <c r="D25" t="s">
+        <v>576</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="F25" t="s">
+        <v>578</v>
+      </c>
+      <c r="G25" t="s">
+        <v>63</v>
+      </c>
+      <c r="H25" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add (codebook.xslsx) added columns and causal relationships to explore for test_mother_highest_education, test_father_highest_education and test_parents_highest_education
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Vaccine Uptake - R\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5ABCF75-4078-44CB-A516-6FB65FD4E987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E8D7D0F-CDFE-4BF6-B830-1E5DBBB78030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1714" uniqueCount="598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1737" uniqueCount="601">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -1888,6 +1888,15 @@
   </si>
   <si>
     <t>The highest level of education that the child of interest's father has completed but JCs, TCs And VCs are classd as their own schooling categories</t>
+  </si>
+  <si>
+    <t>mother_employment_status(0) * mother_stay_home (0) * test_household_income</t>
+  </si>
+  <si>
+    <t>test_mother_highest_father_highest_education_</t>
+  </si>
+  <si>
+    <t>difference in vax levels between VS, TS, JC?</t>
   </si>
 </sst>
 </file>
@@ -7534,7 +7543,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9521944E-28B4-4113-A27F-3B841E118807}">
-  <dimension ref="A1:AQ52"/>
+  <dimension ref="A1:AT55"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
@@ -7552,16 +7561,18 @@
     <col min="32" max="32" width="9.1796875" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="9.26953125" customWidth="1"/>
     <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="8.6328125" customWidth="1"/>
-    <col min="38" max="38" width="9.26953125" customWidth="1"/>
-    <col min="39" max="39" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="18" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="8.7265625" style="11"/>
+    <col min="35" max="35" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="37" max="39" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8.6328125" customWidth="1"/>
+    <col min="41" max="41" width="9.26953125" customWidth="1"/>
+    <col min="42" max="42" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="18" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="8.7265625" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="2" customFormat="1" ht="30" customHeight="1">
+    <row r="1" spans="1:46" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A1" s="18" t="s">
         <v>391</v>
       </c>
@@ -7668,99 +7679,108 @@
         <v>87</v>
       </c>
       <c r="AJ1" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="AK1" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="AL1" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
+        <v>589</v>
+      </c>
+      <c r="AN1" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AR1" t="s">
         <v>379</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AS1" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="AQ1" s="19" t="s">
+      <c r="AT1" s="19" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="2" spans="1:43">
+    <row r="2" spans="1:46">
       <c r="A2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:43">
+    <row r="3" spans="1:46">
       <c r="A3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:43">
+    <row r="4" spans="1:46">
       <c r="A4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:43">
+    <row r="5" spans="1:46">
       <c r="A5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:43">
+    <row r="6" spans="1:46">
       <c r="A6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:43">
+    <row r="7" spans="1:46">
       <c r="A7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:43">
+    <row r="8" spans="1:46">
       <c r="A8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:43">
+    <row r="9" spans="1:46">
       <c r="A9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:43">
+    <row r="10" spans="1:46">
       <c r="A10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:43">
+    <row r="11" spans="1:46">
       <c r="A11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:43">
+    <row r="12" spans="1:46">
       <c r="A12" t="s">
         <v>15</v>
       </c>
       <c r="U12" s="16"/>
       <c r="AF12" s="16"/>
-      <c r="AP12" s="16"/>
-      <c r="AQ12" s="11" t="s">
+      <c r="AS12" s="16"/>
+      <c r="AT12" s="11" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="13" spans="1:43">
+    <row r="13" spans="1:46">
       <c r="A13" t="s">
         <v>385</v>
       </c>
       <c r="L13" s="23"/>
-      <c r="AP13" s="16"/>
-    </row>
-    <row r="14" spans="1:43">
+      <c r="AS13" s="16"/>
+    </row>
+    <row r="14" spans="1:46">
       <c r="A14" t="s">
         <v>60</v>
       </c>
@@ -7770,69 +7790,69 @@
       </c>
       <c r="AE14" s="16"/>
       <c r="AF14" s="16"/>
-      <c r="AP14" s="16"/>
-    </row>
-    <row r="15" spans="1:43">
+      <c r="AS14" s="16"/>
+    </row>
+    <row r="15" spans="1:46">
       <c r="A15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:43">
+    <row r="16" spans="1:46">
       <c r="A16" t="s">
         <v>62</v>
       </c>
-      <c r="AO16" s="16"/>
-    </row>
-    <row r="17" spans="1:42">
+      <c r="AR16" s="16"/>
+    </row>
+    <row r="17" spans="1:45">
       <c r="A17" t="s">
         <v>63</v>
       </c>
       <c r="AB17" s="16"/>
-      <c r="AO17" s="16"/>
-    </row>
-    <row r="18" spans="1:42">
+      <c r="AR17" s="16"/>
+    </row>
+    <row r="18" spans="1:45">
       <c r="A18" t="s">
         <v>64</v>
       </c>
       <c r="Q18" s="23"/>
-      <c r="AO18" s="16"/>
-    </row>
-    <row r="19" spans="1:42">
+      <c r="AR18" s="16"/>
+    </row>
+    <row r="19" spans="1:45">
       <c r="A19" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:42">
+    <row r="20" spans="1:45">
       <c r="A20" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:42">
+    <row r="21" spans="1:45">
       <c r="A21" t="s">
         <v>502</v>
       </c>
       <c r="L21" s="23"/>
-      <c r="AO21" s="16"/>
-    </row>
-    <row r="22" spans="1:42">
+      <c r="AR21" s="16"/>
+    </row>
+    <row r="22" spans="1:45">
       <c r="A22" t="s">
         <v>495</v>
       </c>
       <c r="L22" s="23"/>
       <c r="M22" s="23"/>
       <c r="Q22" s="23"/>
-      <c r="AO22" s="16"/>
-    </row>
-    <row r="23" spans="1:42">
+      <c r="AR22" s="16"/>
+    </row>
+    <row r="23" spans="1:45">
       <c r="A23" t="s">
         <v>69</v>
       </c>
       <c r="L23" s="23"/>
       <c r="M23" s="23"/>
       <c r="Q23" s="23"/>
-      <c r="AO23" s="16"/>
-    </row>
-    <row r="24" spans="1:42">
+      <c r="AR23" s="16"/>
+    </row>
+    <row r="24" spans="1:45">
       <c r="A24" t="s">
         <v>71</v>
       </c>
@@ -7851,26 +7871,26 @@
       <c r="AF24" s="16" t="s">
         <v>416</v>
       </c>
-      <c r="AO24" s="16"/>
-    </row>
-    <row r="25" spans="1:42">
+      <c r="AR24" s="16"/>
+    </row>
+    <row r="25" spans="1:45">
       <c r="A25" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="26" spans="1:42">
+    <row r="26" spans="1:45">
       <c r="A26" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="27" spans="1:42">
+    <row r="27" spans="1:45">
       <c r="A27" t="s">
         <v>75</v>
       </c>
       <c r="AC27" s="16"/>
-      <c r="AO27" s="16"/>
-    </row>
-    <row r="28" spans="1:42">
+      <c r="AR27" s="16"/>
+    </row>
+    <row r="28" spans="1:45">
       <c r="A28" t="s">
         <v>77</v>
       </c>
@@ -7882,10 +7902,10 @@
       <c r="W28" s="16" t="s">
         <v>419</v>
       </c>
-      <c r="AO28" s="16"/>
-      <c r="AP28" s="16"/>
-    </row>
-    <row r="29" spans="1:42">
+      <c r="AR28" s="16"/>
+      <c r="AS28" s="16"/>
+    </row>
+    <row r="29" spans="1:45">
       <c r="A29" t="s">
         <v>78</v>
       </c>
@@ -7893,23 +7913,23 @@
         <v>429</v>
       </c>
       <c r="X29" s="16"/>
-      <c r="AK29" s="16" t="s">
+      <c r="AN29" s="16" t="s">
         <v>430</v>
       </c>
-      <c r="AL29" s="16"/>
-      <c r="AM29" s="16" t="s">
+      <c r="AO29" s="16"/>
+      <c r="AP29" s="16" t="s">
         <v>431</v>
       </c>
-      <c r="AP29" s="16"/>
-    </row>
-    <row r="30" spans="1:42">
+      <c r="AS29" s="16"/>
+    </row>
+    <row r="30" spans="1:45">
       <c r="A30" t="s">
         <v>79</v>
       </c>
       <c r="R30" s="16"/>
       <c r="AB30" s="23"/>
     </row>
-    <row r="31" spans="1:42">
+    <row r="31" spans="1:45">
       <c r="A31" t="s">
         <v>80</v>
       </c>
@@ -7921,7 +7941,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="32" spans="1:42">
+    <row r="32" spans="1:45">
       <c r="A32" t="s">
         <v>84</v>
       </c>
@@ -7932,24 +7952,24 @@
         <v>433</v>
       </c>
     </row>
-    <row r="33" spans="1:42">
+    <row r="33" spans="1:45">
       <c r="A33" t="s">
         <v>85</v>
       </c>
-      <c r="AK33" s="16" t="s">
+      <c r="AN33" s="16" t="s">
         <v>425</v>
       </c>
-      <c r="AL33" s="16" t="s">
+      <c r="AO33" s="16" t="s">
         <v>426</v>
       </c>
-      <c r="AM33" s="16" t="s">
+      <c r="AP33" s="16" t="s">
         <v>427</v>
       </c>
-      <c r="AN33" s="16" t="s">
+      <c r="AQ33" s="16" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="34" spans="1:42">
+    <row r="34" spans="1:45">
       <c r="A34" t="s">
         <v>86</v>
       </c>
@@ -7959,10 +7979,11 @@
         <v>437</v>
       </c>
       <c r="AD34" s="16"/>
-      <c r="AJ34" s="16"/>
-      <c r="AP34" s="16"/>
-    </row>
-    <row r="35" spans="1:42">
+      <c r="AL34" s="16"/>
+      <c r="AM34" s="16"/>
+      <c r="AS34" s="16"/>
+    </row>
+    <row r="35" spans="1:45">
       <c r="A35" t="s">
         <v>87</v>
       </c>
@@ -7973,121 +7994,161 @@
       </c>
       <c r="AE35" s="16"/>
       <c r="AF35" s="16"/>
-      <c r="AJ35" s="16"/>
-      <c r="AP35" s="16"/>
-    </row>
-    <row r="36" spans="1:42" ht="14" customHeight="1">
+      <c r="AL35" s="16"/>
+      <c r="AM35" s="16"/>
+      <c r="AS35" s="16"/>
+    </row>
+    <row r="36" spans="1:45">
       <c r="A36" t="s">
+        <v>382</v>
+      </c>
+      <c r="V36" s="16"/>
+      <c r="W36" s="16"/>
+      <c r="AB36" s="16" t="s">
+        <v>437</v>
+      </c>
+      <c r="AD36" s="16"/>
+      <c r="AL36" s="16"/>
+      <c r="AM36" s="16"/>
+      <c r="AS36" s="16"/>
+    </row>
+    <row r="37" spans="1:45">
+      <c r="A37" t="s">
+        <v>383</v>
+      </c>
+      <c r="V37" s="16"/>
+      <c r="W37" s="16"/>
+      <c r="AB37" s="16" t="s">
+        <v>436</v>
+      </c>
+      <c r="AE37" s="16"/>
+      <c r="AF37" s="16"/>
+      <c r="AL37" s="16"/>
+      <c r="AM37" s="16"/>
+      <c r="AS37" s="16"/>
+    </row>
+    <row r="38" spans="1:45" ht="14" customHeight="1">
+      <c r="A38" t="s">
         <v>89</v>
       </c>
-      <c r="Q36" s="23" t="s">
+      <c r="Q38" s="23" t="s">
         <v>421</v>
       </c>
-      <c r="V36" s="16"/>
-      <c r="W36" s="16" t="s">
+      <c r="V38" s="16"/>
+      <c r="W38" s="16" t="s">
         <v>422</v>
       </c>
-      <c r="AB36" s="23" t="s">
+      <c r="AB38" s="23" t="s">
         <v>438</v>
       </c>
-      <c r="AF36" s="16" t="s">
+      <c r="AF38" s="16" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="37" spans="1:42">
-      <c r="A37" t="s">
+    <row r="39" spans="1:45" ht="14" customHeight="1">
+      <c r="A39" t="s">
+        <v>589</v>
+      </c>
+      <c r="Q39" s="16"/>
+      <c r="V39" s="16"/>
+      <c r="W39" s="16"/>
+      <c r="AB39" s="16"/>
+      <c r="AF39" s="16"/>
+    </row>
+    <row r="40" spans="1:45">
+      <c r="A40" t="s">
         <v>90</v>
       </c>
-      <c r="AP37" s="16"/>
-    </row>
-    <row r="38" spans="1:42">
-      <c r="A38" t="s">
+      <c r="AS40" s="16"/>
+    </row>
+    <row r="41" spans="1:45">
+      <c r="A41" t="s">
         <v>91</v>
       </c>
-      <c r="AP38" s="16"/>
-    </row>
-    <row r="39" spans="1:42">
-      <c r="A39" t="s">
+      <c r="AS41" s="16"/>
+    </row>
+    <row r="42" spans="1:45">
+      <c r="A42" t="s">
         <v>92</v>
       </c>
-      <c r="AP39" s="16"/>
-    </row>
-    <row r="40" spans="1:42">
-      <c r="A40" t="s">
+      <c r="AS42" s="16"/>
+    </row>
+    <row r="43" spans="1:45">
+      <c r="A43" t="s">
         <v>93</v>
       </c>
-      <c r="AK40" s="16" t="s">
+      <c r="AN43" s="16" t="s">
         <v>428</v>
       </c>
-      <c r="AP40" s="16"/>
-    </row>
-    <row r="41" spans="1:42">
-      <c r="A41" t="s">
+      <c r="AS43" s="16"/>
+    </row>
+    <row r="44" spans="1:45">
+      <c r="A44" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="42" spans="1:42">
-      <c r="A42" t="s">
+    <row r="45" spans="1:45">
+      <c r="A45" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="44" spans="1:42" s="11" customFormat="1">
-      <c r="A44" s="11" t="s">
+    <row r="47" spans="1:45" s="11" customFormat="1">
+      <c r="A47" s="11" t="s">
         <v>455</v>
       </c>
-      <c r="P44" s="4"/>
-    </row>
-    <row r="46" spans="1:42">
-      <c r="B46" s="12" t="s">
+      <c r="P47" s="4"/>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="B49" s="12" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="47" spans="1:42">
-      <c r="A47" s="12"/>
-      <c r="B47" s="13"/>
-      <c r="C47" t="s">
+    <row r="50" spans="1:3">
+      <c r="A50" s="12"/>
+      <c r="B50" s="13"/>
+      <c r="C50" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="48" spans="1:42">
-      <c r="B48" s="14"/>
-      <c r="C48" t="s">
+    <row r="51" spans="1:3">
+      <c r="B51" s="14"/>
+      <c r="C51" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="49" spans="2:3">
-      <c r="B49" s="15"/>
-      <c r="C49" t="s">
+    <row r="52" spans="1:3">
+      <c r="B52" s="15"/>
+      <c r="C52" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="50" spans="2:3">
-      <c r="B50" s="16"/>
-      <c r="C50" t="s">
+    <row r="53" spans="1:3">
+      <c r="B53" s="16"/>
+      <c r="C53" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="51" spans="2:3">
-      <c r="B51" s="1" t="s">
+    <row r="54" spans="1:3">
+      <c r="B54" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C54" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="52" spans="2:3">
-      <c r="B52" s="23"/>
-      <c r="C52" t="s">
+    <row r="55" spans="1:3">
+      <c r="B55" s="23"/>
+      <c r="C55" t="s">
         <v>476</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B33:AM33">
+  <conditionalFormatting sqref="B33:AP33">
     <cfRule type="expression" dxfId="4" priority="3">
       <formula>$A33=B$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:AP23 B2:M24 N24:AN24 AP24 B25:AP27 X28:AN28 B28:W29 Y29:AP29 B30:AA32 AC30:AP32 AN33:AP34 AC34:AL34 B34:AA37 AC35:AP37 B38:AP43 B50">
+  <conditionalFormatting sqref="B2:AI27 AS24 X28:AI28 B28:W29 Y29:AI29 B30:AA32 AC30:AI32 AQ33:AS34 B41:AI46 B53 AQ36:AS36 B34:AA40 AC34:AI40 AM36:AO36 AM37:AS46 AM35:AS35 AM34:AO34 AM29:AS32 AM28:AQ28 AM25:AS27 AM24:AQ24 AM2:AS23 AJ34:AL46 AJ2:AL32">
     <cfRule type="expression" dxfId="3" priority="60">
       <formula>$A2=B$1</formula>
     </cfRule>
@@ -8097,14 +8158,14 @@
       <formula>$A29=#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB36">
+  <conditionalFormatting sqref="AB38:AB39">
     <cfRule type="expression" dxfId="1" priority="1">
-      <formula>$A36=AB$1</formula>
+      <formula>$A38=AB$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AO24 AO28:AP28">
+  <conditionalFormatting sqref="AR24 AR28:AS28">
     <cfRule type="expression" dxfId="0" priority="9">
-      <formula>#REF!=AO$1</formula>
+      <formula>#REF!=AR$1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8114,7 +8175,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313888EE-552D-40AA-8234-3B847E46EF43}">
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="55.7265625" bestFit="1" customWidth="1"/>
@@ -8258,136 +8319,133 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="43.5">
-      <c r="B6" s="29" t="s">
+    <row r="6" spans="1:10">
+      <c r="B6" s="27" t="s">
+        <v>519</v>
+      </c>
+      <c r="D6" t="s">
+        <v>599</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="F6" t="s">
+        <v>482</v>
+      </c>
+      <c r="G6" t="s">
+        <v>382</v>
+      </c>
+      <c r="H6" t="s">
+        <v>383</v>
+      </c>
+      <c r="I6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="B7" s="27" t="s">
+        <v>519</v>
+      </c>
+      <c r="D7" t="s">
+        <v>599</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="F7" t="s">
+        <v>482</v>
+      </c>
+      <c r="G7" t="s">
+        <v>382</v>
+      </c>
+      <c r="H7" t="s">
+        <v>383</v>
+      </c>
+      <c r="I7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="43.5">
+      <c r="B8" s="29" t="s">
         <v>587</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C8" t="s">
         <v>472</v>
-      </c>
-      <c r="D6" t="s">
-        <v>460</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="F6" t="s">
-        <v>525</v>
-      </c>
-      <c r="G6" t="s">
-        <v>526</v>
-      </c>
-      <c r="H6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="43.5">
-      <c r="B7" s="29" t="s">
-        <v>588</v>
-      </c>
-      <c r="C7" t="s">
-        <v>470</v>
-      </c>
-      <c r="D7" t="s">
-        <v>460</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>521</v>
-      </c>
-      <c r="F7" t="s">
-        <v>522</v>
-      </c>
-      <c r="G7" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="43.5">
-      <c r="B8" s="26" t="s">
-        <v>518</v>
-      </c>
-      <c r="C8" t="s">
-        <v>470</v>
       </c>
       <c r="D8" t="s">
         <v>460</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>485</v>
+        <v>524</v>
       </c>
       <c r="F8" t="s">
-        <v>486</v>
+        <v>525</v>
       </c>
       <c r="G8" t="s">
-        <v>89</v>
+        <v>526</v>
       </c>
       <c r="H8" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="29">
-      <c r="B9" s="28" t="s">
-        <v>520</v>
+    <row r="9" spans="1:10" ht="43.5">
+      <c r="B9" s="29" t="s">
+        <v>588</v>
       </c>
       <c r="C9" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D9" t="s">
-        <v>473</v>
+        <v>460</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>479</v>
+        <v>521</v>
       </c>
       <c r="F9" t="s">
-        <v>480</v>
+        <v>522</v>
       </c>
       <c r="G9" t="s">
-        <v>84</v>
-      </c>
-      <c r="H9" t="s">
-        <v>77</v>
+        <v>523</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.5">
-      <c r="A10" s="2" t="s">
-        <v>531</v>
-      </c>
-      <c r="B10" s="27" t="s">
-        <v>519</v>
+      <c r="B10" s="26" t="s">
+        <v>518</v>
       </c>
       <c r="C10" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D10" t="s">
-        <v>477</v>
+        <v>460</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
       <c r="F10" t="s">
-        <v>169</v>
+        <v>486</v>
       </c>
       <c r="G10" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H10" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="43.5">
+    <row r="11" spans="1:10" ht="29">
       <c r="B11" s="28" t="s">
         <v>520</v>
       </c>
       <c r="C11" t="s">
-        <v>169</v>
+        <v>471</v>
       </c>
       <c r="D11" t="s">
-        <v>483</v>
+        <v>473</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="F11" t="s">
-        <v>169</v>
+        <v>480</v>
       </c>
       <c r="G11" t="s">
         <v>84</v>
@@ -8395,227 +8453,221 @@
       <c r="H11" t="s">
         <v>77</v>
       </c>
-      <c r="I11" t="s">
+    </row>
+    <row r="12" spans="1:10" ht="43.5">
+      <c r="A12" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B12" s="31" t="s">
+        <v>518</v>
+      </c>
+      <c r="C12" t="s">
+        <v>471</v>
+      </c>
+      <c r="D12" t="s">
+        <v>477</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="F12" t="s">
+        <v>598</v>
+      </c>
+      <c r="G12" t="s">
+        <v>80</v>
+      </c>
+      <c r="H12" t="s">
+        <v>77</v>
+      </c>
+      <c r="I12" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="43.5">
+      <c r="B13" s="28" t="s">
+        <v>520</v>
+      </c>
+      <c r="C13" t="s">
+        <v>169</v>
+      </c>
+      <c r="D13" t="s">
+        <v>483</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="F13" t="s">
+        <v>169</v>
+      </c>
+      <c r="G13" t="s">
+        <v>84</v>
+      </c>
+      <c r="H13" t="s">
+        <v>77</v>
+      </c>
+      <c r="I13" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="58">
-      <c r="A12" t="s">
+    <row r="14" spans="1:10" ht="58">
+      <c r="A14" t="s">
         <v>493</v>
       </c>
-      <c r="B12" s="30" t="s">
+      <c r="B14" s="30" t="s">
         <v>586</v>
-      </c>
-      <c r="C12" t="s">
-        <v>472</v>
-      </c>
-      <c r="D12" t="s">
-        <v>494</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>492</v>
-      </c>
-      <c r="F12" t="s">
-        <v>491</v>
-      </c>
-      <c r="G12" t="s">
-        <v>385</v>
-      </c>
-      <c r="H12" t="s">
-        <v>15</v>
-      </c>
-      <c r="I12" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="29">
-      <c r="A13" t="s">
-        <v>536</v>
-      </c>
-      <c r="B13" s="31" t="s">
-        <v>518</v>
-      </c>
-      <c r="C13" t="s">
-        <v>472</v>
-      </c>
-      <c r="D13" t="s">
-        <v>517</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>516</v>
-      </c>
-      <c r="F13" t="s">
-        <v>515</v>
-      </c>
-      <c r="G13" t="s">
-        <v>514</v>
-      </c>
-      <c r="H13" t="s">
-        <v>15</v>
-      </c>
-      <c r="I13" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="B14" s="31" t="s">
-        <v>518</v>
       </c>
       <c r="C14" t="s">
         <v>472</v>
       </c>
+      <c r="D14" t="s">
+        <v>494</v>
+      </c>
       <c r="E14" s="2" t="s">
-        <v>529</v>
+        <v>492</v>
       </c>
       <c r="F14" t="s">
-        <v>530</v>
+        <v>491</v>
       </c>
       <c r="G14" t="s">
-        <v>502</v>
+        <v>385</v>
       </c>
       <c r="H14" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" ht="58">
+      <c r="I14" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="29">
       <c r="A15" t="s">
-        <v>534</v>
-      </c>
-      <c r="B15" s="30" t="s">
-        <v>586</v>
+        <v>536</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>518</v>
       </c>
       <c r="C15" t="s">
         <v>472</v>
       </c>
       <c r="D15" t="s">
+        <v>517</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="F15" t="s">
+        <v>515</v>
+      </c>
+      <c r="G15" t="s">
+        <v>514</v>
+      </c>
+      <c r="H15" t="s">
+        <v>15</v>
+      </c>
+      <c r="I15" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="B16" s="31" t="s">
+        <v>518</v>
+      </c>
+      <c r="C16" t="s">
+        <v>472</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="F16" t="s">
+        <v>530</v>
+      </c>
+      <c r="G16" t="s">
+        <v>502</v>
+      </c>
+      <c r="H16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="58">
+      <c r="A17" t="s">
+        <v>534</v>
+      </c>
+      <c r="B17" s="30" t="s">
+        <v>586</v>
+      </c>
+      <c r="C17" t="s">
+        <v>472</v>
+      </c>
+      <c r="D17" t="s">
         <v>535</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F17" t="s">
         <v>533</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G17" t="s">
         <v>71</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H17" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="43.5">
-      <c r="A16" t="s">
-        <v>541</v>
-      </c>
-      <c r="B16" s="30" t="s">
-        <v>586</v>
-      </c>
-      <c r="C16" t="s">
-        <v>470</v>
-      </c>
-      <c r="D16" t="s">
-        <v>537</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>540</v>
-      </c>
-      <c r="F16" t="s">
-        <v>538</v>
-      </c>
-      <c r="G16" t="s">
-        <v>539</v>
-      </c>
-      <c r="H16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="29">
-      <c r="A17" t="s">
-        <v>545</v>
-      </c>
-      <c r="B17" s="31" t="s">
-        <v>518</v>
-      </c>
-      <c r="C17" t="s">
-        <v>470</v>
-      </c>
-      <c r="D17" t="s">
-        <v>542</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="F17" t="s">
-        <v>544</v>
-      </c>
-      <c r="G17" t="s">
-        <v>539</v>
-      </c>
-      <c r="H17" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="43.5">
       <c r="A18" t="s">
-        <v>548</v>
+        <v>541</v>
       </c>
       <c r="B18" s="30" t="s">
         <v>586</v>
       </c>
       <c r="C18" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="D18" t="s">
-        <v>546</v>
+        <v>537</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>547</v>
+        <v>540</v>
       </c>
       <c r="F18" t="s">
-        <v>549</v>
+        <v>538</v>
       </c>
       <c r="G18" t="s">
         <v>539</v>
       </c>
       <c r="H18" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="29">
       <c r="A19" t="s">
-        <v>552</v>
-      </c>
-      <c r="B19" s="30" t="s">
-        <v>573</v>
+        <v>545</v>
+      </c>
+      <c r="B19" s="31" t="s">
+        <v>518</v>
       </c>
       <c r="C19" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="D19" t="s">
-        <v>553</v>
+        <v>542</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>551</v>
+        <v>543</v>
       </c>
       <c r="F19" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="G19" t="s">
         <v>539</v>
       </c>
       <c r="H19" t="s">
-        <v>64</v>
-      </c>
-      <c r="I19" t="s">
-        <v>78</v>
-      </c>
-      <c r="J19" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="72.5">
+    <row r="20" spans="1:10" ht="43.5">
       <c r="A20" t="s">
-        <v>559</v>
+        <v>548</v>
       </c>
       <c r="B20" s="30" t="s">
         <v>586</v>
@@ -8624,54 +8676,57 @@
         <v>472</v>
       </c>
       <c r="D20" t="s">
-        <v>561</v>
+        <v>546</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>560</v>
+        <v>547</v>
       </c>
       <c r="F20" t="s">
-        <v>558</v>
+        <v>549</v>
       </c>
       <c r="G20" t="s">
-        <v>63</v>
+        <v>539</v>
       </c>
       <c r="H20" t="s">
-        <v>557</v>
-      </c>
-      <c r="I20" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="87">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>562</v>
+        <v>552</v>
       </c>
       <c r="B21" s="30" t="s">
-        <v>586</v>
+        <v>573</v>
       </c>
       <c r="C21" t="s">
         <v>472</v>
       </c>
       <c r="D21" t="s">
-        <v>563</v>
+        <v>553</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>565</v>
+        <v>551</v>
       </c>
       <c r="F21" t="s">
-        <v>564</v>
+        <v>550</v>
       </c>
       <c r="G21" t="s">
-        <v>63</v>
+        <v>539</v>
       </c>
       <c r="H21" t="s">
         <v>64</v>
       </c>
       <c r="I21" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="43.5">
+        <v>78</v>
+      </c>
+      <c r="J21" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="72.5">
+      <c r="A22" t="s">
+        <v>559</v>
+      </c>
       <c r="B22" s="30" t="s">
         <v>586</v>
       </c>
@@ -8679,48 +8734,54 @@
         <v>472</v>
       </c>
       <c r="D22" t="s">
-        <v>554</v>
+        <v>561</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="F22" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="G22" t="s">
         <v>63</v>
       </c>
       <c r="H22" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="43.5">
+        <v>557</v>
+      </c>
+      <c r="I22" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="87">
+      <c r="A23" t="s">
+        <v>562</v>
+      </c>
       <c r="B23" s="30" t="s">
         <v>586</v>
       </c>
       <c r="C23" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D23" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="F23" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="G23" t="s">
         <v>63</v>
       </c>
       <c r="H23" t="s">
+        <v>64</v>
+      </c>
+      <c r="I23" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="58">
-      <c r="A24" t="s">
-        <v>569</v>
-      </c>
+    <row r="24" spans="1:10" ht="43.5">
       <c r="B24" s="30" t="s">
         <v>586</v>
       </c>
@@ -8728,73 +8789,122 @@
         <v>472</v>
       </c>
       <c r="D24" t="s">
-        <v>570</v>
+        <v>554</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>571</v>
+        <v>555</v>
       </c>
       <c r="F24" t="s">
-        <v>572</v>
+        <v>556</v>
       </c>
       <c r="G24" t="s">
         <v>63</v>
       </c>
       <c r="H24" t="s">
-        <v>71</v>
-      </c>
-      <c r="I24" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="58">
-      <c r="A25" t="s">
-        <v>577</v>
-      </c>
-      <c r="B25" s="31" t="s">
-        <v>518</v>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="43.5">
+      <c r="B25" s="30" t="s">
+        <v>586</v>
       </c>
       <c r="C25" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D25" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>575</v>
+        <v>567</v>
       </c>
       <c r="F25" t="s">
-        <v>576</v>
+        <v>566</v>
       </c>
       <c r="G25" t="s">
         <v>63</v>
       </c>
       <c r="H25" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="116">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="58">
       <c r="A26" t="s">
-        <v>581</v>
+        <v>569</v>
       </c>
       <c r="B26" s="30" t="s">
         <v>586</v>
       </c>
       <c r="C26" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D26" t="s">
-        <v>578</v>
+        <v>570</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>579</v>
+        <v>571</v>
       </c>
       <c r="F26" t="s">
-        <v>580</v>
+        <v>572</v>
       </c>
       <c r="G26" t="s">
         <v>63</v>
       </c>
       <c r="H26" t="s">
+        <v>71</v>
+      </c>
+      <c r="I26" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="58">
+      <c r="A27" t="s">
+        <v>577</v>
+      </c>
+      <c r="B27" s="31" t="s">
+        <v>518</v>
+      </c>
+      <c r="C27" t="s">
+        <v>472</v>
+      </c>
+      <c r="D27" t="s">
+        <v>574</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="F27" t="s">
+        <v>576</v>
+      </c>
+      <c r="G27" t="s">
+        <v>63</v>
+      </c>
+      <c r="H27" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="116">
+      <c r="A28" t="s">
+        <v>581</v>
+      </c>
+      <c r="B28" s="30" t="s">
+        <v>586</v>
+      </c>
+      <c r="C28" t="s">
+        <v>471</v>
+      </c>
+      <c r="D28" t="s">
+        <v>578</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F28" t="s">
+        <v>580</v>
+      </c>
+      <c r="G28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H28" t="s">
         <v>495</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add (codebook.xslsx) (exploratory_dag) added links for siblings_over_18
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Vaccine Uptake - R\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E8D7D0F-CDFE-4BF6-B830-1E5DBBB78030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7296CF7-FCF5-4422-9C76-307471315E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1737" uniqueCount="601">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1743" uniqueCount="605">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -1896,7 +1896,19 @@
     <t>test_mother_highest_father_highest_education_</t>
   </si>
   <si>
-    <t>difference in vax levels between VS, TS, JC?</t>
+    <t>test_mother_highest_test_father_highest_education_</t>
+  </si>
+  <si>
+    <t>Having fathers in JC or VS significantly decreases the uptake of the covid vaccine</t>
+  </si>
+  <si>
+    <t>test_father_highest_education (VS) * test_mother_highest_education (VS, JC)</t>
+  </si>
+  <si>
+    <t>mother_highest_test_father_highest_education</t>
+  </si>
+  <si>
+    <t>test_father_highest_education (VS)</t>
   </si>
 </sst>
 </file>
@@ -2084,7 +2096,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2136,6 +2148,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7543,7 +7556,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9521944E-28B4-4113-A27F-3B841E118807}">
-  <dimension ref="A1:AT55"/>
+  <dimension ref="A1:AU56"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
@@ -7552,27 +7565,28 @@
     <col min="15" max="15" width="8.6328125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10.6328125" style="4" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8.36328125" customWidth="1"/>
-    <col min="28" max="28" width="11.08984375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="9.26953125" customWidth="1"/>
-    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="37" max="39" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="8.6328125" customWidth="1"/>
-    <col min="41" max="41" width="9.26953125" customWidth="1"/>
-    <col min="42" max="42" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="18" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="8.7265625" style="11"/>
+    <col min="24" max="24" width="8.54296875" customWidth="1"/>
+    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="8.36328125" customWidth="1"/>
+    <col min="29" max="29" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.26953125" customWidth="1"/>
+    <col min="35" max="35" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="38" max="40" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="8.6328125" customWidth="1"/>
+    <col min="42" max="42" width="9.26953125" customWidth="1"/>
+    <col min="43" max="43" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="18" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="8.7265625" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" s="2" customFormat="1" ht="30" customHeight="1">
+    <row r="1" spans="1:47" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A1" s="18" t="s">
         <v>391</v>
       </c>
@@ -7643,529 +7657,550 @@
         <v>69</v>
       </c>
       <c r="X1" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="Y1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AB1" s="17" t="s">
+      <c r="AC1" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>589</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AR1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>379</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AT1" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="AT1" s="19" t="s">
+      <c r="AU1" s="19" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="2" spans="1:46">
+    <row r="2" spans="1:47">
       <c r="A2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:46">
+    <row r="3" spans="1:47">
       <c r="A3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:46">
+    <row r="4" spans="1:47">
       <c r="A4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:46">
+    <row r="5" spans="1:47">
       <c r="A5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:46">
+    <row r="6" spans="1:47">
       <c r="A6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:46">
+    <row r="7" spans="1:47">
       <c r="A7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:46">
+    <row r="8" spans="1:47">
       <c r="A8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:46">
+    <row r="9" spans="1:47">
       <c r="A9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:46">
+    <row r="10" spans="1:47">
       <c r="A10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:46">
+    <row r="11" spans="1:47">
       <c r="A11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:46">
+    <row r="12" spans="1:47">
       <c r="A12" t="s">
         <v>15</v>
       </c>
       <c r="U12" s="16"/>
-      <c r="AF12" s="16"/>
-      <c r="AS12" s="16"/>
-      <c r="AT12" s="11" t="s">
+      <c r="AG12" s="16"/>
+      <c r="AT12" s="16"/>
+      <c r="AU12" s="11" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="13" spans="1:46">
+    <row r="13" spans="1:47">
       <c r="A13" t="s">
         <v>385</v>
       </c>
       <c r="L13" s="23"/>
-      <c r="AS13" s="16"/>
-    </row>
-    <row r="14" spans="1:46">
+      <c r="AT13" s="16"/>
+    </row>
+    <row r="14" spans="1:47">
       <c r="A14" t="s">
         <v>60</v>
       </c>
       <c r="R14" s="16"/>
-      <c r="AB14" s="23" t="s">
+      <c r="AC14" s="23" t="s">
         <v>394</v>
       </c>
-      <c r="AE14" s="16"/>
       <c r="AF14" s="16"/>
-      <c r="AS14" s="16"/>
-    </row>
-    <row r="15" spans="1:46">
+      <c r="AG14" s="16"/>
+      <c r="AT14" s="16"/>
+    </row>
+    <row r="15" spans="1:47">
       <c r="A15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:46">
+    <row r="16" spans="1:47">
       <c r="A16" t="s">
         <v>62</v>
       </c>
-      <c r="AR16" s="16"/>
-    </row>
-    <row r="17" spans="1:45">
+      <c r="AS16" s="16"/>
+    </row>
+    <row r="17" spans="1:46">
       <c r="A17" t="s">
         <v>63</v>
       </c>
-      <c r="AB17" s="16"/>
-      <c r="AR17" s="16"/>
-    </row>
-    <row r="18" spans="1:45">
+      <c r="AC17" s="16"/>
+      <c r="AS17" s="16"/>
+    </row>
+    <row r="18" spans="1:46">
       <c r="A18" t="s">
         <v>64</v>
       </c>
       <c r="Q18" s="23"/>
-      <c r="AR18" s="16"/>
-    </row>
-    <row r="19" spans="1:45">
+      <c r="AS18" s="16"/>
+    </row>
+    <row r="19" spans="1:46">
       <c r="A19" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:45">
+    <row r="20" spans="1:46">
       <c r="A20" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:45">
+    <row r="21" spans="1:46">
       <c r="A21" t="s">
         <v>502</v>
       </c>
       <c r="L21" s="23"/>
-      <c r="AR21" s="16"/>
-    </row>
-    <row r="22" spans="1:45">
+      <c r="AS21" s="16"/>
+    </row>
+    <row r="22" spans="1:46">
       <c r="A22" t="s">
         <v>495</v>
       </c>
       <c r="L22" s="23"/>
       <c r="M22" s="23"/>
       <c r="Q22" s="23"/>
-      <c r="AR22" s="16"/>
-    </row>
-    <row r="23" spans="1:45">
+      <c r="AS22" s="16"/>
+    </row>
+    <row r="23" spans="1:46">
       <c r="A23" t="s">
         <v>69</v>
       </c>
       <c r="L23" s="23"/>
-      <c r="M23" s="23"/>
+      <c r="M23" s="33"/>
       <c r="Q23" s="23"/>
-      <c r="AR23" s="16"/>
-    </row>
-    <row r="24" spans="1:45">
+      <c r="AS23" s="16"/>
+    </row>
+    <row r="24" spans="1:46">
       <c r="A24" t="s">
+        <v>582</v>
+      </c>
+      <c r="L24" s="33"/>
+      <c r="M24" s="16"/>
+      <c r="Q24" s="16"/>
+      <c r="R24" s="16"/>
+      <c r="AC24" s="16"/>
+      <c r="AS24" s="16"/>
+    </row>
+    <row r="25" spans="1:46">
+      <c r="A25" t="s">
         <v>71</v>
       </c>
-      <c r="N24" s="23" t="s">
+      <c r="N25" s="23" t="s">
         <v>418</v>
       </c>
-      <c r="Q24" s="23" t="s">
+      <c r="Q25" s="23" t="s">
         <v>417</v>
       </c>
-      <c r="AB24" s="15" t="s">
+      <c r="AC25" s="15" t="s">
         <v>415</v>
       </c>
-      <c r="AC24" s="16" t="s">
+      <c r="AD25" s="16" t="s">
         <v>432</v>
       </c>
-      <c r="AF24" s="16" t="s">
+      <c r="AG25" s="16" t="s">
         <v>416</v>
       </c>
-      <c r="AR24" s="16"/>
-    </row>
-    <row r="25" spans="1:45">
-      <c r="A25" t="s">
+      <c r="AS25" s="16"/>
+    </row>
+    <row r="26" spans="1:46">
+      <c r="A26" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="26" spans="1:45">
-      <c r="A26" t="s">
+    <row r="27" spans="1:46">
+      <c r="A27" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="27" spans="1:45">
-      <c r="A27" t="s">
+    <row r="28" spans="1:46">
+      <c r="A28" t="s">
         <v>75</v>
       </c>
-      <c r="AC27" s="16"/>
-      <c r="AR27" s="16"/>
-    </row>
-    <row r="28" spans="1:45">
-      <c r="A28" t="s">
+      <c r="AD28" s="16"/>
+      <c r="AS28" s="16"/>
+    </row>
+    <row r="29" spans="1:46">
+      <c r="A29" t="s">
         <v>77</v>
       </c>
-      <c r="P28" s="15"/>
-      <c r="R28" s="16" t="s">
+      <c r="P29" s="15"/>
+      <c r="R29" s="16" t="s">
         <v>423</v>
       </c>
-      <c r="V28" s="16"/>
-      <c r="W28" s="16" t="s">
+      <c r="V29" s="16"/>
+      <c r="W29" s="16" t="s">
         <v>419</v>
       </c>
-      <c r="AR28" s="16"/>
-      <c r="AS28" s="16"/>
-    </row>
-    <row r="29" spans="1:45">
-      <c r="A29" t="s">
+      <c r="X29" s="16"/>
+      <c r="AS29" s="16"/>
+      <c r="AT29" s="16"/>
+    </row>
+    <row r="30" spans="1:46">
+      <c r="A30" t="s">
         <v>78</v>
       </c>
-      <c r="P29" s="4" t="s">
+      <c r="P30" s="4" t="s">
         <v>429</v>
       </c>
-      <c r="X29" s="16"/>
-      <c r="AN29" s="16" t="s">
+      <c r="Y30" s="16"/>
+      <c r="AO30" s="16" t="s">
         <v>430</v>
       </c>
-      <c r="AO29" s="16"/>
-      <c r="AP29" s="16" t="s">
+      <c r="AP30" s="16"/>
+      <c r="AQ30" s="16" t="s">
         <v>431</v>
       </c>
-      <c r="AS29" s="16"/>
-    </row>
-    <row r="30" spans="1:45">
-      <c r="A30" t="s">
+      <c r="AT30" s="16"/>
+    </row>
+    <row r="31" spans="1:46">
+      <c r="A31" t="s">
         <v>79</v>
       </c>
-      <c r="R30" s="16"/>
-      <c r="AB30" s="23"/>
-    </row>
-    <row r="31" spans="1:45">
-      <c r="A31" t="s">
+      <c r="R31" s="16"/>
+      <c r="AC31" s="23"/>
+    </row>
+    <row r="32" spans="1:46">
+      <c r="A32" t="s">
         <v>80</v>
       </c>
-      <c r="R31" s="16"/>
-      <c r="AB31" s="24" t="s">
+      <c r="R32" s="16"/>
+      <c r="AC32" s="24" t="s">
         <v>475</v>
       </c>
-      <c r="AF31" s="16" t="s">
+      <c r="AG32" s="16" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="32" spans="1:45">
-      <c r="A32" t="s">
+    <row r="33" spans="1:46">
+      <c r="A33" t="s">
         <v>84</v>
       </c>
-      <c r="R32" s="16" t="s">
+      <c r="R33" s="16" t="s">
         <v>434</v>
       </c>
-      <c r="AB32" s="23" t="s">
+      <c r="AC33" s="23" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="33" spans="1:45">
-      <c r="A33" t="s">
+    <row r="34" spans="1:46">
+      <c r="A34" t="s">
         <v>85</v>
       </c>
-      <c r="AN33" s="16" t="s">
+      <c r="AO34" s="16" t="s">
         <v>425</v>
       </c>
-      <c r="AO33" s="16" t="s">
+      <c r="AP34" s="16" t="s">
         <v>426</v>
       </c>
-      <c r="AP33" s="16" t="s">
+      <c r="AQ34" s="16" t="s">
         <v>427</v>
       </c>
-      <c r="AQ33" s="16" t="s">
+      <c r="AR34" s="16" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="34" spans="1:45">
-      <c r="A34" t="s">
+    <row r="35" spans="1:46">
+      <c r="A35" t="s">
         <v>86</v>
-      </c>
-      <c r="V34" s="16"/>
-      <c r="W34" s="16"/>
-      <c r="AB34" s="23" t="s">
-        <v>437</v>
-      </c>
-      <c r="AD34" s="16"/>
-      <c r="AL34" s="16"/>
-      <c r="AM34" s="16"/>
-      <c r="AS34" s="16"/>
-    </row>
-    <row r="35" spans="1:45">
-      <c r="A35" t="s">
-        <v>87</v>
       </c>
       <c r="V35" s="16"/>
       <c r="W35" s="16"/>
-      <c r="AB35" s="23" t="s">
-        <v>436</v>
+      <c r="X35" s="16"/>
+      <c r="AC35" s="23" t="s">
+        <v>437</v>
       </c>
       <c r="AE35" s="16"/>
-      <c r="AF35" s="16"/>
-      <c r="AL35" s="16"/>
       <c r="AM35" s="16"/>
-      <c r="AS35" s="16"/>
-    </row>
-    <row r="36" spans="1:45">
+      <c r="AN35" s="16"/>
+      <c r="AT35" s="16"/>
+    </row>
+    <row r="36" spans="1:46">
       <c r="A36" t="s">
-        <v>382</v>
+        <v>87</v>
       </c>
       <c r="V36" s="16"/>
       <c r="W36" s="16"/>
-      <c r="AB36" s="16" t="s">
-        <v>437</v>
-      </c>
-      <c r="AD36" s="16"/>
-      <c r="AL36" s="16"/>
+      <c r="X36" s="16"/>
+      <c r="AC36" s="23" t="s">
+        <v>436</v>
+      </c>
+      <c r="AF36" s="16"/>
+      <c r="AG36" s="16"/>
       <c r="AM36" s="16"/>
-      <c r="AS36" s="16"/>
-    </row>
-    <row r="37" spans="1:45">
+      <c r="AN36" s="16"/>
+      <c r="AT36" s="16"/>
+    </row>
+    <row r="37" spans="1:46">
       <c r="A37" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="V37" s="16"/>
       <c r="W37" s="16"/>
-      <c r="AB37" s="16" t="s">
+      <c r="X37" s="16"/>
+      <c r="AC37" s="16" t="s">
+        <v>437</v>
+      </c>
+      <c r="AE37" s="16"/>
+      <c r="AM37" s="16"/>
+      <c r="AN37" s="16"/>
+      <c r="AT37" s="16"/>
+    </row>
+    <row r="38" spans="1:46">
+      <c r="A38" t="s">
+        <v>383</v>
+      </c>
+      <c r="V38" s="16"/>
+      <c r="W38" s="16"/>
+      <c r="X38" s="16"/>
+      <c r="AC38" s="16" t="s">
         <v>436</v>
       </c>
-      <c r="AE37" s="16"/>
-      <c r="AF37" s="16"/>
-      <c r="AL37" s="16"/>
-      <c r="AM37" s="16"/>
-      <c r="AS37" s="16"/>
-    </row>
-    <row r="38" spans="1:45" ht="14" customHeight="1">
-      <c r="A38" t="s">
+      <c r="AF38" s="16"/>
+      <c r="AG38" s="16"/>
+      <c r="AM38" s="16"/>
+      <c r="AN38" s="16"/>
+      <c r="AT38" s="16"/>
+    </row>
+    <row r="39" spans="1:46" ht="14" customHeight="1">
+      <c r="A39" t="s">
         <v>89</v>
       </c>
-      <c r="Q38" s="23" t="s">
+      <c r="Q39" s="23" t="s">
         <v>421</v>
       </c>
-      <c r="V38" s="16"/>
-      <c r="W38" s="16" t="s">
+      <c r="V39" s="16"/>
+      <c r="W39" s="16" t="s">
         <v>422</v>
       </c>
-      <c r="AB38" s="23" t="s">
+      <c r="X39" s="16"/>
+      <c r="AC39" s="23" t="s">
         <v>438</v>
       </c>
-      <c r="AF38" s="16" t="s">
+      <c r="AG39" s="16" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="39" spans="1:45" ht="14" customHeight="1">
-      <c r="A39" t="s">
+    <row r="40" spans="1:46" ht="14" customHeight="1">
+      <c r="A40" t="s">
         <v>589</v>
       </c>
-      <c r="Q39" s="16"/>
-      <c r="V39" s="16"/>
-      <c r="W39" s="16"/>
-      <c r="AB39" s="16"/>
-      <c r="AF39" s="16"/>
-    </row>
-    <row r="40" spans="1:45">
-      <c r="A40" t="s">
+      <c r="Q40" s="16"/>
+      <c r="V40" s="16"/>
+      <c r="W40" s="16"/>
+      <c r="X40" s="16"/>
+      <c r="AC40" s="16"/>
+      <c r="AG40" s="16"/>
+    </row>
+    <row r="41" spans="1:46">
+      <c r="A41" t="s">
         <v>90</v>
       </c>
-      <c r="AS40" s="16"/>
-    </row>
-    <row r="41" spans="1:45">
-      <c r="A41" t="s">
+      <c r="AT41" s="16"/>
+    </row>
+    <row r="42" spans="1:46">
+      <c r="A42" t="s">
         <v>91</v>
       </c>
-      <c r="AS41" s="16"/>
-    </row>
-    <row r="42" spans="1:45">
-      <c r="A42" t="s">
+      <c r="AT42" s="16"/>
+    </row>
+    <row r="43" spans="1:46">
+      <c r="A43" t="s">
         <v>92</v>
       </c>
-      <c r="AS42" s="16"/>
-    </row>
-    <row r="43" spans="1:45">
-      <c r="A43" t="s">
+      <c r="AT43" s="16"/>
+    </row>
+    <row r="44" spans="1:46">
+      <c r="A44" t="s">
         <v>93</v>
       </c>
-      <c r="AN43" s="16" t="s">
+      <c r="AO44" s="16" t="s">
         <v>428</v>
       </c>
-      <c r="AS43" s="16"/>
-    </row>
-    <row r="44" spans="1:45">
-      <c r="A44" t="s">
+      <c r="AT44" s="16"/>
+    </row>
+    <row r="45" spans="1:46">
+      <c r="A45" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="45" spans="1:45">
-      <c r="A45" t="s">
+    <row r="46" spans="1:46">
+      <c r="A46" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="47" spans="1:45" s="11" customFormat="1">
-      <c r="A47" s="11" t="s">
+    <row r="48" spans="1:46" s="11" customFormat="1">
+      <c r="A48" s="11" t="s">
         <v>455</v>
       </c>
-      <c r="P47" s="4"/>
-    </row>
-    <row r="49" spans="1:3">
-      <c r="B49" s="12" t="s">
+      <c r="P48" s="4"/>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="B50" s="12" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
-      <c r="A50" s="12"/>
-      <c r="B50" s="13"/>
-      <c r="C50" t="s">
+    <row r="51" spans="1:3">
+      <c r="A51" s="12"/>
+      <c r="B51" s="13"/>
+      <c r="C51" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
-      <c r="B51" s="14"/>
-      <c r="C51" t="s">
+    <row r="52" spans="1:3">
+      <c r="B52" s="14"/>
+      <c r="C52" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
-      <c r="B52" s="15"/>
-      <c r="C52" t="s">
+    <row r="53" spans="1:3">
+      <c r="B53" s="15"/>
+      <c r="C53" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
-      <c r="B53" s="16"/>
-      <c r="C53" t="s">
+    <row r="54" spans="1:3">
+      <c r="B54" s="16"/>
+      <c r="C54" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
-      <c r="B54" s="1" t="s">
+    <row r="55" spans="1:3">
+      <c r="B55" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C55" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
-      <c r="B55" s="23"/>
-      <c r="C55" t="s">
+    <row r="56" spans="1:3">
+      <c r="B56" s="23"/>
+      <c r="C56" t="s">
         <v>476</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B33:AP33">
+  <conditionalFormatting sqref="B2:AJ22 B23:P24 B34:AQ34 AC39:AC40 AN2:AT24 AK2:AM33 AN25:AR25 AT25 AN26:AT28 Y29:AJ29 AN29:AR29 B29:X30 Z30:AJ30 AN30:AT33 B31:AB33 AD31:AJ33 AR34:AT35 AN35:AP35 B35:AB41 AD35:AJ41 AK35:AM47 AN36:AT36 AN37:AP37 AR37:AT37 AN38:AT47 B42:AJ47 B25:AJ28 R23:AJ24">
     <cfRule type="expression" dxfId="4" priority="3">
-      <formula>$A33=B$1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:AI27 AS24 X28:AI28 B28:W29 Y29:AI29 B30:AA32 AC30:AI32 AQ33:AS34 B41:AI46 B53 AQ36:AS36 B34:AA40 AC34:AI40 AM36:AO36 AM37:AS46 AM35:AS35 AM34:AO34 AM29:AS32 AM28:AQ28 AM25:AS27 AM24:AQ24 AM2:AS23 AJ34:AL46 AJ2:AL32">
-    <cfRule type="expression" dxfId="3" priority="60">
       <formula>$A2=B$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X29">
-    <cfRule type="expression" dxfId="2" priority="7">
-      <formula>$A29=#REF!</formula>
+  <conditionalFormatting sqref="Y30">
+    <cfRule type="expression" dxfId="3" priority="7">
+      <formula>$A30=#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB38:AB39">
-    <cfRule type="expression" dxfId="1" priority="1">
-      <formula>$A38=AB$1</formula>
+  <conditionalFormatting sqref="B54">
+    <cfRule type="expression" dxfId="2" priority="60">
+      <formula>$A54=B$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AR24 AR28:AS28">
-    <cfRule type="expression" dxfId="0" priority="9">
-      <formula>#REF!=AR$1</formula>
+  <conditionalFormatting sqref="AS25 AS29:AT29">
+    <cfRule type="expression" dxfId="1" priority="9">
+      <formula>#REF!=AS$1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q23">
+    <cfRule type="expression" dxfId="0" priority="86">
+      <formula>$A23=Q$1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8175,7 +8210,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313888EE-552D-40AA-8234-3B847E46EF43}">
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="55.7265625" bestFit="1" customWidth="1"/>
@@ -8319,21 +8354,24 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" ht="29">
       <c r="B6" s="27" t="s">
         <v>519</v>
       </c>
+      <c r="C6" t="s">
+        <v>471</v>
+      </c>
       <c r="D6" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="F6" t="s">
-        <v>482</v>
+        <v>602</v>
       </c>
       <c r="G6" t="s">
-        <v>382</v>
+        <v>604</v>
       </c>
       <c r="H6" t="s">
         <v>383</v>
@@ -8349,9 +8387,6 @@
       <c r="D7" t="s">
         <v>599</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>599</v>
-      </c>
       <c r="F7" t="s">
         <v>482</v>
       </c>
@@ -8359,58 +8394,53 @@
         <v>382</v>
       </c>
       <c r="H7" t="s">
-        <v>383</v>
+        <v>87</v>
       </c>
       <c r="I7" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="43.5">
-      <c r="B8" s="29" t="s">
-        <v>587</v>
-      </c>
-      <c r="C8" t="s">
-        <v>472</v>
-      </c>
+    <row r="8" spans="1:10">
+      <c r="B8" s="27"/>
       <c r="D8" t="s">
-        <v>460</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="F8" t="s">
-        <v>525</v>
+        <v>603</v>
       </c>
       <c r="G8" t="s">
-        <v>526</v>
+        <v>86</v>
       </c>
       <c r="H8" t="s">
+        <v>383</v>
+      </c>
+      <c r="I8" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.5">
       <c r="B9" s="29" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="C9" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="D9" t="s">
         <v>460</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="F9" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="G9" t="s">
-        <v>523</v>
+        <v>526</v>
+      </c>
+      <c r="H9" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.5">
-      <c r="B10" s="26" t="s">
-        <v>518</v>
+      <c r="B10" s="29" t="s">
+        <v>588</v>
       </c>
       <c r="C10" t="s">
         <v>470</v>
@@ -8419,146 +8449,137 @@
         <v>460</v>
       </c>
       <c r="E10" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="F10" t="s">
+        <v>522</v>
+      </c>
+      <c r="G10" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="43.5">
+      <c r="B11" s="26" t="s">
+        <v>518</v>
+      </c>
+      <c r="C11" t="s">
+        <v>470</v>
+      </c>
+      <c r="D11" t="s">
+        <v>460</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>485</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F11" t="s">
         <v>486</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G11" t="s">
         <v>89</v>
-      </c>
-      <c r="H10" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="29">
-      <c r="B11" s="28" t="s">
-        <v>520</v>
-      </c>
-      <c r="C11" t="s">
-        <v>471</v>
-      </c>
-      <c r="D11" t="s">
-        <v>473</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>479</v>
-      </c>
-      <c r="F11" t="s">
-        <v>480</v>
-      </c>
-      <c r="G11" t="s">
-        <v>84</v>
       </c>
       <c r="H11" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="43.5">
-      <c r="A12" s="2" t="s">
-        <v>531</v>
-      </c>
-      <c r="B12" s="31" t="s">
-        <v>518</v>
+    <row r="12" spans="1:10" ht="29">
+      <c r="B12" s="28" t="s">
+        <v>520</v>
       </c>
       <c r="C12" t="s">
         <v>471</v>
       </c>
       <c r="D12" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="F12" t="s">
-        <v>598</v>
+        <v>480</v>
       </c>
       <c r="G12" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H12" t="s">
         <v>77</v>
       </c>
-      <c r="I12" t="s">
-        <v>84</v>
-      </c>
     </row>
     <row r="13" spans="1:10" ht="43.5">
-      <c r="B13" s="28" t="s">
-        <v>520</v>
+      <c r="A13" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B13" s="31" t="s">
+        <v>518</v>
       </c>
       <c r="C13" t="s">
-        <v>169</v>
+        <v>471</v>
       </c>
       <c r="D13" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
       <c r="F13" t="s">
-        <v>169</v>
+        <v>598</v>
       </c>
       <c r="G13" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="H13" t="s">
         <v>77</v>
       </c>
       <c r="I13" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="43.5">
+      <c r="B14" s="28" t="s">
+        <v>520</v>
+      </c>
+      <c r="C14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D14" t="s">
+        <v>483</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="F14" t="s">
+        <v>169</v>
+      </c>
+      <c r="G14" t="s">
+        <v>84</v>
+      </c>
+      <c r="H14" t="s">
+        <v>77</v>
+      </c>
+      <c r="I14" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="58">
-      <c r="A14" t="s">
+    <row r="15" spans="1:10" ht="58">
+      <c r="A15" t="s">
         <v>493</v>
       </c>
-      <c r="B14" s="30" t="s">
+      <c r="B15" s="30" t="s">
         <v>586</v>
-      </c>
-      <c r="C14" t="s">
-        <v>472</v>
-      </c>
-      <c r="D14" t="s">
-        <v>494</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>492</v>
-      </c>
-      <c r="F14" t="s">
-        <v>491</v>
-      </c>
-      <c r="G14" t="s">
-        <v>385</v>
-      </c>
-      <c r="H14" t="s">
-        <v>15</v>
-      </c>
-      <c r="I14" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="29">
-      <c r="A15" t="s">
-        <v>536</v>
-      </c>
-      <c r="B15" s="31" t="s">
-        <v>518</v>
       </c>
       <c r="C15" t="s">
         <v>472</v>
       </c>
       <c r="D15" t="s">
-        <v>517</v>
+        <v>494</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>516</v>
+        <v>492</v>
       </c>
       <c r="F15" t="s">
-        <v>515</v>
+        <v>491</v>
       </c>
       <c r="G15" t="s">
-        <v>514</v>
+        <v>385</v>
       </c>
       <c r="H15" t="s">
         <v>15</v>
@@ -8567,194 +8588,194 @@
         <v>502</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" ht="29">
+      <c r="A16" t="s">
+        <v>536</v>
+      </c>
       <c r="B16" s="31" t="s">
         <v>518</v>
       </c>
       <c r="C16" t="s">
         <v>472</v>
       </c>
+      <c r="D16" t="s">
+        <v>517</v>
+      </c>
       <c r="E16" s="2" t="s">
-        <v>529</v>
+        <v>516</v>
       </c>
       <c r="F16" t="s">
-        <v>530</v>
+        <v>515</v>
       </c>
       <c r="G16" t="s">
-        <v>502</v>
+        <v>514</v>
       </c>
       <c r="H16" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" ht="58">
-      <c r="A17" t="s">
-        <v>534</v>
-      </c>
-      <c r="B17" s="30" t="s">
-        <v>586</v>
+      <c r="I16" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
+      <c r="B17" s="31" t="s">
+        <v>518</v>
       </c>
       <c r="C17" t="s">
         <v>472</v>
       </c>
-      <c r="D17" t="s">
-        <v>535</v>
-      </c>
       <c r="E17" s="2" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="F17" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="G17" t="s">
-        <v>71</v>
+        <v>502</v>
       </c>
       <c r="H17" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="43.5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="58">
       <c r="A18" t="s">
-        <v>541</v>
+        <v>534</v>
       </c>
       <c r="B18" s="30" t="s">
         <v>586</v>
       </c>
       <c r="C18" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="D18" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>540</v>
+        <v>532</v>
       </c>
       <c r="F18" t="s">
-        <v>538</v>
+        <v>533</v>
       </c>
       <c r="G18" t="s">
-        <v>539</v>
+        <v>71</v>
       </c>
       <c r="H18" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="29">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="43.5">
       <c r="A19" t="s">
-        <v>545</v>
-      </c>
-      <c r="B19" s="31" t="s">
-        <v>518</v>
+        <v>541</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>586</v>
       </c>
       <c r="C19" t="s">
         <v>470</v>
       </c>
       <c r="D19" t="s">
-        <v>542</v>
+        <v>537</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="F19" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="G19" t="s">
         <v>539</v>
       </c>
       <c r="H19" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="43.5">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="29">
       <c r="A20" t="s">
-        <v>548</v>
-      </c>
-      <c r="B20" s="30" t="s">
-        <v>586</v>
+        <v>545</v>
+      </c>
+      <c r="B20" s="31" t="s">
+        <v>518</v>
       </c>
       <c r="C20" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="D20" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="F20" t="s">
-        <v>549</v>
+        <v>544</v>
       </c>
       <c r="G20" t="s">
         <v>539</v>
       </c>
       <c r="H20" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="43.5">
       <c r="A21" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="B21" s="30" t="s">
-        <v>573</v>
+        <v>586</v>
       </c>
       <c r="C21" t="s">
         <v>472</v>
       </c>
       <c r="D21" t="s">
-        <v>553</v>
+        <v>546</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>551</v>
+        <v>547</v>
       </c>
       <c r="F21" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="G21" t="s">
         <v>539</v>
       </c>
       <c r="H21" t="s">
-        <v>64</v>
-      </c>
-      <c r="I21" t="s">
         <v>78</v>
       </c>
-      <c r="J21" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="72.5">
+    </row>
+    <row r="22" spans="1:10">
       <c r="A22" t="s">
-        <v>559</v>
+        <v>552</v>
       </c>
       <c r="B22" s="30" t="s">
-        <v>586</v>
+        <v>573</v>
       </c>
       <c r="C22" t="s">
         <v>472</v>
       </c>
       <c r="D22" t="s">
-        <v>561</v>
+        <v>553</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>560</v>
+        <v>551</v>
       </c>
       <c r="F22" t="s">
-        <v>558</v>
+        <v>550</v>
       </c>
       <c r="G22" t="s">
-        <v>63</v>
+        <v>539</v>
       </c>
       <c r="H22" t="s">
-        <v>557</v>
+        <v>64</v>
       </c>
       <c r="I22" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="87">
+        <v>78</v>
+      </c>
+      <c r="J22" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="72.5">
       <c r="A23" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="B23" s="30" t="s">
         <v>586</v>
@@ -8763,25 +8784,28 @@
         <v>472</v>
       </c>
       <c r="D23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="F23" t="s">
-        <v>564</v>
+        <v>558</v>
       </c>
       <c r="G23" t="s">
         <v>63</v>
       </c>
       <c r="H23" t="s">
-        <v>64</v>
+        <v>557</v>
       </c>
       <c r="I23" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="43.5">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="87">
+      <c r="A24" t="s">
+        <v>562</v>
+      </c>
       <c r="B24" s="30" t="s">
         <v>586</v>
       </c>
@@ -8789,19 +8813,22 @@
         <v>472</v>
       </c>
       <c r="D24" t="s">
-        <v>554</v>
+        <v>563</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>555</v>
+        <v>565</v>
       </c>
       <c r="F24" t="s">
-        <v>556</v>
+        <v>564</v>
       </c>
       <c r="G24" t="s">
         <v>63</v>
       </c>
       <c r="H24" t="s">
         <v>64</v>
+      </c>
+      <c r="I24" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="43.5">
@@ -8809,42 +8836,39 @@
         <v>586</v>
       </c>
       <c r="C25" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D25" t="s">
-        <v>568</v>
+        <v>554</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>567</v>
+        <v>555</v>
       </c>
       <c r="F25" t="s">
-        <v>566</v>
+        <v>556</v>
       </c>
       <c r="G25" t="s">
         <v>63</v>
       </c>
       <c r="H25" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="58">
-      <c r="A26" t="s">
-        <v>569</v>
-      </c>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="43.5">
       <c r="B26" s="30" t="s">
         <v>586</v>
       </c>
       <c r="C26" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D26" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="F26" t="s">
-        <v>572</v>
+        <v>566</v>
       </c>
       <c r="G26" t="s">
         <v>63</v>
@@ -8852,59 +8876,85 @@
       <c r="H26" t="s">
         <v>71</v>
       </c>
-      <c r="I26" t="s">
-        <v>77</v>
-      </c>
     </row>
     <row r="27" spans="1:10" ht="58">
       <c r="A27" t="s">
-        <v>577</v>
-      </c>
-      <c r="B27" s="31" t="s">
-        <v>518</v>
+        <v>569</v>
+      </c>
+      <c r="B27" s="30" t="s">
+        <v>586</v>
       </c>
       <c r="C27" t="s">
         <v>472</v>
       </c>
       <c r="D27" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="F27" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="G27" t="s">
         <v>63</v>
       </c>
       <c r="H27" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="116">
+        <v>71</v>
+      </c>
+      <c r="I27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="58">
       <c r="A28" t="s">
-        <v>581</v>
-      </c>
-      <c r="B28" s="30" t="s">
-        <v>586</v>
+        <v>577</v>
+      </c>
+      <c r="B28" s="31" t="s">
+        <v>518</v>
       </c>
       <c r="C28" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D28" t="s">
-        <v>578</v>
+        <v>574</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="F28" t="s">
-        <v>580</v>
+        <v>576</v>
       </c>
       <c r="G28" t="s">
         <v>63</v>
       </c>
       <c r="H28" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="116">
+      <c r="A29" t="s">
+        <v>581</v>
+      </c>
+      <c r="B29" s="30" t="s">
+        <v>586</v>
+      </c>
+      <c r="C29" t="s">
+        <v>471</v>
+      </c>
+      <c r="D29" t="s">
+        <v>578</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F29" t="s">
+        <v>580</v>
+      </c>
+      <c r="G29" t="s">
+        <v>63</v>
+      </c>
+      <c r="H29" t="s">
         <v>495</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add (codebook) (investigating interdependence) (exploratory dags) added some graphs and documentation for siblings over 18 and child grand
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Vaccine Uptake - R\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7296CF7-FCF5-4422-9C76-307471315E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{255CEB4E-5ABA-4F44-ABD7-5717E230D679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1743" uniqueCount="605">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1773" uniqueCount="620">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -1909,6 +1909,51 @@
   </si>
   <si>
     <t>test_father_highest_education (VS)</t>
+  </si>
+  <si>
+    <t>Yes?</t>
+  </si>
+  <si>
+    <t>child_grand_income</t>
+  </si>
+  <si>
+    <t>child_grand * test_household_income</t>
+  </si>
+  <si>
+    <t>Having a (presence) grandparent reduces the uptake of both vaccines as household income increases, whereas the uptake increases with household income otherwise</t>
+  </si>
+  <si>
+    <t>child_grand_parents</t>
+  </si>
+  <si>
+    <t>An increasing number of grandparents reduces the uptakeof both vaccines when the child only has 1 parent as opposed to increasing the uptake of vaccines when the child has 2 parents</t>
+  </si>
+  <si>
+    <t>child_grand * child_parents</t>
+  </si>
+  <si>
+    <t>child_grand_parents_income</t>
+  </si>
+  <si>
+    <t>child_grand * child_parents * test_household_income</t>
+  </si>
+  <si>
+    <t>Having 1 or 2 parents doesn't change the relationship between the number of grandparents and test_household_income on vaccine uptake</t>
+  </si>
+  <si>
+    <t>Too many outliers that are skewing the results</t>
+  </si>
+  <si>
+    <t>child_grand_siblings_over_18_income</t>
+  </si>
+  <si>
+    <t>child_grand * siblings_over_18 * test_household_income</t>
+  </si>
+  <si>
+    <t>Not enough data to determine how the number of siblings over 18 impacts the relationship between income and uptake for different number of grandparents in a household</t>
+  </si>
+  <si>
+    <t>Too little data</t>
   </si>
 </sst>
 </file>
@@ -7801,7 +7846,7 @@
       <c r="A14" t="s">
         <v>60</v>
       </c>
-      <c r="R14" s="16"/>
+      <c r="R14" s="23"/>
       <c r="AC14" s="23" t="s">
         <v>394</v>
       </c>
@@ -7923,7 +7968,7 @@
         <v>77</v>
       </c>
       <c r="P29" s="15"/>
-      <c r="R29" s="16" t="s">
+      <c r="R29" s="23" t="s">
         <v>423</v>
       </c>
       <c r="V29" s="16"/>
@@ -8210,7 +8255,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313888EE-552D-40AA-8234-3B847E46EF43}">
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="55.7265625" bestFit="1" customWidth="1"/>
@@ -8956,6 +9001,104 @@
       </c>
       <c r="H29" t="s">
         <v>495</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="58">
+      <c r="B30" s="25" t="s">
+        <v>605</v>
+      </c>
+      <c r="C30" t="s">
+        <v>472</v>
+      </c>
+      <c r="D30" t="s">
+        <v>606</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="F30" t="s">
+        <v>607</v>
+      </c>
+      <c r="G30" t="s">
+        <v>64</v>
+      </c>
+      <c r="H30" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="72.5">
+      <c r="B31" s="25" t="s">
+        <v>605</v>
+      </c>
+      <c r="C31" t="s">
+        <v>472</v>
+      </c>
+      <c r="D31" t="s">
+        <v>609</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="F31" t="s">
+        <v>611</v>
+      </c>
+      <c r="G31" t="s">
+        <v>64</v>
+      </c>
+      <c r="H31" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="58">
+      <c r="A32" t="s">
+        <v>615</v>
+      </c>
+      <c r="B32" s="25" t="s">
+        <v>573</v>
+      </c>
+      <c r="D32" t="s">
+        <v>612</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="F32" t="s">
+        <v>613</v>
+      </c>
+      <c r="G32" t="s">
+        <v>64</v>
+      </c>
+      <c r="H32" t="s">
+        <v>60</v>
+      </c>
+      <c r="I32" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="72.5">
+      <c r="A33" t="s">
+        <v>619</v>
+      </c>
+      <c r="B33" s="25" t="s">
+        <v>573</v>
+      </c>
+      <c r="D33" t="s">
+        <v>616</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="F33" t="s">
+        <v>617</v>
+      </c>
+      <c r="G33" t="s">
+        <v>64</v>
+      </c>
+      <c r="H33" t="s">
+        <v>582</v>
+      </c>
+      <c r="I33" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
edit (codebook.xlsx) removed the following redundant variables from the causal relationships page and greyed them out from the codebook page: test_mother_highest_education test_father_highest_education test_parents_highest_education vulnerable_individuals mother_stay_home
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Vaccine Uptake - R\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{255CEB4E-5ABA-4F44-ABD7-5717E230D679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{802C7D65-13CF-44BB-B2AA-FB06500EB096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1773" uniqueCount="620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1794" uniqueCount="631">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -1248,9 +1248,6 @@
     <t>test_mother_highest_education</t>
   </si>
   <si>
-    <t>Majority of the unemployed population are mothers and (1415 / 1525 unemployed mothers are stay home mothers)</t>
-  </si>
-  <si>
     <t>birth_order</t>
   </si>
   <si>
@@ -1344,9 +1341,6 @@
     <t>unmarried have a lower mean income (4.6 M JPY/Y vs 7.6 M JPY/Y)</t>
   </si>
   <si>
-    <t>almost no mothers stay home if they're divorced vs ~25% stay home if they’re married</t>
-  </si>
-  <si>
     <t>mean household size increases with marriage (3.2 v 3.9)</t>
   </si>
   <si>
@@ -1356,9 +1350,6 @@
     <t>siblings = -(income)^2</t>
   </si>
   <si>
-    <t>parents highest education doesn't impact the proportion of mothers who stay home (26% to 33%)</t>
-  </si>
-  <si>
     <t>mean size doesn't change but more highsch/junior high have larger families (&gt;= 5)</t>
   </si>
   <si>
@@ -1383,9 +1374,6 @@
     <t>a more recen t covid vaccination is associated with having obtained more doses of the vaccine</t>
   </si>
   <si>
-    <t>having a parent with chronic illness isn't assocaited with vulnerable individuals</t>
-  </si>
-  <si>
     <t>fathers and mothers with chronic illnesses were more likely to have the influenza vaccine</t>
   </si>
   <si>
@@ -1395,12 +1383,6 @@
     <t>being unmarried is associated with current chronic illness</t>
   </si>
   <si>
-    <t>mothers staying home is associated with lower income</t>
-  </si>
-  <si>
-    <t>no stay-home mum is associated with more grandparents at home (6.8 %  vs 3.6%)</t>
-  </si>
-  <si>
     <t>the age of children of single fathers Is much higher</t>
   </si>
   <si>
@@ -1644,9 +1626,6 @@
     <t>child_siblings*age_of_interest*age_cat (??)</t>
   </si>
   <si>
-    <t>The increase in full vaccination increases as the number of siblings increases</t>
-  </si>
-  <si>
     <t>age_child_siblings_</t>
   </si>
   <si>
@@ -1911,18 +1890,12 @@
     <t>test_father_highest_education (VS)</t>
   </si>
   <si>
-    <t>Yes?</t>
-  </si>
-  <si>
     <t>child_grand_income</t>
   </si>
   <si>
     <t>child_grand * test_household_income</t>
   </si>
   <si>
-    <t>Having a (presence) grandparent reduces the uptake of both vaccines as household income increases, whereas the uptake increases with household income otherwise</t>
-  </si>
-  <si>
     <t>child_grand_parents</t>
   </si>
   <si>
@@ -1950,10 +1923,70 @@
     <t>child_grand * siblings_over_18 * test_household_income</t>
   </si>
   <si>
-    <t>Not enough data to determine how the number of siblings over 18 impacts the relationship between income and uptake for different number of grandparents in a household</t>
-  </si>
-  <si>
     <t>Too little data</t>
+  </si>
+  <si>
+    <t>Not enough data to determine how the number of siblings over 18 impacts the relationship between income and uptake for different number of grandparents in a household. (and thus we can't determine how the slope differs with different number of gr</t>
+  </si>
+  <si>
+    <t>the relationship between Vaccine uptake and income varies for families where the COI has 0, 1 and 2+ grandparents respectively</t>
+  </si>
+  <si>
+    <t>The increase in full vaccination increases as the number of siblings increases across ages and age categories</t>
+  </si>
+  <si>
+    <t>child_grand_siblings_over_18</t>
+  </si>
+  <si>
+    <t>Insufficient data to determine how the uptake varies with no. of grandparents for diff number of siblings over 18</t>
+  </si>
+  <si>
+    <t>child_grand * siblings_over_18</t>
+  </si>
+  <si>
+    <t>Run regresssions</t>
+  </si>
+  <si>
+    <t>Include in diff models</t>
+  </si>
+  <si>
+    <t>income_father_mother_education_</t>
+  </si>
+  <si>
+    <t>child_grand_father_employment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">There is insufficient data to determine if </t>
+  </si>
+  <si>
+    <t>child_grand*father_employment_status</t>
+  </si>
+  <si>
+    <t>child_grand_mother_employment_status</t>
+  </si>
+  <si>
+    <t>Unemployed or mothers doing part-time work showed decreased lack of uptake as compared to mothers working full-time</t>
+  </si>
+  <si>
+    <t>child_grand*mother_employment_status</t>
+  </si>
+  <si>
+    <t>The anova test for interaction wasn't significant</t>
+  </si>
+  <si>
+    <t>child_grand_mother_stay_home</t>
+  </si>
+  <si>
+    <t>for children whose mothers stay home, there seems to be an increasing uptake as the number of grandparents also increases</t>
+  </si>
+  <si>
+    <t>child_grand*mother_stay_home</t>
+  </si>
+  <si>
+    <t>Too little data?</t>
+  </si>
+  <si>
+    <t>reference age_child_siblings</t>
   </si>
 </sst>
 </file>
@@ -2013,7 +2046,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2092,14 +2125,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2122,26 +2149,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="2"/>
-      </left>
-      <right style="thin">
-        <color theme="2"/>
-      </right>
-      <top style="thin">
-        <color theme="2"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2151,9 +2163,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2189,36 +2198,14 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font>
-        <color theme="2" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="2" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color theme="2" tint="-0.24994659260841701"/>
@@ -2569,27 +2556,29 @@
     <col min="20" max="20" width="25.453125" bestFit="1" customWidth="1"/>
     <col min="21" max="22" width="24.90625" bestFit="1" customWidth="1"/>
     <col min="23" max="54" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="55" max="61" width="35.81640625" bestFit="1" customWidth="1"/>
+    <col min="55" max="56" width="35.81640625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="58" max="61" width="35.81640625" bestFit="1" customWidth="1"/>
     <col min="62" max="62" width="22.90625" bestFit="1" customWidth="1"/>
     <col min="63" max="63" width="22.90625" customWidth="1"/>
-    <col min="64" max="64" width="35.81640625" style="21" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="35.81640625" style="20" bestFit="1" customWidth="1"/>
     <col min="65" max="65" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="66" max="66" width="35.81640625" bestFit="1" customWidth="1"/>
     <col min="67" max="68" width="35.81640625" customWidth="1"/>
     <col min="69" max="69" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="35.81640625" style="13" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="35.81640625" style="12" bestFit="1" customWidth="1"/>
     <col min="71" max="71" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="72" max="74" width="35.81640625" bestFit="1" customWidth="1"/>
     <col min="75" max="75" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="76" max="79" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="80" max="82" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="83" max="86" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="87" max="88" width="35.81640625" style="6" customWidth="1"/>
-    <col min="89" max="89" width="35.81640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="80" max="83" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="84" max="86" width="35.81640625" bestFit="1" customWidth="1"/>
+    <col min="87" max="88" width="35.81640625" style="4" customWidth="1"/>
+    <col min="89" max="89" width="35.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="90" max="90" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="35.81640625" style="6" customWidth="1"/>
+    <col min="91" max="91" width="35.81640625" style="4" customWidth="1"/>
     <col min="92" max="95" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="96" max="97" width="35.81640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="96" max="97" width="35.81640625" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:98">
@@ -2630,7 +2619,7 @@
         <v>15</v>
       </c>
       <c r="M1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="N1" t="s">
         <v>17</v>
@@ -2761,7 +2750,7 @@
       <c r="BD1" t="s">
         <v>61</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BE1" s="4" t="s">
         <v>62</v>
       </c>
       <c r="BF1" t="s">
@@ -2780,9 +2769,9 @@
         <v>15</v>
       </c>
       <c r="BK1" t="s">
-        <v>502</v>
-      </c>
-      <c r="BL1" s="21" t="s">
+        <v>496</v>
+      </c>
+      <c r="BL1" s="20" t="s">
         <v>67</v>
       </c>
       <c r="BM1" s="4" t="s">
@@ -2792,15 +2781,15 @@
         <v>69</v>
       </c>
       <c r="BO1" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
       <c r="BP1" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="BQ1" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="BR1" s="13" t="s">
+      <c r="BR1" s="12" t="s">
         <v>71</v>
       </c>
       <c r="BS1" s="4" t="s">
@@ -2839,7 +2828,7 @@
       <c r="CD1" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CE1" s="4" t="s">
         <v>84</v>
       </c>
       <c r="CF1" t="s">
@@ -2851,20 +2840,20 @@
       <c r="CH1" t="s">
         <v>87</v>
       </c>
-      <c r="CI1" s="6" t="s">
+      <c r="CI1" s="4" t="s">
         <v>382</v>
       </c>
-      <c r="CJ1" s="6" t="s">
+      <c r="CJ1" s="4" t="s">
         <v>383</v>
       </c>
-      <c r="CK1" s="8" t="s">
+      <c r="CK1" s="4" t="s">
         <v>88</v>
       </c>
       <c r="CL1" t="s">
         <v>89</v>
       </c>
-      <c r="CM1" s="6" t="s">
-        <v>589</v>
+      <c r="CM1" s="4" t="s">
+        <v>582</v>
       </c>
       <c r="CN1" t="s">
         <v>90</v>
@@ -2878,10 +2867,10 @@
       <c r="CQ1" t="s">
         <v>93</v>
       </c>
-      <c r="CR1" s="8" t="s">
+      <c r="CR1" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="CS1" s="8" t="s">
+      <c r="CS1" s="7" t="s">
         <v>95</v>
       </c>
       <c r="CT1" s="2"/>
@@ -3055,7 +3044,7 @@
       <c r="BD2" t="s">
         <v>96</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BE2" s="4" t="s">
         <v>96</v>
       </c>
       <c r="BF2" t="s">
@@ -3076,7 +3065,7 @@
       <c r="BK2" t="s">
         <v>96</v>
       </c>
-      <c r="BL2" s="21" t="s">
+      <c r="BL2" s="20" t="s">
         <v>96</v>
       </c>
       <c r="BM2" s="4" t="s">
@@ -3086,15 +3075,15 @@
         <v>96</v>
       </c>
       <c r="BO2" t="s">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="BP2" t="s">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="BQ2" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="BR2" s="13" t="s">
+      <c r="BR2" s="12" t="s">
         <v>96</v>
       </c>
       <c r="BS2" s="4" t="s">
@@ -3133,7 +3122,7 @@
       <c r="CD2" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="CE2" t="s">
+      <c r="CE2" s="4" t="s">
         <v>96</v>
       </c>
       <c r="CF2" t="s">
@@ -3145,19 +3134,19 @@
       <c r="CH2" t="s">
         <v>96</v>
       </c>
-      <c r="CI2" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="CJ2" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="CK2" s="8" t="s">
+      <c r="CI2" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="CJ2" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="CK2" s="4" t="s">
         <v>96</v>
       </c>
       <c r="CL2" t="s">
         <v>96</v>
       </c>
-      <c r="CM2" s="6" t="s">
+      <c r="CM2" s="4" t="s">
         <v>96</v>
       </c>
       <c r="CN2" t="s">
@@ -3172,16 +3161,16 @@
       <c r="CQ2" t="s">
         <v>96</v>
       </c>
-      <c r="CR2" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="CS2" s="8" t="s">
+      <c r="CR2" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="CS2" s="7" t="s">
         <v>96</v>
       </c>
       <c r="CT2" s="2"/>
     </row>
     <row r="3" spans="1:98" s="2" customFormat="1" ht="101.5">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -3218,7 +3207,7 @@
         <v>117</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="N3" s="2" t="s">
         <v>118</v>
@@ -3285,7 +3274,7 @@
       <c r="BD3" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="BE3" s="2" t="s">
+      <c r="BE3" s="3" t="s">
         <v>129</v>
       </c>
       <c r="BF3" s="2" t="s">
@@ -3304,27 +3293,27 @@
         <v>117</v>
       </c>
       <c r="BK3" s="2" t="s">
-        <v>503</v>
-      </c>
-      <c r="BL3" s="22" t="s">
-        <v>451</v>
+        <v>497</v>
+      </c>
+      <c r="BL3" s="21" t="s">
+        <v>445</v>
       </c>
       <c r="BM3" s="3" t="s">
-        <v>452</v>
+        <v>446</v>
       </c>
       <c r="BN3" s="2" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="BO3" t="s">
-        <v>497</v>
+        <v>491</v>
       </c>
       <c r="BP3" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="BQ3" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="BR3" s="17" t="s">
+      <c r="BR3" s="16" t="s">
         <v>135</v>
       </c>
       <c r="BS3" s="3" t="s">
@@ -3360,7 +3349,7 @@
       <c r="CD3" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="CE3" s="2" t="s">
+      <c r="CE3" s="3" t="s">
         <v>147</v>
       </c>
       <c r="CF3" s="2" t="s">
@@ -3372,18 +3361,18 @@
       <c r="CH3" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="CI3" s="5" t="s">
-        <v>597</v>
-      </c>
-      <c r="CJ3" s="5" t="s">
-        <v>597</v>
-      </c>
-      <c r="CK3" s="7"/>
+      <c r="CI3" s="3" t="s">
+        <v>590</v>
+      </c>
+      <c r="CJ3" s="3" t="s">
+        <v>590</v>
+      </c>
+      <c r="CK3" s="3"/>
       <c r="CL3" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="CM3" s="5" t="s">
-        <v>596</v>
+      <c r="CM3" s="3" t="s">
+        <v>589</v>
       </c>
       <c r="CN3" s="2" t="s">
         <v>152</v>
@@ -3397,11 +3386,11 @@
       <c r="CQ3" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="CR3" s="7"/>
-      <c r="CS3" s="7"/>
+      <c r="CR3" s="6"/>
+      <c r="CS3" s="6"/>
     </row>
     <row r="4" spans="1:98">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B4" t="s">
@@ -3563,13 +3552,13 @@
       <c r="BB4" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="BC4" s="11" t="s">
+      <c r="BC4" s="10" t="s">
         <v>100</v>
       </c>
       <c r="BD4" t="s">
         <v>100</v>
       </c>
-      <c r="BE4" t="s">
+      <c r="BE4" s="4" t="s">
         <v>100</v>
       </c>
       <c r="BF4" t="s">
@@ -3581,7 +3570,7 @@
       <c r="BH4" t="s">
         <v>99</v>
       </c>
-      <c r="BI4" s="11" t="s">
+      <c r="BI4" s="10" t="s">
         <v>99</v>
       </c>
       <c r="BJ4" t="s">
@@ -3590,7 +3579,7 @@
       <c r="BK4" t="s">
         <v>99</v>
       </c>
-      <c r="BL4" s="21" t="s">
+      <c r="BL4" s="20" t="s">
         <v>98</v>
       </c>
       <c r="BM4" s="4" t="s">
@@ -3608,16 +3597,16 @@
       <c r="BQ4" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="BR4" s="13" t="s">
+      <c r="BR4" s="12" t="s">
         <v>99</v>
       </c>
       <c r="BS4" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="BT4" s="11" t="s">
+      <c r="BT4" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="BU4" s="11" t="s">
+      <c r="BU4" s="10" t="s">
         <v>99</v>
       </c>
       <c r="BV4" t="s">
@@ -3627,7 +3616,7 @@
         <v>260</v>
       </c>
       <c r="BX4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="BY4" t="s">
         <v>99</v>
@@ -3647,7 +3636,7 @@
       <c r="CD4" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="CE4" s="11" t="s">
+      <c r="CE4" s="4" t="s">
         <v>99</v>
       </c>
       <c r="CF4" t="s">
@@ -3659,19 +3648,19 @@
       <c r="CH4" t="s">
         <v>99</v>
       </c>
-      <c r="CI4" s="6" t="s">
+      <c r="CI4" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="CJ4" s="6" t="s">
+      <c r="CJ4" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="CK4" s="8" t="s">
+      <c r="CK4" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="CL4" s="11" t="s">
+      <c r="CL4" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="CM4" s="6" t="s">
+      <c r="CM4" s="4" t="s">
         <v>99</v>
       </c>
       <c r="CN4" t="s">
@@ -3686,10 +3675,10 @@
       <c r="CQ4" t="s">
         <v>99</v>
       </c>
-      <c r="CR4" s="8" t="s">
+      <c r="CR4" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="CS4" s="8" t="s">
+      <c r="CS4" s="7" t="s">
         <v>99</v>
       </c>
     </row>
@@ -3712,13 +3701,13 @@
       <c r="F5" t="s">
         <v>103</v>
       </c>
-      <c r="CR5" s="8"/>
-      <c r="CS5" s="8"/>
+      <c r="CR5" s="7"/>
+      <c r="CS5" s="7"/>
     </row>
     <row r="6" spans="1:98">
       <c r="A6" s="1"/>
-      <c r="CR6" s="8"/>
-      <c r="CS6" s="8"/>
+      <c r="CR6" s="7"/>
+      <c r="CS6" s="7"/>
     </row>
     <row r="7" spans="1:98">
       <c r="A7" s="1" t="s">
@@ -3778,7 +3767,7 @@
       <c r="BD7" t="s">
         <v>109</v>
       </c>
-      <c r="BE7" t="s">
+      <c r="BE7" s="4" t="s">
         <v>109</v>
       </c>
       <c r="BF7" t="s">
@@ -3790,7 +3779,7 @@
       <c r="BJ7" t="s">
         <v>108</v>
       </c>
-      <c r="BL7" s="21" t="s">
+      <c r="BL7" s="20" t="s">
         <v>109</v>
       </c>
       <c r="BM7" s="4" t="s">
@@ -3809,20 +3798,20 @@
         <v>108</v>
       </c>
       <c r="BW7" s="4" t="s">
-        <v>414</v>
-      </c>
-      <c r="CR7" s="8"/>
-      <c r="CS7" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="CR7" s="7"/>
+      <c r="CS7" s="7"/>
     </row>
     <row r="8" spans="1:98">
       <c r="A8" s="1"/>
-      <c r="CR8" s="8"/>
-      <c r="CS8" s="8"/>
+      <c r="CR8" s="7"/>
+      <c r="CS8" s="7"/>
     </row>
     <row r="9" spans="1:98">
       <c r="A9" s="1"/>
-      <c r="CR9" s="8"/>
-      <c r="CS9" s="8"/>
+      <c r="CR9" s="7"/>
+      <c r="CS9" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
@@ -4278,7 +4267,7 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C14" t="s">
         <v>260</v>
@@ -4287,10 +4276,10 @@
         <v>109</v>
       </c>
       <c r="E14" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F14" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="G14" t="s">
         <v>283</v>
@@ -4299,7 +4288,7 @@
         <v>275</v>
       </c>
       <c r="I14" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="J14" t="s">
         <v>307</v>
@@ -4824,41 +4813,41 @@
         <v>307</v>
       </c>
     </row>
-    <row r="39" spans="1:14">
-      <c r="A39" t="s">
-        <v>96</v>
-      </c>
-      <c r="B39" t="s">
+    <row r="39" spans="1:14" s="4" customFormat="1">
+      <c r="A39" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B39" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E39" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F39" s="4" t="s">
         <v>349</v>
       </c>
-      <c r="G39" t="s">
+      <c r="G39" s="4" t="s">
         <v>309</v>
       </c>
-      <c r="H39" t="s">
-        <v>307</v>
-      </c>
-      <c r="I39" t="s">
+      <c r="H39" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="I39" s="4" t="s">
         <v>310</v>
       </c>
-      <c r="J39" t="s">
-        <v>307</v>
-      </c>
-      <c r="K39" t="s">
+      <c r="J39" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="K39" s="4" t="s">
         <v>311</v>
       </c>
-      <c r="L39" t="s">
+      <c r="L39" s="4" t="s">
         <v>307</v>
       </c>
     </row>
@@ -5034,7 +5023,7 @@
         <v>117</v>
       </c>
       <c r="F47" t="s">
-        <v>501</v>
+        <v>495</v>
       </c>
       <c r="G47" t="s">
         <v>15</v>
@@ -5048,19 +5037,19 @@
         <v>96</v>
       </c>
       <c r="B48" t="s">
-        <v>502</v>
+        <v>496</v>
       </c>
       <c r="C48" t="s">
         <v>261</v>
       </c>
       <c r="D48" t="s">
-        <v>504</v>
+        <v>498</v>
       </c>
       <c r="E48" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="F48" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="G48" t="s">
         <v>15</v>
@@ -5080,13 +5069,13 @@
         <v>96</v>
       </c>
       <c r="D49" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="E49" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="F49" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -5094,13 +5083,13 @@
         <v>96</v>
       </c>
       <c r="D50" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="E50" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="F50" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -5114,7 +5103,7 @@
         <v>169</v>
       </c>
       <c r="F51" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
     </row>
     <row r="52" spans="1:12" s="4" customFormat="1">
@@ -5131,7 +5120,7 @@
         <v>109</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="F52" s="4" t="s">
         <v>318</v>
@@ -5163,7 +5152,7 @@
         <v>109</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>319</v>
@@ -5186,7 +5175,7 @@
         <v>96</v>
       </c>
       <c r="B54" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
       <c r="C54" t="s">
         <v>260</v>
@@ -5195,10 +5184,10 @@
         <v>109</v>
       </c>
       <c r="E54" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
       <c r="F54" t="s">
-        <v>500</v>
+        <v>494</v>
       </c>
       <c r="G54" t="s">
         <v>68</v>
@@ -5213,7 +5202,7 @@
         <v>307</v>
       </c>
       <c r="K54" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="L54" t="s">
         <v>307</v>
@@ -5233,10 +5222,10 @@
         <v>109</v>
       </c>
       <c r="E55" t="s">
-        <v>499</v>
+        <v>493</v>
       </c>
       <c r="F55" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="G55" t="s">
         <v>68</v>
@@ -5256,7 +5245,7 @@
         <v>96</v>
       </c>
       <c r="B56" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="C56" t="s">
         <v>260</v>
@@ -5265,13 +5254,13 @@
         <v>109</v>
       </c>
       <c r="E56" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
       <c r="F56" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="G56" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="H56" t="s">
         <v>307</v>
@@ -5465,28 +5454,28 @@
       <c r="E68" t="s">
         <v>167</v>
       </c>
-      <c r="F68" s="11" t="s">
+      <c r="F68" s="10" t="s">
         <v>355</v>
       </c>
-      <c r="G68" s="11" t="s">
+      <c r="G68" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H68" s="11" t="s">
-        <v>307</v>
-      </c>
-      <c r="I68" s="11" t="s">
+      <c r="H68" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="I68" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="J68" s="11" t="s">
-        <v>307</v>
-      </c>
-      <c r="K68" s="11" t="s">
+      <c r="J68" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="K68" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="L68" s="11" t="s">
-        <v>307</v>
-      </c>
-      <c r="M68" s="11"/>
+      <c r="L68" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="M68" s="10"/>
     </row>
     <row r="69" spans="1:13">
       <c r="A69" t="s">
@@ -5719,7 +5708,7 @@
         <v>181</v>
       </c>
       <c r="F86" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="G86" t="s">
         <v>321</v>
@@ -5737,7 +5726,7 @@
         <v>2</v>
       </c>
       <c r="E87" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -5749,7 +5738,7 @@
         <v>3</v>
       </c>
       <c r="E88" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -5761,7 +5750,7 @@
         <v>4</v>
       </c>
       <c r="E89" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="90" spans="1:8">
@@ -5773,7 +5762,7 @@
         <v>5</v>
       </c>
       <c r="E90" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="91" spans="1:8">
@@ -5785,7 +5774,7 @@
         <v>6</v>
       </c>
       <c r="E91" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -5797,7 +5786,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -5809,7 +5798,7 @@
         <v>8</v>
       </c>
       <c r="E93" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -5821,7 +5810,7 @@
         <v>9</v>
       </c>
       <c r="E94" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -5833,7 +5822,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="96" spans="1:8">
@@ -5845,7 +5834,7 @@
         <v>11</v>
       </c>
       <c r="E96" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="97" spans="1:16">
@@ -5857,7 +5846,7 @@
         <v>12</v>
       </c>
       <c r="E97" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="98" spans="1:16">
@@ -5869,7 +5858,7 @@
         <v>13</v>
       </c>
       <c r="E98" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="99" spans="1:16">
@@ -5881,7 +5870,7 @@
         <v>14</v>
       </c>
       <c r="E99" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="100" spans="1:16">
@@ -5892,8 +5881,8 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="E100" s="20" t="s">
-        <v>411</v>
+      <c r="E100" s="19" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="101" spans="1:16">
@@ -5905,7 +5894,7 @@
         <v>16</v>
       </c>
       <c r="E101" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="102" spans="1:16">
@@ -5917,7 +5906,7 @@
         <v>17</v>
       </c>
       <c r="E102" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="103" spans="1:16">
@@ -6182,7 +6171,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="118" spans="1:17" s="6" customFormat="1">
+    <row r="118" spans="1:17" s="5" customFormat="1">
       <c r="A118" t="s">
         <v>96</v>
       </c>
@@ -6489,75 +6478,75 @@
         <v>215</v>
       </c>
     </row>
-    <row r="134" spans="1:16">
-      <c r="A134" t="s">
-        <v>96</v>
-      </c>
-      <c r="B134" t="s">
+    <row r="134" spans="1:16" s="4" customFormat="1">
+      <c r="A134" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B134" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="C134" t="s">
+      <c r="C134" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="D134">
+      <c r="D134" s="4">
         <v>0</v>
       </c>
-      <c r="E134" t="s">
+      <c r="E134" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="F134" t="s">
+      <c r="F134" s="4" t="s">
         <v>364</v>
       </c>
-      <c r="G134" t="s">
+      <c r="G134" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="H134" t="s">
-        <v>307</v>
-      </c>
-      <c r="I134" t="s">
+      <c r="H134" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="I134" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="J134" t="s">
-        <v>307</v>
-      </c>
-      <c r="K134" t="s">
+      <c r="J134" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="K134" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="L134" t="s">
-        <v>307</v>
-      </c>
-      <c r="M134" t="s">
+      <c r="L134" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="M134" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="N134" t="s">
-        <v>307</v>
-      </c>
-      <c r="O134" t="s">
+      <c r="N134" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="O134" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="P134" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="135" spans="1:16">
-      <c r="A135" t="s">
-        <v>96</v>
-      </c>
-      <c r="D135">
+      <c r="P134" s="4" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="135" spans="1:16" s="4" customFormat="1">
+      <c r="A135" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D135" s="4">
         <v>1</v>
       </c>
-      <c r="E135" t="s">
+      <c r="E135" s="4" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="136" spans="1:16">
-      <c r="A136" t="s">
-        <v>96</v>
-      </c>
-      <c r="D136" t="s">
+    <row r="136" spans="1:16" s="4" customFormat="1">
+      <c r="A136" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D136" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="E136" t="s">
+      <c r="E136" s="4" t="s">
         <v>223</v>
       </c>
     </row>
@@ -6658,7 +6647,7 @@
         <v>0</v>
       </c>
       <c r="E141" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F141" t="s">
         <v>366</v>
@@ -6702,7 +6691,7 @@
         <v>1</v>
       </c>
       <c r="E142" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="143" spans="1:16">
@@ -6752,7 +6741,7 @@
         <v>0</v>
       </c>
       <c r="E146" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F146" t="s">
         <v>367</v>
@@ -6796,7 +6785,7 @@
         <v>1</v>
       </c>
       <c r="E147" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="148" spans="1:16">
@@ -6846,7 +6835,7 @@
         <v>0</v>
       </c>
       <c r="E151" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F151" t="s">
         <v>368</v>
@@ -6878,7 +6867,7 @@
         <v>1</v>
       </c>
       <c r="E152" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="153" spans="1:16">
@@ -7257,339 +7246,339 @@
         <v>253</v>
       </c>
     </row>
-    <row r="179" spans="1:16" s="32" customFormat="1">
-      <c r="A179" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="B179" s="32" t="s">
+    <row r="179" spans="1:16" s="4" customFormat="1">
+      <c r="A179" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B179" s="4" t="s">
         <v>382</v>
       </c>
-      <c r="C179" s="32" t="s">
+      <c r="C179" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="D179" s="32">
+      <c r="D179" s="4">
         <v>0</v>
       </c>
-      <c r="E179" s="32" t="s">
-        <v>389</v>
-      </c>
-      <c r="F179" s="32" t="s">
-        <v>594</v>
-      </c>
-      <c r="G179" s="32" t="s">
+      <c r="E179" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="F179" s="4" t="s">
+        <v>587</v>
+      </c>
+      <c r="G179" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="H179" s="32" t="s">
-        <v>307</v>
-      </c>
-      <c r="I179" s="32" t="s">
+      <c r="H179" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="I179" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="J179" s="32" t="s">
-        <v>307</v>
-      </c>
-      <c r="K179" s="32" t="s">
+      <c r="J179" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="K179" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="L179" s="32" t="s">
-        <v>307</v>
-      </c>
-      <c r="M179" s="32" t="s">
+      <c r="L179" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="M179" s="4" t="s">
         <v>325</v>
       </c>
-      <c r="N179" s="32" t="s">
-        <v>307</v>
-      </c>
-      <c r="O179" s="32" t="s">
+      <c r="N179" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="O179" s="4" t="s">
         <v>326</v>
       </c>
-      <c r="P179" s="32" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="180" spans="1:16" s="32" customFormat="1">
-      <c r="A180" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D180" s="32">
+      <c r="P179" s="4" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="180" spans="1:16" s="4" customFormat="1">
+      <c r="A180" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D180" s="4">
         <v>1</v>
       </c>
-      <c r="E180" s="32" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="181" spans="1:16" s="32" customFormat="1">
-      <c r="A181" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D181" s="32">
+      <c r="E180" s="4" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="181" spans="1:16" s="4" customFormat="1">
+      <c r="A181" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D181" s="4">
         <v>1.5</v>
       </c>
-      <c r="E181" s="32" t="s">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="182" spans="1:16" s="32" customFormat="1">
-      <c r="A182" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D182" s="32">
+      <c r="E181" s="4" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="182" spans="1:16" s="4" customFormat="1">
+      <c r="A182" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D182" s="4">
         <v>2</v>
       </c>
-      <c r="E182" s="32" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="183" spans="1:16" s="32" customFormat="1">
-      <c r="A183" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D183" s="32">
+      <c r="E182" s="4" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="183" spans="1:16" s="4" customFormat="1">
+      <c r="A183" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D183" s="4">
         <v>3</v>
       </c>
-      <c r="E183" s="32" t="s">
+      <c r="E183" s="4" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="184" spans="1:16" s="32" customFormat="1">
-      <c r="A184" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D184" s="32">
+    <row r="184" spans="1:16" s="4" customFormat="1">
+      <c r="A184" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D184" s="4">
         <v>4</v>
       </c>
-      <c r="E184" s="32" t="s">
+      <c r="E184" s="4" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="185" spans="1:16" s="32" customFormat="1">
-      <c r="A185" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D185" s="32" t="s">
+    <row r="185" spans="1:16" s="4" customFormat="1">
+      <c r="A185" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D185" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="E185" s="32" t="s">
+      <c r="E185" s="4" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="186" spans="1:16" s="32" customFormat="1">
-      <c r="A186" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="B186" s="32" t="s">
+    <row r="186" spans="1:16" s="4" customFormat="1">
+      <c r="A186" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B186" s="4" t="s">
         <v>383</v>
       </c>
-      <c r="C186" s="32" t="s">
+      <c r="C186" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="D186" s="32">
+      <c r="D186" s="4">
         <v>0</v>
       </c>
-      <c r="E186" s="32" t="s">
-        <v>389</v>
-      </c>
-      <c r="F186" s="32" t="s">
-        <v>593</v>
-      </c>
-      <c r="G186" s="32" t="s">
+      <c r="E186" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="F186" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="G186" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="H186" s="32" t="s">
-        <v>307</v>
-      </c>
-      <c r="I186" s="32" t="s">
+      <c r="H186" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="I186" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="J186" s="32" t="s">
-        <v>307</v>
-      </c>
-      <c r="K186" s="32" t="s">
+      <c r="J186" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="K186" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="L186" s="32" t="s">
-        <v>307</v>
-      </c>
-      <c r="M186" s="32" t="s">
+      <c r="L186" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="M186" s="4" t="s">
         <v>325</v>
       </c>
-      <c r="N186" s="32" t="s">
-        <v>307</v>
-      </c>
-      <c r="O186" s="32" t="s">
+      <c r="N186" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="O186" s="4" t="s">
         <v>326</v>
       </c>
-      <c r="P186" s="32" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="187" spans="1:16" s="32" customFormat="1">
-      <c r="A187" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D187" s="32">
+      <c r="P186" s="4" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="187" spans="1:16" s="4" customFormat="1">
+      <c r="A187" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D187" s="4">
         <v>1</v>
       </c>
-      <c r="E187" s="32" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="188" spans="1:16" s="32" customFormat="1">
-      <c r="A188" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D188" s="32">
+      <c r="E187" s="4" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="188" spans="1:16" s="4" customFormat="1">
+      <c r="A188" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D188" s="4">
         <v>1.5</v>
       </c>
-      <c r="E188" s="32" t="s">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="189" spans="1:16" s="32" customFormat="1">
-      <c r="A189" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D189" s="32">
+      <c r="E188" s="4" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="189" spans="1:16" s="4" customFormat="1">
+      <c r="A189" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D189" s="4">
         <v>2</v>
       </c>
-      <c r="E189" s="32" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="190" spans="1:16" s="32" customFormat="1">
-      <c r="A190" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D190" s="32">
+      <c r="E189" s="4" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="190" spans="1:16" s="4" customFormat="1">
+      <c r="A190" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D190" s="4">
         <v>3</v>
       </c>
-      <c r="E190" s="32" t="s">
+      <c r="E190" s="4" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="191" spans="1:16" s="32" customFormat="1">
-      <c r="A191" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D191" s="32">
+    <row r="191" spans="1:16" s="4" customFormat="1">
+      <c r="A191" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D191" s="4">
         <v>4</v>
       </c>
-      <c r="E191" s="32" t="s">
+      <c r="E191" s="4" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="192" spans="1:16" s="32" customFormat="1">
-      <c r="A192" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D192" s="32" t="s">
+    <row r="192" spans="1:16" s="4" customFormat="1">
+      <c r="A192" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D192" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="E192" s="32" t="s">
+      <c r="E192" s="4" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="193" spans="1:12" s="32" customFormat="1">
-      <c r="A193" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="B193" s="32" t="s">
-        <v>589</v>
-      </c>
-      <c r="C193" s="32" t="s">
+    <row r="193" spans="1:12" s="4" customFormat="1">
+      <c r="A193" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B193" s="4" t="s">
+        <v>582</v>
+      </c>
+      <c r="C193" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="D193" s="32">
+      <c r="D193" s="4">
         <v>0</v>
       </c>
-      <c r="E193" s="32" t="s">
-        <v>389</v>
-      </c>
-      <c r="F193" s="32" t="s">
-        <v>595</v>
-      </c>
-      <c r="G193" s="32" t="s">
+      <c r="E193" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="F193" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="G193" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="H193" s="32" t="s">
+      <c r="H193" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="I193" s="32" t="s">
+      <c r="I193" s="4" t="s">
         <v>382</v>
       </c>
-      <c r="J193" s="32" t="s">
-        <v>307</v>
-      </c>
-      <c r="K193" s="32" t="s">
+      <c r="J193" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="K193" s="4" t="s">
         <v>383</v>
       </c>
-      <c r="L193" s="32" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="194" spans="1:12" s="32" customFormat="1">
-      <c r="A194" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D194" s="32">
+      <c r="L193" s="4" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="194" spans="1:12" s="4" customFormat="1">
+      <c r="A194" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D194" s="4">
         <v>1</v>
       </c>
-      <c r="E194" s="32" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="195" spans="1:12" s="32" customFormat="1">
-      <c r="A195" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D195" s="32">
+      <c r="E194" s="4" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="195" spans="1:12" s="4" customFormat="1">
+      <c r="A195" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D195" s="4">
         <v>1.5</v>
       </c>
-      <c r="E195" s="32" t="s">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="196" spans="1:12" s="32" customFormat="1">
-      <c r="A196" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D196" s="32">
+      <c r="E195" s="4" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="196" spans="1:12" s="4" customFormat="1">
+      <c r="A196" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D196" s="4">
         <v>2</v>
       </c>
-      <c r="E196" s="32" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="197" spans="1:12" s="32" customFormat="1">
-      <c r="A197" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D197" s="32">
+      <c r="E196" s="4" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="197" spans="1:12" s="4" customFormat="1">
+      <c r="A197" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D197" s="4">
         <v>3</v>
       </c>
-      <c r="E197" s="32" t="s">
+      <c r="E197" s="4" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="198" spans="1:12" s="32" customFormat="1">
-      <c r="A198" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D198" s="32">
+    <row r="198" spans="1:12" s="4" customFormat="1">
+      <c r="A198" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D198" s="4">
         <v>4</v>
       </c>
-      <c r="E198" s="32" t="s">
+      <c r="E198" s="4" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="199" spans="1:12" s="32" customFormat="1">
-      <c r="A199" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D199" s="32" t="s">
+    <row r="199" spans="1:12" s="4" customFormat="1">
+      <c r="A199" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D199" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="E199" s="32" t="s">
+      <c r="E199" s="4" t="s">
         <v>231</v>
       </c>
     </row>
@@ -7601,39 +7590,35 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9521944E-28B4-4113-A27F-3B841E118807}">
-  <dimension ref="A1:AU56"/>
+  <dimension ref="A1:AP52"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.36328125" customWidth="1"/>
     <col min="4" max="6" width="8.6328125" customWidth="1"/>
     <col min="15" max="15" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.6328125" style="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.54296875" customWidth="1"/>
-    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="8.36328125" customWidth="1"/>
-    <col min="29" max="29" width="11.08984375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="9.26953125" customWidth="1"/>
-    <col min="35" max="35" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="38" max="40" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="8.6328125" customWidth="1"/>
-    <col min="42" max="42" width="9.26953125" customWidth="1"/>
-    <col min="43" max="43" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="18" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="8.7265625" style="11"/>
+    <col min="22" max="22" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.54296875" customWidth="1"/>
+    <col min="24" max="24" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.36328125" customWidth="1"/>
+    <col min="28" max="28" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="9.26953125" customWidth="1"/>
+    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="8.6328125" customWidth="1"/>
+    <col min="37" max="37" width="9.26953125" customWidth="1"/>
+    <col min="38" max="38" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="18" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="8.7265625" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" s="2" customFormat="1" ht="30" customHeight="1">
-      <c r="A1" s="18" t="s">
-        <v>391</v>
+    <row r="1" spans="1:42" s="2" customFormat="1" ht="30" customHeight="1">
+      <c r="A1" s="17" t="s">
+        <v>390</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>5</v>
@@ -7669,7 +7654,7 @@
         <v>15</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="N1" s="2" t="s">
         <v>60</v>
@@ -7677,575 +7662,476 @@
       <c r="O1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="P1" s="3" t="s">
-        <v>62</v>
+      <c r="P1" s="2" t="s">
+        <v>63</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>66</v>
+        <v>496</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>502</v>
+        <v>489</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>495</v>
+        <v>69</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>69</v>
+        <v>575</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>582</v>
+        <v>71</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Z1" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AA1" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AB1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AC1" s="17" t="s">
+      <c r="AB1" s="16" t="s">
         <v>77</v>
       </c>
+      <c r="AC1" s="2" t="s">
+        <v>78</v>
+      </c>
       <c r="AD1" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AE1" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AF1" s="2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="AG1" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AH1" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AI1" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="AJ1" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="AK1" s="2" t="s">
-        <v>382</v>
+        <v>91</v>
       </c>
       <c r="AL1" s="2" t="s">
-        <v>383</v>
+        <v>92</v>
       </c>
       <c r="AM1" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AN1" s="2" t="s">
-        <v>589</v>
+        <v>93</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>379</v>
       </c>
       <c r="AO1" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="AP1" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AQ1" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="AR1" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="AS1" t="s">
-        <v>379</v>
-      </c>
-      <c r="AT1" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="AU1" s="19" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="2" spans="1:47">
+      <c r="AP1" s="18" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="2" spans="1:42">
       <c r="A2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:47">
+    <row r="3" spans="1:42">
       <c r="A3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:47">
+    <row r="4" spans="1:42">
       <c r="A4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:47">
+    <row r="5" spans="1:42">
       <c r="A5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:47">
+    <row r="6" spans="1:42">
       <c r="A6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:47">
+    <row r="7" spans="1:42">
       <c r="A7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:47">
+    <row r="8" spans="1:42">
       <c r="A8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:47">
+    <row r="9" spans="1:42">
       <c r="A9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:47">
+    <row r="10" spans="1:42">
       <c r="A10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:47">
+    <row r="11" spans="1:42">
       <c r="A11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:47">
+    <row r="12" spans="1:42">
       <c r="A12" t="s">
         <v>15</v>
       </c>
-      <c r="U12" s="16"/>
-      <c r="AG12" s="16"/>
-      <c r="AT12" s="16"/>
-      <c r="AU12" s="11" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="13" spans="1:47">
+      <c r="T12" s="22"/>
+      <c r="AO12" s="15"/>
+      <c r="AP12" s="10" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="13" spans="1:42">
       <c r="A13" t="s">
-        <v>385</v>
-      </c>
-      <c r="L13" s="23"/>
-      <c r="AT13" s="16"/>
-    </row>
-    <row r="14" spans="1:47">
+        <v>384</v>
+      </c>
+      <c r="L13" s="22"/>
+      <c r="AO13" s="15"/>
+    </row>
+    <row r="14" spans="1:42">
       <c r="A14" t="s">
         <v>60</v>
       </c>
-      <c r="R14" s="23"/>
-      <c r="AC14" s="23" t="s">
-        <v>394</v>
-      </c>
-      <c r="AF14" s="16"/>
-      <c r="AG14" s="16"/>
-      <c r="AT14" s="16"/>
-    </row>
-    <row r="15" spans="1:47">
+      <c r="Q14" s="22"/>
+      <c r="AB14" s="22" t="s">
+        <v>393</v>
+      </c>
+      <c r="AE14" s="15"/>
+      <c r="AO14" s="15"/>
+    </row>
+    <row r="15" spans="1:42">
       <c r="A15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:47">
+    <row r="16" spans="1:42">
       <c r="A16" t="s">
         <v>62</v>
       </c>
-      <c r="AS16" s="16"/>
-    </row>
-    <row r="17" spans="1:46">
+      <c r="AN16" s="15"/>
+    </row>
+    <row r="17" spans="1:41">
       <c r="A17" t="s">
         <v>63</v>
       </c>
-      <c r="AC17" s="16"/>
-      <c r="AS17" s="16"/>
-    </row>
-    <row r="18" spans="1:46">
+      <c r="AB17" s="15"/>
+      <c r="AN17" s="15"/>
+    </row>
+    <row r="18" spans="1:41">
       <c r="A18" t="s">
         <v>64</v>
       </c>
-      <c r="Q18" s="23"/>
-      <c r="AS18" s="16"/>
-    </row>
-    <row r="19" spans="1:46">
+      <c r="P18" s="22"/>
+      <c r="AN18" s="15"/>
+    </row>
+    <row r="19" spans="1:41">
       <c r="A19" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:46">
+    <row r="20" spans="1:41">
       <c r="A20" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:46">
+    <row r="21" spans="1:41">
       <c r="A21" t="s">
-        <v>502</v>
-      </c>
-      <c r="L21" s="23"/>
-      <c r="AS21" s="16"/>
-    </row>
-    <row r="22" spans="1:46">
+        <v>496</v>
+      </c>
+      <c r="L21" s="22"/>
+      <c r="AN21" s="15"/>
+    </row>
+    <row r="22" spans="1:41">
       <c r="A22" t="s">
-        <v>495</v>
-      </c>
-      <c r="L22" s="23"/>
-      <c r="M22" s="23"/>
-      <c r="Q22" s="23"/>
-      <c r="AS22" s="16"/>
-    </row>
-    <row r="23" spans="1:46">
+        <v>489</v>
+      </c>
+      <c r="L22" s="22"/>
+      <c r="M22" s="22"/>
+      <c r="P22" s="22"/>
+      <c r="AN22" s="15"/>
+    </row>
+    <row r="23" spans="1:41">
       <c r="A23" t="s">
         <v>69</v>
       </c>
-      <c r="L23" s="23"/>
-      <c r="M23" s="33"/>
-      <c r="Q23" s="23"/>
-      <c r="AS23" s="16"/>
-    </row>
-    <row r="24" spans="1:46">
+      <c r="L23" s="22"/>
+      <c r="P23" s="22"/>
+      <c r="AN23" s="15"/>
+    </row>
+    <row r="24" spans="1:41">
       <c r="A24" t="s">
-        <v>582</v>
-      </c>
-      <c r="L24" s="33"/>
-      <c r="M24" s="16"/>
-      <c r="Q24" s="16"/>
-      <c r="R24" s="16"/>
-      <c r="AC24" s="16"/>
-      <c r="AS24" s="16"/>
-    </row>
-    <row r="25" spans="1:46">
+        <v>575</v>
+      </c>
+      <c r="M24" s="15"/>
+      <c r="P24" s="15"/>
+      <c r="Q24" s="22"/>
+      <c r="AB24" s="15"/>
+      <c r="AN24" s="15"/>
+    </row>
+    <row r="25" spans="1:41">
       <c r="A25" t="s">
         <v>71</v>
       </c>
-      <c r="N25" s="23" t="s">
-        <v>418</v>
-      </c>
-      <c r="Q25" s="23" t="s">
-        <v>417</v>
+      <c r="N25" s="22" t="s">
+        <v>416</v>
+      </c>
+      <c r="P25" s="22" t="s">
+        <v>415</v>
+      </c>
+      <c r="AB25" s="14" t="s">
+        <v>414</v>
       </c>
       <c r="AC25" s="15" t="s">
-        <v>415</v>
-      </c>
-      <c r="AD25" s="16" t="s">
-        <v>432</v>
-      </c>
-      <c r="AG25" s="16" t="s">
-        <v>416</v>
-      </c>
-      <c r="AS25" s="16"/>
-    </row>
-    <row r="26" spans="1:46">
+        <v>428</v>
+      </c>
+      <c r="AN25" s="15"/>
+    </row>
+    <row r="26" spans="1:41">
       <c r="A26" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="27" spans="1:46">
+    <row r="27" spans="1:41">
       <c r="A27" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:46">
+    <row r="28" spans="1:41">
       <c r="A28" t="s">
         <v>75</v>
       </c>
-      <c r="AD28" s="16"/>
-      <c r="AS28" s="16"/>
-    </row>
-    <row r="29" spans="1:46">
+      <c r="AC28" s="15"/>
+      <c r="AN28" s="15"/>
+    </row>
+    <row r="29" spans="1:41">
       <c r="A29" t="s">
         <v>77</v>
       </c>
-      <c r="P29" s="15"/>
-      <c r="R29" s="23" t="s">
-        <v>423</v>
-      </c>
-      <c r="V29" s="16"/>
-      <c r="W29" s="16" t="s">
-        <v>419</v>
-      </c>
-      <c r="X29" s="16"/>
-      <c r="AS29" s="16"/>
-      <c r="AT29" s="16"/>
-    </row>
-    <row r="30" spans="1:46">
+      <c r="Q29" s="22" t="s">
+        <v>420</v>
+      </c>
+      <c r="U29" s="15"/>
+      <c r="V29" s="15" t="s">
+        <v>417</v>
+      </c>
+      <c r="W29" s="15"/>
+      <c r="AN29" s="15"/>
+      <c r="AO29" s="15"/>
+    </row>
+    <row r="30" spans="1:41">
       <c r="A30" t="s">
         <v>78</v>
       </c>
-      <c r="P30" s="4" t="s">
-        <v>429</v>
-      </c>
-      <c r="Y30" s="16"/>
-      <c r="AO30" s="16" t="s">
-        <v>430</v>
-      </c>
-      <c r="AP30" s="16"/>
-      <c r="AQ30" s="16" t="s">
-        <v>431</v>
-      </c>
-      <c r="AT30" s="16"/>
-    </row>
-    <row r="31" spans="1:46">
+      <c r="X30" s="15"/>
+      <c r="AJ30" s="15" t="s">
+        <v>426</v>
+      </c>
+      <c r="AK30" s="15"/>
+      <c r="AL30" s="15" t="s">
+        <v>427</v>
+      </c>
+      <c r="AO30" s="15"/>
+    </row>
+    <row r="31" spans="1:41">
       <c r="A31" t="s">
         <v>79</v>
       </c>
-      <c r="R31" s="16"/>
-      <c r="AC31" s="23"/>
-    </row>
-    <row r="32" spans="1:46">
+      <c r="Q31" s="22"/>
+      <c r="AB31" s="22"/>
+    </row>
+    <row r="32" spans="1:41">
       <c r="A32" t="s">
         <v>80</v>
       </c>
-      <c r="R32" s="16"/>
-      <c r="AC32" s="24" t="s">
-        <v>475</v>
-      </c>
-      <c r="AG32" s="16" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="33" spans="1:46">
+      <c r="Q32" s="22"/>
+      <c r="AB32" s="23" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="33" spans="1:41">
       <c r="A33" t="s">
-        <v>84</v>
-      </c>
-      <c r="R33" s="16" t="s">
-        <v>434</v>
-      </c>
-      <c r="AC33" s="23" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="34" spans="1:46">
+        <v>85</v>
+      </c>
+      <c r="AJ33" s="15" t="s">
+        <v>422</v>
+      </c>
+      <c r="AK33" s="15" t="s">
+        <v>423</v>
+      </c>
+      <c r="AL33" s="15" t="s">
+        <v>424</v>
+      </c>
+      <c r="AM33" s="15" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="34" spans="1:41">
       <c r="A34" t="s">
-        <v>85</v>
-      </c>
-      <c r="AO34" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="U34" s="15"/>
+      <c r="V34" s="15"/>
+      <c r="W34" s="15"/>
+      <c r="AB34" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="AD34" s="15"/>
+      <c r="AI34" s="15"/>
+      <c r="AO34" s="15"/>
+    </row>
+    <row r="35" spans="1:41">
+      <c r="A35" t="s">
+        <v>87</v>
+      </c>
+      <c r="U35" s="15"/>
+      <c r="V35" s="15"/>
+      <c r="W35" s="15"/>
+      <c r="AB35" s="22" t="s">
+        <v>430</v>
+      </c>
+      <c r="AE35" s="15"/>
+      <c r="AI35" s="15"/>
+      <c r="AO35" s="15"/>
+    </row>
+    <row r="36" spans="1:41" ht="14" customHeight="1">
+      <c r="A36" t="s">
+        <v>89</v>
+      </c>
+      <c r="P36" s="22" t="s">
+        <v>418</v>
+      </c>
+      <c r="U36" s="15"/>
+      <c r="V36" s="15" t="s">
+        <v>419</v>
+      </c>
+      <c r="W36" s="15"/>
+      <c r="AB36" s="22" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="37" spans="1:41">
+      <c r="A37" t="s">
+        <v>90</v>
+      </c>
+      <c r="AO37" s="15"/>
+    </row>
+    <row r="38" spans="1:41">
+      <c r="A38" t="s">
+        <v>91</v>
+      </c>
+      <c r="AO38" s="15"/>
+    </row>
+    <row r="39" spans="1:41">
+      <c r="A39" t="s">
+        <v>92</v>
+      </c>
+      <c r="AO39" s="15"/>
+    </row>
+    <row r="40" spans="1:41">
+      <c r="A40" t="s">
+        <v>93</v>
+      </c>
+      <c r="AJ40" s="15" t="s">
         <v>425</v>
       </c>
-      <c r="AP34" s="16" t="s">
-        <v>426</v>
-      </c>
-      <c r="AQ34" s="16" t="s">
-        <v>427</v>
-      </c>
-      <c r="AR34" s="16" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="35" spans="1:46">
-      <c r="A35" t="s">
-        <v>86</v>
-      </c>
-      <c r="V35" s="16"/>
-      <c r="W35" s="16"/>
-      <c r="X35" s="16"/>
-      <c r="AC35" s="23" t="s">
-        <v>437</v>
-      </c>
-      <c r="AE35" s="16"/>
-      <c r="AM35" s="16"/>
-      <c r="AN35" s="16"/>
-      <c r="AT35" s="16"/>
-    </row>
-    <row r="36" spans="1:46">
-      <c r="A36" t="s">
-        <v>87</v>
-      </c>
-      <c r="V36" s="16"/>
-      <c r="W36" s="16"/>
-      <c r="X36" s="16"/>
-      <c r="AC36" s="23" t="s">
-        <v>436</v>
-      </c>
-      <c r="AF36" s="16"/>
-      <c r="AG36" s="16"/>
-      <c r="AM36" s="16"/>
-      <c r="AN36" s="16"/>
-      <c r="AT36" s="16"/>
-    </row>
-    <row r="37" spans="1:46">
-      <c r="A37" t="s">
-        <v>382</v>
-      </c>
-      <c r="V37" s="16"/>
-      <c r="W37" s="16"/>
-      <c r="X37" s="16"/>
-      <c r="AC37" s="16" t="s">
-        <v>437</v>
-      </c>
-      <c r="AE37" s="16"/>
-      <c r="AM37" s="16"/>
-      <c r="AN37" s="16"/>
-      <c r="AT37" s="16"/>
-    </row>
-    <row r="38" spans="1:46">
-      <c r="A38" t="s">
-        <v>383</v>
-      </c>
-      <c r="V38" s="16"/>
-      <c r="W38" s="16"/>
-      <c r="X38" s="16"/>
-      <c r="AC38" s="16" t="s">
-        <v>436</v>
-      </c>
-      <c r="AF38" s="16"/>
-      <c r="AG38" s="16"/>
-      <c r="AM38" s="16"/>
-      <c r="AN38" s="16"/>
-      <c r="AT38" s="16"/>
-    </row>
-    <row r="39" spans="1:46" ht="14" customHeight="1">
-      <c r="A39" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q39" s="23" t="s">
-        <v>421</v>
-      </c>
-      <c r="V39" s="16"/>
-      <c r="W39" s="16" t="s">
-        <v>422</v>
-      </c>
-      <c r="X39" s="16"/>
-      <c r="AC39" s="23" t="s">
-        <v>438</v>
-      </c>
-      <c r="AG39" s="16" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="40" spans="1:46" ht="14" customHeight="1">
-      <c r="A40" t="s">
-        <v>589</v>
-      </c>
-      <c r="Q40" s="16"/>
-      <c r="V40" s="16"/>
-      <c r="W40" s="16"/>
-      <c r="X40" s="16"/>
-      <c r="AC40" s="16"/>
-      <c r="AG40" s="16"/>
-    </row>
-    <row r="41" spans="1:46">
+      <c r="AO40" s="15"/>
+    </row>
+    <row r="41" spans="1:41">
       <c r="A41" t="s">
-        <v>90</v>
-      </c>
-      <c r="AT41" s="16"/>
-    </row>
-    <row r="42" spans="1:46">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="42" spans="1:41">
       <c r="A42" t="s">
-        <v>91</v>
-      </c>
-      <c r="AT42" s="16"/>
-    </row>
-    <row r="43" spans="1:46">
-      <c r="A43" t="s">
-        <v>92</v>
-      </c>
-      <c r="AT43" s="16"/>
-    </row>
-    <row r="44" spans="1:46">
-      <c r="A44" t="s">
-        <v>93</v>
-      </c>
-      <c r="AO44" s="16" t="s">
-        <v>428</v>
-      </c>
-      <c r="AT44" s="16"/>
-    </row>
-    <row r="45" spans="1:46">
-      <c r="A45" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="46" spans="1:46">
-      <c r="A46" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="48" spans="1:46" s="11" customFormat="1">
-      <c r="A48" s="11" t="s">
-        <v>455</v>
-      </c>
-      <c r="P48" s="4"/>
-    </row>
-    <row r="50" spans="1:3">
-      <c r="B50" s="12" t="s">
+    <row r="44" spans="1:41" s="10" customFormat="1">
+      <c r="A44" s="10" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="46" spans="1:41">
+      <c r="B46" s="11" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
-      <c r="A51" s="12"/>
-      <c r="B51" s="13"/>
+    <row r="47" spans="1:41">
+      <c r="A47" s="11"/>
+      <c r="B47" s="12"/>
+      <c r="C47" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="48" spans="1:41">
+      <c r="B48" s="13"/>
+      <c r="C48" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3">
+      <c r="B49" s="14"/>
+      <c r="C49" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3">
+      <c r="B50" s="15"/>
+      <c r="C50" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3">
+      <c r="B51" s="1" t="s">
+        <v>380</v>
+      </c>
       <c r="C51" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="B52" s="14"/>
+        <v>381</v>
+      </c>
+    </row>
+    <row r="52" spans="2:3">
+      <c r="B52" s="22"/>
       <c r="C52" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="B53" s="15"/>
-      <c r="C53" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3">
-      <c r="B54" s="16"/>
-      <c r="C54" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="B55" s="1" t="s">
-        <v>380</v>
-      </c>
-      <c r="C55" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3">
-      <c r="B56" s="23"/>
-      <c r="C56" t="s">
-        <v>476</v>
+        <v>470</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:AJ22 B23:P24 B34:AQ34 AC39:AC40 AN2:AT24 AK2:AM33 AN25:AR25 AT25 AN26:AT28 Y29:AJ29 AN29:AR29 B29:X30 Z30:AJ30 AN30:AT33 B31:AB33 AD31:AJ33 AR34:AT35 AN35:AP35 B35:AB41 AD35:AJ41 AK35:AM47 AN36:AT36 AN37:AP37 AR37:AT37 AN38:AT47 B42:AJ47 B25:AJ28 R23:AJ24">
-    <cfRule type="expression" dxfId="4" priority="3">
+  <conditionalFormatting sqref="P2:AH22 B2:O24 AJ2:AO24 AI2:AI32 P23 Q23:AH24 AJ25:AM25 AO25 B25:AH28 AJ26:AO28 X29:AH29 AJ29:AM29 B29:W30 Y30:AH30 AJ30:AO32 B31:AA32 AC31:AH32 B33:AL33 AM33:AO34 AJ34:AK34 B34:AA37 AC34:AH37 AI34:AI43 AJ35:AO43 AB36 B38:AH43 B50">
+    <cfRule type="expression" dxfId="2" priority="60">
       <formula>$A2=B$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y30">
-    <cfRule type="expression" dxfId="3" priority="7">
+  <conditionalFormatting sqref="X30">
+    <cfRule type="expression" dxfId="1" priority="7">
       <formula>$A30=#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B54">
-    <cfRule type="expression" dxfId="2" priority="60">
-      <formula>$A54=B$1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AS25 AS29:AT29">
-    <cfRule type="expression" dxfId="1" priority="9">
-      <formula>#REF!=AS$1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q23">
-    <cfRule type="expression" dxfId="0" priority="86">
-      <formula>$A23=Q$1</formula>
+  <conditionalFormatting sqref="AN25 AN29:AO29">
+    <cfRule type="expression" dxfId="0" priority="9">
+      <formula>#REF!=AN$1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8255,11 +8141,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313888EE-552D-40AA-8234-3B847E46EF43}">
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="55.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.36328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.36328125" style="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.36328125" customWidth="1"/>
     <col min="4" max="4" width="38" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="38" style="2" customWidth="1"/>
@@ -8271,45 +8157,45 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
-        <v>464</v>
-      </c>
-      <c r="B1" s="25" t="s">
-        <v>456</v>
+        <v>458</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>450</v>
       </c>
       <c r="C1" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
       <c r="D1" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="F1" t="s">
-        <v>481</v>
+        <v>475</v>
       </c>
       <c r="G1" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
       <c r="H1" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="29">
       <c r="A2" t="s">
-        <v>488</v>
-      </c>
-      <c r="B2" s="28" t="s">
-        <v>520</v>
+        <v>482</v>
+      </c>
+      <c r="B2" s="27" t="s">
+        <v>513</v>
       </c>
       <c r="C2" t="s">
         <v>169</v>
       </c>
       <c r="D2" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>490</v>
+        <v>484</v>
       </c>
       <c r="F2" t="s">
         <v>169</v>
@@ -8323,25 +8209,25 @@
     </row>
     <row r="3" spans="1:10" ht="58">
       <c r="A3" t="s">
-        <v>465</v>
-      </c>
-      <c r="B3" s="28" t="s">
-        <v>520</v>
+        <v>459</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>513</v>
       </c>
       <c r="C3" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D3" t="s">
-        <v>459</v>
+        <v>453</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="F3" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
       <c r="G3" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="H3" t="s">
         <v>77</v>
@@ -8354,69 +8240,78 @@
       </c>
     </row>
     <row r="4" spans="1:10" ht="43.5">
-      <c r="B4" s="27" t="s">
-        <v>519</v>
+      <c r="A4" s="22" t="s">
+        <v>616</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>512</v>
       </c>
       <c r="C4" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="D4" t="s">
-        <v>460</v>
+        <v>618</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
       <c r="F4" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="G4" t="s">
-        <v>528</v>
+        <v>521</v>
       </c>
       <c r="H4" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="43.5">
-      <c r="B5" s="27" t="s">
-        <v>519</v>
+      <c r="A5" s="22" t="s">
+        <v>616</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>512</v>
       </c>
       <c r="C5" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="D5" t="s">
-        <v>460</v>
+        <v>618</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="F5" t="s">
         <v>462</v>
       </c>
-      <c r="F5" t="s">
-        <v>468</v>
-      </c>
       <c r="G5" t="s">
-        <v>527</v>
+        <v>520</v>
       </c>
       <c r="H5" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="29">
-      <c r="B6" s="27" t="s">
-        <v>519</v>
+      <c r="A6" s="22" t="s">
+        <v>616</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>512</v>
       </c>
       <c r="C6" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="D6" t="s">
-        <v>600</v>
+        <v>593</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>601</v>
+        <v>594</v>
       </c>
       <c r="F6" t="s">
-        <v>602</v>
+        <v>595</v>
       </c>
       <c r="G6" t="s">
-        <v>604</v>
+        <v>597</v>
       </c>
       <c r="H6" t="s">
         <v>383</v>
@@ -8426,14 +8321,17 @@
       </c>
     </row>
     <row r="7" spans="1:10">
-      <c r="B7" s="27" t="s">
-        <v>519</v>
+      <c r="A7" s="22" t="s">
+        <v>616</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>512</v>
       </c>
       <c r="D7" t="s">
-        <v>599</v>
+        <v>592</v>
       </c>
       <c r="F7" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
       <c r="G7" t="s">
         <v>382</v>
@@ -8446,9 +8344,12 @@
       </c>
     </row>
     <row r="8" spans="1:10">
-      <c r="B8" s="27"/>
+      <c r="A8" s="22" t="s">
+        <v>616</v>
+      </c>
+      <c r="B8" s="26"/>
       <c r="D8" t="s">
-        <v>603</v>
+        <v>596</v>
       </c>
       <c r="G8" t="s">
         <v>86</v>
@@ -8461,63 +8362,63 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.5">
-      <c r="B9" s="29" t="s">
-        <v>587</v>
+      <c r="B9" s="30" t="s">
+        <v>580</v>
       </c>
       <c r="C9" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D9" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>524</v>
+        <v>517</v>
       </c>
       <c r="F9" t="s">
-        <v>525</v>
+        <v>518</v>
       </c>
       <c r="G9" t="s">
-        <v>526</v>
+        <v>519</v>
       </c>
       <c r="H9" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.5">
-      <c r="B10" s="29" t="s">
-        <v>588</v>
+      <c r="B10" s="30" t="s">
+        <v>581</v>
       </c>
       <c r="C10" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="D10" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>521</v>
+        <v>514</v>
       </c>
       <c r="F10" t="s">
-        <v>522</v>
+        <v>515</v>
       </c>
       <c r="G10" t="s">
-        <v>523</v>
+        <v>516</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="43.5">
-      <c r="B11" s="26" t="s">
-        <v>518</v>
+      <c r="B11" s="25" t="s">
+        <v>511</v>
       </c>
       <c r="C11" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="D11" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
       <c r="F11" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="G11" t="s">
         <v>89</v>
@@ -8527,20 +8428,20 @@
       </c>
     </row>
     <row r="12" spans="1:10" ht="29">
-      <c r="B12" s="28" t="s">
-        <v>520</v>
+      <c r="B12" s="26" t="s">
+        <v>513</v>
       </c>
       <c r="C12" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="D12" t="s">
+        <v>467</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>473</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>479</v>
-      </c>
       <c r="F12" t="s">
-        <v>480</v>
+        <v>474</v>
       </c>
       <c r="G12" t="s">
         <v>84</v>
@@ -8551,22 +8452,22 @@
     </row>
     <row r="13" spans="1:10" ht="43.5">
       <c r="A13" s="2" t="s">
-        <v>531</v>
-      </c>
-      <c r="B13" s="31" t="s">
-        <v>518</v>
+        <v>524</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>511</v>
       </c>
       <c r="C13" t="s">
+        <v>465</v>
+      </c>
+      <c r="D13" t="s">
         <v>471</v>
       </c>
-      <c r="D13" t="s">
-        <v>477</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="F13" t="s">
-        <v>598</v>
+        <v>591</v>
       </c>
       <c r="G13" t="s">
         <v>80</v>
@@ -8579,17 +8480,17 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="43.5">
-      <c r="B14" s="28" t="s">
-        <v>520</v>
+      <c r="B14" s="27" t="s">
+        <v>513</v>
       </c>
       <c r="C14" t="s">
         <v>169</v>
       </c>
       <c r="D14" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
       <c r="F14" t="s">
         <v>169</v>
@@ -8606,77 +8507,80 @@
     </row>
     <row r="15" spans="1:10" ht="58">
       <c r="A15" t="s">
-        <v>493</v>
-      </c>
-      <c r="B15" s="30" t="s">
-        <v>586</v>
+        <v>487</v>
+      </c>
+      <c r="B15" s="28" t="s">
+        <v>579</v>
       </c>
       <c r="C15" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D15" t="s">
-        <v>494</v>
+        <v>488</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
       <c r="F15" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="G15" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H15" t="s">
         <v>15</v>
       </c>
       <c r="I15" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="29">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="43.5">
       <c r="A16" t="s">
-        <v>536</v>
-      </c>
-      <c r="B16" s="31" t="s">
-        <v>518</v>
+        <v>529</v>
+      </c>
+      <c r="B16" s="29" t="s">
+        <v>511</v>
       </c>
       <c r="C16" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D16" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>516</v>
+        <v>612</v>
       </c>
       <c r="F16" t="s">
-        <v>515</v>
+        <v>509</v>
       </c>
       <c r="G16" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="H16" t="s">
         <v>15</v>
       </c>
       <c r="I16" t="s">
-        <v>502</v>
+        <v>496</v>
       </c>
     </row>
     <row r="17" spans="1:10">
-      <c r="B17" s="31" t="s">
-        <v>518</v>
+      <c r="B17" s="29" t="s">
+        <v>511</v>
       </c>
       <c r="C17" t="s">
-        <v>472</v>
+        <v>466</v>
+      </c>
+      <c r="D17" t="s">
+        <v>630</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>529</v>
+        <v>522</v>
       </c>
       <c r="F17" t="s">
-        <v>530</v>
+        <v>523</v>
       </c>
       <c r="G17" t="s">
-        <v>502</v>
+        <v>496</v>
       </c>
       <c r="H17" t="s">
         <v>15</v>
@@ -8684,22 +8588,22 @@
     </row>
     <row r="18" spans="1:10" ht="58">
       <c r="A18" t="s">
-        <v>534</v>
-      </c>
-      <c r="B18" s="30" t="s">
-        <v>586</v>
+        <v>527</v>
+      </c>
+      <c r="B18" s="28" t="s">
+        <v>579</v>
       </c>
       <c r="C18" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D18" t="s">
-        <v>535</v>
+        <v>528</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>532</v>
+        <v>525</v>
       </c>
       <c r="F18" t="s">
-        <v>533</v>
+        <v>526</v>
       </c>
       <c r="G18" t="s">
         <v>71</v>
@@ -8710,25 +8614,25 @@
     </row>
     <row r="19" spans="1:10" ht="43.5">
       <c r="A19" t="s">
-        <v>541</v>
-      </c>
-      <c r="B19" s="30" t="s">
-        <v>586</v>
+        <v>534</v>
+      </c>
+      <c r="B19" s="28" t="s">
+        <v>579</v>
       </c>
       <c r="C19" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="D19" t="s">
-        <v>537</v>
+        <v>530</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>540</v>
+        <v>533</v>
       </c>
       <c r="F19" t="s">
-        <v>538</v>
+        <v>531</v>
       </c>
       <c r="G19" t="s">
-        <v>539</v>
+        <v>532</v>
       </c>
       <c r="H19" t="s">
         <v>64</v>
@@ -8736,25 +8640,25 @@
     </row>
     <row r="20" spans="1:10" ht="29">
       <c r="A20" t="s">
-        <v>545</v>
-      </c>
-      <c r="B20" s="31" t="s">
-        <v>518</v>
+        <v>538</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>511</v>
       </c>
       <c r="C20" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="D20" t="s">
-        <v>542</v>
+        <v>535</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>543</v>
+        <v>536</v>
       </c>
       <c r="F20" t="s">
-        <v>544</v>
+        <v>537</v>
       </c>
       <c r="G20" t="s">
-        <v>539</v>
+        <v>532</v>
       </c>
       <c r="H20" t="s">
         <v>77</v>
@@ -8762,25 +8666,25 @@
     </row>
     <row r="21" spans="1:10" ht="43.5">
       <c r="A21" t="s">
-        <v>548</v>
-      </c>
-      <c r="B21" s="30" t="s">
-        <v>586</v>
+        <v>541</v>
+      </c>
+      <c r="B21" s="28" t="s">
+        <v>579</v>
       </c>
       <c r="C21" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D21" t="s">
-        <v>546</v>
+        <v>539</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>547</v>
+        <v>540</v>
       </c>
       <c r="F21" t="s">
-        <v>549</v>
+        <v>542</v>
       </c>
       <c r="G21" t="s">
-        <v>539</v>
+        <v>532</v>
       </c>
       <c r="H21" t="s">
         <v>78</v>
@@ -8788,25 +8692,25 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" t="s">
-        <v>552</v>
-      </c>
-      <c r="B22" s="30" t="s">
-        <v>573</v>
+        <v>545</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>566</v>
       </c>
       <c r="C22" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D22" t="s">
-        <v>553</v>
+        <v>546</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>551</v>
+        <v>544</v>
       </c>
       <c r="F22" t="s">
-        <v>550</v>
+        <v>543</v>
       </c>
       <c r="G22" t="s">
-        <v>539</v>
+        <v>532</v>
       </c>
       <c r="H22" t="s">
         <v>64</v>
@@ -8820,28 +8724,28 @@
     </row>
     <row r="23" spans="1:10" ht="72.5">
       <c r="A23" t="s">
-        <v>559</v>
-      </c>
-      <c r="B23" s="30" t="s">
-        <v>586</v>
+        <v>552</v>
+      </c>
+      <c r="B23" s="28" t="s">
+        <v>579</v>
       </c>
       <c r="C23" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D23" t="s">
-        <v>561</v>
+        <v>554</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>560</v>
+        <v>553</v>
       </c>
       <c r="F23" t="s">
-        <v>558</v>
+        <v>551</v>
       </c>
       <c r="G23" t="s">
         <v>63</v>
       </c>
       <c r="H23" t="s">
-        <v>557</v>
+        <v>550</v>
       </c>
       <c r="I23" t="s">
         <v>89</v>
@@ -8849,22 +8753,22 @@
     </row>
     <row r="24" spans="1:10" ht="87">
       <c r="A24" t="s">
-        <v>562</v>
-      </c>
-      <c r="B24" s="30" t="s">
-        <v>586</v>
+        <v>555</v>
+      </c>
+      <c r="B24" s="28" t="s">
+        <v>579</v>
       </c>
       <c r="C24" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D24" t="s">
-        <v>563</v>
+        <v>556</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>565</v>
+        <v>558</v>
       </c>
       <c r="F24" t="s">
-        <v>564</v>
+        <v>557</v>
       </c>
       <c r="G24" t="s">
         <v>63</v>
@@ -8877,20 +8781,20 @@
       </c>
     </row>
     <row r="25" spans="1:10" ht="43.5">
-      <c r="B25" s="30" t="s">
-        <v>586</v>
+      <c r="B25" s="28" t="s">
+        <v>579</v>
       </c>
       <c r="C25" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D25" t="s">
-        <v>554</v>
+        <v>547</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>555</v>
+        <v>548</v>
       </c>
       <c r="F25" t="s">
-        <v>556</v>
+        <v>549</v>
       </c>
       <c r="G25" t="s">
         <v>63</v>
@@ -8900,20 +8804,20 @@
       </c>
     </row>
     <row r="26" spans="1:10" ht="43.5">
-      <c r="B26" s="30" t="s">
-        <v>586</v>
+      <c r="B26" s="28" t="s">
+        <v>579</v>
       </c>
       <c r="C26" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="D26" t="s">
-        <v>568</v>
+        <v>561</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>567</v>
+        <v>560</v>
       </c>
       <c r="F26" t="s">
-        <v>566</v>
+        <v>559</v>
       </c>
       <c r="G26" t="s">
         <v>63</v>
@@ -8924,22 +8828,22 @@
     </row>
     <row r="27" spans="1:10" ht="58">
       <c r="A27" t="s">
-        <v>569</v>
-      </c>
-      <c r="B27" s="30" t="s">
-        <v>586</v>
+        <v>562</v>
+      </c>
+      <c r="B27" s="28" t="s">
+        <v>579</v>
       </c>
       <c r="C27" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D27" t="s">
-        <v>570</v>
+        <v>563</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>571</v>
+        <v>564</v>
       </c>
       <c r="F27" t="s">
-        <v>572</v>
+        <v>565</v>
       </c>
       <c r="G27" t="s">
         <v>63</v>
@@ -8953,22 +8857,22 @@
     </row>
     <row r="28" spans="1:10" ht="58">
       <c r="A28" t="s">
-        <v>577</v>
-      </c>
-      <c r="B28" s="31" t="s">
-        <v>518</v>
+        <v>570</v>
+      </c>
+      <c r="B28" s="29" t="s">
+        <v>511</v>
       </c>
       <c r="C28" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D28" t="s">
-        <v>574</v>
+        <v>567</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>575</v>
+        <v>568</v>
       </c>
       <c r="F28" t="s">
-        <v>576</v>
+        <v>569</v>
       </c>
       <c r="G28" t="s">
         <v>63</v>
@@ -8979,45 +8883,45 @@
     </row>
     <row r="29" spans="1:10" ht="116">
       <c r="A29" t="s">
-        <v>581</v>
-      </c>
-      <c r="B29" s="30" t="s">
-        <v>586</v>
+        <v>574</v>
+      </c>
+      <c r="B29" s="28" t="s">
+        <v>579</v>
       </c>
       <c r="C29" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="D29" t="s">
-        <v>578</v>
+        <v>571</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>579</v>
+        <v>572</v>
       </c>
       <c r="F29" t="s">
-        <v>580</v>
+        <v>573</v>
       </c>
       <c r="G29" t="s">
         <v>63</v>
       </c>
       <c r="H29" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="58">
-      <c r="B30" s="25" t="s">
-        <v>605</v>
+      <c r="B30" s="29" t="s">
+        <v>511</v>
       </c>
       <c r="C30" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D30" t="s">
-        <v>606</v>
+        <v>598</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="F30" t="s">
-        <v>607</v>
+        <v>599</v>
       </c>
       <c r="G30" t="s">
         <v>64</v>
@@ -9027,20 +8931,20 @@
       </c>
     </row>
     <row r="31" spans="1:10" ht="72.5">
-      <c r="B31" s="25" t="s">
-        <v>605</v>
+      <c r="B31" s="30" t="s">
+        <v>617</v>
       </c>
       <c r="C31" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D31" t="s">
-        <v>609</v>
+        <v>600</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>610</v>
+        <v>601</v>
       </c>
       <c r="F31" t="s">
-        <v>611</v>
+        <v>602</v>
       </c>
       <c r="G31" t="s">
         <v>64</v>
@@ -9051,19 +8955,19 @@
     </row>
     <row r="32" spans="1:10" ht="58">
       <c r="A32" t="s">
-        <v>615</v>
-      </c>
-      <c r="B32" s="25" t="s">
-        <v>573</v>
+        <v>606</v>
+      </c>
+      <c r="B32" s="30" t="s">
+        <v>617</v>
       </c>
       <c r="D32" t="s">
-        <v>612</v>
+        <v>603</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>614</v>
+        <v>605</v>
       </c>
       <c r="F32" t="s">
-        <v>613</v>
+        <v>604</v>
       </c>
       <c r="G32" t="s">
         <v>64</v>
@@ -9075,31 +8979,138 @@
         <v>77</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="72.5">
+    <row r="33" spans="1:9" ht="101.5">
       <c r="A33" t="s">
-        <v>619</v>
-      </c>
-      <c r="B33" s="25" t="s">
-        <v>573</v>
+        <v>609</v>
+      </c>
+      <c r="B33" s="28" t="s">
+        <v>579</v>
+      </c>
+      <c r="C33" t="s">
+        <v>465</v>
       </c>
       <c r="D33" t="s">
-        <v>616</v>
+        <v>607</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>618</v>
+        <v>610</v>
       </c>
       <c r="F33" t="s">
-        <v>617</v>
+        <v>608</v>
       </c>
       <c r="G33" t="s">
         <v>64</v>
       </c>
       <c r="H33" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="I33" t="s">
         <v>77</v>
       </c>
+    </row>
+    <row r="34" spans="1:9" ht="43.5">
+      <c r="B34" s="28" t="s">
+        <v>579</v>
+      </c>
+      <c r="C34" t="s">
+        <v>466</v>
+      </c>
+      <c r="D34" t="s">
+        <v>613</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="F34" t="s">
+        <v>615</v>
+      </c>
+      <c r="G34" t="s">
+        <v>64</v>
+      </c>
+      <c r="H34" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" t="s">
+        <v>609</v>
+      </c>
+      <c r="B35" s="28" t="s">
+        <v>579</v>
+      </c>
+      <c r="C35" t="s">
+        <v>466</v>
+      </c>
+      <c r="D35" t="s">
+        <v>619</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>620</v>
+      </c>
+      <c r="F35" t="s">
+        <v>621</v>
+      </c>
+      <c r="G35" t="s">
+        <v>64</v>
+      </c>
+      <c r="H35" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="43.5">
+      <c r="A36" t="s">
+        <v>625</v>
+      </c>
+      <c r="B36" s="28" t="s">
+        <v>579</v>
+      </c>
+      <c r="C36" t="s">
+        <v>465</v>
+      </c>
+      <c r="D36" t="s">
+        <v>622</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="F36" t="s">
+        <v>624</v>
+      </c>
+      <c r="G36" t="s">
+        <v>64</v>
+      </c>
+      <c r="H36" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="43.5">
+      <c r="A37" t="s">
+        <v>629</v>
+      </c>
+      <c r="B37" s="28" t="s">
+        <v>579</v>
+      </c>
+      <c r="C37" t="s">
+        <v>465</v>
+      </c>
+      <c r="D37" t="s">
+        <v>626</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>627</v>
+      </c>
+      <c r="F37" t="s">
+        <v>628</v>
+      </c>
+      <c r="G37" t="s">
+        <v>64</v>
+      </c>
+      <c r="H37" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="B38" s="29"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9120,18 +9131,18 @@
   <sheetData>
     <row r="1" spans="2:6">
       <c r="B1" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C1" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="D1" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
     </row>
     <row r="2" spans="2:6" ht="29">
       <c r="B2" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C2" t="s">
         <v>77</v>
@@ -9145,7 +9156,7 @@
     </row>
     <row r="3" spans="2:6" ht="29">
       <c r="B3" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C3" t="s">
         <v>77</v>
@@ -9157,23 +9168,23 @@
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="2:6" s="11" customFormat="1">
-      <c r="B5" s="19" t="s">
-        <v>435</v>
-      </c>
-      <c r="C5" s="11" t="s">
+    <row r="5" spans="2:6" s="10" customFormat="1">
+      <c r="B5" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="10" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="29">
       <c r="B7" s="2" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
       <c r="C7" t="s">
         <v>77</v>
@@ -9187,7 +9198,7 @@
     </row>
     <row r="8" spans="2:6" ht="29">
       <c r="B8" s="2" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
       <c r="C8" t="s">
         <v>77</v>
@@ -9212,7 +9223,7 @@
     </row>
     <row r="12" spans="2:6" ht="29">
       <c r="B12" s="2" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
       <c r="C12" t="s">
         <v>87</v>
@@ -9226,7 +9237,7 @@
     </row>
     <row r="17" spans="2:5" ht="43.5">
       <c r="B17" s="2" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
       <c r="C17" t="s">
         <v>84</v>
@@ -9235,7 +9246,7 @@
         <v>320</v>
       </c>
       <c r="E17" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add (codebook, 02_clean_data.R) added the variables and documentation for responding parents daily childcare time, respondng parents weekly working time, spouse's weekly working time;
to translate this into variables in 03_transform_data.R
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Vaccine Uptake - R\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4939D138-0F19-482F-819C-E3751D300180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B1D30C-94AA-4104-82B2-FBD934DB2275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -71,6 +71,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={869B55B9-3B1F-4453-9A39-E466CC7906FC}</author>
+    <author>tc={443BE410-81F7-49D5-89CA-23D177220CB4}</author>
   </authors>
   <commentList>
     <comment ref="L68" authorId="0" shapeId="0" xr:uid="{869B55B9-3B1F-4453-9A39-E466CC7906FC}">
@@ -84,12 +85,21 @@
 </t>
       </text>
     </comment>
+    <comment ref="E238" authorId="1" shapeId="0" xr:uid="{443BE410-81F7-49D5-89CA-23D177220CB4}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Come back and change the time bins based on how the data behaves
+</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1886" uniqueCount="635">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1934" uniqueCount="652">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -1999,13 +2009,64 @@
   </si>
   <si>
     <t>household_mortgage</t>
+  </si>
+  <si>
+    <t>The amount of time per day, which the responding parent spent on childcare</t>
+  </si>
+  <si>
+    <t>Numerical</t>
+  </si>
+  <si>
+    <t>parent_daily_childcare</t>
+  </si>
+  <si>
+    <t>The number of hours spent at work per week</t>
+  </si>
+  <si>
+    <t>parent_childcare_daily</t>
+  </si>
+  <si>
+    <t>hours</t>
+  </si>
+  <si>
+    <t>The number of hours the responding parent spends on childcare in a week</t>
+  </si>
+  <si>
+    <t>father_work_weekly</t>
+  </si>
+  <si>
+    <t>mother_work_weekly</t>
+  </si>
+  <si>
+    <t>The number of hours the COI's father spends at work per week</t>
+  </si>
+  <si>
+    <t>The number of hours the COI's mother spends at work per week</t>
+  </si>
+  <si>
+    <t>use the median value of the time bin of the number of hours spent per week on childcare by the responding parent</t>
+  </si>
+  <si>
+    <t>childcare_daily</t>
+  </si>
+  <si>
+    <t>take the approximate number of hours worked by the responding parent/spouse and determine which is the father respectively</t>
+  </si>
+  <si>
+    <t>parent_work_weekly</t>
+  </si>
+  <si>
+    <t>spouse_work_weekly</t>
+  </si>
+  <si>
+    <t>take the approximate number of hours worked by the responding parent/spouse and determine which is the mother respectively</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2056,6 +2117,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="14">
@@ -2165,7 +2232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2213,6 +2280,8 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2548,12 +2617,16 @@
 cases where parents = 2 but they arent married, i.e. divorced both parents might still have a say in the child’s vaccination
 </text>
   </threadedComment>
+  <threadedComment ref="E238" dT="2025-06-10T09:37:58.90" personId="{018BAD65-E158-4456-AEB2-B6F599AC9FA9}" id="{443BE410-81F7-49D5-89CA-23D177220CB4}">
+    <text xml:space="preserve">Come back and change the time bins based on how the data behaves
+</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CU9"/>
+  <dimension ref="A1:CW9"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="20.1796875" bestFit="1" customWidth="1"/>
@@ -2593,9 +2666,12 @@
     <col min="92" max="92" width="35.81640625" style="4" customWidth="1"/>
     <col min="93" max="96" width="35.81640625" bestFit="1" customWidth="1"/>
     <col min="97" max="98" width="35.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="22.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:99">
+    <row r="1" spans="1:101" ht="29">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2890,9 +2966,17 @@
       <c r="CT1" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="CU1" s="2"/>
-    </row>
-    <row r="2" spans="1:99">
+      <c r="CU1" s="2" t="s">
+        <v>637</v>
+      </c>
+      <c r="CV1" t="s">
+        <v>642</v>
+      </c>
+      <c r="CW1" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="2" spans="1:101" ht="72.5">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -3187,9 +3271,17 @@
       <c r="CT2" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="CU2" s="2"/>
-    </row>
-    <row r="3" spans="1:99" s="2" customFormat="1" ht="101.5">
+      <c r="CU2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="CV2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="CW2" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:101" s="2" customFormat="1" ht="101.5">
       <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
@@ -3411,8 +3503,17 @@
       </c>
       <c r="CS3" s="6"/>
       <c r="CT3" s="6"/>
-    </row>
-    <row r="4" spans="1:99">
+      <c r="CU3" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="CV3" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="CW3" s="2" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="4" spans="1:101">
       <c r="A4" s="9" t="s">
         <v>2</v>
       </c>
@@ -3707,8 +3808,17 @@
       <c r="CT4" s="7" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="5" spans="1:99">
+      <c r="CU4" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="CV4" t="s">
+        <v>636</v>
+      </c>
+      <c r="CW4" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="5" spans="1:101">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -3730,12 +3840,12 @@
       <c r="CS5" s="7"/>
       <c r="CT5" s="7"/>
     </row>
-    <row r="6" spans="1:99">
+    <row r="6" spans="1:101">
       <c r="A6" s="1"/>
       <c r="CS6" s="7"/>
       <c r="CT6" s="7"/>
     </row>
-    <row r="7" spans="1:99">
+    <row r="7" spans="1:101">
       <c r="A7" s="1" t="s">
         <v>106</v>
       </c>
@@ -3829,12 +3939,12 @@
       <c r="CS7" s="7"/>
       <c r="CT7" s="7"/>
     </row>
-    <row r="8" spans="1:99">
+    <row r="8" spans="1:101">
       <c r="A8" s="1"/>
       <c r="CS8" s="7"/>
       <c r="CT8" s="7"/>
     </row>
-    <row r="9" spans="1:99">
+    <row r="9" spans="1:101">
       <c r="A9" s="1"/>
       <c r="CS9" s="7"/>
       <c r="CT9" s="7"/>
@@ -3848,7 +3958,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83406F25-8B9E-4B45-BE5A-CFE07640E852}">
-  <dimension ref="A1:XFA237"/>
+  <dimension ref="A1:XFA240"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="35.81640625" bestFit="1" customWidth="1"/>
@@ -6188,7 +6298,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="123" spans="1:8" customFormat="1">
+    <row r="123" spans="1:8">
       <c r="A123" t="s">
         <v>96</v>
       </c>
@@ -6199,7 +6309,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="124" spans="1:8" customFormat="1">
+    <row r="124" spans="1:8">
       <c r="A124" t="s">
         <v>96</v>
       </c>
@@ -6225,19 +6335,19 @@
         <v>307</v>
       </c>
     </row>
-    <row r="125" spans="1:8" customFormat="1">
+    <row r="125" spans="1:8">
       <c r="A125" t="s">
         <v>96</v>
       </c>
       <c r="D125">
-        <f t="shared" ref="D125:L140" si="2">D124 +1</f>
+        <f t="shared" ref="D125:D140" si="2">D124 +1</f>
         <v>2</v>
       </c>
       <c r="E125" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="126" spans="1:8" customFormat="1">
+    <row r="126" spans="1:8">
       <c r="A126" t="s">
         <v>96</v>
       </c>
@@ -6249,7 +6359,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="127" spans="1:8" customFormat="1">
+    <row r="127" spans="1:8">
       <c r="A127" t="s">
         <v>96</v>
       </c>
@@ -6261,7 +6371,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="128" spans="1:8" customFormat="1">
+    <row r="128" spans="1:8">
       <c r="A128" t="s">
         <v>96</v>
       </c>
@@ -6273,7 +6383,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="129" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="129" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A129" t="s">
         <v>96</v>
       </c>
@@ -6285,7 +6395,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="130" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="130" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A130" t="s">
         <v>96</v>
       </c>
@@ -6297,7 +6407,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="131" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="131" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A131" t="s">
         <v>96</v>
       </c>
@@ -6309,7 +6419,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="132" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="132" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A132" t="s">
         <v>96</v>
       </c>
@@ -6321,7 +6431,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="133" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="133" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A133" t="s">
         <v>96</v>
       </c>
@@ -6333,7 +6443,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="134" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="134" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A134" t="s">
         <v>96</v>
       </c>
@@ -6345,7 +6455,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="135" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="135" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A135" t="s">
         <v>96</v>
       </c>
@@ -6357,7 +6467,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="136" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="136" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A136" t="s">
         <v>96</v>
       </c>
@@ -6369,7 +6479,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="137" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="137" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A137" t="s">
         <v>96</v>
       </c>
@@ -6381,7 +6491,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="138" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="138" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A138" t="s">
         <v>96</v>
       </c>
@@ -8440,7 +8550,7 @@
       <c r="XES138" s="19"/>
       <c r="XFA138" s="19"/>
     </row>
-    <row r="139" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="139" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A139" t="s">
         <v>96</v>
       </c>
@@ -8452,7 +8562,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="140" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="140" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A140" t="s">
         <v>96</v>
       </c>
@@ -8464,19 +8574,19 @@
         <v>411</v>
       </c>
     </row>
-    <row r="141" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="141" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A141" t="s">
         <v>96</v>
       </c>
       <c r="D141">
-        <f t="shared" ref="D141:BO141" si="3">D140 +1</f>
+        <f t="shared" ref="D141" si="3">D140 +1</f>
         <v>18</v>
       </c>
       <c r="E141" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="142" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="142" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A142" t="s">
         <v>96</v>
       </c>
@@ -8487,7 +8597,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="143" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="143" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A143" t="s">
         <v>96</v>
       </c>
@@ -8516,7 +8626,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="144" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" customFormat="1">
+    <row r="144" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381">
       <c r="A144" t="s">
         <v>96</v>
       </c>
@@ -9967,7 +10077,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="225" spans="1:12" s="4" customFormat="1">
+    <row r="225" spans="1:14" s="4" customFormat="1">
       <c r="A225" s="4" t="s">
         <v>96</v>
       </c>
@@ -9978,7 +10088,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="226" spans="1:12" s="4" customFormat="1">
+    <row r="226" spans="1:14" s="4" customFormat="1">
       <c r="A226" s="4" t="s">
         <v>96</v>
       </c>
@@ -9989,7 +10099,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="227" spans="1:12" s="4" customFormat="1">
+    <row r="227" spans="1:14" s="4" customFormat="1">
       <c r="A227" s="4" t="s">
         <v>96</v>
       </c>
@@ -10000,7 +10110,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="228" spans="1:12" s="4" customFormat="1">
+    <row r="228" spans="1:14" s="4" customFormat="1">
       <c r="A228" s="4" t="s">
         <v>96</v>
       </c>
@@ -10011,7 +10121,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="229" spans="1:12" s="4" customFormat="1">
+    <row r="229" spans="1:14" s="4" customFormat="1">
       <c r="A229" s="4" t="s">
         <v>96</v>
       </c>
@@ -10022,7 +10132,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="230" spans="1:12" s="4" customFormat="1">
+    <row r="230" spans="1:14" s="4" customFormat="1">
       <c r="A230" s="4" t="s">
         <v>96</v>
       </c>
@@ -10033,7 +10143,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="231" spans="1:12" s="4" customFormat="1">
+    <row r="231" spans="1:14" s="4" customFormat="1">
       <c r="A231" s="4" t="s">
         <v>96</v>
       </c>
@@ -10071,7 +10181,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="232" spans="1:12" s="4" customFormat="1">
+    <row r="232" spans="1:14" s="4" customFormat="1">
       <c r="A232" s="4" t="s">
         <v>96</v>
       </c>
@@ -10082,7 +10192,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="233" spans="1:12" s="4" customFormat="1">
+    <row r="233" spans="1:14" s="4" customFormat="1">
       <c r="A233" s="4" t="s">
         <v>96</v>
       </c>
@@ -10093,7 +10203,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="234" spans="1:12" s="4" customFormat="1">
+    <row r="234" spans="1:14" s="4" customFormat="1">
       <c r="A234" s="4" t="s">
         <v>96</v>
       </c>
@@ -10104,7 +10214,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="235" spans="1:12" s="4" customFormat="1">
+    <row r="235" spans="1:14" s="4" customFormat="1">
       <c r="A235" s="4" t="s">
         <v>96</v>
       </c>
@@ -10115,7 +10225,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="236" spans="1:12" s="4" customFormat="1">
+    <row r="236" spans="1:14" s="4" customFormat="1">
       <c r="A236" s="4" t="s">
         <v>96</v>
       </c>
@@ -10126,7 +10236,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="237" spans="1:12" s="4" customFormat="1">
+    <row r="237" spans="1:14" s="4" customFormat="1">
       <c r="A237" s="4" t="s">
         <v>96</v>
       </c>
@@ -10135,6 +10245,120 @@
       </c>
       <c r="E237" s="4" t="s">
         <v>231</v>
+      </c>
+    </row>
+    <row r="238" spans="1:14">
+      <c r="A238" t="s">
+        <v>96</v>
+      </c>
+      <c r="B238" t="s">
+        <v>639</v>
+      </c>
+      <c r="C238" t="s">
+        <v>260</v>
+      </c>
+      <c r="D238" t="s">
+        <v>640</v>
+      </c>
+      <c r="E238" s="31" t="s">
+        <v>641</v>
+      </c>
+      <c r="F238" t="s">
+        <v>646</v>
+      </c>
+      <c r="G238" t="s">
+        <v>647</v>
+      </c>
+      <c r="H238" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="239" spans="1:14">
+      <c r="A239" t="s">
+        <v>96</v>
+      </c>
+      <c r="B239" t="s">
+        <v>642</v>
+      </c>
+      <c r="C239" t="s">
+        <v>260</v>
+      </c>
+      <c r="D239" s="31" t="s">
+        <v>640</v>
+      </c>
+      <c r="E239" s="32" t="s">
+        <v>644</v>
+      </c>
+      <c r="F239" t="s">
+        <v>648</v>
+      </c>
+      <c r="G239" t="s">
+        <v>649</v>
+      </c>
+      <c r="H239" t="s">
+        <v>307</v>
+      </c>
+      <c r="I239" t="s">
+        <v>650</v>
+      </c>
+      <c r="J239" t="s">
+        <v>307</v>
+      </c>
+      <c r="K239" t="s">
+        <v>73</v>
+      </c>
+      <c r="L239" t="s">
+        <v>307</v>
+      </c>
+      <c r="M239" t="s">
+        <v>74</v>
+      </c>
+      <c r="N239" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="240" spans="1:14">
+      <c r="A240" t="s">
+        <v>96</v>
+      </c>
+      <c r="B240" t="s">
+        <v>643</v>
+      </c>
+      <c r="C240" t="s">
+        <v>260</v>
+      </c>
+      <c r="D240" s="32" t="s">
+        <v>640</v>
+      </c>
+      <c r="E240" s="32" t="s">
+        <v>645</v>
+      </c>
+      <c r="F240" t="s">
+        <v>651</v>
+      </c>
+      <c r="G240" t="s">
+        <v>649</v>
+      </c>
+      <c r="H240" t="s">
+        <v>307</v>
+      </c>
+      <c r="I240" t="s">
+        <v>650</v>
+      </c>
+      <c r="J240" t="s">
+        <v>307</v>
+      </c>
+      <c r="K240" t="s">
+        <v>73</v>
+      </c>
+      <c r="L240" t="s">
+        <v>307</v>
+      </c>
+      <c r="M240" t="s">
+        <v>74</v>
+      </c>
+      <c r="N240" t="s">
+        <v>307</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Master, added file to resolve functions with the same name
transform, added variable for mother and father's weekly working hours
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Vaccine Uptake - R\Data\JACSIS2023\processed\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangk\Desktop\vaccination_uptake_jacsis2023\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9911AA4B-6AA5-4FB1-928A-F6B74261CC51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A3E3069-EFCA-4065-9513-89A555A26DC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10890" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3470" yWindow="690" windowWidth="14400" windowHeight="8710" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -98,8 +98,63 @@
 </comments>
 </file>
 
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={7F40D788-9EC4-40FB-A9F9-AD66BD761ADD}</author>
+    <author>Kevin Wang</author>
+    <author>tc={96A696B5-9B70-421D-BAE5-16DC63333B7B}</author>
+  </authors>
+  <commentList>
+    <comment ref="D18" authorId="0" shapeId="0" xr:uid="{7F40D788-9EC4-40FB-A9F9-AD66BD761ADD}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Should be age_cat and age_of_interest
+I will figure it out and update once I find out which graph this is referring to</t>
+      </text>
+    </comment>
+    <comment ref="A44" authorId="1" shapeId="0" xr:uid="{596F102C-84BE-40F1-A512-14A8EBE941E9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Kevin Wang:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Has already been investigated by household_total * test_marital_status
+found to be null
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A45" authorId="2" shapeId="0" xr:uid="{96A696B5-9B70-421D-BAE5-16DC63333B7B}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Will be interesting to see if marital status (i..e single parents) are affected by the number of children they have to care for.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2015" uniqueCount="666">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2024" uniqueCount="673">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -1552,9 +1607,6 @@
     <t>The proportion of children who received no coverage, for single mothers (parents'marital status == 1), increased with increasing income</t>
   </si>
   <si>
-    <t>I don't think there's any sort of interaction here with the exception that the income levels generally cut off at half of the maximum level</t>
-  </si>
-  <si>
     <t>income_child_parents_</t>
   </si>
   <si>
@@ -2102,13 +2154,37 @@
   </si>
   <si>
     <t xml:space="preserve">translate the values of the survey responses directly </t>
+  </si>
+  <si>
+    <t>Investigate</t>
+  </si>
+  <si>
+    <t>Logically it makes sense that there is some interaction even though I don't think there's any sort of interaction here with the exception that the income levels generally cut off at half of the maximum level</t>
+  </si>
+  <si>
+    <t>This needs to be plotted</t>
+  </si>
+  <si>
+    <t>mother_employment_status * test_household_income</t>
+  </si>
+  <si>
+    <t>To investigate</t>
+  </si>
+  <si>
+    <t>mother's employment (i..e stay home or not proxy) and household income</t>
+  </si>
+  <si>
+    <t>marital status and total no. of indivs</t>
+  </si>
+  <si>
+    <t>marital status and total no. of siblings</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2166,8 +2242,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2258,6 +2347,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF99CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -2286,7 +2381,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2346,11 +2441,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2388,6 +2485,13 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF99CC"/>
+      <color rgb="FFFF99FF"/>
+      <color rgb="FFFF66CC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2402,6 +2506,7 @@
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="Kevin Wang" id="{018BAD65-E158-4456-AEB2-B6F599AC9FA9}" userId="aa11382e36a27e4c" providerId="Windows Live"/>
+  <person displayName="Wang Kevin" id="{F1230DF4-625E-4957-ABA0-003D3672236E}" userId="S::e1697655@u.nus.edu::ed0a20a1-e08d-41cd-86f8-80056833cbbd" providerId="AD"/>
 </personList>
 </file>
 
@@ -2693,6 +2798,18 @@
 </ThreadedComments>
 </file>
 
+<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="D18" dT="2025-12-10T07:33:20.85" personId="{F1230DF4-625E-4957-ABA0-003D3672236E}" id="{7F40D788-9EC4-40FB-A9F9-AD66BD761ADD}">
+    <text>Should be age_cat and age_of_interest
+I will figure it out and update once I find out which graph this is referring to</text>
+  </threadedComment>
+  <threadedComment ref="A45" dT="2025-12-10T07:47:28.93" personId="{F1230DF4-625E-4957-ABA0-003D3672236E}" id="{96A696B5-9B70-421D-BAE5-16DC63333B7B}">
+    <text>Will be interesting to see if marital status (i..e single parents) are affected by the number of children they have to care for.</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:DF9"/>
@@ -2738,7 +2855,7 @@
     <col min="99" max="99" width="19.54296875" style="7" bestFit="1" customWidth="1"/>
     <col min="100" max="100" width="21.453125" style="7" bestFit="1" customWidth="1"/>
     <col min="101" max="101" width="22.453125" style="7" bestFit="1" customWidth="1"/>
-    <col min="102" max="109" width="37.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="102" max="109" width="37.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:110" ht="29">
@@ -2929,7 +3046,7 @@
         <v>15</v>
       </c>
       <c r="BK1" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="BL1" s="20" t="s">
         <v>67</v>
@@ -2941,10 +3058,10 @@
         <v>69</v>
       </c>
       <c r="BO1" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="BP1" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="BQ1" s="4" t="s">
         <v>70</v>
@@ -2971,7 +3088,7 @@
         <v>77</v>
       </c>
       <c r="BY1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="BZ1" t="s">
         <v>78</v>
@@ -3016,7 +3133,7 @@
         <v>89</v>
       </c>
       <c r="CN1" s="4" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="CO1" t="s">
         <v>90</v>
@@ -3037,36 +3154,36 @@
         <v>95</v>
       </c>
       <c r="CU1" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="CV1" s="7" t="s">
+        <v>639</v>
+      </c>
+      <c r="CW1" s="7" t="s">
         <v>640</v>
       </c>
-      <c r="CW1" s="7" t="s">
-        <v>641</v>
-      </c>
-      <c r="CX1" s="39" t="s">
-        <v>653</v>
-      </c>
-      <c r="CY1" s="39" t="s">
+      <c r="CX1" t="s">
+        <v>652</v>
+      </c>
+      <c r="CY1" t="s">
         <v>56</v>
       </c>
-      <c r="CZ1" s="39" t="s">
+      <c r="CZ1" t="s">
         <v>55</v>
       </c>
-      <c r="DA1" s="39" t="s">
+      <c r="DA1" t="s">
         <v>54</v>
       </c>
-      <c r="DB1" s="39" t="s">
+      <c r="DB1" t="s">
         <v>53</v>
       </c>
-      <c r="DC1" s="39" t="s">
+      <c r="DC1" t="s">
         <v>52</v>
       </c>
-      <c r="DD1" s="39" t="s">
+      <c r="DD1" t="s">
         <v>51</v>
       </c>
-      <c r="DE1" s="39" t="s">
+      <c r="DE1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -3270,10 +3387,10 @@
         <v>96</v>
       </c>
       <c r="BO2" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="BP2" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="BQ2" s="4" t="s">
         <v>96</v>
@@ -3374,35 +3491,35 @@
       <c r="CW2" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="CX2" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="CY2" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="CZ2" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="DA2" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="DB2" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="DC2" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="DD2" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="DE2" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="DF2" s="39" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="3" spans="1:110" s="2" customFormat="1" ht="246.5">
+      <c r="CX2" t="s">
+        <v>96</v>
+      </c>
+      <c r="CY2" t="s">
+        <v>96</v>
+      </c>
+      <c r="CZ2" t="s">
+        <v>96</v>
+      </c>
+      <c r="DA2" t="s">
+        <v>96</v>
+      </c>
+      <c r="DB2" t="s">
+        <v>96</v>
+      </c>
+      <c r="DC2" t="s">
+        <v>96</v>
+      </c>
+      <c r="DD2" t="s">
+        <v>96</v>
+      </c>
+      <c r="DE2" t="s">
+        <v>96</v>
+      </c>
+      <c r="DF2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:110" s="2" customFormat="1" ht="101.5">
       <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
@@ -3526,7 +3643,7 @@
         <v>117</v>
       </c>
       <c r="BK3" s="2" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="BL3" s="21" t="s">
         <v>445</v>
@@ -3538,10 +3655,10 @@
         <v>444</v>
       </c>
       <c r="BO3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="BP3" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="BQ3" s="3" t="s">
         <v>134</v>
@@ -3565,7 +3682,7 @@
         <v>140</v>
       </c>
       <c r="BY3" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="BZ3" s="2" t="s">
         <v>141</v>
@@ -3598,17 +3715,17 @@
         <v>150</v>
       </c>
       <c r="CJ3" s="3" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="CK3" s="3" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="CL3" s="3"/>
       <c r="CM3" s="2" t="s">
         <v>151</v>
       </c>
       <c r="CN3" s="3" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="CO3" s="2" t="s">
         <v>152</v>
@@ -3625,37 +3742,37 @@
       <c r="CS3" s="6"/>
       <c r="CT3" s="6"/>
       <c r="CU3" s="6" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="CV3" s="6" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="CW3" s="6" t="s">
-        <v>636</v>
-      </c>
-      <c r="CX3" s="40" t="s">
+        <v>635</v>
+      </c>
+      <c r="CX3" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="CY3" s="2" t="s">
         <v>654</v>
       </c>
-      <c r="CY3" s="40" t="s">
+      <c r="CZ3" s="2" t="s">
         <v>655</v>
       </c>
-      <c r="CZ3" s="40" t="s">
+      <c r="DA3" s="2" t="s">
         <v>656</v>
       </c>
-      <c r="DA3" s="40" t="s">
+      <c r="DB3" s="2" t="s">
         <v>657</v>
       </c>
-      <c r="DB3" s="40" t="s">
+      <c r="DC3" s="2" t="s">
         <v>658</v>
       </c>
-      <c r="DC3" s="40" t="s">
+      <c r="DD3" s="2" t="s">
         <v>659</v>
       </c>
-      <c r="DD3" s="40" t="s">
+      <c r="DE3" s="2" t="s">
         <v>660</v>
-      </c>
-      <c r="DE3" s="40" t="s">
-        <v>661</v>
       </c>
     </row>
     <row r="4" spans="1:110">
@@ -3954,37 +4071,37 @@
         <v>99</v>
       </c>
       <c r="CU4" s="6" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="CV4" s="7" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="CW4" s="7" t="s">
-        <v>634</v>
-      </c>
-      <c r="CX4" s="39" t="s">
-        <v>662</v>
-      </c>
-      <c r="CY4" s="39" t="s">
-        <v>662</v>
-      </c>
-      <c r="CZ4" s="39" t="s">
-        <v>662</v>
-      </c>
-      <c r="DA4" s="39" t="s">
-        <v>662</v>
-      </c>
-      <c r="DB4" s="39" t="s">
-        <v>662</v>
-      </c>
-      <c r="DC4" s="39" t="s">
-        <v>662</v>
-      </c>
-      <c r="DD4" s="39" t="s">
-        <v>662</v>
-      </c>
-      <c r="DE4" s="39" t="s">
-        <v>662</v>
+        <v>633</v>
+      </c>
+      <c r="CX4" t="s">
+        <v>661</v>
+      </c>
+      <c r="CY4" t="s">
+        <v>661</v>
+      </c>
+      <c r="CZ4" t="s">
+        <v>661</v>
+      </c>
+      <c r="DA4" t="s">
+        <v>661</v>
+      </c>
+      <c r="DB4" t="s">
+        <v>661</v>
+      </c>
+      <c r="DC4" t="s">
+        <v>661</v>
+      </c>
+      <c r="DD4" t="s">
+        <v>661</v>
+      </c>
+      <c r="DE4" t="s">
+        <v>661</v>
       </c>
     </row>
     <row r="5" spans="1:110">
@@ -5328,7 +5445,7 @@
         <v>117</v>
       </c>
       <c r="F47" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="G47" t="s">
         <v>15</v>
@@ -5342,19 +5459,19 @@
         <v>96</v>
       </c>
       <c r="B48" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C48" t="s">
         <v>261</v>
       </c>
       <c r="D48" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="E48" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="F48" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="G48" t="s">
         <v>15</v>
@@ -5374,13 +5491,13 @@
         <v>96</v>
       </c>
       <c r="D49" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="E49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="F49" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -5388,13 +5505,13 @@
         <v>96</v>
       </c>
       <c r="D50" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="E50" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="F50" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -5408,7 +5525,7 @@
         <v>169</v>
       </c>
       <c r="F51" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="52" spans="1:12" s="4" customFormat="1">
@@ -5480,7 +5597,7 @@
         <v>96</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>260</v>
@@ -5489,10 +5606,10 @@
         <v>109</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="G54" s="4" t="s">
         <v>68</v>
@@ -5527,7 +5644,7 @@
         <v>109</v>
       </c>
       <c r="E55" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="F55" t="s">
         <v>442</v>
@@ -5550,7 +5667,7 @@
         <v>96</v>
       </c>
       <c r="B56" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C56" t="s">
         <v>260</v>
@@ -5559,10 +5676,10 @@
         <v>109</v>
       </c>
       <c r="E56" t="s">
+        <v>574</v>
+      </c>
+      <c r="F56" t="s">
         <v>575</v>
-      </c>
-      <c r="F56" t="s">
-        <v>576</v>
       </c>
       <c r="G56" t="s">
         <v>441</v>
@@ -6242,7 +6359,7 @@
         <v>96</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="C105" s="4" t="s">
         <v>260</v>
@@ -6254,10 +6371,10 @@
         <v>181</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="G105" s="4" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="H105" s="4" t="s">
         <v>307</v>
@@ -6483,7 +6600,7 @@
         <v>96</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="C124" s="4" t="s">
         <v>260</v>
@@ -6495,10 +6612,10 @@
         <v>181</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="G124" s="4" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="H124" s="4" t="s">
         <v>307</v>
@@ -10097,7 +10214,7 @@
         <v>388</v>
       </c>
       <c r="F217" s="4" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="G217" s="4" t="s">
         <v>66</v>
@@ -10138,7 +10255,7 @@
         <v>1</v>
       </c>
       <c r="E218" s="4" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="219" spans="1:16" s="4" customFormat="1">
@@ -10149,7 +10266,7 @@
         <v>1.5</v>
       </c>
       <c r="E219" s="4" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="220" spans="1:16" s="4" customFormat="1">
@@ -10160,7 +10277,7 @@
         <v>2</v>
       </c>
       <c r="E220" s="4" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="221" spans="1:16" s="4" customFormat="1">
@@ -10213,7 +10330,7 @@
         <v>388</v>
       </c>
       <c r="F224" s="4" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="G224" s="4" t="s">
         <v>66</v>
@@ -10254,7 +10371,7 @@
         <v>1</v>
       </c>
       <c r="E225" s="4" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="226" spans="1:14" s="4" customFormat="1">
@@ -10265,7 +10382,7 @@
         <v>1.5</v>
       </c>
       <c r="E226" s="4" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="227" spans="1:14" s="4" customFormat="1">
@@ -10276,7 +10393,7 @@
         <v>2</v>
       </c>
       <c r="E227" s="4" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="228" spans="1:14" s="4" customFormat="1">
@@ -10317,7 +10434,7 @@
         <v>96</v>
       </c>
       <c r="B231" s="4" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="C231" s="4" t="s">
         <v>261</v>
@@ -10329,7 +10446,7 @@
         <v>388</v>
       </c>
       <c r="F231" s="4" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="G231" s="4" t="s">
         <v>66</v>
@@ -10358,7 +10475,7 @@
         <v>1</v>
       </c>
       <c r="E232" s="4" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="233" spans="1:14" s="4" customFormat="1">
@@ -10369,7 +10486,7 @@
         <v>1.5</v>
       </c>
       <c r="E233" s="4" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="234" spans="1:14" s="4" customFormat="1">
@@ -10380,7 +10497,7 @@
         <v>2</v>
       </c>
       <c r="E234" s="4" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="235" spans="1:14" s="4" customFormat="1">
@@ -10421,22 +10538,22 @@
         <v>96</v>
       </c>
       <c r="B238" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="C238" t="s">
         <v>260</v>
       </c>
       <c r="D238" t="s">
+        <v>637</v>
+      </c>
+      <c r="E238" s="31" t="s">
         <v>638</v>
       </c>
-      <c r="E238" s="31" t="s">
-        <v>639</v>
-      </c>
       <c r="F238" t="s">
+        <v>643</v>
+      </c>
+      <c r="G238" t="s">
         <v>644</v>
-      </c>
-      <c r="G238" t="s">
-        <v>645</v>
       </c>
       <c r="H238" t="s">
         <v>307</v>
@@ -10447,28 +10564,28 @@
         <v>96</v>
       </c>
       <c r="B239" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="C239" t="s">
         <v>260</v>
       </c>
       <c r="D239" s="31" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="E239" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="F239" t="s">
+        <v>645</v>
+      </c>
+      <c r="G239" t="s">
         <v>646</v>
-      </c>
-      <c r="G239" t="s">
-        <v>647</v>
       </c>
       <c r="H239" t="s">
         <v>307</v>
       </c>
       <c r="I239" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="J239" t="s">
         <v>307</v>
@@ -10491,28 +10608,28 @@
         <v>96</v>
       </c>
       <c r="B240" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="C240" t="s">
         <v>260</v>
       </c>
       <c r="D240" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="E240" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="F240" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="G240" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="H240" t="s">
         <v>307</v>
       </c>
       <c r="I240" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="J240" t="s">
         <v>307</v>
@@ -10534,160 +10651,160 @@
       <c r="A241" t="s">
         <v>96</v>
       </c>
-      <c r="B241" s="39" t="s">
+      <c r="B241" t="s">
+        <v>652</v>
+      </c>
+      <c r="C241" t="s">
+        <v>662</v>
+      </c>
+      <c r="D241" s="39" t="s">
+        <v>663</v>
+      </c>
+      <c r="E241" s="2" t="s">
         <v>653</v>
       </c>
-      <c r="C241" t="s">
-        <v>663</v>
-      </c>
-      <c r="D241" s="41" t="s">
+      <c r="F241" t="s">
         <v>664</v>
-      </c>
-      <c r="E241" s="40" t="s">
-        <v>654</v>
-      </c>
-      <c r="F241" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="242" spans="1:6">
       <c r="A242" t="s">
         <v>96</v>
       </c>
-      <c r="B242" s="39" t="s">
+      <c r="B242" t="s">
         <v>56</v>
       </c>
       <c r="C242" t="s">
+        <v>662</v>
+      </c>
+      <c r="D242" s="39" t="s">
         <v>663</v>
       </c>
-      <c r="D242" s="41" t="s">
+      <c r="E242" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="F242" t="s">
         <v>664</v>
-      </c>
-      <c r="E242" s="40" t="s">
-        <v>655</v>
-      </c>
-      <c r="F242" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="243" spans="1:6">
       <c r="A243" t="s">
         <v>96</v>
       </c>
-      <c r="B243" s="39" t="s">
+      <c r="B243" t="s">
         <v>55</v>
       </c>
       <c r="C243" t="s">
+        <v>662</v>
+      </c>
+      <c r="D243" s="39" t="s">
         <v>663</v>
       </c>
-      <c r="D243" s="41" t="s">
+      <c r="E243" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="F243" t="s">
         <v>664</v>
-      </c>
-      <c r="E243" s="40" t="s">
-        <v>656</v>
-      </c>
-      <c r="F243" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="244" spans="1:6">
       <c r="A244" t="s">
         <v>96</v>
       </c>
-      <c r="B244" s="39" t="s">
+      <c r="B244" t="s">
         <v>54</v>
       </c>
       <c r="C244" t="s">
+        <v>662</v>
+      </c>
+      <c r="D244" s="39" t="s">
         <v>663</v>
       </c>
-      <c r="D244" s="41" t="s">
+      <c r="E244" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="F244" t="s">
         <v>664</v>
-      </c>
-      <c r="E244" s="40" t="s">
-        <v>657</v>
-      </c>
-      <c r="F244" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="245" spans="1:6">
       <c r="A245" t="s">
         <v>96</v>
       </c>
-      <c r="B245" s="39" t="s">
+      <c r="B245" t="s">
         <v>53</v>
       </c>
       <c r="C245" t="s">
+        <v>662</v>
+      </c>
+      <c r="D245" s="39" t="s">
         <v>663</v>
       </c>
-      <c r="D245" s="41" t="s">
+      <c r="E245" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="F245" t="s">
         <v>664</v>
-      </c>
-      <c r="E245" s="40" t="s">
-        <v>658</v>
-      </c>
-      <c r="F245" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="246" spans="1:6">
       <c r="A246" t="s">
         <v>96</v>
       </c>
-      <c r="B246" s="39" t="s">
+      <c r="B246" t="s">
         <v>52</v>
       </c>
       <c r="C246" t="s">
+        <v>662</v>
+      </c>
+      <c r="D246" s="39" t="s">
         <v>663</v>
       </c>
-      <c r="D246" s="41" t="s">
+      <c r="E246" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="F246" t="s">
         <v>664</v>
-      </c>
-      <c r="E246" s="40" t="s">
-        <v>659</v>
-      </c>
-      <c r="F246" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="247" spans="1:6">
       <c r="A247" t="s">
         <v>96</v>
       </c>
-      <c r="B247" s="39" t="s">
+      <c r="B247" t="s">
         <v>51</v>
       </c>
       <c r="C247" t="s">
+        <v>662</v>
+      </c>
+      <c r="D247" s="39" t="s">
         <v>663</v>
       </c>
-      <c r="D247" s="41" t="s">
+      <c r="E247" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="F247" t="s">
         <v>664</v>
-      </c>
-      <c r="E247" s="40" t="s">
-        <v>660</v>
-      </c>
-      <c r="F247" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="248" spans="1:6">
       <c r="A248" t="s">
         <v>96</v>
       </c>
-      <c r="B248" s="39" t="s">
+      <c r="B248" t="s">
         <v>50</v>
       </c>
       <c r="C248" t="s">
+        <v>662</v>
+      </c>
+      <c r="D248" s="39" t="s">
         <v>663</v>
       </c>
-      <c r="D248" s="41" t="s">
+      <c r="E248" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="F248" t="s">
         <v>664</v>
-      </c>
-      <c r="E248" s="40" t="s">
-        <v>661</v>
-      </c>
-      <c r="F248" t="s">
-        <v>665</v>
       </c>
     </row>
   </sheetData>
@@ -10784,16 +10901,16 @@
         <v>66</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="V1" s="2" t="s">
         <v>69</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="X1" s="2" t="s">
         <v>71</v>
@@ -10968,14 +11085,14 @@
     </row>
     <row r="21" spans="1:41">
       <c r="A21" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="L21" s="22"/>
       <c r="AN21" s="15"/>
     </row>
     <row r="22" spans="1:41">
       <c r="A22" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="L22" s="22"/>
       <c r="M22" s="22"/>
@@ -10992,7 +11109,7 @@
     </row>
     <row r="24" spans="1:41">
       <c r="A24" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="M24" s="15"/>
       <c r="P24" s="15"/>
@@ -11249,8 +11366,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313888EE-552D-40AA-8234-3B847E46EF43}">
-  <dimension ref="A1:J38"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313888EE-552D-40AA-8234-3B847E46EF43}">
+  <dimension ref="A1:J45"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="55.7265625" bestFit="1" customWidth="1"/>
@@ -11290,21 +11407,21 @@
         <v>460</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="29">
-      <c r="A2" t="s">
-        <v>482</v>
-      </c>
-      <c r="B2" s="27" t="s">
-        <v>513</v>
+    <row r="2" spans="1:10" ht="61.5" customHeight="1">
+      <c r="A2" s="22" t="s">
+        <v>666</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>665</v>
       </c>
       <c r="C2" t="s">
         <v>169</v>
       </c>
       <c r="D2" t="s">
+        <v>482</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>483</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>484</v>
       </c>
       <c r="F2" t="s">
         <v>169</v>
@@ -11321,7 +11438,7 @@
         <v>459</v>
       </c>
       <c r="B3" s="27" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C3" t="s">
         <v>466</v>
@@ -11350,16 +11467,16 @@
     </row>
     <row r="4" spans="1:10" ht="43.5">
       <c r="A4" s="22" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C4" t="s">
         <v>464</v>
       </c>
       <c r="D4" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>457</v>
@@ -11368,7 +11485,7 @@
         <v>461</v>
       </c>
       <c r="G4" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="H4" t="s">
         <v>77</v>
@@ -11376,16 +11493,16 @@
     </row>
     <row r="5" spans="1:10" ht="43.5">
       <c r="A5" s="22" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C5" t="s">
         <v>464</v>
       </c>
       <c r="D5" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>456</v>
@@ -11394,7 +11511,7 @@
         <v>462</v>
       </c>
       <c r="G5" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="H5" t="s">
         <v>77</v>
@@ -11402,25 +11519,25 @@
     </row>
     <row r="6" spans="1:10" s="32" customFormat="1" ht="29">
       <c r="A6" s="32" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C6" s="32" t="s">
         <v>465</v>
       </c>
       <c r="D6" s="32" t="s">
+        <v>590</v>
+      </c>
+      <c r="E6" s="34" t="s">
         <v>591</v>
       </c>
-      <c r="E6" s="34" t="s">
+      <c r="F6" s="32" t="s">
         <v>592</v>
       </c>
-      <c r="F6" s="32" t="s">
-        <v>593</v>
-      </c>
       <c r="G6" s="32" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="H6" s="32" t="s">
         <v>383</v>
@@ -11431,13 +11548,13 @@
     </row>
     <row r="7" spans="1:10" s="32" customFormat="1">
       <c r="A7" s="32" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E7" s="34"/>
       <c r="F7" s="32" t="s">
@@ -11455,11 +11572,11 @@
     </row>
     <row r="8" spans="1:10" s="32" customFormat="1">
       <c r="A8" s="32" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B8" s="33"/>
       <c r="D8" s="32" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="E8" s="34"/>
       <c r="G8" s="32" t="s">
@@ -11474,7 +11591,7 @@
     </row>
     <row r="9" spans="1:10" ht="43.5">
       <c r="B9" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C9" t="s">
         <v>466</v>
@@ -11483,13 +11600,13 @@
         <v>454</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="F9" t="s">
         <v>517</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>518</v>
-      </c>
-      <c r="G9" t="s">
-        <v>519</v>
       </c>
       <c r="H9" t="s">
         <v>77</v>
@@ -11497,7 +11614,7 @@
     </row>
     <row r="10" spans="1:10" ht="43.5">
       <c r="B10" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="C10" t="s">
         <v>464</v>
@@ -11506,18 +11623,18 @@
         <v>454</v>
       </c>
       <c r="E10" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="F10" t="s">
         <v>514</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>515</v>
-      </c>
-      <c r="G10" t="s">
-        <v>516</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="43.5">
       <c r="B11" s="25" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C11" t="s">
         <v>464</v>
@@ -11538,374 +11655,348 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="29">
-      <c r="B12" s="26" t="s">
-        <v>513</v>
-      </c>
-      <c r="C12" t="s">
+    <row r="13" spans="1:10" ht="29">
+      <c r="B13" s="28" t="s">
+        <v>512</v>
+      </c>
+      <c r="C13" t="s">
         <v>465</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D13" t="s">
         <v>467</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>473</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F13" t="s">
         <v>474</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G13" t="s">
         <v>84</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H13" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:10" s="32" customFormat="1" ht="43.5">
-      <c r="A13" s="34" t="s">
-        <v>651</v>
-      </c>
-      <c r="B13" s="33" t="s">
-        <v>511</v>
-      </c>
-      <c r="C13" s="32" t="s">
+    <row r="14" spans="1:10" s="32" customFormat="1" ht="43.5">
+      <c r="A14" s="34" t="s">
+        <v>650</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>510</v>
+      </c>
+      <c r="C14" s="32" t="s">
         <v>465</v>
       </c>
-      <c r="D13" s="32" t="s">
+      <c r="D14" s="32" t="s">
         <v>471</v>
       </c>
-      <c r="E13" s="34" t="s">
+      <c r="E14" s="34" t="s">
         <v>472</v>
       </c>
-      <c r="F13" s="32" t="s">
-        <v>589</v>
-      </c>
-      <c r="G13" s="32" t="s">
+      <c r="F14" s="32" t="s">
+        <v>588</v>
+      </c>
+      <c r="G14" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="H13" s="32" t="s">
+      <c r="H14" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="I13" s="32" t="s">
+      <c r="I14" s="32" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="43.5">
-      <c r="B14" s="27" t="s">
-        <v>513</v>
-      </c>
-      <c r="C14" t="s">
+    <row r="15" spans="1:10" ht="43.5">
+      <c r="B15" s="27" t="s">
+        <v>512</v>
+      </c>
+      <c r="C15" t="s">
         <v>169</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D15" t="s">
         <v>477</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>478</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F15" t="s">
         <v>169</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G15" t="s">
         <v>84</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H15" t="s">
         <v>77</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I15" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="58">
-      <c r="A15" t="s">
-        <v>487</v>
-      </c>
-      <c r="B15" s="28" t="s">
-        <v>577</v>
-      </c>
-      <c r="C15" t="s">
-        <v>466</v>
-      </c>
-      <c r="D15" t="s">
-        <v>488</v>
-      </c>
-      <c r="E15" s="2" t="s">
+    <row r="16" spans="1:10" ht="58">
+      <c r="A16" t="s">
         <v>486</v>
       </c>
-      <c r="F15" t="s">
-        <v>485</v>
-      </c>
-      <c r="G15" t="s">
-        <v>384</v>
-      </c>
-      <c r="H15" t="s">
-        <v>15</v>
-      </c>
-      <c r="I15" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="43.5">
-      <c r="A16" t="s">
-        <v>528</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>511</v>
+      <c r="B16" s="28" t="s">
+        <v>576</v>
       </c>
       <c r="C16" t="s">
         <v>466</v>
       </c>
       <c r="D16" t="s">
-        <v>510</v>
+        <v>487</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>610</v>
+        <v>485</v>
       </c>
       <c r="F16" t="s">
-        <v>509</v>
+        <v>484</v>
       </c>
       <c r="G16" t="s">
-        <v>508</v>
+        <v>384</v>
       </c>
       <c r="H16" t="s">
         <v>15</v>
       </c>
       <c r="I16" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="43.5">
+      <c r="A17" t="s">
+        <v>527</v>
+      </c>
       <c r="B17" s="29" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C17" t="s">
         <v>466</v>
       </c>
       <c r="D17" t="s">
-        <v>628</v>
+        <v>509</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>522</v>
+        <v>609</v>
       </c>
       <c r="F17" t="s">
-        <v>523</v>
+        <v>508</v>
       </c>
       <c r="G17" t="s">
-        <v>496</v>
+        <v>507</v>
       </c>
       <c r="H17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" ht="58">
-      <c r="A18" t="s">
-        <v>526</v>
-      </c>
-      <c r="B18" s="28" t="s">
-        <v>577</v>
+      <c r="I17" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="B18" s="29" t="s">
+        <v>510</v>
       </c>
       <c r="C18" t="s">
         <v>466</v>
       </c>
       <c r="D18" t="s">
-        <v>527</v>
+        <v>627</v>
       </c>
       <c r="E18" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="F18" t="s">
+        <v>522</v>
+      </c>
+      <c r="G18" t="s">
+        <v>495</v>
+      </c>
+      <c r="H18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="58">
+      <c r="A19" t="s">
+        <v>525</v>
+      </c>
+      <c r="B19" s="28" t="s">
+        <v>576</v>
+      </c>
+      <c r="C19" t="s">
+        <v>466</v>
+      </c>
+      <c r="D19" t="s">
+        <v>526</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="F19" t="s">
         <v>524</v>
       </c>
-      <c r="F18" t="s">
-        <v>525</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="G19" t="s">
         <v>71</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H19" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="43.5">
-      <c r="A19" t="s">
+    <row r="20" spans="1:10" ht="43.5">
+      <c r="A20" t="s">
+        <v>532</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>576</v>
+      </c>
+      <c r="C20" t="s">
+        <v>464</v>
+      </c>
+      <c r="D20" t="s">
+        <v>528</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="F20" t="s">
+        <v>529</v>
+      </c>
+      <c r="G20" t="s">
+        <v>530</v>
+      </c>
+      <c r="H20" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" s="35" customFormat="1" ht="29">
+      <c r="A21" s="35" t="s">
+        <v>651</v>
+      </c>
+      <c r="B21" s="36" t="s">
+        <v>510</v>
+      </c>
+      <c r="C21" s="35" t="s">
+        <v>464</v>
+      </c>
+      <c r="D21" s="35" t="s">
         <v>533</v>
       </c>
-      <c r="B19" s="28" t="s">
-        <v>577</v>
-      </c>
-      <c r="C19" t="s">
-        <v>464</v>
-      </c>
-      <c r="D19" t="s">
-        <v>529</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>532</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="E21" s="37" t="s">
+        <v>534</v>
+      </c>
+      <c r="F21" s="35" t="s">
+        <v>535</v>
+      </c>
+      <c r="G21" s="35" t="s">
         <v>530</v>
       </c>
-      <c r="G19" t="s">
-        <v>531</v>
-      </c>
-      <c r="H19" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" s="35" customFormat="1" ht="29">
-      <c r="A20" s="35" t="s">
-        <v>652</v>
-      </c>
-      <c r="B20" s="36" t="s">
-        <v>511</v>
-      </c>
-      <c r="C20" s="35" t="s">
-        <v>464</v>
-      </c>
-      <c r="D20" s="35" t="s">
-        <v>534</v>
-      </c>
-      <c r="E20" s="37" t="s">
-        <v>535</v>
-      </c>
-      <c r="F20" s="35" t="s">
-        <v>536</v>
-      </c>
-      <c r="G20" s="35" t="s">
-        <v>531</v>
-      </c>
-      <c r="H20" s="35" t="s">
+      <c r="H21" s="35" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="43.5">
-      <c r="A21" t="s">
-        <v>539</v>
-      </c>
-      <c r="B21" s="28" t="s">
-        <v>577</v>
-      </c>
-      <c r="C21" t="s">
-        <v>466</v>
-      </c>
-      <c r="D21" t="s">
-        <v>537</v>
-      </c>
-      <c r="E21" s="2" t="s">
+    <row r="22" spans="1:10" ht="43.5">
+      <c r="A22" t="s">
         <v>538</v>
       </c>
-      <c r="F21" t="s">
-        <v>540</v>
-      </c>
-      <c r="G21" t="s">
-        <v>531</v>
-      </c>
-      <c r="H21" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10">
-      <c r="A22" t="s">
-        <v>543</v>
-      </c>
       <c r="B22" s="28" t="s">
-        <v>564</v>
+        <v>576</v>
       </c>
       <c r="C22" t="s">
         <v>466</v>
       </c>
       <c r="D22" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="E22" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="F22" t="s">
+        <v>539</v>
+      </c>
+      <c r="G22" t="s">
+        <v>530</v>
+      </c>
+      <c r="H22" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10">
+      <c r="A23" t="s">
         <v>542</v>
       </c>
-      <c r="F22" t="s">
-        <v>541</v>
-      </c>
-      <c r="G22" t="s">
-        <v>531</v>
-      </c>
-      <c r="H22" t="s">
-        <v>64</v>
-      </c>
-      <c r="I22" t="s">
-        <v>78</v>
-      </c>
-      <c r="J22" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="72.5">
-      <c r="A23" t="s">
-        <v>550</v>
-      </c>
       <c r="B23" s="28" t="s">
-        <v>577</v>
+        <v>563</v>
       </c>
       <c r="C23" t="s">
         <v>466</v>
       </c>
       <c r="D23" t="s">
-        <v>552</v>
+        <v>543</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>551</v>
+        <v>541</v>
       </c>
       <c r="F23" t="s">
+        <v>540</v>
+      </c>
+      <c r="G23" t="s">
+        <v>530</v>
+      </c>
+      <c r="H23" t="s">
+        <v>64</v>
+      </c>
+      <c r="I23" t="s">
+        <v>78</v>
+      </c>
+      <c r="J23" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="72.5">
+      <c r="A24" t="s">
         <v>549</v>
       </c>
-      <c r="G23" t="s">
-        <v>63</v>
-      </c>
-      <c r="H23" t="s">
-        <v>548</v>
-      </c>
-      <c r="I23" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="87">
-      <c r="A24" t="s">
-        <v>553</v>
-      </c>
       <c r="B24" s="28" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C24" t="s">
         <v>466</v>
       </c>
       <c r="D24" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>556</v>
+        <v>550</v>
       </c>
       <c r="F24" t="s">
-        <v>555</v>
+        <v>548</v>
       </c>
       <c r="G24" t="s">
         <v>63</v>
       </c>
       <c r="H24" t="s">
-        <v>64</v>
+        <v>547</v>
       </c>
       <c r="I24" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="43.5">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="87">
+      <c r="A25" t="s">
+        <v>552</v>
+      </c>
       <c r="B25" s="28" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C25" t="s">
         <v>466</v>
       </c>
       <c r="D25" t="s">
-        <v>545</v>
+        <v>553</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>546</v>
+        <v>555</v>
       </c>
       <c r="F25" t="s">
-        <v>547</v>
+        <v>554</v>
       </c>
       <c r="G25" t="s">
         <v>63</v>
@@ -11913,48 +12004,48 @@
       <c r="H25" t="s">
         <v>64</v>
       </c>
+      <c r="I25" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="26" spans="1:10" ht="43.5">
       <c r="B26" s="28" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C26" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D26" t="s">
-        <v>559</v>
+        <v>544</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>558</v>
+        <v>545</v>
       </c>
       <c r="F26" t="s">
-        <v>557</v>
+        <v>546</v>
       </c>
       <c r="G26" t="s">
         <v>63</v>
       </c>
       <c r="H26" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="58">
-      <c r="A27" t="s">
-        <v>560</v>
-      </c>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="43.5">
       <c r="B27" s="28" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C27" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="D27" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="F27" t="s">
-        <v>563</v>
+        <v>556</v>
       </c>
       <c r="G27" t="s">
         <v>63</v>
@@ -11962,123 +12053,126 @@
       <c r="H27" t="s">
         <v>71</v>
       </c>
-      <c r="I27" t="s">
-        <v>77</v>
-      </c>
     </row>
     <row r="28" spans="1:10" ht="58">
       <c r="A28" t="s">
-        <v>568</v>
-      </c>
-      <c r="B28" s="29" t="s">
-        <v>511</v>
+        <v>559</v>
+      </c>
+      <c r="B28" s="28" t="s">
+        <v>576</v>
       </c>
       <c r="C28" t="s">
         <v>466</v>
       </c>
       <c r="D28" t="s">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>566</v>
+        <v>561</v>
       </c>
       <c r="F28" t="s">
-        <v>567</v>
+        <v>562</v>
       </c>
       <c r="G28" t="s">
         <v>63</v>
       </c>
       <c r="H28" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="116">
+        <v>71</v>
+      </c>
+      <c r="I28" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="58">
       <c r="A29" t="s">
-        <v>572</v>
-      </c>
-      <c r="B29" s="28" t="s">
-        <v>577</v>
+        <v>567</v>
+      </c>
+      <c r="B29" s="29" t="s">
+        <v>510</v>
       </c>
       <c r="C29" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D29" t="s">
-        <v>569</v>
+        <v>564</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>570</v>
+        <v>565</v>
       </c>
       <c r="F29" t="s">
-        <v>571</v>
+        <v>566</v>
       </c>
       <c r="G29" t="s">
         <v>63</v>
       </c>
       <c r="H29" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="58">
-      <c r="B30" s="29" t="s">
-        <v>511</v>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="116">
+      <c r="A30" t="s">
+        <v>571</v>
+      </c>
+      <c r="B30" s="28" t="s">
+        <v>576</v>
       </c>
       <c r="C30" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="D30" t="s">
-        <v>596</v>
+        <v>568</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>609</v>
+        <v>569</v>
       </c>
       <c r="F30" t="s">
-        <v>597</v>
+        <v>570</v>
       </c>
       <c r="G30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H30" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="72.5">
-      <c r="B31" s="30" t="s">
-        <v>615</v>
+        <v>488</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="58">
+      <c r="B31" s="29" t="s">
+        <v>510</v>
       </c>
       <c r="C31" t="s">
         <v>466</v>
       </c>
       <c r="D31" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>599</v>
+        <v>608</v>
       </c>
       <c r="F31" t="s">
-        <v>600</v>
+        <v>596</v>
       </c>
       <c r="G31" t="s">
         <v>64</v>
       </c>
       <c r="H31" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="58">
-      <c r="A32" t="s">
-        <v>604</v>
-      </c>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="72.5">
       <c r="B32" s="30" t="s">
-        <v>615</v>
+        <v>614</v>
+      </c>
+      <c r="C32" t="s">
+        <v>466</v>
       </c>
       <c r="D32" t="s">
-        <v>601</v>
+        <v>597</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>603</v>
+        <v>598</v>
       </c>
       <c r="F32" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="G32" t="s">
         <v>64</v>
@@ -12086,145 +12180,219 @@
       <c r="H32" t="s">
         <v>60</v>
       </c>
-      <c r="I32" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="101.5">
+    </row>
+    <row r="33" spans="1:9" ht="58">
       <c r="A33" t="s">
-        <v>607</v>
-      </c>
-      <c r="B33" s="28" t="s">
-        <v>577</v>
-      </c>
-      <c r="C33" t="s">
-        <v>465</v>
+        <v>603</v>
+      </c>
+      <c r="B33" s="30" t="s">
+        <v>614</v>
       </c>
       <c r="D33" t="s">
-        <v>605</v>
+        <v>600</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>608</v>
+        <v>602</v>
       </c>
       <c r="F33" t="s">
-        <v>606</v>
+        <v>601</v>
       </c>
       <c r="G33" t="s">
         <v>64</v>
       </c>
       <c r="H33" t="s">
-        <v>573</v>
+        <v>60</v>
       </c>
       <c r="I33" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="43.5">
+    <row r="34" spans="1:9" ht="101.5">
+      <c r="A34" t="s">
+        <v>606</v>
+      </c>
       <c r="B34" s="28" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C34" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="D34" t="s">
-        <v>611</v>
+        <v>604</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>612</v>
+        <v>607</v>
       </c>
       <c r="F34" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="G34" t="s">
         <v>64</v>
       </c>
       <c r="H34" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9">
-      <c r="A35" t="s">
-        <v>607</v>
-      </c>
+        <v>572</v>
+      </c>
+      <c r="I34" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="43.5">
       <c r="B35" s="28" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C35" t="s">
         <v>466</v>
       </c>
       <c r="D35" t="s">
-        <v>617</v>
+        <v>610</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>618</v>
+        <v>611</v>
       </c>
       <c r="F35" t="s">
-        <v>619</v>
+        <v>612</v>
       </c>
       <c r="G35" t="s">
         <v>64</v>
       </c>
       <c r="H35" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="43.5">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
       <c r="A36" t="s">
-        <v>623</v>
+        <v>606</v>
       </c>
       <c r="B36" s="28" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C36" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D36" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="F36" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
       <c r="G36" t="s">
         <v>64</v>
       </c>
       <c r="H36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="43.5">
       <c r="A37" t="s">
-        <v>627</v>
+        <v>622</v>
       </c>
       <c r="B37" s="28" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C37" t="s">
         <v>465</v>
       </c>
       <c r="D37" t="s">
-        <v>624</v>
+        <v>619</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>625</v>
+        <v>620</v>
       </c>
       <c r="F37" t="s">
-        <v>626</v>
+        <v>621</v>
       </c>
       <c r="G37" t="s">
         <v>64</v>
       </c>
       <c r="H37" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="43.5">
+      <c r="A38" t="s">
+        <v>626</v>
+      </c>
+      <c r="B38" s="28" t="s">
+        <v>576</v>
+      </c>
+      <c r="C38" t="s">
+        <v>465</v>
+      </c>
+      <c r="D38" t="s">
+        <v>623</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="F38" t="s">
+        <v>625</v>
+      </c>
+      <c r="G38" t="s">
+        <v>64</v>
+      </c>
+      <c r="H38" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="38" spans="1:9">
-      <c r="B38" s="29"/>
+    <row r="39" spans="1:9">
+      <c r="B39" s="29"/>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" s="40" t="s">
+        <v>669</v>
+      </c>
+      <c r="B42" s="41"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="40"/>
+      <c r="E42" s="42"/>
+      <c r="F42" s="40"/>
+      <c r="G42" s="40"/>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="41" t="s">
+        <v>670</v>
+      </c>
+      <c r="B43" s="40" t="s">
+        <v>466</v>
+      </c>
+      <c r="C43" s="40" t="s">
+        <v>667</v>
+      </c>
+      <c r="D43" s="42"/>
+      <c r="E43" s="40" t="s">
+        <v>668</v>
+      </c>
+      <c r="F43" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="G43" s="40" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" s="4" customFormat="1">
+      <c r="A44" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="B44" s="43"/>
+      <c r="E44" s="3"/>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" s="40" t="s">
+        <v>672</v>
+      </c>
+      <c r="B45" s="41"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="40"/>
+      <c r="E45" s="42"/>
+      <c r="F45" s="40"/>
+      <c r="G45" s="40"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
updated documentation regarding father_weekly_work and mother_weekly_work
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangk\Desktop\vaccination_uptake_jacsis2023\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A3E3069-EFCA-4065-9513-89A555A26DC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715EDCA9-7DC8-49E7-88B3-0C75CD25A558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3470" yWindow="690" windowWidth="14400" windowHeight="8710" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3470" yWindow="690" windowWidth="14400" windowHeight="8710" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -115,7 +115,7 @@
 I will figure it out and update once I find out which graph this is referring to</t>
       </text>
     </comment>
-    <comment ref="A44" authorId="1" shapeId="0" xr:uid="{596F102C-84BE-40F1-A512-14A8EBE941E9}">
+    <comment ref="A46" authorId="1" shapeId="0" xr:uid="{596F102C-84BE-40F1-A512-14A8EBE941E9}">
       <text>
         <r>
           <rPr>
@@ -141,7 +141,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A45" authorId="2" shapeId="0" xr:uid="{96A696B5-9B70-421D-BAE5-16DC63333B7B}">
+    <comment ref="A47" authorId="2" shapeId="0" xr:uid="{96A696B5-9B70-421D-BAE5-16DC63333B7B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2024" uniqueCount="673">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2034" uniqueCount="681">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -2084,12 +2084,6 @@
     <t>mother_work_weekly</t>
   </si>
   <si>
-    <t>The number of hours the COI's father spends at work per week</t>
-  </si>
-  <si>
-    <t>The number of hours the COI's mother spends at work per week</t>
-  </si>
-  <si>
     <t>use the median value of the time bin of the number of hours spent per week on childcare by the responding parent</t>
   </si>
   <si>
@@ -2178,6 +2172,36 @@
   </si>
   <si>
     <t>marital status and total no. of siblings</t>
+  </si>
+  <si>
+    <t>mother's working hours (and maybe fathers)</t>
+  </si>
+  <si>
+    <t>this needs to be plotted</t>
+  </si>
+  <si>
+    <t>mother_weekly_work * test_household_income</t>
+  </si>
+  <si>
+    <t>mother_weekly_work</t>
+  </si>
+  <si>
+    <t>father;s weekly working hours</t>
+  </si>
+  <si>
+    <t>needs to be plotted</t>
+  </si>
+  <si>
+    <t>father_weekly_work</t>
+  </si>
+  <si>
+    <t>father_weekly_work * test_household_income</t>
+  </si>
+  <si>
+    <t>The number of hours the COI's father spends at work per week (in the past month prior to submitting the survey)</t>
+  </si>
+  <si>
+    <t>The number of hours the COI's mother spends at work per week (in the past month prior to submitting the survey)</t>
   </si>
 </sst>
 </file>
@@ -2256,7 +2280,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2353,6 +2377,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -2381,7 +2411,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2448,6 +2478,8 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2804,7 +2836,7 @@
     <text>Should be age_cat and age_of_interest
 I will figure it out and update once I find out which graph this is referring to</text>
   </threadedComment>
-  <threadedComment ref="A45" dT="2025-12-10T07:47:28.93" personId="{F1230DF4-625E-4957-ABA0-003D3672236E}" id="{96A696B5-9B70-421D-BAE5-16DC63333B7B}">
+  <threadedComment ref="A47" dT="2025-12-10T07:47:28.93" personId="{F1230DF4-625E-4957-ABA0-003D3672236E}" id="{96A696B5-9B70-421D-BAE5-16DC63333B7B}">
     <text>Will be interesting to see if marital status (i..e single parents) are affected by the number of children they have to care for.</text>
   </threadedComment>
 </ThreadedComments>
@@ -3163,7 +3195,7 @@
         <v>640</v>
       </c>
       <c r="CX1" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="CY1" t="s">
         <v>56</v>
@@ -3751,28 +3783,28 @@
         <v>635</v>
       </c>
       <c r="CX3" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="CY3" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="CZ3" s="2" t="s">
         <v>653</v>
       </c>
-      <c r="CY3" s="2" t="s">
+      <c r="DA3" s="2" t="s">
         <v>654</v>
       </c>
-      <c r="CZ3" s="2" t="s">
+      <c r="DB3" s="2" t="s">
         <v>655</v>
       </c>
-      <c r="DA3" s="2" t="s">
+      <c r="DC3" s="2" t="s">
         <v>656</v>
       </c>
-      <c r="DB3" s="2" t="s">
+      <c r="DD3" s="2" t="s">
         <v>657</v>
       </c>
-      <c r="DC3" s="2" t="s">
+      <c r="DE3" s="2" t="s">
         <v>658</v>
-      </c>
-      <c r="DD3" s="2" t="s">
-        <v>659</v>
-      </c>
-      <c r="DE3" s="2" t="s">
-        <v>660</v>
       </c>
     </row>
     <row r="4" spans="1:110">
@@ -4080,28 +4112,28 @@
         <v>633</v>
       </c>
       <c r="CX4" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="CY4" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="CZ4" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="DA4" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="DB4" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="DC4" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="DD4" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="DE4" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
     </row>
     <row r="5" spans="1:110">
@@ -10550,10 +10582,10 @@
         <v>638</v>
       </c>
       <c r="F238" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="G238" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="H238" t="s">
         <v>307</v>
@@ -10573,19 +10605,19 @@
         <v>637</v>
       </c>
       <c r="E239" t="s">
-        <v>641</v>
+        <v>679</v>
       </c>
       <c r="F239" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="G239" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="H239" t="s">
         <v>307</v>
       </c>
       <c r="I239" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="J239" t="s">
         <v>307</v>
@@ -10617,19 +10649,19 @@
         <v>637</v>
       </c>
       <c r="E240" t="s">
-        <v>642</v>
+        <v>680</v>
       </c>
       <c r="F240" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="G240" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="H240" t="s">
         <v>307</v>
       </c>
       <c r="I240" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="J240" t="s">
         <v>307</v>
@@ -10652,19 +10684,19 @@
         <v>96</v>
       </c>
       <c r="B241" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="C241" t="s">
+        <v>660</v>
+      </c>
+      <c r="D241" s="39" t="s">
+        <v>661</v>
+      </c>
+      <c r="E241" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="F241" t="s">
         <v>662</v>
-      </c>
-      <c r="D241" s="39" t="s">
-        <v>663</v>
-      </c>
-      <c r="E241" s="2" t="s">
-        <v>653</v>
-      </c>
-      <c r="F241" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="242" spans="1:6">
@@ -10675,16 +10707,16 @@
         <v>56</v>
       </c>
       <c r="C242" t="s">
+        <v>660</v>
+      </c>
+      <c r="D242" s="39" t="s">
+        <v>661</v>
+      </c>
+      <c r="E242" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="F242" t="s">
         <v>662</v>
-      </c>
-      <c r="D242" s="39" t="s">
-        <v>663</v>
-      </c>
-      <c r="E242" s="2" t="s">
-        <v>654</v>
-      </c>
-      <c r="F242" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="243" spans="1:6">
@@ -10695,16 +10727,16 @@
         <v>55</v>
       </c>
       <c r="C243" t="s">
+        <v>660</v>
+      </c>
+      <c r="D243" s="39" t="s">
+        <v>661</v>
+      </c>
+      <c r="E243" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="F243" t="s">
         <v>662</v>
-      </c>
-      <c r="D243" s="39" t="s">
-        <v>663</v>
-      </c>
-      <c r="E243" s="2" t="s">
-        <v>655</v>
-      </c>
-      <c r="F243" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="244" spans="1:6">
@@ -10715,16 +10747,16 @@
         <v>54</v>
       </c>
       <c r="C244" t="s">
+        <v>660</v>
+      </c>
+      <c r="D244" s="39" t="s">
+        <v>661</v>
+      </c>
+      <c r="E244" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="F244" t="s">
         <v>662</v>
-      </c>
-      <c r="D244" s="39" t="s">
-        <v>663</v>
-      </c>
-      <c r="E244" s="2" t="s">
-        <v>656</v>
-      </c>
-      <c r="F244" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="245" spans="1:6">
@@ -10735,16 +10767,16 @@
         <v>53</v>
       </c>
       <c r="C245" t="s">
+        <v>660</v>
+      </c>
+      <c r="D245" s="39" t="s">
+        <v>661</v>
+      </c>
+      <c r="E245" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="F245" t="s">
         <v>662</v>
-      </c>
-      <c r="D245" s="39" t="s">
-        <v>663</v>
-      </c>
-      <c r="E245" s="2" t="s">
-        <v>657</v>
-      </c>
-      <c r="F245" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="246" spans="1:6">
@@ -10755,16 +10787,16 @@
         <v>52</v>
       </c>
       <c r="C246" t="s">
+        <v>660</v>
+      </c>
+      <c r="D246" s="39" t="s">
+        <v>661</v>
+      </c>
+      <c r="E246" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="F246" t="s">
         <v>662</v>
-      </c>
-      <c r="D246" s="39" t="s">
-        <v>663</v>
-      </c>
-      <c r="E246" s="2" t="s">
-        <v>658</v>
-      </c>
-      <c r="F246" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="247" spans="1:6">
@@ -10775,16 +10807,16 @@
         <v>51</v>
       </c>
       <c r="C247" t="s">
+        <v>660</v>
+      </c>
+      <c r="D247" s="39" t="s">
+        <v>661</v>
+      </c>
+      <c r="E247" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="F247" t="s">
         <v>662</v>
-      </c>
-      <c r="D247" s="39" t="s">
-        <v>663</v>
-      </c>
-      <c r="E247" s="2" t="s">
-        <v>659</v>
-      </c>
-      <c r="F247" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="248" spans="1:6">
@@ -10795,16 +10827,16 @@
         <v>50</v>
       </c>
       <c r="C248" t="s">
+        <v>660</v>
+      </c>
+      <c r="D248" s="39" t="s">
+        <v>661</v>
+      </c>
+      <c r="E248" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="F248" t="s">
         <v>662</v>
-      </c>
-      <c r="D248" s="39" t="s">
-        <v>663</v>
-      </c>
-      <c r="E248" s="2" t="s">
-        <v>660</v>
-      </c>
-      <c r="F248" t="s">
-        <v>664</v>
       </c>
     </row>
   </sheetData>
@@ -11367,7 +11399,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313888EE-552D-40AA-8234-3B847E46EF43}">
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="55.7265625" bestFit="1" customWidth="1"/>
@@ -11409,10 +11441,10 @@
     </row>
     <row r="2" spans="1:10" ht="61.5" customHeight="1">
       <c r="A2" s="22" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="C2" t="s">
         <v>169</v>
@@ -11519,7 +11551,7 @@
     </row>
     <row r="6" spans="1:10" s="32" customFormat="1" ht="29">
       <c r="A6" s="32" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="B6" s="33" t="s">
         <v>511</v>
@@ -11548,7 +11580,7 @@
     </row>
     <row r="7" spans="1:10" s="32" customFormat="1">
       <c r="A7" s="32" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="B7" s="33" t="s">
         <v>511</v>
@@ -11572,7 +11604,7 @@
     </row>
     <row r="8" spans="1:10" s="32" customFormat="1">
       <c r="A8" s="32" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="B8" s="33"/>
       <c r="D8" s="32" t="s">
@@ -11680,7 +11712,7 @@
     </row>
     <row r="14" spans="1:10" s="32" customFormat="1" ht="43.5">
       <c r="A14" s="34" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="B14" s="33" t="s">
         <v>510</v>
@@ -11868,7 +11900,7 @@
     </row>
     <row r="21" spans="1:10" s="35" customFormat="1" ht="29">
       <c r="A21" s="35" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B21" s="36" t="s">
         <v>510</v>
@@ -12342,7 +12374,7 @@
     </row>
     <row r="42" spans="1:9">
       <c r="A42" s="40" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="B42" s="41"/>
       <c r="C42" s="40"/>
@@ -12353,42 +12385,80 @@
     </row>
     <row r="43" spans="1:9">
       <c r="A43" s="41" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="B43" s="40" t="s">
         <v>466</v>
       </c>
-      <c r="C43" s="40" t="s">
-        <v>667</v>
+      <c r="C43" s="45" t="s">
+        <v>665</v>
       </c>
       <c r="D43" s="42"/>
-      <c r="E43" s="40" t="s">
-        <v>668</v>
-      </c>
       <c r="F43" s="40" t="s">
-        <v>80</v>
+        <v>666</v>
       </c>
       <c r="G43" s="40" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" s="4" customFormat="1">
-      <c r="A44" s="4" t="s">
+      <c r="H43" s="40" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" s="44" t="s">
+        <v>675</v>
+      </c>
+      <c r="B44" s="40"/>
+      <c r="C44" s="40" t="s">
+        <v>676</v>
+      </c>
+      <c r="D44" s="42"/>
+      <c r="F44" s="40" t="s">
+        <v>678</v>
+      </c>
+      <c r="G44" s="40" t="s">
+        <v>77</v>
+      </c>
+      <c r="H44" s="40" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" s="44" t="s">
         <v>671</v>
       </c>
-      <c r="B44" s="43"/>
-      <c r="E44" s="3"/>
-    </row>
-    <row r="45" spans="1:9">
-      <c r="A45" s="40" t="s">
+      <c r="B45" s="40"/>
+      <c r="C45" s="40" t="s">
         <v>672</v>
       </c>
-      <c r="B45" s="41"/>
-      <c r="C45" s="40"/>
-      <c r="D45" s="40"/>
-      <c r="E45" s="42"/>
-      <c r="F45" s="40"/>
-      <c r="G45" s="40"/>
+      <c r="D45" s="42"/>
+      <c r="F45" s="40" t="s">
+        <v>673</v>
+      </c>
+      <c r="G45" s="40" t="s">
+        <v>77</v>
+      </c>
+      <c r="H45" s="40" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" s="4" customFormat="1">
+      <c r="A46" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="B46" s="43"/>
+      <c r="E46" s="3"/>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" s="40" t="s">
+        <v>670</v>
+      </c>
+      <c r="B47" s="41"/>
+      <c r="C47" s="40"/>
+      <c r="D47" s="40"/>
+      <c r="E47" s="42"/>
+      <c r="F47" s="40"/>
+      <c r="G47" s="40"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix father_work_weekly and mother_work_weekly to depend on parent_1_sex and parent_2_sex, additionally allocated unemployed parents 0 work hours/week instead of NA and for the parents who are working (father/mother_employment_status != 0) to have the number of hours reported as worked by the spouse/respondent parent
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangk\Desktop\vaccination_uptake_jacsis2023\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715EDCA9-7DC8-49E7-88B3-0C75CD25A558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7CE101-A666-43E2-AF8A-C4635380440D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3470" yWindow="690" windowWidth="14400" windowHeight="8710" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1238,12 +1238,6 @@
     <t>where "chronic_illness" represents the 20 chronic illnesses asked about in the survey, we derive the responding parent's experience with chronic illnesses as: never (for never had for all 20 illnesses), previously had (if not currently having a chronic illness and previously had at least one chronic illness), currently having (when at least 1 chronic illness corresponds to currently have)</t>
   </si>
   <si>
-    <t>stratify the type of employment that the child's father, based on the respodnent's sex (parent_1_sex) or the partner's sex (parent_2_sex) which will be mapped to the respondent or partner's employment status</t>
-  </si>
-  <si>
-    <t>stratify the type of employment that the child's mother, based on the respodnent's sex (parent_1_sex) or the partner's sex (parent_2_sex) which will be mapped to the respondent or partner's employment status</t>
-  </si>
-  <si>
     <t>determine if the child's mother, father or both parents are students, based on the respodnent's sex (parent_1_sex) or the partner's sex (parent_2_sex) which will be mapped to the respondent or partner's employment status</t>
   </si>
   <si>
@@ -2090,18 +2084,12 @@
     <t>childcare_daily</t>
   </si>
   <si>
-    <t>take the approximate number of hours worked by the responding parent/spouse and determine which is the father respectively</t>
-  </si>
-  <si>
     <t>parent_work_weekly</t>
   </si>
   <si>
     <t>spouse_work_weekly</t>
   </si>
   <si>
-    <t>take the approximate number of hours worked by the responding parent/spouse and determine which is the mother respectively</t>
-  </si>
-  <si>
     <t>Retired test_mother/father_education</t>
   </si>
   <si>
@@ -2202,6 +2190,18 @@
   </si>
   <si>
     <t>The number of hours the COI's mother spends at work per week (in the past month prior to submitting the survey)</t>
+  </si>
+  <si>
+    <t>stratify the type of employment that the child's mother, based on the respodnent's sex (parent_1_sex) or the partner's sex (parent_2_sex) which will be mapped to the respondent or partner's employment status. If parent_2_sex is NA (ie responding parent is unmarried then if the father doesn't exist, their employment status is by default NA)</t>
+  </si>
+  <si>
+    <t>stratify the type of employment that the child's father, based on the respodnent's sex (parent_1_sex) or the partner's sex (parent_2_sex) which will be mapped to the respondent or partner's employment status. If parent_2_sex is NA, and parent_1_sex is female then there is no father in this family (i..e single mother family) and this value will be NA</t>
+  </si>
+  <si>
+    <t>take the approximate number of hours worked by the responding parent/spouse and determine which is the father respectively. Derived from parent_1_sex and parent_2_sex, which correspond to the sex of the responding parent and the spouse of the responding parent respectively, which are then matched to parent_work_weekly and spouse_work_weekly. NA is assigned when there is no father in the family (i..e single parent family) and 0 is assigned either when reported as 0 or when father is unemployed</t>
+  </si>
+  <si>
+    <t>take the approximate number of hours worked by the responding parent/spouse and determine which is the mother respectively. Derived from parent_1_sex and parent_2_sex, which correspond to the sex of the responding parent and the spouse of the responding parent respectively, which are then matched to parent_work_weekly and spouse_work_weekly. NA is assigned when there is no mother in the family (i..e single parent family) and 0 is assigned either when reported as 0 or when mother is unemployed</t>
   </si>
 </sst>
 </file>
@@ -2411,7 +2411,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2478,7 +2478,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2928,7 +2927,7 @@
         <v>15</v>
       </c>
       <c r="M1" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="N1" t="s">
         <v>17</v>
@@ -3078,7 +3077,7 @@
         <v>15</v>
       </c>
       <c r="BK1" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="BL1" s="20" t="s">
         <v>67</v>
@@ -3090,10 +3089,10 @@
         <v>69</v>
       </c>
       <c r="BO1" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="BP1" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="BQ1" s="4" t="s">
         <v>70</v>
@@ -3120,7 +3119,7 @@
         <v>77</v>
       </c>
       <c r="BY1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="BZ1" t="s">
         <v>78</v>
@@ -3153,10 +3152,10 @@
         <v>87</v>
       </c>
       <c r="CJ1" s="4" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="CK1" s="4" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="CL1" s="4" t="s">
         <v>88</v>
@@ -3165,7 +3164,7 @@
         <v>89</v>
       </c>
       <c r="CN1" s="4" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="CO1" t="s">
         <v>90</v>
@@ -3186,16 +3185,16 @@
         <v>95</v>
       </c>
       <c r="CU1" s="6" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="CV1" s="7" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="CW1" s="7" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="CX1" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="CY1" t="s">
         <v>56</v>
@@ -3419,10 +3418,10 @@
         <v>96</v>
       </c>
       <c r="BO2" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="BP2" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="BQ2" s="4" t="s">
         <v>96</v>
@@ -3589,7 +3588,7 @@
         <v>117</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="N3" s="2" t="s">
         <v>118</v>
@@ -3675,22 +3674,22 @@
         <v>117</v>
       </c>
       <c r="BK3" s="2" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="BL3" s="21" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="BM3" s="3" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="BN3" s="2" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="BO3" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="BP3" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="BQ3" s="3" t="s">
         <v>134</v>
@@ -3714,7 +3713,7 @@
         <v>140</v>
       </c>
       <c r="BY3" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="BZ3" s="2" t="s">
         <v>141</v>
@@ -3747,17 +3746,17 @@
         <v>150</v>
       </c>
       <c r="CJ3" s="3" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="CK3" s="3" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="CL3" s="3"/>
       <c r="CM3" s="2" t="s">
         <v>151</v>
       </c>
       <c r="CN3" s="3" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="CO3" s="2" t="s">
         <v>152</v>
@@ -3774,37 +3773,37 @@
       <c r="CS3" s="6"/>
       <c r="CT3" s="6"/>
       <c r="CU3" s="6" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="CV3" s="6" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="CW3" s="6" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="CX3" s="2" t="s">
+        <v>647</v>
+      </c>
+      <c r="CY3" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="CZ3" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="DA3" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="DB3" s="2" t="s">
         <v>651</v>
       </c>
-      <c r="CY3" s="2" t="s">
+      <c r="DC3" s="2" t="s">
         <v>652</v>
       </c>
-      <c r="CZ3" s="2" t="s">
+      <c r="DD3" s="2" t="s">
         <v>653</v>
       </c>
-      <c r="DA3" s="2" t="s">
+      <c r="DE3" s="2" t="s">
         <v>654</v>
-      </c>
-      <c r="DB3" s="2" t="s">
-        <v>655</v>
-      </c>
-      <c r="DC3" s="2" t="s">
-        <v>656</v>
-      </c>
-      <c r="DD3" s="2" t="s">
-        <v>657</v>
-      </c>
-      <c r="DE3" s="2" t="s">
-        <v>658</v>
       </c>
     </row>
     <row r="4" spans="1:110">
@@ -4034,10 +4033,10 @@
         <v>260</v>
       </c>
       <c r="BX4" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="BY4" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="BZ4" t="s">
         <v>99</v>
@@ -4103,37 +4102,37 @@
         <v>99</v>
       </c>
       <c r="CU4" s="6" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="CV4" s="7" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="CW4" s="7" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="CX4" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="CY4" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="CZ4" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="DA4" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="DB4" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="DC4" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="DD4" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="DE4" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
     </row>
     <row r="5" spans="1:110">
@@ -4252,7 +4251,7 @@
         <v>108</v>
       </c>
       <c r="BW7" s="4" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="CS7" s="7"/>
       <c r="CT7" s="7"/>
@@ -4721,7 +4720,7 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C14" t="s">
         <v>260</v>
@@ -4730,10 +4729,10 @@
         <v>109</v>
       </c>
       <c r="E14" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="F14" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="G14" t="s">
         <v>283</v>
@@ -4742,7 +4741,7 @@
         <v>275</v>
       </c>
       <c r="I14" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="J14" t="s">
         <v>307</v>
@@ -5477,7 +5476,7 @@
         <v>117</v>
       </c>
       <c r="F47" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="G47" t="s">
         <v>15</v>
@@ -5491,19 +5490,19 @@
         <v>96</v>
       </c>
       <c r="B48" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="C48" t="s">
         <v>261</v>
       </c>
       <c r="D48" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="E48" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="F48" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="G48" t="s">
         <v>15</v>
@@ -5523,13 +5522,13 @@
         <v>96</v>
       </c>
       <c r="D49" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="E49" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="F49" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -5537,13 +5536,13 @@
         <v>96</v>
       </c>
       <c r="D50" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="E50" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="F50" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -5557,7 +5556,7 @@
         <v>169</v>
       </c>
       <c r="F51" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="52" spans="1:12" s="4" customFormat="1">
@@ -5574,7 +5573,7 @@
         <v>109</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="F52" s="4" t="s">
         <v>318</v>
@@ -5606,7 +5605,7 @@
         <v>109</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>319</v>
@@ -5629,7 +5628,7 @@
         <v>96</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>260</v>
@@ -5638,10 +5637,10 @@
         <v>109</v>
       </c>
       <c r="E54" s="4" t="s">
+        <v>489</v>
+      </c>
+      <c r="F54" s="4" t="s">
         <v>491</v>
-      </c>
-      <c r="F54" s="4" t="s">
-        <v>493</v>
       </c>
       <c r="G54" s="4" t="s">
         <v>68</v>
@@ -5656,7 +5655,7 @@
         <v>307</v>
       </c>
       <c r="K54" s="4" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="L54" s="4" t="s">
         <v>307</v>
@@ -5676,10 +5675,10 @@
         <v>109</v>
       </c>
       <c r="E55" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="F55" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="G55" t="s">
         <v>68</v>
@@ -5699,7 +5698,7 @@
         <v>96</v>
       </c>
       <c r="B56" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="C56" t="s">
         <v>260</v>
@@ -5708,13 +5707,13 @@
         <v>109</v>
       </c>
       <c r="E56" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="F56" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="G56" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="H56" t="s">
         <v>307</v>
@@ -6162,7 +6161,7 @@
         <v>181</v>
       </c>
       <c r="F86" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="G86" t="s">
         <v>321</v>
@@ -6180,7 +6179,7 @@
         <v>2</v>
       </c>
       <c r="E87" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -6192,7 +6191,7 @@
         <v>3</v>
       </c>
       <c r="E88" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -6204,7 +6203,7 @@
         <v>4</v>
       </c>
       <c r="E89" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="90" spans="1:8">
@@ -6216,7 +6215,7 @@
         <v>5</v>
       </c>
       <c r="E90" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="91" spans="1:8">
@@ -6228,7 +6227,7 @@
         <v>6</v>
       </c>
       <c r="E91" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -6240,7 +6239,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -6252,7 +6251,7 @@
         <v>8</v>
       </c>
       <c r="E93" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -6264,7 +6263,7 @@
         <v>9</v>
       </c>
       <c r="E94" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -6276,7 +6275,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="96" spans="1:8">
@@ -6288,7 +6287,7 @@
         <v>11</v>
       </c>
       <c r="E96" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="97" spans="1:8">
@@ -6300,7 +6299,7 @@
         <v>12</v>
       </c>
       <c r="E97" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="98" spans="1:8">
@@ -6312,7 +6311,7 @@
         <v>13</v>
       </c>
       <c r="E98" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="99" spans="1:8">
@@ -6324,7 +6323,7 @@
         <v>14</v>
       </c>
       <c r="E99" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="100" spans="1:8">
@@ -6336,7 +6335,7 @@
         <v>15</v>
       </c>
       <c r="E100" s="19" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="101" spans="1:8">
@@ -6348,7 +6347,7 @@
         <v>16</v>
       </c>
       <c r="E101" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="102" spans="1:8">
@@ -6360,7 +6359,7 @@
         <v>17</v>
       </c>
       <c r="E102" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="103" spans="1:8">
@@ -6391,7 +6390,7 @@
         <v>96</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="C105" s="4" t="s">
         <v>260</v>
@@ -6403,10 +6402,10 @@
         <v>181</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="G105" s="4" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="H105" s="4" t="s">
         <v>307</v>
@@ -6421,7 +6420,7 @@
         <v>2</v>
       </c>
       <c r="E106" s="4" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="107" spans="1:8" s="4" customFormat="1">
@@ -6433,7 +6432,7 @@
         <v>3</v>
       </c>
       <c r="E107" s="4" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="108" spans="1:8" s="4" customFormat="1">
@@ -6445,7 +6444,7 @@
         <v>4</v>
       </c>
       <c r="E108" s="4" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="109" spans="1:8" s="4" customFormat="1">
@@ -6457,7 +6456,7 @@
         <v>5</v>
       </c>
       <c r="E109" s="4" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="110" spans="1:8" s="4" customFormat="1">
@@ -6469,7 +6468,7 @@
         <v>6</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="111" spans="1:8" s="4" customFormat="1">
@@ -6481,7 +6480,7 @@
         <v>7</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="112" spans="1:8" s="4" customFormat="1">
@@ -6493,7 +6492,7 @@
         <v>8</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="113" spans="1:8" s="4" customFormat="1">
@@ -6505,7 +6504,7 @@
         <v>9</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="114" spans="1:8" s="4" customFormat="1">
@@ -6517,7 +6516,7 @@
         <v>10</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="115" spans="1:8" s="4" customFormat="1">
@@ -6529,7 +6528,7 @@
         <v>11</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="116" spans="1:8" s="4" customFormat="1">
@@ -6541,7 +6540,7 @@
         <v>12</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="117" spans="1:8" s="4" customFormat="1">
@@ -6553,7 +6552,7 @@
         <v>13</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="118" spans="1:8" s="4" customFormat="1">
@@ -6565,7 +6564,7 @@
         <v>14</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="119" spans="1:8" s="4" customFormat="1">
@@ -6577,7 +6576,7 @@
         <v>15</v>
       </c>
       <c r="E119" s="38" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="120" spans="1:8" s="4" customFormat="1">
@@ -6589,7 +6588,7 @@
         <v>16</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="121" spans="1:8" s="4" customFormat="1">
@@ -6601,7 +6600,7 @@
         <v>17</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="122" spans="1:8" s="4" customFormat="1">
@@ -6632,7 +6631,7 @@
         <v>96</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="C124" s="4" t="s">
         <v>260</v>
@@ -6644,10 +6643,10 @@
         <v>181</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="G124" s="4" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="H124" s="4" t="s">
         <v>307</v>
@@ -6662,7 +6661,7 @@
         <v>2</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="126" spans="1:8" s="4" customFormat="1">
@@ -6674,7 +6673,7 @@
         <v>3</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="127" spans="1:8" s="4" customFormat="1">
@@ -6686,7 +6685,7 @@
         <v>4</v>
       </c>
       <c r="E127" s="4" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="128" spans="1:8" s="4" customFormat="1">
@@ -6698,7 +6697,7 @@
         <v>5</v>
       </c>
       <c r="E128" s="4" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="129" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
@@ -6710,7 +6709,7 @@
         <v>6</v>
       </c>
       <c r="E129" s="4" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="130" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
@@ -6722,7 +6721,7 @@
         <v>7</v>
       </c>
       <c r="E130" s="4" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="131" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
@@ -6734,7 +6733,7 @@
         <v>8</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="132" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
@@ -6746,7 +6745,7 @@
         <v>9</v>
       </c>
       <c r="E132" s="4" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="133" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
@@ -6758,7 +6757,7 @@
         <v>10</v>
       </c>
       <c r="E133" s="4" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="134" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
@@ -6770,7 +6769,7 @@
         <v>11</v>
       </c>
       <c r="E134" s="4" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="135" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
@@ -6782,7 +6781,7 @@
         <v>12</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="136" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
@@ -6794,7 +6793,7 @@
         <v>13</v>
       </c>
       <c r="E136" s="4" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="137" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
@@ -6806,7 +6805,7 @@
         <v>14</v>
       </c>
       <c r="E137" s="4" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="138" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
@@ -6818,7 +6817,7 @@
         <v>15</v>
       </c>
       <c r="E138" s="38" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="M138" s="38"/>
       <c r="U138" s="38"/>
@@ -8877,7 +8876,7 @@
         <v>16</v>
       </c>
       <c r="E139" s="4" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="140" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
@@ -8889,7 +8888,7 @@
         <v>17</v>
       </c>
       <c r="E140" s="4" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="141" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
@@ -8994,7 +8993,7 @@
         <v>201</v>
       </c>
       <c r="F147" t="s">
-        <v>359</v>
+        <v>678</v>
       </c>
       <c r="G147" t="s">
         <v>66</v>
@@ -9088,7 +9087,7 @@
         <v>201</v>
       </c>
       <c r="F152" t="s">
-        <v>360</v>
+        <v>677</v>
       </c>
       <c r="G152" t="s">
         <v>66</v>
@@ -9196,7 +9195,7 @@
         <v>217</v>
       </c>
       <c r="F157" s="4" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="G157" s="4" t="s">
         <v>66</v>
@@ -9290,7 +9289,7 @@
         <v>211</v>
       </c>
       <c r="F162" s="4" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="G162" s="4" t="s">
         <v>66</v>
@@ -9384,7 +9383,7 @@
         <v>216</v>
       </c>
       <c r="F167" s="4" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="G167" s="4" t="s">
         <v>66</v>
@@ -9478,7 +9477,7 @@
         <v>221</v>
       </c>
       <c r="F172" s="4" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="G172" s="4" t="s">
         <v>66</v>
@@ -9550,7 +9549,7 @@
         <v>225</v>
       </c>
       <c r="F175" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="G175" t="s">
         <v>66</v>
@@ -9630,10 +9629,10 @@
         <v>0</v>
       </c>
       <c r="E179" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="F179" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G179" t="s">
         <v>66</v>
@@ -9674,7 +9673,7 @@
         <v>1</v>
       </c>
       <c r="E180" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="181" spans="1:16">
@@ -9724,10 +9723,10 @@
         <v>0</v>
       </c>
       <c r="E184" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="F184" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="G184" t="s">
         <v>66</v>
@@ -9768,7 +9767,7 @@
         <v>1</v>
       </c>
       <c r="E185" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="186" spans="1:16">
@@ -9818,10 +9817,10 @@
         <v>0</v>
       </c>
       <c r="E189" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="F189" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="G189" t="s">
         <v>66</v>
@@ -9850,7 +9849,7 @@
         <v>1</v>
       </c>
       <c r="E190" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="191" spans="1:16">
@@ -9903,7 +9902,7 @@
         <v>235</v>
       </c>
       <c r="F194" s="4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="G194" s="4" t="s">
         <v>66</v>
@@ -9957,7 +9956,7 @@
         <v>233</v>
       </c>
       <c r="F197" s="4" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="G197" s="4" t="s">
         <v>66</v>
@@ -10077,7 +10076,7 @@
         <v>245</v>
       </c>
       <c r="F206" s="4" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="G206" s="4" t="s">
         <v>66</v>
@@ -10175,7 +10174,7 @@
         <v>251</v>
       </c>
       <c r="F213" s="4" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="G213" s="4" t="s">
         <v>66</v>
@@ -10215,7 +10214,7 @@
         <v>2</v>
       </c>
       <c r="E215" s="4" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="216" spans="1:16" s="4" customFormat="1">
@@ -10234,7 +10233,7 @@
         <v>96</v>
       </c>
       <c r="B217" s="4" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C217" s="4" t="s">
         <v>261</v>
@@ -10243,10 +10242,10 @@
         <v>0</v>
       </c>
       <c r="E217" s="4" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="F217" s="4" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="G217" s="4" t="s">
         <v>66</v>
@@ -10287,7 +10286,7 @@
         <v>1</v>
       </c>
       <c r="E218" s="4" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="219" spans="1:16" s="4" customFormat="1">
@@ -10298,7 +10297,7 @@
         <v>1.5</v>
       </c>
       <c r="E219" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
     </row>
     <row r="220" spans="1:16" s="4" customFormat="1">
@@ -10309,7 +10308,7 @@
         <v>2</v>
       </c>
       <c r="E220" s="4" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="221" spans="1:16" s="4" customFormat="1">
@@ -10350,7 +10349,7 @@
         <v>96</v>
       </c>
       <c r="B224" s="4" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="C224" s="4" t="s">
         <v>261</v>
@@ -10359,10 +10358,10 @@
         <v>0</v>
       </c>
       <c r="E224" s="4" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="F224" s="4" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="G224" s="4" t="s">
         <v>66</v>
@@ -10403,7 +10402,7 @@
         <v>1</v>
       </c>
       <c r="E225" s="4" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="226" spans="1:14" s="4" customFormat="1">
@@ -10414,7 +10413,7 @@
         <v>1.5</v>
       </c>
       <c r="E226" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
     </row>
     <row r="227" spans="1:14" s="4" customFormat="1">
@@ -10425,7 +10424,7 @@
         <v>2</v>
       </c>
       <c r="E227" s="4" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="228" spans="1:14" s="4" customFormat="1">
@@ -10466,7 +10465,7 @@
         <v>96</v>
       </c>
       <c r="B231" s="4" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C231" s="4" t="s">
         <v>261</v>
@@ -10475,10 +10474,10 @@
         <v>0</v>
       </c>
       <c r="E231" s="4" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="F231" s="4" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="G231" s="4" t="s">
         <v>66</v>
@@ -10487,13 +10486,13 @@
         <v>327</v>
       </c>
       <c r="I231" s="4" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="J231" s="4" t="s">
         <v>307</v>
       </c>
       <c r="K231" s="4" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="L231" s="4" t="s">
         <v>307</v>
@@ -10507,7 +10506,7 @@
         <v>1</v>
       </c>
       <c r="E232" s="4" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="233" spans="1:14" s="4" customFormat="1">
@@ -10518,7 +10517,7 @@
         <v>1.5</v>
       </c>
       <c r="E233" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
     </row>
     <row r="234" spans="1:14" s="4" customFormat="1">
@@ -10529,7 +10528,7 @@
         <v>2</v>
       </c>
       <c r="E234" s="4" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="235" spans="1:14" s="4" customFormat="1">
@@ -10570,22 +10569,22 @@
         <v>96</v>
       </c>
       <c r="B238" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="C238" t="s">
         <v>260</v>
       </c>
       <c r="D238" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="E238" s="31" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="F238" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="G238" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="H238" t="s">
         <v>307</v>
@@ -10596,28 +10595,28 @@
         <v>96</v>
       </c>
       <c r="B239" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="C239" t="s">
         <v>260</v>
       </c>
       <c r="D239" s="31" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="E239" t="s">
+        <v>675</v>
+      </c>
+      <c r="F239" t="s">
         <v>679</v>
       </c>
-      <c r="F239" t="s">
-        <v>643</v>
-      </c>
       <c r="G239" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="H239" t="s">
         <v>307</v>
       </c>
       <c r="I239" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="J239" t="s">
         <v>307</v>
@@ -10640,28 +10639,28 @@
         <v>96</v>
       </c>
       <c r="B240" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="C240" t="s">
         <v>260</v>
       </c>
       <c r="D240" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="E240" t="s">
+        <v>676</v>
+      </c>
+      <c r="F240" t="s">
         <v>680</v>
       </c>
-      <c r="F240" t="s">
-        <v>646</v>
-      </c>
       <c r="G240" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="H240" t="s">
         <v>307</v>
       </c>
       <c r="I240" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="J240" t="s">
         <v>307</v>
@@ -10684,19 +10683,19 @@
         <v>96</v>
       </c>
       <c r="B241" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C241" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="D241" s="39" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="E241" s="2" t="s">
-        <v>651</v>
+        <v>647</v>
       </c>
       <c r="F241" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
     </row>
     <row r="242" spans="1:6">
@@ -10707,16 +10706,16 @@
         <v>56</v>
       </c>
       <c r="C242" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="D242" s="39" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="E242" s="2" t="s">
-        <v>652</v>
+        <v>648</v>
       </c>
       <c r="F242" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
     </row>
     <row r="243" spans="1:6">
@@ -10727,16 +10726,16 @@
         <v>55</v>
       </c>
       <c r="C243" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="D243" s="39" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="E243" s="2" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="F243" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
     </row>
     <row r="244" spans="1:6">
@@ -10747,16 +10746,16 @@
         <v>54</v>
       </c>
       <c r="C244" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="D244" s="39" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="E244" s="2" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="F244" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
     </row>
     <row r="245" spans="1:6">
@@ -10767,16 +10766,16 @@
         <v>53</v>
       </c>
       <c r="C245" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="D245" s="39" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="E245" s="2" t="s">
-        <v>655</v>
+        <v>651</v>
       </c>
       <c r="F245" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
     </row>
     <row r="246" spans="1:6">
@@ -10787,16 +10786,16 @@
         <v>52</v>
       </c>
       <c r="C246" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="D246" s="39" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="E246" s="2" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="F246" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
     </row>
     <row r="247" spans="1:6">
@@ -10807,16 +10806,16 @@
         <v>51</v>
       </c>
       <c r="C247" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="D247" s="39" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="E247" s="2" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="F247" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
     </row>
     <row r="248" spans="1:6">
@@ -10827,16 +10826,16 @@
         <v>50</v>
       </c>
       <c r="C248" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="D248" s="39" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="E248" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="F248" t="s">
         <v>658</v>
-      </c>
-      <c r="F248" t="s">
-        <v>662</v>
       </c>
     </row>
   </sheetData>
@@ -10876,7 +10875,7 @@
   <sheetData>
     <row r="1" spans="1:42" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A1" s="17" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>5</v>
@@ -10912,7 +10911,7 @@
         <v>15</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="N1" s="2" t="s">
         <v>60</v>
@@ -10933,16 +10932,16 @@
         <v>66</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="V1" s="2" t="s">
         <v>69</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="X1" s="2" t="s">
         <v>71</v>
@@ -10993,13 +10992,13 @@
         <v>93</v>
       </c>
       <c r="AN1" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="AO1" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="AP1" s="18" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="2" spans="1:42">
@@ -11059,12 +11058,12 @@
       <c r="T12" s="22"/>
       <c r="AO12" s="15"/>
       <c r="AP12" s="10" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="13" spans="1:42">
       <c r="A13" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="L13" s="22"/>
       <c r="AO13" s="15"/>
@@ -11075,7 +11074,7 @@
       </c>
       <c r="Q14" s="22"/>
       <c r="AB14" s="22" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="AE14" s="15"/>
       <c r="AO14" s="15"/>
@@ -11117,14 +11116,14 @@
     </row>
     <row r="21" spans="1:41">
       <c r="A21" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="L21" s="22"/>
       <c r="AN21" s="15"/>
     </row>
     <row r="22" spans="1:41">
       <c r="A22" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="L22" s="22"/>
       <c r="M22" s="22"/>
@@ -11141,7 +11140,7 @@
     </row>
     <row r="24" spans="1:41">
       <c r="A24" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="M24" s="15"/>
       <c r="P24" s="15"/>
@@ -11154,16 +11153,16 @@
         <v>71</v>
       </c>
       <c r="N25" s="22" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="P25" s="22" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="AB25" s="14" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="AC25" s="15" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="AN25" s="15"/>
     </row>
@@ -11189,11 +11188,11 @@
         <v>77</v>
       </c>
       <c r="Q29" s="22" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="U29" s="15"/>
       <c r="V29" s="15" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="W29" s="15"/>
       <c r="AN29" s="15"/>
@@ -11205,11 +11204,11 @@
       </c>
       <c r="X30" s="15"/>
       <c r="AJ30" s="15" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="AK30" s="15"/>
       <c r="AL30" s="15" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="AO30" s="15"/>
     </row>
@@ -11226,7 +11225,7 @@
       </c>
       <c r="Q32" s="22"/>
       <c r="AB32" s="23" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="33" spans="1:41">
@@ -11234,16 +11233,16 @@
         <v>85</v>
       </c>
       <c r="AJ33" s="15" t="s">
+        <v>420</v>
+      </c>
+      <c r="AK33" s="15" t="s">
+        <v>421</v>
+      </c>
+      <c r="AL33" s="15" t="s">
         <v>422</v>
       </c>
-      <c r="AK33" s="15" t="s">
-        <v>423</v>
-      </c>
-      <c r="AL33" s="15" t="s">
-        <v>424</v>
-      </c>
       <c r="AM33" s="15" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="34" spans="1:41">
@@ -11254,7 +11253,7 @@
       <c r="V34" s="15"/>
       <c r="W34" s="15"/>
       <c r="AB34" s="22" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="AD34" s="15"/>
       <c r="AI34" s="15"/>
@@ -11268,7 +11267,7 @@
       <c r="V35" s="15"/>
       <c r="W35" s="15"/>
       <c r="AB35" s="22" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="AE35" s="15"/>
       <c r="AI35" s="15"/>
@@ -11279,15 +11278,15 @@
         <v>89</v>
       </c>
       <c r="P36" s="22" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="U36" s="15"/>
       <c r="V36" s="15" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="W36" s="15"/>
       <c r="AB36" s="22" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="37" spans="1:41">
@@ -11313,67 +11312,67 @@
         <v>93</v>
       </c>
       <c r="AJ40" s="15" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="AO40" s="15"/>
     </row>
     <row r="41" spans="1:41">
       <c r="A41" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="42" spans="1:41">
       <c r="A42" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="44" spans="1:41" s="10" customFormat="1">
       <c r="A44" s="10" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
     </row>
     <row r="46" spans="1:41">
       <c r="B46" s="11" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="47" spans="1:41">
       <c r="A47" s="11"/>
       <c r="B47" s="12"/>
       <c r="C47" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="48" spans="1:41">
       <c r="B48" s="13"/>
       <c r="C48" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="49" spans="2:3">
       <c r="B49" s="14"/>
       <c r="C49" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="50" spans="2:3">
       <c r="B50" s="15"/>
       <c r="C50" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="51" spans="2:3">
       <c r="B51" s="1" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C51" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="52" spans="2:3">
       <c r="B52" s="22"/>
       <c r="C52" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
   </sheetData>
@@ -11415,45 +11414,45 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>456</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>448</v>
+      </c>
+      <c r="C1" t="s">
+        <v>461</v>
+      </c>
+      <c r="D1" t="s">
+        <v>450</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="F1" t="s">
+        <v>473</v>
+      </c>
+      <c r="G1" t="s">
+        <v>449</v>
+      </c>
+      <c r="H1" t="s">
         <v>458</v>
-      </c>
-      <c r="B1" s="24" t="s">
-        <v>450</v>
-      </c>
-      <c r="C1" t="s">
-        <v>463</v>
-      </c>
-      <c r="D1" t="s">
-        <v>452</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="F1" t="s">
-        <v>475</v>
-      </c>
-      <c r="G1" t="s">
-        <v>451</v>
-      </c>
-      <c r="H1" t="s">
-        <v>460</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="61.5" customHeight="1">
       <c r="A2" s="22" t="s">
-        <v>664</v>
+        <v>660</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="C2" t="s">
         <v>169</v>
       </c>
       <c r="D2" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F2" t="s">
         <v>169</v>
@@ -11467,25 +11466,25 @@
     </row>
     <row r="3" spans="1:10" ht="58">
       <c r="A3" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="B3" s="27" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C3" t="s">
+        <v>464</v>
+      </c>
+      <c r="D3" t="s">
+        <v>451</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="F3" t="s">
+        <v>474</v>
+      </c>
+      <c r="G3" t="s">
         <v>466</v>
-      </c>
-      <c r="D3" t="s">
-        <v>453</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>481</v>
-      </c>
-      <c r="F3" t="s">
-        <v>476</v>
-      </c>
-      <c r="G3" t="s">
-        <v>468</v>
       </c>
       <c r="H3" t="s">
         <v>77</v>
@@ -11499,25 +11498,25 @@
     </row>
     <row r="4" spans="1:10" ht="43.5">
       <c r="A4" s="22" t="s">
+        <v>611</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>509</v>
+      </c>
+      <c r="C4" t="s">
+        <v>462</v>
+      </c>
+      <c r="D4" t="s">
         <v>613</v>
       </c>
-      <c r="B4" s="26" t="s">
-        <v>511</v>
-      </c>
-      <c r="C4" t="s">
-        <v>464</v>
-      </c>
-      <c r="D4" t="s">
-        <v>615</v>
-      </c>
       <c r="E4" s="2" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="F4" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="G4" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="H4" t="s">
         <v>77</v>
@@ -11525,25 +11524,25 @@
     </row>
     <row r="5" spans="1:10" ht="43.5">
       <c r="A5" s="22" t="s">
+        <v>611</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>509</v>
+      </c>
+      <c r="C5" t="s">
+        <v>462</v>
+      </c>
+      <c r="D5" t="s">
         <v>613</v>
       </c>
-      <c r="B5" s="26" t="s">
-        <v>511</v>
-      </c>
-      <c r="C5" t="s">
-        <v>464</v>
-      </c>
-      <c r="D5" t="s">
-        <v>615</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="F5" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="G5" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="H5" t="s">
         <v>77</v>
@@ -11551,28 +11550,28 @@
     </row>
     <row r="6" spans="1:10" s="32" customFormat="1" ht="29">
       <c r="A6" s="32" t="s">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="C6" s="32" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="D6" s="32" t="s">
+        <v>588</v>
+      </c>
+      <c r="E6" s="34" t="s">
+        <v>589</v>
+      </c>
+      <c r="F6" s="32" t="s">
         <v>590</v>
       </c>
-      <c r="E6" s="34" t="s">
-        <v>591</v>
-      </c>
-      <c r="F6" s="32" t="s">
+      <c r="G6" s="32" t="s">
         <v>592</v>
       </c>
-      <c r="G6" s="32" t="s">
-        <v>594</v>
-      </c>
       <c r="H6" s="32" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="I6" s="32" t="s">
         <v>77</v>
@@ -11580,20 +11579,20 @@
     </row>
     <row r="7" spans="1:10" s="32" customFormat="1">
       <c r="A7" s="32" t="s">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="E7" s="34"/>
       <c r="F7" s="32" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="G7" s="32" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="H7" s="32" t="s">
         <v>87</v>
@@ -11604,18 +11603,18 @@
     </row>
     <row r="8" spans="1:10" s="32" customFormat="1">
       <c r="A8" s="32" t="s">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="B8" s="33"/>
       <c r="D8" s="32" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="E8" s="34"/>
       <c r="G8" s="32" t="s">
         <v>86</v>
       </c>
       <c r="H8" s="32" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="I8" s="32" t="s">
         <v>77</v>
@@ -11623,22 +11622,22 @@
     </row>
     <row r="9" spans="1:10" ht="43.5">
       <c r="B9" s="30" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C9" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D9" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="F9" t="s">
+        <v>515</v>
+      </c>
+      <c r="G9" t="s">
         <v>516</v>
-      </c>
-      <c r="F9" t="s">
-        <v>517</v>
-      </c>
-      <c r="G9" t="s">
-        <v>518</v>
       </c>
       <c r="H9" t="s">
         <v>77</v>
@@ -11646,39 +11645,39 @@
     </row>
     <row r="10" spans="1:10" ht="43.5">
       <c r="B10" s="30" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="C10" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D10" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="E10" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="F10" t="s">
+        <v>512</v>
+      </c>
+      <c r="G10" t="s">
         <v>513</v>
-      </c>
-      <c r="F10" t="s">
-        <v>514</v>
-      </c>
-      <c r="G10" t="s">
-        <v>515</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="43.5">
       <c r="B11" s="25" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C11" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D11" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="F11" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="G11" t="s">
         <v>89</v>
@@ -11689,19 +11688,19 @@
     </row>
     <row r="13" spans="1:10" ht="29">
       <c r="B13" s="28" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C13" t="s">
+        <v>463</v>
+      </c>
+      <c r="D13" t="s">
         <v>465</v>
       </c>
-      <c r="D13" t="s">
-        <v>467</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="F13" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="G13" t="s">
         <v>84</v>
@@ -11712,22 +11711,22 @@
     </row>
     <row r="14" spans="1:10" s="32" customFormat="1" ht="43.5">
       <c r="A14" s="34" t="s">
-        <v>648</v>
+        <v>644</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C14" s="32" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="F14" s="32" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="G14" s="32" t="s">
         <v>80</v>
@@ -11741,16 +11740,16 @@
     </row>
     <row r="15" spans="1:10" ht="43.5">
       <c r="B15" s="27" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C15" t="s">
         <v>169</v>
       </c>
       <c r="D15" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="F15" t="s">
         <v>169</v>
@@ -11767,80 +11766,80 @@
     </row>
     <row r="16" spans="1:10" ht="58">
       <c r="A16" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C16" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D16" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="F16" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="G16" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H16" t="s">
         <v>15</v>
       </c>
       <c r="I16" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="43.5">
       <c r="A17" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C17" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D17" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="F17" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="G17" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="H17" t="s">
         <v>15</v>
       </c>
       <c r="I17" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="B18" s="29" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C18" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D18" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="F18" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="G18" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="H18" t="s">
         <v>15</v>
@@ -11848,22 +11847,22 @@
     </row>
     <row r="19" spans="1:10" ht="58">
       <c r="A19" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="B19" s="28" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C19" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D19" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="F19" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="G19" t="s">
         <v>71</v>
@@ -11874,25 +11873,25 @@
     </row>
     <row r="20" spans="1:10" ht="43.5">
       <c r="A20" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="B20" s="28" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C20" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D20" t="s">
+        <v>526</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="F20" t="s">
+        <v>527</v>
+      </c>
+      <c r="G20" t="s">
         <v>528</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>531</v>
-      </c>
-      <c r="F20" t="s">
-        <v>529</v>
-      </c>
-      <c r="G20" t="s">
-        <v>530</v>
       </c>
       <c r="H20" t="s">
         <v>64</v>
@@ -11900,25 +11899,25 @@
     </row>
     <row r="21" spans="1:10" s="35" customFormat="1" ht="29">
       <c r="A21" s="35" t="s">
-        <v>649</v>
+        <v>645</v>
       </c>
       <c r="B21" s="36" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C21" s="35" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D21" s="35" t="s">
+        <v>531</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>532</v>
+      </c>
+      <c r="F21" s="35" t="s">
         <v>533</v>
       </c>
-      <c r="E21" s="37" t="s">
-        <v>534</v>
-      </c>
-      <c r="F21" s="35" t="s">
-        <v>535</v>
-      </c>
       <c r="G21" s="35" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="H21" s="35" t="s">
         <v>77</v>
@@ -11926,25 +11925,25 @@
     </row>
     <row r="22" spans="1:10" ht="43.5">
       <c r="A22" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C22" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D22" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="E22" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="F22" t="s">
         <v>537</v>
       </c>
-      <c r="F22" t="s">
-        <v>539</v>
-      </c>
       <c r="G22" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="H22" t="s">
         <v>78</v>
@@ -11952,25 +11951,25 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="B23" s="28" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="C23" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D23" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="F23" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="G23" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="H23" t="s">
         <v>64</v>
@@ -11984,28 +11983,28 @@
     </row>
     <row r="24" spans="1:10" ht="72.5">
       <c r="A24" t="s">
+        <v>547</v>
+      </c>
+      <c r="B24" s="28" t="s">
+        <v>574</v>
+      </c>
+      <c r="C24" t="s">
+        <v>464</v>
+      </c>
+      <c r="D24" t="s">
         <v>549</v>
       </c>
-      <c r="B24" s="28" t="s">
-        <v>576</v>
-      </c>
-      <c r="C24" t="s">
-        <v>466</v>
-      </c>
-      <c r="D24" t="s">
-        <v>551</v>
-      </c>
       <c r="E24" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="F24" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="G24" t="s">
         <v>63</v>
       </c>
       <c r="H24" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="I24" t="s">
         <v>89</v>
@@ -12013,22 +12012,22 @@
     </row>
     <row r="25" spans="1:10" ht="87">
       <c r="A25" t="s">
+        <v>550</v>
+      </c>
+      <c r="B25" s="28" t="s">
+        <v>574</v>
+      </c>
+      <c r="C25" t="s">
+        <v>464</v>
+      </c>
+      <c r="D25" t="s">
+        <v>551</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="F25" t="s">
         <v>552</v>
-      </c>
-      <c r="B25" s="28" t="s">
-        <v>576</v>
-      </c>
-      <c r="C25" t="s">
-        <v>466</v>
-      </c>
-      <c r="D25" t="s">
-        <v>553</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>555</v>
-      </c>
-      <c r="F25" t="s">
-        <v>554</v>
       </c>
       <c r="G25" t="s">
         <v>63</v>
@@ -12042,19 +12041,19 @@
     </row>
     <row r="26" spans="1:10" ht="43.5">
       <c r="B26" s="28" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C26" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D26" t="s">
+        <v>542</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="F26" t="s">
         <v>544</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>545</v>
-      </c>
-      <c r="F26" t="s">
-        <v>546</v>
       </c>
       <c r="G26" t="s">
         <v>63</v>
@@ -12065,19 +12064,19 @@
     </row>
     <row r="27" spans="1:10" ht="43.5">
       <c r="B27" s="28" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C27" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="D27" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="F27" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="G27" t="s">
         <v>63</v>
@@ -12088,22 +12087,22 @@
     </row>
     <row r="28" spans="1:10" ht="58">
       <c r="A28" t="s">
+        <v>557</v>
+      </c>
+      <c r="B28" s="28" t="s">
+        <v>574</v>
+      </c>
+      <c r="C28" t="s">
+        <v>464</v>
+      </c>
+      <c r="D28" t="s">
+        <v>558</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>559</v>
       </c>
-      <c r="B28" s="28" t="s">
-        <v>576</v>
-      </c>
-      <c r="C28" t="s">
-        <v>466</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="F28" t="s">
         <v>560</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>561</v>
-      </c>
-      <c r="F28" t="s">
-        <v>562</v>
       </c>
       <c r="G28" t="s">
         <v>63</v>
@@ -12117,22 +12116,22 @@
     </row>
     <row r="29" spans="1:10" ht="58">
       <c r="A29" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B29" s="29" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C29" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D29" t="s">
+        <v>562</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="F29" t="s">
         <v>564</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>565</v>
-      </c>
-      <c r="F29" t="s">
-        <v>566</v>
       </c>
       <c r="G29" t="s">
         <v>63</v>
@@ -12143,45 +12142,45 @@
     </row>
     <row r="30" spans="1:10" ht="116">
       <c r="A30" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="B30" s="28" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C30" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="D30" t="s">
+        <v>566</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="F30" t="s">
         <v>568</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="F30" t="s">
-        <v>570</v>
       </c>
       <c r="G30" t="s">
         <v>63</v>
       </c>
       <c r="H30" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="58">
       <c r="B31" s="29" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C31" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D31" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="F31" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="G31" t="s">
         <v>64</v>
@@ -12192,19 +12191,19 @@
     </row>
     <row r="32" spans="1:10" ht="72.5">
       <c r="B32" s="30" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="C32" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D32" t="s">
+        <v>595</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="F32" t="s">
         <v>597</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>598</v>
-      </c>
-      <c r="F32" t="s">
-        <v>599</v>
       </c>
       <c r="G32" t="s">
         <v>64</v>
@@ -12215,19 +12214,19 @@
     </row>
     <row r="33" spans="1:9" ht="58">
       <c r="A33" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B33" s="30" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="D33" t="s">
+        <v>598</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>600</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>602</v>
-      </c>
       <c r="F33" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="G33" t="s">
         <v>64</v>
@@ -12241,28 +12240,28 @@
     </row>
     <row r="34" spans="1:9" ht="101.5">
       <c r="A34" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="B34" s="28" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C34" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="D34" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="F34" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="G34" t="s">
         <v>64</v>
       </c>
       <c r="H34" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="I34" t="s">
         <v>77</v>
@@ -12270,45 +12269,45 @@
     </row>
     <row r="35" spans="1:9" ht="43.5">
       <c r="B35" s="28" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C35" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D35" t="s">
+        <v>608</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="F35" t="s">
         <v>610</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>611</v>
-      </c>
-      <c r="F35" t="s">
-        <v>612</v>
       </c>
       <c r="G35" t="s">
         <v>64</v>
       </c>
       <c r="H35" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="36" spans="1:9">
       <c r="A36" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="B36" s="28" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C36" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D36" t="s">
+        <v>614</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="F36" t="s">
         <v>616</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="F36" t="s">
-        <v>618</v>
       </c>
       <c r="G36" t="s">
         <v>64</v>
@@ -12319,22 +12318,22 @@
     </row>
     <row r="37" spans="1:9" ht="43.5">
       <c r="A37" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B37" s="28" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C37" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="D37" t="s">
+        <v>617</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="F37" t="s">
         <v>619</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>620</v>
-      </c>
-      <c r="F37" t="s">
-        <v>621</v>
       </c>
       <c r="G37" t="s">
         <v>64</v>
@@ -12345,22 +12344,22 @@
     </row>
     <row r="38" spans="1:9" ht="43.5">
       <c r="A38" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="B38" s="28" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C38" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="D38" t="s">
+        <v>621</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="F38" t="s">
         <v>623</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>624</v>
-      </c>
-      <c r="F38" t="s">
-        <v>625</v>
       </c>
       <c r="G38" t="s">
         <v>64</v>
@@ -12374,7 +12373,7 @@
     </row>
     <row r="42" spans="1:9">
       <c r="A42" s="40" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="B42" s="41"/>
       <c r="C42" s="40"/>
@@ -12385,17 +12384,17 @@
     </row>
     <row r="43" spans="1:9">
       <c r="A43" s="41" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
       <c r="B43" s="40" t="s">
-        <v>466</v>
-      </c>
-      <c r="C43" s="45" t="s">
-        <v>665</v>
+        <v>464</v>
+      </c>
+      <c r="C43" s="44" t="s">
+        <v>661</v>
       </c>
       <c r="D43" s="42"/>
       <c r="F43" s="40" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="G43" s="40" t="s">
         <v>77</v>
@@ -12405,53 +12404,53 @@
       </c>
     </row>
     <row r="44" spans="1:9">
-      <c r="A44" s="44" t="s">
-        <v>675</v>
+      <c r="A44" s="40" t="s">
+        <v>671</v>
       </c>
       <c r="B44" s="40"/>
       <c r="C44" s="40" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="D44" s="42"/>
       <c r="F44" s="40" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="G44" s="40" t="s">
         <v>77</v>
       </c>
       <c r="H44" s="40" t="s">
-        <v>677</v>
+        <v>673</v>
       </c>
     </row>
     <row r="45" spans="1:9">
-      <c r="A45" s="44" t="s">
-        <v>671</v>
+      <c r="A45" s="40" t="s">
+        <v>667</v>
       </c>
       <c r="B45" s="40"/>
       <c r="C45" s="40" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="D45" s="42"/>
       <c r="F45" s="40" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="G45" s="40" t="s">
         <v>77</v>
       </c>
       <c r="H45" s="40" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
     </row>
     <row r="46" spans="1:9" s="4" customFormat="1">
       <c r="A46" s="4" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="B46" s="43"/>
       <c r="E46" s="3"/>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" s="40" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="B47" s="41"/>
       <c r="C47" s="40"/>
@@ -12480,18 +12479,18 @@
   <sheetData>
     <row r="1" spans="2:6">
       <c r="B1" s="2" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D1" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="2" spans="2:6" ht="29">
       <c r="B2" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C2" t="s">
         <v>77</v>
@@ -12505,7 +12504,7 @@
     </row>
     <row r="3" spans="2:6" ht="29">
       <c r="B3" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C3" t="s">
         <v>77</v>
@@ -12519,7 +12518,7 @@
     </row>
     <row r="5" spans="2:6" s="10" customFormat="1">
       <c r="B5" s="18" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>15</v>
@@ -12533,7 +12532,7 @@
     </row>
     <row r="7" spans="2:6" ht="29">
       <c r="B7" s="2" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C7" t="s">
         <v>77</v>
@@ -12547,7 +12546,7 @@
     </row>
     <row r="8" spans="2:6" ht="29">
       <c r="B8" s="2" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="C8" t="s">
         <v>77</v>
@@ -12572,7 +12571,7 @@
     </row>
     <row r="12" spans="2:6" ht="29">
       <c r="B12" s="2" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C12" t="s">
         <v>87</v>
@@ -12586,7 +12585,7 @@
     </row>
     <row r="17" spans="2:5" ht="43.5">
       <c r="B17" s="2" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="C17" t="s">
         <v>84</v>
@@ -12595,7 +12594,7 @@
         <v>320</v>
       </c>
       <c r="E17" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add added regression plots for mother working hours together with income -- no significant interaction
and some minor changes
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangk\Desktop\vaccination_uptake_jacsis2023\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7CE101-A666-43E2-AF8A-C4635380440D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D265FA1-66AC-4DA9-868C-7AC720AB1487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3470" yWindow="690" windowWidth="14400" windowHeight="8710" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3470" yWindow="690" windowWidth="14400" windowHeight="8710" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -48,17 +48,17 @@
   <commentList>
     <comment ref="AZ1" authorId="0" shapeId="0" xr:uid="{F627B11A-9966-4DAF-9CD9-36B5D028D9EE}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     Remove once we’ve determined how to stratify by disease</t>
       </text>
     </comment>
     <comment ref="CE1" authorId="1" shapeId="0" xr:uid="{E5BA077E-7025-4391-8B23-A38BD7E65674}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t xml:space="preserve">[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     Remove retired status and student status? (due to the low number of respondents who fall into these categories)
 </t>
       </text>
@@ -76,9 +76,9 @@
   <commentList>
     <comment ref="L68" authorId="0" shapeId="0" xr:uid="{869B55B9-3B1F-4453-9A39-E466CC7906FC}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t xml:space="preserve">[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     How should we define the number of parents a child has, the numebr of spouses livignin the same household? Or the marital status of the responding parent
 there are cases where parents = 1 but the responding parent is still married, and in such cases where the other parent isn’t living in the same hosuehold as them they still may have an influence on their childs’vaccination
 cases where parents = 2 but they arent married, i.e. divorced both parents might still have a say in the child’s vaccination
@@ -87,9 +87,9 @@
     </comment>
     <comment ref="E238" authorId="1" shapeId="0" xr:uid="{443BE410-81F7-49D5-89CA-23D177220CB4}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t xml:space="preserve">[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     Come back and change the time bins based on how the data behaves
 </t>
       </text>
@@ -108,9 +108,9 @@
   <commentList>
     <comment ref="D18" authorId="0" shapeId="0" xr:uid="{7F40D788-9EC4-40FB-A9F9-AD66BD761ADD}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     Should be age_cat and age_of_interest
 I will figure it out and update once I find out which graph this is referring to</t>
       </text>
@@ -143,9 +143,9 @@
     </comment>
     <comment ref="A47" authorId="2" shapeId="0" xr:uid="{96A696B5-9B70-421D-BAE5-16DC63333B7B}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     Will be interesting to see if marital status (i..e single parents) are affected by the number of children they have to care for.</t>
       </text>
     </comment>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2034" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2036" uniqueCount="683">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -2202,6 +2202,12 @@
   </si>
   <si>
     <t>take the approximate number of hours worked by the responding parent/spouse and determine which is the mother respectively. Derived from parent_1_sex and parent_2_sex, which correspond to the sex of the responding parent and the spouse of the responding parent respectively, which are then matched to parent_work_weekly and spouse_work_weekly. NA is assigned when there is no mother in the family (i..e single parent family) and 0 is assigned either when reported as 0 or when mother is unemployed</t>
+  </si>
+  <si>
+    <t>No interaction</t>
+  </si>
+  <si>
+    <t>mother's working hours</t>
   </si>
 </sst>
 </file>
@@ -2280,7 +2286,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2377,12 +2383,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -2411,7 +2411,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2459,7 +2459,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -2478,10 +2477,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
@@ -6575,7 +6576,7 @@
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="E119" s="38" t="s">
+      <c r="E119" s="37" t="s">
         <v>408</v>
       </c>
     </row>
@@ -6816,2056 +6817,2056 @@
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="E138" s="38" t="s">
+      <c r="E138" s="37" t="s">
         <v>408</v>
       </c>
-      <c r="M138" s="38"/>
-      <c r="U138" s="38"/>
-      <c r="AC138" s="38"/>
-      <c r="AK138" s="38"/>
-      <c r="AS138" s="38"/>
-      <c r="BA138" s="38"/>
-      <c r="BI138" s="38"/>
-      <c r="BQ138" s="38"/>
-      <c r="BY138" s="38"/>
-      <c r="CG138" s="38"/>
-      <c r="CO138" s="38"/>
-      <c r="CW138" s="38"/>
-      <c r="DE138" s="38"/>
-      <c r="DM138" s="38"/>
-      <c r="DU138" s="38"/>
-      <c r="EC138" s="38"/>
-      <c r="EK138" s="38"/>
-      <c r="ES138" s="38"/>
-      <c r="FA138" s="38"/>
-      <c r="FI138" s="38"/>
-      <c r="FQ138" s="38"/>
-      <c r="FY138" s="38"/>
-      <c r="GG138" s="38"/>
-      <c r="GO138" s="38"/>
-      <c r="GW138" s="38"/>
-      <c r="HE138" s="38"/>
-      <c r="HM138" s="38"/>
-      <c r="HU138" s="38"/>
-      <c r="IC138" s="38"/>
-      <c r="IK138" s="38"/>
-      <c r="IS138" s="38"/>
-      <c r="JA138" s="38"/>
-      <c r="JI138" s="38"/>
-      <c r="JQ138" s="38"/>
-      <c r="JY138" s="38"/>
-      <c r="KG138" s="38"/>
-      <c r="KO138" s="38"/>
-      <c r="KW138" s="38"/>
-      <c r="LE138" s="38"/>
-      <c r="LM138" s="38"/>
-      <c r="LU138" s="38"/>
-      <c r="MC138" s="38"/>
-      <c r="MK138" s="38"/>
-      <c r="MS138" s="38"/>
-      <c r="NA138" s="38"/>
-      <c r="NI138" s="38"/>
-      <c r="NQ138" s="38"/>
-      <c r="NY138" s="38"/>
-      <c r="OG138" s="38"/>
-      <c r="OO138" s="38"/>
-      <c r="OW138" s="38"/>
-      <c r="PE138" s="38"/>
-      <c r="PM138" s="38"/>
-      <c r="PU138" s="38"/>
-      <c r="QC138" s="38"/>
-      <c r="QK138" s="38"/>
-      <c r="QS138" s="38"/>
-      <c r="RA138" s="38"/>
-      <c r="RI138" s="38"/>
-      <c r="RQ138" s="38"/>
-      <c r="RY138" s="38"/>
-      <c r="SG138" s="38"/>
-      <c r="SO138" s="38"/>
-      <c r="SW138" s="38"/>
-      <c r="TE138" s="38"/>
-      <c r="TM138" s="38"/>
-      <c r="TU138" s="38"/>
-      <c r="UC138" s="38"/>
-      <c r="UK138" s="38"/>
-      <c r="US138" s="38"/>
-      <c r="VA138" s="38"/>
-      <c r="VI138" s="38"/>
-      <c r="VQ138" s="38"/>
-      <c r="VY138" s="38"/>
-      <c r="WG138" s="38"/>
-      <c r="WO138" s="38"/>
-      <c r="WW138" s="38"/>
-      <c r="XE138" s="38"/>
-      <c r="XM138" s="38"/>
-      <c r="XU138" s="38"/>
-      <c r="YC138" s="38"/>
-      <c r="YK138" s="38"/>
-      <c r="YS138" s="38"/>
-      <c r="ZA138" s="38"/>
-      <c r="ZI138" s="38"/>
-      <c r="ZQ138" s="38"/>
-      <c r="ZY138" s="38"/>
-      <c r="AAG138" s="38"/>
-      <c r="AAO138" s="38"/>
-      <c r="AAW138" s="38"/>
-      <c r="ABE138" s="38"/>
-      <c r="ABM138" s="38"/>
-      <c r="ABU138" s="38"/>
-      <c r="ACC138" s="38"/>
-      <c r="ACK138" s="38"/>
-      <c r="ACS138" s="38"/>
-      <c r="ADA138" s="38"/>
-      <c r="ADI138" s="38"/>
-      <c r="ADQ138" s="38"/>
-      <c r="ADY138" s="38"/>
-      <c r="AEG138" s="38"/>
-      <c r="AEO138" s="38"/>
-      <c r="AEW138" s="38"/>
-      <c r="AFE138" s="38"/>
-      <c r="AFM138" s="38"/>
-      <c r="AFU138" s="38"/>
-      <c r="AGC138" s="38"/>
-      <c r="AGK138" s="38"/>
-      <c r="AGS138" s="38"/>
-      <c r="AHA138" s="38"/>
-      <c r="AHI138" s="38"/>
-      <c r="AHQ138" s="38"/>
-      <c r="AHY138" s="38"/>
-      <c r="AIG138" s="38"/>
-      <c r="AIO138" s="38"/>
-      <c r="AIW138" s="38"/>
-      <c r="AJE138" s="38"/>
-      <c r="AJM138" s="38"/>
-      <c r="AJU138" s="38"/>
-      <c r="AKC138" s="38"/>
-      <c r="AKK138" s="38"/>
-      <c r="AKS138" s="38"/>
-      <c r="ALA138" s="38"/>
-      <c r="ALI138" s="38"/>
-      <c r="ALQ138" s="38"/>
-      <c r="ALY138" s="38"/>
-      <c r="AMG138" s="38"/>
-      <c r="AMO138" s="38"/>
-      <c r="AMW138" s="38"/>
-      <c r="ANE138" s="38"/>
-      <c r="ANM138" s="38"/>
-      <c r="ANU138" s="38"/>
-      <c r="AOC138" s="38"/>
-      <c r="AOK138" s="38"/>
-      <c r="AOS138" s="38"/>
-      <c r="APA138" s="38"/>
-      <c r="API138" s="38"/>
-      <c r="APQ138" s="38"/>
-      <c r="APY138" s="38"/>
-      <c r="AQG138" s="38"/>
-      <c r="AQO138" s="38"/>
-      <c r="AQW138" s="38"/>
-      <c r="ARE138" s="38"/>
-      <c r="ARM138" s="38"/>
-      <c r="ARU138" s="38"/>
-      <c r="ASC138" s="38"/>
-      <c r="ASK138" s="38"/>
-      <c r="ASS138" s="38"/>
-      <c r="ATA138" s="38"/>
-      <c r="ATI138" s="38"/>
-      <c r="ATQ138" s="38"/>
-      <c r="ATY138" s="38"/>
-      <c r="AUG138" s="38"/>
-      <c r="AUO138" s="38"/>
-      <c r="AUW138" s="38"/>
-      <c r="AVE138" s="38"/>
-      <c r="AVM138" s="38"/>
-      <c r="AVU138" s="38"/>
-      <c r="AWC138" s="38"/>
-      <c r="AWK138" s="38"/>
-      <c r="AWS138" s="38"/>
-      <c r="AXA138" s="38"/>
-      <c r="AXI138" s="38"/>
-      <c r="AXQ138" s="38"/>
-      <c r="AXY138" s="38"/>
-      <c r="AYG138" s="38"/>
-      <c r="AYO138" s="38"/>
-      <c r="AYW138" s="38"/>
-      <c r="AZE138" s="38"/>
-      <c r="AZM138" s="38"/>
-      <c r="AZU138" s="38"/>
-      <c r="BAC138" s="38"/>
-      <c r="BAK138" s="38"/>
-      <c r="BAS138" s="38"/>
-      <c r="BBA138" s="38"/>
-      <c r="BBI138" s="38"/>
-      <c r="BBQ138" s="38"/>
-      <c r="BBY138" s="38"/>
-      <c r="BCG138" s="38"/>
-      <c r="BCO138" s="38"/>
-      <c r="BCW138" s="38"/>
-      <c r="BDE138" s="38"/>
-      <c r="BDM138" s="38"/>
-      <c r="BDU138" s="38"/>
-      <c r="BEC138" s="38"/>
-      <c r="BEK138" s="38"/>
-      <c r="BES138" s="38"/>
-      <c r="BFA138" s="38"/>
-      <c r="BFI138" s="38"/>
-      <c r="BFQ138" s="38"/>
-      <c r="BFY138" s="38"/>
-      <c r="BGG138" s="38"/>
-      <c r="BGO138" s="38"/>
-      <c r="BGW138" s="38"/>
-      <c r="BHE138" s="38"/>
-      <c r="BHM138" s="38"/>
-      <c r="BHU138" s="38"/>
-      <c r="BIC138" s="38"/>
-      <c r="BIK138" s="38"/>
-      <c r="BIS138" s="38"/>
-      <c r="BJA138" s="38"/>
-      <c r="BJI138" s="38"/>
-      <c r="BJQ138" s="38"/>
-      <c r="BJY138" s="38"/>
-      <c r="BKG138" s="38"/>
-      <c r="BKO138" s="38"/>
-      <c r="BKW138" s="38"/>
-      <c r="BLE138" s="38"/>
-      <c r="BLM138" s="38"/>
-      <c r="BLU138" s="38"/>
-      <c r="BMC138" s="38"/>
-      <c r="BMK138" s="38"/>
-      <c r="BMS138" s="38"/>
-      <c r="BNA138" s="38"/>
-      <c r="BNI138" s="38"/>
-      <c r="BNQ138" s="38"/>
-      <c r="BNY138" s="38"/>
-      <c r="BOG138" s="38"/>
-      <c r="BOO138" s="38"/>
-      <c r="BOW138" s="38"/>
-      <c r="BPE138" s="38"/>
-      <c r="BPM138" s="38"/>
-      <c r="BPU138" s="38"/>
-      <c r="BQC138" s="38"/>
-      <c r="BQK138" s="38"/>
-      <c r="BQS138" s="38"/>
-      <c r="BRA138" s="38"/>
-      <c r="BRI138" s="38"/>
-      <c r="BRQ138" s="38"/>
-      <c r="BRY138" s="38"/>
-      <c r="BSG138" s="38"/>
-      <c r="BSO138" s="38"/>
-      <c r="BSW138" s="38"/>
-      <c r="BTE138" s="38"/>
-      <c r="BTM138" s="38"/>
-      <c r="BTU138" s="38"/>
-      <c r="BUC138" s="38"/>
-      <c r="BUK138" s="38"/>
-      <c r="BUS138" s="38"/>
-      <c r="BVA138" s="38"/>
-      <c r="BVI138" s="38"/>
-      <c r="BVQ138" s="38"/>
-      <c r="BVY138" s="38"/>
-      <c r="BWG138" s="38"/>
-      <c r="BWO138" s="38"/>
-      <c r="BWW138" s="38"/>
-      <c r="BXE138" s="38"/>
-      <c r="BXM138" s="38"/>
-      <c r="BXU138" s="38"/>
-      <c r="BYC138" s="38"/>
-      <c r="BYK138" s="38"/>
-      <c r="BYS138" s="38"/>
-      <c r="BZA138" s="38"/>
-      <c r="BZI138" s="38"/>
-      <c r="BZQ138" s="38"/>
-      <c r="BZY138" s="38"/>
-      <c r="CAG138" s="38"/>
-      <c r="CAO138" s="38"/>
-      <c r="CAW138" s="38"/>
-      <c r="CBE138" s="38"/>
-      <c r="CBM138" s="38"/>
-      <c r="CBU138" s="38"/>
-      <c r="CCC138" s="38"/>
-      <c r="CCK138" s="38"/>
-      <c r="CCS138" s="38"/>
-      <c r="CDA138" s="38"/>
-      <c r="CDI138" s="38"/>
-      <c r="CDQ138" s="38"/>
-      <c r="CDY138" s="38"/>
-      <c r="CEG138" s="38"/>
-      <c r="CEO138" s="38"/>
-      <c r="CEW138" s="38"/>
-      <c r="CFE138" s="38"/>
-      <c r="CFM138" s="38"/>
-      <c r="CFU138" s="38"/>
-      <c r="CGC138" s="38"/>
-      <c r="CGK138" s="38"/>
-      <c r="CGS138" s="38"/>
-      <c r="CHA138" s="38"/>
-      <c r="CHI138" s="38"/>
-      <c r="CHQ138" s="38"/>
-      <c r="CHY138" s="38"/>
-      <c r="CIG138" s="38"/>
-      <c r="CIO138" s="38"/>
-      <c r="CIW138" s="38"/>
-      <c r="CJE138" s="38"/>
-      <c r="CJM138" s="38"/>
-      <c r="CJU138" s="38"/>
-      <c r="CKC138" s="38"/>
-      <c r="CKK138" s="38"/>
-      <c r="CKS138" s="38"/>
-      <c r="CLA138" s="38"/>
-      <c r="CLI138" s="38"/>
-      <c r="CLQ138" s="38"/>
-      <c r="CLY138" s="38"/>
-      <c r="CMG138" s="38"/>
-      <c r="CMO138" s="38"/>
-      <c r="CMW138" s="38"/>
-      <c r="CNE138" s="38"/>
-      <c r="CNM138" s="38"/>
-      <c r="CNU138" s="38"/>
-      <c r="COC138" s="38"/>
-      <c r="COK138" s="38"/>
-      <c r="COS138" s="38"/>
-      <c r="CPA138" s="38"/>
-      <c r="CPI138" s="38"/>
-      <c r="CPQ138" s="38"/>
-      <c r="CPY138" s="38"/>
-      <c r="CQG138" s="38"/>
-      <c r="CQO138" s="38"/>
-      <c r="CQW138" s="38"/>
-      <c r="CRE138" s="38"/>
-      <c r="CRM138" s="38"/>
-      <c r="CRU138" s="38"/>
-      <c r="CSC138" s="38"/>
-      <c r="CSK138" s="38"/>
-      <c r="CSS138" s="38"/>
-      <c r="CTA138" s="38"/>
-      <c r="CTI138" s="38"/>
-      <c r="CTQ138" s="38"/>
-      <c r="CTY138" s="38"/>
-      <c r="CUG138" s="38"/>
-      <c r="CUO138" s="38"/>
-      <c r="CUW138" s="38"/>
-      <c r="CVE138" s="38"/>
-      <c r="CVM138" s="38"/>
-      <c r="CVU138" s="38"/>
-      <c r="CWC138" s="38"/>
-      <c r="CWK138" s="38"/>
-      <c r="CWS138" s="38"/>
-      <c r="CXA138" s="38"/>
-      <c r="CXI138" s="38"/>
-      <c r="CXQ138" s="38"/>
-      <c r="CXY138" s="38"/>
-      <c r="CYG138" s="38"/>
-      <c r="CYO138" s="38"/>
-      <c r="CYW138" s="38"/>
-      <c r="CZE138" s="38"/>
-      <c r="CZM138" s="38"/>
-      <c r="CZU138" s="38"/>
-      <c r="DAC138" s="38"/>
-      <c r="DAK138" s="38"/>
-      <c r="DAS138" s="38"/>
-      <c r="DBA138" s="38"/>
-      <c r="DBI138" s="38"/>
-      <c r="DBQ138" s="38"/>
-      <c r="DBY138" s="38"/>
-      <c r="DCG138" s="38"/>
-      <c r="DCO138" s="38"/>
-      <c r="DCW138" s="38"/>
-      <c r="DDE138" s="38"/>
-      <c r="DDM138" s="38"/>
-      <c r="DDU138" s="38"/>
-      <c r="DEC138" s="38"/>
-      <c r="DEK138" s="38"/>
-      <c r="DES138" s="38"/>
-      <c r="DFA138" s="38"/>
-      <c r="DFI138" s="38"/>
-      <c r="DFQ138" s="38"/>
-      <c r="DFY138" s="38"/>
-      <c r="DGG138" s="38"/>
-      <c r="DGO138" s="38"/>
-      <c r="DGW138" s="38"/>
-      <c r="DHE138" s="38"/>
-      <c r="DHM138" s="38"/>
-      <c r="DHU138" s="38"/>
-      <c r="DIC138" s="38"/>
-      <c r="DIK138" s="38"/>
-      <c r="DIS138" s="38"/>
-      <c r="DJA138" s="38"/>
-      <c r="DJI138" s="38"/>
-      <c r="DJQ138" s="38"/>
-      <c r="DJY138" s="38"/>
-      <c r="DKG138" s="38"/>
-      <c r="DKO138" s="38"/>
-      <c r="DKW138" s="38"/>
-      <c r="DLE138" s="38"/>
-      <c r="DLM138" s="38"/>
-      <c r="DLU138" s="38"/>
-      <c r="DMC138" s="38"/>
-      <c r="DMK138" s="38"/>
-      <c r="DMS138" s="38"/>
-      <c r="DNA138" s="38"/>
-      <c r="DNI138" s="38"/>
-      <c r="DNQ138" s="38"/>
-      <c r="DNY138" s="38"/>
-      <c r="DOG138" s="38"/>
-      <c r="DOO138" s="38"/>
-      <c r="DOW138" s="38"/>
-      <c r="DPE138" s="38"/>
-      <c r="DPM138" s="38"/>
-      <c r="DPU138" s="38"/>
-      <c r="DQC138" s="38"/>
-      <c r="DQK138" s="38"/>
-      <c r="DQS138" s="38"/>
-      <c r="DRA138" s="38"/>
-      <c r="DRI138" s="38"/>
-      <c r="DRQ138" s="38"/>
-      <c r="DRY138" s="38"/>
-      <c r="DSG138" s="38"/>
-      <c r="DSO138" s="38"/>
-      <c r="DSW138" s="38"/>
-      <c r="DTE138" s="38"/>
-      <c r="DTM138" s="38"/>
-      <c r="DTU138" s="38"/>
-      <c r="DUC138" s="38"/>
-      <c r="DUK138" s="38"/>
-      <c r="DUS138" s="38"/>
-      <c r="DVA138" s="38"/>
-      <c r="DVI138" s="38"/>
-      <c r="DVQ138" s="38"/>
-      <c r="DVY138" s="38"/>
-      <c r="DWG138" s="38"/>
-      <c r="DWO138" s="38"/>
-      <c r="DWW138" s="38"/>
-      <c r="DXE138" s="38"/>
-      <c r="DXM138" s="38"/>
-      <c r="DXU138" s="38"/>
-      <c r="DYC138" s="38"/>
-      <c r="DYK138" s="38"/>
-      <c r="DYS138" s="38"/>
-      <c r="DZA138" s="38"/>
-      <c r="DZI138" s="38"/>
-      <c r="DZQ138" s="38"/>
-      <c r="DZY138" s="38"/>
-      <c r="EAG138" s="38"/>
-      <c r="EAO138" s="38"/>
-      <c r="EAW138" s="38"/>
-      <c r="EBE138" s="38"/>
-      <c r="EBM138" s="38"/>
-      <c r="EBU138" s="38"/>
-      <c r="ECC138" s="38"/>
-      <c r="ECK138" s="38"/>
-      <c r="ECS138" s="38"/>
-      <c r="EDA138" s="38"/>
-      <c r="EDI138" s="38"/>
-      <c r="EDQ138" s="38"/>
-      <c r="EDY138" s="38"/>
-      <c r="EEG138" s="38"/>
-      <c r="EEO138" s="38"/>
-      <c r="EEW138" s="38"/>
-      <c r="EFE138" s="38"/>
-      <c r="EFM138" s="38"/>
-      <c r="EFU138" s="38"/>
-      <c r="EGC138" s="38"/>
-      <c r="EGK138" s="38"/>
-      <c r="EGS138" s="38"/>
-      <c r="EHA138" s="38"/>
-      <c r="EHI138" s="38"/>
-      <c r="EHQ138" s="38"/>
-      <c r="EHY138" s="38"/>
-      <c r="EIG138" s="38"/>
-      <c r="EIO138" s="38"/>
-      <c r="EIW138" s="38"/>
-      <c r="EJE138" s="38"/>
-      <c r="EJM138" s="38"/>
-      <c r="EJU138" s="38"/>
-      <c r="EKC138" s="38"/>
-      <c r="EKK138" s="38"/>
-      <c r="EKS138" s="38"/>
-      <c r="ELA138" s="38"/>
-      <c r="ELI138" s="38"/>
-      <c r="ELQ138" s="38"/>
-      <c r="ELY138" s="38"/>
-      <c r="EMG138" s="38"/>
-      <c r="EMO138" s="38"/>
-      <c r="EMW138" s="38"/>
-      <c r="ENE138" s="38"/>
-      <c r="ENM138" s="38"/>
-      <c r="ENU138" s="38"/>
-      <c r="EOC138" s="38"/>
-      <c r="EOK138" s="38"/>
-      <c r="EOS138" s="38"/>
-      <c r="EPA138" s="38"/>
-      <c r="EPI138" s="38"/>
-      <c r="EPQ138" s="38"/>
-      <c r="EPY138" s="38"/>
-      <c r="EQG138" s="38"/>
-      <c r="EQO138" s="38"/>
-      <c r="EQW138" s="38"/>
-      <c r="ERE138" s="38"/>
-      <c r="ERM138" s="38"/>
-      <c r="ERU138" s="38"/>
-      <c r="ESC138" s="38"/>
-      <c r="ESK138" s="38"/>
-      <c r="ESS138" s="38"/>
-      <c r="ETA138" s="38"/>
-      <c r="ETI138" s="38"/>
-      <c r="ETQ138" s="38"/>
-      <c r="ETY138" s="38"/>
-      <c r="EUG138" s="38"/>
-      <c r="EUO138" s="38"/>
-      <c r="EUW138" s="38"/>
-      <c r="EVE138" s="38"/>
-      <c r="EVM138" s="38"/>
-      <c r="EVU138" s="38"/>
-      <c r="EWC138" s="38"/>
-      <c r="EWK138" s="38"/>
-      <c r="EWS138" s="38"/>
-      <c r="EXA138" s="38"/>
-      <c r="EXI138" s="38"/>
-      <c r="EXQ138" s="38"/>
-      <c r="EXY138" s="38"/>
-      <c r="EYG138" s="38"/>
-      <c r="EYO138" s="38"/>
-      <c r="EYW138" s="38"/>
-      <c r="EZE138" s="38"/>
-      <c r="EZM138" s="38"/>
-      <c r="EZU138" s="38"/>
-      <c r="FAC138" s="38"/>
-      <c r="FAK138" s="38"/>
-      <c r="FAS138" s="38"/>
-      <c r="FBA138" s="38"/>
-      <c r="FBI138" s="38"/>
-      <c r="FBQ138" s="38"/>
-      <c r="FBY138" s="38"/>
-      <c r="FCG138" s="38"/>
-      <c r="FCO138" s="38"/>
-      <c r="FCW138" s="38"/>
-      <c r="FDE138" s="38"/>
-      <c r="FDM138" s="38"/>
-      <c r="FDU138" s="38"/>
-      <c r="FEC138" s="38"/>
-      <c r="FEK138" s="38"/>
-      <c r="FES138" s="38"/>
-      <c r="FFA138" s="38"/>
-      <c r="FFI138" s="38"/>
-      <c r="FFQ138" s="38"/>
-      <c r="FFY138" s="38"/>
-      <c r="FGG138" s="38"/>
-      <c r="FGO138" s="38"/>
-      <c r="FGW138" s="38"/>
-      <c r="FHE138" s="38"/>
-      <c r="FHM138" s="38"/>
-      <c r="FHU138" s="38"/>
-      <c r="FIC138" s="38"/>
-      <c r="FIK138" s="38"/>
-      <c r="FIS138" s="38"/>
-      <c r="FJA138" s="38"/>
-      <c r="FJI138" s="38"/>
-      <c r="FJQ138" s="38"/>
-      <c r="FJY138" s="38"/>
-      <c r="FKG138" s="38"/>
-      <c r="FKO138" s="38"/>
-      <c r="FKW138" s="38"/>
-      <c r="FLE138" s="38"/>
-      <c r="FLM138" s="38"/>
-      <c r="FLU138" s="38"/>
-      <c r="FMC138" s="38"/>
-      <c r="FMK138" s="38"/>
-      <c r="FMS138" s="38"/>
-      <c r="FNA138" s="38"/>
-      <c r="FNI138" s="38"/>
-      <c r="FNQ138" s="38"/>
-      <c r="FNY138" s="38"/>
-      <c r="FOG138" s="38"/>
-      <c r="FOO138" s="38"/>
-      <c r="FOW138" s="38"/>
-      <c r="FPE138" s="38"/>
-      <c r="FPM138" s="38"/>
-      <c r="FPU138" s="38"/>
-      <c r="FQC138" s="38"/>
-      <c r="FQK138" s="38"/>
-      <c r="FQS138" s="38"/>
-      <c r="FRA138" s="38"/>
-      <c r="FRI138" s="38"/>
-      <c r="FRQ138" s="38"/>
-      <c r="FRY138" s="38"/>
-      <c r="FSG138" s="38"/>
-      <c r="FSO138" s="38"/>
-      <c r="FSW138" s="38"/>
-      <c r="FTE138" s="38"/>
-      <c r="FTM138" s="38"/>
-      <c r="FTU138" s="38"/>
-      <c r="FUC138" s="38"/>
-      <c r="FUK138" s="38"/>
-      <c r="FUS138" s="38"/>
-      <c r="FVA138" s="38"/>
-      <c r="FVI138" s="38"/>
-      <c r="FVQ138" s="38"/>
-      <c r="FVY138" s="38"/>
-      <c r="FWG138" s="38"/>
-      <c r="FWO138" s="38"/>
-      <c r="FWW138" s="38"/>
-      <c r="FXE138" s="38"/>
-      <c r="FXM138" s="38"/>
-      <c r="FXU138" s="38"/>
-      <c r="FYC138" s="38"/>
-      <c r="FYK138" s="38"/>
-      <c r="FYS138" s="38"/>
-      <c r="FZA138" s="38"/>
-      <c r="FZI138" s="38"/>
-      <c r="FZQ138" s="38"/>
-      <c r="FZY138" s="38"/>
-      <c r="GAG138" s="38"/>
-      <c r="GAO138" s="38"/>
-      <c r="GAW138" s="38"/>
-      <c r="GBE138" s="38"/>
-      <c r="GBM138" s="38"/>
-      <c r="GBU138" s="38"/>
-      <c r="GCC138" s="38"/>
-      <c r="GCK138" s="38"/>
-      <c r="GCS138" s="38"/>
-      <c r="GDA138" s="38"/>
-      <c r="GDI138" s="38"/>
-      <c r="GDQ138" s="38"/>
-      <c r="GDY138" s="38"/>
-      <c r="GEG138" s="38"/>
-      <c r="GEO138" s="38"/>
-      <c r="GEW138" s="38"/>
-      <c r="GFE138" s="38"/>
-      <c r="GFM138" s="38"/>
-      <c r="GFU138" s="38"/>
-      <c r="GGC138" s="38"/>
-      <c r="GGK138" s="38"/>
-      <c r="GGS138" s="38"/>
-      <c r="GHA138" s="38"/>
-      <c r="GHI138" s="38"/>
-      <c r="GHQ138" s="38"/>
-      <c r="GHY138" s="38"/>
-      <c r="GIG138" s="38"/>
-      <c r="GIO138" s="38"/>
-      <c r="GIW138" s="38"/>
-      <c r="GJE138" s="38"/>
-      <c r="GJM138" s="38"/>
-      <c r="GJU138" s="38"/>
-      <c r="GKC138" s="38"/>
-      <c r="GKK138" s="38"/>
-      <c r="GKS138" s="38"/>
-      <c r="GLA138" s="38"/>
-      <c r="GLI138" s="38"/>
-      <c r="GLQ138" s="38"/>
-      <c r="GLY138" s="38"/>
-      <c r="GMG138" s="38"/>
-      <c r="GMO138" s="38"/>
-      <c r="GMW138" s="38"/>
-      <c r="GNE138" s="38"/>
-      <c r="GNM138" s="38"/>
-      <c r="GNU138" s="38"/>
-      <c r="GOC138" s="38"/>
-      <c r="GOK138" s="38"/>
-      <c r="GOS138" s="38"/>
-      <c r="GPA138" s="38"/>
-      <c r="GPI138" s="38"/>
-      <c r="GPQ138" s="38"/>
-      <c r="GPY138" s="38"/>
-      <c r="GQG138" s="38"/>
-      <c r="GQO138" s="38"/>
-      <c r="GQW138" s="38"/>
-      <c r="GRE138" s="38"/>
-      <c r="GRM138" s="38"/>
-      <c r="GRU138" s="38"/>
-      <c r="GSC138" s="38"/>
-      <c r="GSK138" s="38"/>
-      <c r="GSS138" s="38"/>
-      <c r="GTA138" s="38"/>
-      <c r="GTI138" s="38"/>
-      <c r="GTQ138" s="38"/>
-      <c r="GTY138" s="38"/>
-      <c r="GUG138" s="38"/>
-      <c r="GUO138" s="38"/>
-      <c r="GUW138" s="38"/>
-      <c r="GVE138" s="38"/>
-      <c r="GVM138" s="38"/>
-      <c r="GVU138" s="38"/>
-      <c r="GWC138" s="38"/>
-      <c r="GWK138" s="38"/>
-      <c r="GWS138" s="38"/>
-      <c r="GXA138" s="38"/>
-      <c r="GXI138" s="38"/>
-      <c r="GXQ138" s="38"/>
-      <c r="GXY138" s="38"/>
-      <c r="GYG138" s="38"/>
-      <c r="GYO138" s="38"/>
-      <c r="GYW138" s="38"/>
-      <c r="GZE138" s="38"/>
-      <c r="GZM138" s="38"/>
-      <c r="GZU138" s="38"/>
-      <c r="HAC138" s="38"/>
-      <c r="HAK138" s="38"/>
-      <c r="HAS138" s="38"/>
-      <c r="HBA138" s="38"/>
-      <c r="HBI138" s="38"/>
-      <c r="HBQ138" s="38"/>
-      <c r="HBY138" s="38"/>
-      <c r="HCG138" s="38"/>
-      <c r="HCO138" s="38"/>
-      <c r="HCW138" s="38"/>
-      <c r="HDE138" s="38"/>
-      <c r="HDM138" s="38"/>
-      <c r="HDU138" s="38"/>
-      <c r="HEC138" s="38"/>
-      <c r="HEK138" s="38"/>
-      <c r="HES138" s="38"/>
-      <c r="HFA138" s="38"/>
-      <c r="HFI138" s="38"/>
-      <c r="HFQ138" s="38"/>
-      <c r="HFY138" s="38"/>
-      <c r="HGG138" s="38"/>
-      <c r="HGO138" s="38"/>
-      <c r="HGW138" s="38"/>
-      <c r="HHE138" s="38"/>
-      <c r="HHM138" s="38"/>
-      <c r="HHU138" s="38"/>
-      <c r="HIC138" s="38"/>
-      <c r="HIK138" s="38"/>
-      <c r="HIS138" s="38"/>
-      <c r="HJA138" s="38"/>
-      <c r="HJI138" s="38"/>
-      <c r="HJQ138" s="38"/>
-      <c r="HJY138" s="38"/>
-      <c r="HKG138" s="38"/>
-      <c r="HKO138" s="38"/>
-      <c r="HKW138" s="38"/>
-      <c r="HLE138" s="38"/>
-      <c r="HLM138" s="38"/>
-      <c r="HLU138" s="38"/>
-      <c r="HMC138" s="38"/>
-      <c r="HMK138" s="38"/>
-      <c r="HMS138" s="38"/>
-      <c r="HNA138" s="38"/>
-      <c r="HNI138" s="38"/>
-      <c r="HNQ138" s="38"/>
-      <c r="HNY138" s="38"/>
-      <c r="HOG138" s="38"/>
-      <c r="HOO138" s="38"/>
-      <c r="HOW138" s="38"/>
-      <c r="HPE138" s="38"/>
-      <c r="HPM138" s="38"/>
-      <c r="HPU138" s="38"/>
-      <c r="HQC138" s="38"/>
-      <c r="HQK138" s="38"/>
-      <c r="HQS138" s="38"/>
-      <c r="HRA138" s="38"/>
-      <c r="HRI138" s="38"/>
-      <c r="HRQ138" s="38"/>
-      <c r="HRY138" s="38"/>
-      <c r="HSG138" s="38"/>
-      <c r="HSO138" s="38"/>
-      <c r="HSW138" s="38"/>
-      <c r="HTE138" s="38"/>
-      <c r="HTM138" s="38"/>
-      <c r="HTU138" s="38"/>
-      <c r="HUC138" s="38"/>
-      <c r="HUK138" s="38"/>
-      <c r="HUS138" s="38"/>
-      <c r="HVA138" s="38"/>
-      <c r="HVI138" s="38"/>
-      <c r="HVQ138" s="38"/>
-      <c r="HVY138" s="38"/>
-      <c r="HWG138" s="38"/>
-      <c r="HWO138" s="38"/>
-      <c r="HWW138" s="38"/>
-      <c r="HXE138" s="38"/>
-      <c r="HXM138" s="38"/>
-      <c r="HXU138" s="38"/>
-      <c r="HYC138" s="38"/>
-      <c r="HYK138" s="38"/>
-      <c r="HYS138" s="38"/>
-      <c r="HZA138" s="38"/>
-      <c r="HZI138" s="38"/>
-      <c r="HZQ138" s="38"/>
-      <c r="HZY138" s="38"/>
-      <c r="IAG138" s="38"/>
-      <c r="IAO138" s="38"/>
-      <c r="IAW138" s="38"/>
-      <c r="IBE138" s="38"/>
-      <c r="IBM138" s="38"/>
-      <c r="IBU138" s="38"/>
-      <c r="ICC138" s="38"/>
-      <c r="ICK138" s="38"/>
-      <c r="ICS138" s="38"/>
-      <c r="IDA138" s="38"/>
-      <c r="IDI138" s="38"/>
-      <c r="IDQ138" s="38"/>
-      <c r="IDY138" s="38"/>
-      <c r="IEG138" s="38"/>
-      <c r="IEO138" s="38"/>
-      <c r="IEW138" s="38"/>
-      <c r="IFE138" s="38"/>
-      <c r="IFM138" s="38"/>
-      <c r="IFU138" s="38"/>
-      <c r="IGC138" s="38"/>
-      <c r="IGK138" s="38"/>
-      <c r="IGS138" s="38"/>
-      <c r="IHA138" s="38"/>
-      <c r="IHI138" s="38"/>
-      <c r="IHQ138" s="38"/>
-      <c r="IHY138" s="38"/>
-      <c r="IIG138" s="38"/>
-      <c r="IIO138" s="38"/>
-      <c r="IIW138" s="38"/>
-      <c r="IJE138" s="38"/>
-      <c r="IJM138" s="38"/>
-      <c r="IJU138" s="38"/>
-      <c r="IKC138" s="38"/>
-      <c r="IKK138" s="38"/>
-      <c r="IKS138" s="38"/>
-      <c r="ILA138" s="38"/>
-      <c r="ILI138" s="38"/>
-      <c r="ILQ138" s="38"/>
-      <c r="ILY138" s="38"/>
-      <c r="IMG138" s="38"/>
-      <c r="IMO138" s="38"/>
-      <c r="IMW138" s="38"/>
-      <c r="INE138" s="38"/>
-      <c r="INM138" s="38"/>
-      <c r="INU138" s="38"/>
-      <c r="IOC138" s="38"/>
-      <c r="IOK138" s="38"/>
-      <c r="IOS138" s="38"/>
-      <c r="IPA138" s="38"/>
-      <c r="IPI138" s="38"/>
-      <c r="IPQ138" s="38"/>
-      <c r="IPY138" s="38"/>
-      <c r="IQG138" s="38"/>
-      <c r="IQO138" s="38"/>
-      <c r="IQW138" s="38"/>
-      <c r="IRE138" s="38"/>
-      <c r="IRM138" s="38"/>
-      <c r="IRU138" s="38"/>
-      <c r="ISC138" s="38"/>
-      <c r="ISK138" s="38"/>
-      <c r="ISS138" s="38"/>
-      <c r="ITA138" s="38"/>
-      <c r="ITI138" s="38"/>
-      <c r="ITQ138" s="38"/>
-      <c r="ITY138" s="38"/>
-      <c r="IUG138" s="38"/>
-      <c r="IUO138" s="38"/>
-      <c r="IUW138" s="38"/>
-      <c r="IVE138" s="38"/>
-      <c r="IVM138" s="38"/>
-      <c r="IVU138" s="38"/>
-      <c r="IWC138" s="38"/>
-      <c r="IWK138" s="38"/>
-      <c r="IWS138" s="38"/>
-      <c r="IXA138" s="38"/>
-      <c r="IXI138" s="38"/>
-      <c r="IXQ138" s="38"/>
-      <c r="IXY138" s="38"/>
-      <c r="IYG138" s="38"/>
-      <c r="IYO138" s="38"/>
-      <c r="IYW138" s="38"/>
-      <c r="IZE138" s="38"/>
-      <c r="IZM138" s="38"/>
-      <c r="IZU138" s="38"/>
-      <c r="JAC138" s="38"/>
-      <c r="JAK138" s="38"/>
-      <c r="JAS138" s="38"/>
-      <c r="JBA138" s="38"/>
-      <c r="JBI138" s="38"/>
-      <c r="JBQ138" s="38"/>
-      <c r="JBY138" s="38"/>
-      <c r="JCG138" s="38"/>
-      <c r="JCO138" s="38"/>
-      <c r="JCW138" s="38"/>
-      <c r="JDE138" s="38"/>
-      <c r="JDM138" s="38"/>
-      <c r="JDU138" s="38"/>
-      <c r="JEC138" s="38"/>
-      <c r="JEK138" s="38"/>
-      <c r="JES138" s="38"/>
-      <c r="JFA138" s="38"/>
-      <c r="JFI138" s="38"/>
-      <c r="JFQ138" s="38"/>
-      <c r="JFY138" s="38"/>
-      <c r="JGG138" s="38"/>
-      <c r="JGO138" s="38"/>
-      <c r="JGW138" s="38"/>
-      <c r="JHE138" s="38"/>
-      <c r="JHM138" s="38"/>
-      <c r="JHU138" s="38"/>
-      <c r="JIC138" s="38"/>
-      <c r="JIK138" s="38"/>
-      <c r="JIS138" s="38"/>
-      <c r="JJA138" s="38"/>
-      <c r="JJI138" s="38"/>
-      <c r="JJQ138" s="38"/>
-      <c r="JJY138" s="38"/>
-      <c r="JKG138" s="38"/>
-      <c r="JKO138" s="38"/>
-      <c r="JKW138" s="38"/>
-      <c r="JLE138" s="38"/>
-      <c r="JLM138" s="38"/>
-      <c r="JLU138" s="38"/>
-      <c r="JMC138" s="38"/>
-      <c r="JMK138" s="38"/>
-      <c r="JMS138" s="38"/>
-      <c r="JNA138" s="38"/>
-      <c r="JNI138" s="38"/>
-      <c r="JNQ138" s="38"/>
-      <c r="JNY138" s="38"/>
-      <c r="JOG138" s="38"/>
-      <c r="JOO138" s="38"/>
-      <c r="JOW138" s="38"/>
-      <c r="JPE138" s="38"/>
-      <c r="JPM138" s="38"/>
-      <c r="JPU138" s="38"/>
-      <c r="JQC138" s="38"/>
-      <c r="JQK138" s="38"/>
-      <c r="JQS138" s="38"/>
-      <c r="JRA138" s="38"/>
-      <c r="JRI138" s="38"/>
-      <c r="JRQ138" s="38"/>
-      <c r="JRY138" s="38"/>
-      <c r="JSG138" s="38"/>
-      <c r="JSO138" s="38"/>
-      <c r="JSW138" s="38"/>
-      <c r="JTE138" s="38"/>
-      <c r="JTM138" s="38"/>
-      <c r="JTU138" s="38"/>
-      <c r="JUC138" s="38"/>
-      <c r="JUK138" s="38"/>
-      <c r="JUS138" s="38"/>
-      <c r="JVA138" s="38"/>
-      <c r="JVI138" s="38"/>
-      <c r="JVQ138" s="38"/>
-      <c r="JVY138" s="38"/>
-      <c r="JWG138" s="38"/>
-      <c r="JWO138" s="38"/>
-      <c r="JWW138" s="38"/>
-      <c r="JXE138" s="38"/>
-      <c r="JXM138" s="38"/>
-      <c r="JXU138" s="38"/>
-      <c r="JYC138" s="38"/>
-      <c r="JYK138" s="38"/>
-      <c r="JYS138" s="38"/>
-      <c r="JZA138" s="38"/>
-      <c r="JZI138" s="38"/>
-      <c r="JZQ138" s="38"/>
-      <c r="JZY138" s="38"/>
-      <c r="KAG138" s="38"/>
-      <c r="KAO138" s="38"/>
-      <c r="KAW138" s="38"/>
-      <c r="KBE138" s="38"/>
-      <c r="KBM138" s="38"/>
-      <c r="KBU138" s="38"/>
-      <c r="KCC138" s="38"/>
-      <c r="KCK138" s="38"/>
-      <c r="KCS138" s="38"/>
-      <c r="KDA138" s="38"/>
-      <c r="KDI138" s="38"/>
-      <c r="KDQ138" s="38"/>
-      <c r="KDY138" s="38"/>
-      <c r="KEG138" s="38"/>
-      <c r="KEO138" s="38"/>
-      <c r="KEW138" s="38"/>
-      <c r="KFE138" s="38"/>
-      <c r="KFM138" s="38"/>
-      <c r="KFU138" s="38"/>
-      <c r="KGC138" s="38"/>
-      <c r="KGK138" s="38"/>
-      <c r="KGS138" s="38"/>
-      <c r="KHA138" s="38"/>
-      <c r="KHI138" s="38"/>
-      <c r="KHQ138" s="38"/>
-      <c r="KHY138" s="38"/>
-      <c r="KIG138" s="38"/>
-      <c r="KIO138" s="38"/>
-      <c r="KIW138" s="38"/>
-      <c r="KJE138" s="38"/>
-      <c r="KJM138" s="38"/>
-      <c r="KJU138" s="38"/>
-      <c r="KKC138" s="38"/>
-      <c r="KKK138" s="38"/>
-      <c r="KKS138" s="38"/>
-      <c r="KLA138" s="38"/>
-      <c r="KLI138" s="38"/>
-      <c r="KLQ138" s="38"/>
-      <c r="KLY138" s="38"/>
-      <c r="KMG138" s="38"/>
-      <c r="KMO138" s="38"/>
-      <c r="KMW138" s="38"/>
-      <c r="KNE138" s="38"/>
-      <c r="KNM138" s="38"/>
-      <c r="KNU138" s="38"/>
-      <c r="KOC138" s="38"/>
-      <c r="KOK138" s="38"/>
-      <c r="KOS138" s="38"/>
-      <c r="KPA138" s="38"/>
-      <c r="KPI138" s="38"/>
-      <c r="KPQ138" s="38"/>
-      <c r="KPY138" s="38"/>
-      <c r="KQG138" s="38"/>
-      <c r="KQO138" s="38"/>
-      <c r="KQW138" s="38"/>
-      <c r="KRE138" s="38"/>
-      <c r="KRM138" s="38"/>
-      <c r="KRU138" s="38"/>
-      <c r="KSC138" s="38"/>
-      <c r="KSK138" s="38"/>
-      <c r="KSS138" s="38"/>
-      <c r="KTA138" s="38"/>
-      <c r="KTI138" s="38"/>
-      <c r="KTQ138" s="38"/>
-      <c r="KTY138" s="38"/>
-      <c r="KUG138" s="38"/>
-      <c r="KUO138" s="38"/>
-      <c r="KUW138" s="38"/>
-      <c r="KVE138" s="38"/>
-      <c r="KVM138" s="38"/>
-      <c r="KVU138" s="38"/>
-      <c r="KWC138" s="38"/>
-      <c r="KWK138" s="38"/>
-      <c r="KWS138" s="38"/>
-      <c r="KXA138" s="38"/>
-      <c r="KXI138" s="38"/>
-      <c r="KXQ138" s="38"/>
-      <c r="KXY138" s="38"/>
-      <c r="KYG138" s="38"/>
-      <c r="KYO138" s="38"/>
-      <c r="KYW138" s="38"/>
-      <c r="KZE138" s="38"/>
-      <c r="KZM138" s="38"/>
-      <c r="KZU138" s="38"/>
-      <c r="LAC138" s="38"/>
-      <c r="LAK138" s="38"/>
-      <c r="LAS138" s="38"/>
-      <c r="LBA138" s="38"/>
-      <c r="LBI138" s="38"/>
-      <c r="LBQ138" s="38"/>
-      <c r="LBY138" s="38"/>
-      <c r="LCG138" s="38"/>
-      <c r="LCO138" s="38"/>
-      <c r="LCW138" s="38"/>
-      <c r="LDE138" s="38"/>
-      <c r="LDM138" s="38"/>
-      <c r="LDU138" s="38"/>
-      <c r="LEC138" s="38"/>
-      <c r="LEK138" s="38"/>
-      <c r="LES138" s="38"/>
-      <c r="LFA138" s="38"/>
-      <c r="LFI138" s="38"/>
-      <c r="LFQ138" s="38"/>
-      <c r="LFY138" s="38"/>
-      <c r="LGG138" s="38"/>
-      <c r="LGO138" s="38"/>
-      <c r="LGW138" s="38"/>
-      <c r="LHE138" s="38"/>
-      <c r="LHM138" s="38"/>
-      <c r="LHU138" s="38"/>
-      <c r="LIC138" s="38"/>
-      <c r="LIK138" s="38"/>
-      <c r="LIS138" s="38"/>
-      <c r="LJA138" s="38"/>
-      <c r="LJI138" s="38"/>
-      <c r="LJQ138" s="38"/>
-      <c r="LJY138" s="38"/>
-      <c r="LKG138" s="38"/>
-      <c r="LKO138" s="38"/>
-      <c r="LKW138" s="38"/>
-      <c r="LLE138" s="38"/>
-      <c r="LLM138" s="38"/>
-      <c r="LLU138" s="38"/>
-      <c r="LMC138" s="38"/>
-      <c r="LMK138" s="38"/>
-      <c r="LMS138" s="38"/>
-      <c r="LNA138" s="38"/>
-      <c r="LNI138" s="38"/>
-      <c r="LNQ138" s="38"/>
-      <c r="LNY138" s="38"/>
-      <c r="LOG138" s="38"/>
-      <c r="LOO138" s="38"/>
-      <c r="LOW138" s="38"/>
-      <c r="LPE138" s="38"/>
-      <c r="LPM138" s="38"/>
-      <c r="LPU138" s="38"/>
-      <c r="LQC138" s="38"/>
-      <c r="LQK138" s="38"/>
-      <c r="LQS138" s="38"/>
-      <c r="LRA138" s="38"/>
-      <c r="LRI138" s="38"/>
-      <c r="LRQ138" s="38"/>
-      <c r="LRY138" s="38"/>
-      <c r="LSG138" s="38"/>
-      <c r="LSO138" s="38"/>
-      <c r="LSW138" s="38"/>
-      <c r="LTE138" s="38"/>
-      <c r="LTM138" s="38"/>
-      <c r="LTU138" s="38"/>
-      <c r="LUC138" s="38"/>
-      <c r="LUK138" s="38"/>
-      <c r="LUS138" s="38"/>
-      <c r="LVA138" s="38"/>
-      <c r="LVI138" s="38"/>
-      <c r="LVQ138" s="38"/>
-      <c r="LVY138" s="38"/>
-      <c r="LWG138" s="38"/>
-      <c r="LWO138" s="38"/>
-      <c r="LWW138" s="38"/>
-      <c r="LXE138" s="38"/>
-      <c r="LXM138" s="38"/>
-      <c r="LXU138" s="38"/>
-      <c r="LYC138" s="38"/>
-      <c r="LYK138" s="38"/>
-      <c r="LYS138" s="38"/>
-      <c r="LZA138" s="38"/>
-      <c r="LZI138" s="38"/>
-      <c r="LZQ138" s="38"/>
-      <c r="LZY138" s="38"/>
-      <c r="MAG138" s="38"/>
-      <c r="MAO138" s="38"/>
-      <c r="MAW138" s="38"/>
-      <c r="MBE138" s="38"/>
-      <c r="MBM138" s="38"/>
-      <c r="MBU138" s="38"/>
-      <c r="MCC138" s="38"/>
-      <c r="MCK138" s="38"/>
-      <c r="MCS138" s="38"/>
-      <c r="MDA138" s="38"/>
-      <c r="MDI138" s="38"/>
-      <c r="MDQ138" s="38"/>
-      <c r="MDY138" s="38"/>
-      <c r="MEG138" s="38"/>
-      <c r="MEO138" s="38"/>
-      <c r="MEW138" s="38"/>
-      <c r="MFE138" s="38"/>
-      <c r="MFM138" s="38"/>
-      <c r="MFU138" s="38"/>
-      <c r="MGC138" s="38"/>
-      <c r="MGK138" s="38"/>
-      <c r="MGS138" s="38"/>
-      <c r="MHA138" s="38"/>
-      <c r="MHI138" s="38"/>
-      <c r="MHQ138" s="38"/>
-      <c r="MHY138" s="38"/>
-      <c r="MIG138" s="38"/>
-      <c r="MIO138" s="38"/>
-      <c r="MIW138" s="38"/>
-      <c r="MJE138" s="38"/>
-      <c r="MJM138" s="38"/>
-      <c r="MJU138" s="38"/>
-      <c r="MKC138" s="38"/>
-      <c r="MKK138" s="38"/>
-      <c r="MKS138" s="38"/>
-      <c r="MLA138" s="38"/>
-      <c r="MLI138" s="38"/>
-      <c r="MLQ138" s="38"/>
-      <c r="MLY138" s="38"/>
-      <c r="MMG138" s="38"/>
-      <c r="MMO138" s="38"/>
-      <c r="MMW138" s="38"/>
-      <c r="MNE138" s="38"/>
-      <c r="MNM138" s="38"/>
-      <c r="MNU138" s="38"/>
-      <c r="MOC138" s="38"/>
-      <c r="MOK138" s="38"/>
-      <c r="MOS138" s="38"/>
-      <c r="MPA138" s="38"/>
-      <c r="MPI138" s="38"/>
-      <c r="MPQ138" s="38"/>
-      <c r="MPY138" s="38"/>
-      <c r="MQG138" s="38"/>
-      <c r="MQO138" s="38"/>
-      <c r="MQW138" s="38"/>
-      <c r="MRE138" s="38"/>
-      <c r="MRM138" s="38"/>
-      <c r="MRU138" s="38"/>
-      <c r="MSC138" s="38"/>
-      <c r="MSK138" s="38"/>
-      <c r="MSS138" s="38"/>
-      <c r="MTA138" s="38"/>
-      <c r="MTI138" s="38"/>
-      <c r="MTQ138" s="38"/>
-      <c r="MTY138" s="38"/>
-      <c r="MUG138" s="38"/>
-      <c r="MUO138" s="38"/>
-      <c r="MUW138" s="38"/>
-      <c r="MVE138" s="38"/>
-      <c r="MVM138" s="38"/>
-      <c r="MVU138" s="38"/>
-      <c r="MWC138" s="38"/>
-      <c r="MWK138" s="38"/>
-      <c r="MWS138" s="38"/>
-      <c r="MXA138" s="38"/>
-      <c r="MXI138" s="38"/>
-      <c r="MXQ138" s="38"/>
-      <c r="MXY138" s="38"/>
-      <c r="MYG138" s="38"/>
-      <c r="MYO138" s="38"/>
-      <c r="MYW138" s="38"/>
-      <c r="MZE138" s="38"/>
-      <c r="MZM138" s="38"/>
-      <c r="MZU138" s="38"/>
-      <c r="NAC138" s="38"/>
-      <c r="NAK138" s="38"/>
-      <c r="NAS138" s="38"/>
-      <c r="NBA138" s="38"/>
-      <c r="NBI138" s="38"/>
-      <c r="NBQ138" s="38"/>
-      <c r="NBY138" s="38"/>
-      <c r="NCG138" s="38"/>
-      <c r="NCO138" s="38"/>
-      <c r="NCW138" s="38"/>
-      <c r="NDE138" s="38"/>
-      <c r="NDM138" s="38"/>
-      <c r="NDU138" s="38"/>
-      <c r="NEC138" s="38"/>
-      <c r="NEK138" s="38"/>
-      <c r="NES138" s="38"/>
-      <c r="NFA138" s="38"/>
-      <c r="NFI138" s="38"/>
-      <c r="NFQ138" s="38"/>
-      <c r="NFY138" s="38"/>
-      <c r="NGG138" s="38"/>
-      <c r="NGO138" s="38"/>
-      <c r="NGW138" s="38"/>
-      <c r="NHE138" s="38"/>
-      <c r="NHM138" s="38"/>
-      <c r="NHU138" s="38"/>
-      <c r="NIC138" s="38"/>
-      <c r="NIK138" s="38"/>
-      <c r="NIS138" s="38"/>
-      <c r="NJA138" s="38"/>
-      <c r="NJI138" s="38"/>
-      <c r="NJQ138" s="38"/>
-      <c r="NJY138" s="38"/>
-      <c r="NKG138" s="38"/>
-      <c r="NKO138" s="38"/>
-      <c r="NKW138" s="38"/>
-      <c r="NLE138" s="38"/>
-      <c r="NLM138" s="38"/>
-      <c r="NLU138" s="38"/>
-      <c r="NMC138" s="38"/>
-      <c r="NMK138" s="38"/>
-      <c r="NMS138" s="38"/>
-      <c r="NNA138" s="38"/>
-      <c r="NNI138" s="38"/>
-      <c r="NNQ138" s="38"/>
-      <c r="NNY138" s="38"/>
-      <c r="NOG138" s="38"/>
-      <c r="NOO138" s="38"/>
-      <c r="NOW138" s="38"/>
-      <c r="NPE138" s="38"/>
-      <c r="NPM138" s="38"/>
-      <c r="NPU138" s="38"/>
-      <c r="NQC138" s="38"/>
-      <c r="NQK138" s="38"/>
-      <c r="NQS138" s="38"/>
-      <c r="NRA138" s="38"/>
-      <c r="NRI138" s="38"/>
-      <c r="NRQ138" s="38"/>
-      <c r="NRY138" s="38"/>
-      <c r="NSG138" s="38"/>
-      <c r="NSO138" s="38"/>
-      <c r="NSW138" s="38"/>
-      <c r="NTE138" s="38"/>
-      <c r="NTM138" s="38"/>
-      <c r="NTU138" s="38"/>
-      <c r="NUC138" s="38"/>
-      <c r="NUK138" s="38"/>
-      <c r="NUS138" s="38"/>
-      <c r="NVA138" s="38"/>
-      <c r="NVI138" s="38"/>
-      <c r="NVQ138" s="38"/>
-      <c r="NVY138" s="38"/>
-      <c r="NWG138" s="38"/>
-      <c r="NWO138" s="38"/>
-      <c r="NWW138" s="38"/>
-      <c r="NXE138" s="38"/>
-      <c r="NXM138" s="38"/>
-      <c r="NXU138" s="38"/>
-      <c r="NYC138" s="38"/>
-      <c r="NYK138" s="38"/>
-      <c r="NYS138" s="38"/>
-      <c r="NZA138" s="38"/>
-      <c r="NZI138" s="38"/>
-      <c r="NZQ138" s="38"/>
-      <c r="NZY138" s="38"/>
-      <c r="OAG138" s="38"/>
-      <c r="OAO138" s="38"/>
-      <c r="OAW138" s="38"/>
-      <c r="OBE138" s="38"/>
-      <c r="OBM138" s="38"/>
-      <c r="OBU138" s="38"/>
-      <c r="OCC138" s="38"/>
-      <c r="OCK138" s="38"/>
-      <c r="OCS138" s="38"/>
-      <c r="ODA138" s="38"/>
-      <c r="ODI138" s="38"/>
-      <c r="ODQ138" s="38"/>
-      <c r="ODY138" s="38"/>
-      <c r="OEG138" s="38"/>
-      <c r="OEO138" s="38"/>
-      <c r="OEW138" s="38"/>
-      <c r="OFE138" s="38"/>
-      <c r="OFM138" s="38"/>
-      <c r="OFU138" s="38"/>
-      <c r="OGC138" s="38"/>
-      <c r="OGK138" s="38"/>
-      <c r="OGS138" s="38"/>
-      <c r="OHA138" s="38"/>
-      <c r="OHI138" s="38"/>
-      <c r="OHQ138" s="38"/>
-      <c r="OHY138" s="38"/>
-      <c r="OIG138" s="38"/>
-      <c r="OIO138" s="38"/>
-      <c r="OIW138" s="38"/>
-      <c r="OJE138" s="38"/>
-      <c r="OJM138" s="38"/>
-      <c r="OJU138" s="38"/>
-      <c r="OKC138" s="38"/>
-      <c r="OKK138" s="38"/>
-      <c r="OKS138" s="38"/>
-      <c r="OLA138" s="38"/>
-      <c r="OLI138" s="38"/>
-      <c r="OLQ138" s="38"/>
-      <c r="OLY138" s="38"/>
-      <c r="OMG138" s="38"/>
-      <c r="OMO138" s="38"/>
-      <c r="OMW138" s="38"/>
-      <c r="ONE138" s="38"/>
-      <c r="ONM138" s="38"/>
-      <c r="ONU138" s="38"/>
-      <c r="OOC138" s="38"/>
-      <c r="OOK138" s="38"/>
-      <c r="OOS138" s="38"/>
-      <c r="OPA138" s="38"/>
-      <c r="OPI138" s="38"/>
-      <c r="OPQ138" s="38"/>
-      <c r="OPY138" s="38"/>
-      <c r="OQG138" s="38"/>
-      <c r="OQO138" s="38"/>
-      <c r="OQW138" s="38"/>
-      <c r="ORE138" s="38"/>
-      <c r="ORM138" s="38"/>
-      <c r="ORU138" s="38"/>
-      <c r="OSC138" s="38"/>
-      <c r="OSK138" s="38"/>
-      <c r="OSS138" s="38"/>
-      <c r="OTA138" s="38"/>
-      <c r="OTI138" s="38"/>
-      <c r="OTQ138" s="38"/>
-      <c r="OTY138" s="38"/>
-      <c r="OUG138" s="38"/>
-      <c r="OUO138" s="38"/>
-      <c r="OUW138" s="38"/>
-      <c r="OVE138" s="38"/>
-      <c r="OVM138" s="38"/>
-      <c r="OVU138" s="38"/>
-      <c r="OWC138" s="38"/>
-      <c r="OWK138" s="38"/>
-      <c r="OWS138" s="38"/>
-      <c r="OXA138" s="38"/>
-      <c r="OXI138" s="38"/>
-      <c r="OXQ138" s="38"/>
-      <c r="OXY138" s="38"/>
-      <c r="OYG138" s="38"/>
-      <c r="OYO138" s="38"/>
-      <c r="OYW138" s="38"/>
-      <c r="OZE138" s="38"/>
-      <c r="OZM138" s="38"/>
-      <c r="OZU138" s="38"/>
-      <c r="PAC138" s="38"/>
-      <c r="PAK138" s="38"/>
-      <c r="PAS138" s="38"/>
-      <c r="PBA138" s="38"/>
-      <c r="PBI138" s="38"/>
-      <c r="PBQ138" s="38"/>
-      <c r="PBY138" s="38"/>
-      <c r="PCG138" s="38"/>
-      <c r="PCO138" s="38"/>
-      <c r="PCW138" s="38"/>
-      <c r="PDE138" s="38"/>
-      <c r="PDM138" s="38"/>
-      <c r="PDU138" s="38"/>
-      <c r="PEC138" s="38"/>
-      <c r="PEK138" s="38"/>
-      <c r="PES138" s="38"/>
-      <c r="PFA138" s="38"/>
-      <c r="PFI138" s="38"/>
-      <c r="PFQ138" s="38"/>
-      <c r="PFY138" s="38"/>
-      <c r="PGG138" s="38"/>
-      <c r="PGO138" s="38"/>
-      <c r="PGW138" s="38"/>
-      <c r="PHE138" s="38"/>
-      <c r="PHM138" s="38"/>
-      <c r="PHU138" s="38"/>
-      <c r="PIC138" s="38"/>
-      <c r="PIK138" s="38"/>
-      <c r="PIS138" s="38"/>
-      <c r="PJA138" s="38"/>
-      <c r="PJI138" s="38"/>
-      <c r="PJQ138" s="38"/>
-      <c r="PJY138" s="38"/>
-      <c r="PKG138" s="38"/>
-      <c r="PKO138" s="38"/>
-      <c r="PKW138" s="38"/>
-      <c r="PLE138" s="38"/>
-      <c r="PLM138" s="38"/>
-      <c r="PLU138" s="38"/>
-      <c r="PMC138" s="38"/>
-      <c r="PMK138" s="38"/>
-      <c r="PMS138" s="38"/>
-      <c r="PNA138" s="38"/>
-      <c r="PNI138" s="38"/>
-      <c r="PNQ138" s="38"/>
-      <c r="PNY138" s="38"/>
-      <c r="POG138" s="38"/>
-      <c r="POO138" s="38"/>
-      <c r="POW138" s="38"/>
-      <c r="PPE138" s="38"/>
-      <c r="PPM138" s="38"/>
-      <c r="PPU138" s="38"/>
-      <c r="PQC138" s="38"/>
-      <c r="PQK138" s="38"/>
-      <c r="PQS138" s="38"/>
-      <c r="PRA138" s="38"/>
-      <c r="PRI138" s="38"/>
-      <c r="PRQ138" s="38"/>
-      <c r="PRY138" s="38"/>
-      <c r="PSG138" s="38"/>
-      <c r="PSO138" s="38"/>
-      <c r="PSW138" s="38"/>
-      <c r="PTE138" s="38"/>
-      <c r="PTM138" s="38"/>
-      <c r="PTU138" s="38"/>
-      <c r="PUC138" s="38"/>
-      <c r="PUK138" s="38"/>
-      <c r="PUS138" s="38"/>
-      <c r="PVA138" s="38"/>
-      <c r="PVI138" s="38"/>
-      <c r="PVQ138" s="38"/>
-      <c r="PVY138" s="38"/>
-      <c r="PWG138" s="38"/>
-      <c r="PWO138" s="38"/>
-      <c r="PWW138" s="38"/>
-      <c r="PXE138" s="38"/>
-      <c r="PXM138" s="38"/>
-      <c r="PXU138" s="38"/>
-      <c r="PYC138" s="38"/>
-      <c r="PYK138" s="38"/>
-      <c r="PYS138" s="38"/>
-      <c r="PZA138" s="38"/>
-      <c r="PZI138" s="38"/>
-      <c r="PZQ138" s="38"/>
-      <c r="PZY138" s="38"/>
-      <c r="QAG138" s="38"/>
-      <c r="QAO138" s="38"/>
-      <c r="QAW138" s="38"/>
-      <c r="QBE138" s="38"/>
-      <c r="QBM138" s="38"/>
-      <c r="QBU138" s="38"/>
-      <c r="QCC138" s="38"/>
-      <c r="QCK138" s="38"/>
-      <c r="QCS138" s="38"/>
-      <c r="QDA138" s="38"/>
-      <c r="QDI138" s="38"/>
-      <c r="QDQ138" s="38"/>
-      <c r="QDY138" s="38"/>
-      <c r="QEG138" s="38"/>
-      <c r="QEO138" s="38"/>
-      <c r="QEW138" s="38"/>
-      <c r="QFE138" s="38"/>
-      <c r="QFM138" s="38"/>
-      <c r="QFU138" s="38"/>
-      <c r="QGC138" s="38"/>
-      <c r="QGK138" s="38"/>
-      <c r="QGS138" s="38"/>
-      <c r="QHA138" s="38"/>
-      <c r="QHI138" s="38"/>
-      <c r="QHQ138" s="38"/>
-      <c r="QHY138" s="38"/>
-      <c r="QIG138" s="38"/>
-      <c r="QIO138" s="38"/>
-      <c r="QIW138" s="38"/>
-      <c r="QJE138" s="38"/>
-      <c r="QJM138" s="38"/>
-      <c r="QJU138" s="38"/>
-      <c r="QKC138" s="38"/>
-      <c r="QKK138" s="38"/>
-      <c r="QKS138" s="38"/>
-      <c r="QLA138" s="38"/>
-      <c r="QLI138" s="38"/>
-      <c r="QLQ138" s="38"/>
-      <c r="QLY138" s="38"/>
-      <c r="QMG138" s="38"/>
-      <c r="QMO138" s="38"/>
-      <c r="QMW138" s="38"/>
-      <c r="QNE138" s="38"/>
-      <c r="QNM138" s="38"/>
-      <c r="QNU138" s="38"/>
-      <c r="QOC138" s="38"/>
-      <c r="QOK138" s="38"/>
-      <c r="QOS138" s="38"/>
-      <c r="QPA138" s="38"/>
-      <c r="QPI138" s="38"/>
-      <c r="QPQ138" s="38"/>
-      <c r="QPY138" s="38"/>
-      <c r="QQG138" s="38"/>
-      <c r="QQO138" s="38"/>
-      <c r="QQW138" s="38"/>
-      <c r="QRE138" s="38"/>
-      <c r="QRM138" s="38"/>
-      <c r="QRU138" s="38"/>
-      <c r="QSC138" s="38"/>
-      <c r="QSK138" s="38"/>
-      <c r="QSS138" s="38"/>
-      <c r="QTA138" s="38"/>
-      <c r="QTI138" s="38"/>
-      <c r="QTQ138" s="38"/>
-      <c r="QTY138" s="38"/>
-      <c r="QUG138" s="38"/>
-      <c r="QUO138" s="38"/>
-      <c r="QUW138" s="38"/>
-      <c r="QVE138" s="38"/>
-      <c r="QVM138" s="38"/>
-      <c r="QVU138" s="38"/>
-      <c r="QWC138" s="38"/>
-      <c r="QWK138" s="38"/>
-      <c r="QWS138" s="38"/>
-      <c r="QXA138" s="38"/>
-      <c r="QXI138" s="38"/>
-      <c r="QXQ138" s="38"/>
-      <c r="QXY138" s="38"/>
-      <c r="QYG138" s="38"/>
-      <c r="QYO138" s="38"/>
-      <c r="QYW138" s="38"/>
-      <c r="QZE138" s="38"/>
-      <c r="QZM138" s="38"/>
-      <c r="QZU138" s="38"/>
-      <c r="RAC138" s="38"/>
-      <c r="RAK138" s="38"/>
-      <c r="RAS138" s="38"/>
-      <c r="RBA138" s="38"/>
-      <c r="RBI138" s="38"/>
-      <c r="RBQ138" s="38"/>
-      <c r="RBY138" s="38"/>
-      <c r="RCG138" s="38"/>
-      <c r="RCO138" s="38"/>
-      <c r="RCW138" s="38"/>
-      <c r="RDE138" s="38"/>
-      <c r="RDM138" s="38"/>
-      <c r="RDU138" s="38"/>
-      <c r="REC138" s="38"/>
-      <c r="REK138" s="38"/>
-      <c r="RES138" s="38"/>
-      <c r="RFA138" s="38"/>
-      <c r="RFI138" s="38"/>
-      <c r="RFQ138" s="38"/>
-      <c r="RFY138" s="38"/>
-      <c r="RGG138" s="38"/>
-      <c r="RGO138" s="38"/>
-      <c r="RGW138" s="38"/>
-      <c r="RHE138" s="38"/>
-      <c r="RHM138" s="38"/>
-      <c r="RHU138" s="38"/>
-      <c r="RIC138" s="38"/>
-      <c r="RIK138" s="38"/>
-      <c r="RIS138" s="38"/>
-      <c r="RJA138" s="38"/>
-      <c r="RJI138" s="38"/>
-      <c r="RJQ138" s="38"/>
-      <c r="RJY138" s="38"/>
-      <c r="RKG138" s="38"/>
-      <c r="RKO138" s="38"/>
-      <c r="RKW138" s="38"/>
-      <c r="RLE138" s="38"/>
-      <c r="RLM138" s="38"/>
-      <c r="RLU138" s="38"/>
-      <c r="RMC138" s="38"/>
-      <c r="RMK138" s="38"/>
-      <c r="RMS138" s="38"/>
-      <c r="RNA138" s="38"/>
-      <c r="RNI138" s="38"/>
-      <c r="RNQ138" s="38"/>
-      <c r="RNY138" s="38"/>
-      <c r="ROG138" s="38"/>
-      <c r="ROO138" s="38"/>
-      <c r="ROW138" s="38"/>
-      <c r="RPE138" s="38"/>
-      <c r="RPM138" s="38"/>
-      <c r="RPU138" s="38"/>
-      <c r="RQC138" s="38"/>
-      <c r="RQK138" s="38"/>
-      <c r="RQS138" s="38"/>
-      <c r="RRA138" s="38"/>
-      <c r="RRI138" s="38"/>
-      <c r="RRQ138" s="38"/>
-      <c r="RRY138" s="38"/>
-      <c r="RSG138" s="38"/>
-      <c r="RSO138" s="38"/>
-      <c r="RSW138" s="38"/>
-      <c r="RTE138" s="38"/>
-      <c r="RTM138" s="38"/>
-      <c r="RTU138" s="38"/>
-      <c r="RUC138" s="38"/>
-      <c r="RUK138" s="38"/>
-      <c r="RUS138" s="38"/>
-      <c r="RVA138" s="38"/>
-      <c r="RVI138" s="38"/>
-      <c r="RVQ138" s="38"/>
-      <c r="RVY138" s="38"/>
-      <c r="RWG138" s="38"/>
-      <c r="RWO138" s="38"/>
-      <c r="RWW138" s="38"/>
-      <c r="RXE138" s="38"/>
-      <c r="RXM138" s="38"/>
-      <c r="RXU138" s="38"/>
-      <c r="RYC138" s="38"/>
-      <c r="RYK138" s="38"/>
-      <c r="RYS138" s="38"/>
-      <c r="RZA138" s="38"/>
-      <c r="RZI138" s="38"/>
-      <c r="RZQ138" s="38"/>
-      <c r="RZY138" s="38"/>
-      <c r="SAG138" s="38"/>
-      <c r="SAO138" s="38"/>
-      <c r="SAW138" s="38"/>
-      <c r="SBE138" s="38"/>
-      <c r="SBM138" s="38"/>
-      <c r="SBU138" s="38"/>
-      <c r="SCC138" s="38"/>
-      <c r="SCK138" s="38"/>
-      <c r="SCS138" s="38"/>
-      <c r="SDA138" s="38"/>
-      <c r="SDI138" s="38"/>
-      <c r="SDQ138" s="38"/>
-      <c r="SDY138" s="38"/>
-      <c r="SEG138" s="38"/>
-      <c r="SEO138" s="38"/>
-      <c r="SEW138" s="38"/>
-      <c r="SFE138" s="38"/>
-      <c r="SFM138" s="38"/>
-      <c r="SFU138" s="38"/>
-      <c r="SGC138" s="38"/>
-      <c r="SGK138" s="38"/>
-      <c r="SGS138" s="38"/>
-      <c r="SHA138" s="38"/>
-      <c r="SHI138" s="38"/>
-      <c r="SHQ138" s="38"/>
-      <c r="SHY138" s="38"/>
-      <c r="SIG138" s="38"/>
-      <c r="SIO138" s="38"/>
-      <c r="SIW138" s="38"/>
-      <c r="SJE138" s="38"/>
-      <c r="SJM138" s="38"/>
-      <c r="SJU138" s="38"/>
-      <c r="SKC138" s="38"/>
-      <c r="SKK138" s="38"/>
-      <c r="SKS138" s="38"/>
-      <c r="SLA138" s="38"/>
-      <c r="SLI138" s="38"/>
-      <c r="SLQ138" s="38"/>
-      <c r="SLY138" s="38"/>
-      <c r="SMG138" s="38"/>
-      <c r="SMO138" s="38"/>
-      <c r="SMW138" s="38"/>
-      <c r="SNE138" s="38"/>
-      <c r="SNM138" s="38"/>
-      <c r="SNU138" s="38"/>
-      <c r="SOC138" s="38"/>
-      <c r="SOK138" s="38"/>
-      <c r="SOS138" s="38"/>
-      <c r="SPA138" s="38"/>
-      <c r="SPI138" s="38"/>
-      <c r="SPQ138" s="38"/>
-      <c r="SPY138" s="38"/>
-      <c r="SQG138" s="38"/>
-      <c r="SQO138" s="38"/>
-      <c r="SQW138" s="38"/>
-      <c r="SRE138" s="38"/>
-      <c r="SRM138" s="38"/>
-      <c r="SRU138" s="38"/>
-      <c r="SSC138" s="38"/>
-      <c r="SSK138" s="38"/>
-      <c r="SSS138" s="38"/>
-      <c r="STA138" s="38"/>
-      <c r="STI138" s="38"/>
-      <c r="STQ138" s="38"/>
-      <c r="STY138" s="38"/>
-      <c r="SUG138" s="38"/>
-      <c r="SUO138" s="38"/>
-      <c r="SUW138" s="38"/>
-      <c r="SVE138" s="38"/>
-      <c r="SVM138" s="38"/>
-      <c r="SVU138" s="38"/>
-      <c r="SWC138" s="38"/>
-      <c r="SWK138" s="38"/>
-      <c r="SWS138" s="38"/>
-      <c r="SXA138" s="38"/>
-      <c r="SXI138" s="38"/>
-      <c r="SXQ138" s="38"/>
-      <c r="SXY138" s="38"/>
-      <c r="SYG138" s="38"/>
-      <c r="SYO138" s="38"/>
-      <c r="SYW138" s="38"/>
-      <c r="SZE138" s="38"/>
-      <c r="SZM138" s="38"/>
-      <c r="SZU138" s="38"/>
-      <c r="TAC138" s="38"/>
-      <c r="TAK138" s="38"/>
-      <c r="TAS138" s="38"/>
-      <c r="TBA138" s="38"/>
-      <c r="TBI138" s="38"/>
-      <c r="TBQ138" s="38"/>
-      <c r="TBY138" s="38"/>
-      <c r="TCG138" s="38"/>
-      <c r="TCO138" s="38"/>
-      <c r="TCW138" s="38"/>
-      <c r="TDE138" s="38"/>
-      <c r="TDM138" s="38"/>
-      <c r="TDU138" s="38"/>
-      <c r="TEC138" s="38"/>
-      <c r="TEK138" s="38"/>
-      <c r="TES138" s="38"/>
-      <c r="TFA138" s="38"/>
-      <c r="TFI138" s="38"/>
-      <c r="TFQ138" s="38"/>
-      <c r="TFY138" s="38"/>
-      <c r="TGG138" s="38"/>
-      <c r="TGO138" s="38"/>
-      <c r="TGW138" s="38"/>
-      <c r="THE138" s="38"/>
-      <c r="THM138" s="38"/>
-      <c r="THU138" s="38"/>
-      <c r="TIC138" s="38"/>
-      <c r="TIK138" s="38"/>
-      <c r="TIS138" s="38"/>
-      <c r="TJA138" s="38"/>
-      <c r="TJI138" s="38"/>
-      <c r="TJQ138" s="38"/>
-      <c r="TJY138" s="38"/>
-      <c r="TKG138" s="38"/>
-      <c r="TKO138" s="38"/>
-      <c r="TKW138" s="38"/>
-      <c r="TLE138" s="38"/>
-      <c r="TLM138" s="38"/>
-      <c r="TLU138" s="38"/>
-      <c r="TMC138" s="38"/>
-      <c r="TMK138" s="38"/>
-      <c r="TMS138" s="38"/>
-      <c r="TNA138" s="38"/>
-      <c r="TNI138" s="38"/>
-      <c r="TNQ138" s="38"/>
-      <c r="TNY138" s="38"/>
-      <c r="TOG138" s="38"/>
-      <c r="TOO138" s="38"/>
-      <c r="TOW138" s="38"/>
-      <c r="TPE138" s="38"/>
-      <c r="TPM138" s="38"/>
-      <c r="TPU138" s="38"/>
-      <c r="TQC138" s="38"/>
-      <c r="TQK138" s="38"/>
-      <c r="TQS138" s="38"/>
-      <c r="TRA138" s="38"/>
-      <c r="TRI138" s="38"/>
-      <c r="TRQ138" s="38"/>
-      <c r="TRY138" s="38"/>
-      <c r="TSG138" s="38"/>
-      <c r="TSO138" s="38"/>
-      <c r="TSW138" s="38"/>
-      <c r="TTE138" s="38"/>
-      <c r="TTM138" s="38"/>
-      <c r="TTU138" s="38"/>
-      <c r="TUC138" s="38"/>
-      <c r="TUK138" s="38"/>
-      <c r="TUS138" s="38"/>
-      <c r="TVA138" s="38"/>
-      <c r="TVI138" s="38"/>
-      <c r="TVQ138" s="38"/>
-      <c r="TVY138" s="38"/>
-      <c r="TWG138" s="38"/>
-      <c r="TWO138" s="38"/>
-      <c r="TWW138" s="38"/>
-      <c r="TXE138" s="38"/>
-      <c r="TXM138" s="38"/>
-      <c r="TXU138" s="38"/>
-      <c r="TYC138" s="38"/>
-      <c r="TYK138" s="38"/>
-      <c r="TYS138" s="38"/>
-      <c r="TZA138" s="38"/>
-      <c r="TZI138" s="38"/>
-      <c r="TZQ138" s="38"/>
-      <c r="TZY138" s="38"/>
-      <c r="UAG138" s="38"/>
-      <c r="UAO138" s="38"/>
-      <c r="UAW138" s="38"/>
-      <c r="UBE138" s="38"/>
-      <c r="UBM138" s="38"/>
-      <c r="UBU138" s="38"/>
-      <c r="UCC138" s="38"/>
-      <c r="UCK138" s="38"/>
-      <c r="UCS138" s="38"/>
-      <c r="UDA138" s="38"/>
-      <c r="UDI138" s="38"/>
-      <c r="UDQ138" s="38"/>
-      <c r="UDY138" s="38"/>
-      <c r="UEG138" s="38"/>
-      <c r="UEO138" s="38"/>
-      <c r="UEW138" s="38"/>
-      <c r="UFE138" s="38"/>
-      <c r="UFM138" s="38"/>
-      <c r="UFU138" s="38"/>
-      <c r="UGC138" s="38"/>
-      <c r="UGK138" s="38"/>
-      <c r="UGS138" s="38"/>
-      <c r="UHA138" s="38"/>
-      <c r="UHI138" s="38"/>
-      <c r="UHQ138" s="38"/>
-      <c r="UHY138" s="38"/>
-      <c r="UIG138" s="38"/>
-      <c r="UIO138" s="38"/>
-      <c r="UIW138" s="38"/>
-      <c r="UJE138" s="38"/>
-      <c r="UJM138" s="38"/>
-      <c r="UJU138" s="38"/>
-      <c r="UKC138" s="38"/>
-      <c r="UKK138" s="38"/>
-      <c r="UKS138" s="38"/>
-      <c r="ULA138" s="38"/>
-      <c r="ULI138" s="38"/>
-      <c r="ULQ138" s="38"/>
-      <c r="ULY138" s="38"/>
-      <c r="UMG138" s="38"/>
-      <c r="UMO138" s="38"/>
-      <c r="UMW138" s="38"/>
-      <c r="UNE138" s="38"/>
-      <c r="UNM138" s="38"/>
-      <c r="UNU138" s="38"/>
-      <c r="UOC138" s="38"/>
-      <c r="UOK138" s="38"/>
-      <c r="UOS138" s="38"/>
-      <c r="UPA138" s="38"/>
-      <c r="UPI138" s="38"/>
-      <c r="UPQ138" s="38"/>
-      <c r="UPY138" s="38"/>
-      <c r="UQG138" s="38"/>
-      <c r="UQO138" s="38"/>
-      <c r="UQW138" s="38"/>
-      <c r="URE138" s="38"/>
-      <c r="URM138" s="38"/>
-      <c r="URU138" s="38"/>
-      <c r="USC138" s="38"/>
-      <c r="USK138" s="38"/>
-      <c r="USS138" s="38"/>
-      <c r="UTA138" s="38"/>
-      <c r="UTI138" s="38"/>
-      <c r="UTQ138" s="38"/>
-      <c r="UTY138" s="38"/>
-      <c r="UUG138" s="38"/>
-      <c r="UUO138" s="38"/>
-      <c r="UUW138" s="38"/>
-      <c r="UVE138" s="38"/>
-      <c r="UVM138" s="38"/>
-      <c r="UVU138" s="38"/>
-      <c r="UWC138" s="38"/>
-      <c r="UWK138" s="38"/>
-      <c r="UWS138" s="38"/>
-      <c r="UXA138" s="38"/>
-      <c r="UXI138" s="38"/>
-      <c r="UXQ138" s="38"/>
-      <c r="UXY138" s="38"/>
-      <c r="UYG138" s="38"/>
-      <c r="UYO138" s="38"/>
-      <c r="UYW138" s="38"/>
-      <c r="UZE138" s="38"/>
-      <c r="UZM138" s="38"/>
-      <c r="UZU138" s="38"/>
-      <c r="VAC138" s="38"/>
-      <c r="VAK138" s="38"/>
-      <c r="VAS138" s="38"/>
-      <c r="VBA138" s="38"/>
-      <c r="VBI138" s="38"/>
-      <c r="VBQ138" s="38"/>
-      <c r="VBY138" s="38"/>
-      <c r="VCG138" s="38"/>
-      <c r="VCO138" s="38"/>
-      <c r="VCW138" s="38"/>
-      <c r="VDE138" s="38"/>
-      <c r="VDM138" s="38"/>
-      <c r="VDU138" s="38"/>
-      <c r="VEC138" s="38"/>
-      <c r="VEK138" s="38"/>
-      <c r="VES138" s="38"/>
-      <c r="VFA138" s="38"/>
-      <c r="VFI138" s="38"/>
-      <c r="VFQ138" s="38"/>
-      <c r="VFY138" s="38"/>
-      <c r="VGG138" s="38"/>
-      <c r="VGO138" s="38"/>
-      <c r="VGW138" s="38"/>
-      <c r="VHE138" s="38"/>
-      <c r="VHM138" s="38"/>
-      <c r="VHU138" s="38"/>
-      <c r="VIC138" s="38"/>
-      <c r="VIK138" s="38"/>
-      <c r="VIS138" s="38"/>
-      <c r="VJA138" s="38"/>
-      <c r="VJI138" s="38"/>
-      <c r="VJQ138" s="38"/>
-      <c r="VJY138" s="38"/>
-      <c r="VKG138" s="38"/>
-      <c r="VKO138" s="38"/>
-      <c r="VKW138" s="38"/>
-      <c r="VLE138" s="38"/>
-      <c r="VLM138" s="38"/>
-      <c r="VLU138" s="38"/>
-      <c r="VMC138" s="38"/>
-      <c r="VMK138" s="38"/>
-      <c r="VMS138" s="38"/>
-      <c r="VNA138" s="38"/>
-      <c r="VNI138" s="38"/>
-      <c r="VNQ138" s="38"/>
-      <c r="VNY138" s="38"/>
-      <c r="VOG138" s="38"/>
-      <c r="VOO138" s="38"/>
-      <c r="VOW138" s="38"/>
-      <c r="VPE138" s="38"/>
-      <c r="VPM138" s="38"/>
-      <c r="VPU138" s="38"/>
-      <c r="VQC138" s="38"/>
-      <c r="VQK138" s="38"/>
-      <c r="VQS138" s="38"/>
-      <c r="VRA138" s="38"/>
-      <c r="VRI138" s="38"/>
-      <c r="VRQ138" s="38"/>
-      <c r="VRY138" s="38"/>
-      <c r="VSG138" s="38"/>
-      <c r="VSO138" s="38"/>
-      <c r="VSW138" s="38"/>
-      <c r="VTE138" s="38"/>
-      <c r="VTM138" s="38"/>
-      <c r="VTU138" s="38"/>
-      <c r="VUC138" s="38"/>
-      <c r="VUK138" s="38"/>
-      <c r="VUS138" s="38"/>
-      <c r="VVA138" s="38"/>
-      <c r="VVI138" s="38"/>
-      <c r="VVQ138" s="38"/>
-      <c r="VVY138" s="38"/>
-      <c r="VWG138" s="38"/>
-      <c r="VWO138" s="38"/>
-      <c r="VWW138" s="38"/>
-      <c r="VXE138" s="38"/>
-      <c r="VXM138" s="38"/>
-      <c r="VXU138" s="38"/>
-      <c r="VYC138" s="38"/>
-      <c r="VYK138" s="38"/>
-      <c r="VYS138" s="38"/>
-      <c r="VZA138" s="38"/>
-      <c r="VZI138" s="38"/>
-      <c r="VZQ138" s="38"/>
-      <c r="VZY138" s="38"/>
-      <c r="WAG138" s="38"/>
-      <c r="WAO138" s="38"/>
-      <c r="WAW138" s="38"/>
-      <c r="WBE138" s="38"/>
-      <c r="WBM138" s="38"/>
-      <c r="WBU138" s="38"/>
-      <c r="WCC138" s="38"/>
-      <c r="WCK138" s="38"/>
-      <c r="WCS138" s="38"/>
-      <c r="WDA138" s="38"/>
-      <c r="WDI138" s="38"/>
-      <c r="WDQ138" s="38"/>
-      <c r="WDY138" s="38"/>
-      <c r="WEG138" s="38"/>
-      <c r="WEO138" s="38"/>
-      <c r="WEW138" s="38"/>
-      <c r="WFE138" s="38"/>
-      <c r="WFM138" s="38"/>
-      <c r="WFU138" s="38"/>
-      <c r="WGC138" s="38"/>
-      <c r="WGK138" s="38"/>
-      <c r="WGS138" s="38"/>
-      <c r="WHA138" s="38"/>
-      <c r="WHI138" s="38"/>
-      <c r="WHQ138" s="38"/>
-      <c r="WHY138" s="38"/>
-      <c r="WIG138" s="38"/>
-      <c r="WIO138" s="38"/>
-      <c r="WIW138" s="38"/>
-      <c r="WJE138" s="38"/>
-      <c r="WJM138" s="38"/>
-      <c r="WJU138" s="38"/>
-      <c r="WKC138" s="38"/>
-      <c r="WKK138" s="38"/>
-      <c r="WKS138" s="38"/>
-      <c r="WLA138" s="38"/>
-      <c r="WLI138" s="38"/>
-      <c r="WLQ138" s="38"/>
-      <c r="WLY138" s="38"/>
-      <c r="WMG138" s="38"/>
-      <c r="WMO138" s="38"/>
-      <c r="WMW138" s="38"/>
-      <c r="WNE138" s="38"/>
-      <c r="WNM138" s="38"/>
-      <c r="WNU138" s="38"/>
-      <c r="WOC138" s="38"/>
-      <c r="WOK138" s="38"/>
-      <c r="WOS138" s="38"/>
-      <c r="WPA138" s="38"/>
-      <c r="WPI138" s="38"/>
-      <c r="WPQ138" s="38"/>
-      <c r="WPY138" s="38"/>
-      <c r="WQG138" s="38"/>
-      <c r="WQO138" s="38"/>
-      <c r="WQW138" s="38"/>
-      <c r="WRE138" s="38"/>
-      <c r="WRM138" s="38"/>
-      <c r="WRU138" s="38"/>
-      <c r="WSC138" s="38"/>
-      <c r="WSK138" s="38"/>
-      <c r="WSS138" s="38"/>
-      <c r="WTA138" s="38"/>
-      <c r="WTI138" s="38"/>
-      <c r="WTQ138" s="38"/>
-      <c r="WTY138" s="38"/>
-      <c r="WUG138" s="38"/>
-      <c r="WUO138" s="38"/>
-      <c r="WUW138" s="38"/>
-      <c r="WVE138" s="38"/>
-      <c r="WVM138" s="38"/>
-      <c r="WVU138" s="38"/>
-      <c r="WWC138" s="38"/>
-      <c r="WWK138" s="38"/>
-      <c r="WWS138" s="38"/>
-      <c r="WXA138" s="38"/>
-      <c r="WXI138" s="38"/>
-      <c r="WXQ138" s="38"/>
-      <c r="WXY138" s="38"/>
-      <c r="WYG138" s="38"/>
-      <c r="WYO138" s="38"/>
-      <c r="WYW138" s="38"/>
-      <c r="WZE138" s="38"/>
-      <c r="WZM138" s="38"/>
-      <c r="WZU138" s="38"/>
-      <c r="XAC138" s="38"/>
-      <c r="XAK138" s="38"/>
-      <c r="XAS138" s="38"/>
-      <c r="XBA138" s="38"/>
-      <c r="XBI138" s="38"/>
-      <c r="XBQ138" s="38"/>
-      <c r="XBY138" s="38"/>
-      <c r="XCG138" s="38"/>
-      <c r="XCO138" s="38"/>
-      <c r="XCW138" s="38"/>
-      <c r="XDE138" s="38"/>
-      <c r="XDM138" s="38"/>
-      <c r="XDU138" s="38"/>
-      <c r="XEC138" s="38"/>
-      <c r="XEK138" s="38"/>
-      <c r="XES138" s="38"/>
-      <c r="XFA138" s="38"/>
+      <c r="M138" s="37"/>
+      <c r="U138" s="37"/>
+      <c r="AC138" s="37"/>
+      <c r="AK138" s="37"/>
+      <c r="AS138" s="37"/>
+      <c r="BA138" s="37"/>
+      <c r="BI138" s="37"/>
+      <c r="BQ138" s="37"/>
+      <c r="BY138" s="37"/>
+      <c r="CG138" s="37"/>
+      <c r="CO138" s="37"/>
+      <c r="CW138" s="37"/>
+      <c r="DE138" s="37"/>
+      <c r="DM138" s="37"/>
+      <c r="DU138" s="37"/>
+      <c r="EC138" s="37"/>
+      <c r="EK138" s="37"/>
+      <c r="ES138" s="37"/>
+      <c r="FA138" s="37"/>
+      <c r="FI138" s="37"/>
+      <c r="FQ138" s="37"/>
+      <c r="FY138" s="37"/>
+      <c r="GG138" s="37"/>
+      <c r="GO138" s="37"/>
+      <c r="GW138" s="37"/>
+      <c r="HE138" s="37"/>
+      <c r="HM138" s="37"/>
+      <c r="HU138" s="37"/>
+      <c r="IC138" s="37"/>
+      <c r="IK138" s="37"/>
+      <c r="IS138" s="37"/>
+      <c r="JA138" s="37"/>
+      <c r="JI138" s="37"/>
+      <c r="JQ138" s="37"/>
+      <c r="JY138" s="37"/>
+      <c r="KG138" s="37"/>
+      <c r="KO138" s="37"/>
+      <c r="KW138" s="37"/>
+      <c r="LE138" s="37"/>
+      <c r="LM138" s="37"/>
+      <c r="LU138" s="37"/>
+      <c r="MC138" s="37"/>
+      <c r="MK138" s="37"/>
+      <c r="MS138" s="37"/>
+      <c r="NA138" s="37"/>
+      <c r="NI138" s="37"/>
+      <c r="NQ138" s="37"/>
+      <c r="NY138" s="37"/>
+      <c r="OG138" s="37"/>
+      <c r="OO138" s="37"/>
+      <c r="OW138" s="37"/>
+      <c r="PE138" s="37"/>
+      <c r="PM138" s="37"/>
+      <c r="PU138" s="37"/>
+      <c r="QC138" s="37"/>
+      <c r="QK138" s="37"/>
+      <c r="QS138" s="37"/>
+      <c r="RA138" s="37"/>
+      <c r="RI138" s="37"/>
+      <c r="RQ138" s="37"/>
+      <c r="RY138" s="37"/>
+      <c r="SG138" s="37"/>
+      <c r="SO138" s="37"/>
+      <c r="SW138" s="37"/>
+      <c r="TE138" s="37"/>
+      <c r="TM138" s="37"/>
+      <c r="TU138" s="37"/>
+      <c r="UC138" s="37"/>
+      <c r="UK138" s="37"/>
+      <c r="US138" s="37"/>
+      <c r="VA138" s="37"/>
+      <c r="VI138" s="37"/>
+      <c r="VQ138" s="37"/>
+      <c r="VY138" s="37"/>
+      <c r="WG138" s="37"/>
+      <c r="WO138" s="37"/>
+      <c r="WW138" s="37"/>
+      <c r="XE138" s="37"/>
+      <c r="XM138" s="37"/>
+      <c r="XU138" s="37"/>
+      <c r="YC138" s="37"/>
+      <c r="YK138" s="37"/>
+      <c r="YS138" s="37"/>
+      <c r="ZA138" s="37"/>
+      <c r="ZI138" s="37"/>
+      <c r="ZQ138" s="37"/>
+      <c r="ZY138" s="37"/>
+      <c r="AAG138" s="37"/>
+      <c r="AAO138" s="37"/>
+      <c r="AAW138" s="37"/>
+      <c r="ABE138" s="37"/>
+      <c r="ABM138" s="37"/>
+      <c r="ABU138" s="37"/>
+      <c r="ACC138" s="37"/>
+      <c r="ACK138" s="37"/>
+      <c r="ACS138" s="37"/>
+      <c r="ADA138" s="37"/>
+      <c r="ADI138" s="37"/>
+      <c r="ADQ138" s="37"/>
+      <c r="ADY138" s="37"/>
+      <c r="AEG138" s="37"/>
+      <c r="AEO138" s="37"/>
+      <c r="AEW138" s="37"/>
+      <c r="AFE138" s="37"/>
+      <c r="AFM138" s="37"/>
+      <c r="AFU138" s="37"/>
+      <c r="AGC138" s="37"/>
+      <c r="AGK138" s="37"/>
+      <c r="AGS138" s="37"/>
+      <c r="AHA138" s="37"/>
+      <c r="AHI138" s="37"/>
+      <c r="AHQ138" s="37"/>
+      <c r="AHY138" s="37"/>
+      <c r="AIG138" s="37"/>
+      <c r="AIO138" s="37"/>
+      <c r="AIW138" s="37"/>
+      <c r="AJE138" s="37"/>
+      <c r="AJM138" s="37"/>
+      <c r="AJU138" s="37"/>
+      <c r="AKC138" s="37"/>
+      <c r="AKK138" s="37"/>
+      <c r="AKS138" s="37"/>
+      <c r="ALA138" s="37"/>
+      <c r="ALI138" s="37"/>
+      <c r="ALQ138" s="37"/>
+      <c r="ALY138" s="37"/>
+      <c r="AMG138" s="37"/>
+      <c r="AMO138" s="37"/>
+      <c r="AMW138" s="37"/>
+      <c r="ANE138" s="37"/>
+      <c r="ANM138" s="37"/>
+      <c r="ANU138" s="37"/>
+      <c r="AOC138" s="37"/>
+      <c r="AOK138" s="37"/>
+      <c r="AOS138" s="37"/>
+      <c r="APA138" s="37"/>
+      <c r="API138" s="37"/>
+      <c r="APQ138" s="37"/>
+      <c r="APY138" s="37"/>
+      <c r="AQG138" s="37"/>
+      <c r="AQO138" s="37"/>
+      <c r="AQW138" s="37"/>
+      <c r="ARE138" s="37"/>
+      <c r="ARM138" s="37"/>
+      <c r="ARU138" s="37"/>
+      <c r="ASC138" s="37"/>
+      <c r="ASK138" s="37"/>
+      <c r="ASS138" s="37"/>
+      <c r="ATA138" s="37"/>
+      <c r="ATI138" s="37"/>
+      <c r="ATQ138" s="37"/>
+      <c r="ATY138" s="37"/>
+      <c r="AUG138" s="37"/>
+      <c r="AUO138" s="37"/>
+      <c r="AUW138" s="37"/>
+      <c r="AVE138" s="37"/>
+      <c r="AVM138" s="37"/>
+      <c r="AVU138" s="37"/>
+      <c r="AWC138" s="37"/>
+      <c r="AWK138" s="37"/>
+      <c r="AWS138" s="37"/>
+      <c r="AXA138" s="37"/>
+      <c r="AXI138" s="37"/>
+      <c r="AXQ138" s="37"/>
+      <c r="AXY138" s="37"/>
+      <c r="AYG138" s="37"/>
+      <c r="AYO138" s="37"/>
+      <c r="AYW138" s="37"/>
+      <c r="AZE138" s="37"/>
+      <c r="AZM138" s="37"/>
+      <c r="AZU138" s="37"/>
+      <c r="BAC138" s="37"/>
+      <c r="BAK138" s="37"/>
+      <c r="BAS138" s="37"/>
+      <c r="BBA138" s="37"/>
+      <c r="BBI138" s="37"/>
+      <c r="BBQ138" s="37"/>
+      <c r="BBY138" s="37"/>
+      <c r="BCG138" s="37"/>
+      <c r="BCO138" s="37"/>
+      <c r="BCW138" s="37"/>
+      <c r="BDE138" s="37"/>
+      <c r="BDM138" s="37"/>
+      <c r="BDU138" s="37"/>
+      <c r="BEC138" s="37"/>
+      <c r="BEK138" s="37"/>
+      <c r="BES138" s="37"/>
+      <c r="BFA138" s="37"/>
+      <c r="BFI138" s="37"/>
+      <c r="BFQ138" s="37"/>
+      <c r="BFY138" s="37"/>
+      <c r="BGG138" s="37"/>
+      <c r="BGO138" s="37"/>
+      <c r="BGW138" s="37"/>
+      <c r="BHE138" s="37"/>
+      <c r="BHM138" s="37"/>
+      <c r="BHU138" s="37"/>
+      <c r="BIC138" s="37"/>
+      <c r="BIK138" s="37"/>
+      <c r="BIS138" s="37"/>
+      <c r="BJA138" s="37"/>
+      <c r="BJI138" s="37"/>
+      <c r="BJQ138" s="37"/>
+      <c r="BJY138" s="37"/>
+      <c r="BKG138" s="37"/>
+      <c r="BKO138" s="37"/>
+      <c r="BKW138" s="37"/>
+      <c r="BLE138" s="37"/>
+      <c r="BLM138" s="37"/>
+      <c r="BLU138" s="37"/>
+      <c r="BMC138" s="37"/>
+      <c r="BMK138" s="37"/>
+      <c r="BMS138" s="37"/>
+      <c r="BNA138" s="37"/>
+      <c r="BNI138" s="37"/>
+      <c r="BNQ138" s="37"/>
+      <c r="BNY138" s="37"/>
+      <c r="BOG138" s="37"/>
+      <c r="BOO138" s="37"/>
+      <c r="BOW138" s="37"/>
+      <c r="BPE138" s="37"/>
+      <c r="BPM138" s="37"/>
+      <c r="BPU138" s="37"/>
+      <c r="BQC138" s="37"/>
+      <c r="BQK138" s="37"/>
+      <c r="BQS138" s="37"/>
+      <c r="BRA138" s="37"/>
+      <c r="BRI138" s="37"/>
+      <c r="BRQ138" s="37"/>
+      <c r="BRY138" s="37"/>
+      <c r="BSG138" s="37"/>
+      <c r="BSO138" s="37"/>
+      <c r="BSW138" s="37"/>
+      <c r="BTE138" s="37"/>
+      <c r="BTM138" s="37"/>
+      <c r="BTU138" s="37"/>
+      <c r="BUC138" s="37"/>
+      <c r="BUK138" s="37"/>
+      <c r="BUS138" s="37"/>
+      <c r="BVA138" s="37"/>
+      <c r="BVI138" s="37"/>
+      <c r="BVQ138" s="37"/>
+      <c r="BVY138" s="37"/>
+      <c r="BWG138" s="37"/>
+      <c r="BWO138" s="37"/>
+      <c r="BWW138" s="37"/>
+      <c r="BXE138" s="37"/>
+      <c r="BXM138" s="37"/>
+      <c r="BXU138" s="37"/>
+      <c r="BYC138" s="37"/>
+      <c r="BYK138" s="37"/>
+      <c r="BYS138" s="37"/>
+      <c r="BZA138" s="37"/>
+      <c r="BZI138" s="37"/>
+      <c r="BZQ138" s="37"/>
+      <c r="BZY138" s="37"/>
+      <c r="CAG138" s="37"/>
+      <c r="CAO138" s="37"/>
+      <c r="CAW138" s="37"/>
+      <c r="CBE138" s="37"/>
+      <c r="CBM138" s="37"/>
+      <c r="CBU138" s="37"/>
+      <c r="CCC138" s="37"/>
+      <c r="CCK138" s="37"/>
+      <c r="CCS138" s="37"/>
+      <c r="CDA138" s="37"/>
+      <c r="CDI138" s="37"/>
+      <c r="CDQ138" s="37"/>
+      <c r="CDY138" s="37"/>
+      <c r="CEG138" s="37"/>
+      <c r="CEO138" s="37"/>
+      <c r="CEW138" s="37"/>
+      <c r="CFE138" s="37"/>
+      <c r="CFM138" s="37"/>
+      <c r="CFU138" s="37"/>
+      <c r="CGC138" s="37"/>
+      <c r="CGK138" s="37"/>
+      <c r="CGS138" s="37"/>
+      <c r="CHA138" s="37"/>
+      <c r="CHI138" s="37"/>
+      <c r="CHQ138" s="37"/>
+      <c r="CHY138" s="37"/>
+      <c r="CIG138" s="37"/>
+      <c r="CIO138" s="37"/>
+      <c r="CIW138" s="37"/>
+      <c r="CJE138" s="37"/>
+      <c r="CJM138" s="37"/>
+      <c r="CJU138" s="37"/>
+      <c r="CKC138" s="37"/>
+      <c r="CKK138" s="37"/>
+      <c r="CKS138" s="37"/>
+      <c r="CLA138" s="37"/>
+      <c r="CLI138" s="37"/>
+      <c r="CLQ138" s="37"/>
+      <c r="CLY138" s="37"/>
+      <c r="CMG138" s="37"/>
+      <c r="CMO138" s="37"/>
+      <c r="CMW138" s="37"/>
+      <c r="CNE138" s="37"/>
+      <c r="CNM138" s="37"/>
+      <c r="CNU138" s="37"/>
+      <c r="COC138" s="37"/>
+      <c r="COK138" s="37"/>
+      <c r="COS138" s="37"/>
+      <c r="CPA138" s="37"/>
+      <c r="CPI138" s="37"/>
+      <c r="CPQ138" s="37"/>
+      <c r="CPY138" s="37"/>
+      <c r="CQG138" s="37"/>
+      <c r="CQO138" s="37"/>
+      <c r="CQW138" s="37"/>
+      <c r="CRE138" s="37"/>
+      <c r="CRM138" s="37"/>
+      <c r="CRU138" s="37"/>
+      <c r="CSC138" s="37"/>
+      <c r="CSK138" s="37"/>
+      <c r="CSS138" s="37"/>
+      <c r="CTA138" s="37"/>
+      <c r="CTI138" s="37"/>
+      <c r="CTQ138" s="37"/>
+      <c r="CTY138" s="37"/>
+      <c r="CUG138" s="37"/>
+      <c r="CUO138" s="37"/>
+      <c r="CUW138" s="37"/>
+      <c r="CVE138" s="37"/>
+      <c r="CVM138" s="37"/>
+      <c r="CVU138" s="37"/>
+      <c r="CWC138" s="37"/>
+      <c r="CWK138" s="37"/>
+      <c r="CWS138" s="37"/>
+      <c r="CXA138" s="37"/>
+      <c r="CXI138" s="37"/>
+      <c r="CXQ138" s="37"/>
+      <c r="CXY138" s="37"/>
+      <c r="CYG138" s="37"/>
+      <c r="CYO138" s="37"/>
+      <c r="CYW138" s="37"/>
+      <c r="CZE138" s="37"/>
+      <c r="CZM138" s="37"/>
+      <c r="CZU138" s="37"/>
+      <c r="DAC138" s="37"/>
+      <c r="DAK138" s="37"/>
+      <c r="DAS138" s="37"/>
+      <c r="DBA138" s="37"/>
+      <c r="DBI138" s="37"/>
+      <c r="DBQ138" s="37"/>
+      <c r="DBY138" s="37"/>
+      <c r="DCG138" s="37"/>
+      <c r="DCO138" s="37"/>
+      <c r="DCW138" s="37"/>
+      <c r="DDE138" s="37"/>
+      <c r="DDM138" s="37"/>
+      <c r="DDU138" s="37"/>
+      <c r="DEC138" s="37"/>
+      <c r="DEK138" s="37"/>
+      <c r="DES138" s="37"/>
+      <c r="DFA138" s="37"/>
+      <c r="DFI138" s="37"/>
+      <c r="DFQ138" s="37"/>
+      <c r="DFY138" s="37"/>
+      <c r="DGG138" s="37"/>
+      <c r="DGO138" s="37"/>
+      <c r="DGW138" s="37"/>
+      <c r="DHE138" s="37"/>
+      <c r="DHM138" s="37"/>
+      <c r="DHU138" s="37"/>
+      <c r="DIC138" s="37"/>
+      <c r="DIK138" s="37"/>
+      <c r="DIS138" s="37"/>
+      <c r="DJA138" s="37"/>
+      <c r="DJI138" s="37"/>
+      <c r="DJQ138" s="37"/>
+      <c r="DJY138" s="37"/>
+      <c r="DKG138" s="37"/>
+      <c r="DKO138" s="37"/>
+      <c r="DKW138" s="37"/>
+      <c r="DLE138" s="37"/>
+      <c r="DLM138" s="37"/>
+      <c r="DLU138" s="37"/>
+      <c r="DMC138" s="37"/>
+      <c r="DMK138" s="37"/>
+      <c r="DMS138" s="37"/>
+      <c r="DNA138" s="37"/>
+      <c r="DNI138" s="37"/>
+      <c r="DNQ138" s="37"/>
+      <c r="DNY138" s="37"/>
+      <c r="DOG138" s="37"/>
+      <c r="DOO138" s="37"/>
+      <c r="DOW138" s="37"/>
+      <c r="DPE138" s="37"/>
+      <c r="DPM138" s="37"/>
+      <c r="DPU138" s="37"/>
+      <c r="DQC138" s="37"/>
+      <c r="DQK138" s="37"/>
+      <c r="DQS138" s="37"/>
+      <c r="DRA138" s="37"/>
+      <c r="DRI138" s="37"/>
+      <c r="DRQ138" s="37"/>
+      <c r="DRY138" s="37"/>
+      <c r="DSG138" s="37"/>
+      <c r="DSO138" s="37"/>
+      <c r="DSW138" s="37"/>
+      <c r="DTE138" s="37"/>
+      <c r="DTM138" s="37"/>
+      <c r="DTU138" s="37"/>
+      <c r="DUC138" s="37"/>
+      <c r="DUK138" s="37"/>
+      <c r="DUS138" s="37"/>
+      <c r="DVA138" s="37"/>
+      <c r="DVI138" s="37"/>
+      <c r="DVQ138" s="37"/>
+      <c r="DVY138" s="37"/>
+      <c r="DWG138" s="37"/>
+      <c r="DWO138" s="37"/>
+      <c r="DWW138" s="37"/>
+      <c r="DXE138" s="37"/>
+      <c r="DXM138" s="37"/>
+      <c r="DXU138" s="37"/>
+      <c r="DYC138" s="37"/>
+      <c r="DYK138" s="37"/>
+      <c r="DYS138" s="37"/>
+      <c r="DZA138" s="37"/>
+      <c r="DZI138" s="37"/>
+      <c r="DZQ138" s="37"/>
+      <c r="DZY138" s="37"/>
+      <c r="EAG138" s="37"/>
+      <c r="EAO138" s="37"/>
+      <c r="EAW138" s="37"/>
+      <c r="EBE138" s="37"/>
+      <c r="EBM138" s="37"/>
+      <c r="EBU138" s="37"/>
+      <c r="ECC138" s="37"/>
+      <c r="ECK138" s="37"/>
+      <c r="ECS138" s="37"/>
+      <c r="EDA138" s="37"/>
+      <c r="EDI138" s="37"/>
+      <c r="EDQ138" s="37"/>
+      <c r="EDY138" s="37"/>
+      <c r="EEG138" s="37"/>
+      <c r="EEO138" s="37"/>
+      <c r="EEW138" s="37"/>
+      <c r="EFE138" s="37"/>
+      <c r="EFM138" s="37"/>
+      <c r="EFU138" s="37"/>
+      <c r="EGC138" s="37"/>
+      <c r="EGK138" s="37"/>
+      <c r="EGS138" s="37"/>
+      <c r="EHA138" s="37"/>
+      <c r="EHI138" s="37"/>
+      <c r="EHQ138" s="37"/>
+      <c r="EHY138" s="37"/>
+      <c r="EIG138" s="37"/>
+      <c r="EIO138" s="37"/>
+      <c r="EIW138" s="37"/>
+      <c r="EJE138" s="37"/>
+      <c r="EJM138" s="37"/>
+      <c r="EJU138" s="37"/>
+      <c r="EKC138" s="37"/>
+      <c r="EKK138" s="37"/>
+      <c r="EKS138" s="37"/>
+      <c r="ELA138" s="37"/>
+      <c r="ELI138" s="37"/>
+      <c r="ELQ138" s="37"/>
+      <c r="ELY138" s="37"/>
+      <c r="EMG138" s="37"/>
+      <c r="EMO138" s="37"/>
+      <c r="EMW138" s="37"/>
+      <c r="ENE138" s="37"/>
+      <c r="ENM138" s="37"/>
+      <c r="ENU138" s="37"/>
+      <c r="EOC138" s="37"/>
+      <c r="EOK138" s="37"/>
+      <c r="EOS138" s="37"/>
+      <c r="EPA138" s="37"/>
+      <c r="EPI138" s="37"/>
+      <c r="EPQ138" s="37"/>
+      <c r="EPY138" s="37"/>
+      <c r="EQG138" s="37"/>
+      <c r="EQO138" s="37"/>
+      <c r="EQW138" s="37"/>
+      <c r="ERE138" s="37"/>
+      <c r="ERM138" s="37"/>
+      <c r="ERU138" s="37"/>
+      <c r="ESC138" s="37"/>
+      <c r="ESK138" s="37"/>
+      <c r="ESS138" s="37"/>
+      <c r="ETA138" s="37"/>
+      <c r="ETI138" s="37"/>
+      <c r="ETQ138" s="37"/>
+      <c r="ETY138" s="37"/>
+      <c r="EUG138" s="37"/>
+      <c r="EUO138" s="37"/>
+      <c r="EUW138" s="37"/>
+      <c r="EVE138" s="37"/>
+      <c r="EVM138" s="37"/>
+      <c r="EVU138" s="37"/>
+      <c r="EWC138" s="37"/>
+      <c r="EWK138" s="37"/>
+      <c r="EWS138" s="37"/>
+      <c r="EXA138" s="37"/>
+      <c r="EXI138" s="37"/>
+      <c r="EXQ138" s="37"/>
+      <c r="EXY138" s="37"/>
+      <c r="EYG138" s="37"/>
+      <c r="EYO138" s="37"/>
+      <c r="EYW138" s="37"/>
+      <c r="EZE138" s="37"/>
+      <c r="EZM138" s="37"/>
+      <c r="EZU138" s="37"/>
+      <c r="FAC138" s="37"/>
+      <c r="FAK138" s="37"/>
+      <c r="FAS138" s="37"/>
+      <c r="FBA138" s="37"/>
+      <c r="FBI138" s="37"/>
+      <c r="FBQ138" s="37"/>
+      <c r="FBY138" s="37"/>
+      <c r="FCG138" s="37"/>
+      <c r="FCO138" s="37"/>
+      <c r="FCW138" s="37"/>
+      <c r="FDE138" s="37"/>
+      <c r="FDM138" s="37"/>
+      <c r="FDU138" s="37"/>
+      <c r="FEC138" s="37"/>
+      <c r="FEK138" s="37"/>
+      <c r="FES138" s="37"/>
+      <c r="FFA138" s="37"/>
+      <c r="FFI138" s="37"/>
+      <c r="FFQ138" s="37"/>
+      <c r="FFY138" s="37"/>
+      <c r="FGG138" s="37"/>
+      <c r="FGO138" s="37"/>
+      <c r="FGW138" s="37"/>
+      <c r="FHE138" s="37"/>
+      <c r="FHM138" s="37"/>
+      <c r="FHU138" s="37"/>
+      <c r="FIC138" s="37"/>
+      <c r="FIK138" s="37"/>
+      <c r="FIS138" s="37"/>
+      <c r="FJA138" s="37"/>
+      <c r="FJI138" s="37"/>
+      <c r="FJQ138" s="37"/>
+      <c r="FJY138" s="37"/>
+      <c r="FKG138" s="37"/>
+      <c r="FKO138" s="37"/>
+      <c r="FKW138" s="37"/>
+      <c r="FLE138" s="37"/>
+      <c r="FLM138" s="37"/>
+      <c r="FLU138" s="37"/>
+      <c r="FMC138" s="37"/>
+      <c r="FMK138" s="37"/>
+      <c r="FMS138" s="37"/>
+      <c r="FNA138" s="37"/>
+      <c r="FNI138" s="37"/>
+      <c r="FNQ138" s="37"/>
+      <c r="FNY138" s="37"/>
+      <c r="FOG138" s="37"/>
+      <c r="FOO138" s="37"/>
+      <c r="FOW138" s="37"/>
+      <c r="FPE138" s="37"/>
+      <c r="FPM138" s="37"/>
+      <c r="FPU138" s="37"/>
+      <c r="FQC138" s="37"/>
+      <c r="FQK138" s="37"/>
+      <c r="FQS138" s="37"/>
+      <c r="FRA138" s="37"/>
+      <c r="FRI138" s="37"/>
+      <c r="FRQ138" s="37"/>
+      <c r="FRY138" s="37"/>
+      <c r="FSG138" s="37"/>
+      <c r="FSO138" s="37"/>
+      <c r="FSW138" s="37"/>
+      <c r="FTE138" s="37"/>
+      <c r="FTM138" s="37"/>
+      <c r="FTU138" s="37"/>
+      <c r="FUC138" s="37"/>
+      <c r="FUK138" s="37"/>
+      <c r="FUS138" s="37"/>
+      <c r="FVA138" s="37"/>
+      <c r="FVI138" s="37"/>
+      <c r="FVQ138" s="37"/>
+      <c r="FVY138" s="37"/>
+      <c r="FWG138" s="37"/>
+      <c r="FWO138" s="37"/>
+      <c r="FWW138" s="37"/>
+      <c r="FXE138" s="37"/>
+      <c r="FXM138" s="37"/>
+      <c r="FXU138" s="37"/>
+      <c r="FYC138" s="37"/>
+      <c r="FYK138" s="37"/>
+      <c r="FYS138" s="37"/>
+      <c r="FZA138" s="37"/>
+      <c r="FZI138" s="37"/>
+      <c r="FZQ138" s="37"/>
+      <c r="FZY138" s="37"/>
+      <c r="GAG138" s="37"/>
+      <c r="GAO138" s="37"/>
+      <c r="GAW138" s="37"/>
+      <c r="GBE138" s="37"/>
+      <c r="GBM138" s="37"/>
+      <c r="GBU138" s="37"/>
+      <c r="GCC138" s="37"/>
+      <c r="GCK138" s="37"/>
+      <c r="GCS138" s="37"/>
+      <c r="GDA138" s="37"/>
+      <c r="GDI138" s="37"/>
+      <c r="GDQ138" s="37"/>
+      <c r="GDY138" s="37"/>
+      <c r="GEG138" s="37"/>
+      <c r="GEO138" s="37"/>
+      <c r="GEW138" s="37"/>
+      <c r="GFE138" s="37"/>
+      <c r="GFM138" s="37"/>
+      <c r="GFU138" s="37"/>
+      <c r="GGC138" s="37"/>
+      <c r="GGK138" s="37"/>
+      <c r="GGS138" s="37"/>
+      <c r="GHA138" s="37"/>
+      <c r="GHI138" s="37"/>
+      <c r="GHQ138" s="37"/>
+      <c r="GHY138" s="37"/>
+      <c r="GIG138" s="37"/>
+      <c r="GIO138" s="37"/>
+      <c r="GIW138" s="37"/>
+      <c r="GJE138" s="37"/>
+      <c r="GJM138" s="37"/>
+      <c r="GJU138" s="37"/>
+      <c r="GKC138" s="37"/>
+      <c r="GKK138" s="37"/>
+      <c r="GKS138" s="37"/>
+      <c r="GLA138" s="37"/>
+      <c r="GLI138" s="37"/>
+      <c r="GLQ138" s="37"/>
+      <c r="GLY138" s="37"/>
+      <c r="GMG138" s="37"/>
+      <c r="GMO138" s="37"/>
+      <c r="GMW138" s="37"/>
+      <c r="GNE138" s="37"/>
+      <c r="GNM138" s="37"/>
+      <c r="GNU138" s="37"/>
+      <c r="GOC138" s="37"/>
+      <c r="GOK138" s="37"/>
+      <c r="GOS138" s="37"/>
+      <c r="GPA138" s="37"/>
+      <c r="GPI138" s="37"/>
+      <c r="GPQ138" s="37"/>
+      <c r="GPY138" s="37"/>
+      <c r="GQG138" s="37"/>
+      <c r="GQO138" s="37"/>
+      <c r="GQW138" s="37"/>
+      <c r="GRE138" s="37"/>
+      <c r="GRM138" s="37"/>
+      <c r="GRU138" s="37"/>
+      <c r="GSC138" s="37"/>
+      <c r="GSK138" s="37"/>
+      <c r="GSS138" s="37"/>
+      <c r="GTA138" s="37"/>
+      <c r="GTI138" s="37"/>
+      <c r="GTQ138" s="37"/>
+      <c r="GTY138" s="37"/>
+      <c r="GUG138" s="37"/>
+      <c r="GUO138" s="37"/>
+      <c r="GUW138" s="37"/>
+      <c r="GVE138" s="37"/>
+      <c r="GVM138" s="37"/>
+      <c r="GVU138" s="37"/>
+      <c r="GWC138" s="37"/>
+      <c r="GWK138" s="37"/>
+      <c r="GWS138" s="37"/>
+      <c r="GXA138" s="37"/>
+      <c r="GXI138" s="37"/>
+      <c r="GXQ138" s="37"/>
+      <c r="GXY138" s="37"/>
+      <c r="GYG138" s="37"/>
+      <c r="GYO138" s="37"/>
+      <c r="GYW138" s="37"/>
+      <c r="GZE138" s="37"/>
+      <c r="GZM138" s="37"/>
+      <c r="GZU138" s="37"/>
+      <c r="HAC138" s="37"/>
+      <c r="HAK138" s="37"/>
+      <c r="HAS138" s="37"/>
+      <c r="HBA138" s="37"/>
+      <c r="HBI138" s="37"/>
+      <c r="HBQ138" s="37"/>
+      <c r="HBY138" s="37"/>
+      <c r="HCG138" s="37"/>
+      <c r="HCO138" s="37"/>
+      <c r="HCW138" s="37"/>
+      <c r="HDE138" s="37"/>
+      <c r="HDM138" s="37"/>
+      <c r="HDU138" s="37"/>
+      <c r="HEC138" s="37"/>
+      <c r="HEK138" s="37"/>
+      <c r="HES138" s="37"/>
+      <c r="HFA138" s="37"/>
+      <c r="HFI138" s="37"/>
+      <c r="HFQ138" s="37"/>
+      <c r="HFY138" s="37"/>
+      <c r="HGG138" s="37"/>
+      <c r="HGO138" s="37"/>
+      <c r="HGW138" s="37"/>
+      <c r="HHE138" s="37"/>
+      <c r="HHM138" s="37"/>
+      <c r="HHU138" s="37"/>
+      <c r="HIC138" s="37"/>
+      <c r="HIK138" s="37"/>
+      <c r="HIS138" s="37"/>
+      <c r="HJA138" s="37"/>
+      <c r="HJI138" s="37"/>
+      <c r="HJQ138" s="37"/>
+      <c r="HJY138" s="37"/>
+      <c r="HKG138" s="37"/>
+      <c r="HKO138" s="37"/>
+      <c r="HKW138" s="37"/>
+      <c r="HLE138" s="37"/>
+      <c r="HLM138" s="37"/>
+      <c r="HLU138" s="37"/>
+      <c r="HMC138" s="37"/>
+      <c r="HMK138" s="37"/>
+      <c r="HMS138" s="37"/>
+      <c r="HNA138" s="37"/>
+      <c r="HNI138" s="37"/>
+      <c r="HNQ138" s="37"/>
+      <c r="HNY138" s="37"/>
+      <c r="HOG138" s="37"/>
+      <c r="HOO138" s="37"/>
+      <c r="HOW138" s="37"/>
+      <c r="HPE138" s="37"/>
+      <c r="HPM138" s="37"/>
+      <c r="HPU138" s="37"/>
+      <c r="HQC138" s="37"/>
+      <c r="HQK138" s="37"/>
+      <c r="HQS138" s="37"/>
+      <c r="HRA138" s="37"/>
+      <c r="HRI138" s="37"/>
+      <c r="HRQ138" s="37"/>
+      <c r="HRY138" s="37"/>
+      <c r="HSG138" s="37"/>
+      <c r="HSO138" s="37"/>
+      <c r="HSW138" s="37"/>
+      <c r="HTE138" s="37"/>
+      <c r="HTM138" s="37"/>
+      <c r="HTU138" s="37"/>
+      <c r="HUC138" s="37"/>
+      <c r="HUK138" s="37"/>
+      <c r="HUS138" s="37"/>
+      <c r="HVA138" s="37"/>
+      <c r="HVI138" s="37"/>
+      <c r="HVQ138" s="37"/>
+      <c r="HVY138" s="37"/>
+      <c r="HWG138" s="37"/>
+      <c r="HWO138" s="37"/>
+      <c r="HWW138" s="37"/>
+      <c r="HXE138" s="37"/>
+      <c r="HXM138" s="37"/>
+      <c r="HXU138" s="37"/>
+      <c r="HYC138" s="37"/>
+      <c r="HYK138" s="37"/>
+      <c r="HYS138" s="37"/>
+      <c r="HZA138" s="37"/>
+      <c r="HZI138" s="37"/>
+      <c r="HZQ138" s="37"/>
+      <c r="HZY138" s="37"/>
+      <c r="IAG138" s="37"/>
+      <c r="IAO138" s="37"/>
+      <c r="IAW138" s="37"/>
+      <c r="IBE138" s="37"/>
+      <c r="IBM138" s="37"/>
+      <c r="IBU138" s="37"/>
+      <c r="ICC138" s="37"/>
+      <c r="ICK138" s="37"/>
+      <c r="ICS138" s="37"/>
+      <c r="IDA138" s="37"/>
+      <c r="IDI138" s="37"/>
+      <c r="IDQ138" s="37"/>
+      <c r="IDY138" s="37"/>
+      <c r="IEG138" s="37"/>
+      <c r="IEO138" s="37"/>
+      <c r="IEW138" s="37"/>
+      <c r="IFE138" s="37"/>
+      <c r="IFM138" s="37"/>
+      <c r="IFU138" s="37"/>
+      <c r="IGC138" s="37"/>
+      <c r="IGK138" s="37"/>
+      <c r="IGS138" s="37"/>
+      <c r="IHA138" s="37"/>
+      <c r="IHI138" s="37"/>
+      <c r="IHQ138" s="37"/>
+      <c r="IHY138" s="37"/>
+      <c r="IIG138" s="37"/>
+      <c r="IIO138" s="37"/>
+      <c r="IIW138" s="37"/>
+      <c r="IJE138" s="37"/>
+      <c r="IJM138" s="37"/>
+      <c r="IJU138" s="37"/>
+      <c r="IKC138" s="37"/>
+      <c r="IKK138" s="37"/>
+      <c r="IKS138" s="37"/>
+      <c r="ILA138" s="37"/>
+      <c r="ILI138" s="37"/>
+      <c r="ILQ138" s="37"/>
+      <c r="ILY138" s="37"/>
+      <c r="IMG138" s="37"/>
+      <c r="IMO138" s="37"/>
+      <c r="IMW138" s="37"/>
+      <c r="INE138" s="37"/>
+      <c r="INM138" s="37"/>
+      <c r="INU138" s="37"/>
+      <c r="IOC138" s="37"/>
+      <c r="IOK138" s="37"/>
+      <c r="IOS138" s="37"/>
+      <c r="IPA138" s="37"/>
+      <c r="IPI138" s="37"/>
+      <c r="IPQ138" s="37"/>
+      <c r="IPY138" s="37"/>
+      <c r="IQG138" s="37"/>
+      <c r="IQO138" s="37"/>
+      <c r="IQW138" s="37"/>
+      <c r="IRE138" s="37"/>
+      <c r="IRM138" s="37"/>
+      <c r="IRU138" s="37"/>
+      <c r="ISC138" s="37"/>
+      <c r="ISK138" s="37"/>
+      <c r="ISS138" s="37"/>
+      <c r="ITA138" s="37"/>
+      <c r="ITI138" s="37"/>
+      <c r="ITQ138" s="37"/>
+      <c r="ITY138" s="37"/>
+      <c r="IUG138" s="37"/>
+      <c r="IUO138" s="37"/>
+      <c r="IUW138" s="37"/>
+      <c r="IVE138" s="37"/>
+      <c r="IVM138" s="37"/>
+      <c r="IVU138" s="37"/>
+      <c r="IWC138" s="37"/>
+      <c r="IWK138" s="37"/>
+      <c r="IWS138" s="37"/>
+      <c r="IXA138" s="37"/>
+      <c r="IXI138" s="37"/>
+      <c r="IXQ138" s="37"/>
+      <c r="IXY138" s="37"/>
+      <c r="IYG138" s="37"/>
+      <c r="IYO138" s="37"/>
+      <c r="IYW138" s="37"/>
+      <c r="IZE138" s="37"/>
+      <c r="IZM138" s="37"/>
+      <c r="IZU138" s="37"/>
+      <c r="JAC138" s="37"/>
+      <c r="JAK138" s="37"/>
+      <c r="JAS138" s="37"/>
+      <c r="JBA138" s="37"/>
+      <c r="JBI138" s="37"/>
+      <c r="JBQ138" s="37"/>
+      <c r="JBY138" s="37"/>
+      <c r="JCG138" s="37"/>
+      <c r="JCO138" s="37"/>
+      <c r="JCW138" s="37"/>
+      <c r="JDE138" s="37"/>
+      <c r="JDM138" s="37"/>
+      <c r="JDU138" s="37"/>
+      <c r="JEC138" s="37"/>
+      <c r="JEK138" s="37"/>
+      <c r="JES138" s="37"/>
+      <c r="JFA138" s="37"/>
+      <c r="JFI138" s="37"/>
+      <c r="JFQ138" s="37"/>
+      <c r="JFY138" s="37"/>
+      <c r="JGG138" s="37"/>
+      <c r="JGO138" s="37"/>
+      <c r="JGW138" s="37"/>
+      <c r="JHE138" s="37"/>
+      <c r="JHM138" s="37"/>
+      <c r="JHU138" s="37"/>
+      <c r="JIC138" s="37"/>
+      <c r="JIK138" s="37"/>
+      <c r="JIS138" s="37"/>
+      <c r="JJA138" s="37"/>
+      <c r="JJI138" s="37"/>
+      <c r="JJQ138" s="37"/>
+      <c r="JJY138" s="37"/>
+      <c r="JKG138" s="37"/>
+      <c r="JKO138" s="37"/>
+      <c r="JKW138" s="37"/>
+      <c r="JLE138" s="37"/>
+      <c r="JLM138" s="37"/>
+      <c r="JLU138" s="37"/>
+      <c r="JMC138" s="37"/>
+      <c r="JMK138" s="37"/>
+      <c r="JMS138" s="37"/>
+      <c r="JNA138" s="37"/>
+      <c r="JNI138" s="37"/>
+      <c r="JNQ138" s="37"/>
+      <c r="JNY138" s="37"/>
+      <c r="JOG138" s="37"/>
+      <c r="JOO138" s="37"/>
+      <c r="JOW138" s="37"/>
+      <c r="JPE138" s="37"/>
+      <c r="JPM138" s="37"/>
+      <c r="JPU138" s="37"/>
+      <c r="JQC138" s="37"/>
+      <c r="JQK138" s="37"/>
+      <c r="JQS138" s="37"/>
+      <c r="JRA138" s="37"/>
+      <c r="JRI138" s="37"/>
+      <c r="JRQ138" s="37"/>
+      <c r="JRY138" s="37"/>
+      <c r="JSG138" s="37"/>
+      <c r="JSO138" s="37"/>
+      <c r="JSW138" s="37"/>
+      <c r="JTE138" s="37"/>
+      <c r="JTM138" s="37"/>
+      <c r="JTU138" s="37"/>
+      <c r="JUC138" s="37"/>
+      <c r="JUK138" s="37"/>
+      <c r="JUS138" s="37"/>
+      <c r="JVA138" s="37"/>
+      <c r="JVI138" s="37"/>
+      <c r="JVQ138" s="37"/>
+      <c r="JVY138" s="37"/>
+      <c r="JWG138" s="37"/>
+      <c r="JWO138" s="37"/>
+      <c r="JWW138" s="37"/>
+      <c r="JXE138" s="37"/>
+      <c r="JXM138" s="37"/>
+      <c r="JXU138" s="37"/>
+      <c r="JYC138" s="37"/>
+      <c r="JYK138" s="37"/>
+      <c r="JYS138" s="37"/>
+      <c r="JZA138" s="37"/>
+      <c r="JZI138" s="37"/>
+      <c r="JZQ138" s="37"/>
+      <c r="JZY138" s="37"/>
+      <c r="KAG138" s="37"/>
+      <c r="KAO138" s="37"/>
+      <c r="KAW138" s="37"/>
+      <c r="KBE138" s="37"/>
+      <c r="KBM138" s="37"/>
+      <c r="KBU138" s="37"/>
+      <c r="KCC138" s="37"/>
+      <c r="KCK138" s="37"/>
+      <c r="KCS138" s="37"/>
+      <c r="KDA138" s="37"/>
+      <c r="KDI138" s="37"/>
+      <c r="KDQ138" s="37"/>
+      <c r="KDY138" s="37"/>
+      <c r="KEG138" s="37"/>
+      <c r="KEO138" s="37"/>
+      <c r="KEW138" s="37"/>
+      <c r="KFE138" s="37"/>
+      <c r="KFM138" s="37"/>
+      <c r="KFU138" s="37"/>
+      <c r="KGC138" s="37"/>
+      <c r="KGK138" s="37"/>
+      <c r="KGS138" s="37"/>
+      <c r="KHA138" s="37"/>
+      <c r="KHI138" s="37"/>
+      <c r="KHQ138" s="37"/>
+      <c r="KHY138" s="37"/>
+      <c r="KIG138" s="37"/>
+      <c r="KIO138" s="37"/>
+      <c r="KIW138" s="37"/>
+      <c r="KJE138" s="37"/>
+      <c r="KJM138" s="37"/>
+      <c r="KJU138" s="37"/>
+      <c r="KKC138" s="37"/>
+      <c r="KKK138" s="37"/>
+      <c r="KKS138" s="37"/>
+      <c r="KLA138" s="37"/>
+      <c r="KLI138" s="37"/>
+      <c r="KLQ138" s="37"/>
+      <c r="KLY138" s="37"/>
+      <c r="KMG138" s="37"/>
+      <c r="KMO138" s="37"/>
+      <c r="KMW138" s="37"/>
+      <c r="KNE138" s="37"/>
+      <c r="KNM138" s="37"/>
+      <c r="KNU138" s="37"/>
+      <c r="KOC138" s="37"/>
+      <c r="KOK138" s="37"/>
+      <c r="KOS138" s="37"/>
+      <c r="KPA138" s="37"/>
+      <c r="KPI138" s="37"/>
+      <c r="KPQ138" s="37"/>
+      <c r="KPY138" s="37"/>
+      <c r="KQG138" s="37"/>
+      <c r="KQO138" s="37"/>
+      <c r="KQW138" s="37"/>
+      <c r="KRE138" s="37"/>
+      <c r="KRM138" s="37"/>
+      <c r="KRU138" s="37"/>
+      <c r="KSC138" s="37"/>
+      <c r="KSK138" s="37"/>
+      <c r="KSS138" s="37"/>
+      <c r="KTA138" s="37"/>
+      <c r="KTI138" s="37"/>
+      <c r="KTQ138" s="37"/>
+      <c r="KTY138" s="37"/>
+      <c r="KUG138" s="37"/>
+      <c r="KUO138" s="37"/>
+      <c r="KUW138" s="37"/>
+      <c r="KVE138" s="37"/>
+      <c r="KVM138" s="37"/>
+      <c r="KVU138" s="37"/>
+      <c r="KWC138" s="37"/>
+      <c r="KWK138" s="37"/>
+      <c r="KWS138" s="37"/>
+      <c r="KXA138" s="37"/>
+      <c r="KXI138" s="37"/>
+      <c r="KXQ138" s="37"/>
+      <c r="KXY138" s="37"/>
+      <c r="KYG138" s="37"/>
+      <c r="KYO138" s="37"/>
+      <c r="KYW138" s="37"/>
+      <c r="KZE138" s="37"/>
+      <c r="KZM138" s="37"/>
+      <c r="KZU138" s="37"/>
+      <c r="LAC138" s="37"/>
+      <c r="LAK138" s="37"/>
+      <c r="LAS138" s="37"/>
+      <c r="LBA138" s="37"/>
+      <c r="LBI138" s="37"/>
+      <c r="LBQ138" s="37"/>
+      <c r="LBY138" s="37"/>
+      <c r="LCG138" s="37"/>
+      <c r="LCO138" s="37"/>
+      <c r="LCW138" s="37"/>
+      <c r="LDE138" s="37"/>
+      <c r="LDM138" s="37"/>
+      <c r="LDU138" s="37"/>
+      <c r="LEC138" s="37"/>
+      <c r="LEK138" s="37"/>
+      <c r="LES138" s="37"/>
+      <c r="LFA138" s="37"/>
+      <c r="LFI138" s="37"/>
+      <c r="LFQ138" s="37"/>
+      <c r="LFY138" s="37"/>
+      <c r="LGG138" s="37"/>
+      <c r="LGO138" s="37"/>
+      <c r="LGW138" s="37"/>
+      <c r="LHE138" s="37"/>
+      <c r="LHM138" s="37"/>
+      <c r="LHU138" s="37"/>
+      <c r="LIC138" s="37"/>
+      <c r="LIK138" s="37"/>
+      <c r="LIS138" s="37"/>
+      <c r="LJA138" s="37"/>
+      <c r="LJI138" s="37"/>
+      <c r="LJQ138" s="37"/>
+      <c r="LJY138" s="37"/>
+      <c r="LKG138" s="37"/>
+      <c r="LKO138" s="37"/>
+      <c r="LKW138" s="37"/>
+      <c r="LLE138" s="37"/>
+      <c r="LLM138" s="37"/>
+      <c r="LLU138" s="37"/>
+      <c r="LMC138" s="37"/>
+      <c r="LMK138" s="37"/>
+      <c r="LMS138" s="37"/>
+      <c r="LNA138" s="37"/>
+      <c r="LNI138" s="37"/>
+      <c r="LNQ138" s="37"/>
+      <c r="LNY138" s="37"/>
+      <c r="LOG138" s="37"/>
+      <c r="LOO138" s="37"/>
+      <c r="LOW138" s="37"/>
+      <c r="LPE138" s="37"/>
+      <c r="LPM138" s="37"/>
+      <c r="LPU138" s="37"/>
+      <c r="LQC138" s="37"/>
+      <c r="LQK138" s="37"/>
+      <c r="LQS138" s="37"/>
+      <c r="LRA138" s="37"/>
+      <c r="LRI138" s="37"/>
+      <c r="LRQ138" s="37"/>
+      <c r="LRY138" s="37"/>
+      <c r="LSG138" s="37"/>
+      <c r="LSO138" s="37"/>
+      <c r="LSW138" s="37"/>
+      <c r="LTE138" s="37"/>
+      <c r="LTM138" s="37"/>
+      <c r="LTU138" s="37"/>
+      <c r="LUC138" s="37"/>
+      <c r="LUK138" s="37"/>
+      <c r="LUS138" s="37"/>
+      <c r="LVA138" s="37"/>
+      <c r="LVI138" s="37"/>
+      <c r="LVQ138" s="37"/>
+      <c r="LVY138" s="37"/>
+      <c r="LWG138" s="37"/>
+      <c r="LWO138" s="37"/>
+      <c r="LWW138" s="37"/>
+      <c r="LXE138" s="37"/>
+      <c r="LXM138" s="37"/>
+      <c r="LXU138" s="37"/>
+      <c r="LYC138" s="37"/>
+      <c r="LYK138" s="37"/>
+      <c r="LYS138" s="37"/>
+      <c r="LZA138" s="37"/>
+      <c r="LZI138" s="37"/>
+      <c r="LZQ138" s="37"/>
+      <c r="LZY138" s="37"/>
+      <c r="MAG138" s="37"/>
+      <c r="MAO138" s="37"/>
+      <c r="MAW138" s="37"/>
+      <c r="MBE138" s="37"/>
+      <c r="MBM138" s="37"/>
+      <c r="MBU138" s="37"/>
+      <c r="MCC138" s="37"/>
+      <c r="MCK138" s="37"/>
+      <c r="MCS138" s="37"/>
+      <c r="MDA138" s="37"/>
+      <c r="MDI138" s="37"/>
+      <c r="MDQ138" s="37"/>
+      <c r="MDY138" s="37"/>
+      <c r="MEG138" s="37"/>
+      <c r="MEO138" s="37"/>
+      <c r="MEW138" s="37"/>
+      <c r="MFE138" s="37"/>
+      <c r="MFM138" s="37"/>
+      <c r="MFU138" s="37"/>
+      <c r="MGC138" s="37"/>
+      <c r="MGK138" s="37"/>
+      <c r="MGS138" s="37"/>
+      <c r="MHA138" s="37"/>
+      <c r="MHI138" s="37"/>
+      <c r="MHQ138" s="37"/>
+      <c r="MHY138" s="37"/>
+      <c r="MIG138" s="37"/>
+      <c r="MIO138" s="37"/>
+      <c r="MIW138" s="37"/>
+      <c r="MJE138" s="37"/>
+      <c r="MJM138" s="37"/>
+      <c r="MJU138" s="37"/>
+      <c r="MKC138" s="37"/>
+      <c r="MKK138" s="37"/>
+      <c r="MKS138" s="37"/>
+      <c r="MLA138" s="37"/>
+      <c r="MLI138" s="37"/>
+      <c r="MLQ138" s="37"/>
+      <c r="MLY138" s="37"/>
+      <c r="MMG138" s="37"/>
+      <c r="MMO138" s="37"/>
+      <c r="MMW138" s="37"/>
+      <c r="MNE138" s="37"/>
+      <c r="MNM138" s="37"/>
+      <c r="MNU138" s="37"/>
+      <c r="MOC138" s="37"/>
+      <c r="MOK138" s="37"/>
+      <c r="MOS138" s="37"/>
+      <c r="MPA138" s="37"/>
+      <c r="MPI138" s="37"/>
+      <c r="MPQ138" s="37"/>
+      <c r="MPY138" s="37"/>
+      <c r="MQG138" s="37"/>
+      <c r="MQO138" s="37"/>
+      <c r="MQW138" s="37"/>
+      <c r="MRE138" s="37"/>
+      <c r="MRM138" s="37"/>
+      <c r="MRU138" s="37"/>
+      <c r="MSC138" s="37"/>
+      <c r="MSK138" s="37"/>
+      <c r="MSS138" s="37"/>
+      <c r="MTA138" s="37"/>
+      <c r="MTI138" s="37"/>
+      <c r="MTQ138" s="37"/>
+      <c r="MTY138" s="37"/>
+      <c r="MUG138" s="37"/>
+      <c r="MUO138" s="37"/>
+      <c r="MUW138" s="37"/>
+      <c r="MVE138" s="37"/>
+      <c r="MVM138" s="37"/>
+      <c r="MVU138" s="37"/>
+      <c r="MWC138" s="37"/>
+      <c r="MWK138" s="37"/>
+      <c r="MWS138" s="37"/>
+      <c r="MXA138" s="37"/>
+      <c r="MXI138" s="37"/>
+      <c r="MXQ138" s="37"/>
+      <c r="MXY138" s="37"/>
+      <c r="MYG138" s="37"/>
+      <c r="MYO138" s="37"/>
+      <c r="MYW138" s="37"/>
+      <c r="MZE138" s="37"/>
+      <c r="MZM138" s="37"/>
+      <c r="MZU138" s="37"/>
+      <c r="NAC138" s="37"/>
+      <c r="NAK138" s="37"/>
+      <c r="NAS138" s="37"/>
+      <c r="NBA138" s="37"/>
+      <c r="NBI138" s="37"/>
+      <c r="NBQ138" s="37"/>
+      <c r="NBY138" s="37"/>
+      <c r="NCG138" s="37"/>
+      <c r="NCO138" s="37"/>
+      <c r="NCW138" s="37"/>
+      <c r="NDE138" s="37"/>
+      <c r="NDM138" s="37"/>
+      <c r="NDU138" s="37"/>
+      <c r="NEC138" s="37"/>
+      <c r="NEK138" s="37"/>
+      <c r="NES138" s="37"/>
+      <c r="NFA138" s="37"/>
+      <c r="NFI138" s="37"/>
+      <c r="NFQ138" s="37"/>
+      <c r="NFY138" s="37"/>
+      <c r="NGG138" s="37"/>
+      <c r="NGO138" s="37"/>
+      <c r="NGW138" s="37"/>
+      <c r="NHE138" s="37"/>
+      <c r="NHM138" s="37"/>
+      <c r="NHU138" s="37"/>
+      <c r="NIC138" s="37"/>
+      <c r="NIK138" s="37"/>
+      <c r="NIS138" s="37"/>
+      <c r="NJA138" s="37"/>
+      <c r="NJI138" s="37"/>
+      <c r="NJQ138" s="37"/>
+      <c r="NJY138" s="37"/>
+      <c r="NKG138" s="37"/>
+      <c r="NKO138" s="37"/>
+      <c r="NKW138" s="37"/>
+      <c r="NLE138" s="37"/>
+      <c r="NLM138" s="37"/>
+      <c r="NLU138" s="37"/>
+      <c r="NMC138" s="37"/>
+      <c r="NMK138" s="37"/>
+      <c r="NMS138" s="37"/>
+      <c r="NNA138" s="37"/>
+      <c r="NNI138" s="37"/>
+      <c r="NNQ138" s="37"/>
+      <c r="NNY138" s="37"/>
+      <c r="NOG138" s="37"/>
+      <c r="NOO138" s="37"/>
+      <c r="NOW138" s="37"/>
+      <c r="NPE138" s="37"/>
+      <c r="NPM138" s="37"/>
+      <c r="NPU138" s="37"/>
+      <c r="NQC138" s="37"/>
+      <c r="NQK138" s="37"/>
+      <c r="NQS138" s="37"/>
+      <c r="NRA138" s="37"/>
+      <c r="NRI138" s="37"/>
+      <c r="NRQ138" s="37"/>
+      <c r="NRY138" s="37"/>
+      <c r="NSG138" s="37"/>
+      <c r="NSO138" s="37"/>
+      <c r="NSW138" s="37"/>
+      <c r="NTE138" s="37"/>
+      <c r="NTM138" s="37"/>
+      <c r="NTU138" s="37"/>
+      <c r="NUC138" s="37"/>
+      <c r="NUK138" s="37"/>
+      <c r="NUS138" s="37"/>
+      <c r="NVA138" s="37"/>
+      <c r="NVI138" s="37"/>
+      <c r="NVQ138" s="37"/>
+      <c r="NVY138" s="37"/>
+      <c r="NWG138" s="37"/>
+      <c r="NWO138" s="37"/>
+      <c r="NWW138" s="37"/>
+      <c r="NXE138" s="37"/>
+      <c r="NXM138" s="37"/>
+      <c r="NXU138" s="37"/>
+      <c r="NYC138" s="37"/>
+      <c r="NYK138" s="37"/>
+      <c r="NYS138" s="37"/>
+      <c r="NZA138" s="37"/>
+      <c r="NZI138" s="37"/>
+      <c r="NZQ138" s="37"/>
+      <c r="NZY138" s="37"/>
+      <c r="OAG138" s="37"/>
+      <c r="OAO138" s="37"/>
+      <c r="OAW138" s="37"/>
+      <c r="OBE138" s="37"/>
+      <c r="OBM138" s="37"/>
+      <c r="OBU138" s="37"/>
+      <c r="OCC138" s="37"/>
+      <c r="OCK138" s="37"/>
+      <c r="OCS138" s="37"/>
+      <c r="ODA138" s="37"/>
+      <c r="ODI138" s="37"/>
+      <c r="ODQ138" s="37"/>
+      <c r="ODY138" s="37"/>
+      <c r="OEG138" s="37"/>
+      <c r="OEO138" s="37"/>
+      <c r="OEW138" s="37"/>
+      <c r="OFE138" s="37"/>
+      <c r="OFM138" s="37"/>
+      <c r="OFU138" s="37"/>
+      <c r="OGC138" s="37"/>
+      <c r="OGK138" s="37"/>
+      <c r="OGS138" s="37"/>
+      <c r="OHA138" s="37"/>
+      <c r="OHI138" s="37"/>
+      <c r="OHQ138" s="37"/>
+      <c r="OHY138" s="37"/>
+      <c r="OIG138" s="37"/>
+      <c r="OIO138" s="37"/>
+      <c r="OIW138" s="37"/>
+      <c r="OJE138" s="37"/>
+      <c r="OJM138" s="37"/>
+      <c r="OJU138" s="37"/>
+      <c r="OKC138" s="37"/>
+      <c r="OKK138" s="37"/>
+      <c r="OKS138" s="37"/>
+      <c r="OLA138" s="37"/>
+      <c r="OLI138" s="37"/>
+      <c r="OLQ138" s="37"/>
+      <c r="OLY138" s="37"/>
+      <c r="OMG138" s="37"/>
+      <c r="OMO138" s="37"/>
+      <c r="OMW138" s="37"/>
+      <c r="ONE138" s="37"/>
+      <c r="ONM138" s="37"/>
+      <c r="ONU138" s="37"/>
+      <c r="OOC138" s="37"/>
+      <c r="OOK138" s="37"/>
+      <c r="OOS138" s="37"/>
+      <c r="OPA138" s="37"/>
+      <c r="OPI138" s="37"/>
+      <c r="OPQ138" s="37"/>
+      <c r="OPY138" s="37"/>
+      <c r="OQG138" s="37"/>
+      <c r="OQO138" s="37"/>
+      <c r="OQW138" s="37"/>
+      <c r="ORE138" s="37"/>
+      <c r="ORM138" s="37"/>
+      <c r="ORU138" s="37"/>
+      <c r="OSC138" s="37"/>
+      <c r="OSK138" s="37"/>
+      <c r="OSS138" s="37"/>
+      <c r="OTA138" s="37"/>
+      <c r="OTI138" s="37"/>
+      <c r="OTQ138" s="37"/>
+      <c r="OTY138" s="37"/>
+      <c r="OUG138" s="37"/>
+      <c r="OUO138" s="37"/>
+      <c r="OUW138" s="37"/>
+      <c r="OVE138" s="37"/>
+      <c r="OVM138" s="37"/>
+      <c r="OVU138" s="37"/>
+      <c r="OWC138" s="37"/>
+      <c r="OWK138" s="37"/>
+      <c r="OWS138" s="37"/>
+      <c r="OXA138" s="37"/>
+      <c r="OXI138" s="37"/>
+      <c r="OXQ138" s="37"/>
+      <c r="OXY138" s="37"/>
+      <c r="OYG138" s="37"/>
+      <c r="OYO138" s="37"/>
+      <c r="OYW138" s="37"/>
+      <c r="OZE138" s="37"/>
+      <c r="OZM138" s="37"/>
+      <c r="OZU138" s="37"/>
+      <c r="PAC138" s="37"/>
+      <c r="PAK138" s="37"/>
+      <c r="PAS138" s="37"/>
+      <c r="PBA138" s="37"/>
+      <c r="PBI138" s="37"/>
+      <c r="PBQ138" s="37"/>
+      <c r="PBY138" s="37"/>
+      <c r="PCG138" s="37"/>
+      <c r="PCO138" s="37"/>
+      <c r="PCW138" s="37"/>
+      <c r="PDE138" s="37"/>
+      <c r="PDM138" s="37"/>
+      <c r="PDU138" s="37"/>
+      <c r="PEC138" s="37"/>
+      <c r="PEK138" s="37"/>
+      <c r="PES138" s="37"/>
+      <c r="PFA138" s="37"/>
+      <c r="PFI138" s="37"/>
+      <c r="PFQ138" s="37"/>
+      <c r="PFY138" s="37"/>
+      <c r="PGG138" s="37"/>
+      <c r="PGO138" s="37"/>
+      <c r="PGW138" s="37"/>
+      <c r="PHE138" s="37"/>
+      <c r="PHM138" s="37"/>
+      <c r="PHU138" s="37"/>
+      <c r="PIC138" s="37"/>
+      <c r="PIK138" s="37"/>
+      <c r="PIS138" s="37"/>
+      <c r="PJA138" s="37"/>
+      <c r="PJI138" s="37"/>
+      <c r="PJQ138" s="37"/>
+      <c r="PJY138" s="37"/>
+      <c r="PKG138" s="37"/>
+      <c r="PKO138" s="37"/>
+      <c r="PKW138" s="37"/>
+      <c r="PLE138" s="37"/>
+      <c r="PLM138" s="37"/>
+      <c r="PLU138" s="37"/>
+      <c r="PMC138" s="37"/>
+      <c r="PMK138" s="37"/>
+      <c r="PMS138" s="37"/>
+      <c r="PNA138" s="37"/>
+      <c r="PNI138" s="37"/>
+      <c r="PNQ138" s="37"/>
+      <c r="PNY138" s="37"/>
+      <c r="POG138" s="37"/>
+      <c r="POO138" s="37"/>
+      <c r="POW138" s="37"/>
+      <c r="PPE138" s="37"/>
+      <c r="PPM138" s="37"/>
+      <c r="PPU138" s="37"/>
+      <c r="PQC138" s="37"/>
+      <c r="PQK138" s="37"/>
+      <c r="PQS138" s="37"/>
+      <c r="PRA138" s="37"/>
+      <c r="PRI138" s="37"/>
+      <c r="PRQ138" s="37"/>
+      <c r="PRY138" s="37"/>
+      <c r="PSG138" s="37"/>
+      <c r="PSO138" s="37"/>
+      <c r="PSW138" s="37"/>
+      <c r="PTE138" s="37"/>
+      <c r="PTM138" s="37"/>
+      <c r="PTU138" s="37"/>
+      <c r="PUC138" s="37"/>
+      <c r="PUK138" s="37"/>
+      <c r="PUS138" s="37"/>
+      <c r="PVA138" s="37"/>
+      <c r="PVI138" s="37"/>
+      <c r="PVQ138" s="37"/>
+      <c r="PVY138" s="37"/>
+      <c r="PWG138" s="37"/>
+      <c r="PWO138" s="37"/>
+      <c r="PWW138" s="37"/>
+      <c r="PXE138" s="37"/>
+      <c r="PXM138" s="37"/>
+      <c r="PXU138" s="37"/>
+      <c r="PYC138" s="37"/>
+      <c r="PYK138" s="37"/>
+      <c r="PYS138" s="37"/>
+      <c r="PZA138" s="37"/>
+      <c r="PZI138" s="37"/>
+      <c r="PZQ138" s="37"/>
+      <c r="PZY138" s="37"/>
+      <c r="QAG138" s="37"/>
+      <c r="QAO138" s="37"/>
+      <c r="QAW138" s="37"/>
+      <c r="QBE138" s="37"/>
+      <c r="QBM138" s="37"/>
+      <c r="QBU138" s="37"/>
+      <c r="QCC138" s="37"/>
+      <c r="QCK138" s="37"/>
+      <c r="QCS138" s="37"/>
+      <c r="QDA138" s="37"/>
+      <c r="QDI138" s="37"/>
+      <c r="QDQ138" s="37"/>
+      <c r="QDY138" s="37"/>
+      <c r="QEG138" s="37"/>
+      <c r="QEO138" s="37"/>
+      <c r="QEW138" s="37"/>
+      <c r="QFE138" s="37"/>
+      <c r="QFM138" s="37"/>
+      <c r="QFU138" s="37"/>
+      <c r="QGC138" s="37"/>
+      <c r="QGK138" s="37"/>
+      <c r="QGS138" s="37"/>
+      <c r="QHA138" s="37"/>
+      <c r="QHI138" s="37"/>
+      <c r="QHQ138" s="37"/>
+      <c r="QHY138" s="37"/>
+      <c r="QIG138" s="37"/>
+      <c r="QIO138" s="37"/>
+      <c r="QIW138" s="37"/>
+      <c r="QJE138" s="37"/>
+      <c r="QJM138" s="37"/>
+      <c r="QJU138" s="37"/>
+      <c r="QKC138" s="37"/>
+      <c r="QKK138" s="37"/>
+      <c r="QKS138" s="37"/>
+      <c r="QLA138" s="37"/>
+      <c r="QLI138" s="37"/>
+      <c r="QLQ138" s="37"/>
+      <c r="QLY138" s="37"/>
+      <c r="QMG138" s="37"/>
+      <c r="QMO138" s="37"/>
+      <c r="QMW138" s="37"/>
+      <c r="QNE138" s="37"/>
+      <c r="QNM138" s="37"/>
+      <c r="QNU138" s="37"/>
+      <c r="QOC138" s="37"/>
+      <c r="QOK138" s="37"/>
+      <c r="QOS138" s="37"/>
+      <c r="QPA138" s="37"/>
+      <c r="QPI138" s="37"/>
+      <c r="QPQ138" s="37"/>
+      <c r="QPY138" s="37"/>
+      <c r="QQG138" s="37"/>
+      <c r="QQO138" s="37"/>
+      <c r="QQW138" s="37"/>
+      <c r="QRE138" s="37"/>
+      <c r="QRM138" s="37"/>
+      <c r="QRU138" s="37"/>
+      <c r="QSC138" s="37"/>
+      <c r="QSK138" s="37"/>
+      <c r="QSS138" s="37"/>
+      <c r="QTA138" s="37"/>
+      <c r="QTI138" s="37"/>
+      <c r="QTQ138" s="37"/>
+      <c r="QTY138" s="37"/>
+      <c r="QUG138" s="37"/>
+      <c r="QUO138" s="37"/>
+      <c r="QUW138" s="37"/>
+      <c r="QVE138" s="37"/>
+      <c r="QVM138" s="37"/>
+      <c r="QVU138" s="37"/>
+      <c r="QWC138" s="37"/>
+      <c r="QWK138" s="37"/>
+      <c r="QWS138" s="37"/>
+      <c r="QXA138" s="37"/>
+      <c r="QXI138" s="37"/>
+      <c r="QXQ138" s="37"/>
+      <c r="QXY138" s="37"/>
+      <c r="QYG138" s="37"/>
+      <c r="QYO138" s="37"/>
+      <c r="QYW138" s="37"/>
+      <c r="QZE138" s="37"/>
+      <c r="QZM138" s="37"/>
+      <c r="QZU138" s="37"/>
+      <c r="RAC138" s="37"/>
+      <c r="RAK138" s="37"/>
+      <c r="RAS138" s="37"/>
+      <c r="RBA138" s="37"/>
+      <c r="RBI138" s="37"/>
+      <c r="RBQ138" s="37"/>
+      <c r="RBY138" s="37"/>
+      <c r="RCG138" s="37"/>
+      <c r="RCO138" s="37"/>
+      <c r="RCW138" s="37"/>
+      <c r="RDE138" s="37"/>
+      <c r="RDM138" s="37"/>
+      <c r="RDU138" s="37"/>
+      <c r="REC138" s="37"/>
+      <c r="REK138" s="37"/>
+      <c r="RES138" s="37"/>
+      <c r="RFA138" s="37"/>
+      <c r="RFI138" s="37"/>
+      <c r="RFQ138" s="37"/>
+      <c r="RFY138" s="37"/>
+      <c r="RGG138" s="37"/>
+      <c r="RGO138" s="37"/>
+      <c r="RGW138" s="37"/>
+      <c r="RHE138" s="37"/>
+      <c r="RHM138" s="37"/>
+      <c r="RHU138" s="37"/>
+      <c r="RIC138" s="37"/>
+      <c r="RIK138" s="37"/>
+      <c r="RIS138" s="37"/>
+      <c r="RJA138" s="37"/>
+      <c r="RJI138" s="37"/>
+      <c r="RJQ138" s="37"/>
+      <c r="RJY138" s="37"/>
+      <c r="RKG138" s="37"/>
+      <c r="RKO138" s="37"/>
+      <c r="RKW138" s="37"/>
+      <c r="RLE138" s="37"/>
+      <c r="RLM138" s="37"/>
+      <c r="RLU138" s="37"/>
+      <c r="RMC138" s="37"/>
+      <c r="RMK138" s="37"/>
+      <c r="RMS138" s="37"/>
+      <c r="RNA138" s="37"/>
+      <c r="RNI138" s="37"/>
+      <c r="RNQ138" s="37"/>
+      <c r="RNY138" s="37"/>
+      <c r="ROG138" s="37"/>
+      <c r="ROO138" s="37"/>
+      <c r="ROW138" s="37"/>
+      <c r="RPE138" s="37"/>
+      <c r="RPM138" s="37"/>
+      <c r="RPU138" s="37"/>
+      <c r="RQC138" s="37"/>
+      <c r="RQK138" s="37"/>
+      <c r="RQS138" s="37"/>
+      <c r="RRA138" s="37"/>
+      <c r="RRI138" s="37"/>
+      <c r="RRQ138" s="37"/>
+      <c r="RRY138" s="37"/>
+      <c r="RSG138" s="37"/>
+      <c r="RSO138" s="37"/>
+      <c r="RSW138" s="37"/>
+      <c r="RTE138" s="37"/>
+      <c r="RTM138" s="37"/>
+      <c r="RTU138" s="37"/>
+      <c r="RUC138" s="37"/>
+      <c r="RUK138" s="37"/>
+      <c r="RUS138" s="37"/>
+      <c r="RVA138" s="37"/>
+      <c r="RVI138" s="37"/>
+      <c r="RVQ138" s="37"/>
+      <c r="RVY138" s="37"/>
+      <c r="RWG138" s="37"/>
+      <c r="RWO138" s="37"/>
+      <c r="RWW138" s="37"/>
+      <c r="RXE138" s="37"/>
+      <c r="RXM138" s="37"/>
+      <c r="RXU138" s="37"/>
+      <c r="RYC138" s="37"/>
+      <c r="RYK138" s="37"/>
+      <c r="RYS138" s="37"/>
+      <c r="RZA138" s="37"/>
+      <c r="RZI138" s="37"/>
+      <c r="RZQ138" s="37"/>
+      <c r="RZY138" s="37"/>
+      <c r="SAG138" s="37"/>
+      <c r="SAO138" s="37"/>
+      <c r="SAW138" s="37"/>
+      <c r="SBE138" s="37"/>
+      <c r="SBM138" s="37"/>
+      <c r="SBU138" s="37"/>
+      <c r="SCC138" s="37"/>
+      <c r="SCK138" s="37"/>
+      <c r="SCS138" s="37"/>
+      <c r="SDA138" s="37"/>
+      <c r="SDI138" s="37"/>
+      <c r="SDQ138" s="37"/>
+      <c r="SDY138" s="37"/>
+      <c r="SEG138" s="37"/>
+      <c r="SEO138" s="37"/>
+      <c r="SEW138" s="37"/>
+      <c r="SFE138" s="37"/>
+      <c r="SFM138" s="37"/>
+      <c r="SFU138" s="37"/>
+      <c r="SGC138" s="37"/>
+      <c r="SGK138" s="37"/>
+      <c r="SGS138" s="37"/>
+      <c r="SHA138" s="37"/>
+      <c r="SHI138" s="37"/>
+      <c r="SHQ138" s="37"/>
+      <c r="SHY138" s="37"/>
+      <c r="SIG138" s="37"/>
+      <c r="SIO138" s="37"/>
+      <c r="SIW138" s="37"/>
+      <c r="SJE138" s="37"/>
+      <c r="SJM138" s="37"/>
+      <c r="SJU138" s="37"/>
+      <c r="SKC138" s="37"/>
+      <c r="SKK138" s="37"/>
+      <c r="SKS138" s="37"/>
+      <c r="SLA138" s="37"/>
+      <c r="SLI138" s="37"/>
+      <c r="SLQ138" s="37"/>
+      <c r="SLY138" s="37"/>
+      <c r="SMG138" s="37"/>
+      <c r="SMO138" s="37"/>
+      <c r="SMW138" s="37"/>
+      <c r="SNE138" s="37"/>
+      <c r="SNM138" s="37"/>
+      <c r="SNU138" s="37"/>
+      <c r="SOC138" s="37"/>
+      <c r="SOK138" s="37"/>
+      <c r="SOS138" s="37"/>
+      <c r="SPA138" s="37"/>
+      <c r="SPI138" s="37"/>
+      <c r="SPQ138" s="37"/>
+      <c r="SPY138" s="37"/>
+      <c r="SQG138" s="37"/>
+      <c r="SQO138" s="37"/>
+      <c r="SQW138" s="37"/>
+      <c r="SRE138" s="37"/>
+      <c r="SRM138" s="37"/>
+      <c r="SRU138" s="37"/>
+      <c r="SSC138" s="37"/>
+      <c r="SSK138" s="37"/>
+      <c r="SSS138" s="37"/>
+      <c r="STA138" s="37"/>
+      <c r="STI138" s="37"/>
+      <c r="STQ138" s="37"/>
+      <c r="STY138" s="37"/>
+      <c r="SUG138" s="37"/>
+      <c r="SUO138" s="37"/>
+      <c r="SUW138" s="37"/>
+      <c r="SVE138" s="37"/>
+      <c r="SVM138" s="37"/>
+      <c r="SVU138" s="37"/>
+      <c r="SWC138" s="37"/>
+      <c r="SWK138" s="37"/>
+      <c r="SWS138" s="37"/>
+      <c r="SXA138" s="37"/>
+      <c r="SXI138" s="37"/>
+      <c r="SXQ138" s="37"/>
+      <c r="SXY138" s="37"/>
+      <c r="SYG138" s="37"/>
+      <c r="SYO138" s="37"/>
+      <c r="SYW138" s="37"/>
+      <c r="SZE138" s="37"/>
+      <c r="SZM138" s="37"/>
+      <c r="SZU138" s="37"/>
+      <c r="TAC138" s="37"/>
+      <c r="TAK138" s="37"/>
+      <c r="TAS138" s="37"/>
+      <c r="TBA138" s="37"/>
+      <c r="TBI138" s="37"/>
+      <c r="TBQ138" s="37"/>
+      <c r="TBY138" s="37"/>
+      <c r="TCG138" s="37"/>
+      <c r="TCO138" s="37"/>
+      <c r="TCW138" s="37"/>
+      <c r="TDE138" s="37"/>
+      <c r="TDM138" s="37"/>
+      <c r="TDU138" s="37"/>
+      <c r="TEC138" s="37"/>
+      <c r="TEK138" s="37"/>
+      <c r="TES138" s="37"/>
+      <c r="TFA138" s="37"/>
+      <c r="TFI138" s="37"/>
+      <c r="TFQ138" s="37"/>
+      <c r="TFY138" s="37"/>
+      <c r="TGG138" s="37"/>
+      <c r="TGO138" s="37"/>
+      <c r="TGW138" s="37"/>
+      <c r="THE138" s="37"/>
+      <c r="THM138" s="37"/>
+      <c r="THU138" s="37"/>
+      <c r="TIC138" s="37"/>
+      <c r="TIK138" s="37"/>
+      <c r="TIS138" s="37"/>
+      <c r="TJA138" s="37"/>
+      <c r="TJI138" s="37"/>
+      <c r="TJQ138" s="37"/>
+      <c r="TJY138" s="37"/>
+      <c r="TKG138" s="37"/>
+      <c r="TKO138" s="37"/>
+      <c r="TKW138" s="37"/>
+      <c r="TLE138" s="37"/>
+      <c r="TLM138" s="37"/>
+      <c r="TLU138" s="37"/>
+      <c r="TMC138" s="37"/>
+      <c r="TMK138" s="37"/>
+      <c r="TMS138" s="37"/>
+      <c r="TNA138" s="37"/>
+      <c r="TNI138" s="37"/>
+      <c r="TNQ138" s="37"/>
+      <c r="TNY138" s="37"/>
+      <c r="TOG138" s="37"/>
+      <c r="TOO138" s="37"/>
+      <c r="TOW138" s="37"/>
+      <c r="TPE138" s="37"/>
+      <c r="TPM138" s="37"/>
+      <c r="TPU138" s="37"/>
+      <c r="TQC138" s="37"/>
+      <c r="TQK138" s="37"/>
+      <c r="TQS138" s="37"/>
+      <c r="TRA138" s="37"/>
+      <c r="TRI138" s="37"/>
+      <c r="TRQ138" s="37"/>
+      <c r="TRY138" s="37"/>
+      <c r="TSG138" s="37"/>
+      <c r="TSO138" s="37"/>
+      <c r="TSW138" s="37"/>
+      <c r="TTE138" s="37"/>
+      <c r="TTM138" s="37"/>
+      <c r="TTU138" s="37"/>
+      <c r="TUC138" s="37"/>
+      <c r="TUK138" s="37"/>
+      <c r="TUS138" s="37"/>
+      <c r="TVA138" s="37"/>
+      <c r="TVI138" s="37"/>
+      <c r="TVQ138" s="37"/>
+      <c r="TVY138" s="37"/>
+      <c r="TWG138" s="37"/>
+      <c r="TWO138" s="37"/>
+      <c r="TWW138" s="37"/>
+      <c r="TXE138" s="37"/>
+      <c r="TXM138" s="37"/>
+      <c r="TXU138" s="37"/>
+      <c r="TYC138" s="37"/>
+      <c r="TYK138" s="37"/>
+      <c r="TYS138" s="37"/>
+      <c r="TZA138" s="37"/>
+      <c r="TZI138" s="37"/>
+      <c r="TZQ138" s="37"/>
+      <c r="TZY138" s="37"/>
+      <c r="UAG138" s="37"/>
+      <c r="UAO138" s="37"/>
+      <c r="UAW138" s="37"/>
+      <c r="UBE138" s="37"/>
+      <c r="UBM138" s="37"/>
+      <c r="UBU138" s="37"/>
+      <c r="UCC138" s="37"/>
+      <c r="UCK138" s="37"/>
+      <c r="UCS138" s="37"/>
+      <c r="UDA138" s="37"/>
+      <c r="UDI138" s="37"/>
+      <c r="UDQ138" s="37"/>
+      <c r="UDY138" s="37"/>
+      <c r="UEG138" s="37"/>
+      <c r="UEO138" s="37"/>
+      <c r="UEW138" s="37"/>
+      <c r="UFE138" s="37"/>
+      <c r="UFM138" s="37"/>
+      <c r="UFU138" s="37"/>
+      <c r="UGC138" s="37"/>
+      <c r="UGK138" s="37"/>
+      <c r="UGS138" s="37"/>
+      <c r="UHA138" s="37"/>
+      <c r="UHI138" s="37"/>
+      <c r="UHQ138" s="37"/>
+      <c r="UHY138" s="37"/>
+      <c r="UIG138" s="37"/>
+      <c r="UIO138" s="37"/>
+      <c r="UIW138" s="37"/>
+      <c r="UJE138" s="37"/>
+      <c r="UJM138" s="37"/>
+      <c r="UJU138" s="37"/>
+      <c r="UKC138" s="37"/>
+      <c r="UKK138" s="37"/>
+      <c r="UKS138" s="37"/>
+      <c r="ULA138" s="37"/>
+      <c r="ULI138" s="37"/>
+      <c r="ULQ138" s="37"/>
+      <c r="ULY138" s="37"/>
+      <c r="UMG138" s="37"/>
+      <c r="UMO138" s="37"/>
+      <c r="UMW138" s="37"/>
+      <c r="UNE138" s="37"/>
+      <c r="UNM138" s="37"/>
+      <c r="UNU138" s="37"/>
+      <c r="UOC138" s="37"/>
+      <c r="UOK138" s="37"/>
+      <c r="UOS138" s="37"/>
+      <c r="UPA138" s="37"/>
+      <c r="UPI138" s="37"/>
+      <c r="UPQ138" s="37"/>
+      <c r="UPY138" s="37"/>
+      <c r="UQG138" s="37"/>
+      <c r="UQO138" s="37"/>
+      <c r="UQW138" s="37"/>
+      <c r="URE138" s="37"/>
+      <c r="URM138" s="37"/>
+      <c r="URU138" s="37"/>
+      <c r="USC138" s="37"/>
+      <c r="USK138" s="37"/>
+      <c r="USS138" s="37"/>
+      <c r="UTA138" s="37"/>
+      <c r="UTI138" s="37"/>
+      <c r="UTQ138" s="37"/>
+      <c r="UTY138" s="37"/>
+      <c r="UUG138" s="37"/>
+      <c r="UUO138" s="37"/>
+      <c r="UUW138" s="37"/>
+      <c r="UVE138" s="37"/>
+      <c r="UVM138" s="37"/>
+      <c r="UVU138" s="37"/>
+      <c r="UWC138" s="37"/>
+      <c r="UWK138" s="37"/>
+      <c r="UWS138" s="37"/>
+      <c r="UXA138" s="37"/>
+      <c r="UXI138" s="37"/>
+      <c r="UXQ138" s="37"/>
+      <c r="UXY138" s="37"/>
+      <c r="UYG138" s="37"/>
+      <c r="UYO138" s="37"/>
+      <c r="UYW138" s="37"/>
+      <c r="UZE138" s="37"/>
+      <c r="UZM138" s="37"/>
+      <c r="UZU138" s="37"/>
+      <c r="VAC138" s="37"/>
+      <c r="VAK138" s="37"/>
+      <c r="VAS138" s="37"/>
+      <c r="VBA138" s="37"/>
+      <c r="VBI138" s="37"/>
+      <c r="VBQ138" s="37"/>
+      <c r="VBY138" s="37"/>
+      <c r="VCG138" s="37"/>
+      <c r="VCO138" s="37"/>
+      <c r="VCW138" s="37"/>
+      <c r="VDE138" s="37"/>
+      <c r="VDM138" s="37"/>
+      <c r="VDU138" s="37"/>
+      <c r="VEC138" s="37"/>
+      <c r="VEK138" s="37"/>
+      <c r="VES138" s="37"/>
+      <c r="VFA138" s="37"/>
+      <c r="VFI138" s="37"/>
+      <c r="VFQ138" s="37"/>
+      <c r="VFY138" s="37"/>
+      <c r="VGG138" s="37"/>
+      <c r="VGO138" s="37"/>
+      <c r="VGW138" s="37"/>
+      <c r="VHE138" s="37"/>
+      <c r="VHM138" s="37"/>
+      <c r="VHU138" s="37"/>
+      <c r="VIC138" s="37"/>
+      <c r="VIK138" s="37"/>
+      <c r="VIS138" s="37"/>
+      <c r="VJA138" s="37"/>
+      <c r="VJI138" s="37"/>
+      <c r="VJQ138" s="37"/>
+      <c r="VJY138" s="37"/>
+      <c r="VKG138" s="37"/>
+      <c r="VKO138" s="37"/>
+      <c r="VKW138" s="37"/>
+      <c r="VLE138" s="37"/>
+      <c r="VLM138" s="37"/>
+      <c r="VLU138" s="37"/>
+      <c r="VMC138" s="37"/>
+      <c r="VMK138" s="37"/>
+      <c r="VMS138" s="37"/>
+      <c r="VNA138" s="37"/>
+      <c r="VNI138" s="37"/>
+      <c r="VNQ138" s="37"/>
+      <c r="VNY138" s="37"/>
+      <c r="VOG138" s="37"/>
+      <c r="VOO138" s="37"/>
+      <c r="VOW138" s="37"/>
+      <c r="VPE138" s="37"/>
+      <c r="VPM138" s="37"/>
+      <c r="VPU138" s="37"/>
+      <c r="VQC138" s="37"/>
+      <c r="VQK138" s="37"/>
+      <c r="VQS138" s="37"/>
+      <c r="VRA138" s="37"/>
+      <c r="VRI138" s="37"/>
+      <c r="VRQ138" s="37"/>
+      <c r="VRY138" s="37"/>
+      <c r="VSG138" s="37"/>
+      <c r="VSO138" s="37"/>
+      <c r="VSW138" s="37"/>
+      <c r="VTE138" s="37"/>
+      <c r="VTM138" s="37"/>
+      <c r="VTU138" s="37"/>
+      <c r="VUC138" s="37"/>
+      <c r="VUK138" s="37"/>
+      <c r="VUS138" s="37"/>
+      <c r="VVA138" s="37"/>
+      <c r="VVI138" s="37"/>
+      <c r="VVQ138" s="37"/>
+      <c r="VVY138" s="37"/>
+      <c r="VWG138" s="37"/>
+      <c r="VWO138" s="37"/>
+      <c r="VWW138" s="37"/>
+      <c r="VXE138" s="37"/>
+      <c r="VXM138" s="37"/>
+      <c r="VXU138" s="37"/>
+      <c r="VYC138" s="37"/>
+      <c r="VYK138" s="37"/>
+      <c r="VYS138" s="37"/>
+      <c r="VZA138" s="37"/>
+      <c r="VZI138" s="37"/>
+      <c r="VZQ138" s="37"/>
+      <c r="VZY138" s="37"/>
+      <c r="WAG138" s="37"/>
+      <c r="WAO138" s="37"/>
+      <c r="WAW138" s="37"/>
+      <c r="WBE138" s="37"/>
+      <c r="WBM138" s="37"/>
+      <c r="WBU138" s="37"/>
+      <c r="WCC138" s="37"/>
+      <c r="WCK138" s="37"/>
+      <c r="WCS138" s="37"/>
+      <c r="WDA138" s="37"/>
+      <c r="WDI138" s="37"/>
+      <c r="WDQ138" s="37"/>
+      <c r="WDY138" s="37"/>
+      <c r="WEG138" s="37"/>
+      <c r="WEO138" s="37"/>
+      <c r="WEW138" s="37"/>
+      <c r="WFE138" s="37"/>
+      <c r="WFM138" s="37"/>
+      <c r="WFU138" s="37"/>
+      <c r="WGC138" s="37"/>
+      <c r="WGK138" s="37"/>
+      <c r="WGS138" s="37"/>
+      <c r="WHA138" s="37"/>
+      <c r="WHI138" s="37"/>
+      <c r="WHQ138" s="37"/>
+      <c r="WHY138" s="37"/>
+      <c r="WIG138" s="37"/>
+      <c r="WIO138" s="37"/>
+      <c r="WIW138" s="37"/>
+      <c r="WJE138" s="37"/>
+      <c r="WJM138" s="37"/>
+      <c r="WJU138" s="37"/>
+      <c r="WKC138" s="37"/>
+      <c r="WKK138" s="37"/>
+      <c r="WKS138" s="37"/>
+      <c r="WLA138" s="37"/>
+      <c r="WLI138" s="37"/>
+      <c r="WLQ138" s="37"/>
+      <c r="WLY138" s="37"/>
+      <c r="WMG138" s="37"/>
+      <c r="WMO138" s="37"/>
+      <c r="WMW138" s="37"/>
+      <c r="WNE138" s="37"/>
+      <c r="WNM138" s="37"/>
+      <c r="WNU138" s="37"/>
+      <c r="WOC138" s="37"/>
+      <c r="WOK138" s="37"/>
+      <c r="WOS138" s="37"/>
+      <c r="WPA138" s="37"/>
+      <c r="WPI138" s="37"/>
+      <c r="WPQ138" s="37"/>
+      <c r="WPY138" s="37"/>
+      <c r="WQG138" s="37"/>
+      <c r="WQO138" s="37"/>
+      <c r="WQW138" s="37"/>
+      <c r="WRE138" s="37"/>
+      <c r="WRM138" s="37"/>
+      <c r="WRU138" s="37"/>
+      <c r="WSC138" s="37"/>
+      <c r="WSK138" s="37"/>
+      <c r="WSS138" s="37"/>
+      <c r="WTA138" s="37"/>
+      <c r="WTI138" s="37"/>
+      <c r="WTQ138" s="37"/>
+      <c r="WTY138" s="37"/>
+      <c r="WUG138" s="37"/>
+      <c r="WUO138" s="37"/>
+      <c r="WUW138" s="37"/>
+      <c r="WVE138" s="37"/>
+      <c r="WVM138" s="37"/>
+      <c r="WVU138" s="37"/>
+      <c r="WWC138" s="37"/>
+      <c r="WWK138" s="37"/>
+      <c r="WWS138" s="37"/>
+      <c r="WXA138" s="37"/>
+      <c r="WXI138" s="37"/>
+      <c r="WXQ138" s="37"/>
+      <c r="WXY138" s="37"/>
+      <c r="WYG138" s="37"/>
+      <c r="WYO138" s="37"/>
+      <c r="WYW138" s="37"/>
+      <c r="WZE138" s="37"/>
+      <c r="WZM138" s="37"/>
+      <c r="WZU138" s="37"/>
+      <c r="XAC138" s="37"/>
+      <c r="XAK138" s="37"/>
+      <c r="XAS138" s="37"/>
+      <c r="XBA138" s="37"/>
+      <c r="XBI138" s="37"/>
+      <c r="XBQ138" s="37"/>
+      <c r="XBY138" s="37"/>
+      <c r="XCG138" s="37"/>
+      <c r="XCO138" s="37"/>
+      <c r="XCW138" s="37"/>
+      <c r="XDE138" s="37"/>
+      <c r="XDM138" s="37"/>
+      <c r="XDU138" s="37"/>
+      <c r="XEC138" s="37"/>
+      <c r="XEK138" s="37"/>
+      <c r="XES138" s="37"/>
+      <c r="XFA138" s="37"/>
     </row>
     <row r="139" spans="1:1021 1029:2045 2053:3069 3077:4093 4101:5117 5125:6141 6149:7165 7173:8189 8197:9213 9221:10237 10245:11261 11269:12285 12293:13309 13317:14333 14341:15357 15365:16381" s="4" customFormat="1">
       <c r="A139" s="4" t="s">
@@ -10564,73 +10565,73 @@
         <v>231</v>
       </c>
     </row>
-    <row r="238" spans="1:14">
-      <c r="A238" t="s">
-        <v>96</v>
-      </c>
-      <c r="B238" t="s">
+    <row r="238" spans="1:14" s="34" customFormat="1">
+      <c r="A238" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="B238" s="34" t="s">
         <v>634</v>
       </c>
-      <c r="C238" t="s">
+      <c r="C238" s="34" t="s">
         <v>260</v>
       </c>
-      <c r="D238" t="s">
+      <c r="D238" s="34" t="s">
         <v>635</v>
       </c>
-      <c r="E238" s="31" t="s">
+      <c r="E238" s="45" t="s">
         <v>636</v>
       </c>
-      <c r="F238" t="s">
+      <c r="F238" s="34" t="s">
         <v>639</v>
       </c>
-      <c r="G238" t="s">
+      <c r="G238" s="34" t="s">
         <v>640</v>
       </c>
-      <c r="H238" t="s">
+      <c r="H238" s="34" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="239" spans="1:14">
-      <c r="A239" t="s">
-        <v>96</v>
-      </c>
-      <c r="B239" t="s">
+    <row r="239" spans="1:14" s="34" customFormat="1">
+      <c r="A239" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="B239" s="34" t="s">
         <v>637</v>
       </c>
-      <c r="C239" t="s">
+      <c r="C239" s="34" t="s">
         <v>260</v>
       </c>
-      <c r="D239" s="31" t="s">
+      <c r="D239" s="45" t="s">
         <v>635</v>
       </c>
-      <c r="E239" t="s">
+      <c r="E239" s="34" t="s">
         <v>675</v>
       </c>
-      <c r="F239" t="s">
+      <c r="F239" s="34" t="s">
         <v>679</v>
       </c>
-      <c r="G239" t="s">
+      <c r="G239" s="34" t="s">
         <v>641</v>
       </c>
-      <c r="H239" t="s">
+      <c r="H239" s="34" t="s">
         <v>307</v>
       </c>
-      <c r="I239" t="s">
+      <c r="I239" s="34" t="s">
         <v>642</v>
       </c>
-      <c r="J239" t="s">
+      <c r="J239" s="34" t="s">
         <v>307</v>
       </c>
-      <c r="K239" t="s">
+      <c r="K239" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="L239" t="s">
+      <c r="L239" s="34" t="s">
         <v>307</v>
       </c>
-      <c r="M239" t="s">
+      <c r="M239" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="N239" t="s">
+      <c r="N239" s="34" t="s">
         <v>307</v>
       </c>
     </row>
@@ -10688,7 +10689,7 @@
       <c r="C241" t="s">
         <v>656</v>
       </c>
-      <c r="D241" s="39" t="s">
+      <c r="D241" s="38" t="s">
         <v>657</v>
       </c>
       <c r="E241" s="2" t="s">
@@ -10708,7 +10709,7 @@
       <c r="C242" t="s">
         <v>656</v>
       </c>
-      <c r="D242" s="39" t="s">
+      <c r="D242" s="38" t="s">
         <v>657</v>
       </c>
       <c r="E242" s="2" t="s">
@@ -10728,7 +10729,7 @@
       <c r="C243" t="s">
         <v>656</v>
       </c>
-      <c r="D243" s="39" t="s">
+      <c r="D243" s="38" t="s">
         <v>657</v>
       </c>
       <c r="E243" s="2" t="s">
@@ -10748,7 +10749,7 @@
       <c r="C244" t="s">
         <v>656</v>
       </c>
-      <c r="D244" s="39" t="s">
+      <c r="D244" s="38" t="s">
         <v>657</v>
       </c>
       <c r="E244" s="2" t="s">
@@ -10768,7 +10769,7 @@
       <c r="C245" t="s">
         <v>656</v>
       </c>
-      <c r="D245" s="39" t="s">
+      <c r="D245" s="38" t="s">
         <v>657</v>
       </c>
       <c r="E245" s="2" t="s">
@@ -10788,7 +10789,7 @@
       <c r="C246" t="s">
         <v>656</v>
       </c>
-      <c r="D246" s="39" t="s">
+      <c r="D246" s="38" t="s">
         <v>657</v>
       </c>
       <c r="E246" s="2" t="s">
@@ -10808,7 +10809,7 @@
       <c r="C247" t="s">
         <v>656</v>
       </c>
-      <c r="D247" s="39" t="s">
+      <c r="D247" s="38" t="s">
         <v>657</v>
       </c>
       <c r="E247" s="2" t="s">
@@ -10828,7 +10829,7 @@
       <c r="C248" t="s">
         <v>656</v>
       </c>
-      <c r="D248" s="39" t="s">
+      <c r="D248" s="38" t="s">
         <v>657</v>
       </c>
       <c r="E248" s="2" t="s">
@@ -11324,6 +11325,11 @@
     <row r="42" spans="1:41">
       <c r="A42" t="s">
         <v>376</v>
+      </c>
+    </row>
+    <row r="43" spans="1:41">
+      <c r="A43" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="44" spans="1:41" s="10" customFormat="1">
@@ -11548,75 +11554,75 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:10" s="32" customFormat="1" ht="29">
-      <c r="A6" s="32" t="s">
+    <row r="6" spans="1:10" s="31" customFormat="1" ht="29">
+      <c r="A6" s="31" t="s">
         <v>643</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="32" t="s">
         <v>509</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="31" t="s">
         <v>463</v>
       </c>
-      <c r="D6" s="32" t="s">
+      <c r="D6" s="31" t="s">
         <v>588</v>
       </c>
-      <c r="E6" s="34" t="s">
+      <c r="E6" s="33" t="s">
         <v>589</v>
       </c>
-      <c r="F6" s="32" t="s">
+      <c r="F6" s="31" t="s">
         <v>590</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="G6" s="31" t="s">
         <v>592</v>
       </c>
-      <c r="H6" s="32" t="s">
+      <c r="H6" s="31" t="s">
         <v>381</v>
       </c>
-      <c r="I6" s="32" t="s">
+      <c r="I6" s="31" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:10" s="32" customFormat="1">
-      <c r="A7" s="32" t="s">
+    <row r="7" spans="1:10" s="31" customFormat="1">
+      <c r="A7" s="31" t="s">
         <v>643</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="32" t="s">
         <v>509</v>
       </c>
-      <c r="D7" s="32" t="s">
+      <c r="D7" s="31" t="s">
         <v>587</v>
       </c>
-      <c r="E7" s="34"/>
-      <c r="F7" s="32" t="s">
+      <c r="E7" s="33"/>
+      <c r="F7" s="31" t="s">
         <v>474</v>
       </c>
-      <c r="G7" s="32" t="s">
+      <c r="G7" s="31" t="s">
         <v>380</v>
       </c>
-      <c r="H7" s="32" t="s">
+      <c r="H7" s="31" t="s">
         <v>87</v>
       </c>
-      <c r="I7" s="32" t="s">
+      <c r="I7" s="31" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:10" s="32" customFormat="1">
-      <c r="A8" s="32" t="s">
+    <row r="8" spans="1:10" s="31" customFormat="1">
+      <c r="A8" s="31" t="s">
         <v>643</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="D8" s="32" t="s">
+      <c r="B8" s="32"/>
+      <c r="D8" s="31" t="s">
         <v>591</v>
       </c>
-      <c r="E8" s="34"/>
-      <c r="G8" s="32" t="s">
+      <c r="E8" s="33"/>
+      <c r="G8" s="31" t="s">
         <v>86</v>
       </c>
-      <c r="H8" s="32" t="s">
+      <c r="H8" s="31" t="s">
         <v>381</v>
       </c>
-      <c r="I8" s="32" t="s">
+      <c r="I8" s="31" t="s">
         <v>77</v>
       </c>
     </row>
@@ -11709,32 +11715,32 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:10" s="32" customFormat="1" ht="43.5">
-      <c r="A14" s="34" t="s">
+    <row r="14" spans="1:10" s="31" customFormat="1" ht="43.5">
+      <c r="A14" s="33" t="s">
         <v>644</v>
       </c>
-      <c r="B14" s="33" t="s">
+      <c r="B14" s="32" t="s">
         <v>508</v>
       </c>
-      <c r="C14" s="32" t="s">
+      <c r="C14" s="31" t="s">
         <v>463</v>
       </c>
-      <c r="D14" s="32" t="s">
+      <c r="D14" s="31" t="s">
         <v>469</v>
       </c>
-      <c r="E14" s="34" t="s">
+      <c r="E14" s="33" t="s">
         <v>470</v>
       </c>
-      <c r="F14" s="32" t="s">
+      <c r="F14" s="31" t="s">
         <v>586</v>
       </c>
-      <c r="G14" s="32" t="s">
+      <c r="G14" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="32" t="s">
+      <c r="H14" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="I14" s="32" t="s">
+      <c r="I14" s="31" t="s">
         <v>84</v>
       </c>
     </row>
@@ -11897,29 +11903,29 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:10" s="35" customFormat="1" ht="29">
-      <c r="A21" s="35" t="s">
+    <row r="21" spans="1:10" s="34" customFormat="1" ht="29">
+      <c r="A21" s="34" t="s">
         <v>645</v>
       </c>
-      <c r="B21" s="36" t="s">
+      <c r="B21" s="35" t="s">
         <v>508</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="34" t="s">
         <v>462</v>
       </c>
-      <c r="D21" s="35" t="s">
+      <c r="D21" s="34" t="s">
         <v>531</v>
       </c>
-      <c r="E21" s="37" t="s">
+      <c r="E21" s="36" t="s">
         <v>532</v>
       </c>
-      <c r="F21" s="35" t="s">
+      <c r="F21" s="34" t="s">
         <v>533</v>
       </c>
-      <c r="G21" s="35" t="s">
+      <c r="G21" s="34" t="s">
         <v>528</v>
       </c>
-      <c r="H21" s="35" t="s">
+      <c r="H21" s="34" t="s">
         <v>77</v>
       </c>
     </row>
@@ -12372,72 +12378,76 @@
       <c r="B39" s="29"/>
     </row>
     <row r="42" spans="1:9">
-      <c r="A42" s="40" t="s">
+      <c r="A42" s="39" t="s">
         <v>663</v>
       </c>
-      <c r="B42" s="41"/>
-      <c r="C42" s="40"/>
-      <c r="D42" s="40"/>
-      <c r="E42" s="42"/>
-      <c r="F42" s="40"/>
-      <c r="G42" s="40"/>
-    </row>
-    <row r="43" spans="1:9">
-      <c r="A43" s="41" t="s">
+      <c r="B42" s="40"/>
+      <c r="C42" s="39"/>
+      <c r="D42" s="39"/>
+      <c r="E42" s="41"/>
+      <c r="F42" s="39"/>
+      <c r="G42" s="39"/>
+    </row>
+    <row r="43" spans="1:9" s="7" customFormat="1">
+      <c r="A43" s="43" t="s">
         <v>664</v>
       </c>
-      <c r="B43" s="40" t="s">
+      <c r="B43" s="7" t="s">
         <v>464</v>
       </c>
-      <c r="C43" s="44" t="s">
+      <c r="C43" s="7" t="s">
         <v>661</v>
       </c>
-      <c r="D43" s="42"/>
-      <c r="F43" s="40" t="s">
+      <c r="D43" s="6"/>
+      <c r="E43" s="6"/>
+      <c r="F43" s="7" t="s">
         <v>662</v>
       </c>
-      <c r="G43" s="40" t="s">
+      <c r="G43" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="H43" s="40" t="s">
+      <c r="H43" s="7" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="44" spans="1:9">
-      <c r="A44" s="40" t="s">
+      <c r="A44" s="39" t="s">
         <v>671</v>
       </c>
-      <c r="B44" s="40"/>
-      <c r="C44" s="40" t="s">
+      <c r="B44" s="39"/>
+      <c r="C44" s="39" t="s">
         <v>672</v>
       </c>
-      <c r="D44" s="42"/>
-      <c r="F44" s="40" t="s">
+      <c r="D44" s="41"/>
+      <c r="F44" s="39" t="s">
         <v>674</v>
       </c>
-      <c r="G44" s="40" t="s">
+      <c r="G44" s="39" t="s">
         <v>77</v>
       </c>
-      <c r="H44" s="40" t="s">
+      <c r="H44" s="39" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="45" spans="1:9">
-      <c r="A45" s="40" t="s">
+    <row r="45" spans="1:9" s="12" customFormat="1">
+      <c r="A45" s="12" t="s">
         <v>667</v>
       </c>
-      <c r="B45" s="40"/>
-      <c r="C45" s="40" t="s">
+      <c r="B45" s="44" t="s">
+        <v>681</v>
+      </c>
+      <c r="C45" s="12" t="s">
         <v>668</v>
       </c>
-      <c r="D45" s="42"/>
-      <c r="F45" s="40" t="s">
+      <c r="D45" s="16"/>
+      <c r="E45" s="16"/>
+      <c r="F45" s="12" t="s">
         <v>669</v>
       </c>
-      <c r="G45" s="40" t="s">
+      <c r="G45" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="H45" s="40" t="s">
+      <c r="H45" s="12" t="s">
         <v>670</v>
       </c>
     </row>
@@ -12445,19 +12455,15 @@
       <c r="A46" s="4" t="s">
         <v>665</v>
       </c>
-      <c r="B46" s="43"/>
+      <c r="B46" s="42"/>
       <c r="E46" s="3"/>
     </row>
-    <row r="47" spans="1:9">
-      <c r="A47" s="40" t="s">
+    <row r="47" spans="1:9" s="7" customFormat="1">
+      <c r="A47" s="7" t="s">
         <v>666</v>
       </c>
-      <c r="B47" s="41"/>
-      <c r="C47" s="40"/>
-      <c r="D47" s="40"/>
-      <c r="E47" s="42"/>
-      <c r="F47" s="40"/>
-      <c r="G47" s="40"/>
+      <c r="B47" s="43"/>
+      <c r="E47" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added code to process parent_childcare_daily, father_work_weekly, mother_work_weekly
</commit_message>
<xml_diff>
--- a/Data/JACSIS2023/processed/codebook.xlsx
+++ b/Data/JACSIS2023/processed/codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangk\Desktop\vaccination_uptake_jacsis2023\Data\JACSIS2023\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D265FA1-66AC-4DA9-868C-7AC720AB1487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F7FE580-0D5D-402B-ACF9-BD18F1E2012D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3470" yWindow="690" windowWidth="14400" windowHeight="8710" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codebook" sheetId="1" r:id="rId1"/>
@@ -48,17 +48,17 @@
   <commentList>
     <comment ref="AZ1" authorId="0" shapeId="0" xr:uid="{F627B11A-9966-4DAF-9CD9-36B5D028D9EE}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     Remove once we’ve determined how to stratify by disease</t>
       </text>
     </comment>
     <comment ref="CE1" authorId="1" shapeId="0" xr:uid="{E5BA077E-7025-4391-8B23-A38BD7E65674}">
       <text>
-        <t xml:space="preserve">[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     Remove retired status and student status? (due to the low number of respondents who fall into these categories)
 </t>
       </text>
@@ -72,13 +72,16 @@
   <authors>
     <author>tc={869B55B9-3B1F-4453-9A39-E466CC7906FC}</author>
     <author>tc={443BE410-81F7-49D5-89CA-23D177220CB4}</author>
+    <author>tc={BAE8D65E-3045-43EB-8774-A318AAC7DD18}</author>
+    <author>tc={659E73EF-A20A-4A59-9B55-54ABF25C8CD7}</author>
+    <author>tc={B95C5CB8-3E03-4E35-BDF4-3319FA60D693}</author>
   </authors>
   <commentList>
     <comment ref="L68" authorId="0" shapeId="0" xr:uid="{869B55B9-3B1F-4453-9A39-E466CC7906FC}">
       <text>
-        <t xml:space="preserve">[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     How should we define the number of parents a child has, the numebr of spouses livignin the same household? Or the marital status of the responding parent
 there are cases where parents = 1 but the responding parent is still married, and in such cases where the other parent isn’t living in the same hosuehold as them they still may have an influence on their childs’vaccination
 cases where parents = 2 but they arent married, i.e. divorced both parents might still have a say in the child’s vaccination
@@ -87,11 +90,36 @@
     </comment>
     <comment ref="E238" authorId="1" shapeId="0" xr:uid="{443BE410-81F7-49D5-89CA-23D177220CB4}">
       <text>
-        <t xml:space="preserve">[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     Come back and change the time bins based on how the data behaves
 </t>
+      </text>
+    </comment>
+    <comment ref="F238" authorId="2" shapeId="0" xr:uid="{BAE8D65E-3045-43EB-8774-A318AAC7DD18}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Is bunching those from less than 30, less than 1 hour and 1 hour together into the same bin which is 1 hour valid? 
+Assumption that those who don’t know their timing == 0 hours of childcare is not valid ?</t>
+      </text>
+    </comment>
+    <comment ref="B240" authorId="3" shapeId="0" xr:uid="{659E73EF-A20A-4A59-9B55-54ABF25C8CD7}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    To add to transform_data</t>
+      </text>
+    </comment>
+    <comment ref="B242" authorId="4" shapeId="0" xr:uid="{B95C5CB8-3E03-4E35-BDF4-3319FA60D693}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    To add to transform_data</t>
       </text>
     </comment>
   </commentList>
@@ -108,9 +136,9 @@
   <commentList>
     <comment ref="D18" authorId="0" shapeId="0" xr:uid="{7F40D788-9EC4-40FB-A9F9-AD66BD761ADD}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     Should be age_cat and age_of_interest
 I will figure it out and update once I find out which graph this is referring to</t>
       </text>
@@ -143,9 +171,9 @@
     </comment>
     <comment ref="A47" authorId="2" shapeId="0" xr:uid="{96A696B5-9B70-421D-BAE5-16DC63333B7B}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     Will be interesting to see if marital status (i..e single parents) are affected by the number of children they have to care for.</t>
       </text>
     </comment>
@@ -154,7 +182,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2036" uniqueCount="683">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2046" uniqueCount="688">
   <si>
     <t>Variable Name</t>
     <phoneticPr fontId="2"/>
@@ -2069,18 +2097,12 @@
     <t>hours</t>
   </si>
   <si>
-    <t>The number of hours the responding parent spends on childcare in a week</t>
-  </si>
-  <si>
     <t>father_work_weekly</t>
   </si>
   <si>
     <t>mother_work_weekly</t>
   </si>
   <si>
-    <t>use the median value of the time bin of the number of hours spent per week on childcare by the responding parent</t>
-  </si>
-  <si>
     <t>childcare_daily</t>
   </si>
   <si>
@@ -2208,6 +2230,27 @@
   </si>
   <si>
     <t>mother's working hours</t>
+  </si>
+  <si>
+    <t>The average number of hours the responding parent spends on childcare a day (over the past month)</t>
+  </si>
+  <si>
+    <t>use the median value of the time bin of the number of hours spent per week on childcare by the responding parent`; Bunch 0 to 1 hour bins together as 1 hour; For parents who don't know code them as 0 hours</t>
+  </si>
+  <si>
+    <t>log(father_work_weekly)</t>
+  </si>
+  <si>
+    <t>log hours</t>
+  </si>
+  <si>
+    <t>log of father_work_weekly as it's right skewed with a few EXTREMELY HIGH observations. We want to reduce the impact of these high working hours; log values ar NA and anything &gt; 0 as the hours provided are integers thus the lowest possible log is log 1 = 0</t>
+  </si>
+  <si>
+    <t>log(mother_work_weekly)</t>
+  </si>
+  <si>
+    <t>log of mother_work_weekly as it's right skewed with a few EXTREMELY HIGH observations. We want to reduce the impact of these high working hours; log values ar NA and anything &gt; 0 as the hours provided are integers thus the lowest possible log is log 1 = 0</t>
   </si>
 </sst>
 </file>
@@ -2411,7 +2454,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2479,10 +2522,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
@@ -2823,9 +2868,19 @@
 cases where parents = 2 but they arent married, i.e. divorced both parents might still have a say in the child’s vaccination
 </text>
   </threadedComment>
-  <threadedComment ref="E238" dT="2025-06-10T09:37:58.90" personId="{018BAD65-E158-4456-AEB2-B6F599AC9FA9}" id="{443BE410-81F7-49D5-89CA-23D177220CB4}">
+  <threadedComment ref="E238" dT="2025-06-10T09:37:58.90" personId="{018BAD65-E158-4456-AEB2-B6F599AC9FA9}" id="{443BE410-81F7-49D5-89CA-23D177220CB4}" done="1">
     <text xml:space="preserve">Come back and change the time bins based on how the data behaves
 </text>
+  </threadedComment>
+  <threadedComment ref="F238" dT="2026-05-21T00:40:01.67" personId="{F1230DF4-625E-4957-ABA0-003D3672236E}" id="{BAE8D65E-3045-43EB-8774-A318AAC7DD18}">
+    <text>Is bunching those from less than 30, less than 1 hour and 1 hour together into the same bin which is 1 hour valid? 
+Assumption that those who don’t know their timing == 0 hours of childcare is not valid ?</text>
+  </threadedComment>
+  <threadedComment ref="B240" dT="2026-05-21T02:47:05.83" personId="{F1230DF4-625E-4957-ABA0-003D3672236E}" id="{659E73EF-A20A-4A59-9B55-54ABF25C8CD7}">
+    <text>To add to transform_data</text>
+  </threadedComment>
+  <threadedComment ref="B242" dT="2026-05-21T02:47:05.83" personId="{F1230DF4-625E-4957-ABA0-003D3672236E}" id="{B95C5CB8-3E03-4E35-BDF4-3319FA60D693}">
+    <text>To add to transform_data</text>
   </threadedComment>
 </ThreadedComments>
 </file>
@@ -3189,13 +3244,13 @@
         <v>632</v>
       </c>
       <c r="CV1" s="7" t="s">
+        <v>636</v>
+      </c>
+      <c r="CW1" s="7" t="s">
         <v>637</v>
       </c>
-      <c r="CW1" s="7" t="s">
-        <v>638</v>
-      </c>
       <c r="CX1" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="CY1" t="s">
         <v>56</v>
@@ -3783,28 +3838,28 @@
         <v>633</v>
       </c>
       <c r="CX3" s="2" t="s">
+        <v>645</v>
+      </c>
+      <c r="CY3" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="CZ3" s="2" t="s">
         <v>647</v>
       </c>
-      <c r="CY3" s="2" t="s">
+      <c r="DA3" s="2" t="s">
         <v>648</v>
       </c>
-      <c r="CZ3" s="2" t="s">
+      <c r="DB3" s="2" t="s">
         <v>649</v>
       </c>
-      <c r="DA3" s="2" t="s">
+      <c r="DC3" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="DB3" s="2" t="s">
+      <c r="DD3" s="2" t="s">
         <v>651</v>
       </c>
-      <c r="DC3" s="2" t="s">
+      <c r="DE3" s="2" t="s">
         <v>652</v>
-      </c>
-      <c r="DD3" s="2" t="s">
-        <v>653</v>
-      </c>
-      <c r="DE3" s="2" t="s">
-        <v>654</v>
       </c>
     </row>
     <row r="4" spans="1:110">
@@ -4112,28 +4167,28 @@
         <v>631</v>
       </c>
       <c r="CX4" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="CY4" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="CZ4" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="DA4" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="DB4" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="DC4" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="DD4" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="DE4" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
     </row>
     <row r="5" spans="1:110">
@@ -4276,7 +4331,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83406F25-8B9E-4B45-BE5A-CFE07640E852}">
-  <dimension ref="A1:XFA248"/>
+  <dimension ref="A1:XFA250"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="35.81640625" bestFit="1" customWidth="1"/>
@@ -8994,7 +9049,7 @@
         <v>201</v>
       </c>
       <c r="F147" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="G147" t="s">
         <v>66</v>
@@ -9088,7 +9143,7 @@
         <v>201</v>
       </c>
       <c r="F152" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="G152" t="s">
         <v>66</v>
@@ -10565,278 +10620,312 @@
         <v>231</v>
       </c>
     </row>
-    <row r="238" spans="1:14" s="34" customFormat="1">
-      <c r="A238" s="34" t="s">
-        <v>96</v>
-      </c>
-      <c r="B238" s="34" t="s">
+    <row r="238" spans="1:14" s="46" customFormat="1">
+      <c r="A238" s="46" t="s">
+        <v>96</v>
+      </c>
+      <c r="B238" s="46" t="s">
         <v>634</v>
       </c>
-      <c r="C238" s="34" t="s">
+      <c r="C238" s="46" t="s">
         <v>260</v>
       </c>
-      <c r="D238" s="34" t="s">
+      <c r="D238" s="46" t="s">
         <v>635</v>
       </c>
-      <c r="E238" s="45" t="s">
+      <c r="E238" s="47" t="s">
+        <v>681</v>
+      </c>
+      <c r="F238" s="46" t="s">
+        <v>682</v>
+      </c>
+      <c r="G238" s="46" t="s">
+        <v>638</v>
+      </c>
+      <c r="H238" s="46" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="239" spans="1:14" s="46" customFormat="1">
+      <c r="A239" s="46" t="s">
+        <v>96</v>
+      </c>
+      <c r="B239" s="46" t="s">
         <v>636</v>
       </c>
-      <c r="F238" s="34" t="s">
+      <c r="C239" s="46" t="s">
+        <v>260</v>
+      </c>
+      <c r="D239" s="47" t="s">
+        <v>635</v>
+      </c>
+      <c r="E239" s="46" t="s">
+        <v>673</v>
+      </c>
+      <c r="F239" s="46" t="s">
+        <v>677</v>
+      </c>
+      <c r="G239" s="46" t="s">
         <v>639</v>
       </c>
-      <c r="G238" s="34" t="s">
+      <c r="H239" s="46" t="s">
+        <v>307</v>
+      </c>
+      <c r="I239" s="46" t="s">
         <v>640</v>
       </c>
-      <c r="H238" s="34" t="s">
+      <c r="J239" s="46" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="239" spans="1:14" s="34" customFormat="1">
-      <c r="A239" s="34" t="s">
-        <v>96</v>
-      </c>
-      <c r="B239" s="34" t="s">
+      <c r="K239" s="46" t="s">
+        <v>73</v>
+      </c>
+      <c r="L239" s="46" t="s">
+        <v>307</v>
+      </c>
+      <c r="M239" s="46" t="s">
+        <v>74</v>
+      </c>
+      <c r="N239" s="46" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="240" spans="1:14" s="22" customFormat="1">
+      <c r="A240" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="B240" s="22" t="s">
+        <v>683</v>
+      </c>
+      <c r="C240" s="22" t="s">
+        <v>260</v>
+      </c>
+      <c r="D240" s="45" t="s">
+        <v>684</v>
+      </c>
+      <c r="E240" s="22" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="241" spans="1:14">
+      <c r="A241" t="s">
+        <v>96</v>
+      </c>
+      <c r="B241" t="s">
         <v>637</v>
       </c>
-      <c r="C239" s="34" t="s">
+      <c r="C241" t="s">
         <v>260</v>
       </c>
-      <c r="D239" s="45" t="s">
+      <c r="D241" t="s">
         <v>635</v>
       </c>
-      <c r="E239" s="34" t="s">
-        <v>675</v>
-      </c>
-      <c r="F239" s="34" t="s">
-        <v>679</v>
-      </c>
-      <c r="G239" s="34" t="s">
-        <v>641</v>
-      </c>
-      <c r="H239" s="34" t="s">
+      <c r="E241" t="s">
+        <v>674</v>
+      </c>
+      <c r="F241" t="s">
+        <v>678</v>
+      </c>
+      <c r="G241" t="s">
+        <v>639</v>
+      </c>
+      <c r="H241" t="s">
         <v>307</v>
       </c>
-      <c r="I239" s="34" t="s">
-        <v>642</v>
-      </c>
-      <c r="J239" s="34" t="s">
+      <c r="I241" t="s">
+        <v>640</v>
+      </c>
+      <c r="J241" t="s">
         <v>307</v>
       </c>
-      <c r="K239" s="34" t="s">
+      <c r="K241" t="s">
         <v>73</v>
       </c>
-      <c r="L239" s="34" t="s">
+      <c r="L241" t="s">
         <v>307</v>
       </c>
-      <c r="M239" s="34" t="s">
+      <c r="M241" t="s">
         <v>74</v>
       </c>
-      <c r="N239" s="34" t="s">
+      <c r="N241" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="240" spans="1:14">
-      <c r="A240" t="s">
-        <v>96</v>
-      </c>
-      <c r="B240" t="s">
-        <v>638</v>
-      </c>
-      <c r="C240" t="s">
+    <row r="242" spans="1:14" s="22" customFormat="1">
+      <c r="A242" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="B242" s="22" t="s">
+        <v>686</v>
+      </c>
+      <c r="C242" s="22" t="s">
         <v>260</v>
       </c>
-      <c r="D240" t="s">
-        <v>635</v>
-      </c>
-      <c r="E240" t="s">
-        <v>676</v>
-      </c>
-      <c r="F240" t="s">
-        <v>680</v>
-      </c>
-      <c r="G240" t="s">
-        <v>641</v>
-      </c>
-      <c r="H240" t="s">
-        <v>307</v>
-      </c>
-      <c r="I240" t="s">
-        <v>642</v>
-      </c>
-      <c r="J240" t="s">
-        <v>307</v>
-      </c>
-      <c r="K240" t="s">
-        <v>73</v>
-      </c>
-      <c r="L240" t="s">
-        <v>307</v>
-      </c>
-      <c r="M240" t="s">
-        <v>74</v>
-      </c>
-      <c r="N240" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="241" spans="1:6">
-      <c r="A241" t="s">
-        <v>96</v>
-      </c>
-      <c r="B241" t="s">
+      <c r="D242" s="45" t="s">
+        <v>684</v>
+      </c>
+      <c r="E242" s="22" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="243" spans="1:14">
+      <c r="A243" t="s">
+        <v>96</v>
+      </c>
+      <c r="B243" t="s">
+        <v>644</v>
+      </c>
+      <c r="C243" t="s">
+        <v>654</v>
+      </c>
+      <c r="D243" s="38" t="s">
+        <v>655</v>
+      </c>
+      <c r="E243" s="2" t="s">
+        <v>645</v>
+      </c>
+      <c r="F243" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="244" spans="1:14">
+      <c r="A244" t="s">
+        <v>96</v>
+      </c>
+      <c r="B244" t="s">
+        <v>56</v>
+      </c>
+      <c r="C244" t="s">
+        <v>654</v>
+      </c>
+      <c r="D244" s="38" t="s">
+        <v>655</v>
+      </c>
+      <c r="E244" s="2" t="s">
         <v>646</v>
       </c>
-      <c r="C241" t="s">
+      <c r="F244" t="s">
         <v>656</v>
       </c>
-      <c r="D241" s="38" t="s">
-        <v>657</v>
-      </c>
-      <c r="E241" s="2" t="s">
+    </row>
+    <row r="245" spans="1:14">
+      <c r="A245" t="s">
+        <v>96</v>
+      </c>
+      <c r="B245" t="s">
+        <v>55</v>
+      </c>
+      <c r="C245" t="s">
+        <v>654</v>
+      </c>
+      <c r="D245" s="38" t="s">
+        <v>655</v>
+      </c>
+      <c r="E245" s="2" t="s">
         <v>647</v>
       </c>
-      <c r="F241" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="242" spans="1:6">
-      <c r="A242" t="s">
-        <v>96</v>
-      </c>
-      <c r="B242" t="s">
-        <v>56</v>
-      </c>
-      <c r="C242" t="s">
+      <c r="F245" t="s">
         <v>656</v>
       </c>
-      <c r="D242" s="38" t="s">
-        <v>657</v>
-      </c>
-      <c r="E242" s="2" t="s">
+    </row>
+    <row r="246" spans="1:14">
+      <c r="A246" t="s">
+        <v>96</v>
+      </c>
+      <c r="B246" t="s">
+        <v>54</v>
+      </c>
+      <c r="C246" t="s">
+        <v>654</v>
+      </c>
+      <c r="D246" s="38" t="s">
+        <v>655</v>
+      </c>
+      <c r="E246" s="2" t="s">
         <v>648</v>
       </c>
-      <c r="F242" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="243" spans="1:6">
-      <c r="A243" t="s">
-        <v>96</v>
-      </c>
-      <c r="B243" t="s">
-        <v>55</v>
-      </c>
-      <c r="C243" t="s">
+      <c r="F246" t="s">
         <v>656</v>
       </c>
-      <c r="D243" s="38" t="s">
-        <v>657</v>
-      </c>
-      <c r="E243" s="2" t="s">
+    </row>
+    <row r="247" spans="1:14">
+      <c r="A247" t="s">
+        <v>96</v>
+      </c>
+      <c r="B247" t="s">
+        <v>53</v>
+      </c>
+      <c r="C247" t="s">
+        <v>654</v>
+      </c>
+      <c r="D247" s="38" t="s">
+        <v>655</v>
+      </c>
+      <c r="E247" s="2" t="s">
         <v>649</v>
       </c>
-      <c r="F243" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="244" spans="1:6">
-      <c r="A244" t="s">
-        <v>96</v>
-      </c>
-      <c r="B244" t="s">
-        <v>54</v>
-      </c>
-      <c r="C244" t="s">
+      <c r="F247" t="s">
         <v>656</v>
       </c>
-      <c r="D244" s="38" t="s">
-        <v>657</v>
-      </c>
-      <c r="E244" s="2" t="s">
+    </row>
+    <row r="248" spans="1:14">
+      <c r="A248" t="s">
+        <v>96</v>
+      </c>
+      <c r="B248" t="s">
+        <v>52</v>
+      </c>
+      <c r="C248" t="s">
+        <v>654</v>
+      </c>
+      <c r="D248" s="38" t="s">
+        <v>655</v>
+      </c>
+      <c r="E248" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="F244" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="245" spans="1:6">
-      <c r="A245" t="s">
-        <v>96</v>
-      </c>
-      <c r="B245" t="s">
-        <v>53</v>
-      </c>
-      <c r="C245" t="s">
+      <c r="F248" t="s">
         <v>656</v>
       </c>
-      <c r="D245" s="38" t="s">
-        <v>657</v>
-      </c>
-      <c r="E245" s="2" t="s">
+    </row>
+    <row r="249" spans="1:14">
+      <c r="A249" t="s">
+        <v>96</v>
+      </c>
+      <c r="B249" t="s">
+        <v>51</v>
+      </c>
+      <c r="C249" t="s">
+        <v>654</v>
+      </c>
+      <c r="D249" s="38" t="s">
+        <v>655</v>
+      </c>
+      <c r="E249" s="2" t="s">
         <v>651</v>
       </c>
-      <c r="F245" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="246" spans="1:6">
-      <c r="A246" t="s">
-        <v>96</v>
-      </c>
-      <c r="B246" t="s">
-        <v>52</v>
-      </c>
-      <c r="C246" t="s">
+      <c r="F249" t="s">
         <v>656</v>
       </c>
-      <c r="D246" s="38" t="s">
-        <v>657</v>
-      </c>
-      <c r="E246" s="2" t="s">
+    </row>
+    <row r="250" spans="1:14">
+      <c r="A250" t="s">
+        <v>96</v>
+      </c>
+      <c r="B250" t="s">
+        <v>50</v>
+      </c>
+      <c r="C250" t="s">
+        <v>654</v>
+      </c>
+      <c r="D250" s="38" t="s">
+        <v>655</v>
+      </c>
+      <c r="E250" s="2" t="s">
         <v>652</v>
       </c>
-      <c r="F246" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="247" spans="1:6">
-      <c r="A247" t="s">
-        <v>96</v>
-      </c>
-      <c r="B247" t="s">
-        <v>51</v>
-      </c>
-      <c r="C247" t="s">
+      <c r="F250" t="s">
         <v>656</v>
-      </c>
-      <c r="D247" s="38" t="s">
-        <v>657</v>
-      </c>
-      <c r="E247" s="2" t="s">
-        <v>653</v>
-      </c>
-      <c r="F247" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="248" spans="1:6">
-      <c r="A248" t="s">
-        <v>96</v>
-      </c>
-      <c r="B248" t="s">
-        <v>50</v>
-      </c>
-      <c r="C248" t="s">
-        <v>656</v>
-      </c>
-      <c r="D248" s="38" t="s">
-        <v>657</v>
-      </c>
-      <c r="E248" s="2" t="s">
-        <v>654</v>
-      </c>
-      <c r="F248" t="s">
-        <v>658</v>
       </c>
     </row>
   </sheetData>
@@ -11329,7 +11418,7 @@
     </row>
     <row r="43" spans="1:41">
       <c r="A43" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
     </row>
     <row r="44" spans="1:41" s="10" customFormat="1">
@@ -11446,10 +11535,10 @@
     </row>
     <row r="2" spans="1:10" ht="61.5" customHeight="1">
       <c r="A2" s="22" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="C2" t="s">
         <v>169</v>
@@ -11556,7 +11645,7 @@
     </row>
     <row r="6" spans="1:10" s="31" customFormat="1" ht="29">
       <c r="A6" s="31" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B6" s="32" t="s">
         <v>509</v>
@@ -11585,7 +11674,7 @@
     </row>
     <row r="7" spans="1:10" s="31" customFormat="1">
       <c r="A7" s="31" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B7" s="32" t="s">
         <v>509</v>
@@ -11609,7 +11698,7 @@
     </row>
     <row r="8" spans="1:10" s="31" customFormat="1">
       <c r="A8" s="31" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B8" s="32"/>
       <c r="D8" s="31" t="s">
@@ -11717,7 +11806,7 @@
     </row>
     <row r="14" spans="1:10" s="31" customFormat="1" ht="43.5">
       <c r="A14" s="33" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="B14" s="32" t="s">
         <v>508</v>
@@ -11905,7 +11994,7 @@
     </row>
     <row r="21" spans="1:10" s="34" customFormat="1" ht="29">
       <c r="A21" s="34" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="B21" s="35" t="s">
         <v>508</v>
@@ -12379,7 +12468,7 @@
     </row>
     <row r="42" spans="1:9">
       <c r="A42" s="39" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="B42" s="40"/>
       <c r="C42" s="39"/>
@@ -12390,18 +12479,18 @@
     </row>
     <row r="43" spans="1:9" s="7" customFormat="1">
       <c r="A43" s="43" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="B43" s="7" t="s">
         <v>464</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="D43" s="6"/>
       <c r="E43" s="6"/>
       <c r="F43" s="7" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="G43" s="7" t="s">
         <v>77</v>
@@ -12412,55 +12501,55 @@
     </row>
     <row r="44" spans="1:9">
       <c r="A44" s="39" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B44" s="39"/>
       <c r="C44" s="39" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="D44" s="41"/>
       <c r="F44" s="39" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="G44" s="39" t="s">
         <v>77</v>
       </c>
       <c r="H44" s="39" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
     </row>
     <row r="45" spans="1:9" s="12" customFormat="1">
       <c r="A45" s="12" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="B45" s="44" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="D45" s="16"/>
       <c r="E45" s="16"/>
       <c r="F45" s="12" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="G45" s="12" t="s">
         <v>77</v>
       </c>
       <c r="H45" s="12" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
     </row>
     <row r="46" spans="1:9" s="4" customFormat="1">
       <c r="A46" s="4" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="B46" s="42"/>
       <c r="E46" s="3"/>
     </row>
     <row r="47" spans="1:9" s="7" customFormat="1">
       <c r="A47" s="7" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B47" s="43"/>
       <c r="E47" s="6"/>

</xml_diff>